<commit_message>
fix: Update deploy-prod.yml for consistency and improve formatting
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEA0539A-E3B2-471B-A5C3-C935FFE7D995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5714CB3A-6746-40FF-BD27-9210676A98A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,8 @@
     <sheet name="ToDo" sheetId="2" r:id="rId3"/>
     <sheet name="linter" sheetId="3" r:id="rId4"/>
     <sheet name="テストカバレッジ" sheetId="5" r:id="rId5"/>
+    <sheet name="API呼び出し" sheetId="6" r:id="rId6"/>
+    <sheet name="不具合修正" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -104,6 +106,46 @@
     <t>テスト対象</t>
     <rPh sb="3" eb="5">
       <t>タイショウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>flutter pub run build_runner build --delete-conflicting-outputs</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>dart run build_runner build --delete-conflicting-outputs
+flutter test --coverage</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>flutter clean
+flutter pub get
+dart fix --apply
+dart format .
+flutter analyze
+dart run build_runner build --delete-conflicting-outputs
+flutter test --coverage</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リアル断捨離カメラ</t>
+    <rPh sb="3" eb="6">
+      <t>ダンシャリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AI稼働モニター</t>
+    <rPh sb="2" eb="4">
+      <t>カドウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CI/CDのスラック通知でエラー</t>
+    <rPh sb="10" eb="12">
+      <t>ツウチ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -456,11 +498,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBDB197-A587-49EA-9FC4-8E4B6580D845}">
-  <dimension ref="B3:D8"/>
+  <dimension ref="B3:D11"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="60" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4">
@@ -510,6 +552,33 @@
       </c>
       <c r="C8" s="1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="B9">
+        <f>B8+1</f>
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="131.25">
+      <c r="B10">
+        <f>B9+1</f>
+        <v>7</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="37.5">
+      <c r="B11">
+        <f>B10+1</f>
+        <v>8</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -633,4 +702,66 @@
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
+  <dimension ref="B3:E4"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3">
+        <v>46036</v>
+      </c>
+      <c r="E3" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCCFC25C-982C-4873-AE2A-E40A864E9987}">
+  <dimension ref="B3:C3"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:3">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Refactor AI model fetching and response handling in ai_status_page.dart; update Supabase function to return model data; enhance error handling and null safety; modify tests for improved clarity and functionality.
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5714CB3A-6746-40FF-BD27-9210676A98A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11DD3DF-60F9-45A0-B3DA-09D2ED780F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -147,6 +147,10 @@
     <rPh sb="10" eb="12">
       <t>ツウチ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>404 not found</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -706,15 +710,17 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
-  <dimension ref="B3:E4"/>
+  <dimension ref="B3:F4"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:5">
+    <row r="3" spans="2:6">
       <c r="B3">
         <v>1</v>
       </c>
@@ -724,17 +730,24 @@
       <c r="D3" s="3">
         <v>46036</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="3"/>
+      <c r="F3" s="3">
         <v>46036</v>
       </c>
     </row>
-    <row r="4" spans="2:5">
+    <row r="4" spans="2:6">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
       </c>
       <c r="C4" t="s">
         <v>17</v>
+      </c>
+      <c r="D4" s="3">
+        <v>46036</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -745,19 +758,23 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCCFC25C-982C-4873-AE2A-E40A864E9987}">
-  <dimension ref="B3:C3"/>
+  <dimension ref="B3:D3"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:3">
+    <row r="3" spans="2:4">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>18</v>
+      </c>
+      <c r="D3" s="3">
+        <v>46036</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update my_web_app.xlsx with latest changes
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F11DD3DF-60F9-45A0-B3DA-09D2ED780F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CC6565-4B82-4BFF-A38A-050E828ED859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="テストカバレッジ" sheetId="5" r:id="rId5"/>
     <sheet name="API呼び出し" sheetId="6" r:id="rId6"/>
     <sheet name="不具合修正" sheetId="7" r:id="rId7"/>
+    <sheet name="機能一覧" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -116,6 +117,35 @@
   <si>
     <t>dart run build_runner build --delete-conflicting-outputs
 flutter test --coverage</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リアル断捨離カメラ</t>
+    <rPh sb="3" eb="6">
+      <t>ダンシャリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AI稼働モニター</t>
+    <rPh sb="2" eb="4">
+      <t>カドウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CI/CDのスラック通知でエラー</t>
+    <rPh sb="10" eb="12">
+      <t>ツウチ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>404 not found</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase functions deploy ai-assistant</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -125,32 +155,21 @@
 dart format .
 flutter analyze
 dart run build_runner build --delete-conflicting-outputs
-flutter test --coverage</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>リアル断捨離カメラ</t>
-    <rPh sb="3" eb="6">
-      <t>ダンシャリ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>AI稼働モニター</t>
+flutter test --coverage
+supabase functions deploy ai-assistant</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>緊急役員会議</t>
+    <rPh sb="0" eb="2">
+      <t>キンキュウ</t>
+    </rPh>
     <rPh sb="2" eb="4">
-      <t>カドウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>CI/CDのスラック通知でエラー</t>
-    <rPh sb="10" eb="12">
-      <t>ツウチ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>404 not found</t>
+      <t>ヤクイン</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>カイギ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -502,7 +521,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBDB197-A587-49EA-9FC4-8E4B6580D845}">
-  <dimension ref="B3:D11"/>
+  <dimension ref="B3:D12"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -567,13 +586,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="131.25">
+    <row r="10" spans="2:4" ht="150">
       <c r="B10">
         <f>B9+1</f>
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="37.5">
@@ -583,6 +602,15 @@
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4">
+      <c r="B12">
+        <f>B11+1</f>
+        <v>9</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -710,7 +738,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
-  <dimension ref="B3:F4"/>
+  <dimension ref="B2:F5"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -720,12 +748,20 @@
     <col min="6" max="6" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="2" spans="2:6">
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+    </row>
     <row r="3" spans="2:6">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" s="3">
         <v>46036</v>
@@ -741,13 +777,22 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D4" s="3">
         <v>46036</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>18</v>
+      </c>
+      <c r="F4" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -771,7 +816,39 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="D3" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
+  <dimension ref="B2:D3"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4">
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
       </c>
       <c r="D3" s="3">
         <v>46036</v>

</xml_diff>

<commit_message>
fix: Update Slack notification payloads for deployment success and failure
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37890C47-556A-44E4-BFA6-1A10E24B2EBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9500DFD-1078-444A-92E2-0B9B42F6BDAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -907,7 +907,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
-  <dimension ref="B2:D3"/>
+  <dimension ref="B2:E3"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -915,12 +915,15 @@
     <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4">
+    <row r="2" spans="2:5">
       <c r="D2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="2:4">
+      <c r="E2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
       <c r="B3">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Refactor Gemini University Page and Update Imports
- Renamed 'gemini_university_page.dart' to 'gemini_university_v2_page.dart' and updated all relevant imports.
- Enhanced coverage in various files, increasing line execution counts.
- Added new 'GeminiUniversityPage' class with curriculum and quiz functionalities.
- Updated 'main.dart' and 'home_page.dart' to reflect the new page structure.
- Adjusted test files to include the new page.
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9500DFD-1078-444A-92E2-0B9B42F6BDAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE5C30F-864A-43C6-8A05-143762C3E131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -186,6 +186,189 @@
   </si>
   <si>
     <t>lib\pages\emergency_meeting_page.dart</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>断捨離（デジタル）</t>
+    <rPh sb="0" eb="3">
+      <t>ダンシャリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>断捨離（リアル）</t>
+    <rPh sb="0" eb="3">
+      <t>ダンシャリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>財務管理（CFO）</t>
+    <rPh sb="0" eb="2">
+      <t>ザイム</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>固定費削減室（サブスク管理）</t>
+    <rPh sb="0" eb="3">
+      <t>コテイヒ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>サクゲン</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>シツ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>決済チャネル台帳</t>
+    <rPh sb="0" eb="2">
+      <t>ケッサイ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ダイチョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>月次決算レポート</t>
+    <rPh sb="0" eb="2">
+      <t>ゲツジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ケッサン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>健康管理（CHO）</t>
+    <rPh sb="0" eb="2">
+      <t>ケンコウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>健康管理室（Health Log）</t>
+    <rPh sb="0" eb="2">
+      <t>ケンコウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>シツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>メンタルチェック</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>定期健康診断</t>
+    <rPh sb="0" eb="2">
+      <t>テイキ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ケンコウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>シンダン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人事厚生（CHRO）</t>
+    <rPh sb="0" eb="2">
+      <t>ジンジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>福利厚生課（Rewards）</t>
+    <rPh sb="0" eb="2">
+      <t>フクリ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウセイ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人事評価室（Stats）</t>
+    <rPh sb="0" eb="2">
+      <t>ジンジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒョウカ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>シツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>社員研修センター（Help）</t>
+    <rPh sb="0" eb="2">
+      <t>シャイン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ケンシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>市場分析（CMO）</t>
+    <rPh sb="0" eb="2">
+      <t>シジョウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ブンセキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>メモ一覧（CKO）</t>
+    <rPh sb="2" eb="4">
+      <t>イチラン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>新規事業起案</t>
+    <rPh sb="0" eb="2">
+      <t>シンキ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ジギョウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>キアン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini大学</t>
+    <rPh sb="6" eb="8">
+      <t>ダイガク</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -907,31 +1090,224 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
-  <dimension ref="B2:E3"/>
+  <dimension ref="B2:F19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5">
-      <c r="D2" t="s">
+    <row r="2" spans="2:6">
+      <c r="E2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:5">
+    <row r="3" spans="2:6">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="3">
-        <v>46036</v>
+      <c r="E3" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F3" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F4" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="5" spans="2:6">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F5" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F6" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F7" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6">
+      <c r="B9">
+        <f>B8+1</f>
+        <v>7</v>
+      </c>
+      <c r="D9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6">
+      <c r="B10">
+        <f>B9+1</f>
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F10" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="11" spans="2:6">
+      <c r="B11">
+        <f>B10+1</f>
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6">
+      <c r="B12">
+        <f>B11+1</f>
+        <v>10</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6">
+      <c r="B13">
+        <f>B12+1</f>
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E13" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F13" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6">
+      <c r="B14">
+        <f>B13+1</f>
+        <v>12</v>
+      </c>
+      <c r="D14" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15" spans="2:6">
+      <c r="B15">
+        <f>B14+1</f>
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6">
+      <c r="B16">
+        <f>B15+1</f>
+        <v>14</v>
+      </c>
+      <c r="C16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17">
+        <f>B16+1</f>
+        <v>15</v>
+      </c>
+      <c r="C17" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18">
+        <f>B17+1</f>
+        <v>16</v>
+      </c>
+      <c r="C18" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19">
+        <f>B18+1</f>
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update Slack GitHub action version and enhance success notification message
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE5C30F-864A-43C6-8A05-143762C3E131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71720FE9-08C1-4986-B920-31C03F7BEACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
     <sheet name="コマンド一覧" sheetId="4" r:id="rId2"/>
-    <sheet name="ToDo" sheetId="2" r:id="rId3"/>
-    <sheet name="linter" sheetId="3" r:id="rId4"/>
-    <sheet name="テストカバレッジ" sheetId="5" r:id="rId5"/>
-    <sheet name="API呼び出し" sheetId="6" r:id="rId6"/>
-    <sheet name="不具合修正" sheetId="7" r:id="rId7"/>
-    <sheet name="機能一覧" sheetId="8" r:id="rId8"/>
+    <sheet name="VSCodeExtensions" sheetId="9" r:id="rId3"/>
+    <sheet name="ToDo" sheetId="2" r:id="rId4"/>
+    <sheet name="linter" sheetId="3" r:id="rId5"/>
+    <sheet name="テストカバレッジ" sheetId="5" r:id="rId6"/>
+    <sheet name="API呼び出し" sheetId="6" r:id="rId7"/>
+    <sheet name="不具合修正" sheetId="7" r:id="rId8"/>
+    <sheet name="機能一覧" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -146,6 +147,218 @@
   </si>
   <si>
     <t>supabase functions deploy ai-assistant</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>緊急役員会議</t>
+    <rPh sb="0" eb="2">
+      <t>キンキュウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヤクイン</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>カイギ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>lib\main.dart</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>lib\models\board_meeting_model.dart</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>lib\pages\ai_status_page.dart</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>lib\pages\emergency_meeting_page.dart</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>断捨離（デジタル）</t>
+    <rPh sb="0" eb="3">
+      <t>ダンシャリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>断捨離（リアル）</t>
+    <rPh sb="0" eb="3">
+      <t>ダンシャリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>財務管理（CFO）</t>
+    <rPh sb="0" eb="2">
+      <t>ザイム</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>固定費削減室（サブスク管理）</t>
+    <rPh sb="0" eb="3">
+      <t>コテイヒ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>サクゲン</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>シツ</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>決済チャネル台帳</t>
+    <rPh sb="0" eb="2">
+      <t>ケッサイ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ダイチョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>月次決算レポート</t>
+    <rPh sb="0" eb="2">
+      <t>ゲツジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ケッサン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>健康管理（CHO）</t>
+    <rPh sb="0" eb="2">
+      <t>ケンコウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>健康管理室（Health Log）</t>
+    <rPh sb="0" eb="2">
+      <t>ケンコウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>シツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>メンタルチェック</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>定期健康診断</t>
+    <rPh sb="0" eb="2">
+      <t>テイキ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ケンコウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>シンダン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人事厚生（CHRO）</t>
+    <rPh sb="0" eb="2">
+      <t>ジンジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>福利厚生課（Rewards）</t>
+    <rPh sb="0" eb="2">
+      <t>フクリ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウセイ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人事評価室（Stats）</t>
+    <rPh sb="0" eb="2">
+      <t>ジンジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ヒョウカ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>シツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>社員研修センター（Help）</t>
+    <rPh sb="0" eb="2">
+      <t>シャイン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ケンシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>市場分析（CMO）</t>
+    <rPh sb="0" eb="2">
+      <t>シジョウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ブンセキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>メモ一覧（CKO）</t>
+    <rPh sb="2" eb="4">
+      <t>イチラン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>新規事業起案</t>
+    <rPh sb="0" eb="2">
+      <t>シンキ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ジギョウ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>キアン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini大学</t>
+    <rPh sb="6" eb="8">
+      <t>ダイガク</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -156,219 +369,12 @@
 flutter analyze
 dart run build_runner build --delete-conflicting-outputs
 flutter test --coverage
-supabase functions deploy ai-assistant</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>緊急役員会議</t>
-    <rPh sb="0" eb="2">
-      <t>キンキュウ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ヤクイン</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>カイギ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>lib\main.dart</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>lib\models\board_meeting_model.dart</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>lib\pages\ai_status_page.dart</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>lib\pages\emergency_meeting_page.dart</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>断捨離（デジタル）</t>
-    <rPh sb="0" eb="3">
-      <t>ダンシャリ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>断捨離（リアル）</t>
-    <rPh sb="0" eb="3">
-      <t>ダンシャリ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>財務管理（CFO）</t>
-    <rPh sb="0" eb="2">
-      <t>ザイム</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>カンリ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>固定費削減室（サブスク管理）</t>
-    <rPh sb="0" eb="3">
-      <t>コテイヒ</t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t>サクゲン</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>シツ</t>
-    </rPh>
-    <rPh sb="11" eb="13">
-      <t>カンリ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>決済チャネル台帳</t>
-    <rPh sb="0" eb="2">
-      <t>ケッサイ</t>
-    </rPh>
-    <rPh sb="6" eb="8">
-      <t>ダイチョウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>月次決算レポート</t>
-    <rPh sb="0" eb="2">
-      <t>ゲツジ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ケッサン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>健康管理（CHO）</t>
-    <rPh sb="0" eb="2">
-      <t>ケンコウ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>カンリ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>健康管理室（Health Log）</t>
-    <rPh sb="0" eb="2">
-      <t>ケンコウ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>カンリ</t>
-    </rPh>
-    <rPh sb="4" eb="5">
-      <t>シツ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>メンタルチェック</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>定期健康診断</t>
-    <rPh sb="0" eb="2">
-      <t>テイキ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ケンコウ</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>シンダン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>人事厚生（CHRO）</t>
-    <rPh sb="0" eb="2">
-      <t>ジンジ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>コウセイ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>福利厚生課（Rewards）</t>
-    <rPh sb="0" eb="2">
-      <t>フクリ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>コウセイ</t>
-    </rPh>
-    <rPh sb="4" eb="5">
-      <t>カ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>人事評価室（Stats）</t>
-    <rPh sb="0" eb="2">
-      <t>ジンジ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ヒョウカ</t>
-    </rPh>
-    <rPh sb="4" eb="5">
-      <t>シツ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>社員研修センター（Help）</t>
-    <rPh sb="0" eb="2">
-      <t>シャイン</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ケンシュウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>市場分析（CMO）</t>
-    <rPh sb="0" eb="2">
-      <t>シジョウ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ブンセキ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>メモ一覧（CKO）</t>
-    <rPh sb="2" eb="4">
-      <t>イチラン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>新規事業起案</t>
-    <rPh sb="0" eb="2">
-      <t>シンキ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ジギョウ</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>キアン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Gemini大学</t>
-    <rPh sb="6" eb="8">
-      <t>ダイガク</t>
-    </rPh>
+supabase functions deploy ai-assistant
+flutter build web --release --no-tree-shake-icons</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GitHub Copilot Chat</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -786,13 +792,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="150">
+    <row r="10" spans="2:4" ht="168.75">
       <c r="B10">
         <f>B9+1</f>
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="37.5">
@@ -820,6 +826,42 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{831F138C-7B13-4940-8512-4B95D1A24D44}">
+  <dimension ref="B2:F3"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6">
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="2:6">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="3">
+        <v>46037</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB9A9986-272E-4F2B-8815-9B72212F3499}">
   <dimension ref="B3:F5"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -871,7 +913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEF53A6-A89B-421F-A561-8936407ADCF5}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -881,7 +923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62C7C188-6DA4-4CDE-8831-D70FA561BA5F}">
   <dimension ref="B3:G8"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -927,7 +969,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E5" s="3">
         <v>46031</v>
@@ -945,7 +987,7 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="3">
         <v>46036</v>
@@ -963,7 +1005,7 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E7" s="3">
         <v>46036</v>
@@ -981,7 +1023,7 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" s="3">
         <v>46036</v>
@@ -996,7 +1038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
   <dimension ref="B2:F5"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -1061,7 +1103,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCCFC25C-982C-4873-AE2A-E40A864E9987}">
   <dimension ref="B3:D3"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -1088,7 +1130,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
   <dimension ref="B2:F19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -1112,7 +1154,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E3" s="3">
         <v>46036</v>
@@ -1127,7 +1169,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E4" s="3">
         <v>46036</v>
@@ -1142,7 +1184,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" s="3">
         <v>46036</v>
@@ -1172,10 +1214,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
         <v>28</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
       </c>
       <c r="E7" s="3">
         <v>46036</v>
@@ -1190,7 +1232,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="2:6">
@@ -1199,7 +1241,7 @@
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="2:6">
@@ -1208,10 +1250,10 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
         <v>32</v>
-      </c>
-      <c r="D10" t="s">
-        <v>33</v>
       </c>
       <c r="E10" s="3">
         <v>46036</v>
@@ -1226,7 +1268,7 @@
         <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="2:6">
@@ -1235,7 +1277,7 @@
         <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="2:6">
@@ -1244,10 +1286,10 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" t="s">
         <v>36</v>
-      </c>
-      <c r="D13" t="s">
-        <v>37</v>
       </c>
       <c r="E13" s="3">
         <v>46036</v>
@@ -1262,7 +1304,7 @@
         <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" spans="2:6">
@@ -1271,7 +1313,7 @@
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="2:6">
@@ -1280,7 +1322,7 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="2:3">
@@ -1289,7 +1331,7 @@
         <v>15</v>
       </c>
       <c r="C17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="2:3">
@@ -1298,7 +1340,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="2:3">
@@ -1307,7 +1349,7 @@
         <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update Slack GitHub action version for deployment notifications
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71720FE9-08C1-4986-B920-31C03F7BEACD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63F5BEA-623D-499C-A9E7-82A61E6A02AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -375,6 +375,26 @@
   </si>
   <si>
     <t>GitHub Copilot Chat</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>改善着手</t>
+    <rPh sb="0" eb="2">
+      <t>カイゼン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>チャクシュ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>改善完了</t>
+    <rPh sb="0" eb="2">
+      <t>カイゼン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリョウ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1132,24 +1152,30 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
-  <dimension ref="B2:F19"/>
+  <dimension ref="B2:H19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6">
+    <row r="2" spans="2:8">
       <c r="E2" t="s">
         <v>1</v>
       </c>
       <c r="F2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="2:6">
+      <c r="G2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8">
       <c r="B3">
         <v>1</v>
       </c>
@@ -1163,7 +1189,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="4" spans="2:6">
+    <row r="4" spans="2:8">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
@@ -1178,7 +1204,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="5" spans="2:6">
+    <row r="5" spans="2:8">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
@@ -1193,7 +1219,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="6" spans="2:6">
+    <row r="6" spans="2:8">
       <c r="B6">
         <f>B5+1</f>
         <v>4</v>
@@ -1208,7 +1234,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="7" spans="2:6">
+    <row r="7" spans="2:8">
       <c r="B7">
         <f>B6+1</f>
         <v>5</v>
@@ -1226,7 +1252,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="8" spans="2:6">
+    <row r="8" spans="2:8">
       <c r="B8">
         <f>B7+1</f>
         <v>6</v>
@@ -1235,7 +1261,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="2:6">
+    <row r="9" spans="2:8">
       <c r="B9">
         <f>B8+1</f>
         <v>7</v>
@@ -1244,7 +1270,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="2:6">
+    <row r="10" spans="2:8">
       <c r="B10">
         <f>B9+1</f>
         <v>8</v>
@@ -1262,7 +1288,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="11" spans="2:6">
+    <row r="11" spans="2:8">
       <c r="B11">
         <f>B10+1</f>
         <v>9</v>
@@ -1271,7 +1297,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="2:6">
+    <row r="12" spans="2:8">
       <c r="B12">
         <f>B11+1</f>
         <v>10</v>
@@ -1280,7 +1306,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="2:6">
+    <row r="13" spans="2:8">
       <c r="B13">
         <f>B12+1</f>
         <v>11</v>
@@ -1298,7 +1324,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="14" spans="2:6">
+    <row r="14" spans="2:8">
       <c r="B14">
         <f>B13+1</f>
         <v>12</v>
@@ -1307,7 +1333,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="2:6">
+    <row r="15" spans="2:8">
       <c r="B15">
         <f>B14+1</f>
         <v>13</v>
@@ -1316,7 +1342,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="2:6">
+    <row r="16" spans="2:8">
       <c r="B16">
         <f>B15+1</f>
         <v>14</v>
@@ -1325,7 +1351,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" spans="2:3">
+    <row r="17" spans="2:7">
       <c r="B17">
         <f>B16+1</f>
         <v>15</v>
@@ -1334,7 +1360,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="2:3">
+    <row r="18" spans="2:7">
       <c r="B18">
         <f>B17+1</f>
         <v>16</v>
@@ -1343,13 +1369,22 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="2:3">
+    <row r="19" spans="2:7">
       <c r="B19">
         <f>B18+1</f>
         <v>17</v>
       </c>
       <c r="C19" t="s">
         <v>42</v>
+      </c>
+      <c r="E19" s="3">
+        <v>46037</v>
+      </c>
+      <c r="F19" s="3">
+        <v>46037</v>
+      </c>
+      <c r="G19" s="3">
+        <v>46037</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: enhance deployment notifications and improve official documentation structure
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63F5BEA-623D-499C-A9E7-82A61E6A02AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB59AE4D-B414-482C-AC25-0E2ADDBAE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="API呼び出し" sheetId="6" r:id="rId7"/>
     <sheet name="不具合修正" sheetId="7" r:id="rId8"/>
     <sheet name="機能一覧" sheetId="8" r:id="rId9"/>
+    <sheet name="デイリータスク" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -395,6 +396,27 @@
     <rPh sb="2" eb="4">
       <t>カンリョウ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>洗い物</t>
+    <rPh sb="0" eb="1">
+      <t>アラ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>モノ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>洗濯</t>
+    <rPh sb="0" eb="2">
+      <t>センタク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>シュレッダー</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -745,6 +767,174 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32515FA5-1C1F-4EBA-80C2-D5F40752231E}">
+  <dimension ref="B1:H19"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="2" spans="2:8">
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E3" s="3">
+        <v>46037</v>
+      </c>
+      <c r="F3" s="3">
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="2:8">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="2:8">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="2:8">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="2:8">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8">
+      <c r="B9">
+        <f>B8+1</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10">
+        <f>B9+1</f>
+        <v>8</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11">
+        <f>B10+1</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12">
+        <f>B11+1</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13">
+        <f>B12+1</f>
+        <v>11</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14">
+        <f>B13+1</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15">
+        <f>B14+1</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8">
+      <c r="B16">
+        <f>B15+1</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7">
+      <c r="B17">
+        <f>B16+1</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7">
+      <c r="B18">
+        <f>B17+1</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7">
+      <c r="B19">
+        <f>B18+1</f>
+        <v>17</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBDB197-A587-49EA-9FC4-8E4B6580D845}">
   <dimension ref="B3:D12"/>

</xml_diff>

<commit_message>
refactor: improve type safety and error handling in various pages and services
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB59AE4D-B414-482C-AC25-0E2ADDBAE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD06B287-9C16-4CF8-BE5E-08FA25043488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,8 @@
     <sheet name="不具合修正" sheetId="7" r:id="rId8"/>
     <sheet name="機能一覧" sheetId="8" r:id="rId9"/>
     <sheet name="デイリータスク" sheetId="10" r:id="rId10"/>
+    <sheet name="追加したい機能" sheetId="11" r:id="rId11"/>
+    <sheet name="Gemini API reference" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="63">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -417,6 +419,61 @@
   </si>
   <si>
     <t>シュレッダー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デイリーTODO管理</t>
+    <rPh sb="8" eb="10">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>本棚</t>
+    <rPh sb="0" eb="2">
+      <t>ホンダナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リマインダー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Gemini API</t>
+  </si>
+  <si>
+    <t>API reference</t>
+  </si>
+  <si>
+    <t>Gemini API reference</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini API リファレンス</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>We have updated our Terms of Service.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>利用規約を更新しました。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>This API reference describes the standard, streaming, and realtime APIs you can use to interact with the Gemini models.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>このAPIリファレンスは、Geminiモデルとのやり取りに使用できる標準API、ストリーミングAPI、リアルタイムAPIについて説明します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>You can use the REST APIs in any environment that supports HTTP requests.</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -469,7 +526,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -478,6 +535,9 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -935,6 +995,233 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A27E184-E904-4778-A996-9404F32C3EC7}">
+  <dimension ref="B1:H19"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="2" spans="2:8">
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="2:8">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="2:8">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="2:8">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="2:8">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="2:8">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8">
+      <c r="B9">
+        <f>B8+1</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10">
+        <f>B9+1</f>
+        <v>8</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11">
+        <f>B10+1</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12">
+        <f>B11+1</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13">
+        <f>B12+1</f>
+        <v>11</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14">
+        <f>B13+1</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15">
+        <f>B14+1</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8">
+      <c r="B16">
+        <f>B15+1</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7">
+      <c r="B17">
+        <f>B16+1</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7">
+      <c r="B18">
+        <f>B17+1</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7">
+      <c r="B19">
+        <f>B18+1</f>
+        <v>17</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
+  <dimension ref="B2:C9"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3">
+      <c r="B2" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3">
+      <c r="B3" s="6" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="B4" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3">
+      <c r="B6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" ht="56.25">
+      <c r="B8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" ht="37.5">
+      <c r="B9" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://ai.google.dev/" xr:uid="{D6844177-6821-498C-95D2-F6B6D63F1D22}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://ai.google.dev/gemini-api" xr:uid="{2CDC8D53-0630-4185-9E29-7B79EBBE1F53}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://ai.google.dev/api" xr:uid="{4A9752DB-169C-4F26-B3F6-A0018804884D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBDB197-A587-49EA-9FC4-8E4B6580D845}">
   <dimension ref="B3:D12"/>

</xml_diff>

<commit_message>
refactor: add Gemini API reference module with quiz and official documentation links
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD06B287-9C16-4CF8-BE5E-08FA25043488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AF72F14-9D89-4A94-91E8-0E1C0DA5FA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="66">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -474,6 +474,18 @@
   </si>
   <si>
     <t>You can use the REST APIs in any environment that supports HTTP requests.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>HTTPリクエストをサポートする環境であれば、どの環境でもREST APIを利用できます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Refer to the Quickstart guide for how to get started with your first API call.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最初のAPI呼び出しを開始する方法については、クイックスタートガイドを参照してください。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1160,11 +1172,11 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B2:C9"/>
+  <dimension ref="B2:C10"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="37.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.625" customWidth="1"/>
+    <col min="3" max="3" width="43.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3">
@@ -1209,6 +1221,17 @@
     <row r="9" spans="2:3" ht="37.5">
       <c r="B9" s="1" t="s">
         <v>62</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" ht="37.5">
+      <c r="B10" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update Gemini API documentation and quiz content for clarity
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AF72F14-9D89-4A94-91E8-0E1C0DA5FA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD8D538-CB16-4208-BE5C-D3F50219E798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="74">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -486,6 +486,38 @@
   </si>
   <si>
     <t>最初のAPI呼び出しを開始する方法については、クイックスタートガイドを参照してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>If you're looking for the references for our language-specific libraries and SDKs, go to the link for that language in the left navigation under SDK references.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>言語固有のライブラリおよびSDKの参照情報をお探しの場合は、左ナビゲーションの「SDKリファレンス」にある該当言語のリンクをご覧ください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Primary endpoints</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>主要評価項目</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>The Gemini API is organized around the following major endpoints:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini APIは以下の主要なエンドポイントを中心に構成されています：</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Standard content generation (generateContent): A standard REST endpoint that processes your request and returns the model's full response in a single package. This is best for non-interactive tasks where you can wait for the entire result.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>標準コンテンツ生成（generateContent）：リクエストを処理し、モデルの完全な応答を単一のパッケージで返す標準的なRESTエンドポイントです。結果全体を待機できる非対話型タスクに最適です。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1172,29 +1204,36 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B2:C10"/>
+  <dimension ref="B1:E17"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="37.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="43.5" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3">
+    <row r="1" spans="2:5">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="2:3">
+    <row r="3" spans="2:5">
       <c r="B3" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="2:3">
+    <row r="4" spans="2:5">
       <c r="B4" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="2:3">
+    <row r="6" spans="2:5">
       <c r="B6" t="s">
         <v>56</v>
       </c>
@@ -1202,7 +1241,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="2:3">
+    <row r="7" spans="2:5">
       <c r="B7" t="s">
         <v>58</v>
       </c>
@@ -1210,7 +1249,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="2:3" ht="56.25">
+    <row r="8" spans="2:5" ht="56.25">
       <c r="B8" s="1" t="s">
         <v>60</v>
       </c>
@@ -1218,7 +1257,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="37.5">
+    <row r="9" spans="2:5" ht="37.5">
       <c r="B9" s="1" t="s">
         <v>62</v>
       </c>
@@ -1226,12 +1265,47 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="37.5">
+    <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="75">
+      <c r="B11" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="3">
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5">
+      <c r="B13" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="37.5">
+      <c r="B15" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" ht="131.25">
+      <c r="B17" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update Gemini API documentation for accuracy and clarity
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AD8D538-CB16-4208-BE5C-D3F50219E798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73C22E3-D0DC-4AD6-9957-AD3CB988D3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -518,6 +518,29 @@
   </si>
   <si>
     <t>標準コンテンツ生成（generateContent）：リクエストを処理し、モデルの完全な応答を単一のパッケージで返す標準的なRESTエンドポイントです。結果全体を待機できる非対話型タスクに最適です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Streaming content generation (streamGenerateContent): Uses Server-Sent Events (SSE) to push chunks of the response to you as they are generated. This provides a faster, more interactive experience for applications like chatbots.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ストリーミングコンテンツ生成 (streamGenerateContent): サーバー送信イベント (SSE) を使用して、生成されたレスポンスのチャンクをプッシュ配信します。これにより、チャットボットなどのアプリケーションにおいて、より高速でインタラクティブな体験を提供します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Live API (BidiGenerateContent): A stateful WebSocket-based API for bi-directional streaming, designed for real-time conversational use cases.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ライブAPI（BidiGenerateContent）：双方向ストリーミングのためのステートフルWebSocketベースのAPI。リアルタイム会話ユースケース向けに設計されています。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>夕食</t>
+    <rPh sb="0" eb="2">
+      <t>ユウショク</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -943,6 +966,9 @@
         <f>B5+1</f>
         <v>4</v>
       </c>
+      <c r="C6" t="s">
+        <v>78</v>
+      </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
@@ -1204,7 +1230,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E17"/>
+  <dimension ref="B1:E19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="37.5" bestFit="1" customWidth="1"/>
@@ -1280,9 +1306,7 @@
       <c r="C11" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="3">
-        <v>46037</v>
-      </c>
+      <c r="E11" s="3"/>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="1" t="s">
@@ -1300,12 +1324,33 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="2:3" ht="131.25">
+    <row r="17" spans="2:5" ht="131.25">
       <c r="B17" s="1" t="s">
         <v>72</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>73</v>
+      </c>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="2:5" ht="112.5">
+      <c r="B18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="2:5" ht="75">
+      <c r="B19" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E19" s="3">
+        <v>46037</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: improve error handling and code readability in CmoPage, adjust padding in GeminiUniversityV2Page, and enhance sound notification in TimerService
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73C22E3-D0DC-4AD6-9957-AD3CB988D3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54335534-41BA-4E09-A5F8-7535551AA306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="83">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -541,6 +541,21 @@
     <rPh sb="0" eb="2">
       <t>ユウショク</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>linter!A1</t>
+  </si>
+  <si>
+    <t>○</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>lib\models\achievement.dart</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>lib\models\app_timer.dart</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -908,7 +923,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46037</v>
+        <v>46038</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -1078,7 +1093,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46037</v>
+        <v>46038</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -1241,7 +1256,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46037</v>
+        <v>46038</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -1502,7 +1517,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB9A9986-272E-4F2B-8815-9B72212F3499}">
-  <dimension ref="B3:F5"/>
+  <dimension ref="B3:F6"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -1527,6 +1542,9 @@
       <c r="C4" t="s">
         <v>0</v>
       </c>
+      <c r="D4" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="5" spans="2:6">
       <c r="B5">
@@ -1543,10 +1561,17 @@
         <v>46031</v>
       </c>
     </row>
+    <row r="6" spans="2:6">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
     <hyperlink ref="D5" location="テストカバレッジ!A1" display="テストカバレッジ!A1" xr:uid="{D25F68D0-C78F-4FF1-ABD2-D974080835FC}"/>
+    <hyperlink ref="D4" location="linter!A1" display="linter!A1" xr:uid="{2F08201A-392B-43E2-8926-23FB861EC50A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1564,7 +1589,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62C7C188-6DA4-4CDE-8831-D70FA561BA5F}">
-  <dimension ref="B3:G8"/>
+  <dimension ref="B3:H11"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -1574,7 +1599,7 @@
     <col min="7" max="7" width="7.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:7">
+    <row r="3" spans="2:8">
       <c r="C3" t="s">
         <v>12</v>
       </c>
@@ -1585,66 +1610,48 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="2:7">
+    <row r="4" spans="2:8">
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="3">
-        <v>46031</v>
-      </c>
-      <c r="F4" s="3">
-        <v>46031</v>
-      </c>
-      <c r="G4" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="2:7">
+        <v>21</v>
+      </c>
+      <c r="G4" s="5">
+        <v>0.80900000000000005</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8">
       <c r="B5">
         <f>B4+1</f>
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="3">
-        <v>46031</v>
-      </c>
-      <c r="F5" s="3">
-        <v>46036</v>
+        <v>81</v>
       </c>
       <c r="G5" s="5">
-        <v>0.82599999999999996</v>
-      </c>
-    </row>
-    <row r="6" spans="2:7">
+        <v>0.33300000000000002</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8">
       <c r="B6">
         <f>B5+1</f>
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" s="3">
-        <v>46036</v>
-      </c>
-      <c r="F6" s="3">
-        <v>46036</v>
+        <v>82</v>
       </c>
       <c r="G6" s="5">
-        <v>0.875</v>
-      </c>
-    </row>
-    <row r="7" spans="2:7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8">
       <c r="B7">
         <f>B6+1</f>
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="3">
         <v>46036</v>
@@ -1653,22 +1660,79 @@
         <v>46036</v>
       </c>
       <c r="G7" s="5">
-        <v>0.90500000000000003</v>
-      </c>
-    </row>
-    <row r="8" spans="2:7">
+        <v>0.95799999999999996</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8">
       <c r="B8">
         <f>B7+1</f>
         <v>5</v>
       </c>
       <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="3">
+        <v>46031</v>
+      </c>
+      <c r="F8" s="3">
+        <v>46031</v>
+      </c>
+      <c r="G8" s="4">
+        <v>1</v>
+      </c>
+      <c r="H8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8">
+      <c r="B9">
+        <f>B8+1</f>
+        <v>6</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="3">
+        <v>46031</v>
+      </c>
+      <c r="F9" s="3">
+        <v>46036</v>
+      </c>
+      <c r="G9" s="5">
+        <v>0.82599999999999996</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10">
+        <f>B9+1</f>
+        <v>7</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="3">
+        <v>46036</v>
+      </c>
+      <c r="F10" s="3">
+        <v>46036</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0.90500000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11">
+        <f>B10+1</f>
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="3">
-        <v>46036</v>
-      </c>
-      <c r="G8" s="5">
-        <v>0.127</v>
+      <c r="E11" s="3">
+        <v>46036</v>
+      </c>
+      <c r="G11" s="5">
+        <v>0.626</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: disable sound and browser notifications on web due to dart:html deprecation
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54335534-41BA-4E09-A5F8-7535551AA306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFC72C90-9A94-4B40-86CA-4E094BED60C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <sheet name="デイリータスク" sheetId="10" r:id="rId10"/>
     <sheet name="追加したい機能" sheetId="11" r:id="rId11"/>
     <sheet name="Gemini API reference" sheetId="12" r:id="rId12"/>
+    <sheet name="プロンプト集" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="90">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -557,6 +558,30 @@
   <si>
     <t>lib\models\app_timer.dart</t>
     <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Batch mode (batchGenerateContent): A standard REST endpoint for submitting batches of generateContent requests.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>バッチモード (batchGenerateContent): generateContentリクエストのバッチを送信するための標準的なRESTエンドポイント。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>下記をGemini大学機能に反映してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>コマンド一覧!A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   info - 'dart:html' is deprecated and shouldn't be used. Use package:web and dart:js_interop instead - lib\services\timer_service.dart:2:1 - deprecated_member_use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   info - Don't use web-only libraries outside Flutter web plugins - lib\services\timer_service.dart:2:1 - avoid_web_libraries_in_flutter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   info - Method invocation or property access on a 'dynamic' target - lib\widgets\note_editor\ai_assistant_menu.dart:76:24 - avoid_dynamic_calls</t>
   </si>
 </sst>
 </file>
@@ -901,10 +926,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="C3"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="16.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:3">
+      <c r="C3" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="C3" location="コマンド一覧!A1" display="コマンド一覧!A1" xr:uid="{513A6E0C-B4B5-4FF3-8DC6-4373BA414EA5}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1245,7 +1282,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E19"/>
+  <dimension ref="B1:E20"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="37.5" bestFit="1" customWidth="1"/>
@@ -1368,6 +1405,17 @@
         <v>46037</v>
       </c>
     </row>
+    <row r="20" spans="2:5" ht="56.25">
+      <c r="B20" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E20" s="3">
+        <v>46038</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
@@ -1379,8 +1427,169 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{475FE61E-6EC0-4C61-9FD0-98172694F2E5}">
+  <dimension ref="B1:H19"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="2" spans="2:8">
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>45</v>
+      </c>
+      <c r="H2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="2:8">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="2:8">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="2:8">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="2:8">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="2:8">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8">
+      <c r="B9">
+        <f>B8+1</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8">
+      <c r="B10">
+        <f>B9+1</f>
+        <v>8</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="2:8">
+      <c r="B11">
+        <f>B10+1</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12">
+        <f>B11+1</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8">
+      <c r="B13">
+        <f>B12+1</f>
+        <v>11</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14">
+        <f>B13+1</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8">
+      <c r="B15">
+        <f>B14+1</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8">
+      <c r="B16">
+        <f>B15+1</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7">
+      <c r="B17">
+        <f>B16+1</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7">
+      <c r="B18">
+        <f>B17+1</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7">
+      <c r="B19">
+        <f>B18+1</f>
+        <v>17</v>
+      </c>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBDB197-A587-49EA-9FC4-8E4B6580D845}">
+  <sheetPr>
+    <tabColor rgb="FFC00000"/>
+  </sheetPr>
   <dimension ref="B3:D12"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
@@ -1579,9 +1788,43 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEF53A6-A89B-421F-A561-8936407ADCF5}">
-  <dimension ref="A1"/>
+  <dimension ref="C2:E5"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="157.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:5">
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="3:5">
+      <c r="C3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5">
+      <c r="C4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5">
+      <c r="C5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D5" s="3">
+        <v>46038</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: add PaymentChannelLedgerPage with basic UI structure
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFC72C90-9A94-4B40-86CA-4E094BED60C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A5E4E8-224E-4CC3-81FC-B050EE3F3EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="4" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,7 @@
     <sheet name="追加したい機能" sheetId="11" r:id="rId11"/>
     <sheet name="Gemini API reference" sheetId="12" r:id="rId12"/>
     <sheet name="プロンプト集" sheetId="13" r:id="rId13"/>
+    <sheet name="Sheet13" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="102">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -583,12 +584,154 @@
   <si>
     <t xml:space="preserve">   info - Method invocation or property access on a 'dynamic' target - lib\widgets\note_editor\ai_assistant_menu.dart:76:24 - avoid_dynamic_calls</t>
   </si>
+  <si>
+    <t>未実装機能にはTODOコメントをつけてください。不要な機能は削除してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Embeddings (embedContent): A standard REST endpoint that generates a text embedding vector from the input Content.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>埋め込み（embedContent）：入力コンテンツからテキスト埋め込みベクトルを生成する標準的なRESTエンドポイント。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Step1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（朝）</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>まず「嫌な未来」をはっきりさせる（20〜30分）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最初にやるのは、理想探しじゃない。この先も続くとマズい人生を言語化する。紙にそのまま書く。
+・最近ずっと我慢している小さな不満は？
+・毎年同じように言ってる愚痴は？
+・このまま5年経った「普通の平日」はどんな1日？
+・10年後、何を失っていそう？
+ポイントは、感情が少し重くなるくらい、具体的に書くこと。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Step2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（朝）</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なぜ変われていないかを正直に書く
+・本当は何から逃げている？
+（失敗／評価／恥／安心／役割）
+・変わるために手放す必要がある「私はこういう人間だ」という思い込みは？
+ここは綺麗な答えじゃなくていい。ダサい本音でOK。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>なぜ変われていないかを正直に書く</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Step3（朝）</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最低限の「向かう先」を決める
+完璧な理想はいらない。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>低限の「向かう先」を決める
+完璧な理想はいらない。
+・3年後の「普通の平日」はどんな感じ？
+・その生活を送っている人にとって、今やろうとしている行動は「努力」？それとも「日常」？
+そして、これを1文で。
+私は「◯◯する人間」だ
+さらに、
+「その人なら今週、何を1つやる？」
+を決める。</t>
+    <phoneticPr fontId="1"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -610,6 +753,18 @@
       <name val="Yu Gothic"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1282,7 +1437,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E20"/>
+  <dimension ref="B1:E21"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="37.5" bestFit="1" customWidth="1"/>
@@ -1413,6 +1568,17 @@
         <v>84</v>
       </c>
       <c r="E20" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="56.25">
+      <c r="B21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="3">
         <v>46038</v>
       </c>
     </row>
@@ -1468,10 +1634,13 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="2:8">
+    <row r="4" spans="2:8" ht="37.5">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -1578,6 +1747,55 @@
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
+  <dimension ref="C3:E5"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="3" max="3" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="94" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:5" ht="206.25">
+      <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5" ht="150">
+      <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" ht="300">
+      <c r="C5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>101</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -2186,6 +2404,9 @@
       <c r="D8" t="s">
         <v>29</v>
       </c>
+      <c r="E8" s="3">
+        <v>46038</v>
+      </c>
     </row>
     <row r="9" spans="2:8">
       <c r="B9">

</xml_diff>

<commit_message>
refactor: improve database schema documentation for clarity and organization
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13A5E4E8-224E-4CC3-81FC-B050EE3F3EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D072C9-7383-490F-9030-67EE7A2C24CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="4" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="114">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -724,6 +724,105 @@
 さらに、
 「その人なら今週、何を1つやる？」
 を決める。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>こちらの詳細設計書にもとづいて、未実装な機能を実装してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CMO OFFICE（市場広報）</t>
+    <rPh sb="11" eb="13">
+      <t>シジョウ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>コウホウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>株主総会へ報告（SNSシェア）</t>
+    <rPh sb="0" eb="2">
+      <t>カブヌシ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ソウカイ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ホウコク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>市場調査（フィードバック）</t>
+    <rPh sb="0" eb="2">
+      <t>シジョウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>チョウサ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CKO OFFICE（知識）</t>
+    <rPh sb="11" eb="13">
+      <t>チシキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>保存</t>
+    <rPh sb="0" eb="2">
+      <t>ホゾン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>文章を洗練</t>
+    <rPh sb="0" eb="2">
+      <t>ブンショウ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>センレン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>要約</t>
+    <rPh sb="0" eb="2">
+      <t>ヨウヤク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>CSO分析</t>
+    <rPh sb="3" eb="5">
+      <t>ブンセキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>カリキュラム</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>学位取得</t>
+    <rPh sb="0" eb="2">
+      <t>ガクイ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>シュトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>決済ソース台帳</t>
+    <rPh sb="0" eb="2">
+      <t>ケッサイ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ダイチョウ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1599,7 +1698,7 @@
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.625" customWidth="1"/>
     <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
   </cols>
@@ -1645,10 +1744,13 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="2:8">
+    <row r="5" spans="2:8" ht="37.5">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>102</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -2296,44 +2398,45 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
-  <dimension ref="B2:H19"/>
+  <dimension ref="B2:I25"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8">
-      <c r="E2" t="s">
+    <row r="2" spans="2:9">
+      <c r="F2" t="s">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>2</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>45</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="2:8">
+    <row r="3" spans="2:9">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="3">
-        <v>46036</v>
-      </c>
       <c r="F3" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="4" spans="2:8">
+      <c r="G3" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
@@ -2341,14 +2444,14 @@
       <c r="C4" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="3">
-        <v>46036</v>
-      </c>
       <c r="F4" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="5" spans="2:8">
+      <c r="G4" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
@@ -2356,14 +2459,14 @@
       <c r="C5" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="3">
-        <v>46036</v>
-      </c>
       <c r="F5" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="6" spans="2:8">
+      <c r="G5" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9">
       <c r="B6">
         <f>B5+1</f>
         <v>4</v>
@@ -2371,14 +2474,14 @@
       <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="3">
-        <v>46036</v>
-      </c>
       <c r="F6" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="7" spans="2:8">
+      <c r="G6" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9">
       <c r="B7">
         <f>B6+1</f>
         <v>5</v>
@@ -2389,14 +2492,14 @@
       <c r="D7" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="3">
-        <v>46036</v>
-      </c>
       <c r="F7" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="8" spans="2:8">
+      <c r="G7" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9">
       <c r="B8">
         <f>B7+1</f>
         <v>6</v>
@@ -2404,11 +2507,14 @@
       <c r="D8" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" t="s">
+        <v>113</v>
+      </c>
+      <c r="F8" s="3">
         <v>46038</v>
       </c>
     </row>
-    <row r="9" spans="2:8">
+    <row r="9" spans="2:9">
       <c r="B9">
         <f>B8+1</f>
         <v>7</v>
@@ -2417,7 +2523,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="2:8">
+    <row r="10" spans="2:9">
       <c r="B10">
         <f>B9+1</f>
         <v>8</v>
@@ -2428,14 +2534,14 @@
       <c r="D10" t="s">
         <v>32</v>
       </c>
-      <c r="E10" s="3">
-        <v>46036</v>
-      </c>
       <c r="F10" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="11" spans="2:8">
+      <c r="G10" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9">
       <c r="B11">
         <f>B10+1</f>
         <v>9</v>
@@ -2444,7 +2550,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="2:8">
+    <row r="12" spans="2:9">
       <c r="B12">
         <f>B11+1</f>
         <v>10</v>
@@ -2453,7 +2559,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="2:8">
+    <row r="13" spans="2:9">
       <c r="B13">
         <f>B12+1</f>
         <v>11</v>
@@ -2464,14 +2570,14 @@
       <c r="D13" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="3">
-        <v>46036</v>
-      </c>
       <c r="F13" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="14" spans="2:8">
+      <c r="G13" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9">
       <c r="B14">
         <f>B13+1</f>
         <v>12</v>
@@ -2480,7 +2586,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="2:8">
+    <row r="15" spans="2:9">
       <c r="B15">
         <f>B14+1</f>
         <v>13</v>
@@ -2489,7 +2595,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="2:8">
+    <row r="16" spans="2:9">
       <c r="B16">
         <f>B15+1</f>
         <v>14</v>
@@ -2497,41 +2603,110 @@
       <c r="C16" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="17" spans="2:7">
+      <c r="D16" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9">
       <c r="B17">
         <f>B16+1</f>
         <v>15</v>
       </c>
-      <c r="C17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7">
+      <c r="D17" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9">
       <c r="B18">
         <f>B17+1</f>
         <v>16</v>
       </c>
-      <c r="C18" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7">
+      <c r="D18" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" spans="2:9">
       <c r="B19">
         <f>B18+1</f>
         <v>17</v>
       </c>
       <c r="C19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9">
+      <c r="B20">
+        <f>B19+1</f>
+        <v>18</v>
+      </c>
+      <c r="E20" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9">
+      <c r="B21">
+        <f>B20+1</f>
+        <v>19</v>
+      </c>
+      <c r="E21" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9">
+      <c r="B22">
+        <f>B21+1</f>
+        <v>20</v>
+      </c>
+      <c r="E22" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9">
+      <c r="B23">
+        <f>B22+1</f>
+        <v>21</v>
+      </c>
+      <c r="C23" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9">
+      <c r="B24">
+        <f>B23+1</f>
+        <v>22</v>
+      </c>
+      <c r="C24" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="3">
+      <c r="D24" t="s">
+        <v>111</v>
+      </c>
+      <c r="F24" s="3">
         <v>46037</v>
       </c>
-      <c r="F19" s="3">
+      <c r="G24" s="3">
         <v>46037</v>
       </c>
-      <c r="G19" s="3">
+      <c r="H24" s="3">
         <v>46037</v>
+      </c>
+      <c r="I24" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9">
+      <c r="B25">
+        <f>B24+1</f>
+        <v>23</v>
+      </c>
+      <c r="D25" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: remove unused import and fix formatting in payment channel ledger page
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98D072C9-7383-490F-9030-67EE7A2C24CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A177F151-9F6B-4381-9045-4B1291ABA21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="6" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
     <sheet name="追加したい機能" sheetId="11" r:id="rId11"/>
     <sheet name="Gemini API reference" sheetId="12" r:id="rId12"/>
     <sheet name="プロンプト集" sheetId="13" r:id="rId13"/>
-    <sheet name="Sheet13" sheetId="14" r:id="rId14"/>
+    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="126">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -823,6 +823,198 @@
     <rPh sb="5" eb="7">
       <t>ダイチョウ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Step4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（昼）</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>考え続ける（自動運転を止める）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>考え続ける（自動運転を止める）
+ここからが、この1日のいちばん重要なパート。
+多くの人は、朝に考えて「なるほど」と思っても、
+昼にはいつもの思考と行動に戻ってしまう。
+それは、人が無意識の自動運転で生きている時間の方が圧倒的に長いから。
+だから今日は、「正しい答えを出す日」ではなく、自動運転を止め続ける日にする。
+やり方はシンプル。スマホにリマインダーを入れて、
+1日の中で何度か強制的に立ち止まる。
+リマインダーに入れる質問の例：
+・今、何を避けている？
+・直近2時間の行動は、何を「避ける／守る」ための行動だった？
+・今日いちばん「生きていた」瞬間は？逆に「死んでいた」瞬間は？
+ここで大事なのは、答えを出そうとしないこと。
+・言葉にならなくてもいい
+・モヤっとしたままでいい
+立ち止まって「今、何が起きているか」を見るだけでOK。
+それだけで、無意識のパターンは少しずつ緩む。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Step5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>（夜）</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>全部を短い言葉にまとめる（15分）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>全部を短い言葉にまとめる（15分）
+夜は「整理の時間」。
+1日中考えてきたことを、短い言葉に圧縮する。
+まず、これを自分に問いかける。
+・これまで自分が詰まっていた一番の理由は何だった？
+・本当の敵は何だった？
+（環境や他人ではなく、自分の内側のパターン）
+そして、次の2つを書いたら今日は終わり。
+① 絶対に拒否する人生（1文）
+これは「もう戻りたくない状態」をはっきりさせるため。
+例：「我慢と先延ばしで時間を溶かす人生は、もうやらない」
+② 向かっていく方向（1文）
+完璧な理想じゃなくていい。
+今の自分が**進みたい“方向”**を示すだけでいい。
+例：「自分のエネルギーが上がる方向へ動く」
+この2文は、迷ったときに戻ってくるコンパスになる。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Step6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>｜明日の行動を決める</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最後に、現実へ戻す。
+ここで初めて「行動」を決める。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最後に、現実へ戻す。
+ここで初めて「行動」を決める。
+ただし、欲張らない。
+1年後：これが変わっていたらOK、というものを1つ
+1か月：そのために進めるプロジェクトを1つ
+明日：やることを2〜3個だけ決める。そして行動に移す時間も決める。
+完璧にやる必要はない。
+続ける必要もない。
+明日やる分だけで十分。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>まとめ（いちばん大事なこと）</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人生は気合や根性では変わらない。
+行動が変わるのは、見ている未来が変わったとき。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人生は気合や根性では変わらない。
+行動が変わるのは、見ている未来が変わったとき。
+今日は、人生を変える日じゃなくていい。
+「これからどっちに向かうか」をはっきりさせる日でいい。
+それだけで、次の1年は確実に違ってくる。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1858,10 +2050,10 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
-  <dimension ref="C3:E5"/>
+  <dimension ref="C3:E9"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="13.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="46.625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="94" bestFit="1" customWidth="1"/>
   </cols>
@@ -1897,6 +2089,50 @@
       </c>
       <c r="E5" s="1" t="s">
         <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" ht="409.5">
+      <c r="C6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" ht="409.5">
+      <c r="C7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" ht="262.5">
+      <c r="C8" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" ht="131.25">
+      <c r="C9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update content formatting and add Gemini Code Assist overview in Gemini University page
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A177F151-9F6B-4381-9045-4B1291ABA21D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473F6262-A20C-4BFC-A75D-C7C4F174F8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="6" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -25,8 +25,9 @@
     <sheet name="デイリータスク" sheetId="10" r:id="rId10"/>
     <sheet name="追加したい機能" sheetId="11" r:id="rId11"/>
     <sheet name="Gemini API reference" sheetId="12" r:id="rId12"/>
-    <sheet name="プロンプト集" sheetId="13" r:id="rId13"/>
-    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId14"/>
+    <sheet name="Gemini Code Assist" sheetId="15" r:id="rId13"/>
+    <sheet name="プロンプト集" sheetId="13" r:id="rId14"/>
+    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="133">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1015,6 +1016,31 @@
 今日は、人生を変える日じゃなくていい。
 「これからどっちに向かうか」をはっきりさせる日でいい。
 それだけで、次の1年は確実に違ってくる。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gen Media APIs: Endpoints for generating media with our specialized models such as Imagen for image generation, and Veo for video generation. Gemini also has these capabilities built in which you can access using the generateContent API.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gen Media API: 画像生成用のImagenや動画生成用のVeoなど、当社の専用モデルを用いたメディア生成のためのエンドポイントです。Geminiにも同様の機能が組み込まれており、generateContent APIを使用してアクセスできます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>Gemini Code Assist</t>
+  </si>
+  <si>
+    <t>Guides</t>
+  </si>
+  <si>
+    <t>Gemini Code Assist overview</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ジェミニ・コードアシストの概要</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1406,7 +1432,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46038</v>
+        <v>46039</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -1576,7 +1602,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46038</v>
+        <v>46039</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -1728,10 +1754,10 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E21"/>
+  <dimension ref="B1:E22"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="37.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.5" customWidth="1"/>
     <col min="3" max="3" width="43.5" customWidth="1"/>
     <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
@@ -1739,7 +1765,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46038</v>
+        <v>46039</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -1822,7 +1848,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="131.25">
+    <row r="17" spans="2:5" ht="93.75">
       <c r="B17" s="1" t="s">
         <v>72</v>
       </c>
@@ -1870,6 +1896,17 @@
         <v>92</v>
       </c>
       <c r="E21" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="93.75">
+      <c r="B22" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E22" s="3">
         <v>46038</v>
       </c>
     </row>
@@ -1885,6 +1922,65 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
+  <dimension ref="B1:E7"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5">
+      <c r="B2" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="B7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://developers.google.com/" xr:uid="{29CCC4AC-286B-4EC0-BB01-ECE2B318A3E0}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://developers.google.com/products" xr:uid="{CF0BCE14-7EC1-458F-B767-95D6891C081A}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{DAA66992-CDAB-4563-A108-1D3004893841}"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://developers.google.com/gemini-code-assist/docs/overview" xr:uid="{D4606693-ABC6-4C4C-8030-AFF9956F016B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{475FE61E-6EC0-4C61-9FD0-98172694F2E5}">
   <dimension ref="B1:H19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -1898,7 +1994,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46038</v>
+        <v>46039</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -2048,7 +2144,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
   <dimension ref="C3:E9"/>
   <sheetFormatPr defaultRowHeight="18.75"/>

</xml_diff>

<commit_message>
refactor: update content and structure for Gemini Code Assist overview in Gemini University page
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473F6262-A20C-4BFC-A75D-C7C4F174F8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2641E9-4F29-4C42-B7BE-723A840A20C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="8" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="144">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1041,6 +1041,52 @@
   </si>
   <si>
     <t>ジェミニ・コードアシストの概要</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://developers.google.com/gemini-code-assist/docs/overview</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Spark icon
+Page Summary</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>スパークアイコン
+ページ概要</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist provides AI-powered assistance for the software development lifecycle using the Gemini 2.5 model.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assistは、Gemini 2.5モデルを活用したソフトウェア開発ライフサイクル向けのAI支援を提供します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>It is available in free, Standard, and Enterprise editions, with varying features and target audiences.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>無料版、スタンダード版、エンタープライズ版の3種類が用意されており、それぞれ機能と対象ユーザー層が異なります。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist can be used in supported IDEs to generate code, provide conversational help, and offer features like source citations.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assistは、対応するIDEでコード生成、対話型ヘルプの提供、ソース引用などの機能を利用できます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Standard and Enterprise editions offer additional features outside the IDE, including integration with various Google Cloud services.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Standard版とEnterprise版では、IDE以外の追加機能を提供しており、各種Google Cloudサービスとの連携が含まれます。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1923,11 +1969,11 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E7"/>
+  <dimension ref="B1:E13"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="28" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="56.625" customWidth="1"/>
+    <col min="3" max="3" width="54.5" customWidth="1"/>
     <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1938,43 +1984,90 @@
       </c>
     </row>
     <row r="2" spans="2:5">
-      <c r="B2" s="6" t="s">
-        <v>53</v>
-      </c>
+      <c r="B2" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" s="6" t="s">
-        <v>128</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="6" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="7" spans="2:5">
-      <c r="B7" t="s">
+    <row r="8" spans="2:5">
+      <c r="B8" t="s">
         <v>131</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>132</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E8" s="3">
         <v>46039</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="37.5">
+      <c r="B9" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="37.5">
+      <c r="B10" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="37.5">
+      <c r="B11" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="56.25">
+      <c r="B12" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="37.5">
+      <c r="B13" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://developers.google.com/" xr:uid="{29CCC4AC-286B-4EC0-BB01-ECE2B318A3E0}"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://developers.google.com/products" xr:uid="{CF0BCE14-7EC1-458F-B767-95D6891C081A}"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{DAA66992-CDAB-4563-A108-1D3004893841}"/>
-    <hyperlink ref="B5" r:id="rId4" display="https://developers.google.com/gemini-code-assist/docs/overview" xr:uid="{D4606693-ABC6-4C4C-8030-AFF9956F016B}"/>
+    <hyperlink ref="B3" r:id="rId1" display="https://developers.google.com/" xr:uid="{29CCC4AC-286B-4EC0-BB01-ECE2B318A3E0}"/>
+    <hyperlink ref="B4" r:id="rId2" display="https://developers.google.com/products" xr:uid="{CF0BCE14-7EC1-458F-B767-95D6891C081A}"/>
+    <hyperlink ref="B5" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{DAA66992-CDAB-4563-A108-1D3004893841}"/>
+    <hyperlink ref="B6" r:id="rId4" display="https://developers.google.com/gemini-code-assist/docs/overview" xr:uid="{D4606693-ABC6-4C4C-8030-AFF9956F016B}"/>
+    <hyperlink ref="B2" r:id="rId5" xr:uid="{F2F2C855-BA2E-4DBF-BDB7-B571F8EBFB8B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: improve formatting and structure in various files for consistency
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2641E9-4F29-4C42-B7BE-723A840A20C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A0EA64-C9DE-4719-95D2-C824BF9905F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="8" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="183">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1089,12 +1089,227 @@
     <t>Standard版とEnterprise版では、IDE以外の追加機能を提供しており、各種Google Cloudサービスとの連携が含まれます。</t>
     <phoneticPr fontId="1"/>
   </si>
+  <si>
+    <t>Users should validate output from Gemini Code Assist as it is an early-stage technology and can sometimes generate incorrect information.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ユーザーは、Gemini Code Assistの出力を検証する必要があります。これは初期段階の技術であり、誤った情報を生成する場合があるためです。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>.NET Install Tool</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>結論から申し上げますと、現在「Gemini Code Assist」をメインで使おうとされているのであれば、「GitHub Copilot Chat」は不要（削除または無効化してOK） です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1. 機能が競合しています
+GitHub Copilot Chat: GitHub (Microsoft) 製のAIチャット
+Gemini Code Assist: Google 製のAIチャット
+これらは「ライバル関係」にあり、機能（コード生成、チャットでの質問、リファクタリング提案など）がほぼ完全に重複しています。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>理由1</t>
+    <rPh sb="0" eb="2">
+      <t>リユウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2. 同居させるデメリット
+両方入れていると、以下の問題が起きやすいです。
+UIが散らかる: サイドバーに似たようなAIアイコンが2つ並び、どちらに聞いているのか混乱する。
+ショートカットの競合: コード補完のショートカットキーなどが競合し、意図しない挙動になることがある。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>3. どちらを残すべきか？
+Gemini Code Assist を使う場合（推奨）:
+直近のご質問内容から、Gemini Code Assist の導入を進められているとお見受けします。その場合、GitHub Copilot Chat はアンインストール（または無効化） して、Gemini 一本に絞るのが最もスムーズです。
+GitHub Copilot を使う場合:
+もし「やっぱり GitHub Copilot の方が使い慣れている」という場合は、逆に Gemini Code Assist を無効化し、GitHub Copilot Chat を残します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Emoji"/>
+        <family val="2"/>
+      </rPr>
+      <t>⚠️</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 注意点：課金について
+拡張機能をアンインストールしても、GitHub Copilot の有料サブスクリプション（月額10ドルなど）は自動解約されません。 もし Gemini Code Assist（無料版やGoogle Cloudのプラン）に完全移行する場合は、GitHub側のサブスクリプション契約の解除も忘れずに行ってください。</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>注意点</t>
+    <rPh sb="0" eb="3">
+      <t>チュウイテン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>理由2</t>
+    <rPh sb="0" eb="2">
+      <t>リユウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>理由3</t>
+    <rPh sb="0" eb="2">
+      <t>リユウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AREPL for python</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>対応</t>
+    <rPh sb="0" eb="2">
+      <t>タイオウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>アンインストール</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>結論から申し上げますと、「.NET Install Tool」も不要（アンインストールしてOK） です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1. 開発言語が異なります
+あなたの現在のプロジェクト: Flutter (Dart) と Supabase (TypeScript) を使用した Webアプリケーション開発 です。
+.NET Install Tool: Microsoftの .NET (C# や F# など) の開発環境を整えるためのツールです。
+現在の my_web_app の開発において、.NET ランタイムが必要になる場面はありません。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2. 何のためにインストールされている？
+おそらく、過去に以下のような拡張機能をインストールした際に、依存関係として自動的にインストールされた可能性があります。
+C# (for VS Code)
+C# Dev Kit
+Unity 関連の拡張機能
+Azure Functions (C#版)
+もし現在、C# や Unity の開発を行っていないのであれば、このツールを残しておく必要はありません。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>3. アクション
+アンインストール（または無効化） してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>万が一、今後インストールする別の拡張機能がこれを必要とする場合は、VS Codeが「この拡張機能には .NET Install Tool が必要です」と通知を出して再インストールを促してくれますので、安心して削除して大丈夫です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Auto Rename Tag</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>結論から申し上げますと、「AREPL for python」も不要（アンインストールしてOK） です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1. 開発言語が異なります
+AREPL for python: Python のコードをリアルタイムで評価（実行結果を表示）するためのツールです。
+現在の開発: Flutter (Dart) と Supabase Functions (TypeScript) であり、Python は使用していません。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2. 用途が限定的です
+この拡張機能は、「Pythonのコードを書きながら、その場で変数の値などを確認する」ためのスクラッチパッド的なツールです。 もし、プロジェクトの裏側でデータ処理用のPythonスクリプトなどを書いていない限り、現在のWebアプリ開発プロジェクトでこれが必要になることはありません。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>これで、開発に関係のない「競合AI」「C#/.NET環境」「Python環境」の3つを整理できたことになります。VS Codeがかなり軽量化され、スッキリするはずです。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>auto-git</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>結論から申し上げますと、「Auto Rename Tag」も不要（アンインストールしてOK） です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1. Flutter (Dart) には「タグ」がありません
+Auto Rename Tag の機能: HTMLやXMLで &lt;div class="..."&gt; のように書き始め、閉じタグ &lt;/div&gt; を自動的にリネームするためのツールです。
+現在の開発 (Flutter): Flutter は Container( child: ... ) のような Dart のクラス（ウィジェット） を入れ子にして構築します。HTMLのような「対になるタグ」という概念がないため、この拡張機能は反応しません。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2. VS Code 標準機能で十分です
+もし仮に index.html などを編集する機会があったとしても、最近の VS Code は標準で Linked Editing（開始タグを変更すると終了タグも変わる機能）をサポートし始めています。あえて専用の拡張機能を入れておく必要性は低くなっています。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>整理の結果
+これで、以下の4つすべてが「不要」と判断できました。
+GitHub Copilot Chat → 削除OK（Geminiと競合）
+.NET Install Tool → 削除OK（言語違い）
+AREPL for python → 削除OK（言語違い）
+Auto Rename Tag → 削除OK（HTML用）
+これらを削除することで、VS Code の動作が軽量になり、メニューや右クリックメニューもスッキリして開発に集中しやすくなるはずです。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>VSCodeExtensions!A1</t>
+  </si>
+  <si>
+    <t>lib\models\attachment.dart</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>warning - The declaration '_playSoundNotification' isn't referenced - lib\services\timer_service.dart:210:8 - unused_element</t>
+  </si>
+  <si>
+    <t>warning - The declaration '_showBrowserNotification' isn't referenced - lib\services\timer_service.dart:218:16 - unused_element</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   info - Missing a required trailing comma - test\models\app_timer_test.dart:132:32 - require_trailing_commas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   info - Missing a required trailing comma - test\models\app_timer_test.dart:134:79 - require_trailing_commas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   info - Missing a required trailing comma - test\models\app_timer_test.dart:136:34 - require_trailing_commas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   info - Missing a required trailing comma - test\models\app_timer_test.dart:138:32 - require_trailing_commas</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1127,6 +1342,12 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI Emoji"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -1444,10 +1665,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3"/>
+  <dimension ref="C3:C4"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="16.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:3">
@@ -1455,10 +1676,16 @@
         <v>86</v>
       </c>
     </row>
+    <row r="4" spans="3:3">
+      <c r="C4" s="2" t="s">
+        <v>175</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
     <hyperlink ref="C3" location="コマンド一覧!A1" display="コマンド一覧!A1" xr:uid="{513A6E0C-B4B5-4FF3-8DC6-4373BA414EA5}"/>
+    <hyperlink ref="C4" location="VSCodeExtensions!A1" display="VSCodeExtensions!A1" xr:uid="{6FD37D3F-1015-4471-81AB-2D814C05317F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1969,10 +2196,10 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E13"/>
+  <dimension ref="B1:E14"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="56.625" customWidth="1"/>
+    <col min="2" max="2" width="60.625" customWidth="1"/>
     <col min="3" max="3" width="54.5" customWidth="1"/>
     <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
@@ -2044,7 +2271,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="56.25">
+    <row r="12" spans="2:5" ht="37.5">
       <c r="B12" s="1" t="s">
         <v>140</v>
       </c>
@@ -2058,6 +2285,14 @@
       </c>
       <c r="C13" s="1" t="s">
         <v>143</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="56.25">
+      <c r="B14" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2435,23 +2670,56 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{831F138C-7B13-4940-8512-4B95D1A24D44}">
-  <dimension ref="B2:F3"/>
+  <dimension ref="B1:L8"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.5" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="78" customWidth="1"/>
+    <col min="9" max="9" width="117.5" customWidth="1"/>
+    <col min="10" max="10" width="101.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="196.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="80.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6">
+    <row r="1" spans="2:12">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46039</v>
+      </c>
+      <c r="G1">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="2:12">
       <c r="E2" t="s">
         <v>1</v>
       </c>
       <c r="F2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="2:6">
+      <c r="G2" t="s">
+        <v>158</v>
+      </c>
+      <c r="H2" t="s">
+        <v>148</v>
+      </c>
+      <c r="I2" t="s">
+        <v>150</v>
+      </c>
+      <c r="J2" t="s">
+        <v>155</v>
+      </c>
+      <c r="K2" t="s">
+        <v>156</v>
+      </c>
+      <c r="L2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" ht="150">
       <c r="B3">
         <v>1</v>
       </c>
@@ -2461,7 +2729,138 @@
       <c r="E3" s="3">
         <v>46037</v>
       </c>
-      <c r="F3" s="3"/>
+      <c r="F3" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G3" t="s">
+        <v>159</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" ht="243.75">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46039</v>
+      </c>
+      <c r="F4" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G4" t="s">
+        <v>159</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" ht="75">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>157</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46039</v>
+      </c>
+      <c r="F5" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G5" t="s">
+        <v>159</v>
+      </c>
+      <c r="H5" t="s">
+        <v>166</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="243.75">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>165</v>
+      </c>
+      <c r="E6" s="3">
+        <v>46039</v>
+      </c>
+      <c r="H6" t="s">
+        <v>171</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>170</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -2533,7 +2932,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEF53A6-A89B-421F-A561-8936407ADCF5}">
-  <dimension ref="C2:E5"/>
+  <dimension ref="C2:E11"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="157.625" bestFit="1" customWidth="1"/>
@@ -2552,11 +2951,23 @@
       <c r="C3" t="s">
         <v>87</v>
       </c>
+      <c r="D3" s="3">
+        <v>46039</v>
+      </c>
+      <c r="E3" s="3">
+        <v>46039</v>
+      </c>
     </row>
     <row r="4" spans="3:5">
       <c r="C4" t="s">
         <v>88</v>
       </c>
+      <c r="D4" s="3">
+        <v>46039</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46039</v>
+      </c>
     </row>
     <row r="5" spans="3:5">
       <c r="C5" t="s">
@@ -2567,6 +2978,36 @@
       </c>
       <c r="E5" s="3">
         <v>46038</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5">
+      <c r="C6" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5">
+      <c r="C7" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5">
+      <c r="C8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5">
+      <c r="C9" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="10" spans="3:5">
+      <c r="C10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="3:5">
+      <c r="C11" t="s">
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -2577,7 +3018,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62C7C188-6DA4-4CDE-8831-D70FA561BA5F}">
-  <dimension ref="B3:H11"/>
+  <dimension ref="B3:H12"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -2639,16 +3080,10 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="3">
-        <v>46036</v>
-      </c>
-      <c r="F7" s="3">
-        <v>46036</v>
+        <v>176</v>
       </c>
       <c r="G7" s="5">
-        <v>0.95799999999999996</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="2:8">
@@ -2657,19 +3092,16 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E8" s="3">
-        <v>46031</v>
+        <v>46036</v>
       </c>
       <c r="F8" s="3">
-        <v>46031</v>
-      </c>
-      <c r="G8" s="4">
-        <v>1</v>
-      </c>
-      <c r="H8" t="s">
-        <v>80</v>
+        <v>46036</v>
+      </c>
+      <c r="G8" s="5">
+        <v>0.95799999999999996</v>
       </c>
     </row>
     <row r="9" spans="2:8">
@@ -2678,16 +3110,19 @@
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="E9" s="3">
         <v>46031</v>
       </c>
       <c r="F9" s="3">
-        <v>46036</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0.82599999999999996</v>
+        <v>46031</v>
+      </c>
+      <c r="G9" s="4">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="2:8">
@@ -2696,16 +3131,16 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E10" s="3">
-        <v>46036</v>
+        <v>46031</v>
       </c>
       <c r="F10" s="3">
         <v>46036</v>
       </c>
       <c r="G10" s="5">
-        <v>0.90500000000000003</v>
+        <v>0.82599999999999996</v>
       </c>
     </row>
     <row r="11" spans="2:8">
@@ -2714,12 +3149,30 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E11" s="3">
         <v>46036</v>
       </c>
+      <c r="F11" s="3">
+        <v>46036</v>
+      </c>
       <c r="G11" s="5">
+        <v>0.90500000000000003</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8">
+      <c r="B12">
+        <f>B11+1</f>
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="3">
+        <v>46036</v>
+      </c>
+      <c r="G12" s="5">
         <v>0.626</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: enhance type safety and improve error handling in AI Assistant function
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A0EA64-C9DE-4719-95D2-C824BF9905F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66DDC44E-6492-43BD-A561-E72EC6CE541E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
     <sheet name="コマンド一覧" sheetId="4" r:id="rId2"/>
-    <sheet name="VSCodeExtensions" sheetId="9" r:id="rId3"/>
-    <sheet name="ToDo" sheetId="2" r:id="rId4"/>
-    <sheet name="linter" sheetId="3" r:id="rId5"/>
-    <sheet name="テストカバレッジ" sheetId="5" r:id="rId6"/>
+    <sheet name="ToDo" sheetId="2" r:id="rId3"/>
+    <sheet name="linter" sheetId="3" r:id="rId4"/>
+    <sheet name="テストカバレッジ" sheetId="5" r:id="rId5"/>
+    <sheet name="VSCodeExtensions" sheetId="9" r:id="rId6"/>
     <sheet name="API呼び出し" sheetId="6" r:id="rId7"/>
     <sheet name="不具合修正" sheetId="7" r:id="rId8"/>
     <sheet name="機能一覧" sheetId="8" r:id="rId9"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="228">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -365,18 +365,6 @@
     <rPh sb="6" eb="8">
       <t>ダイガク</t>
     </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>flutter clean
-flutter pub get
-dart fix --apply
-dart format .
-flutter analyze
-dart run build_runner build --delete-conflicting-outputs
-flutter test --coverage
-supabase functions deploy ai-assistant
-flutter build web --release --no-tree-shake-icons</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -1303,6 +1291,287 @@
   </si>
   <si>
     <t xml:space="preserve">   info - Missing a required trailing comma - test\models\app_timer_test.dart:138:32 - require_trailing_commas</t>
+  </si>
+  <si>
+    <t>autoDocstring - Python Docstring Generator</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>VSCodeExtensionsを整理する</t>
+    <rPh sb="17" eb="19">
+      <t>セイリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>API呼び出し!A1</t>
+  </si>
+  <si>
+    <t>API一覧を作成する</t>
+    <rPh sb="3" eb="5">
+      <t>イチラン</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>サクセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Endpoint Path</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/ai-assistant</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Method</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>POST</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Authentication</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>必須 (Supabase Auth User Token)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Content-Type</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>application/json</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ヘッダー (Headers)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ヘッダー名	必須	値の例	説明
+Authorization	YES	Bearer &lt;USER_TOKEN&gt;	ログインユーザーのアクセストークン
+Content-Type	YES	application/json</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>共通リクエストボディ (Request Body)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{
+  "action": "実行したいアクション名 (必須)",
+  "model": "指定したいAIモデル名 (任意)",
+  "content": "テキスト入力 (アクションによる)",
+  "imageBase64": "Base64エンコードされた画像データ (画像分析時)",
+  "mimeType": "画像のMIMEタイプ (例: image/jpeg)"
+}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>model (任意): 指定しない場合、コード内で定義されたフォールバックリスト（Gemini Flash -&gt; GPT-4o-mini -&gt; Claude Haiku）順に試行されます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>機能 (Actions) 一覧</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1. 利用可能モデルの取得
+システムで利用可能なAIモデルの一覧を取得します。
+Action: get_models
+必要なパラメータ: なし</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "models": [
+    { "name": "gemini-2.0-flash", "provider": "Google", "description": "Fast &amp; Versatile" },
+    ...
+  ]
+}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>モデル一覧取得</t>
+    <rPh sb="3" eb="5">
+      <t>イチラン</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>シュトク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>2. リアル断捨離クエスト (画像分析)
+アップロードされた画像を「自分株式会社」のCSO（最高戦略責任者）の視点で分析し、断捨離すべきか判定します。
+Action: analyze_danshari_item
+必要なパラメータ:
+imageBase64 (必須): 画像のBase64文字列
+mimeType (推奨): 画像形式 (デフォルトは image/jpeg)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "result": {
+    "item_name": "アイテム名",
+    "spark_joy_score": 0-100,
+    "decision": "KEEP" | "DISCARD",
+    "reason": "判定理由",
+    "witty_comment": "皮肉やユーモアのあるコメント"
+  }
+}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>緊急役員会議 (Board Meeting)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>入力された議題について、CEO (Steve), CTO (Linus), CMO (Gary), CFO (Warren) の4名が議論するシミュレーションを行います。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>緊急役員会議</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リアル断捨離クエスト (画像分析)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>アップロードされた画像を「自分株式会社」のCSO（最高戦略責任者）の視点で分析し、断捨離すべきか判定します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>システムで利用可能なAIモデルの一覧を取得します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>3. 緊急役員会議 (Board Meeting)
+入力された議題について、CEO (Steve), CTO (Linus), CMO (Gary), CFO (Warren) の4名が議論するシミュレーションを行います。
+Action: hold_board_meeting
+必要なパラメータ:
+content (必須): 会議の議題 (Topic)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>レスポンス (構造化JSON):</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "result": {
+    "meeting_minutes": [
+      { "role": "CEO", "name": "Steve", "text": "発言内容..." },
+      ...
+    ],
+    "conclusion": "最終的な結論"
+  }
+}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>エラーレスポンス</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>処理に失敗した場合、以下の形式で返却されます。
+Status Code: 400 (Bad Request) または 404 (Not Found), 500 (Internal Server Error)
+Body:
+{
+  "success": false,
+  "error": "エラーメッセージの詳細"
+}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ノート機能</t>
+    <rPh sb="3" eb="5">
+      <t>キノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>汎用テキスト処理</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>一般的なテキスト生成・加工タスクを実行します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>4. 汎用テキスト処理
+一般的なテキスト生成・加工タスクを実行します。
+Actions: 以下のいずれか
+improve (文章の改善)
+summarize (要約)
+expand (話を広げる)
+translate (翻訳)
+suggest_title (タイトル提案)
+必要なパラメータ:
+content (必須): 対象となるテキスト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{
+  "success": true,
+  "result": "AIによって生成されたテキスト結果"
+}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>呼び出し結果</t>
+    <rPh sb="0" eb="1">
+      <t>ヨ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ダ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ケッカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>deno cache supabase/functions/ai-assistant/index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>irm https://deno.land/install.ps1 | iex</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>deno check supabase/functions/ai-assistant/index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>deno lint supabase/functions/ai-assistant/index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>deno lint supabase</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>flutter clean
+flutter pub get
+dart fix --apply
+dart format .
+flutter analyze
+deno lint supabase
+dart run build_runner build --delete-conflicting-outputs
+flutter test --coverage
+supabase functions deploy ai-assistant
+flutter build web --release --no-tree-shake-icons</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -1673,12 +1942,12 @@
   <sheetData>
     <row r="3" spans="3:3">
       <c r="C3" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="3:3">
       <c r="C4" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -1716,10 +1985,10 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" t="s">
         <v>45</v>
-      </c>
-      <c r="H2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="2:8">
@@ -1727,7 +1996,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E3" s="3">
         <v>46037</v>
@@ -1742,7 +2011,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -1753,7 +2022,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -1764,7 +2033,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -1886,10 +2155,10 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" t="s">
         <v>45</v>
-      </c>
-      <c r="H2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="2:8">
@@ -1897,7 +2166,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -1908,7 +2177,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -1919,7 +2188,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -2043,108 +2312,108 @@
     </row>
     <row r="2" spans="2:5">
       <c r="B2" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C6" t="s">
         <v>56</v>
-      </c>
-      <c r="C6" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" t="s">
         <v>58</v>
-      </c>
-      <c r="C7" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="56.25">
       <c r="B8" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="37.5">
       <c r="B9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="75">
       <c r="B11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="E11" s="3"/>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="37.5">
       <c r="B15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="93.75">
       <c r="B17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="2:5" ht="112.5">
       <c r="B18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="E18" s="3"/>
     </row>
     <row r="19" spans="2:5" ht="75">
       <c r="B19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="E19" s="3">
         <v>46037</v>
@@ -2152,10 +2421,10 @@
     </row>
     <row r="20" spans="2:5" ht="56.25">
       <c r="B20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>84</v>
       </c>
       <c r="E20" s="3">
         <v>46038</v>
@@ -2163,10 +2432,10 @@
     </row>
     <row r="21" spans="2:5" ht="56.25">
       <c r="B21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="E21" s="3">
         <v>46038</v>
@@ -2174,10 +2443,10 @@
     </row>
     <row r="22" spans="2:5" ht="93.75">
       <c r="B22" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="E22" s="3">
         <v>46038</v>
@@ -2212,36 +2481,36 @@
     </row>
     <row r="2" spans="2:5">
       <c r="B2" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C8" t="s">
         <v>131</v>
-      </c>
-      <c r="C8" t="s">
-        <v>132</v>
       </c>
       <c r="E8" s="3">
         <v>46039</v>
@@ -2249,50 +2518,50 @@
     </row>
     <row r="9" spans="2:5" ht="37.5">
       <c r="B9" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>136</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="37.5">
       <c r="B11" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="37.5">
       <c r="B12" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>140</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="37.5">
       <c r="B13" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="56.25">
       <c r="B14" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>144</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2333,10 +2602,10 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H2" t="s">
         <v>45</v>
-      </c>
-      <c r="H2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="2:8">
@@ -2344,7 +2613,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -2355,7 +2624,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -2366,7 +2635,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -2484,79 +2753,79 @@
   <sheetData>
     <row r="3" spans="3:5" ht="206.25">
       <c r="C3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" t="s">
         <v>93</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="4" spans="3:5" ht="150">
       <c r="C4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="D4" t="s">
-        <v>98</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="300">
       <c r="C5" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="6" spans="3:5" ht="409.5">
       <c r="C6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D6" t="s">
         <v>114</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="7" spans="3:5" ht="409.5">
       <c r="C7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" t="s">
         <v>117</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="8" spans="3:5" ht="262.5">
       <c r="C8" t="s">
+        <v>119</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="9" spans="3:5" ht="131.25">
       <c r="C9" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2570,10 +2839,10 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="B3:D12"/>
+  <dimension ref="B3:D17"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="60" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2635,13 +2904,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="168.75">
+    <row r="10" spans="2:4" ht="187.5">
       <c r="B10">
         <f>B9+1</f>
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>43</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="37.5">
@@ -2660,6 +2929,51 @@
       </c>
       <c r="C12" s="1" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4">
+      <c r="B13">
+        <f>B12+1</f>
+        <v>10</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4">
+      <c r="B14">
+        <f>B13+1</f>
+        <v>11</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4">
+      <c r="B15">
+        <f>B14+1</f>
+        <v>12</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4">
+      <c r="B16">
+        <f>B15+1</f>
+        <v>13</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17">
+        <f>B16+1</f>
+        <v>14</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>
@@ -2669,214 +2983,14 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{831F138C-7B13-4940-8512-4B95D1A24D44}">
-  <dimension ref="B1:L8"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
-  <cols>
-    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="78" customWidth="1"/>
-    <col min="9" max="9" width="117.5" customWidth="1"/>
-    <col min="10" max="10" width="101.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="196.625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="80.25" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:12">
-      <c r="E1" s="3">
-        <f ca="1">TODAY()</f>
-        <v>46039</v>
-      </c>
-      <c r="G1">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="2" spans="2:12">
-      <c r="E2" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>2</v>
-      </c>
-      <c r="G2" t="s">
-        <v>158</v>
-      </c>
-      <c r="H2" t="s">
-        <v>148</v>
-      </c>
-      <c r="I2" t="s">
-        <v>150</v>
-      </c>
-      <c r="J2" t="s">
-        <v>155</v>
-      </c>
-      <c r="K2" t="s">
-        <v>156</v>
-      </c>
-      <c r="L2" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="3" spans="2:12" ht="150">
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E3" s="3">
-        <v>46037</v>
-      </c>
-      <c r="F3" s="3">
-        <v>46039</v>
-      </c>
-      <c r="G3" t="s">
-        <v>159</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="4" spans="2:12" ht="243.75">
-      <c r="B4">
-        <f>B3+1</f>
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>146</v>
-      </c>
-      <c r="E4" s="3">
-        <v>46039</v>
-      </c>
-      <c r="F4" s="3">
-        <v>46039</v>
-      </c>
-      <c r="G4" t="s">
-        <v>159</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="5" spans="2:12" ht="75">
-      <c r="B5">
-        <f>B4+1</f>
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>157</v>
-      </c>
-      <c r="E5" s="3">
-        <v>46039</v>
-      </c>
-      <c r="F5" s="3">
-        <v>46039</v>
-      </c>
-      <c r="G5" t="s">
-        <v>159</v>
-      </c>
-      <c r="H5" t="s">
-        <v>166</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" ht="243.75">
-      <c r="B6">
-        <f>B5+1</f>
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E6" s="3">
-        <v>46039</v>
-      </c>
-      <c r="H6" t="s">
-        <v>171</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12">
-      <c r="B7">
-        <f>B6+1</f>
-        <v>5</v>
-      </c>
-      <c r="C7" t="s">
-        <v>170</v>
-      </c>
-      <c r="E7" s="3">
-        <v>46039</v>
-      </c>
-    </row>
-    <row r="8" spans="2:12">
-      <c r="B8">
-        <f>B7+1</f>
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB9A9986-272E-4F2B-8815-9B72212F3499}">
-  <dimension ref="B3:F6"/>
+  <dimension ref="B3:F7"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2896,7 +3010,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="2:6">
@@ -2918,6 +3032,27 @@
       <c r="B6">
         <f>B5+1</f>
         <v>3</v>
+      </c>
+      <c r="C6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>185</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46039</v>
       </c>
     </row>
   </sheetData>
@@ -2925,12 +3060,14 @@
   <hyperlinks>
     <hyperlink ref="D5" location="テストカバレッジ!A1" display="テストカバレッジ!A1" xr:uid="{D25F68D0-C78F-4FF1-ABD2-D974080835FC}"/>
     <hyperlink ref="D4" location="linter!A1" display="linter!A1" xr:uid="{2F08201A-392B-43E2-8926-23FB861EC50A}"/>
+    <hyperlink ref="D6" location="VSCodeExtensions!A1" display="VSCodeExtensions!A1" xr:uid="{8DEA63B7-005F-48BD-BB37-28E553CC1988}"/>
+    <hyperlink ref="D7" location="API呼び出し!A1" display="API呼び出し!A1" xr:uid="{03F8098F-7CB3-480C-BBDF-9E03B8A5E4A0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEF53A6-A89B-421F-A561-8936407ADCF5}">
   <dimension ref="C2:E11"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -2949,7 +3086,7 @@
     </row>
     <row r="3" spans="3:5">
       <c r="C3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D3" s="3">
         <v>46039</v>
@@ -2960,7 +3097,7 @@
     </row>
     <row r="4" spans="3:5">
       <c r="C4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D4" s="3">
         <v>46039</v>
@@ -2971,7 +3108,7 @@
     </row>
     <row r="5" spans="3:5">
       <c r="C5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D5" s="3">
         <v>46038</v>
@@ -2982,32 +3119,32 @@
     </row>
     <row r="6" spans="3:5">
       <c r="C6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="3:5">
       <c r="C7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="8" spans="3:5">
       <c r="C8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" spans="3:5">
       <c r="C9" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="10" spans="3:5">
       <c r="C10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" spans="3:5">
       <c r="C11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3016,7 +3153,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62C7C188-6DA4-4CDE-8831-D70FA561BA5F}">
   <dimension ref="B3:H12"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -3056,7 +3193,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G5" s="5">
         <v>0.33300000000000002</v>
@@ -3068,7 +3205,7 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G6" s="5">
         <v>0</v>
@@ -3080,7 +3217,7 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G7" s="5">
         <v>0</v>
@@ -3122,7 +3259,7 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="2:8">
@@ -3174,6 +3311,218 @@
       </c>
       <c r="G12" s="5">
         <v>0.626</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{831F138C-7B13-4940-8512-4B95D1A24D44}">
+  <dimension ref="B1:L8"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="78" customWidth="1"/>
+    <col min="9" max="9" width="117.5" customWidth="1"/>
+    <col min="10" max="10" width="101.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="196.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="80.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:12">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46039</v>
+      </c>
+      <c r="G1">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="2:12">
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
+        <v>157</v>
+      </c>
+      <c r="H2" t="s">
+        <v>147</v>
+      </c>
+      <c r="I2" t="s">
+        <v>149</v>
+      </c>
+      <c r="J2" t="s">
+        <v>154</v>
+      </c>
+      <c r="K2" t="s">
+        <v>155</v>
+      </c>
+      <c r="L2" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" ht="150">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="3">
+        <v>46037</v>
+      </c>
+      <c r="F3" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" ht="243.75">
+      <c r="B4">
+        <f>B3+1</f>
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46039</v>
+      </c>
+      <c r="F4" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G4" t="s">
+        <v>158</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" ht="75">
+      <c r="B5">
+        <f>B4+1</f>
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46039</v>
+      </c>
+      <c r="F5" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G5" t="s">
+        <v>158</v>
+      </c>
+      <c r="H5" t="s">
+        <v>165</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="243.75">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E6" s="3">
+        <v>46039</v>
+      </c>
+      <c r="F6" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G6" t="s">
+        <v>158</v>
+      </c>
+      <c r="H6" t="s">
+        <v>170</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>182</v>
+      </c>
+      <c r="E8" s="3">
+        <v>46039</v>
       </c>
     </row>
   </sheetData>
@@ -3184,40 +3533,117 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
-  <dimension ref="B2:F5"/>
+  <dimension ref="B2:R6"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.25" customWidth="1"/>
+    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="32.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="75.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="65.75" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="65.75" customWidth="1"/>
+    <col min="13" max="13" width="50.125" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="50.125" customWidth="1"/>
+    <col min="16" max="16" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6">
-      <c r="D2" t="s">
+    <row r="2" spans="2:18">
+      <c r="F2" t="s">
+        <v>186</v>
+      </c>
+      <c r="G2" t="s">
+        <v>188</v>
+      </c>
+      <c r="H2" t="s">
+        <v>190</v>
+      </c>
+      <c r="I2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K2" t="s">
+        <v>196</v>
+      </c>
+      <c r="M2" t="s">
+        <v>199</v>
+      </c>
+      <c r="N2" t="s">
+        <v>212</v>
+      </c>
+      <c r="O2" t="s">
+        <v>214</v>
+      </c>
+      <c r="P2" t="s">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="Q2" t="s">
+        <v>221</v>
+      </c>
+      <c r="R2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:6">
+    <row r="3" spans="2:18" ht="225">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" t="s">
+        <v>208</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F3" t="s">
+        <v>187</v>
+      </c>
+      <c r="G3" t="s">
+        <v>189</v>
+      </c>
+      <c r="H3" t="s">
+        <v>191</v>
+      </c>
+      <c r="I3" t="s">
+        <v>193</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="P3" s="3">
         <v>46036</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3">
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3">
         <v>46036</v>
       </c>
     </row>
-    <row r="4" spans="2:6">
+    <row r="4" spans="2:18" ht="206.25">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
@@ -3225,20 +3651,146 @@
       <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" t="s">
+        <v>202</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F4" t="s">
+        <v>187</v>
+      </c>
+      <c r="G4" t="s">
+        <v>189</v>
+      </c>
+      <c r="H4" t="s">
+        <v>191</v>
+      </c>
+      <c r="I4" t="s">
+        <v>193</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="P4" s="3">
         <v>46036</v>
       </c>
-      <c r="E4" t="s">
+      <c r="Q4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="3">
+      <c r="R4" s="3">
         <v>46036</v>
       </c>
     </row>
-    <row r="5" spans="2:6">
+    <row r="5" spans="2:18" ht="206.25">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>205</v>
+      </c>
+      <c r="D5" t="s">
+        <v>207</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F5" t="s">
+        <v>187</v>
+      </c>
+      <c r="G5" t="s">
+        <v>189</v>
+      </c>
+      <c r="H5" t="s">
+        <v>191</v>
+      </c>
+      <c r="I5" t="s">
+        <v>193</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="P5" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="6" spans="2:18" ht="337.5">
+      <c r="B6">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>216</v>
+      </c>
+      <c r="D6" t="s">
+        <v>217</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F6" t="s">
+        <v>187</v>
+      </c>
+      <c r="G6" t="s">
+        <v>189</v>
+      </c>
+      <c r="H6" t="s">
+        <v>191</v>
+      </c>
+      <c r="I6" t="s">
+        <v>193</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="P6" s="3">
+        <v>46039</v>
       </c>
     </row>
   </sheetData>
@@ -3294,10 +3846,10 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" t="s">
         <v>45</v>
-      </c>
-      <c r="I2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="3" spans="2:9">
@@ -3386,7 +3938,7 @@
         <v>29</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F8" s="3">
         <v>46038</v>
@@ -3482,7 +4034,7 @@
         <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="2:9">
@@ -3491,7 +4043,7 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="2:9">
@@ -3500,7 +4052,7 @@
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="19" spans="2:9">
@@ -3512,10 +4064,10 @@
         <v>40</v>
       </c>
       <c r="D19" t="s">
+        <v>105</v>
+      </c>
+      <c r="E19" t="s">
         <v>106</v>
-      </c>
-      <c r="E19" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="20" spans="2:9">
@@ -3524,7 +4076,7 @@
         <v>18</v>
       </c>
       <c r="E20" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="2:9">
@@ -3533,7 +4085,7 @@
         <v>19</v>
       </c>
       <c r="E21" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" spans="2:9">
@@ -3542,7 +4094,7 @@
         <v>20</v>
       </c>
       <c r="E22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="2:9">
@@ -3563,7 +4115,7 @@
         <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F24" s="3">
         <v>46037</v>
@@ -3584,7 +4136,7 @@
         <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: enhance type safety by replacing 'any' with specific types and adding type definitions in AI functions
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66DDC44E-6492-43BD-A561-E72EC6CE541E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F7F5AA1-A687-43F5-9DDB-67FD56DF6064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="248">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -145,10 +145,6 @@
     <rPh sb="10" eb="12">
       <t>ツウチ</t>
     </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>404 not found</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -1571,6 +1567,115 @@
 flutter test --coverage
 supabase functions deploy ai-assistant
 flutter build web --release --no-tree-shake-icons</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Note: If you're at a business or would like more team-level benefits, consider Gemini Code Assist Standard or Enterprise.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>注：ビジネス利用の場合、またはチームレベルの特典をさらにご利用になりたい場合は、Gemini Code Assist Standard または Enterprise のご利用をご検討ください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist offers AI-powered assistance to help your development team build, deploy, and operate applications throughout the software development lifecycle. Gemini Code Assist is available in the following editions:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assistは、ソフトウェア開発ライフサイクル全体を通じて、開発チームがアプリケーションを構築、デプロイ、運用するためのAIを活用した支援を提供します。Gemini Code Assistは以下のエディションで利用可能です：</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist for individuals, available at no cost.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>個人向けジェミニ・コードアシスト、無料でご利用いただけます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist Standard, a product in the Gemini for Google Cloud portfolio.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist Standard（Gemini for Google Cloud ポートフォリオの製品）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist Enterprise, a product in the Gemini for Google Cloud portfolio.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist Enterprise（Gemini for Google Cloud ポートフォリオの製品）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>{
+    "success": true,
+    "models": [
+        {
+            "name": "gemini-2.0-flash",
+            "provider": "Google",
+            "description": "Fast &amp; Versatile"
+        },
+        {
+            "name": "gpt-4o",
+            "provider": "OpenAI",
+            "description": "High Intelligence"
+        },
+        {
+            "name": "claude-3-opus",
+            "provider": "Anthropic",
+            "description": "Complex Tasks"
+        }
+    ]
+}</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>UIからの操作手順</t>
+    <rPh sb="5" eb="7">
+      <t>ソウサ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>テジュン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ソースコード</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\ai-assistant\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\ai-search\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\ai-suggest-tags\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\daily-judgment\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\generate-daily-challenges\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\generate-quote-image\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\get-ogp\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase\functions\share-quote\index.ts</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1641,14 +1746,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
@@ -1942,12 +2046,12 @@
   <sheetData>
     <row r="3" spans="3:3">
       <c r="C3" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="3:3">
       <c r="C4" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -1985,10 +2089,10 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
         <v>44</v>
-      </c>
-      <c r="H2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="2:8">
@@ -1996,7 +2100,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E3" s="3">
         <v>46037</v>
@@ -2011,7 +2115,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -2022,7 +2126,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -2033,7 +2137,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -2155,10 +2259,10 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
         <v>44</v>
-      </c>
-      <c r="H2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="2:8">
@@ -2166,7 +2270,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -2177,7 +2281,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -2188,7 +2292,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -2311,109 +2415,109 @@
       </c>
     </row>
     <row r="2" spans="2:5">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="5" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="2:5">
-      <c r="B3" s="6" t="s">
+    <row r="4" spans="2:5">
+      <c r="B4" s="5" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5">
-      <c r="B4" s="6" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s">
         <v>55</v>
-      </c>
-      <c r="C6" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" t="s">
         <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="56.25">
       <c r="B8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="37.5">
       <c r="B9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="75">
       <c r="B11" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>66</v>
       </c>
       <c r="E11" s="3"/>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>67</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="37.5">
       <c r="B15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="93.75">
       <c r="B17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>72</v>
       </c>
       <c r="E17" s="3"/>
     </row>
     <row r="18" spans="2:5" ht="112.5">
       <c r="B18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>74</v>
       </c>
       <c r="E18" s="3"/>
     </row>
     <row r="19" spans="2:5" ht="75">
       <c r="B19" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="E19" s="3">
         <v>46037</v>
@@ -2421,10 +2525,10 @@
     </row>
     <row r="20" spans="2:5" ht="56.25">
       <c r="B20" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="E20" s="3">
         <v>46038</v>
@@ -2432,10 +2536,10 @@
     </row>
     <row r="21" spans="2:5" ht="56.25">
       <c r="B21" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="E21" s="3">
         <v>46038</v>
@@ -2443,10 +2547,10 @@
     </row>
     <row r="22" spans="2:5" ht="93.75">
       <c r="B22" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>125</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>126</v>
       </c>
       <c r="E22" s="3">
         <v>46038</v>
@@ -2465,11 +2569,11 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E14"/>
+  <dimension ref="B1:E19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="60.625" customWidth="1"/>
-    <col min="3" max="3" width="54.5" customWidth="1"/>
+    <col min="2" max="2" width="73.125" customWidth="1"/>
+    <col min="3" max="3" width="72.5" customWidth="1"/>
     <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2481,36 +2585,36 @@
     </row>
     <row r="2" spans="2:5">
       <c r="B2" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E2" s="3"/>
     </row>
     <row r="3" spans="2:5">
-      <c r="B3" s="6" t="s">
-        <v>52</v>
+      <c r="B3" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="2:5">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="5" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="2:5">
-      <c r="B5" s="6" t="s">
+    <row r="6" spans="2:5">
+      <c r="B6" s="5" t="s">
         <v>128</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5">
-      <c r="B6" s="6" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" t="s">
         <v>130</v>
-      </c>
-      <c r="C8" t="s">
-        <v>131</v>
       </c>
       <c r="E8" s="3">
         <v>46039</v>
@@ -2518,50 +2622,90 @@
     </row>
     <row r="9" spans="2:5" ht="37.5">
       <c r="B9" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="37.5">
       <c r="B11" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="37.5">
       <c r="B12" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="37.5">
       <c r="B13" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="C13" s="1" t="s">
+    </row>
+    <row r="14" spans="2:5" ht="37.5">
+      <c r="B14" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="14" spans="2:5" ht="56.25">
-      <c r="B14" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>144</v>
+    </row>
+    <row r="15" spans="2:5" ht="37.5">
+      <c r="B15" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="56.25">
+      <c r="B16" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -2602,10 +2746,10 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
+        <v>43</v>
+      </c>
+      <c r="H2" t="s">
         <v>44</v>
-      </c>
-      <c r="H2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="2:8">
@@ -2613,7 +2757,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -2624,7 +2768,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -2635,7 +2779,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -2753,79 +2897,79 @@
   <sheetData>
     <row r="3" spans="3:5" ht="206.25">
       <c r="C3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" t="s">
         <v>92</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="4" spans="3:5" ht="150">
       <c r="C4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="D4" t="s">
-        <v>97</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="5" spans="3:5" ht="300">
       <c r="C5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="6" spans="3:5" ht="409.5">
       <c r="C6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6" t="s">
         <v>113</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="7" spans="3:5" ht="409.5">
       <c r="C7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" t="s">
         <v>116</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="8" spans="3:5" ht="262.5">
       <c r="C8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="9" spans="3:5" ht="131.25">
       <c r="C9" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2910,7 +3054,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="37.5">
@@ -2928,7 +3072,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="2:4">
@@ -2937,7 +3081,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14" spans="2:4">
@@ -2946,7 +3090,7 @@
         <v>11</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="15" spans="2:4">
@@ -2955,7 +3099,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="16" spans="2:4">
@@ -2964,7 +3108,7 @@
         <v>13</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="17" spans="2:3">
@@ -2973,7 +3117,7 @@
         <v>14</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -3010,7 +3154,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="2:6">
@@ -3034,10 +3178,10 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="2:6">
@@ -3046,10 +3190,10 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E7" s="3">
         <v>46039</v>
@@ -3086,7 +3230,7 @@
     </row>
     <row r="3" spans="3:5">
       <c r="C3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D3" s="3">
         <v>46039</v>
@@ -3097,7 +3241,7 @@
     </row>
     <row r="4" spans="3:5">
       <c r="C4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D4" s="3">
         <v>46039</v>
@@ -3108,7 +3252,7 @@
     </row>
     <row r="5" spans="3:5">
       <c r="C5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D5" s="3">
         <v>46038</v>
@@ -3119,32 +3263,32 @@
     </row>
     <row r="6" spans="3:5">
       <c r="C6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="3:5">
       <c r="C7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="8" spans="3:5">
       <c r="C8" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" spans="3:5">
       <c r="C9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="3:5">
       <c r="C10" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="11" spans="3:5">
       <c r="C11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -3162,7 +3306,7 @@
     <col min="3" max="3" width="36.875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.375" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:8">
@@ -3181,9 +3325,9 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="5">
+        <v>20</v>
+      </c>
+      <c r="G4" s="4">
         <v>0.80900000000000005</v>
       </c>
     </row>
@@ -3193,9 +3337,9 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G5" s="5">
+        <v>79</v>
+      </c>
+      <c r="G5" s="4">
         <v>0.33300000000000002</v>
       </c>
     </row>
@@ -3205,10 +3349,16 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
-      </c>
-      <c r="G6" s="5">
-        <v>0</v>
+        <v>80</v>
+      </c>
+      <c r="E6" s="3">
+        <v>46039</v>
+      </c>
+      <c r="F6" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G6" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="2:8">
@@ -3217,9 +3367,9 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>175</v>
-      </c>
-      <c r="G7" s="5">
+        <v>174</v>
+      </c>
+      <c r="G7" s="4">
         <v>0</v>
       </c>
     </row>
@@ -3229,7 +3379,7 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E8" s="3">
         <v>46036</v>
@@ -3237,7 +3387,7 @@
       <c r="F8" s="3">
         <v>46036</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="4">
         <v>0.95799999999999996</v>
       </c>
     </row>
@@ -3259,7 +3409,7 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="2:8">
@@ -3268,7 +3418,7 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E10" s="3">
         <v>46031</v>
@@ -3276,7 +3426,7 @@
       <c r="F10" s="3">
         <v>46036</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="4">
         <v>0.82599999999999996</v>
       </c>
     </row>
@@ -3286,7 +3436,7 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E11" s="3">
         <v>46036</v>
@@ -3294,7 +3444,7 @@
       <c r="F11" s="3">
         <v>46036</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <v>0.90500000000000003</v>
       </c>
     </row>
@@ -3304,12 +3454,12 @@
         <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E12" s="3">
         <v>46036</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <v>0.626</v>
       </c>
     </row>
@@ -3352,22 +3502,22 @@
         <v>2</v>
       </c>
       <c r="G2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J2" t="s">
+        <v>153</v>
+      </c>
+      <c r="K2" t="s">
         <v>154</v>
       </c>
-      <c r="K2" t="s">
-        <v>155</v>
-      </c>
       <c r="L2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="150">
@@ -3375,7 +3525,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E3" s="3">
         <v>46037</v>
@@ -3384,22 +3534,22 @@
         <v>46039</v>
       </c>
       <c r="G3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J3" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K3" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="4" spans="2:12" ht="243.75">
@@ -3408,7 +3558,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E4" s="3">
         <v>46039</v>
@@ -3417,22 +3567,22 @@
         <v>46039</v>
       </c>
       <c r="G4" t="s">
+        <v>157</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="5" spans="2:12" ht="75">
@@ -3441,7 +3591,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E5" s="3">
         <v>46039</v>
@@ -3450,22 +3600,22 @@
         <v>46039</v>
       </c>
       <c r="G5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H5" t="s">
+        <v>164</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="J5" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="K5" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="6" spans="2:12" ht="243.75">
@@ -3474,7 +3624,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E6" s="3">
         <v>46039</v>
@@ -3483,22 +3633,22 @@
         <v>46039</v>
       </c>
       <c r="G6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I6" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="L6" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="7" spans="2:12">
@@ -3507,7 +3657,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E7" s="3">
         <v>46039</v>
@@ -3519,7 +3669,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E8" s="3">
         <v>46039</v>
@@ -3533,66 +3683,74 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
-  <dimension ref="B2:R6"/>
+  <dimension ref="B2:T13"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.75" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34.25" customWidth="1"/>
-    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="32.625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="75.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="65.75" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="65.75" customWidth="1"/>
-    <col min="13" max="13" width="50.125" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="50.125" customWidth="1"/>
-    <col min="16" max="16" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="54.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.25" customWidth="1"/>
+    <col min="8" max="8" width="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="32.625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="75.5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="65.75" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="65.75" customWidth="1"/>
+    <col min="15" max="15" width="50.125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="50.125" customWidth="1"/>
     <col min="18" max="18" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="47" customWidth="1"/>
+    <col min="20" max="20" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18">
+    <row r="2" spans="2:20">
       <c r="F2" t="s">
-        <v>186</v>
+        <v>239</v>
       </c>
       <c r="G2" t="s">
-        <v>188</v>
+        <v>238</v>
       </c>
       <c r="H2" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="I2" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="J2" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K2" t="s">
-        <v>196</v>
+        <v>191</v>
+      </c>
+      <c r="L2" t="s">
+        <v>193</v>
       </c>
       <c r="M2" t="s">
-        <v>199</v>
-      </c>
-      <c r="N2" t="s">
-        <v>212</v>
+        <v>195</v>
       </c>
       <c r="O2" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="P2" t="s">
+        <v>211</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>213</v>
+      </c>
+      <c r="R2" t="s">
         <v>1</v>
       </c>
-      <c r="Q2" t="s">
-        <v>221</v>
-      </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
+        <v>220</v>
+      </c>
+      <c r="T2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:18" ht="225">
+    <row r="3" spans="2:20" ht="225">
       <c r="B3">
         <v>1</v>
       </c>
@@ -3600,50 +3758,54 @@
         <v>15</v>
       </c>
       <c r="D3" t="s">
+        <v>207</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="F3" t="s">
-        <v>187</v>
-      </c>
-      <c r="G3" t="s">
-        <v>189</v>
-      </c>
+      <c r="F3" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G3" s="1"/>
       <c r="H3" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="I3" t="s">
-        <v>193</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="K3" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="J3" t="s">
+        <v>190</v>
+      </c>
+      <c r="K3" t="s">
+        <v>192</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="N3" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="M3" s="1" t="s">
+      <c r="O3" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="P3" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="P3" s="3">
-        <v>46036</v>
-      </c>
-      <c r="Q3" s="3"/>
+      <c r="Q3" s="1" t="s">
+        <v>214</v>
+      </c>
       <c r="R3" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="4" spans="2:18" ht="206.25">
+      <c r="S3" s="3"/>
+      <c r="T3" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="4" spans="2:20" ht="375">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
@@ -3652,145 +3814,220 @@
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="F4" t="s">
-        <v>187</v>
-      </c>
-      <c r="G4" t="s">
-        <v>189</v>
-      </c>
+        <v>209</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G4" s="1"/>
       <c r="H4" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="I4" t="s">
-        <v>193</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="K4" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="J4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K4" t="s">
+        <v>192</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="N4" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="L4" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="M4" s="1" t="s">
+      <c r="O4" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="P4" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="P4" s="3">
-        <v>46036</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>18</v>
+      <c r="Q4" s="1" t="s">
+        <v>214</v>
       </c>
       <c r="R4" s="3">
         <v>46036</v>
       </c>
-    </row>
-    <row r="5" spans="2:18" ht="206.25">
+      <c r="S4" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="T4" s="3">
+        <v>46036</v>
+      </c>
+    </row>
+    <row r="5" spans="2:20" ht="206.25">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>204</v>
+      </c>
+      <c r="D5" t="s">
+        <v>206</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="D5" t="s">
-        <v>207</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="F5" t="s">
-        <v>187</v>
-      </c>
-      <c r="G5" t="s">
-        <v>189</v>
-      </c>
+      <c r="F5" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G5" s="1"/>
       <c r="H5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="I5" t="s">
-        <v>193</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="K5" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="J5" t="s">
+        <v>190</v>
+      </c>
+      <c r="K5" t="s">
+        <v>192</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="N5" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="L5" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>213</v>
-      </c>
       <c r="O5" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="P5" s="3">
+        <v>210</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="R5" s="3">
         <v>46039</v>
       </c>
     </row>
-    <row r="6" spans="2:18" ht="337.5">
+    <row r="6" spans="2:20" ht="337.5">
       <c r="B6">
         <f>B5+1</f>
         <v>4</v>
       </c>
       <c r="C6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D6" t="s">
         <v>216</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="G6" s="1"/>
+      <c r="H6" t="s">
+        <v>186</v>
+      </c>
+      <c r="I6" t="s">
+        <v>188</v>
+      </c>
+      <c r="J6" t="s">
+        <v>190</v>
+      </c>
+      <c r="K6" t="s">
+        <v>192</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="O6" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F6" t="s">
-        <v>187</v>
-      </c>
-      <c r="G6" t="s">
-        <v>189</v>
-      </c>
-      <c r="H6" t="s">
-        <v>191</v>
-      </c>
-      <c r="I6" t="s">
-        <v>193</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="M6" s="1" t="s">
+      <c r="P6" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="P6" s="3">
+      <c r="Q6" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="R6" s="3">
         <v>46039</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20">
+      <c r="B7">
+        <f>B6+1</f>
+        <v>5</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="8" spans="2:20">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>6</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20">
+      <c r="B9">
+        <f>B8+1</f>
+        <v>7</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="10" spans="2:20" ht="37.5">
+      <c r="B10">
+        <f>B9+1</f>
+        <v>8</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="11" spans="2:20">
+      <c r="B11">
+        <f>B10+1</f>
+        <v>9</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="12" spans="2:20">
+      <c r="B12">
+        <f>B11+1</f>
+        <v>10</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="13" spans="2:20">
+      <c r="B13">
+        <f>B12+1</f>
+        <v>11</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -3846,10 +4083,10 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" t="s">
         <v>44</v>
-      </c>
-      <c r="I2" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="3" spans="2:9">
@@ -3857,7 +4094,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F3" s="3">
         <v>46036</v>
@@ -3872,7 +4109,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F4" s="3">
         <v>46036</v>
@@ -3887,7 +4124,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F5" s="3">
         <v>46036</v>
@@ -3917,10 +4154,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
         <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
       </c>
       <c r="F7" s="3">
         <v>46036</v>
@@ -3935,10 +4172,10 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F8" s="3">
         <v>46038</v>
@@ -3950,7 +4187,7 @@
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="2:9">
@@ -3959,10 +4196,10 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
         <v>31</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
       </c>
       <c r="F10" s="3">
         <v>46036</v>
@@ -3977,7 +4214,7 @@
         <v>9</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="2:9">
@@ -3986,7 +4223,7 @@
         <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="2:9">
@@ -3995,10 +4232,10 @@
         <v>11</v>
       </c>
       <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
         <v>35</v>
-      </c>
-      <c r="D13" t="s">
-        <v>36</v>
       </c>
       <c r="F13" s="3">
         <v>46036</v>
@@ -4013,7 +4250,7 @@
         <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15" spans="2:9">
@@ -4022,7 +4259,7 @@
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="16" spans="2:9">
@@ -4031,10 +4268,10 @@
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="2:9">
@@ -4043,7 +4280,7 @@
         <v>15</v>
       </c>
       <c r="D17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="2:9">
@@ -4052,7 +4289,7 @@
         <v>16</v>
       </c>
       <c r="D18" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="2:9">
@@ -4061,13 +4298,13 @@
         <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D19" t="s">
+        <v>104</v>
+      </c>
+      <c r="E19" t="s">
         <v>105</v>
-      </c>
-      <c r="E19" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="20" spans="2:9">
@@ -4076,7 +4313,7 @@
         <v>18</v>
       </c>
       <c r="E20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="2:9">
@@ -4085,7 +4322,7 @@
         <v>19</v>
       </c>
       <c r="E21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="2:9">
@@ -4094,7 +4331,7 @@
         <v>20</v>
       </c>
       <c r="E22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="2:9">
@@ -4103,7 +4340,7 @@
         <v>21</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="2:9">
@@ -4112,10 +4349,10 @@
         <v>22</v>
       </c>
       <c r="C24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F24" s="3">
         <v>46037</v>
@@ -4136,7 +4373,7 @@
         <v>23</v>
       </c>
       <c r="D25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: update RealWorldDanshariPage to require ImagePicker and enhance integration test setup
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F7F5AA1-A687-43F5-9DDB-67FD56DF6064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4F8712-50F2-4C8C-98C8-FF0F36B9D760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="289">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1557,19 +1557,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>flutter clean
-flutter pub get
-dart fix --apply
-dart format .
-flutter analyze
-deno lint supabase
-dart run build_runner build --delete-conflicting-outputs
-flutter test --coverage
-supabase functions deploy ai-assistant
-flutter build web --release --no-tree-shake-icons</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Note: If you're at a business or would like more team-level benefits, consider Gemini Code Assist Standard or Enterprise.</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -1676,6 +1663,250 @@
   </si>
   <si>
     <t>supabase\functions\share-quote\index.ts</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>supabase functions deploy</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>flutter clean
+flutter pub get
+dart fix --apply
+dart format .
+flutter analyze
+deno lint supabase
+dart run build_runner build --delete-conflicting-outputs
+flutter test --coverage
+supabase functions deploy
+flutter build web --release --no-tree-shake-icons</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>API名 (Function Name)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ai-assistant</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ai-search</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/ai-search</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>概要 (Description)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>主要パラメータ (Params)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>action (必須), model, content, imageBase64</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>query (必須), limit</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AI統合アシスタント
+モデル取得、画像分析（断捨離）、会議シミュレーション、汎用テキスト処理を行うマルチ機能API。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AIセマンティック検索
+OpenAI Embeddingsとpgvectorを使用し、メモの意味検索とAIによる再ランク付けを行う。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>名言画像生成 (OGP)
+指定されたIDの名言をSVG画像（OGPサイズ）として動的に生成して返す。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GET</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/get-ogp</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>OGP情報取得
+URLからメタデータ（タイトル、画像、説明文）を取得する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>url</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>generate-quote-image</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今日使ったお金を確認する</t>
+    <rPh sb="0" eb="2">
+      <t>キョウ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ツカ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>カネ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今月の支出額を確認する</t>
+    <rPh sb="0" eb="2">
+      <t>コンゲツ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シシュツ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ガク</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今月の支出予定を確認する</t>
+    <rPh sb="0" eb="2">
+      <t>コンゲツ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シシュツ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ヨテイ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>不要なサブスクを解約する</t>
+    <rPh sb="0" eb="2">
+      <t>フヨウ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カイヤク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/generate-quote-image</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>id (クエリパラメータ)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/daily-judgment</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>daily-judgment</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>日次評価システム
+ユーザーの活動データを分析し、信頼スコアの更新や警告メールの送信を行う。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>(内部処理用 / CRON想定)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>generate-daily-challenges</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>get-ogp</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>share-quote</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/share-quote</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/generate-daily-challenges</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デイリークエスト生成
+ユーザーの過去の行動や目標に基づいて、その日のタスク（クエスト）を生成する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>名言シェア機能
+名言をSNS等でシェアするための短縮URLや共有用データを生成する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>quoteId</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>大機能</t>
+    <rPh sb="0" eb="3">
+      <t>ダイキノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>中機能</t>
+    <rPh sb="0" eb="1">
+      <t>チュウ</t>
+    </rPh>
+    <rPh sb="1" eb="3">
+      <t>キノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>処理内容</t>
+    <rPh sb="0" eb="2">
+      <t>ショリ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ナイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Action</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>analyze_danshari_item</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ホーム画面またはメニューから「リアル断捨離」を選択する。
+カメラアイコンをタップし、カメラで撮影またはギャラリーから画像を選択する。
+画像が表示されたら「AIに判定してもらう」ボタンをタップする。
+AI（CSO）による判定結果（KEEP/DISCARD）と辛口コメントが表示されることを確認する。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2070,7 +2301,7 @@
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.625" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
@@ -2147,6 +2378,9 @@
         <f>B6+1</f>
         <v>5</v>
       </c>
+      <c r="C7" t="s">
+        <v>265</v>
+      </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
     </row>
@@ -2155,17 +2389,26 @@
         <f>B7+1</f>
         <v>6</v>
       </c>
+      <c r="C8" t="s">
+        <v>266</v>
+      </c>
     </row>
     <row r="9" spans="2:8">
       <c r="B9">
         <f>B8+1</f>
         <v>7</v>
       </c>
+      <c r="C9" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="10" spans="2:8">
       <c r="B10">
         <f>B9+1</f>
         <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>268</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -2670,42 +2913,42 @@
     </row>
     <row r="15" spans="2:5" ht="37.5">
       <c r="B15" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>227</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="56.25">
       <c r="B16" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>229</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="17" spans="2:3">
       <c r="B17" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C17" s="1" t="s">
         <v>231</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="18" spans="2:3">
       <c r="B18" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C18" s="1" t="s">
         <v>233</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="19" spans="2:3">
       <c r="B19" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>235</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -2983,7 +3226,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="B3:D17"/>
+  <dimension ref="B3:D18"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
@@ -3054,7 +3297,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="37.5">
@@ -3118,6 +3361,15 @@
       </c>
       <c r="C17" s="1" t="s">
         <v>225</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18">
+        <f>B17+1</f>
+        <v>15</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -3683,7 +3935,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
-  <dimension ref="B2:T13"/>
+  <dimension ref="B2:X13"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.75" bestFit="1" customWidth="1"/>
@@ -3691,66 +3943,91 @@
     <col min="4" max="4" width="31.75" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="34.25" customWidth="1"/>
     <col min="6" max="6" width="54.875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="34.25" customWidth="1"/>
-    <col min="8" max="8" width="26" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="32.625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="75.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="65.75" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="65.75" customWidth="1"/>
-    <col min="15" max="15" width="50.125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="50.125" customWidth="1"/>
-    <col min="18" max="18" width="10.25" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="47" customWidth="1"/>
-    <col min="20" max="20" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.875" customWidth="1"/>
+    <col min="8" max="8" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.625" customWidth="1"/>
+    <col min="10" max="10" width="35.75" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.75" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="32.625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="75.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="65.75" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="65.75" customWidth="1"/>
+    <col min="19" max="19" width="50.125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="50.125" customWidth="1"/>
+    <col min="22" max="22" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="47" customWidth="1"/>
+    <col min="24" max="24" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20">
+    <row r="2" spans="2:24">
+      <c r="C2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" t="s">
+        <v>284</v>
+      </c>
+      <c r="E2" t="s">
+        <v>285</v>
+      </c>
       <c r="F2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H2" t="s">
+        <v>249</v>
+      </c>
+      <c r="I2" t="s">
+        <v>286</v>
+      </c>
+      <c r="J2" t="s">
         <v>185</v>
       </c>
-      <c r="I2" t="s">
+      <c r="K2" t="s">
         <v>187</v>
       </c>
-      <c r="J2" t="s">
+      <c r="L2" t="s">
+        <v>253</v>
+      </c>
+      <c r="M2" t="s">
+        <v>254</v>
+      </c>
+      <c r="N2" t="s">
         <v>189</v>
       </c>
-      <c r="K2" t="s">
+      <c r="O2" t="s">
         <v>191</v>
       </c>
-      <c r="L2" t="s">
+      <c r="P2" t="s">
         <v>193</v>
       </c>
-      <c r="M2" t="s">
+      <c r="Q2" t="s">
         <v>195</v>
       </c>
-      <c r="O2" t="s">
+      <c r="S2" t="s">
         <v>198</v>
       </c>
-      <c r="P2" t="s">
+      <c r="T2" t="s">
         <v>211</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="U2" t="s">
         <v>213</v>
       </c>
-      <c r="R2" t="s">
+      <c r="V2" t="s">
         <v>1</v>
       </c>
-      <c r="S2" t="s">
+      <c r="W2" t="s">
         <v>220</v>
       </c>
-      <c r="T2" t="s">
+      <c r="X2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:20" ht="225">
+    <row r="3" spans="2:24" ht="225">
       <c r="B3">
         <v>1</v>
       </c>
@@ -3764,48 +4041,62 @@
         <v>208</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="G3" s="1"/>
-      <c r="H3" t="s">
+        <v>239</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="J3" t="s">
         <v>186</v>
       </c>
-      <c r="I3" t="s">
+      <c r="K3" t="s">
         <v>188</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="M3" t="s">
+        <v>255</v>
+      </c>
+      <c r="N3" t="s">
         <v>190</v>
       </c>
-      <c r="K3" t="s">
+      <c r="O3" t="s">
         <v>192</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="P3" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="Q3" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="R3" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="S3" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="T3" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="Q3" s="1" t="s">
+      <c r="U3" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="R3" s="3">
+      <c r="V3" s="3">
         <v>46036</v>
       </c>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3">
+      <c r="W3" s="3"/>
+      <c r="X3" s="3">
         <v>46036</v>
       </c>
     </row>
-    <row r="4" spans="2:20" ht="375">
+    <row r="4" spans="2:24" ht="375">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
@@ -3820,50 +4111,60 @@
         <v>209</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G4" s="1"/>
-      <c r="H4" t="s">
+      <c r="H4" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" t="s">
         <v>186</v>
       </c>
-      <c r="I4" t="s">
+      <c r="K4" t="s">
         <v>188</v>
       </c>
-      <c r="J4" t="s">
+      <c r="L4" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="M4" t="s">
+        <v>255</v>
+      </c>
+      <c r="N4" t="s">
         <v>190</v>
       </c>
-      <c r="K4" t="s">
+      <c r="O4" t="s">
         <v>192</v>
       </c>
-      <c r="L4" s="1" t="s">
+      <c r="P4" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="R4" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="S4" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="T4" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="U4" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="R4" s="3">
+      <c r="V4" s="3">
         <v>46036</v>
       </c>
-      <c r="S4" s="1" t="s">
-        <v>237</v>
-      </c>
-      <c r="T4" s="3">
+      <c r="W4" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="X4" s="3">
         <v>46036</v>
       </c>
     </row>
-    <row r="5" spans="2:20" ht="206.25">
+    <row r="5" spans="2:24" ht="206.25">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
@@ -3878,44 +4179,54 @@
         <v>205</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G5" s="1"/>
-      <c r="H5" t="s">
+      <c r="H5" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" t="s">
         <v>186</v>
       </c>
-      <c r="I5" t="s">
+      <c r="K5" t="s">
         <v>188</v>
       </c>
-      <c r="J5" t="s">
+      <c r="L5" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="M5" t="s">
+        <v>255</v>
+      </c>
+      <c r="N5" t="s">
         <v>190</v>
       </c>
-      <c r="K5" t="s">
+      <c r="O5" t="s">
         <v>192</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="P5" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="R5" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="S5" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="T5" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="U5" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="R5" s="3">
+      <c r="V5" s="3">
         <v>46039</v>
       </c>
     </row>
-    <row r="6" spans="2:20" ht="337.5">
+    <row r="6" spans="2:24" ht="337.5">
       <c r="B6">
         <f>B5+1</f>
         <v>4</v>
@@ -3930,104 +4241,229 @@
         <v>217</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G6" s="1"/>
-      <c r="H6" t="s">
+      <c r="H6" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="I6" s="1"/>
+      <c r="J6" t="s">
         <v>186</v>
       </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>188</v>
       </c>
-      <c r="J6" t="s">
+      <c r="L6" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="M6" t="s">
+        <v>255</v>
+      </c>
+      <c r="N6" t="s">
         <v>190</v>
       </c>
-      <c r="K6" t="s">
+      <c r="O6" t="s">
         <v>192</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="P6" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="Q6" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="R6" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="S6" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="T6" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="U6" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="R6" s="3">
+      <c r="V6" s="3">
         <v>46039</v>
       </c>
     </row>
-    <row r="7" spans="2:20">
+    <row r="7" spans="2:24" ht="187.5">
       <c r="B7">
         <f>B6+1</f>
         <v>5</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="8" spans="2:20">
+        <v>240</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" t="s">
+        <v>252</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="N7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="2:24">
       <c r="B8">
         <f>B7+1</f>
         <v>6</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="9" spans="2:20">
+        <v>241</v>
+      </c>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+    </row>
+    <row r="9" spans="2:24" ht="150">
       <c r="B9">
         <f>B8+1</f>
         <v>7</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="10" spans="2:20" ht="37.5">
+        <v>242</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="I9" s="1"/>
+      <c r="J9" t="s">
+        <v>271</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="N9" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="10" spans="2:24" ht="168.75">
       <c r="B10">
         <f>B9+1</f>
         <v>8</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="11" spans="2:20">
+        <v>243</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" t="s">
+        <v>279</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="N10" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="11" spans="2:24" ht="131.25">
       <c r="B11">
         <f>B10+1</f>
         <v>9</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="12" spans="2:20">
+        <v>244</v>
+      </c>
+      <c r="H11" t="s">
+        <v>264</v>
+      </c>
+      <c r="J11" t="s">
+        <v>269</v>
+      </c>
+      <c r="K11" t="s">
+        <v>260</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="M11" t="s">
+        <v>270</v>
+      </c>
+      <c r="N11" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="12" spans="2:24" ht="131.25">
       <c r="B12">
         <f>B11+1</f>
         <v>10</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="13" spans="2:20">
+        <v>245</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" t="s">
+        <v>261</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="M12" t="s">
+        <v>263</v>
+      </c>
+      <c r="N12" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="13" spans="2:24" ht="131.25">
       <c r="B13">
         <f>B12+1</f>
         <v>11</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" t="s">
+        <v>278</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="N13" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add CashManagementPage and integrate it into CfoOfficePage menu
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4F8712-50F2-4C8C-98C8-FF0F36B9D760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DC4D3B-5511-441F-8A50-F0E7271DF208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="291">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1907,6 +1907,24 @@
 カメラアイコンをタップし、カメラで撮影またはギャラリーから画像を選択する。
 画像が表示されたら「AIに判定してもらう」ボタンをタップする。
 AI（CSO）による判定結果（KEEP/DISCARD）と辛口コメントが表示されることを確認する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>財務管理（CFO）機能を改善してください。
+まず、毎日財布の中の現金を登録する機能と、登録された現金の情報を元に現金残高推移をグラフ表示できる機能を追加してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現金残高推移</t>
+    <rPh sb="0" eb="2">
+      <t>ゲンキン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ザンダカ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>スイイ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2480,45 +2498,46 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A27E184-E904-4778-A996-9404F32C3EC7}">
-  <dimension ref="B1:H19"/>
+  <dimension ref="B1:I19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.75" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="6" max="7" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8">
-      <c r="E1" s="3">
+    <row r="1" spans="2:9">
+      <c r="F1" s="3">
         <f ca="1">TODAY()</f>
         <v>46039</v>
       </c>
     </row>
-    <row r="2" spans="2:8">
-      <c r="E2" t="s">
+    <row r="2" spans="2:9">
+      <c r="F2" t="s">
         <v>1</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>2</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>43</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="2:8">
+    <row r="3" spans="2:9">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="3"/>
       <c r="F3" s="3"/>
-    </row>
-    <row r="4" spans="2:8">
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="2:9">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
@@ -2526,10 +2545,10 @@
       <c r="C4" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-    </row>
-    <row r="5" spans="2:8">
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="2:9">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
@@ -2537,103 +2556,109 @@
       <c r="C5" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="3"/>
       <c r="F5" s="3"/>
-    </row>
-    <row r="6" spans="2:8">
+      <c r="G5" s="3"/>
+    </row>
+    <row r="6" spans="2:9" ht="93.75">
       <c r="B6">
         <f>B5+1</f>
         <v>4</v>
       </c>
-      <c r="E6" s="3"/>
+      <c r="C6" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>289</v>
+      </c>
       <c r="F6" s="3"/>
-    </row>
-    <row r="7" spans="2:8">
+      <c r="G6" s="3"/>
+    </row>
+    <row r="7" spans="2:9">
       <c r="B7">
         <f>B6+1</f>
         <v>5</v>
       </c>
-      <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-    </row>
-    <row r="8" spans="2:8">
+      <c r="G7" s="3"/>
+    </row>
+    <row r="8" spans="2:9">
       <c r="B8">
         <f>B7+1</f>
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:8">
+    <row r="9" spans="2:9">
       <c r="B9">
         <f>B8+1</f>
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="2:8">
+    <row r="10" spans="2:9">
       <c r="B10">
         <f>B9+1</f>
         <v>8</v>
       </c>
-      <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-    </row>
-    <row r="11" spans="2:8">
+      <c r="G10" s="3"/>
+    </row>
+    <row r="11" spans="2:9">
       <c r="B11">
         <f>B10+1</f>
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="2:8">
+    <row r="12" spans="2:9">
       <c r="B12">
         <f>B11+1</f>
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="2:8">
+    <row r="13" spans="2:9">
       <c r="B13">
         <f>B12+1</f>
         <v>11</v>
       </c>
-      <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-    </row>
-    <row r="14" spans="2:8">
+      <c r="G13" s="3"/>
+    </row>
+    <row r="14" spans="2:9">
       <c r="B14">
         <f>B13+1</f>
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:8">
+    <row r="15" spans="2:9">
       <c r="B15">
         <f>B14+1</f>
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="2:8">
+    <row r="16" spans="2:9">
       <c r="B16">
         <f>B15+1</f>
         <v>14</v>
       </c>
     </row>
-    <row r="17" spans="2:7">
+    <row r="17" spans="2:8">
       <c r="B17">
         <f>B16+1</f>
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="2:7">
+    <row r="18" spans="2:8">
       <c r="B18">
         <f>B17+1</f>
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="2:7">
+    <row r="19" spans="2:8">
       <c r="B19">
         <f>B18+1</f>
         <v>17</v>
       </c>
-      <c r="E19" s="3"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -4625,6 +4650,9 @@
       <c r="D9" t="s">
         <v>29</v>
       </c>
+      <c r="F9" s="3">
+        <v>46039</v>
+      </c>
     </row>
     <row r="10" spans="2:9">
       <c r="B10">

</xml_diff>

<commit_message>
refactor: update Gemini API reference content and improve quiz question for clarity
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12DC4D3B-5511-441F-8A50-F0E7271DF208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F44E670-0624-4DC3-BDE9-572914F5D2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="296">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1670,11 +1670,257 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>API名 (Function Name)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ai-assistant</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ai-search</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/ai-search</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>概要 (Description)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>主要パラメータ (Params)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>action (必須), model, content, imageBase64</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>query (必須), limit</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AI統合アシスタント
+モデル取得、画像分析（断捨離）、会議シミュレーション、汎用テキスト処理を行うマルチ機能API。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AIセマンティック検索
+OpenAI Embeddingsとpgvectorを使用し、メモの意味検索とAIによる再ランク付けを行う。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>名言画像生成 (OGP)
+指定されたIDの名言をSVG画像（OGPサイズ）として動的に生成して返す。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GET</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/get-ogp</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>OGP情報取得
+URLからメタデータ（タイトル、画像、説明文）を取得する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>url</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>generate-quote-image</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今日使ったお金を確認する</t>
+    <rPh sb="0" eb="2">
+      <t>キョウ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ツカ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>カネ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今月の支出額を確認する</t>
+    <rPh sb="0" eb="2">
+      <t>コンゲツ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シシュツ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ガク</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今月の支出予定を確認する</t>
+    <rPh sb="0" eb="2">
+      <t>コンゲツ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シシュツ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>ヨテイ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カクニン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>不要なサブスクを解約する</t>
+    <rPh sb="0" eb="2">
+      <t>フヨウ</t>
+    </rPh>
+    <rPh sb="8" eb="10">
+      <t>カイヤク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/generate-quote-image</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>id (クエリパラメータ)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/daily-judgment</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>daily-judgment</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>日次評価システム
+ユーザーの活動データを分析し、信頼スコアの更新や警告メールの送信を行う。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>(内部処理用 / CRON想定)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>generate-daily-challenges</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>get-ogp</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>share-quote</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/share-quote</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>/functions/v1/generate-daily-challenges</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デイリークエスト生成
+ユーザーの過去の行動や目標に基づいて、その日のタスク（クエスト）を生成する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>名言シェア機能
+名言をSNS等でシェアするための短縮URLや共有用データを生成する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>quoteId</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>大機能</t>
+    <rPh sb="0" eb="3">
+      <t>ダイキノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>中機能</t>
+    <rPh sb="0" eb="1">
+      <t>チュウ</t>
+    </rPh>
+    <rPh sb="1" eb="3">
+      <t>キノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>処理内容</t>
+    <rPh sb="0" eb="2">
+      <t>ショリ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ナイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Action</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>analyze_danshari_item</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ホーム画面またはメニューから「リアル断捨離」を選択する。
+カメラアイコンをタップし、カメラで撮影またはギャラリーから画像を選択する。
+画像が表示されたら「AIに判定してもらう」ボタンをタップする。
+AI（CSO）による判定結果（KEEP/DISCARD）と辛口コメントが表示されることを確認する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>財務管理（CFO）機能を改善してください。
+まず、毎日財布の中の現金を登録する機能と、登録された現金の情報を元に現金残高推移をグラフ表示できる機能を追加してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現金残高推移</t>
+    <rPh sb="0" eb="2">
+      <t>ゲンキン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ザンダカ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>スイイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>flutter clean
 flutter pub get
 dart fix --apply
 dart format .
 flutter analyze
+deno check supabase
 deno lint supabase
 dart run build_runner build --delete-conflicting-outputs
 flutter test --coverage
@@ -1683,248 +1929,23 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>API名 (Function Name)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ai-assistant</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ai-search</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>/functions/v1/ai-search</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>概要 (Description)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>主要パラメータ (Params)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>action (必須), model, content, imageBase64</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>query (必須), limit</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>AI統合アシスタント
-モデル取得、画像分析（断捨離）、会議シミュレーション、汎用テキスト処理を行うマルチ機能API。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>AIセマンティック検索
-OpenAI Embeddingsとpgvectorを使用し、メモの意味検索とAIによる再ランク付けを行う。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>名言画像生成 (OGP)
-指定されたIDの名言をSVG画像（OGPサイズ）として動的に生成して返す。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>GET</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>/functions/v1/get-ogp</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>OGP情報取得
-URLからメタデータ（タイトル、画像、説明文）を取得する。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>url</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>generate-quote-image</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>今日使ったお金を確認する</t>
-    <rPh sb="0" eb="2">
-      <t>キョウ</t>
-    </rPh>
-    <rPh sb="2" eb="3">
-      <t>ツカ</t>
-    </rPh>
-    <rPh sb="6" eb="7">
-      <t>カネ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>カクニン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>今月の支出額を確認する</t>
-    <rPh sb="0" eb="2">
-      <t>コンゲツ</t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t>シシュツ</t>
-    </rPh>
-    <rPh sb="5" eb="6">
-      <t>ガク</t>
-    </rPh>
-    <rPh sb="7" eb="9">
-      <t>カクニン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>今月の支出予定を確認する</t>
-    <rPh sb="0" eb="2">
-      <t>コンゲツ</t>
-    </rPh>
-    <rPh sb="3" eb="5">
-      <t>シシュツ</t>
-    </rPh>
-    <rPh sb="5" eb="7">
-      <t>ヨテイ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>カクニン</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>不要なサブスクを解約する</t>
-    <rPh sb="0" eb="2">
-      <t>フヨウ</t>
-    </rPh>
-    <rPh sb="8" eb="10">
-      <t>カイヤク</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>/functions/v1/generate-quote-image</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>id (クエリパラメータ)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>/functions/v1/daily-judgment</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>daily-judgment</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>日次評価システム
-ユーザーの活動データを分析し、信頼スコアの更新や警告メールの送信を行う。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>(内部処理用 / CRON想定)</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>generate-daily-challenges</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>get-ogp</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>share-quote</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>/functions/v1/share-quote</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>/functions/v1/generate-daily-challenges</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>デイリークエスト生成
-ユーザーの過去の行動や目標に基づいて、その日のタスク（クエスト）を生成する。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>名言シェア機能
-名言をSNS等でシェアするための短縮URLや共有用データを生成する。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>quoteId</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>大機能</t>
-    <rPh sb="0" eb="3">
-      <t>ダイキノウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>中機能</t>
-    <rPh sb="0" eb="1">
-      <t>チュウ</t>
-    </rPh>
-    <rPh sb="1" eb="3">
-      <t>キノウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>処理内容</t>
-    <rPh sb="0" eb="2">
-      <t>ショリ</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ナイヨウ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>Action</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>analyze_danshari_item</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>ホーム画面またはメニューから「リアル断捨離」を選択する。
-カメラアイコンをタップし、カメラで撮影またはギャラリーから画像を選択する。
-画像が表示されたら「AIに判定してもらう」ボタンをタップする。
-AI（CSO）による判定結果（KEEP/DISCARD）と辛口コメントが表示されることを確認する。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>財務管理（CFO）機能を改善してください。
-まず、毎日財布の中の現金を登録する機能と、登録された現金の情報を元に現金残高推移をグラフ表示できる機能を追加してください。</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>現金残高推移</t>
-    <rPh sb="0" eb="2">
-      <t>ゲンキン</t>
-    </rPh>
-    <rPh sb="2" eb="4">
-      <t>ザンダカ</t>
-    </rPh>
-    <rPh sb="4" eb="6">
-      <t>スイイ</t>
-    </rPh>
+    <t>Platform APIs: Utility endpoints that support core capabilities such as uploading files, and counting tokens.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>プラットフォームAPI：ファイルのアップロードやトークンのカウントといった中核機能をサポートするユーティリティエンドポイント。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>認証</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>All requests to the Gemini API must include an x-goog-api-key header with your API key. Create one with a few clicks in Google AI Studio.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini APIへのすべてのリクエストには、APIキーを含むx-goog-api-keyヘッダーを含める必要があります。Google AI Studioで数クリックで作成できます。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2397,7 +2418,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -2408,7 +2429,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" spans="2:8">
@@ -2417,7 +2438,7 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="10" spans="2:8">
@@ -2426,7 +2447,7 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -2565,10 +2586,10 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -2668,7 +2689,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E22"/>
+  <dimension ref="B1:E27"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="42.5" customWidth="1"/>
@@ -2822,6 +2843,33 @@
       </c>
       <c r="E22" s="3">
         <v>46038</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="56.25">
+      <c r="B23" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E23" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" ht="75">
+      <c r="B27" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -3316,13 +3364,13 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="187.5">
+    <row r="10" spans="2:4" ht="206.25">
       <c r="B10">
         <f>B9+1</f>
         <v>7</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>248</v>
+        <v>290</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="37.5">
@@ -3989,13 +4037,13 @@
   <sheetData>
     <row r="2" spans="2:24">
       <c r="C2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D2" t="s">
         <v>283</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>284</v>
-      </c>
-      <c r="E2" t="s">
-        <v>285</v>
       </c>
       <c r="F2" t="s">
         <v>238</v>
@@ -4004,10 +4052,10 @@
         <v>237</v>
       </c>
       <c r="H2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J2" t="s">
         <v>185</v>
@@ -4016,10 +4064,10 @@
         <v>187</v>
       </c>
       <c r="L2" t="s">
+        <v>252</v>
+      </c>
+      <c r="M2" t="s">
         <v>253</v>
-      </c>
-      <c r="M2" t="s">
-        <v>254</v>
       </c>
       <c r="N2" t="s">
         <v>189</v>
@@ -4069,13 +4117,13 @@
         <v>239</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J3" t="s">
         <v>186</v>
@@ -4084,10 +4132,10 @@
         <v>188</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="M3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="N3" t="s">
         <v>190</v>
@@ -4140,7 +4188,7 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" t="s">
@@ -4150,10 +4198,10 @@
         <v>188</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="M4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="N4" t="s">
         <v>190</v>
@@ -4208,7 +4256,7 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" t="s">
@@ -4218,10 +4266,10 @@
         <v>188</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="M5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="N5" t="s">
         <v>190</v>
@@ -4270,7 +4318,7 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" t="s">
@@ -4280,10 +4328,10 @@
         <v>188</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="M6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="N6" t="s">
         <v>190</v>
@@ -4322,20 +4370,20 @@
         <v>240</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>188</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="N7" t="s">
         <v>190</v>
@@ -4361,20 +4409,20 @@
         <v>242</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>188</v>
       </c>
       <c r="L9" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>273</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>274</v>
       </c>
       <c r="N9" t="s">
         <v>190</v>
@@ -4389,20 +4437,20 @@
         <v>243</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>188</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="N10" t="s">
         <v>190</v>
@@ -4417,19 +4465,19 @@
         <v>244</v>
       </c>
       <c r="H11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="J11" t="s">
+        <v>268</v>
+      </c>
+      <c r="K11" t="s">
+        <v>259</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="M11" t="s">
         <v>269</v>
-      </c>
-      <c r="K11" t="s">
-        <v>260</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="M11" t="s">
-        <v>270</v>
       </c>
       <c r="N11" t="s">
         <v>190</v>
@@ -4444,20 +4492,20 @@
         <v>245</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>188</v>
       </c>
       <c r="L12" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="M12" t="s">
         <v>262</v>
-      </c>
-      <c r="M12" t="s">
-        <v>263</v>
       </c>
       <c r="N12" t="s">
         <v>190</v>
@@ -4472,20 +4520,20 @@
         <v>246</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>188</v>
       </c>
       <c r="L13" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="M13" s="1" t="s">
         <v>281</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>282</v>
       </c>
       <c r="N13" t="s">
         <v>190</v>

</xml_diff>

<commit_message>
Refactor asset management and cash management pages; remove web deployment issues documentation
- Deleted the WEB_DEPLOYMENT_ISSUES.md file as it is no longer needed.
- Updated CashManagementPage to improve text formatting and layout.
- Replaced CashManagementPage with AssetManagementPage in CfoOfficePage.
- Added AssetManagementPage with functionality for managing and visualizing asset data.
- Improved code readability and structure across various files.
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F44E670-0624-4DC3-BDE9-572914F5D2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632B692D-0C42-43E4-A5A1-1E938525BED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,9 @@
     <sheet name="機能一覧" sheetId="8" r:id="rId9"/>
     <sheet name="デイリータスク" sheetId="10" r:id="rId10"/>
     <sheet name="追加したい機能" sheetId="11" r:id="rId11"/>
-    <sheet name="Gemini API reference" sheetId="12" r:id="rId12"/>
-    <sheet name="Gemini Code Assist" sheetId="15" r:id="rId13"/>
-    <sheet name="プロンプト集" sheetId="13" r:id="rId14"/>
+    <sheet name="プロンプト集" sheetId="13" r:id="rId12"/>
+    <sheet name="Gemini API reference" sheetId="12" r:id="rId13"/>
+    <sheet name="Gemini Code Assist" sheetId="15" r:id="rId14"/>
     <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="299">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1946,6 +1946,30 @@
   </si>
   <si>
     <t>Gemini APIへのすべてのリクエストには、APIキーを含むx-goog-api-keyヘッダーを含める必要があります。Google AI Studioで数クリックで作成できます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現金管理</t>
+    <rPh sb="0" eb="2">
+      <t>ゲンキン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現金管理機能ですが、銀行口座残高等も登録して資産管理ができるように更新してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>資産管理</t>
+    <rPh sb="0" eb="2">
+      <t>シサン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンリ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2591,16 +2615,30 @@
       <c r="D6" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-    </row>
-    <row r="7" spans="2:9">
+      <c r="F6" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G6" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" ht="37.5">
       <c r="B7">
         <f>B6+1</f>
         <v>5</v>
       </c>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="C7" t="s">
+        <v>298</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="F7" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G7" s="3">
+        <v>46039</v>
+      </c>
     </row>
     <row r="8" spans="2:9">
       <c r="B8">
@@ -2688,356 +2726,6 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E27"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
-  <cols>
-    <col min="2" max="2" width="42.5" customWidth="1"/>
-    <col min="3" max="3" width="43.5" customWidth="1"/>
-    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:5">
-      <c r="E1" s="3">
-        <f ca="1">TODAY()</f>
-        <v>46039</v>
-      </c>
-    </row>
-    <row r="2" spans="2:5">
-      <c r="B2" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="2:5">
-      <c r="B3" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5">
-      <c r="B4" s="5" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5">
-      <c r="B6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5">
-      <c r="B7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" ht="56.25">
-      <c r="B8" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" ht="37.5">
-      <c r="B9" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" ht="37.5">
-      <c r="B10" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" ht="75">
-      <c r="B11" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="13" spans="2:5">
-      <c r="B13" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" ht="37.5">
-      <c r="B15" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" ht="93.75">
-      <c r="B17" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="2:5" ht="112.5">
-      <c r="B18" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" spans="2:5" ht="75">
-      <c r="B19" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="E19" s="3">
-        <v>46037</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" ht="56.25">
-      <c r="B20" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E20" s="3">
-        <v>46038</v>
-      </c>
-    </row>
-    <row r="21" spans="2:5" ht="56.25">
-      <c r="B21" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="E21" s="3">
-        <v>46038</v>
-      </c>
-    </row>
-    <row r="22" spans="2:5" ht="93.75">
-      <c r="B22" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="E22" s="3">
-        <v>46038</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" ht="56.25">
-      <c r="B23" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="E23" s="3">
-        <v>46039</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5">
-      <c r="B25" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" ht="75">
-      <c r="B27" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>295</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://ai.google.dev/" xr:uid="{D6844177-6821-498C-95D2-F6B6D63F1D22}"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://ai.google.dev/gemini-api" xr:uid="{2CDC8D53-0630-4185-9E29-7B79EBBE1F53}"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://ai.google.dev/api" xr:uid="{4A9752DB-169C-4F26-B3F6-A0018804884D}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E19"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
-  <cols>
-    <col min="2" max="2" width="73.125" customWidth="1"/>
-    <col min="3" max="3" width="72.5" customWidth="1"/>
-    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:5">
-      <c r="E1" s="3">
-        <f ca="1">TODAY()</f>
-        <v>46039</v>
-      </c>
-    </row>
-    <row r="2" spans="2:5">
-      <c r="B2" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="2:5">
-      <c r="B3" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5">
-      <c r="B4" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5">
-      <c r="B5" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5">
-      <c r="B6" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5">
-      <c r="B8" t="s">
-        <v>129</v>
-      </c>
-      <c r="C8" t="s">
-        <v>130</v>
-      </c>
-      <c r="E8" s="3">
-        <v>46039</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" ht="37.5">
-      <c r="B9" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" ht="37.5">
-      <c r="B10" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" ht="37.5">
-      <c r="B11" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" ht="37.5">
-      <c r="B12" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" ht="37.5">
-      <c r="B13" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" ht="37.5">
-      <c r="B14" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" ht="37.5">
-      <c r="B15" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" ht="56.25">
-      <c r="B16" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3">
-      <c r="B17" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3">
-      <c r="B18" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3">
-      <c r="B19" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>235</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" display="https://developers.google.com/" xr:uid="{29CCC4AC-286B-4EC0-BB01-ECE2B318A3E0}"/>
-    <hyperlink ref="B4" r:id="rId2" display="https://developers.google.com/products" xr:uid="{CF0BCE14-7EC1-458F-B767-95D6891C081A}"/>
-    <hyperlink ref="B5" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{DAA66992-CDAB-4563-A108-1D3004893841}"/>
-    <hyperlink ref="B6" r:id="rId4" display="https://developers.google.com/gemini-code-assist/docs/overview" xr:uid="{D4606693-ABC6-4C4C-8030-AFF9956F016B}"/>
-    <hyperlink ref="B2" r:id="rId5" xr:uid="{F2F2C855-BA2E-4DBF-BDB7-B571F8EBFB8B}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{475FE61E-6EC0-4C61-9FD0-98172694F2E5}">
   <dimension ref="B1:H19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -3197,6 +2885,359 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
+  <dimension ref="B1:E27"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="42.5" customWidth="1"/>
+    <col min="3" max="3" width="46.75" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5">
+      <c r="B2" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="B7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="56.25">
+      <c r="B8" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="37.5">
+      <c r="B9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="37.5">
+      <c r="B10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="75">
+      <c r="B11" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E11" s="3"/>
+    </row>
+    <row r="13" spans="2:5">
+      <c r="B13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="37.5">
+      <c r="B15" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="93.75">
+      <c r="B17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="3"/>
+    </row>
+    <row r="18" spans="2:5" ht="112.5">
+      <c r="B18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="2:5" ht="75">
+      <c r="B19" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E19" s="3">
+        <v>46037</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="56.25">
+      <c r="B20" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" ht="56.25">
+      <c r="B21" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" ht="93.75">
+      <c r="B22" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E22" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" ht="56.25">
+      <c r="B23" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="E23" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5">
+      <c r="B25" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" ht="56.25">
+      <c r="B27" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="E27" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://ai.google.dev/" xr:uid="{D6844177-6821-498C-95D2-F6B6D63F1D22}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://ai.google.dev/gemini-api" xr:uid="{2CDC8D53-0630-4185-9E29-7B79EBBE1F53}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://ai.google.dev/api" xr:uid="{4A9752DB-169C-4F26-B3F6-A0018804884D}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
+  <dimension ref="B1:E19"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="73.125" customWidth="1"/>
+    <col min="3" max="3" width="72.5" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5">
+      <c r="B2" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E8" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="37.5">
+      <c r="B9" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="37.5">
+      <c r="B10" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="37.5">
+      <c r="B11" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="37.5">
+      <c r="B12" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="37.5">
+      <c r="B13" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="37.5">
+      <c r="B14" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="37.5">
+      <c r="B15" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="56.25">
+      <c r="B16" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" display="https://developers.google.com/" xr:uid="{29CCC4AC-286B-4EC0-BB01-ECE2B318A3E0}"/>
+    <hyperlink ref="B4" r:id="rId2" display="https://developers.google.com/products" xr:uid="{CF0BCE14-7EC1-458F-B767-95D6891C081A}"/>
+    <hyperlink ref="B5" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{DAA66992-CDAB-4563-A108-1D3004893841}"/>
+    <hyperlink ref="B6" r:id="rId4" display="https://developers.google.com/gemini-code-assist/docs/overview" xr:uid="{D4606693-ABC6-4C4C-8030-AFF9956F016B}"/>
+    <hyperlink ref="B2" r:id="rId5" xr:uid="{F2F2C855-BA2E-4DBF-BDB7-B571F8EBFB8B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4574,7 +4615,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
-  <dimension ref="B2:I25"/>
+  <dimension ref="B2:I26"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
@@ -4659,232 +4700,247 @@
     </row>
     <row r="7" spans="2:9">
       <c r="B7">
+        <f>B5+1</f>
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
+        <v>296</v>
+      </c>
+      <c r="F7" s="3">
+        <v>46039</v>
+      </c>
+      <c r="G7" s="3">
+        <v>46039</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9">
+      <c r="B8">
         <f>B6+1</f>
         <v>5</v>
       </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F8" s="3">
         <v>46036</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G8" s="3">
         <v>46036</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9">
-      <c r="B8">
-        <f>B7+1</f>
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" t="s">
-        <v>111</v>
-      </c>
-      <c r="F8" s="3">
-        <v>46038</v>
       </c>
     </row>
     <row r="9" spans="2:9">
       <c r="B9">
         <f>B8+1</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>28</v>
+      </c>
+      <c r="E9" t="s">
+        <v>111</v>
       </c>
       <c r="F9" s="3">
-        <v>46039</v>
+        <v>46038</v>
       </c>
     </row>
     <row r="10" spans="2:9">
       <c r="B10">
         <f>B9+1</f>
-        <v>8</v>
-      </c>
-      <c r="C10" t="s">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F10" s="3">
-        <v>46036</v>
-      </c>
-      <c r="G10" s="3">
-        <v>46036</v>
+        <v>46039</v>
       </c>
     </row>
     <row r="11" spans="2:9">
       <c r="B11">
         <f>B10+1</f>
-        <v>9</v>
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>31</v>
+      </c>
+      <c r="F11" s="3">
+        <v>46036</v>
+      </c>
+      <c r="G11" s="3">
+        <v>46036</v>
       </c>
     </row>
     <row r="12" spans="2:9">
       <c r="B12">
         <f>B11+1</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="2:9">
       <c r="B13">
         <f>B12+1</f>
-        <v>11</v>
-      </c>
-      <c r="C13" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
-      </c>
-      <c r="F13" s="3">
-        <v>46036</v>
-      </c>
-      <c r="G13" s="3">
-        <v>46036</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="2:9">
       <c r="B14">
         <f>B13+1</f>
-        <v>12</v>
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>35</v>
+      </c>
+      <c r="F14" s="3">
+        <v>46036</v>
+      </c>
+      <c r="G14" s="3">
+        <v>46036</v>
       </c>
     </row>
     <row r="15" spans="2:9">
       <c r="B15">
         <f>B14+1</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="2:9">
       <c r="B16">
         <f>B15+1</f>
-        <v>14</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>101</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="2:9">
       <c r="B17">
         <f>B16+1</f>
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
       </c>
       <c r="D17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="2:9">
       <c r="B18">
         <f>B17+1</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="19" spans="2:9">
       <c r="B19">
         <f>B18+1</f>
-        <v>17</v>
-      </c>
-      <c r="C19" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="D19" t="s">
-        <v>104</v>
-      </c>
-      <c r="E19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" spans="2:9">
       <c r="B20">
         <f>B19+1</f>
-        <v>18</v>
+        <v>17</v>
+      </c>
+      <c r="C20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" t="s">
+        <v>104</v>
       </c>
       <c r="E20" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="2:9">
       <c r="B21">
         <f>B20+1</f>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="2:9">
       <c r="B22">
         <f>B21+1</f>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E22" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="2:9">
       <c r="B23">
         <f>B22+1</f>
-        <v>21</v>
-      </c>
-      <c r="C23" t="s">
-        <v>40</v>
+        <v>20</v>
+      </c>
+      <c r="E23" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="24" spans="2:9">
       <c r="B24">
         <f>B23+1</f>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C24" t="s">
-        <v>41</v>
-      </c>
-      <c r="D24" t="s">
-        <v>109</v>
-      </c>
-      <c r="F24" s="3">
-        <v>46037</v>
-      </c>
-      <c r="G24" s="3">
-        <v>46037</v>
-      </c>
-      <c r="H24" s="3">
-        <v>46037</v>
-      </c>
-      <c r="I24" s="3">
-        <v>46038</v>
+        <v>40</v>
       </c>
     </row>
     <row r="25" spans="2:9">
       <c r="B25">
         <f>B24+1</f>
+        <v>22</v>
+      </c>
+      <c r="C25" t="s">
+        <v>41</v>
+      </c>
+      <c r="D25" t="s">
+        <v>109</v>
+      </c>
+      <c r="F25" s="3">
+        <v>46037</v>
+      </c>
+      <c r="G25" s="3">
+        <v>46037</v>
+      </c>
+      <c r="H25" s="3">
+        <v>46037</v>
+      </c>
+      <c r="I25" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9">
+      <c r="B26">
+        <f>B25+1</f>
         <v>23</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D26" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add last updated date tracking for asset types
- Introduced a new map to store the last updated dates for each asset type.
- Updated the last updated dates whenever asset data is modified.
- Added a widget to display the last updated date or a message indicating no data.
- Improved the layout of the asset input row to include last updated information.
- Refactored code for better readability and consistency.
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{632B692D-0C42-43E4-A5A1-1E938525BED0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F21C417-80C5-4085-A022-7C7627B88994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="301">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1969,6 +1969,26 @@
     </rPh>
     <rPh sb="2" eb="4">
       <t>カンリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最後に現金残高や銀行口座残高が更新された日時を画面に表示するようにしてください。（今日はまだ更新していないということが分かるように）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最終更新日時表示</t>
+    <rPh sb="0" eb="2">
+      <t>サイシュウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウシン</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ニチジ</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ヒョウジ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -2640,10 +2660,19 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="8" spans="2:9">
+    <row r="8" spans="2:9" ht="75">
       <c r="B8">
         <f>B7+1</f>
         <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>300</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="F8" s="3">
+        <v>46039</v>
       </c>
     </row>
     <row r="9" spans="2:9">

</xml_diff>

<commit_message>
Refactor asset management and cash management pages; replace monthly closing report with financial report
- Updated `_buildLastUpdatedText` method in `asset_management_page.dart` for improved readability.
- Removed `cash_management_page.dart` as it is no longer needed.
- Replaced `monthly_closing_report_page.dart` with `financial_report_page.dart` in `cfo_office_page.dart`.
- Deleted `monthly_closing_report_page.dart` file.
- Added new `financial_report_page.dart` with comprehensive financial reporting features including daily, weekly, and monthly reports.
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F21C417-80C5-4085-A022-7C7627B88994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8312F23-19D1-4B68-A0E2-133FCD6800EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="304">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -1990,6 +1990,30 @@
     <rPh sb="6" eb="8">
       <t>ヒョウジ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>日時決算レポート</t>
+    <rPh sb="0" eb="2">
+      <t>ニチジ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ケッサン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>各ページにパンくずリストを表示できるようにしたい</t>
+    <rPh sb="0" eb="1">
+      <t>カク</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>ヒョウジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>トップページにサイトマップをつけたい</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2567,7 +2591,7 @@
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.25" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="6" max="7" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
@@ -2680,19 +2704,28 @@
         <f>B8+1</f>
         <v>7</v>
       </c>
-    </row>
-    <row r="10" spans="2:9">
+      <c r="C9" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" ht="56.25">
       <c r="B10">
         <f>B9+1</f>
         <v>8</v>
       </c>
+      <c r="C10" s="1" t="s">
+        <v>302</v>
+      </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
     </row>
-    <row r="11" spans="2:9">
+    <row r="11" spans="2:9" ht="37.5">
       <c r="B11">
         <f>B10+1</f>
         <v>9</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="12" spans="2:9">

</xml_diff>

<commit_message>
feat: Add Morning Briefing card to HomePage and implement overdue task migration in MorningBriefingPage
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8312F23-19D1-4B68-A0E2-133FCD6800EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CAB1D75-530C-4C69-B4A4-1CF08B5BA9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="306">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2014,6 +2014,20 @@
   </si>
   <si>
     <t>トップページにサイトマップをつけたい</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>依存をコントロールする機能</t>
+    <rPh sb="0" eb="2">
+      <t>イゾン</t>
+    </rPh>
+    <rPh sb="11" eb="13">
+      <t>キノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デイリーTODO機能を追加する場所は別の場所がよいかもしれません。DETAILED_DESIGN.mdを参照して検討してください。また、機能を追加したら、DETAILED_DESIGN.mdも更新してください。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2416,7 +2430,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46039</v>
+        <v>46041</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -2591,7 +2605,7 @@
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.25" customWidth="1"/>
+    <col min="3" max="3" width="27.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
     <col min="6" max="7" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
@@ -2599,7 +2613,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46039</v>
+        <v>46041</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -2616,14 +2630,19 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="2:9">
+    <row r="3" spans="2:9" ht="93.75">
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="3"/>
+      <c r="D3" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="F3" s="3">
+        <v>46041</v>
+      </c>
       <c r="G3" s="3"/>
     </row>
     <row r="4" spans="2:9">
@@ -2732,6 +2751,9 @@
       <c r="B12">
         <f>B11+1</f>
         <v>10</v>
+      </c>
+      <c r="C12" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="13" spans="2:9">
@@ -2801,7 +2823,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46039</v>
+        <v>46041</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -2964,7 +2986,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46039</v>
+        <v>46041</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -3163,7 +3185,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46039</v>
+        <v>46041</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -3916,7 +3938,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46039</v>
+        <v>46041</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
feat: Add edit functionality for todos in Morning Briefing page
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CAB1D75-530C-4C69-B4A4-1CF08B5BA9F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A12155E-C030-4507-8C07-0EFC83688387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="9" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,7 @@
     <sheet name="Gemini API reference" sheetId="12" r:id="rId13"/>
     <sheet name="Gemini Code Assist" sheetId="15" r:id="rId14"/>
     <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId15"/>
+    <sheet name="How to fix" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="313">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2028,6 +2029,34 @@
   </si>
   <si>
     <t>デイリーTODO機能を追加する場所は別の場所がよいかもしれません。DETAILED_DESIGN.mdを参照して検討してください。また、機能を追加したら、DETAILED_DESIGN.mdも更新してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>If you're anything like me, you think new years resolutions are stupid.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>もし君が僕みたいな人間なら、新年の抱負なんて馬鹿げてると思うだろう。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Because most people go about changing their lives in the completely wrong way.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ほとんどの人は、人生を変える方法を完全に間違ったやり方で進めているからだ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/thedankoe/status/2010751592346030461</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>How to fix your entire life in 1 day</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人生を1日で完全に変える方法</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3419,6 +3448,53 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595742A4-FD4B-4501-B5BA-63CBD2F36625}">
+  <dimension ref="C2:D7"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="3" max="3" width="35.75" customWidth="1"/>
+    <col min="4" max="4" width="48.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:4">
+      <c r="C2" s="2" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4">
+      <c r="C4" t="s">
+        <v>311</v>
+      </c>
+      <c r="D4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" ht="37.5">
+      <c r="C6" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" ht="37.5">
+      <c r="C7" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{2D572F08-FF13-4D66-AD9B-8810B4A82168}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EBDB197-A587-49EA-9FC4-8E4B6580D845}">
   <sheetPr>

</xml_diff>

<commit_message>
feat: Add recurrence feature for todos with options for daily, weekly, and monthly tasks
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A12155E-C030-4507-8C07-0EFC83688387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89C9D164-6BC1-458B-94F7-3567921ABEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="9" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="315">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2057,6 +2057,26 @@
   </si>
   <si>
     <t>人生を1日で完全に変える方法</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>flutter pub add confetti</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ユーザー数やサイト利用者を可視化できる機能</t>
+    <rPh sb="4" eb="5">
+      <t>スウ</t>
+    </rPh>
+    <rPh sb="9" eb="12">
+      <t>リヨウシャ</t>
+    </rPh>
+    <rPh sb="13" eb="16">
+      <t>カシカ</t>
+    </rPh>
+    <rPh sb="19" eb="21">
+      <t>キノウ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2785,10 +2805,13 @@
         <v>304</v>
       </c>
     </row>
-    <row r="13" spans="2:9">
+    <row r="13" spans="2:9" ht="37.5">
       <c r="B13">
         <f>B12+1</f>
         <v>11</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>314</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -3500,7 +3523,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="B3:D18"/>
+  <dimension ref="B3:D19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
@@ -3644,6 +3667,15 @@
       </c>
       <c r="C18" s="1" t="s">
         <v>247</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19">
+        <f>B18+1</f>
+        <v>16</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add UUID generation for messages in EmergencyMeetingPage and update message structure
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65713B9C-DF6C-47D1-8958-1C03782515A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F7DDF3-5579-481A-8347-7FA5644F3AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1161" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="540">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2081,12 +2081,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>{</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  "models": [</t>
-  </si>
-  <si>
     <t xml:space="preserve">    {</t>
   </si>
   <si>
@@ -2144,25 +2138,7 @@
     <t xml:space="preserve">      "thinking": true</t>
   </si>
   <si>
-    <t xml:space="preserve">      "name": "models/gemini-2.5-pro",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "version": "2.5",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "displayName": "Gemini 2.5 Pro",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "description": "Stable release (June 17th, 2025) of Gemini 2.5 Pro",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "name": "models/gemini-2.0-flash-exp",</t>
-  </si>
-  <si>
     <t xml:space="preserve">      "version": "2.0",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash Experimental",</t>
   </si>
   <si>
     <t xml:space="preserve">      "description": "Gemini 2.0 Flash Experimental",</t>
@@ -2779,6 +2755,38 @@
   </si>
   <si>
     <t>thinking</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>models/gemini-2.5-pro</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini 2.5 Pro</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Stable release (June 17th, 2025) of Gemini 2.5 Pro</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini 2.5 Pro 安定版リリース（2025年6月17日）</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">      "name": "models/gemini-2.0-flash-exp",</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>models/gemini-2.0-flash-exp</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash Experimental",</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini 2.0 Flash Experimental</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3729,13 +3737,13 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F96D129-34E8-4B10-A261-7AEE00EA03AD}">
-  <dimension ref="C2:Q746"/>
+  <dimension ref="C2:Q729"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="41.75" customWidth="1"/>
+    <col min="7" max="7" width="29.375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="47.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="47.75" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.25" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="29.125" bestFit="1" customWidth="1"/>
@@ -3745,60 +3753,57 @@
   <sheetData>
     <row r="2" spans="3:17">
       <c r="E2" t="s">
+        <v>510</v>
+      </c>
+      <c r="F2" t="s">
+        <v>512</v>
+      </c>
+      <c r="G2" t="s">
+        <v>513</v>
+      </c>
+      <c r="H2" t="s">
+        <v>515</v>
+      </c>
+      <c r="J2" t="s">
+        <v>517</v>
+      </c>
+      <c r="K2" t="s">
         <v>518</v>
       </c>
-      <c r="F2" t="s">
-        <v>520</v>
-      </c>
-      <c r="G2" t="s">
-        <v>521</v>
-      </c>
-      <c r="H2" t="s">
-        <v>523</v>
-      </c>
-      <c r="J2" t="s">
-        <v>525</v>
-      </c>
-      <c r="K2" t="s">
-        <v>526</v>
-      </c>
       <c r="L2" t="s">
+        <v>519</v>
+      </c>
+      <c r="M2" t="s">
         <v>527</v>
       </c>
-      <c r="M2" t="s">
-        <v>535</v>
-      </c>
       <c r="N2" t="s">
-        <v>536</v>
+        <v>528</v>
       </c>
       <c r="O2" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
       <c r="P2" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="Q2" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
     </row>
     <row r="3" spans="3:17" ht="37.5">
-      <c r="C3" t="s">
-        <v>315</v>
-      </c>
       <c r="E3" t="s">
-        <v>519</v>
+        <v>511</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>522</v>
+        <v>514</v>
       </c>
       <c r="H3" t="s">
+        <v>516</v>
+      </c>
+      <c r="I3" t="s">
         <v>524</v>
-      </c>
-      <c r="I3" t="s">
-        <v>532</v>
       </c>
       <c r="J3">
         <v>1024</v>
@@ -3807,27 +3812,24 @@
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>528</v>
+        <v>520</v>
       </c>
     </row>
     <row r="4" spans="3:17" ht="75">
-      <c r="C4" t="s">
-        <v>316</v>
-      </c>
       <c r="E4" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
       <c r="J4">
         <v>1048576</v>
@@ -3836,7 +3838,7 @@
         <v>65536</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>534</v>
+        <v>526</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -3854,104 +3856,147 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="3:17">
-      <c r="C5" t="s">
-        <v>317</v>
+    <row r="5" spans="3:17" ht="75">
+      <c r="E5" t="s">
+        <v>532</v>
+      </c>
+      <c r="F5">
+        <v>2.5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>533</v>
+      </c>
+      <c r="H5" t="s">
+        <v>534</v>
+      </c>
+      <c r="I5" t="s">
+        <v>535</v>
+      </c>
+      <c r="J5">
+        <v>1048576</v>
+      </c>
+      <c r="K5">
+        <v>65536</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+      <c r="N5">
+        <v>0.95</v>
+      </c>
+      <c r="O5">
+        <v>64</v>
+      </c>
+      <c r="P5">
+        <v>2</v>
+      </c>
+      <c r="Q5" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="3:17">
-      <c r="C6" t="s">
-        <v>336</v>
-      </c>
+      <c r="E6" t="s">
+        <v>537</v>
+      </c>
+      <c r="F6">
+        <v>2</v>
+      </c>
+      <c r="G6" t="s">
+        <v>539</v>
+      </c>
+      <c r="L6" s="1"/>
     </row>
     <row r="7" spans="3:17">
       <c r="C7" t="s">
-        <v>337</v>
+        <v>315</v>
       </c>
     </row>
     <row r="8" spans="3:17">
       <c r="C8" t="s">
-        <v>338</v>
+        <v>536</v>
       </c>
     </row>
     <row r="9" spans="3:17">
       <c r="C9" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
     <row r="10" spans="3:17">
       <c r="C10" t="s">
-        <v>324</v>
+        <v>538</v>
       </c>
     </row>
     <row r="11" spans="3:17">
       <c r="C11" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="12" spans="3:17">
       <c r="C12" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="3:17">
       <c r="C13" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
     </row>
     <row r="14" spans="3:17">
       <c r="C14" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="15" spans="3:17">
       <c r="C15" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="16" spans="3:17">
       <c r="C16" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="19" spans="3:3">
       <c r="C19" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="20" spans="3:3">
       <c r="C20" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
     </row>
     <row r="22" spans="3:3">
       <c r="C22" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="25" spans="3:3">
@@ -3961,802 +4006,802 @@
     </row>
     <row r="26" spans="3:3">
       <c r="C26" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" spans="3:3">
       <c r="C27" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="28" spans="3:3">
       <c r="C28" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="29" spans="3:3">
       <c r="C29" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="30" spans="3:3">
       <c r="C30" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
     </row>
     <row r="31" spans="3:3">
       <c r="C31" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="32" spans="3:3">
       <c r="C32" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="33" spans="3:3">
       <c r="C33" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="34" spans="3:3">
       <c r="C34" t="s">
-        <v>345</v>
+        <v>326</v>
       </c>
     </row>
     <row r="35" spans="3:3">
       <c r="C35" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="36" spans="3:3">
       <c r="C36" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="38" spans="3:3">
       <c r="C38" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
     </row>
     <row r="40" spans="3:3">
       <c r="C40" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="42" spans="3:3">
       <c r="C42" t="s">
-        <v>348</v>
+        <v>315</v>
       </c>
     </row>
     <row r="43" spans="3:3">
       <c r="C43" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="44" spans="3:3">
       <c r="C44" t="s">
-        <v>349</v>
+        <v>334</v>
       </c>
     </row>
     <row r="45" spans="3:3">
       <c r="C45" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
     </row>
     <row r="46" spans="3:3">
       <c r="C46" t="s">
-        <v>324</v>
+        <v>345</v>
       </c>
     </row>
     <row r="47" spans="3:3">
       <c r="C47" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
     </row>
     <row r="48" spans="3:3">
       <c r="C48" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
     </row>
     <row r="49" spans="3:3">
       <c r="C49" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="50" spans="3:3">
       <c r="C50" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="51" spans="3:3">
       <c r="C51" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="52" spans="3:3">
       <c r="C52" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="53" spans="3:3">
       <c r="C53" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="54" spans="3:3">
       <c r="C54" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="55" spans="3:3">
       <c r="C55" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="56" spans="3:3">
       <c r="C56" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="57" spans="3:3">
       <c r="C57" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
     </row>
     <row r="58" spans="3:3">
       <c r="C58" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
     </row>
     <row r="59" spans="3:3">
       <c r="C59" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="60" spans="3:3">
       <c r="C60" t="s">
-        <v>351</v>
+        <v>315</v>
       </c>
     </row>
     <row r="61" spans="3:3">
       <c r="C61" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="62" spans="3:3">
       <c r="C62" t="s">
-        <v>352</v>
+        <v>334</v>
       </c>
     </row>
     <row r="63" spans="3:3">
       <c r="C63" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
     </row>
     <row r="64" spans="3:3">
       <c r="C64" t="s">
-        <v>324</v>
+        <v>348</v>
       </c>
     </row>
     <row r="65" spans="3:3">
       <c r="C65" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
     </row>
     <row r="66" spans="3:3">
       <c r="C66" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
     </row>
     <row r="67" spans="3:3">
       <c r="C67" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="68" spans="3:3">
       <c r="C68" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="69" spans="3:3">
       <c r="C69" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="70" spans="3:3">
       <c r="C70" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
     </row>
     <row r="71" spans="3:3">
       <c r="C71" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="72" spans="3:3">
       <c r="C72" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="73" spans="3:3">
       <c r="C73" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="74" spans="3:3">
       <c r="C74" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
     </row>
     <row r="75" spans="3:3">
       <c r="C75" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
     </row>
     <row r="76" spans="3:3">
       <c r="C76" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="77" spans="3:3">
       <c r="C77" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="78" spans="3:3">
       <c r="C78" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
     </row>
     <row r="79" spans="3:3">
       <c r="C79" t="s">
-        <v>341</v>
+        <v>334</v>
       </c>
     </row>
     <row r="80" spans="3:3">
       <c r="C80" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
     </row>
     <row r="81" spans="3:3">
       <c r="C81" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
     </row>
     <row r="82" spans="3:3">
       <c r="C82" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="83" spans="3:3">
       <c r="C83" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
     </row>
     <row r="84" spans="3:3">
       <c r="C84" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="85" spans="3:3">
       <c r="C85" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="86" spans="3:3">
       <c r="C86" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="87" spans="3:3">
       <c r="C87" t="s">
-        <v>345</v>
+        <v>326</v>
       </c>
     </row>
     <row r="88" spans="3:3">
       <c r="C88" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="89" spans="3:3">
       <c r="C89" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="90" spans="3:3">
       <c r="C90" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="91" spans="3:3">
       <c r="C91" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="92" spans="3:3">
       <c r="C92" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
     </row>
     <row r="93" spans="3:3">
       <c r="C93" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
     </row>
     <row r="94" spans="3:3">
       <c r="C94" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="95" spans="3:3">
       <c r="C95" t="s">
-        <v>357</v>
+        <v>315</v>
       </c>
     </row>
     <row r="96" spans="3:3">
       <c r="C96" t="s">
-        <v>341</v>
+        <v>352</v>
       </c>
     </row>
     <row r="97" spans="3:3">
       <c r="C97" t="s">
-        <v>358</v>
+        <v>334</v>
       </c>
     </row>
     <row r="98" spans="3:3">
       <c r="C98" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
     </row>
     <row r="99" spans="3:3">
       <c r="C99" t="s">
-        <v>324</v>
+        <v>354</v>
       </c>
     </row>
     <row r="100" spans="3:3">
       <c r="C100" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
     </row>
     <row r="101" spans="3:3">
       <c r="C101" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
     </row>
     <row r="102" spans="3:3">
       <c r="C102" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="103" spans="3:3">
       <c r="C103" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="104" spans="3:3">
       <c r="C104" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="105" spans="3:3">
       <c r="C105" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="106" spans="3:3">
       <c r="C106" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="107" spans="3:3">
       <c r="C107" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="108" spans="3:3">
       <c r="C108" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="109" spans="3:3">
       <c r="C109" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="110" spans="3:3">
       <c r="C110" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
     </row>
     <row r="111" spans="3:3">
       <c r="C111" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
     </row>
     <row r="112" spans="3:3">
       <c r="C112" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="113" spans="3:3">
       <c r="C113" t="s">
-        <v>360</v>
+        <v>315</v>
       </c>
     </row>
     <row r="114" spans="3:3">
       <c r="C114" t="s">
-        <v>341</v>
+        <v>355</v>
       </c>
     </row>
     <row r="115" spans="3:3">
       <c r="C115" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="116" spans="3:3">
       <c r="C116" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="117" spans="3:3">
       <c r="C117" t="s">
-        <v>324</v>
+        <v>358</v>
       </c>
     </row>
     <row r="118" spans="3:3">
       <c r="C118" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
     </row>
     <row r="119" spans="3:3">
       <c r="C119" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
     </row>
     <row r="120" spans="3:3">
       <c r="C120" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="121" spans="3:3">
       <c r="C121" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="122" spans="3:3">
       <c r="C122" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="123" spans="3:3">
       <c r="C123" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="124" spans="3:3">
       <c r="C124" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="125" spans="3:3">
       <c r="C125" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="126" spans="3:3">
       <c r="C126" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="127" spans="3:3">
       <c r="C127" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="128" spans="3:3">
       <c r="C128" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
     </row>
     <row r="129" spans="3:3">
       <c r="C129" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
     </row>
     <row r="130" spans="3:3">
       <c r="C130" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="131" spans="3:3">
       <c r="C131" t="s">
-        <v>363</v>
+        <v>315</v>
       </c>
     </row>
     <row r="132" spans="3:3">
       <c r="C132" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="133" spans="3:3">
       <c r="C133" t="s">
-        <v>365</v>
+        <v>356</v>
       </c>
     </row>
     <row r="134" spans="3:3">
       <c r="C134" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
     </row>
     <row r="135" spans="3:3">
       <c r="C135" t="s">
-        <v>324</v>
+        <v>358</v>
       </c>
     </row>
     <row r="136" spans="3:3">
       <c r="C136" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
     </row>
     <row r="137" spans="3:3">
       <c r="C137" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
     </row>
     <row r="138" spans="3:3">
       <c r="C138" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="139" spans="3:3">
       <c r="C139" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="140" spans="3:3">
       <c r="C140" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="141" spans="3:3">
       <c r="C141" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="142" spans="3:3">
       <c r="C142" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="143" spans="3:3">
       <c r="C143" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="144" spans="3:3">
       <c r="C144" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="145" spans="3:3">
       <c r="C145" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="146" spans="3:3">
       <c r="C146" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
     </row>
     <row r="147" spans="3:3">
       <c r="C147" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
     </row>
     <row r="148" spans="3:3">
       <c r="C148" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="149" spans="3:3">
       <c r="C149" t="s">
-        <v>367</v>
+        <v>315</v>
       </c>
     </row>
     <row r="150" spans="3:3">
       <c r="C150" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
     </row>
     <row r="151" spans="3:3">
       <c r="C151" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
     </row>
     <row r="152" spans="3:3">
       <c r="C152" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
     </row>
     <row r="153" spans="3:3">
       <c r="C153" t="s">
-        <v>324</v>
+        <v>364</v>
       </c>
     </row>
     <row r="154" spans="3:3">
       <c r="C154" t="s">
-        <v>344</v>
+        <v>322</v>
       </c>
     </row>
     <row r="155" spans="3:3">
       <c r="C155" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="156" spans="3:3">
       <c r="C156" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="157" spans="3:3">
       <c r="C157" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="158" spans="3:3">
       <c r="C158" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="159" spans="3:3">
       <c r="C159" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="160" spans="3:3">
       <c r="C160" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="161" spans="3:3">
       <c r="C161" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="162" spans="3:3">
       <c r="C162" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="163" spans="3:3">
       <c r="C163" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="164" spans="3:3">
       <c r="C164" t="s">
-        <v>347</v>
+        <v>331</v>
       </c>
     </row>
     <row r="165" spans="3:3">
       <c r="C165" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="166" spans="3:3">
       <c r="C166" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="167" spans="3:3">
       <c r="C167" t="s">
-        <v>369</v>
+        <v>321</v>
       </c>
     </row>
     <row r="168" spans="3:3">
       <c r="C168" t="s">
-        <v>370</v>
+        <v>315</v>
       </c>
     </row>
     <row r="169" spans="3:3">
       <c r="C169" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
     </row>
     <row r="170" spans="3:3">
       <c r="C170" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
     </row>
     <row r="171" spans="3:3">
       <c r="C171" t="s">
-        <v>324</v>
+        <v>367</v>
       </c>
     </row>
     <row r="172" spans="3:3">
       <c r="C172" t="s">
-        <v>325</v>
+        <v>368</v>
       </c>
     </row>
     <row r="173" spans="3:3">
       <c r="C173" t="s">
-        <v>321</v>
+        <v>369</v>
       </c>
     </row>
     <row r="174" spans="3:3">
       <c r="C174" t="s">
-        <v>326</v>
+        <v>370</v>
       </c>
     </row>
     <row r="175" spans="3:3">
       <c r="C175" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="176" spans="3:3">
       <c r="C176" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="177" spans="3:3">
       <c r="C177" t="s">
-        <v>329</v>
+        <v>371</v>
       </c>
     </row>
     <row r="178" spans="3:3">
       <c r="C178" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="179" spans="3:3">
       <c r="C179" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="180" spans="3:3">
       <c r="C180" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="181" spans="3:3">
       <c r="C181" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="182" spans="3:3">
       <c r="C182" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
     <row r="183" spans="3:3">
       <c r="C183" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="184" spans="3:3">
       <c r="C184" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
     </row>
     <row r="185" spans="3:3">
       <c r="C185" t="s">
-        <v>317</v>
+        <v>372</v>
       </c>
     </row>
     <row r="186" spans="3:3">
@@ -4776,112 +4821,112 @@
     </row>
     <row r="189" spans="3:3">
       <c r="C189" t="s">
-        <v>376</v>
+        <v>369</v>
       </c>
     </row>
     <row r="190" spans="3:3">
       <c r="C190" t="s">
-        <v>377</v>
+        <v>370</v>
       </c>
     </row>
     <row r="191" spans="3:3">
       <c r="C191" t="s">
-        <v>378</v>
+        <v>319</v>
       </c>
     </row>
     <row r="192" spans="3:3">
       <c r="C192" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="193" spans="3:3">
       <c r="C193" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="194" spans="3:3">
       <c r="C194" t="s">
-        <v>379</v>
+        <v>327</v>
       </c>
     </row>
     <row r="195" spans="3:3">
       <c r="C195" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="196" spans="3:3">
       <c r="C196" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="197" spans="3:3">
       <c r="C197" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="198" spans="3:3">
       <c r="C198" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="199" spans="3:3">
       <c r="C199" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
     </row>
     <row r="200" spans="3:3">
       <c r="C200" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="201" spans="3:3">
       <c r="C201" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="202" spans="3:3">
       <c r="C202" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
     </row>
     <row r="203" spans="3:3">
       <c r="C203" t="s">
-        <v>381</v>
+        <v>316</v>
       </c>
     </row>
     <row r="204" spans="3:3">
       <c r="C204" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
     </row>
     <row r="205" spans="3:3">
       <c r="C205" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
     </row>
     <row r="206" spans="3:3">
       <c r="C206" t="s">
-        <v>377</v>
+        <v>336</v>
       </c>
     </row>
     <row r="207" spans="3:3">
       <c r="C207" t="s">
-        <v>378</v>
+        <v>319</v>
       </c>
     </row>
     <row r="208" spans="3:3">
       <c r="C208" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="209" spans="3:3">
       <c r="C209" t="s">
-        <v>327</v>
+        <v>379</v>
       </c>
     </row>
     <row r="210" spans="3:3">
       <c r="C210" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="211" spans="3:3">
@@ -4896,227 +4941,227 @@
     </row>
     <row r="213" spans="3:3">
       <c r="C213" t="s">
-        <v>331</v>
+        <v>380</v>
       </c>
     </row>
     <row r="214" spans="3:3">
       <c r="C214" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
     </row>
     <row r="215" spans="3:3">
       <c r="C215" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
     </row>
     <row r="216" spans="3:3">
       <c r="C216" t="s">
-        <v>347</v>
+        <v>381</v>
       </c>
     </row>
     <row r="217" spans="3:3">
       <c r="C217" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="218" spans="3:3">
       <c r="C218" t="s">
-        <v>317</v>
+        <v>382</v>
       </c>
     </row>
     <row r="219" spans="3:3">
       <c r="C219" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="220" spans="3:3">
       <c r="C220" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
     </row>
     <row r="221" spans="3:3">
       <c r="C221" t="s">
-        <v>385</v>
+        <v>319</v>
       </c>
     </row>
     <row r="222" spans="3:3">
       <c r="C222" t="s">
-        <v>386</v>
+        <v>324</v>
       </c>
     </row>
     <row r="223" spans="3:3">
       <c r="C223" t="s">
-        <v>344</v>
+        <v>379</v>
       </c>
     </row>
     <row r="224" spans="3:3">
       <c r="C224" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="225" spans="3:3">
       <c r="C225" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="226" spans="3:3">
       <c r="C226" t="s">
-        <v>387</v>
+        <v>330</v>
       </c>
     </row>
     <row r="227" spans="3:3">
       <c r="C227" t="s">
-        <v>330</v>
+        <v>380</v>
       </c>
     </row>
     <row r="228" spans="3:3">
       <c r="C228" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
     </row>
     <row r="229" spans="3:3">
       <c r="C229" t="s">
-        <v>332</v>
+        <v>315</v>
       </c>
     </row>
     <row r="230" spans="3:3">
       <c r="C230" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
     </row>
     <row r="231" spans="3:3">
       <c r="C231" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="232" spans="3:3">
       <c r="C232" t="s">
-        <v>317</v>
+        <v>384</v>
       </c>
     </row>
     <row r="233" spans="3:3">
       <c r="C233" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
     </row>
     <row r="234" spans="3:3">
       <c r="C234" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
     </row>
     <row r="235" spans="3:3">
       <c r="C235" t="s">
-        <v>390</v>
+        <v>319</v>
       </c>
     </row>
     <row r="236" spans="3:3">
       <c r="C236" t="s">
-        <v>386</v>
+        <v>324</v>
       </c>
     </row>
     <row r="237" spans="3:3">
       <c r="C237" t="s">
-        <v>344</v>
+        <v>379</v>
       </c>
     </row>
     <row r="238" spans="3:3">
       <c r="C238" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="239" spans="3:3">
       <c r="C239" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="240" spans="3:3">
       <c r="C240" t="s">
-        <v>387</v>
+        <v>330</v>
       </c>
     </row>
     <row r="241" spans="3:3">
       <c r="C241" t="s">
-        <v>330</v>
+        <v>380</v>
       </c>
     </row>
     <row r="242" spans="3:3">
       <c r="C242" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
     </row>
     <row r="243" spans="3:3">
       <c r="C243" t="s">
-        <v>332</v>
+        <v>315</v>
       </c>
     </row>
     <row r="244" spans="3:3">
       <c r="C244" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
     </row>
     <row r="245" spans="3:3">
       <c r="C245" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="246" spans="3:3">
       <c r="C246" t="s">
-        <v>317</v>
+        <v>386</v>
       </c>
     </row>
     <row r="247" spans="3:3">
       <c r="C247" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
     </row>
     <row r="248" spans="3:3">
       <c r="C248" t="s">
-        <v>318</v>
+        <v>336</v>
       </c>
     </row>
     <row r="249" spans="3:3">
       <c r="C249" t="s">
-        <v>392</v>
+        <v>319</v>
       </c>
     </row>
     <row r="250" spans="3:3">
       <c r="C250" t="s">
-        <v>386</v>
+        <v>324</v>
       </c>
     </row>
     <row r="251" spans="3:3">
       <c r="C251" t="s">
-        <v>344</v>
+        <v>379</v>
       </c>
     </row>
     <row r="252" spans="3:3">
       <c r="C252" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="253" spans="3:3">
       <c r="C253" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="254" spans="3:3">
       <c r="C254" t="s">
-        <v>387</v>
+        <v>330</v>
       </c>
     </row>
     <row r="255" spans="3:3">
       <c r="C255" t="s">
-        <v>330</v>
+        <v>380</v>
       </c>
     </row>
     <row r="256" spans="3:3">
       <c r="C256" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
     </row>
     <row r="257" spans="3:3">
       <c r="C257" t="s">
-        <v>332</v>
+        <v>315</v>
       </c>
     </row>
     <row r="258" spans="3:3">
@@ -5126,182 +5171,182 @@
     </row>
     <row r="259" spans="3:3">
       <c r="C259" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="260" spans="3:3">
       <c r="C260" t="s">
-        <v>317</v>
+        <v>389</v>
       </c>
     </row>
     <row r="261" spans="3:3">
       <c r="C261" t="s">
-        <v>393</v>
+        <v>369</v>
       </c>
     </row>
     <row r="262" spans="3:3">
       <c r="C262" t="s">
-        <v>318</v>
+        <v>390</v>
       </c>
     </row>
     <row r="263" spans="3:3">
       <c r="C263" t="s">
-        <v>394</v>
+        <v>319</v>
       </c>
     </row>
     <row r="264" spans="3:3">
       <c r="C264" t="s">
-        <v>395</v>
+        <v>324</v>
       </c>
     </row>
     <row r="265" spans="3:3">
       <c r="C265" t="s">
-        <v>344</v>
+        <v>379</v>
       </c>
     </row>
     <row r="266" spans="3:3">
       <c r="C266" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="267" spans="3:3">
       <c r="C267" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="268" spans="3:3">
       <c r="C268" t="s">
-        <v>387</v>
+        <v>330</v>
       </c>
     </row>
     <row r="269" spans="3:3">
       <c r="C269" t="s">
-        <v>330</v>
+        <v>380</v>
       </c>
     </row>
     <row r="270" spans="3:3">
       <c r="C270" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
     </row>
     <row r="271" spans="3:3">
       <c r="C271" t="s">
-        <v>332</v>
+        <v>315</v>
       </c>
     </row>
     <row r="272" spans="3:3">
       <c r="C272" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
     </row>
     <row r="273" spans="3:3">
       <c r="C273" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="274" spans="3:3">
       <c r="C274" t="s">
-        <v>317</v>
+        <v>392</v>
       </c>
     </row>
     <row r="275" spans="3:3">
       <c r="C275" t="s">
-        <v>396</v>
+        <v>369</v>
       </c>
     </row>
     <row r="276" spans="3:3">
       <c r="C276" t="s">
-        <v>318</v>
+        <v>390</v>
       </c>
     </row>
     <row r="277" spans="3:3">
       <c r="C277" t="s">
-        <v>397</v>
+        <v>319</v>
       </c>
     </row>
     <row r="278" spans="3:3">
       <c r="C278" t="s">
-        <v>377</v>
+        <v>324</v>
       </c>
     </row>
     <row r="279" spans="3:3">
       <c r="C279" t="s">
-        <v>398</v>
+        <v>379</v>
       </c>
     </row>
     <row r="280" spans="3:3">
       <c r="C280" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="281" spans="3:3">
       <c r="C281" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
     </row>
     <row r="282" spans="3:3">
       <c r="C282" t="s">
-        <v>387</v>
+        <v>330</v>
       </c>
     </row>
     <row r="283" spans="3:3">
       <c r="C283" t="s">
-        <v>330</v>
+        <v>380</v>
       </c>
     </row>
     <row r="284" spans="3:3">
       <c r="C284" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
     </row>
     <row r="285" spans="3:3">
       <c r="C285" t="s">
-        <v>332</v>
+        <v>315</v>
       </c>
     </row>
     <row r="286" spans="3:3">
       <c r="C286" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
     <row r="287" spans="3:3">
       <c r="C287" t="s">
-        <v>323</v>
+        <v>394</v>
       </c>
     </row>
     <row r="288" spans="3:3">
       <c r="C288" t="s">
-        <v>317</v>
+        <v>395</v>
       </c>
     </row>
     <row r="289" spans="3:3">
       <c r="C289" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="290" spans="3:3">
       <c r="C290" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="291" spans="3:3">
       <c r="C291" t="s">
-        <v>400</v>
+        <v>323</v>
       </c>
     </row>
     <row r="292" spans="3:3">
       <c r="C292" t="s">
-        <v>377</v>
+        <v>319</v>
       </c>
     </row>
     <row r="293" spans="3:3">
       <c r="C293" t="s">
-        <v>398</v>
+        <v>324</v>
       </c>
     </row>
     <row r="294" spans="3:3">
       <c r="C294" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="295" spans="3:3">
@@ -5311,1422 +5356,1422 @@
     </row>
     <row r="296" spans="3:3">
       <c r="C296" t="s">
-        <v>387</v>
+        <v>327</v>
       </c>
     </row>
     <row r="297" spans="3:3">
       <c r="C297" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="298" spans="3:3">
       <c r="C298" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="299" spans="3:3">
       <c r="C299" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="300" spans="3:3">
       <c r="C300" t="s">
-        <v>388</v>
+        <v>331</v>
       </c>
     </row>
     <row r="301" spans="3:3">
       <c r="C301" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="302" spans="3:3">
       <c r="C302" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="303" spans="3:3">
       <c r="C303" t="s">
-        <v>401</v>
+        <v>321</v>
       </c>
     </row>
     <row r="304" spans="3:3">
       <c r="C304" t="s">
-        <v>402</v>
+        <v>315</v>
       </c>
     </row>
     <row r="305" spans="3:3">
       <c r="C305" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
     </row>
     <row r="306" spans="3:3">
       <c r="C306" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="307" spans="3:3">
       <c r="C307" t="s">
-        <v>324</v>
+        <v>399</v>
       </c>
     </row>
     <row r="308" spans="3:3">
       <c r="C308" t="s">
-        <v>325</v>
+        <v>400</v>
       </c>
     </row>
     <row r="309" spans="3:3">
       <c r="C309" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="310" spans="3:3">
       <c r="C310" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="311" spans="3:3">
       <c r="C311" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="312" spans="3:3">
       <c r="C312" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="313" spans="3:3">
       <c r="C313" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="314" spans="3:3">
       <c r="C314" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="315" spans="3:3">
       <c r="C315" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="316" spans="3:3">
       <c r="C316" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="317" spans="3:3">
       <c r="C317" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="318" spans="3:3">
       <c r="C318" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="319" spans="3:3">
       <c r="C319" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="320" spans="3:3">
       <c r="C320" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="321" spans="3:3">
       <c r="C321" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="322" spans="3:3">
       <c r="C322" t="s">
-        <v>405</v>
+        <v>321</v>
       </c>
     </row>
     <row r="323" spans="3:3">
       <c r="C323" t="s">
-        <v>406</v>
+        <v>315</v>
       </c>
     </row>
     <row r="324" spans="3:3">
       <c r="C324" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
     </row>
     <row r="325" spans="3:3">
       <c r="C325" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="326" spans="3:3">
       <c r="C326" t="s">
-        <v>324</v>
+        <v>403</v>
       </c>
     </row>
     <row r="327" spans="3:3">
       <c r="C327" t="s">
-        <v>325</v>
+        <v>404</v>
       </c>
     </row>
     <row r="328" spans="3:3">
       <c r="C328" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="329" spans="3:3">
       <c r="C329" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="330" spans="3:3">
       <c r="C330" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="331" spans="3:3">
       <c r="C331" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="332" spans="3:3">
       <c r="C332" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="333" spans="3:3">
       <c r="C333" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="334" spans="3:3">
       <c r="C334" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="335" spans="3:3">
       <c r="C335" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="336" spans="3:3">
       <c r="C336" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="337" spans="3:3">
       <c r="C337" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="338" spans="3:3">
       <c r="C338" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="339" spans="3:3">
       <c r="C339" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="340" spans="3:3">
       <c r="C340" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="341" spans="3:3">
       <c r="C341" t="s">
-        <v>409</v>
+        <v>321</v>
       </c>
     </row>
     <row r="342" spans="3:3">
       <c r="C342" t="s">
-        <v>410</v>
+        <v>315</v>
       </c>
     </row>
     <row r="343" spans="3:3">
       <c r="C343" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
     </row>
     <row r="344" spans="3:3">
       <c r="C344" t="s">
-        <v>412</v>
+        <v>316</v>
       </c>
     </row>
     <row r="345" spans="3:3">
       <c r="C345" t="s">
-        <v>324</v>
+        <v>406</v>
       </c>
     </row>
     <row r="346" spans="3:3">
       <c r="C346" t="s">
-        <v>325</v>
+        <v>407</v>
       </c>
     </row>
     <row r="347" spans="3:3">
       <c r="C347" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="348" spans="3:3">
       <c r="C348" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="349" spans="3:3">
       <c r="C349" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="350" spans="3:3">
       <c r="C350" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="351" spans="3:3">
       <c r="C351" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="352" spans="3:3">
       <c r="C352" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="353" spans="3:3">
       <c r="C353" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="354" spans="3:3">
       <c r="C354" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="355" spans="3:3">
       <c r="C355" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="356" spans="3:3">
       <c r="C356" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="357" spans="3:3">
       <c r="C357" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="358" spans="3:3">
       <c r="C358" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="359" spans="3:3">
       <c r="C359" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="360" spans="3:3">
       <c r="C360" t="s">
-        <v>413</v>
+        <v>321</v>
       </c>
     </row>
     <row r="361" spans="3:3">
       <c r="C361" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="362" spans="3:3">
       <c r="C362" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
     </row>
     <row r="363" spans="3:3">
       <c r="C363" t="s">
-        <v>415</v>
+        <v>334</v>
       </c>
     </row>
     <row r="364" spans="3:3">
       <c r="C364" t="s">
-        <v>324</v>
+        <v>409</v>
       </c>
     </row>
     <row r="365" spans="3:3">
       <c r="C365" t="s">
-        <v>325</v>
+        <v>410</v>
       </c>
     </row>
     <row r="366" spans="3:3">
       <c r="C366" t="s">
-        <v>321</v>
+        <v>378</v>
       </c>
     </row>
     <row r="367" spans="3:3">
       <c r="C367" t="s">
-        <v>326</v>
+        <v>411</v>
       </c>
     </row>
     <row r="368" spans="3:3">
       <c r="C368" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="369" spans="3:3">
       <c r="C369" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="370" spans="3:3">
       <c r="C370" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="371" spans="3:3">
       <c r="C371" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="372" spans="3:3">
       <c r="C372" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="373" spans="3:3">
       <c r="C373" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="374" spans="3:3">
       <c r="C374" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="375" spans="3:3">
       <c r="C375" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
     </row>
     <row r="376" spans="3:3">
       <c r="C376" t="s">
-        <v>335</v>
+        <v>412</v>
       </c>
     </row>
     <row r="377" spans="3:3">
       <c r="C377" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="378" spans="3:3">
       <c r="C378" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="379" spans="3:3">
       <c r="C379" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
     </row>
     <row r="380" spans="3:3">
       <c r="C380" t="s">
-        <v>341</v>
+        <v>414</v>
       </c>
     </row>
     <row r="381" spans="3:3">
       <c r="C381" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="382" spans="3:3">
       <c r="C382" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
     </row>
     <row r="383" spans="3:3">
       <c r="C383" t="s">
-        <v>386</v>
+        <v>322</v>
       </c>
     </row>
     <row r="384" spans="3:3">
       <c r="C384" t="s">
-        <v>419</v>
+        <v>323</v>
       </c>
     </row>
     <row r="385" spans="3:3">
       <c r="C385" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="386" spans="3:3">
       <c r="C386" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="387" spans="3:3">
       <c r="C387" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="388" spans="3:3">
       <c r="C388" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="389" spans="3:3">
       <c r="C389" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="390" spans="3:3">
       <c r="C390" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="391" spans="3:3">
       <c r="C391" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="392" spans="3:3">
       <c r="C392" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="393" spans="3:3">
       <c r="C393" t="s">
-        <v>420</v>
+        <v>331</v>
       </c>
     </row>
     <row r="394" spans="3:3">
       <c r="C394" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="395" spans="3:3">
       <c r="C395" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="396" spans="3:3">
       <c r="C396" t="s">
-        <v>421</v>
+        <v>321</v>
       </c>
     </row>
     <row r="397" spans="3:3">
       <c r="C397" t="s">
-        <v>422</v>
+        <v>315</v>
       </c>
     </row>
     <row r="398" spans="3:3">
       <c r="C398" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
     </row>
     <row r="399" spans="3:3">
       <c r="C399" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
     </row>
     <row r="400" spans="3:3">
       <c r="C400" t="s">
-        <v>324</v>
+        <v>419</v>
       </c>
     </row>
     <row r="401" spans="3:3">
       <c r="C401" t="s">
-        <v>325</v>
+        <v>420</v>
       </c>
     </row>
     <row r="402" spans="3:3">
       <c r="C402" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="403" spans="3:3">
       <c r="C403" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="404" spans="3:3">
       <c r="C404" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="405" spans="3:3">
       <c r="C405" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="406" spans="3:3">
       <c r="C406" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="407" spans="3:3">
       <c r="C407" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="408" spans="3:3">
       <c r="C408" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="409" spans="3:3">
       <c r="C409" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="410" spans="3:3">
       <c r="C410" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="411" spans="3:3">
       <c r="C411" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="412" spans="3:3">
       <c r="C412" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="413" spans="3:3">
       <c r="C413" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="414" spans="3:3">
       <c r="C414" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="415" spans="3:3">
       <c r="C415" t="s">
-        <v>425</v>
+        <v>321</v>
       </c>
     </row>
     <row r="416" spans="3:3">
       <c r="C416" t="s">
-        <v>426</v>
+        <v>315</v>
       </c>
     </row>
     <row r="417" spans="3:3">
       <c r="C417" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
     </row>
     <row r="418" spans="3:3">
       <c r="C418" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
     </row>
     <row r="419" spans="3:3">
       <c r="C419" t="s">
-        <v>324</v>
+        <v>423</v>
       </c>
     </row>
     <row r="420" spans="3:3">
       <c r="C420" t="s">
-        <v>325</v>
+        <v>424</v>
       </c>
     </row>
     <row r="421" spans="3:3">
       <c r="C421" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="422" spans="3:3">
       <c r="C422" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="423" spans="3:3">
       <c r="C423" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="424" spans="3:3">
       <c r="C424" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="425" spans="3:3">
       <c r="C425" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="426" spans="3:3">
       <c r="C426" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="427" spans="3:3">
       <c r="C427" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="428" spans="3:3">
       <c r="C428" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="429" spans="3:3">
       <c r="C429" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="430" spans="3:3">
       <c r="C430" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="431" spans="3:3">
       <c r="C431" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="432" spans="3:3">
       <c r="C432" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="433" spans="3:3">
       <c r="C433" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="434" spans="3:3">
       <c r="C434" t="s">
-        <v>429</v>
+        <v>321</v>
       </c>
     </row>
     <row r="435" spans="3:3">
       <c r="C435" t="s">
-        <v>430</v>
+        <v>315</v>
       </c>
     </row>
     <row r="436" spans="3:3">
       <c r="C436" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
     </row>
     <row r="437" spans="3:3">
       <c r="C437" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
     </row>
     <row r="438" spans="3:3">
       <c r="C438" t="s">
-        <v>324</v>
+        <v>427</v>
       </c>
     </row>
     <row r="439" spans="3:3">
       <c r="C439" t="s">
-        <v>325</v>
+        <v>428</v>
       </c>
     </row>
     <row r="440" spans="3:3">
       <c r="C440" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="441" spans="3:3">
       <c r="C441" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="442" spans="3:3">
       <c r="C442" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="443" spans="3:3">
       <c r="C443" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="444" spans="3:3">
       <c r="C444" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="445" spans="3:3">
       <c r="C445" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="446" spans="3:3">
       <c r="C446" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="447" spans="3:3">
       <c r="C447" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="448" spans="3:3">
       <c r="C448" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="449" spans="3:3">
       <c r="C449" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
     </row>
     <row r="450" spans="3:3">
       <c r="C450" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="451" spans="3:3">
       <c r="C451" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
     </row>
     <row r="452" spans="3:3">
       <c r="C452" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
     </row>
     <row r="453" spans="3:3">
       <c r="C453" t="s">
-        <v>433</v>
+        <v>321</v>
       </c>
     </row>
     <row r="454" spans="3:3">
       <c r="C454" t="s">
-        <v>434</v>
+        <v>315</v>
       </c>
     </row>
     <row r="455" spans="3:3">
       <c r="C455" t="s">
-        <v>435</v>
+        <v>429</v>
       </c>
     </row>
     <row r="456" spans="3:3">
       <c r="C456" t="s">
-        <v>436</v>
+        <v>430</v>
       </c>
     </row>
     <row r="457" spans="3:3">
       <c r="C457" t="s">
-        <v>324</v>
+        <v>431</v>
       </c>
     </row>
     <row r="458" spans="3:3">
       <c r="C458" t="s">
-        <v>325</v>
+        <v>432</v>
       </c>
     </row>
     <row r="459" spans="3:3">
       <c r="C459" t="s">
-        <v>321</v>
+        <v>387</v>
       </c>
     </row>
     <row r="460" spans="3:3">
       <c r="C460" t="s">
-        <v>326</v>
+        <v>411</v>
       </c>
     </row>
     <row r="461" spans="3:3">
       <c r="C461" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="462" spans="3:3">
       <c r="C462" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="463" spans="3:3">
       <c r="C463" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="464" spans="3:3">
       <c r="C464" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="465" spans="3:3">
       <c r="C465" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="466" spans="3:3">
       <c r="C466" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="467" spans="3:3">
       <c r="C467" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="468" spans="3:3">
       <c r="C468" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
     </row>
     <row r="469" spans="3:3">
       <c r="C469" t="s">
-        <v>335</v>
+        <v>433</v>
       </c>
     </row>
     <row r="470" spans="3:3">
       <c r="C470" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
     </row>
     <row r="471" spans="3:3">
       <c r="C471" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="472" spans="3:3">
       <c r="C472" t="s">
-        <v>437</v>
+        <v>315</v>
       </c>
     </row>
     <row r="473" spans="3:3">
       <c r="C473" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
     </row>
     <row r="474" spans="3:3">
       <c r="C474" t="s">
-        <v>439</v>
+        <v>430</v>
       </c>
     </row>
     <row r="475" spans="3:3">
       <c r="C475" t="s">
-        <v>440</v>
+        <v>431</v>
       </c>
     </row>
     <row r="476" spans="3:3">
       <c r="C476" t="s">
-        <v>395</v>
+        <v>432</v>
       </c>
     </row>
     <row r="477" spans="3:3">
       <c r="C477" t="s">
-        <v>419</v>
+        <v>387</v>
       </c>
     </row>
     <row r="478" spans="3:3">
       <c r="C478" t="s">
-        <v>321</v>
+        <v>411</v>
       </c>
     </row>
     <row r="479" spans="3:3">
       <c r="C479" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="480" spans="3:3">
       <c r="C480" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="481" spans="3:3">
       <c r="C481" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="482" spans="3:3">
       <c r="C482" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="483" spans="3:3">
       <c r="C483" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="484" spans="3:3">
       <c r="C484" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="485" spans="3:3">
       <c r="C485" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="486" spans="3:3">
       <c r="C486" t="s">
-        <v>441</v>
+        <v>331</v>
       </c>
     </row>
     <row r="487" spans="3:3">
       <c r="C487" t="s">
-        <v>335</v>
+        <v>433</v>
       </c>
     </row>
     <row r="488" spans="3:3">
       <c r="C488" t="s">
-        <v>323</v>
+        <v>333</v>
       </c>
     </row>
     <row r="489" spans="3:3">
       <c r="C489" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="490" spans="3:3">
       <c r="C490" t="s">
-        <v>442</v>
+        <v>315</v>
       </c>
     </row>
     <row r="491" spans="3:3">
       <c r="C491" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
     </row>
     <row r="492" spans="3:3">
       <c r="C492" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="493" spans="3:3">
       <c r="C493" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="494" spans="3:3">
       <c r="C494" t="s">
-        <v>395</v>
+        <v>438</v>
       </c>
     </row>
     <row r="495" spans="3:3">
       <c r="C495" t="s">
-        <v>419</v>
+        <v>322</v>
       </c>
     </row>
     <row r="496" spans="3:3">
       <c r="C496" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="497" spans="3:3">
       <c r="C497" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="498" spans="3:3">
       <c r="C498" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="499" spans="3:3">
       <c r="C499" t="s">
-        <v>329</v>
+        <v>379</v>
       </c>
     </row>
     <row r="500" spans="3:3">
       <c r="C500" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="501" spans="3:3">
       <c r="C501" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="502" spans="3:3">
       <c r="C502" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="503" spans="3:3">
       <c r="C503" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="504" spans="3:3">
       <c r="C504" t="s">
-        <v>441</v>
+        <v>332</v>
       </c>
     </row>
     <row r="505" spans="3:3">
       <c r="C505" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="506" spans="3:3">
       <c r="C506" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="507" spans="3:3">
       <c r="C507" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="508" spans="3:3">
       <c r="C508" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
     </row>
     <row r="509" spans="3:3">
       <c r="C509" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
     </row>
     <row r="510" spans="3:3">
       <c r="C510" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="511" spans="3:3">
       <c r="C511" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
     </row>
     <row r="512" spans="3:3">
       <c r="C512" t="s">
-        <v>324</v>
+        <v>387</v>
       </c>
     </row>
     <row r="513" spans="3:3">
       <c r="C513" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="514" spans="3:3">
       <c r="C514" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="515" spans="3:3">
       <c r="C515" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="516" spans="3:3">
       <c r="C516" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
     </row>
     <row r="517" spans="3:3">
       <c r="C517" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="518" spans="3:3">
       <c r="C518" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="519" spans="3:3">
       <c r="C519" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="520" spans="3:3">
       <c r="C520" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="521" spans="3:3">
       <c r="C521" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="522" spans="3:3">
       <c r="C522" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="523" spans="3:3">
       <c r="C523" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="524" spans="3:3">
       <c r="C524" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="525" spans="3:3">
       <c r="C525" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
     </row>
     <row r="526" spans="3:3">
       <c r="C526" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
     </row>
     <row r="527" spans="3:3">
       <c r="C527" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
     </row>
     <row r="528" spans="3:3">
       <c r="C528" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
     </row>
     <row r="529" spans="3:3">
       <c r="C529" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
     </row>
     <row r="530" spans="3:3">
       <c r="C530" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="531" spans="3:3">
       <c r="C531" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="532" spans="3:3">
       <c r="C532" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="533" spans="3:3">
       <c r="C533" t="s">
-        <v>387</v>
+        <v>379</v>
       </c>
     </row>
     <row r="534" spans="3:3">
       <c r="C534" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="535" spans="3:3">
       <c r="C535" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="536" spans="3:3">
       <c r="C536" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="537" spans="3:3">
       <c r="C537" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="538" spans="3:3">
       <c r="C538" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="539" spans="3:3">
       <c r="C539" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="540" spans="3:3">
       <c r="C540" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
     </row>
     <row r="541" spans="3:3">
       <c r="C541" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="542" spans="3:3">
       <c r="C542" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
     </row>
     <row r="543" spans="3:3">
       <c r="C543" t="s">
-        <v>452</v>
+        <v>316</v>
       </c>
     </row>
     <row r="544" spans="3:3">
       <c r="C544" t="s">
-        <v>453</v>
+        <v>448</v>
       </c>
     </row>
     <row r="545" spans="3:3">
       <c r="C545" t="s">
-        <v>454</v>
+        <v>317</v>
       </c>
     </row>
     <row r="546" spans="3:3">
       <c r="C546" t="s">
-        <v>395</v>
+        <v>449</v>
       </c>
     </row>
     <row r="547" spans="3:3">
       <c r="C547" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
     </row>
     <row r="548" spans="3:3">
       <c r="C548" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
     </row>
     <row r="549" spans="3:3">
       <c r="C549" t="s">
-        <v>326</v>
+        <v>450</v>
       </c>
     </row>
     <row r="550" spans="3:3">
       <c r="C550" t="s">
-        <v>387</v>
+        <v>320</v>
       </c>
     </row>
     <row r="551" spans="3:3">
       <c r="C551" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="552" spans="3:3">
       <c r="C552" t="s">
-        <v>331</v>
+        <v>315</v>
       </c>
     </row>
     <row r="553" spans="3:3">
       <c r="C553" t="s">
-        <v>332</v>
+        <v>451</v>
       </c>
     </row>
     <row r="554" spans="3:3">
       <c r="C554" t="s">
-        <v>333</v>
+        <v>452</v>
       </c>
     </row>
     <row r="555" spans="3:3">
       <c r="C555" t="s">
-        <v>334</v>
+        <v>453</v>
       </c>
     </row>
     <row r="556" spans="3:3">
       <c r="C556" t="s">
-        <v>335</v>
+        <v>317</v>
       </c>
     </row>
     <row r="557" spans="3:3">
       <c r="C557" t="s">
-        <v>323</v>
+        <v>449</v>
       </c>
     </row>
     <row r="558" spans="3:3">
       <c r="C558" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="559" spans="3:3">
       <c r="C559" t="s">
-        <v>455</v>
+        <v>319</v>
       </c>
     </row>
     <row r="560" spans="3:3">
       <c r="C560" t="s">
-        <v>318</v>
+        <v>450</v>
       </c>
     </row>
     <row r="561" spans="3:3">
       <c r="C561" t="s">
-        <v>456</v>
+        <v>320</v>
       </c>
     </row>
     <row r="562" spans="3:3">
       <c r="C562" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="563" spans="3:3">
       <c r="C563" t="s">
-        <v>457</v>
+        <v>315</v>
       </c>
     </row>
     <row r="564" spans="3:3">
       <c r="C564" t="s">
-        <v>320</v>
+        <v>454</v>
       </c>
     </row>
     <row r="565" spans="3:3">
       <c r="C565" t="s">
-        <v>321</v>
+        <v>455</v>
       </c>
     </row>
     <row r="566" spans="3:3">
       <c r="C566" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="567" spans="3:3">
       <c r="C567" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
     </row>
     <row r="568" spans="3:3">
       <c r="C568" t="s">
-        <v>323</v>
+        <v>369</v>
       </c>
     </row>
     <row r="569" spans="3:3">
       <c r="C569" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="570" spans="3:3">
       <c r="C570" t="s">
-        <v>459</v>
+        <v>319</v>
       </c>
     </row>
     <row r="571" spans="3:3">
       <c r="C571" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
     <row r="572" spans="3:3">
       <c r="C572" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="573" spans="3:3">
       <c r="C573" t="s">
-        <v>319</v>
+        <v>379</v>
       </c>
     </row>
     <row r="574" spans="3:3">
       <c r="C574" t="s">
-        <v>457</v>
+        <v>320</v>
       </c>
     </row>
     <row r="575" spans="3:3">
       <c r="C575" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="576" spans="3:3">
       <c r="C576" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="577" spans="3:3">
       <c r="C577" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="578" spans="3:3">
       <c r="C578" t="s">
-        <v>322</v>
+        <v>455</v>
       </c>
     </row>
     <row r="579" spans="3:3">
       <c r="C579" t="s">
-        <v>323</v>
+        <v>460</v>
       </c>
     </row>
     <row r="580" spans="3:3">
@@ -6736,62 +6781,62 @@
     </row>
     <row r="581" spans="3:3">
       <c r="C581" t="s">
-        <v>462</v>
+        <v>369</v>
       </c>
     </row>
     <row r="582" spans="3:3">
       <c r="C582" t="s">
-        <v>463</v>
+        <v>318</v>
       </c>
     </row>
     <row r="583" spans="3:3">
       <c r="C583" t="s">
-        <v>464</v>
+        <v>319</v>
       </c>
     </row>
     <row r="584" spans="3:3">
       <c r="C584" t="s">
-        <v>319</v>
+        <v>457</v>
       </c>
     </row>
     <row r="585" spans="3:3">
       <c r="C585" t="s">
-        <v>377</v>
+        <v>458</v>
       </c>
     </row>
     <row r="586" spans="3:3">
       <c r="C586" t="s">
-        <v>320</v>
+        <v>379</v>
       </c>
     </row>
     <row r="587" spans="3:3">
       <c r="C587" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="588" spans="3:3">
       <c r="C588" t="s">
-        <v>465</v>
+        <v>321</v>
       </c>
     </row>
     <row r="589" spans="3:3">
       <c r="C589" t="s">
-        <v>466</v>
+        <v>315</v>
       </c>
     </row>
     <row r="590" spans="3:3">
       <c r="C590" t="s">
-        <v>387</v>
+        <v>461</v>
       </c>
     </row>
     <row r="591" spans="3:3">
       <c r="C591" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
     </row>
     <row r="592" spans="3:3">
       <c r="C592" t="s">
-        <v>323</v>
+        <v>462</v>
       </c>
     </row>
     <row r="593" spans="3:3">
@@ -6801,82 +6846,82 @@
     </row>
     <row r="594" spans="3:3">
       <c r="C594" t="s">
-        <v>467</v>
+        <v>449</v>
       </c>
     </row>
     <row r="595" spans="3:3">
       <c r="C595" t="s">
-        <v>463</v>
+        <v>318</v>
       </c>
     </row>
     <row r="596" spans="3:3">
       <c r="C596" t="s">
-        <v>468</v>
+        <v>319</v>
       </c>
     </row>
     <row r="597" spans="3:3">
       <c r="C597" t="s">
-        <v>319</v>
+        <v>457</v>
       </c>
     </row>
     <row r="598" spans="3:3">
       <c r="C598" t="s">
-        <v>377</v>
+        <v>458</v>
       </c>
     </row>
     <row r="599" spans="3:3">
       <c r="C599" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
     <row r="600" spans="3:3">
       <c r="C600" t="s">
-        <v>321</v>
+        <v>463</v>
       </c>
     </row>
     <row r="601" spans="3:3">
       <c r="C601" t="s">
-        <v>465</v>
+        <v>320</v>
       </c>
     </row>
     <row r="602" spans="3:3">
       <c r="C602" t="s">
-        <v>466</v>
+        <v>321</v>
       </c>
     </row>
     <row r="603" spans="3:3">
       <c r="C603" t="s">
-        <v>387</v>
+        <v>315</v>
       </c>
     </row>
     <row r="604" spans="3:3">
       <c r="C604" t="s">
-        <v>322</v>
+        <v>464</v>
       </c>
     </row>
     <row r="605" spans="3:3">
       <c r="C605" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="606" spans="3:3">
       <c r="C606" t="s">
-        <v>317</v>
+        <v>465</v>
       </c>
     </row>
     <row r="607" spans="3:3">
       <c r="C607" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
     <row r="608" spans="3:3">
       <c r="C608" t="s">
-        <v>318</v>
+        <v>467</v>
       </c>
     </row>
     <row r="609" spans="3:3">
       <c r="C609" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
     </row>
     <row r="610" spans="3:3">
@@ -6886,82 +6931,82 @@
     </row>
     <row r="611" spans="3:3">
       <c r="C611" t="s">
-        <v>457</v>
+        <v>469</v>
       </c>
     </row>
     <row r="612" spans="3:3">
       <c r="C612" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
     </row>
     <row r="613" spans="3:3">
       <c r="C613" t="s">
-        <v>321</v>
+        <v>470</v>
       </c>
     </row>
     <row r="614" spans="3:3">
       <c r="C614" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
     </row>
     <row r="615" spans="3:3">
       <c r="C615" t="s">
-        <v>466</v>
+        <v>472</v>
       </c>
     </row>
     <row r="616" spans="3:3">
       <c r="C616" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="617" spans="3:3">
       <c r="C617" t="s">
-        <v>471</v>
+        <v>315</v>
       </c>
     </row>
     <row r="618" spans="3:3">
       <c r="C618" t="s">
-        <v>322</v>
+        <v>473</v>
       </c>
     </row>
     <row r="619" spans="3:3">
       <c r="C619" t="s">
-        <v>323</v>
+        <v>474</v>
       </c>
     </row>
     <row r="620" spans="3:3">
       <c r="C620" t="s">
-        <v>317</v>
+        <v>475</v>
       </c>
     </row>
     <row r="621" spans="3:3">
       <c r="C621" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
     </row>
     <row r="622" spans="3:3">
       <c r="C622" t="s">
-        <v>318</v>
+        <v>477</v>
       </c>
     </row>
     <row r="623" spans="3:3">
       <c r="C623" t="s">
-        <v>473</v>
+        <v>336</v>
       </c>
     </row>
     <row r="624" spans="3:3">
       <c r="C624" t="s">
-        <v>474</v>
+        <v>319</v>
       </c>
     </row>
     <row r="625" spans="3:3">
       <c r="C625" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="626" spans="3:3">
       <c r="C626" t="s">
-        <v>476</v>
+        <v>320</v>
       </c>
     </row>
     <row r="627" spans="3:3">
@@ -6971,597 +7016,512 @@
     </row>
     <row r="628" spans="3:3">
       <c r="C628" t="s">
-        <v>477</v>
+        <v>315</v>
       </c>
     </row>
     <row r="629" spans="3:3">
       <c r="C629" t="s">
-        <v>330</v>
+        <v>479</v>
       </c>
     </row>
     <row r="630" spans="3:3">
       <c r="C630" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
     </row>
     <row r="631" spans="3:3">
       <c r="C631" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
     </row>
     <row r="632" spans="3:3">
       <c r="C632" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
     </row>
     <row r="633" spans="3:3">
       <c r="C633" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="634" spans="3:3">
       <c r="C634" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="635" spans="3:3">
       <c r="C635" t="s">
-        <v>481</v>
+        <v>319</v>
       </c>
     </row>
     <row r="636" spans="3:3">
       <c r="C636" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
     </row>
     <row r="637" spans="3:3">
       <c r="C637" t="s">
-        <v>483</v>
+        <v>320</v>
       </c>
     </row>
     <row r="638" spans="3:3">
       <c r="C638" t="s">
-        <v>484</v>
+        <v>321</v>
       </c>
     </row>
     <row r="639" spans="3:3">
       <c r="C639" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="640" spans="3:3">
       <c r="C640" t="s">
-        <v>344</v>
+        <v>482</v>
       </c>
     </row>
     <row r="641" spans="3:3">
       <c r="C641" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="642" spans="3:3">
       <c r="C642" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
     </row>
     <row r="643" spans="3:3">
       <c r="C643" t="s">
-        <v>322</v>
+        <v>476</v>
       </c>
     </row>
     <row r="644" spans="3:3">
       <c r="C644" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="645" spans="3:3">
       <c r="C645" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="646" spans="3:3">
       <c r="C646" t="s">
-        <v>487</v>
+        <v>319</v>
       </c>
     </row>
     <row r="647" spans="3:3">
       <c r="C647" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
     </row>
     <row r="648" spans="3:3">
       <c r="C648" t="s">
-        <v>488</v>
+        <v>320</v>
       </c>
     </row>
     <row r="649" spans="3:3">
       <c r="C649" t="s">
-        <v>489</v>
+        <v>321</v>
       </c>
     </row>
     <row r="650" spans="3:3">
       <c r="C650" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="651" spans="3:3">
       <c r="C651" t="s">
-        <v>344</v>
+        <v>484</v>
       </c>
     </row>
     <row r="652" spans="3:3">
       <c r="C652" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="653" spans="3:3">
       <c r="C653" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="654" spans="3:3">
       <c r="C654" t="s">
-        <v>322</v>
+        <v>481</v>
       </c>
     </row>
     <row r="655" spans="3:3">
       <c r="C655" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="656" spans="3:3">
       <c r="C656" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="657" spans="3:3">
       <c r="C657" t="s">
-        <v>490</v>
+        <v>319</v>
       </c>
     </row>
     <row r="658" spans="3:3">
       <c r="C658" t="s">
-        <v>318</v>
+        <v>478</v>
       </c>
     </row>
     <row r="659" spans="3:3">
       <c r="C659" t="s">
-        <v>491</v>
+        <v>320</v>
       </c>
     </row>
     <row r="660" spans="3:3">
       <c r="C660" t="s">
-        <v>484</v>
+        <v>321</v>
       </c>
     </row>
     <row r="661" spans="3:3">
       <c r="C661" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="662" spans="3:3">
       <c r="C662" t="s">
-        <v>344</v>
+        <v>486</v>
       </c>
     </row>
     <row r="663" spans="3:3">
       <c r="C663" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="664" spans="3:3">
       <c r="C664" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="665" spans="3:3">
       <c r="C665" t="s">
-        <v>322</v>
+        <v>488</v>
       </c>
     </row>
     <row r="666" spans="3:3">
       <c r="C666" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="667" spans="3:3">
       <c r="C667" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="668" spans="3:3">
       <c r="C668" t="s">
-        <v>492</v>
+        <v>319</v>
       </c>
     </row>
     <row r="669" spans="3:3">
       <c r="C669" t="s">
-        <v>318</v>
+        <v>478</v>
       </c>
     </row>
     <row r="670" spans="3:3">
       <c r="C670" t="s">
-        <v>493</v>
+        <v>320</v>
       </c>
     </row>
     <row r="671" spans="3:3">
       <c r="C671" t="s">
-        <v>489</v>
+        <v>321</v>
       </c>
     </row>
     <row r="672" spans="3:3">
       <c r="C672" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="673" spans="3:3">
       <c r="C673" t="s">
-        <v>344</v>
+        <v>489</v>
       </c>
     </row>
     <row r="674" spans="3:3">
       <c r="C674" t="s">
-        <v>321</v>
+        <v>334</v>
       </c>
     </row>
     <row r="675" spans="3:3">
       <c r="C675" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
     </row>
     <row r="676" spans="3:3">
       <c r="C676" t="s">
-        <v>322</v>
+        <v>491</v>
       </c>
     </row>
     <row r="677" spans="3:3">
       <c r="C677" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="678" spans="3:3">
       <c r="C678" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="679" spans="3:3">
       <c r="C679" t="s">
-        <v>494</v>
+        <v>319</v>
       </c>
     </row>
     <row r="680" spans="3:3">
       <c r="C680" t="s">
-        <v>318</v>
+        <v>492</v>
       </c>
     </row>
     <row r="681" spans="3:3">
       <c r="C681" t="s">
-        <v>495</v>
+        <v>320</v>
       </c>
     </row>
     <row r="682" spans="3:3">
       <c r="C682" t="s">
-        <v>496</v>
+        <v>321</v>
       </c>
     </row>
     <row r="683" spans="3:3">
       <c r="C683" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="684" spans="3:3">
       <c r="C684" t="s">
-        <v>344</v>
+        <v>493</v>
       </c>
     </row>
     <row r="685" spans="3:3">
       <c r="C685" t="s">
-        <v>321</v>
+        <v>430</v>
       </c>
     </row>
     <row r="686" spans="3:3">
       <c r="C686" t="s">
-        <v>486</v>
+        <v>494</v>
       </c>
     </row>
     <row r="687" spans="3:3">
       <c r="C687" t="s">
-        <v>322</v>
+        <v>495</v>
       </c>
     </row>
     <row r="688" spans="3:3">
       <c r="C688" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="689" spans="3:3">
       <c r="C689" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="690" spans="3:3">
       <c r="C690" t="s">
-        <v>497</v>
+        <v>319</v>
       </c>
     </row>
     <row r="691" spans="3:3">
       <c r="C691" t="s">
-        <v>341</v>
+        <v>492</v>
       </c>
     </row>
     <row r="692" spans="3:3">
       <c r="C692" t="s">
-        <v>498</v>
+        <v>320</v>
       </c>
     </row>
     <row r="693" spans="3:3">
       <c r="C693" t="s">
-        <v>499</v>
+        <v>321</v>
       </c>
     </row>
     <row r="694" spans="3:3">
       <c r="C694" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="695" spans="3:3">
       <c r="C695" t="s">
-        <v>344</v>
+        <v>496</v>
       </c>
     </row>
     <row r="696" spans="3:3">
       <c r="C696" t="s">
-        <v>321</v>
+        <v>430</v>
       </c>
     </row>
     <row r="697" spans="3:3">
       <c r="C697" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="698" spans="3:3">
       <c r="C698" t="s">
-        <v>322</v>
+        <v>498</v>
       </c>
     </row>
     <row r="699" spans="3:3">
       <c r="C699" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="700" spans="3:3">
       <c r="C700" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="701" spans="3:3">
       <c r="C701" t="s">
-        <v>501</v>
+        <v>319</v>
       </c>
     </row>
     <row r="702" spans="3:3">
       <c r="C702" t="s">
-        <v>438</v>
+        <v>492</v>
       </c>
     </row>
     <row r="703" spans="3:3">
       <c r="C703" t="s">
-        <v>502</v>
+        <v>320</v>
       </c>
     </row>
     <row r="704" spans="3:3">
       <c r="C704" t="s">
-        <v>503</v>
+        <v>321</v>
       </c>
     </row>
     <row r="705" spans="3:3">
       <c r="C705" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="706" spans="3:3">
       <c r="C706" t="s">
-        <v>344</v>
+        <v>499</v>
       </c>
     </row>
     <row r="707" spans="3:3">
       <c r="C707" t="s">
-        <v>321</v>
+        <v>500</v>
       </c>
     </row>
     <row r="708" spans="3:3">
       <c r="C708" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="709" spans="3:3">
       <c r="C709" t="s">
-        <v>322</v>
+        <v>502</v>
       </c>
     </row>
     <row r="710" spans="3:3">
       <c r="C710" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="711" spans="3:3">
       <c r="C711" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="712" spans="3:3">
       <c r="C712" t="s">
-        <v>504</v>
+        <v>319</v>
       </c>
     </row>
     <row r="713" spans="3:3">
       <c r="C713" t="s">
-        <v>438</v>
+        <v>492</v>
       </c>
     </row>
     <row r="714" spans="3:3">
       <c r="C714" t="s">
-        <v>505</v>
+        <v>320</v>
       </c>
     </row>
     <row r="715" spans="3:3">
       <c r="C715" t="s">
-        <v>506</v>
+        <v>321</v>
       </c>
     </row>
     <row r="716" spans="3:3">
       <c r="C716" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="717" spans="3:3">
       <c r="C717" t="s">
-        <v>344</v>
+        <v>503</v>
       </c>
     </row>
     <row r="718" spans="3:3">
       <c r="C718" t="s">
-        <v>321</v>
+        <v>500</v>
       </c>
     </row>
     <row r="719" spans="3:3">
       <c r="C719" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
     </row>
     <row r="720" spans="3:3">
       <c r="C720" t="s">
-        <v>322</v>
+        <v>505</v>
       </c>
     </row>
     <row r="721" spans="3:3">
       <c r="C721" t="s">
-        <v>323</v>
+        <v>477</v>
       </c>
     </row>
     <row r="722" spans="3:3">
       <c r="C722" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="723" spans="3:3">
       <c r="C723" t="s">
-        <v>507</v>
+        <v>319</v>
       </c>
     </row>
     <row r="724" spans="3:3">
       <c r="C724" t="s">
-        <v>508</v>
+        <v>492</v>
       </c>
     </row>
     <row r="725" spans="3:3">
       <c r="C725" t="s">
-        <v>509</v>
+        <v>320</v>
       </c>
     </row>
     <row r="726" spans="3:3">
       <c r="C726" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
     </row>
     <row r="727" spans="3:3">
       <c r="C727" t="s">
-        <v>485</v>
+        <v>507</v>
       </c>
     </row>
     <row r="728" spans="3:3">
       <c r="C728" t="s">
-        <v>344</v>
+        <v>508</v>
       </c>
     </row>
     <row r="729" spans="3:3">
       <c r="C729" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="730" spans="3:3">
-      <c r="C730" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="731" spans="3:3">
-      <c r="C731" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="732" spans="3:3">
-      <c r="C732" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="733" spans="3:3">
-      <c r="C733" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="734" spans="3:3">
-      <c r="C734" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="735" spans="3:3">
-      <c r="C735" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="736" spans="3:3">
-      <c r="C736" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="737" spans="3:3">
-      <c r="C737" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="738" spans="3:3">
-      <c r="C738" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="739" spans="3:3">
-      <c r="C739" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="740" spans="3:3">
-      <c r="C740" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="741" spans="3:3">
-      <c r="C741" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="742" spans="3:3">
-      <c r="C742" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="743" spans="3:3">
-      <c r="C743" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="744" spans="3:3">
-      <c r="C744" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="745" spans="3:3">
-      <c r="C745" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="746" spans="3:3">
-      <c r="C746" t="s">
-        <v>517</v>
+        <v>509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Update error handling for AI model availability and rate limits in EmergencyMeetingPage
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F7DDF3-5579-481A-8347-7FA5644F3AE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A51C6A-09D8-4E7A-B26D-0DE07BF21416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="542">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2141,9 +2141,6 @@
     <t xml:space="preserve">      "version": "2.0",</t>
   </si>
   <si>
-    <t xml:space="preserve">      "description": "Gemini 2.0 Flash Experimental",</t>
-  </si>
-  <si>
     <t xml:space="preserve">      "outputTokenLimit": 8192,</t>
   </si>
   <si>
@@ -2154,12 +2151,6 @@
   </si>
   <si>
     <t xml:space="preserve">      "maxTemperature": 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "name": "models/gemini-2.0-flash",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash",</t>
   </si>
   <si>
     <t xml:space="preserve">      "description": "Gemini 2.0 Flash",</t>
@@ -2774,19 +2765,41 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">      "name": "models/gemini-2.0-flash-exp",</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>models/gemini-2.0-flash-exp</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash Experimental",</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>Gemini 2.0 Flash Experimental</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ジェミニ2.0 フラッシュ実験版</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>generateContent
+countTokens
+bidiGenerateContent</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">      "name": "models/gemini-2.0-flash",</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>models/gemini-2.0-flash</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">      "version": "2.0",</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash",</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini 2.0 Flash</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3737,7 +3750,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F96D129-34E8-4B10-A261-7AEE00EA03AD}">
-  <dimension ref="C2:Q729"/>
+  <dimension ref="C2:Q713"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
@@ -3753,57 +3766,57 @@
   <sheetData>
     <row r="2" spans="3:17">
       <c r="E2" t="s">
+        <v>507</v>
+      </c>
+      <c r="F2" t="s">
+        <v>509</v>
+      </c>
+      <c r="G2" t="s">
         <v>510</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>512</v>
       </c>
-      <c r="G2" t="s">
-        <v>513</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
+        <v>514</v>
+      </c>
+      <c r="K2" t="s">
         <v>515</v>
       </c>
-      <c r="J2" t="s">
-        <v>517</v>
-      </c>
-      <c r="K2" t="s">
-        <v>518</v>
-      </c>
       <c r="L2" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="M2" t="s">
+        <v>524</v>
+      </c>
+      <c r="N2" t="s">
+        <v>525</v>
+      </c>
+      <c r="O2" t="s">
+        <v>526</v>
+      </c>
+      <c r="P2" t="s">
         <v>527</v>
       </c>
-      <c r="N2" t="s">
+      <c r="Q2" t="s">
         <v>528</v>
-      </c>
-      <c r="O2" t="s">
-        <v>529</v>
-      </c>
-      <c r="P2" t="s">
-        <v>530</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>531</v>
       </c>
     </row>
     <row r="3" spans="3:17" ht="37.5">
       <c r="E3" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="H3" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="I3" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="J3">
         <v>1024</v>
@@ -3812,24 +3825,24 @@
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
     </row>
     <row r="4" spans="3:17" ht="75">
       <c r="E4" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
+        <v>519</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>522</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>523</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>525</v>
       </c>
       <c r="J4">
         <v>1048576</v>
@@ -3838,7 +3851,7 @@
         <v>65536</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -3858,19 +3871,19 @@
     </row>
     <row r="5" spans="3:17" ht="75">
       <c r="E5" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F5">
         <v>2.5</v>
       </c>
       <c r="G5" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="H5" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="I5" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="J5">
         <v>1048576</v>
@@ -3879,7 +3892,7 @@
         <v>65536</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -3897,816 +3910,849 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:17">
+    <row r="6" spans="3:17" ht="56.25">
       <c r="E6" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>539</v>
-      </c>
-      <c r="L6" s="1"/>
+        <v>534</v>
+      </c>
+      <c r="H6" t="s">
+        <v>534</v>
+      </c>
+      <c r="I6" t="s">
+        <v>535</v>
+      </c>
+      <c r="J6">
+        <v>1048576</v>
+      </c>
+      <c r="K6">
+        <v>8192</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+      <c r="N6">
+        <v>0.95</v>
+      </c>
+      <c r="O6">
+        <v>40</v>
+      </c>
+      <c r="P6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7" spans="3:17">
-      <c r="C7" t="s">
-        <v>315</v>
-      </c>
+      <c r="E7" t="s">
+        <v>538</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7" t="s">
+        <v>541</v>
+      </c>
+      <c r="L7" s="1"/>
     </row>
     <row r="8" spans="3:17">
       <c r="C8" t="s">
-        <v>536</v>
+        <v>315</v>
       </c>
     </row>
     <row r="9" spans="3:17">
       <c r="C9" t="s">
-        <v>334</v>
+        <v>537</v>
       </c>
     </row>
     <row r="10" spans="3:17">
       <c r="C10" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="11" spans="3:17">
       <c r="C11" t="s">
-        <v>335</v>
+        <v>540</v>
       </c>
     </row>
     <row r="12" spans="3:17">
       <c r="C12" t="s">
-        <v>322</v>
+        <v>339</v>
       </c>
     </row>
     <row r="13" spans="3:17">
       <c r="C13" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
     </row>
     <row r="14" spans="3:17">
       <c r="C14" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
     </row>
     <row r="15" spans="3:17">
       <c r="C15" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="16" spans="3:17">
       <c r="C16" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="19" spans="3:3">
       <c r="C19" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" spans="3:3">
       <c r="C20" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="22" spans="3:3">
       <c r="C22" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="25" spans="3:3">
       <c r="C25" t="s">
-        <v>340</v>
+        <v>321</v>
       </c>
     </row>
     <row r="26" spans="3:3">
       <c r="C26" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="27" spans="3:3">
       <c r="C27" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="28" spans="3:3">
       <c r="C28" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
     </row>
     <row r="29" spans="3:3">
       <c r="C29" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
     </row>
     <row r="30" spans="3:3">
       <c r="C30" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
     </row>
     <row r="31" spans="3:3">
       <c r="C31" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="32" spans="3:3">
       <c r="C32" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
     </row>
     <row r="33" spans="3:3">
       <c r="C33" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="34" spans="3:3">
       <c r="C34" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="35" spans="3:3">
       <c r="C35" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="36" spans="3:3">
       <c r="C36" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="38" spans="3:3">
       <c r="C38" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="40" spans="3:3">
       <c r="C40" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
     </row>
     <row r="42" spans="3:3">
       <c r="C42" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="43" spans="3:3">
       <c r="C43" t="s">
-        <v>343</v>
+        <v>321</v>
       </c>
     </row>
     <row r="44" spans="3:3">
       <c r="C44" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="45" spans="3:3">
       <c r="C45" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="46" spans="3:3">
       <c r="C46" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
     </row>
     <row r="47" spans="3:3">
       <c r="C47" t="s">
-        <v>322</v>
+        <v>344</v>
       </c>
     </row>
     <row r="48" spans="3:3">
       <c r="C48" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
     </row>
     <row r="49" spans="3:3">
       <c r="C49" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="50" spans="3:3">
       <c r="C50" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
     </row>
     <row r="51" spans="3:3">
       <c r="C51" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="52" spans="3:3">
       <c r="C52" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="53" spans="3:3">
       <c r="C53" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="54" spans="3:3">
       <c r="C54" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
     </row>
     <row r="55" spans="3:3">
       <c r="C55" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="56" spans="3:3">
       <c r="C56" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="57" spans="3:3">
       <c r="C57" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
     </row>
     <row r="58" spans="3:3">
       <c r="C58" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
     </row>
     <row r="59" spans="3:3">
       <c r="C59" t="s">
-        <v>321</v>
+        <v>338</v>
       </c>
     </row>
     <row r="60" spans="3:3">
       <c r="C60" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="61" spans="3:3">
       <c r="C61" t="s">
-        <v>346</v>
+        <v>315</v>
       </c>
     </row>
     <row r="62" spans="3:3">
       <c r="C62" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
     </row>
     <row r="63" spans="3:3">
       <c r="C63" t="s">
-        <v>347</v>
+        <v>334</v>
       </c>
     </row>
     <row r="64" spans="3:3">
       <c r="C64" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="65" spans="3:3">
       <c r="C65" t="s">
-        <v>322</v>
+        <v>348</v>
       </c>
     </row>
     <row r="66" spans="3:3">
       <c r="C66" t="s">
-        <v>336</v>
+        <v>322</v>
       </c>
     </row>
     <row r="67" spans="3:3">
       <c r="C67" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
     </row>
     <row r="68" spans="3:3">
       <c r="C68" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="69" spans="3:3">
       <c r="C69" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="70" spans="3:3">
       <c r="C70" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
     </row>
     <row r="71" spans="3:3">
       <c r="C71" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="72" spans="3:3">
       <c r="C72" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="73" spans="3:3">
       <c r="C73" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="74" spans="3:3">
       <c r="C74" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="75" spans="3:3">
       <c r="C75" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="76" spans="3:3">
       <c r="C76" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
     </row>
     <row r="77" spans="3:3">
       <c r="C77" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="78" spans="3:3">
       <c r="C78" t="s">
-        <v>349</v>
+        <v>321</v>
       </c>
     </row>
     <row r="79" spans="3:3">
       <c r="C79" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="80" spans="3:3">
       <c r="C80" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="81" spans="3:3">
       <c r="C81" t="s">
-        <v>351</v>
+        <v>334</v>
       </c>
     </row>
     <row r="82" spans="3:3">
       <c r="C82" t="s">
-        <v>322</v>
+        <v>350</v>
       </c>
     </row>
     <row r="83" spans="3:3">
       <c r="C83" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
     </row>
     <row r="84" spans="3:3">
       <c r="C84" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="85" spans="3:3">
       <c r="C85" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
     </row>
     <row r="86" spans="3:3">
       <c r="C86" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="87" spans="3:3">
       <c r="C87" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="88" spans="3:3">
       <c r="C88" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="89" spans="3:3">
       <c r="C89" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="90" spans="3:3">
       <c r="C90" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="91" spans="3:3">
       <c r="C91" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="92" spans="3:3">
       <c r="C92" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="93" spans="3:3">
       <c r="C93" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="94" spans="3:3">
       <c r="C94" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
     </row>
     <row r="95" spans="3:3">
       <c r="C95" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="96" spans="3:3">
       <c r="C96" t="s">
-        <v>352</v>
+        <v>321</v>
       </c>
     </row>
     <row r="97" spans="3:3">
       <c r="C97" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="98" spans="3:3">
       <c r="C98" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="99" spans="3:3">
       <c r="C99" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="100" spans="3:3">
       <c r="C100" t="s">
-        <v>322</v>
+        <v>354</v>
       </c>
     </row>
     <row r="101" spans="3:3">
       <c r="C101" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
     </row>
     <row r="102" spans="3:3">
       <c r="C102" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="103" spans="3:3">
       <c r="C103" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
     </row>
     <row r="104" spans="3:3">
       <c r="C104" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="105" spans="3:3">
       <c r="C105" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="106" spans="3:3">
       <c r="C106" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="107" spans="3:3">
       <c r="C107" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="108" spans="3:3">
       <c r="C108" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="109" spans="3:3">
       <c r="C109" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="110" spans="3:3">
       <c r="C110" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="111" spans="3:3">
       <c r="C111" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="112" spans="3:3">
       <c r="C112" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
     </row>
     <row r="113" spans="3:3">
       <c r="C113" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="114" spans="3:3">
       <c r="C114" t="s">
-        <v>355</v>
+        <v>321</v>
       </c>
     </row>
     <row r="115" spans="3:3">
       <c r="C115" t="s">
-        <v>356</v>
+        <v>315</v>
       </c>
     </row>
     <row r="116" spans="3:3">
       <c r="C116" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="117" spans="3:3">
       <c r="C117" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
     </row>
     <row r="118" spans="3:3">
       <c r="C118" t="s">
-        <v>322</v>
+        <v>357</v>
       </c>
     </row>
     <row r="119" spans="3:3">
       <c r="C119" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
     </row>
     <row r="120" spans="3:3">
       <c r="C120" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="121" spans="3:3">
       <c r="C121" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
     </row>
     <row r="122" spans="3:3">
       <c r="C122" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="123" spans="3:3">
       <c r="C123" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="124" spans="3:3">
       <c r="C124" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="125" spans="3:3">
       <c r="C125" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="126" spans="3:3">
       <c r="C126" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="127" spans="3:3">
       <c r="C127" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="128" spans="3:3">
       <c r="C128" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="129" spans="3:3">
       <c r="C129" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="130" spans="3:3">
       <c r="C130" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
     </row>
     <row r="131" spans="3:3">
       <c r="C131" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="132" spans="3:3">
       <c r="C132" t="s">
-        <v>359</v>
+        <v>321</v>
       </c>
     </row>
     <row r="133" spans="3:3">
       <c r="C133" t="s">
-        <v>356</v>
+        <v>315</v>
       </c>
     </row>
     <row r="134" spans="3:3">
       <c r="C134" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
     </row>
     <row r="135" spans="3:3">
       <c r="C135" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="136" spans="3:3">
       <c r="C136" t="s">
-        <v>322</v>
+        <v>360</v>
       </c>
     </row>
     <row r="137" spans="3:3">
       <c r="C137" t="s">
-        <v>336</v>
+        <v>361</v>
       </c>
     </row>
     <row r="138" spans="3:3">
       <c r="C138" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="139" spans="3:3">
       <c r="C139" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="140" spans="3:3">
       <c r="C140" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="141" spans="3:3">
       <c r="C141" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="142" spans="3:3">
       <c r="C142" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="143" spans="3:3">
       <c r="C143" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="144" spans="3:3">
       <c r="C144" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="145" spans="3:3">
       <c r="C145" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="146" spans="3:3">
       <c r="C146" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="147" spans="3:3">
       <c r="C147" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="148" spans="3:3">
       <c r="C148" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="149" spans="3:3">
       <c r="C149" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="150" spans="3:3">
       <c r="C150" t="s">
-        <v>361</v>
+        <v>333</v>
       </c>
     </row>
     <row r="151" spans="3:3">
       <c r="C151" t="s">
-        <v>362</v>
+        <v>321</v>
       </c>
     </row>
     <row r="152" spans="3:3">
       <c r="C152" t="s">
-        <v>363</v>
+        <v>315</v>
       </c>
     </row>
     <row r="153" spans="3:3">
       <c r="C153" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
     </row>
     <row r="154" spans="3:3">
       <c r="C154" t="s">
-        <v>322</v>
+        <v>363</v>
       </c>
     </row>
     <row r="155" spans="3:3">
       <c r="C155" t="s">
-        <v>323</v>
+        <v>364</v>
       </c>
     </row>
     <row r="156" spans="3:3">
       <c r="C156" t="s">
-        <v>319</v>
+        <v>365</v>
       </c>
     </row>
     <row r="157" spans="3:3">
       <c r="C157" t="s">
-        <v>324</v>
+        <v>366</v>
       </c>
     </row>
     <row r="158" spans="3:3">
       <c r="C158" t="s">
-        <v>325</v>
+        <v>367</v>
       </c>
     </row>
     <row r="159" spans="3:3">
       <c r="C159" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="160" spans="3:3">
       <c r="C160" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="161" spans="3:3">
       <c r="C161" t="s">
-        <v>328</v>
+        <v>368</v>
       </c>
     </row>
     <row r="162" spans="3:3">
       <c r="C162" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="163" spans="3:3">
       <c r="C163" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="164" spans="3:3">
       <c r="C164" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="165" spans="3:3">
       <c r="C165" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="166" spans="3:3">
       <c r="C166" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="167" spans="3:3">
@@ -4721,32 +4767,32 @@
     </row>
     <row r="169" spans="3:3">
       <c r="C169" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
     </row>
     <row r="170" spans="3:3">
       <c r="C170" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
     </row>
     <row r="171" spans="3:3">
       <c r="C171" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="172" spans="3:3">
       <c r="C172" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
     </row>
     <row r="173" spans="3:3">
       <c r="C173" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="174" spans="3:3">
       <c r="C174" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="175" spans="3:3">
@@ -4761,47 +4807,47 @@
     </row>
     <row r="177" spans="3:3">
       <c r="C177" t="s">
-        <v>371</v>
+        <v>324</v>
       </c>
     </row>
     <row r="178" spans="3:3">
       <c r="C178" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="179" spans="3:3">
       <c r="C179" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="180" spans="3:3">
       <c r="C180" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="181" spans="3:3">
       <c r="C181" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="182" spans="3:3">
       <c r="C182" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
     </row>
     <row r="183" spans="3:3">
       <c r="C183" t="s">
-        <v>321</v>
+        <v>338</v>
       </c>
     </row>
     <row r="184" spans="3:3">
       <c r="C184" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="185" spans="3:3">
       <c r="C185" t="s">
-        <v>372</v>
+        <v>315</v>
       </c>
     </row>
     <row r="186" spans="3:3">
@@ -4811,22 +4857,22 @@
     </row>
     <row r="187" spans="3:3">
       <c r="C187" t="s">
-        <v>374</v>
+        <v>316</v>
       </c>
     </row>
     <row r="188" spans="3:3">
       <c r="C188" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="189" spans="3:3">
       <c r="C189" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="190" spans="3:3">
       <c r="C190" t="s">
-        <v>370</v>
+        <v>335</v>
       </c>
     </row>
     <row r="191" spans="3:3">
@@ -4836,122 +4882,122 @@
     </row>
     <row r="192" spans="3:3">
       <c r="C192" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="193" spans="3:3">
       <c r="C193" t="s">
-        <v>324</v>
+        <v>376</v>
       </c>
     </row>
     <row r="194" spans="3:3">
       <c r="C194" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="195" spans="3:3">
       <c r="C195" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="196" spans="3:3">
       <c r="C196" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="197" spans="3:3">
       <c r="C197" t="s">
-        <v>330</v>
+        <v>377</v>
       </c>
     </row>
     <row r="198" spans="3:3">
       <c r="C198" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
     </row>
     <row r="199" spans="3:3">
       <c r="C199" t="s">
-        <v>339</v>
+        <v>315</v>
       </c>
     </row>
     <row r="200" spans="3:3">
       <c r="C200" t="s">
-        <v>321</v>
+        <v>378</v>
       </c>
     </row>
     <row r="201" spans="3:3">
       <c r="C201" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="202" spans="3:3">
       <c r="C202" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
     </row>
     <row r="203" spans="3:3">
       <c r="C203" t="s">
-        <v>316</v>
+        <v>375</v>
       </c>
     </row>
     <row r="204" spans="3:3">
       <c r="C204" t="s">
-        <v>377</v>
+        <v>335</v>
       </c>
     </row>
     <row r="205" spans="3:3">
       <c r="C205" t="s">
-        <v>378</v>
+        <v>319</v>
       </c>
     </row>
     <row r="206" spans="3:3">
       <c r="C206" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
     </row>
     <row r="207" spans="3:3">
       <c r="C207" t="s">
-        <v>319</v>
+        <v>376</v>
       </c>
     </row>
     <row r="208" spans="3:3">
       <c r="C208" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="209" spans="3:3">
       <c r="C209" t="s">
-        <v>379</v>
+        <v>329</v>
       </c>
     </row>
     <row r="210" spans="3:3">
       <c r="C210" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="211" spans="3:3">
       <c r="C211" t="s">
-        <v>329</v>
+        <v>377</v>
       </c>
     </row>
     <row r="212" spans="3:3">
       <c r="C212" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="213" spans="3:3">
       <c r="C213" t="s">
-        <v>380</v>
+        <v>315</v>
       </c>
     </row>
     <row r="214" spans="3:3">
       <c r="C214" t="s">
-        <v>321</v>
+        <v>380</v>
       </c>
     </row>
     <row r="215" spans="3:3">
       <c r="C215" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="216" spans="3:3">
@@ -4961,67 +5007,67 @@
     </row>
     <row r="217" spans="3:3">
       <c r="C217" t="s">
-        <v>316</v>
+        <v>375</v>
       </c>
     </row>
     <row r="218" spans="3:3">
       <c r="C218" t="s">
-        <v>382</v>
+        <v>335</v>
       </c>
     </row>
     <row r="219" spans="3:3">
       <c r="C219" t="s">
-        <v>378</v>
+        <v>319</v>
       </c>
     </row>
     <row r="220" spans="3:3">
       <c r="C220" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
     </row>
     <row r="221" spans="3:3">
       <c r="C221" t="s">
-        <v>319</v>
+        <v>376</v>
       </c>
     </row>
     <row r="222" spans="3:3">
       <c r="C222" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="223" spans="3:3">
       <c r="C223" t="s">
-        <v>379</v>
+        <v>329</v>
       </c>
     </row>
     <row r="224" spans="3:3">
       <c r="C224" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="225" spans="3:3">
       <c r="C225" t="s">
-        <v>329</v>
+        <v>377</v>
       </c>
     </row>
     <row r="226" spans="3:3">
       <c r="C226" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="227" spans="3:3">
       <c r="C227" t="s">
-        <v>380</v>
+        <v>315</v>
       </c>
     </row>
     <row r="228" spans="3:3">
       <c r="C228" t="s">
-        <v>321</v>
+        <v>382</v>
       </c>
     </row>
     <row r="229" spans="3:3">
       <c r="C229" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="230" spans="3:3">
@@ -5031,1132 +5077,1132 @@
     </row>
     <row r="231" spans="3:3">
       <c r="C231" t="s">
-        <v>316</v>
+        <v>384</v>
       </c>
     </row>
     <row r="232" spans="3:3">
       <c r="C232" t="s">
-        <v>384</v>
+        <v>335</v>
       </c>
     </row>
     <row r="233" spans="3:3">
       <c r="C233" t="s">
-        <v>378</v>
+        <v>319</v>
       </c>
     </row>
     <row r="234" spans="3:3">
       <c r="C234" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
     </row>
     <row r="235" spans="3:3">
       <c r="C235" t="s">
-        <v>319</v>
+        <v>376</v>
       </c>
     </row>
     <row r="236" spans="3:3">
       <c r="C236" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="237" spans="3:3">
       <c r="C237" t="s">
-        <v>379</v>
+        <v>329</v>
       </c>
     </row>
     <row r="238" spans="3:3">
       <c r="C238" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="239" spans="3:3">
       <c r="C239" t="s">
-        <v>329</v>
+        <v>377</v>
       </c>
     </row>
     <row r="240" spans="3:3">
       <c r="C240" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="241" spans="3:3">
       <c r="C241" t="s">
-        <v>380</v>
+        <v>315</v>
       </c>
     </row>
     <row r="242" spans="3:3">
       <c r="C242" t="s">
-        <v>321</v>
+        <v>385</v>
       </c>
     </row>
     <row r="243" spans="3:3">
       <c r="C243" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="244" spans="3:3">
       <c r="C244" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="245" spans="3:3">
       <c r="C245" t="s">
-        <v>316</v>
+        <v>366</v>
       </c>
     </row>
     <row r="246" spans="3:3">
       <c r="C246" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="247" spans="3:3">
       <c r="C247" t="s">
-        <v>387</v>
+        <v>319</v>
       </c>
     </row>
     <row r="248" spans="3:3">
       <c r="C248" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
     </row>
     <row r="249" spans="3:3">
       <c r="C249" t="s">
-        <v>319</v>
+        <v>376</v>
       </c>
     </row>
     <row r="250" spans="3:3">
       <c r="C250" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="251" spans="3:3">
       <c r="C251" t="s">
-        <v>379</v>
+        <v>329</v>
       </c>
     </row>
     <row r="252" spans="3:3">
       <c r="C252" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="253" spans="3:3">
       <c r="C253" t="s">
-        <v>329</v>
+        <v>377</v>
       </c>
     </row>
     <row r="254" spans="3:3">
       <c r="C254" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="255" spans="3:3">
       <c r="C255" t="s">
-        <v>380</v>
+        <v>315</v>
       </c>
     </row>
     <row r="256" spans="3:3">
       <c r="C256" t="s">
-        <v>321</v>
+        <v>388</v>
       </c>
     </row>
     <row r="257" spans="3:3">
       <c r="C257" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="258" spans="3:3">
       <c r="C258" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="259" spans="3:3">
       <c r="C259" t="s">
-        <v>316</v>
+        <v>366</v>
       </c>
     </row>
     <row r="260" spans="3:3">
       <c r="C260" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
     </row>
     <row r="261" spans="3:3">
       <c r="C261" t="s">
-        <v>369</v>
+        <v>319</v>
       </c>
     </row>
     <row r="262" spans="3:3">
       <c r="C262" t="s">
-        <v>390</v>
+        <v>324</v>
       </c>
     </row>
     <row r="263" spans="3:3">
       <c r="C263" t="s">
-        <v>319</v>
+        <v>376</v>
       </c>
     </row>
     <row r="264" spans="3:3">
       <c r="C264" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
     </row>
     <row r="265" spans="3:3">
       <c r="C265" t="s">
-        <v>379</v>
+        <v>329</v>
       </c>
     </row>
     <row r="266" spans="3:3">
       <c r="C266" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="267" spans="3:3">
       <c r="C267" t="s">
-        <v>329</v>
+        <v>377</v>
       </c>
     </row>
     <row r="268" spans="3:3">
       <c r="C268" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="269" spans="3:3">
       <c r="C269" t="s">
-        <v>380</v>
+        <v>315</v>
       </c>
     </row>
     <row r="270" spans="3:3">
       <c r="C270" t="s">
-        <v>321</v>
+        <v>390</v>
       </c>
     </row>
     <row r="271" spans="3:3">
       <c r="C271" t="s">
-        <v>315</v>
+        <v>391</v>
       </c>
     </row>
     <row r="272" spans="3:3">
       <c r="C272" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="273" spans="3:3">
       <c r="C273" t="s">
-        <v>316</v>
+        <v>393</v>
       </c>
     </row>
     <row r="274" spans="3:3">
       <c r="C274" t="s">
-        <v>392</v>
+        <v>322</v>
       </c>
     </row>
     <row r="275" spans="3:3">
       <c r="C275" t="s">
-        <v>369</v>
+        <v>323</v>
       </c>
     </row>
     <row r="276" spans="3:3">
       <c r="C276" t="s">
-        <v>390</v>
+        <v>319</v>
       </c>
     </row>
     <row r="277" spans="3:3">
       <c r="C277" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="278" spans="3:3">
       <c r="C278" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="279" spans="3:3">
       <c r="C279" t="s">
-        <v>379</v>
+        <v>326</v>
       </c>
     </row>
     <row r="280" spans="3:3">
       <c r="C280" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="281" spans="3:3">
       <c r="C281" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="282" spans="3:3">
       <c r="C282" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="283" spans="3:3">
       <c r="C283" t="s">
-        <v>380</v>
+        <v>330</v>
       </c>
     </row>
     <row r="284" spans="3:3">
       <c r="C284" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="285" spans="3:3">
       <c r="C285" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="286" spans="3:3">
       <c r="C286" t="s">
-        <v>393</v>
+        <v>333</v>
       </c>
     </row>
     <row r="287" spans="3:3">
       <c r="C287" t="s">
-        <v>394</v>
+        <v>321</v>
       </c>
     </row>
     <row r="288" spans="3:3">
       <c r="C288" t="s">
-        <v>395</v>
+        <v>315</v>
       </c>
     </row>
     <row r="289" spans="3:3">
       <c r="C289" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="290" spans="3:3">
       <c r="C290" t="s">
-        <v>322</v>
+        <v>395</v>
       </c>
     </row>
     <row r="291" spans="3:3">
       <c r="C291" t="s">
-        <v>323</v>
+        <v>396</v>
       </c>
     </row>
     <row r="292" spans="3:3">
       <c r="C292" t="s">
-        <v>319</v>
+        <v>397</v>
       </c>
     </row>
     <row r="293" spans="3:3">
       <c r="C293" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="294" spans="3:3">
       <c r="C294" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="295" spans="3:3">
       <c r="C295" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="296" spans="3:3">
       <c r="C296" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="297" spans="3:3">
       <c r="C297" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="298" spans="3:3">
       <c r="C298" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="299" spans="3:3">
       <c r="C299" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="300" spans="3:3">
       <c r="C300" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="301" spans="3:3">
       <c r="C301" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="302" spans="3:3">
       <c r="C302" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="303" spans="3:3">
       <c r="C303" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="304" spans="3:3">
       <c r="C304" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="305" spans="3:3">
       <c r="C305" t="s">
-        <v>397</v>
+        <v>333</v>
       </c>
     </row>
     <row r="306" spans="3:3">
       <c r="C306" t="s">
-        <v>398</v>
+        <v>321</v>
       </c>
     </row>
     <row r="307" spans="3:3">
       <c r="C307" t="s">
-        <v>399</v>
+        <v>315</v>
       </c>
     </row>
     <row r="308" spans="3:3">
       <c r="C308" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="309" spans="3:3">
       <c r="C309" t="s">
-        <v>322</v>
+        <v>399</v>
       </c>
     </row>
     <row r="310" spans="3:3">
       <c r="C310" t="s">
-        <v>323</v>
+        <v>400</v>
       </c>
     </row>
     <row r="311" spans="3:3">
       <c r="C311" t="s">
-        <v>319</v>
+        <v>401</v>
       </c>
     </row>
     <row r="312" spans="3:3">
       <c r="C312" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="313" spans="3:3">
       <c r="C313" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="314" spans="3:3">
       <c r="C314" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="315" spans="3:3">
       <c r="C315" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="316" spans="3:3">
       <c r="C316" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="317" spans="3:3">
       <c r="C317" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="318" spans="3:3">
       <c r="C318" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="319" spans="3:3">
       <c r="C319" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="320" spans="3:3">
       <c r="C320" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="321" spans="3:3">
       <c r="C321" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="322" spans="3:3">
       <c r="C322" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="323" spans="3:3">
       <c r="C323" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="324" spans="3:3">
       <c r="C324" t="s">
-        <v>401</v>
+        <v>333</v>
       </c>
     </row>
     <row r="325" spans="3:3">
       <c r="C325" t="s">
-        <v>402</v>
+        <v>321</v>
       </c>
     </row>
     <row r="326" spans="3:3">
       <c r="C326" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
     </row>
     <row r="327" spans="3:3">
       <c r="C327" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="328" spans="3:3">
       <c r="C328" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
     </row>
     <row r="329" spans="3:3">
       <c r="C329" t="s">
-        <v>323</v>
+        <v>403</v>
       </c>
     </row>
     <row r="330" spans="3:3">
       <c r="C330" t="s">
-        <v>319</v>
+        <v>404</v>
       </c>
     </row>
     <row r="331" spans="3:3">
       <c r="C331" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="332" spans="3:3">
       <c r="C332" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="333" spans="3:3">
       <c r="C333" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="334" spans="3:3">
       <c r="C334" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="335" spans="3:3">
       <c r="C335" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="336" spans="3:3">
       <c r="C336" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="337" spans="3:3">
       <c r="C337" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="338" spans="3:3">
       <c r="C338" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="339" spans="3:3">
       <c r="C339" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="340" spans="3:3">
       <c r="C340" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="341" spans="3:3">
       <c r="C341" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="342" spans="3:3">
       <c r="C342" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="343" spans="3:3">
       <c r="C343" t="s">
-        <v>405</v>
+        <v>333</v>
       </c>
     </row>
     <row r="344" spans="3:3">
       <c r="C344" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
     </row>
     <row r="345" spans="3:3">
       <c r="C345" t="s">
-        <v>406</v>
+        <v>315</v>
       </c>
     </row>
     <row r="346" spans="3:3">
       <c r="C346" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
     </row>
     <row r="347" spans="3:3">
       <c r="C347" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
     </row>
     <row r="348" spans="3:3">
       <c r="C348" t="s">
-        <v>323</v>
+        <v>406</v>
       </c>
     </row>
     <row r="349" spans="3:3">
       <c r="C349" t="s">
-        <v>319</v>
+        <v>407</v>
       </c>
     </row>
     <row r="350" spans="3:3">
       <c r="C350" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
     </row>
     <row r="351" spans="3:3">
       <c r="C351" t="s">
-        <v>325</v>
+        <v>408</v>
       </c>
     </row>
     <row r="352" spans="3:3">
       <c r="C352" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="353" spans="3:3">
       <c r="C353" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="354" spans="3:3">
       <c r="C354" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="355" spans="3:3">
       <c r="C355" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="356" spans="3:3">
       <c r="C356" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="357" spans="3:3">
       <c r="C357" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="358" spans="3:3">
       <c r="C358" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="359" spans="3:3">
       <c r="C359" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="360" spans="3:3">
       <c r="C360" t="s">
-        <v>321</v>
+        <v>409</v>
       </c>
     </row>
     <row r="361" spans="3:3">
       <c r="C361" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="362" spans="3:3">
       <c r="C362" t="s">
-        <v>408</v>
+        <v>315</v>
       </c>
     </row>
     <row r="363" spans="3:3">
       <c r="C363" t="s">
-        <v>334</v>
+        <v>410</v>
       </c>
     </row>
     <row r="364" spans="3:3">
       <c r="C364" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
     </row>
     <row r="365" spans="3:3">
       <c r="C365" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="366" spans="3:3">
       <c r="C366" t="s">
-        <v>378</v>
+        <v>413</v>
       </c>
     </row>
     <row r="367" spans="3:3">
       <c r="C367" t="s">
-        <v>411</v>
+        <v>322</v>
       </c>
     </row>
     <row r="368" spans="3:3">
       <c r="C368" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="369" spans="3:3">
       <c r="C369" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="370" spans="3:3">
       <c r="C370" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="371" spans="3:3">
       <c r="C371" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
     </row>
     <row r="372" spans="3:3">
       <c r="C372" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="373" spans="3:3">
       <c r="C373" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="374" spans="3:3">
       <c r="C374" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="375" spans="3:3">
       <c r="C375" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="376" spans="3:3">
       <c r="C376" t="s">
-        <v>412</v>
+        <v>330</v>
       </c>
     </row>
     <row r="377" spans="3:3">
       <c r="C377" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="378" spans="3:3">
       <c r="C378" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="379" spans="3:3">
       <c r="C379" t="s">
-        <v>413</v>
+        <v>333</v>
       </c>
     </row>
     <row r="380" spans="3:3">
       <c r="C380" t="s">
-        <v>414</v>
+        <v>321</v>
       </c>
     </row>
     <row r="381" spans="3:3">
       <c r="C381" t="s">
-        <v>415</v>
+        <v>315</v>
       </c>
     </row>
     <row r="382" spans="3:3">
       <c r="C382" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
     </row>
     <row r="383" spans="3:3">
       <c r="C383" t="s">
-        <v>322</v>
+        <v>415</v>
       </c>
     </row>
     <row r="384" spans="3:3">
       <c r="C384" t="s">
-        <v>323</v>
+        <v>416</v>
       </c>
     </row>
     <row r="385" spans="3:3">
       <c r="C385" t="s">
-        <v>319</v>
+        <v>417</v>
       </c>
     </row>
     <row r="386" spans="3:3">
       <c r="C386" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="387" spans="3:3">
       <c r="C387" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="388" spans="3:3">
       <c r="C388" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="389" spans="3:3">
       <c r="C389" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="390" spans="3:3">
       <c r="C390" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="391" spans="3:3">
       <c r="C391" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="392" spans="3:3">
       <c r="C392" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="393" spans="3:3">
       <c r="C393" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="394" spans="3:3">
       <c r="C394" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="395" spans="3:3">
       <c r="C395" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="396" spans="3:3">
       <c r="C396" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="397" spans="3:3">
       <c r="C397" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="398" spans="3:3">
       <c r="C398" t="s">
-        <v>417</v>
+        <v>333</v>
       </c>
     </row>
     <row r="399" spans="3:3">
       <c r="C399" t="s">
-        <v>418</v>
+        <v>321</v>
       </c>
     </row>
     <row r="400" spans="3:3">
       <c r="C400" t="s">
-        <v>419</v>
+        <v>315</v>
       </c>
     </row>
     <row r="401" spans="3:3">
       <c r="C401" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
     </row>
     <row r="402" spans="3:3">
       <c r="C402" t="s">
-        <v>322</v>
+        <v>419</v>
       </c>
     </row>
     <row r="403" spans="3:3">
       <c r="C403" t="s">
-        <v>323</v>
+        <v>420</v>
       </c>
     </row>
     <row r="404" spans="3:3">
       <c r="C404" t="s">
-        <v>319</v>
+        <v>421</v>
       </c>
     </row>
     <row r="405" spans="3:3">
       <c r="C405" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="406" spans="3:3">
       <c r="C406" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="407" spans="3:3">
       <c r="C407" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="408" spans="3:3">
       <c r="C408" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="409" spans="3:3">
       <c r="C409" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="410" spans="3:3">
       <c r="C410" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="411" spans="3:3">
       <c r="C411" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="412" spans="3:3">
       <c r="C412" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="413" spans="3:3">
       <c r="C413" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="414" spans="3:3">
       <c r="C414" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="415" spans="3:3">
       <c r="C415" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="416" spans="3:3">
       <c r="C416" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="417" spans="3:3">
       <c r="C417" t="s">
-        <v>421</v>
+        <v>333</v>
       </c>
     </row>
     <row r="418" spans="3:3">
       <c r="C418" t="s">
-        <v>422</v>
+        <v>321</v>
       </c>
     </row>
     <row r="419" spans="3:3">
       <c r="C419" t="s">
-        <v>423</v>
+        <v>315</v>
       </c>
     </row>
     <row r="420" spans="3:3">
       <c r="C420" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
     </row>
     <row r="421" spans="3:3">
       <c r="C421" t="s">
-        <v>322</v>
+        <v>423</v>
       </c>
     </row>
     <row r="422" spans="3:3">
       <c r="C422" t="s">
-        <v>323</v>
+        <v>424</v>
       </c>
     </row>
     <row r="423" spans="3:3">
       <c r="C423" t="s">
-        <v>319</v>
+        <v>425</v>
       </c>
     </row>
     <row r="424" spans="3:3">
       <c r="C424" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="425" spans="3:3">
       <c r="C425" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="426" spans="3:3">
       <c r="C426" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="427" spans="3:3">
       <c r="C427" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="428" spans="3:3">
       <c r="C428" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="429" spans="3:3">
       <c r="C429" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="430" spans="3:3">
       <c r="C430" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="431" spans="3:3">
       <c r="C431" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="432" spans="3:3">
       <c r="C432" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="433" spans="3:3">
       <c r="C433" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="434" spans="3:3">
       <c r="C434" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="435" spans="3:3">
       <c r="C435" t="s">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="436" spans="3:3">
       <c r="C436" t="s">
-        <v>425</v>
+        <v>333</v>
       </c>
     </row>
     <row r="437" spans="3:3">
       <c r="C437" t="s">
-        <v>426</v>
+        <v>321</v>
       </c>
     </row>
     <row r="438" spans="3:3">
       <c r="C438" t="s">
-        <v>427</v>
+        <v>315</v>
       </c>
     </row>
     <row r="439" spans="3:3">
       <c r="C439" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
     </row>
     <row r="440" spans="3:3">
       <c r="C440" t="s">
-        <v>322</v>
+        <v>427</v>
       </c>
     </row>
     <row r="441" spans="3:3">
       <c r="C441" t="s">
-        <v>323</v>
+        <v>428</v>
       </c>
     </row>
     <row r="442" spans="3:3">
       <c r="C442" t="s">
-        <v>319</v>
+        <v>429</v>
       </c>
     </row>
     <row r="443" spans="3:3">
       <c r="C443" t="s">
-        <v>324</v>
+        <v>384</v>
       </c>
     </row>
     <row r="444" spans="3:3">
       <c r="C444" t="s">
-        <v>325</v>
+        <v>408</v>
       </c>
     </row>
     <row r="445" spans="3:3">
       <c r="C445" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="446" spans="3:3">
       <c r="C446" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="447" spans="3:3">
       <c r="C447" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="448" spans="3:3">
       <c r="C448" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="449" spans="3:3">
       <c r="C449" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="450" spans="3:3">
       <c r="C450" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="451" spans="3:3">
       <c r="C451" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="452" spans="3:3">
       <c r="C452" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="453" spans="3:3">
       <c r="C453" t="s">
-        <v>321</v>
+        <v>430</v>
       </c>
     </row>
     <row r="454" spans="3:3">
       <c r="C454" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="455" spans="3:3">
       <c r="C455" t="s">
-        <v>429</v>
+        <v>321</v>
       </c>
     </row>
     <row r="456" spans="3:3">
       <c r="C456" t="s">
-        <v>430</v>
+        <v>315</v>
       </c>
     </row>
     <row r="457" spans="3:3">
@@ -6166,172 +6212,172 @@
     </row>
     <row r="458" spans="3:3">
       <c r="C458" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
     </row>
     <row r="459" spans="3:3">
       <c r="C459" t="s">
-        <v>387</v>
+        <v>428</v>
       </c>
     </row>
     <row r="460" spans="3:3">
       <c r="C460" t="s">
-        <v>411</v>
+        <v>429</v>
       </c>
     </row>
     <row r="461" spans="3:3">
       <c r="C461" t="s">
-        <v>319</v>
+        <v>384</v>
       </c>
     </row>
     <row r="462" spans="3:3">
       <c r="C462" t="s">
-        <v>324</v>
+        <v>408</v>
       </c>
     </row>
     <row r="463" spans="3:3">
       <c r="C463" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="464" spans="3:3">
       <c r="C464" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="465" spans="3:3">
       <c r="C465" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="466" spans="3:3">
       <c r="C466" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="467" spans="3:3">
       <c r="C467" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="468" spans="3:3">
       <c r="C468" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="469" spans="3:3">
       <c r="C469" t="s">
-        <v>433</v>
+        <v>330</v>
       </c>
     </row>
     <row r="470" spans="3:3">
       <c r="C470" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="471" spans="3:3">
       <c r="C471" t="s">
-        <v>321</v>
+        <v>430</v>
       </c>
     </row>
     <row r="472" spans="3:3">
       <c r="C472" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="473" spans="3:3">
       <c r="C473" t="s">
-        <v>434</v>
+        <v>321</v>
       </c>
     </row>
     <row r="474" spans="3:3">
       <c r="C474" t="s">
-        <v>430</v>
+        <v>315</v>
       </c>
     </row>
     <row r="475" spans="3:3">
       <c r="C475" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="476" spans="3:3">
       <c r="C476" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="477" spans="3:3">
       <c r="C477" t="s">
-        <v>387</v>
+        <v>434</v>
       </c>
     </row>
     <row r="478" spans="3:3">
       <c r="C478" t="s">
-        <v>411</v>
+        <v>435</v>
       </c>
     </row>
     <row r="479" spans="3:3">
       <c r="C479" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="480" spans="3:3">
       <c r="C480" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="481" spans="3:3">
       <c r="C481" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="482" spans="3:3">
       <c r="C482" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="483" spans="3:3">
       <c r="C483" t="s">
-        <v>328</v>
+        <v>376</v>
       </c>
     </row>
     <row r="484" spans="3:3">
       <c r="C484" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="485" spans="3:3">
       <c r="C485" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="486" spans="3:3">
       <c r="C486" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="487" spans="3:3">
       <c r="C487" t="s">
-        <v>433</v>
+        <v>331</v>
       </c>
     </row>
     <row r="488" spans="3:3">
       <c r="C488" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="489" spans="3:3">
       <c r="C489" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="490" spans="3:3">
       <c r="C490" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="491" spans="3:3">
       <c r="C491" t="s">
-        <v>435</v>
+        <v>315</v>
       </c>
     </row>
     <row r="492" spans="3:3">
@@ -6351,72 +6397,72 @@
     </row>
     <row r="495" spans="3:3">
       <c r="C495" t="s">
-        <v>322</v>
+        <v>439</v>
       </c>
     </row>
     <row r="496" spans="3:3">
       <c r="C496" t="s">
-        <v>323</v>
+        <v>384</v>
       </c>
     </row>
     <row r="497" spans="3:3">
       <c r="C497" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="498" spans="3:3">
       <c r="C498" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="499" spans="3:3">
       <c r="C499" t="s">
-        <v>379</v>
+        <v>324</v>
       </c>
     </row>
     <row r="500" spans="3:3">
       <c r="C500" t="s">
-        <v>328</v>
+        <v>376</v>
       </c>
     </row>
     <row r="501" spans="3:3">
       <c r="C501" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="502" spans="3:3">
       <c r="C502" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="503" spans="3:3">
       <c r="C503" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="504" spans="3:3">
       <c r="C504" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="505" spans="3:3">
       <c r="C505" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="506" spans="3:3">
       <c r="C506" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="507" spans="3:3">
       <c r="C507" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="508" spans="3:3">
       <c r="C508" t="s">
-        <v>439</v>
+        <v>315</v>
       </c>
     </row>
     <row r="509" spans="3:3">
@@ -6436,72 +6482,72 @@
     </row>
     <row r="512" spans="3:3">
       <c r="C512" t="s">
-        <v>387</v>
+        <v>443</v>
       </c>
     </row>
     <row r="513" spans="3:3">
       <c r="C513" t="s">
-        <v>323</v>
+        <v>384</v>
       </c>
     </row>
     <row r="514" spans="3:3">
       <c r="C514" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="515" spans="3:3">
       <c r="C515" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="516" spans="3:3">
       <c r="C516" t="s">
-        <v>379</v>
+        <v>324</v>
       </c>
     </row>
     <row r="517" spans="3:3">
       <c r="C517" t="s">
-        <v>328</v>
+        <v>376</v>
       </c>
     </row>
     <row r="518" spans="3:3">
       <c r="C518" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="519" spans="3:3">
       <c r="C519" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="520" spans="3:3">
       <c r="C520" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="521" spans="3:3">
       <c r="C521" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="522" spans="3:3">
       <c r="C522" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="523" spans="3:3">
       <c r="C523" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="524" spans="3:3">
       <c r="C524" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="525" spans="3:3">
       <c r="C525" t="s">
-        <v>443</v>
+        <v>315</v>
       </c>
     </row>
     <row r="526" spans="3:3">
@@ -6511,437 +6557,437 @@
     </row>
     <row r="527" spans="3:3">
       <c r="C527" t="s">
-        <v>445</v>
+        <v>316</v>
       </c>
     </row>
     <row r="528" spans="3:3">
       <c r="C528" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="529" spans="3:3">
       <c r="C529" t="s">
-        <v>387</v>
+        <v>317</v>
       </c>
     </row>
     <row r="530" spans="3:3">
       <c r="C530" t="s">
-        <v>323</v>
+        <v>446</v>
       </c>
     </row>
     <row r="531" spans="3:3">
       <c r="C531" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="532" spans="3:3">
       <c r="C532" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="533" spans="3:3">
       <c r="C533" t="s">
-        <v>379</v>
+        <v>447</v>
       </c>
     </row>
     <row r="534" spans="3:3">
       <c r="C534" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
     </row>
     <row r="535" spans="3:3">
       <c r="C535" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
     </row>
     <row r="536" spans="3:3">
       <c r="C536" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="537" spans="3:3">
       <c r="C537" t="s">
-        <v>331</v>
+        <v>448</v>
       </c>
     </row>
     <row r="538" spans="3:3">
       <c r="C538" t="s">
-        <v>332</v>
+        <v>449</v>
       </c>
     </row>
     <row r="539" spans="3:3">
       <c r="C539" t="s">
-        <v>333</v>
+        <v>450</v>
       </c>
     </row>
     <row r="540" spans="3:3">
       <c r="C540" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="541" spans="3:3">
       <c r="C541" t="s">
-        <v>315</v>
+        <v>446</v>
       </c>
     </row>
     <row r="542" spans="3:3">
       <c r="C542" t="s">
-        <v>447</v>
+        <v>318</v>
       </c>
     </row>
     <row r="543" spans="3:3">
       <c r="C543" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="544" spans="3:3">
       <c r="C544" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="545" spans="3:3">
       <c r="C545" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="546" spans="3:3">
       <c r="C546" t="s">
-        <v>449</v>
+        <v>321</v>
       </c>
     </row>
     <row r="547" spans="3:3">
       <c r="C547" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="548" spans="3:3">
       <c r="C548" t="s">
-        <v>319</v>
+        <v>451</v>
       </c>
     </row>
     <row r="549" spans="3:3">
       <c r="C549" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="550" spans="3:3">
       <c r="C550" t="s">
-        <v>320</v>
+        <v>453</v>
       </c>
     </row>
     <row r="551" spans="3:3">
       <c r="C551" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="552" spans="3:3">
       <c r="C552" t="s">
-        <v>315</v>
+        <v>366</v>
       </c>
     </row>
     <row r="553" spans="3:3">
       <c r="C553" t="s">
-        <v>451</v>
+        <v>318</v>
       </c>
     </row>
     <row r="554" spans="3:3">
       <c r="C554" t="s">
-        <v>452</v>
+        <v>319</v>
       </c>
     </row>
     <row r="555" spans="3:3">
       <c r="C555" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
     </row>
     <row r="556" spans="3:3">
       <c r="C556" t="s">
-        <v>317</v>
+        <v>455</v>
       </c>
     </row>
     <row r="557" spans="3:3">
       <c r="C557" t="s">
-        <v>449</v>
+        <v>376</v>
       </c>
     </row>
     <row r="558" spans="3:3">
       <c r="C558" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="559" spans="3:3">
       <c r="C559" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="560" spans="3:3">
       <c r="C560" t="s">
-        <v>450</v>
+        <v>315</v>
       </c>
     </row>
     <row r="561" spans="3:3">
       <c r="C561" t="s">
-        <v>320</v>
+        <v>456</v>
       </c>
     </row>
     <row r="562" spans="3:3">
       <c r="C562" t="s">
-        <v>321</v>
+        <v>452</v>
       </c>
     </row>
     <row r="563" spans="3:3">
       <c r="C563" t="s">
-        <v>315</v>
+        <v>457</v>
       </c>
     </row>
     <row r="564" spans="3:3">
       <c r="C564" t="s">
-        <v>454</v>
+        <v>317</v>
       </c>
     </row>
     <row r="565" spans="3:3">
       <c r="C565" t="s">
-        <v>455</v>
+        <v>366</v>
       </c>
     </row>
     <row r="566" spans="3:3">
       <c r="C566" t="s">
-        <v>456</v>
+        <v>318</v>
       </c>
     </row>
     <row r="567" spans="3:3">
       <c r="C567" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="568" spans="3:3">
       <c r="C568" t="s">
-        <v>369</v>
+        <v>454</v>
       </c>
     </row>
     <row r="569" spans="3:3">
       <c r="C569" t="s">
-        <v>318</v>
+        <v>455</v>
       </c>
     </row>
     <row r="570" spans="3:3">
       <c r="C570" t="s">
-        <v>319</v>
+        <v>376</v>
       </c>
     </row>
     <row r="571" spans="3:3">
       <c r="C571" t="s">
-        <v>457</v>
+        <v>320</v>
       </c>
     </row>
     <row r="572" spans="3:3">
       <c r="C572" t="s">
-        <v>458</v>
+        <v>321</v>
       </c>
     </row>
     <row r="573" spans="3:3">
       <c r="C573" t="s">
-        <v>379</v>
+        <v>315</v>
       </c>
     </row>
     <row r="574" spans="3:3">
       <c r="C574" t="s">
-        <v>320</v>
+        <v>458</v>
       </c>
     </row>
     <row r="575" spans="3:3">
       <c r="C575" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
     </row>
     <row r="576" spans="3:3">
       <c r="C576" t="s">
-        <v>315</v>
+        <v>459</v>
       </c>
     </row>
     <row r="577" spans="3:3">
       <c r="C577" t="s">
-        <v>459</v>
+        <v>317</v>
       </c>
     </row>
     <row r="578" spans="3:3">
       <c r="C578" t="s">
-        <v>455</v>
+        <v>446</v>
       </c>
     </row>
     <row r="579" spans="3:3">
       <c r="C579" t="s">
-        <v>460</v>
+        <v>318</v>
       </c>
     </row>
     <row r="580" spans="3:3">
       <c r="C580" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
     </row>
     <row r="581" spans="3:3">
       <c r="C581" t="s">
-        <v>369</v>
+        <v>454</v>
       </c>
     </row>
     <row r="582" spans="3:3">
       <c r="C582" t="s">
-        <v>318</v>
+        <v>455</v>
       </c>
     </row>
     <row r="583" spans="3:3">
       <c r="C583" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
     </row>
     <row r="584" spans="3:3">
       <c r="C584" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
     </row>
     <row r="585" spans="3:3">
       <c r="C585" t="s">
-        <v>458</v>
+        <v>320</v>
       </c>
     </row>
     <row r="586" spans="3:3">
       <c r="C586" t="s">
-        <v>379</v>
+        <v>321</v>
       </c>
     </row>
     <row r="587" spans="3:3">
       <c r="C587" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
     </row>
     <row r="588" spans="3:3">
       <c r="C588" t="s">
-        <v>321</v>
+        <v>461</v>
       </c>
     </row>
     <row r="589" spans="3:3">
       <c r="C589" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="590" spans="3:3">
       <c r="C590" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="591" spans="3:3">
       <c r="C591" t="s">
-        <v>316</v>
+        <v>463</v>
       </c>
     </row>
     <row r="592" spans="3:3">
       <c r="C592" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="593" spans="3:3">
       <c r="C593" t="s">
-        <v>317</v>
+        <v>465</v>
       </c>
     </row>
     <row r="594" spans="3:3">
       <c r="C594" t="s">
-        <v>449</v>
+        <v>319</v>
       </c>
     </row>
     <row r="595" spans="3:3">
       <c r="C595" t="s">
-        <v>318</v>
+        <v>466</v>
       </c>
     </row>
     <row r="596" spans="3:3">
       <c r="C596" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
     </row>
     <row r="597" spans="3:3">
       <c r="C597" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
     </row>
     <row r="598" spans="3:3">
       <c r="C598" t="s">
-        <v>458</v>
+        <v>468</v>
       </c>
     </row>
     <row r="599" spans="3:3">
       <c r="C599" t="s">
-        <v>325</v>
+        <v>469</v>
       </c>
     </row>
     <row r="600" spans="3:3">
       <c r="C600" t="s">
-        <v>463</v>
+        <v>321</v>
       </c>
     </row>
     <row r="601" spans="3:3">
       <c r="C601" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
     </row>
     <row r="602" spans="3:3">
       <c r="C602" t="s">
-        <v>321</v>
+        <v>470</v>
       </c>
     </row>
     <row r="603" spans="3:3">
       <c r="C603" t="s">
-        <v>315</v>
+        <v>471</v>
       </c>
     </row>
     <row r="604" spans="3:3">
       <c r="C604" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
     </row>
     <row r="605" spans="3:3">
       <c r="C605" t="s">
-        <v>316</v>
+        <v>473</v>
       </c>
     </row>
     <row r="606" spans="3:3">
       <c r="C606" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
     </row>
     <row r="607" spans="3:3">
       <c r="C607" t="s">
-        <v>466</v>
+        <v>335</v>
       </c>
     </row>
     <row r="608" spans="3:3">
       <c r="C608" t="s">
-        <v>467</v>
+        <v>319</v>
       </c>
     </row>
     <row r="609" spans="3:3">
       <c r="C609" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
     </row>
     <row r="610" spans="3:3">
       <c r="C610" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="611" spans="3:3">
       <c r="C611" t="s">
-        <v>469</v>
+        <v>321</v>
       </c>
     </row>
     <row r="612" spans="3:3">
       <c r="C612" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
     </row>
     <row r="613" spans="3:3">
       <c r="C613" t="s">
-        <v>470</v>
+        <v>476</v>
       </c>
     </row>
     <row r="614" spans="3:3">
@@ -6951,27 +6997,27 @@
     </row>
     <row r="615" spans="3:3">
       <c r="C615" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
     </row>
     <row r="616" spans="3:3">
       <c r="C616" t="s">
-        <v>321</v>
+        <v>478</v>
       </c>
     </row>
     <row r="617" spans="3:3">
       <c r="C617" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="618" spans="3:3">
       <c r="C618" t="s">
-        <v>473</v>
+        <v>335</v>
       </c>
     </row>
     <row r="619" spans="3:3">
       <c r="C619" t="s">
-        <v>474</v>
+        <v>319</v>
       </c>
     </row>
     <row r="620" spans="3:3">
@@ -6981,547 +7027,467 @@
     </row>
     <row r="621" spans="3:3">
       <c r="C621" t="s">
-        <v>476</v>
+        <v>320</v>
       </c>
     </row>
     <row r="622" spans="3:3">
       <c r="C622" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="623" spans="3:3">
       <c r="C623" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="624" spans="3:3">
       <c r="C624" t="s">
-        <v>319</v>
+        <v>479</v>
       </c>
     </row>
     <row r="625" spans="3:3">
       <c r="C625" t="s">
-        <v>478</v>
+        <v>316</v>
       </c>
     </row>
     <row r="626" spans="3:3">
       <c r="C626" t="s">
-        <v>320</v>
+        <v>480</v>
       </c>
     </row>
     <row r="627" spans="3:3">
       <c r="C627" t="s">
-        <v>321</v>
+        <v>473</v>
       </c>
     </row>
     <row r="628" spans="3:3">
       <c r="C628" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="629" spans="3:3">
       <c r="C629" t="s">
-        <v>479</v>
+        <v>335</v>
       </c>
     </row>
     <row r="630" spans="3:3">
       <c r="C630" t="s">
-        <v>474</v>
+        <v>319</v>
       </c>
     </row>
     <row r="631" spans="3:3">
       <c r="C631" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
     </row>
     <row r="632" spans="3:3">
       <c r="C632" t="s">
-        <v>481</v>
+        <v>320</v>
       </c>
     </row>
     <row r="633" spans="3:3">
       <c r="C633" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="634" spans="3:3">
       <c r="C634" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="635" spans="3:3">
       <c r="C635" t="s">
-        <v>319</v>
+        <v>481</v>
       </c>
     </row>
     <row r="636" spans="3:3">
       <c r="C636" t="s">
-        <v>478</v>
+        <v>316</v>
       </c>
     </row>
     <row r="637" spans="3:3">
       <c r="C637" t="s">
-        <v>320</v>
+        <v>482</v>
       </c>
     </row>
     <row r="638" spans="3:3">
       <c r="C638" t="s">
-        <v>321</v>
+        <v>478</v>
       </c>
     </row>
     <row r="639" spans="3:3">
       <c r="C639" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="640" spans="3:3">
       <c r="C640" t="s">
-        <v>482</v>
+        <v>335</v>
       </c>
     </row>
     <row r="641" spans="3:3">
       <c r="C641" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="642" spans="3:3">
       <c r="C642" t="s">
-        <v>483</v>
+        <v>475</v>
       </c>
     </row>
     <row r="643" spans="3:3">
       <c r="C643" t="s">
-        <v>476</v>
+        <v>320</v>
       </c>
     </row>
     <row r="644" spans="3:3">
       <c r="C644" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="645" spans="3:3">
       <c r="C645" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="646" spans="3:3">
       <c r="C646" t="s">
-        <v>319</v>
+        <v>483</v>
       </c>
     </row>
     <row r="647" spans="3:3">
       <c r="C647" t="s">
-        <v>478</v>
+        <v>316</v>
       </c>
     </row>
     <row r="648" spans="3:3">
       <c r="C648" t="s">
-        <v>320</v>
+        <v>484</v>
       </c>
     </row>
     <row r="649" spans="3:3">
       <c r="C649" t="s">
-        <v>321</v>
+        <v>485</v>
       </c>
     </row>
     <row r="650" spans="3:3">
       <c r="C650" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="651" spans="3:3">
       <c r="C651" t="s">
-        <v>484</v>
+        <v>335</v>
       </c>
     </row>
     <row r="652" spans="3:3">
       <c r="C652" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="653" spans="3:3">
       <c r="C653" t="s">
-        <v>485</v>
+        <v>475</v>
       </c>
     </row>
     <row r="654" spans="3:3">
       <c r="C654" t="s">
-        <v>481</v>
+        <v>320</v>
       </c>
     </row>
     <row r="655" spans="3:3">
       <c r="C655" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="656" spans="3:3">
       <c r="C656" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="657" spans="3:3">
       <c r="C657" t="s">
-        <v>319</v>
+        <v>486</v>
       </c>
     </row>
     <row r="658" spans="3:3">
       <c r="C658" t="s">
-        <v>478</v>
+        <v>334</v>
       </c>
     </row>
     <row r="659" spans="3:3">
       <c r="C659" t="s">
-        <v>320</v>
+        <v>487</v>
       </c>
     </row>
     <row r="660" spans="3:3">
       <c r="C660" t="s">
-        <v>321</v>
+        <v>488</v>
       </c>
     </row>
     <row r="661" spans="3:3">
       <c r="C661" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="662" spans="3:3">
       <c r="C662" t="s">
-        <v>486</v>
+        <v>335</v>
       </c>
     </row>
     <row r="663" spans="3:3">
       <c r="C663" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="664" spans="3:3">
       <c r="C664" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="665" spans="3:3">
       <c r="C665" t="s">
-        <v>488</v>
+        <v>320</v>
       </c>
     </row>
     <row r="666" spans="3:3">
       <c r="C666" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="667" spans="3:3">
       <c r="C667" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="668" spans="3:3">
       <c r="C668" t="s">
-        <v>319</v>
+        <v>490</v>
       </c>
     </row>
     <row r="669" spans="3:3">
       <c r="C669" t="s">
-        <v>478</v>
+        <v>427</v>
       </c>
     </row>
     <row r="670" spans="3:3">
       <c r="C670" t="s">
-        <v>320</v>
+        <v>491</v>
       </c>
     </row>
     <row r="671" spans="3:3">
       <c r="C671" t="s">
-        <v>321</v>
+        <v>492</v>
       </c>
     </row>
     <row r="672" spans="3:3">
       <c r="C672" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="673" spans="3:3">
       <c r="C673" t="s">
-        <v>489</v>
+        <v>335</v>
       </c>
     </row>
     <row r="674" spans="3:3">
       <c r="C674" t="s">
-        <v>334</v>
+        <v>319</v>
       </c>
     </row>
     <row r="675" spans="3:3">
       <c r="C675" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="676" spans="3:3">
       <c r="C676" t="s">
-        <v>491</v>
+        <v>320</v>
       </c>
     </row>
     <row r="677" spans="3:3">
       <c r="C677" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="678" spans="3:3">
       <c r="C678" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="679" spans="3:3">
       <c r="C679" t="s">
-        <v>319</v>
+        <v>493</v>
       </c>
     </row>
     <row r="680" spans="3:3">
       <c r="C680" t="s">
-        <v>492</v>
+        <v>427</v>
       </c>
     </row>
     <row r="681" spans="3:3">
       <c r="C681" t="s">
-        <v>320</v>
+        <v>494</v>
       </c>
     </row>
     <row r="682" spans="3:3">
       <c r="C682" t="s">
-        <v>321</v>
+        <v>495</v>
       </c>
     </row>
     <row r="683" spans="3:3">
       <c r="C683" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="684" spans="3:3">
       <c r="C684" t="s">
-        <v>493</v>
+        <v>335</v>
       </c>
     </row>
     <row r="685" spans="3:3">
       <c r="C685" t="s">
-        <v>430</v>
+        <v>319</v>
       </c>
     </row>
     <row r="686" spans="3:3">
       <c r="C686" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
     </row>
     <row r="687" spans="3:3">
       <c r="C687" t="s">
-        <v>495</v>
+        <v>320</v>
       </c>
     </row>
     <row r="688" spans="3:3">
       <c r="C688" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="689" spans="3:3">
       <c r="C689" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="690" spans="3:3">
       <c r="C690" t="s">
-        <v>319</v>
+        <v>496</v>
       </c>
     </row>
     <row r="691" spans="3:3">
       <c r="C691" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
     </row>
     <row r="692" spans="3:3">
       <c r="C692" t="s">
-        <v>320</v>
+        <v>498</v>
       </c>
     </row>
     <row r="693" spans="3:3">
       <c r="C693" t="s">
-        <v>321</v>
+        <v>499</v>
       </c>
     </row>
     <row r="694" spans="3:3">
       <c r="C694" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="695" spans="3:3">
       <c r="C695" t="s">
-        <v>496</v>
+        <v>335</v>
       </c>
     </row>
     <row r="696" spans="3:3">
       <c r="C696" t="s">
-        <v>430</v>
+        <v>319</v>
       </c>
     </row>
     <row r="697" spans="3:3">
       <c r="C697" t="s">
-        <v>497</v>
+        <v>489</v>
       </c>
     </row>
     <row r="698" spans="3:3">
       <c r="C698" t="s">
-        <v>498</v>
+        <v>320</v>
       </c>
     </row>
     <row r="699" spans="3:3">
       <c r="C699" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="700" spans="3:3">
       <c r="C700" t="s">
-        <v>336</v>
+        <v>315</v>
       </c>
     </row>
     <row r="701" spans="3:3">
       <c r="C701" t="s">
-        <v>319</v>
+        <v>500</v>
       </c>
     </row>
     <row r="702" spans="3:3">
       <c r="C702" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
     </row>
     <row r="703" spans="3:3">
       <c r="C703" t="s">
-        <v>320</v>
+        <v>501</v>
       </c>
     </row>
     <row r="704" spans="3:3">
       <c r="C704" t="s">
-        <v>321</v>
+        <v>502</v>
       </c>
     </row>
     <row r="705" spans="3:3">
       <c r="C705" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="706" spans="3:3">
       <c r="C706" t="s">
-        <v>499</v>
+        <v>335</v>
       </c>
     </row>
     <row r="707" spans="3:3">
       <c r="C707" t="s">
-        <v>500</v>
+        <v>319</v>
       </c>
     </row>
     <row r="708" spans="3:3">
       <c r="C708" t="s">
-        <v>501</v>
+        <v>489</v>
       </c>
     </row>
     <row r="709" spans="3:3">
       <c r="C709" t="s">
-        <v>502</v>
+        <v>320</v>
       </c>
     </row>
     <row r="710" spans="3:3">
       <c r="C710" t="s">
-        <v>477</v>
+        <v>503</v>
       </c>
     </row>
     <row r="711" spans="3:3">
       <c r="C711" t="s">
-        <v>336</v>
+        <v>504</v>
       </c>
     </row>
     <row r="712" spans="3:3">
       <c r="C712" t="s">
-        <v>319</v>
+        <v>505</v>
       </c>
     </row>
     <row r="713" spans="3:3">
       <c r="C713" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="714" spans="3:3">
-      <c r="C714" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="715" spans="3:3">
-      <c r="C715" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="716" spans="3:3">
-      <c r="C716" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="717" spans="3:3">
-      <c r="C717" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="718" spans="3:3">
-      <c r="C718" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="719" spans="3:3">
-      <c r="C719" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="720" spans="3:3">
-      <c r="C720" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="721" spans="3:3">
-      <c r="C721" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="722" spans="3:3">
-      <c r="C722" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="723" spans="3:3">
-      <c r="C723" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="724" spans="3:3">
-      <c r="C724" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="725" spans="3:3">
-      <c r="C725" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="726" spans="3:3">
-      <c r="C726" t="s">
         <v>506</v>
-      </c>
-    </row>
-    <row r="727" spans="3:3">
-      <c r="C727" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="728" spans="3:3">
-      <c r="C728" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="729" spans="3:3">
-      <c r="C729" t="s">
-        <v>509</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Update speaker regex to match new format and enhance conclusion extraction for CEO messages
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A51C6A-09D8-4E7A-B26D-0DE07BF21416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDA39DB-9185-43B4-A0D6-88F5204BF275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -28,8 +28,9 @@
     <sheet name="model一覧" sheetId="17" r:id="rId13"/>
     <sheet name="Gemini API reference" sheetId="12" r:id="rId14"/>
     <sheet name="Gemini Code Assist" sheetId="15" r:id="rId15"/>
-    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId16"/>
-    <sheet name="How to fix" sheetId="16" r:id="rId17"/>
+    <sheet name="Gemini Code Assist 2" sheetId="18" r:id="rId16"/>
+    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId17"/>
+    <sheet name="How to fix" sheetId="16" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="542">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="549">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2800,6 +2801,33 @@
   </si>
   <si>
     <t>Gemini 2.0 Flash</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Resources</t>
+  </si>
+  <si>
+    <t>Quotas and limits</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>割当と制限</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Page Summary</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ページ概要</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>This document outlines the quotas and system limits for using Gemini Code Assist and Gemini CLI.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>この文書では、Gemini Code Assist および Gemini CLI の使用に関するクォータとシステム制限について説明します。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3202,7 +3230,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46043</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3385,7 +3413,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46043</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -3598,7 +3626,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46043</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -7509,7 +7537,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46043</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -7708,7 +7736,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46043</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -7850,6 +7878,71 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D01CB6-001D-4D20-8CBB-FE510A056DBA}">
+  <dimension ref="B2:C9"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="34.625" customWidth="1"/>
+    <col min="3" max="3" width="37.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3">
+      <c r="B2" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3">
+      <c r="B3" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="B4" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3">
+      <c r="B5" s="5" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3">
+      <c r="B7" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="C7" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3">
+      <c r="B8" t="s">
+        <v>545</v>
+      </c>
+      <c r="C8" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" ht="56.25">
+      <c r="B9" s="1" t="s">
+        <v>547</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>548</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://developers.google.com/" xr:uid="{AB4DF198-4467-43BD-92E5-7F9CEA77AE2D}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://developers.google.com/products" xr:uid="{E0788B1D-CD47-4B9D-A222-F399F4097EB5}"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{59048891-D360-4985-8E21-C2F762568942}"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://developers.google.com/gemini-code-assist/resources/faqs" xr:uid="{B8E91675-F28D-4503-9C6B-4A96AC1B988B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
   <dimension ref="C3:E9"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -7942,7 +8035,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595742A4-FD4B-4501-B5BA-63CBD2F36625}">
   <dimension ref="C2:D7"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -8517,7 +8610,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46043</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
fix: Update default model and enhance model selection logic in EmergencyMeetingPage
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDA39DB-9185-43B4-A0D6-88F5204BF275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB37782E-C90E-42F8-B192-1C258494BD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="557">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2828,6 +2828,38 @@
   </si>
   <si>
     <t>この文書では、Gemini Code Assist および Gemini CLI の使用に関するクォータとシステム制限について説明します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Quotas represent the amount of a shared resource you can use, while system limits are fixed values.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>クォータは共有リソースの使用可能量を表すのに対し、システム制限は固定値です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist and Gemini CLI have quotas for local codebase awareness, code customization repositories, and requests per user per minute/day, which vary depending on the edition or license type.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist および Gemini CLI には、ローカルコードベースの認識、コードカスタマイズリポジトリ、およびユーザーごとの分単位/日単位のリクエスト数に関するクォータが設定されており、これらはエディションまたはライセンスタイプによって異なります。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Usage of Gemini Code Assist on GitHub has separate quotas for pull request reviews.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>GitHubにおけるGemini Code Assistの使用には、プルリクエストのレビュー用に別途クォータが設定されています。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Quotas for Gemini in BigQuery's code assistance features are the same as Gemini Code Assist, with additional quotas for advanced features based on BigQuery usage.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>BigQueryのコードアシスト機能におけるGeminiのクォータは、Gemini Code Assistと同じです。ただし、BigQueryの使用状況に基づく高度な機能については追加のクォータが適用されます。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -7879,11 +7911,11 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D01CB6-001D-4D20-8CBB-FE510A056DBA}">
-  <dimension ref="B2:C9"/>
+  <dimension ref="B2:C13"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="34.625" customWidth="1"/>
-    <col min="3" max="3" width="37.375" customWidth="1"/>
+    <col min="2" max="2" width="45.125" customWidth="1"/>
+    <col min="3" max="3" width="59.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3">
@@ -7928,6 +7960,38 @@
       </c>
       <c r="C9" s="1" t="s">
         <v>548</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" ht="37.5">
+      <c r="B10" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" ht="75">
+      <c r="B11" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" ht="37.5">
+      <c r="B12" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" ht="75">
+      <c r="B13" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Update Gemini API reference with new last updated date and enhance content generation section
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB37782E-C90E-42F8-B192-1C258494BD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01F30B0-272B-4A3F-B080-0AD399C13E9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1153" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="577">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2860,6 +2860,100 @@
   </si>
   <si>
     <t>BigQueryのコードアシスト機能におけるGeminiのクォータは、Gemini Code Assistと同じです。ただし、BigQueryの使用状況に基づく高度な機能については追加のクォータが適用されます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>This document lists the quotas and system limits that apply to your combined use of Gemini Code Assist and Gemini CLI.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>このドキュメントでは、Gemini Code Assist と Gemini CLI の併用におけるクォータとシステム制限を記載しています。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Note: Individual developers using the free version of Gemini Code Assist, Gemini Code Assist for individuals, can get access to higher daily model request limits by purchasing a subscription to Google AI Pro or Ultra. This will enable higher daily model request limits shared across Gemini Code Assist, Gemini CLI and agent mode. Learn more.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>注：Gemini Code Assistの無料版（個人向けGemini Code Assist）をご利用の個人開発者は、Google AI ProまたはUltraのサブスクリプションを購入することで、1日あたりのモデルリクエスト上限を引き上げることができます。これにより、Gemini Code Assist、Gemini CLI、エージェントモードで共有される1日あたりのモデルリクエスト上限が引き上げられます。詳細はこちら。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://ai.google.dev/api</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>The following is an example request with the API key included in the header:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>以下は、ヘッダーにAPIキーを含めたリクエストの例です：</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>curl "https://generativelanguage.googleapis.com/v1beta/models/gemini-2.5-flash:generateContent" \
+  -H "x-goog-api-key: $GEMINI_API_KEY" \
+  -H 'Content-Type: application/json' \
+  -X POST \
+  -d '{
+    "contents": [
+      {
+        "parts": [
+          {
+            "text": "Explain how AI works in a few words"
+          }
+        ]
+      }
+    ]
+  }'</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>For instructions on how to pass your key to the API using Gemini SDKs, see the Using Gemini API keys guide.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini SDKを使用してAPIにキーを渡す方法については、「Gemini APIキーの使用」ガイドを参照してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Content generation</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>コンテンツ生成</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>This is the central endpoint for sending prompts to the model.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>これはモデルにプロンプトを送信するための中央エンドポイントです。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>There are two endpoints for generating content, the key difference is how you receive the response:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>コンテンツ生成には2つのエンドポイントがあり、主な違いはレスポンスの受け取り方です：</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>generateContent (REST): Receives a request and provides a single response after the model has finished its entire generation.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>generateContent (REST): リクエストを受け取り、モデルの生成が完全に終了した後に単一のレスポンスを返します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>streamGenerateContent (SSE): Receives the exact same request, but the model streams back chunks of the response as they are generated. This provides a better user experience for interactive applications as it lets you display partial results immediately.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>streamGenerateContent (SSE): まったく同じリクエストを受け取りますが、モデルが生成されたレスポンスのチャンクをストリーミングで返します。これにより、部分的な結果を即座に表示できるため、インタラクティブなアプリケーションにおいて優れたユーザー体験を提供します。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -7558,7 +7652,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E27"/>
+  <dimension ref="B1:E38"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="42.5" customWidth="1"/>
@@ -7573,191 +7667,278 @@
       </c>
     </row>
     <row r="2" spans="2:5">
-      <c r="B2" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="B2" s="2" t="s">
+        <v>561</v>
+      </c>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="5" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="5" t="s">
         <v>53</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5">
-      <c r="B6" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" t="s">
         <v>56</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="56.25">
-      <c r="B8" s="1" t="s">
+    <row r="9" spans="2:5" ht="56.25">
+      <c r="B9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" ht="37.5">
-      <c r="B9" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="37.5">
+      <c r="B11" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="75">
-      <c r="B11" s="1" t="s">
+    <row r="12" spans="2:5" ht="75">
+      <c r="B12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="13" spans="2:5">
-      <c r="B13" s="1" t="s">
+      <c r="E12" s="3"/>
+    </row>
+    <row r="14" spans="2:5">
+      <c r="B14" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="2:5" ht="37.5">
-      <c r="B15" s="1" t="s">
+    <row r="16" spans="2:5" ht="37.5">
+      <c r="B16" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="93.75">
-      <c r="B17" s="1" t="s">
+    <row r="18" spans="2:5" ht="93.75">
+      <c r="B18" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="2:5" ht="112.5">
-      <c r="B18" s="1" t="s">
+      <c r="E18" s="3"/>
+    </row>
+    <row r="19" spans="2:5" ht="112.5">
+      <c r="B19" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" spans="2:5" ht="75">
-      <c r="B19" s="1" t="s">
+      <c r="E19" s="3"/>
+    </row>
+    <row r="20" spans="2:5" ht="75">
+      <c r="B20" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E19" s="3">
+      <c r="E20" s="3">
         <v>46037</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" ht="56.25">
-      <c r="B20" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="E20" s="3">
-        <v>46038</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="56.25">
       <c r="B21" s="1" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="E21" s="3">
         <v>46038</v>
       </c>
     </row>
-    <row r="22" spans="2:5" ht="93.75">
+    <row r="22" spans="2:5" ht="56.25">
       <c r="B22" s="1" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>125</v>
+        <v>90</v>
       </c>
       <c r="E22" s="3">
         <v>46038</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="56.25">
+    <row r="23" spans="2:5" ht="93.75">
       <c r="B23" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="E23" s="3">
+        <v>46038</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" ht="56.25">
+      <c r="B24" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C24" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E24" s="3">
         <v>46039</v>
       </c>
     </row>
-    <row r="25" spans="2:5">
-      <c r="B25" s="1" t="s">
+    <row r="26" spans="2:5">
+      <c r="B26" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C26" s="1" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="27" spans="2:5" ht="56.25">
-      <c r="B27" s="1" t="s">
+    <row r="28" spans="2:5" ht="56.25">
+      <c r="B28" s="1" t="s">
         <v>294</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C28" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E28" s="3">
         <v>46039</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" ht="37.5">
+      <c r="B29" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="E29" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" ht="337.5">
+      <c r="B30" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" ht="56.25">
+      <c r="B31" s="1" t="s">
+        <v>565</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="E31" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5">
+      <c r="B33" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="E33" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" ht="37.5">
+      <c r="B35" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" ht="56.25">
+      <c r="B36" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="E36" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" ht="56.25">
+      <c r="B37" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="E37" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" ht="112.5">
+      <c r="B38" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="E38" s="3">
+        <v>46043</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://ai.google.dev/" xr:uid="{D6844177-6821-498C-95D2-F6B6D63F1D22}"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://ai.google.dev/gemini-api" xr:uid="{2CDC8D53-0630-4185-9E29-7B79EBBE1F53}"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://ai.google.dev/api" xr:uid="{4A9752DB-169C-4F26-B3F6-A0018804884D}"/>
+    <hyperlink ref="B3" r:id="rId1" display="https://ai.google.dev/" xr:uid="{D6844177-6821-498C-95D2-F6B6D63F1D22}"/>
+    <hyperlink ref="B4" r:id="rId2" display="https://ai.google.dev/gemini-api" xr:uid="{2CDC8D53-0630-4185-9E29-7B79EBBE1F53}"/>
+    <hyperlink ref="B5" r:id="rId3" display="https://ai.google.dev/api" xr:uid="{4A9752DB-169C-4F26-B3F6-A0018804884D}"/>
+    <hyperlink ref="B2" r:id="rId4" xr:uid="{47EA1D9B-75C8-4CFC-95C8-B5BD7FE04536}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E19"/>
+  <dimension ref="B1:E20"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="73.125" customWidth="1"/>
@@ -7872,7 +8053,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="17" spans="2:3">
+    <row r="17" spans="2:5">
       <c r="B17" s="1" t="s">
         <v>230</v>
       </c>
@@ -7880,7 +8061,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="18" spans="2:3">
+    <row r="18" spans="2:5">
       <c r="B18" s="1" t="s">
         <v>232</v>
       </c>
@@ -7888,12 +8069,23 @@
         <v>233</v>
       </c>
     </row>
-    <row r="19" spans="2:3">
+    <row r="19" spans="2:5">
       <c r="B19" s="1" t="s">
         <v>234</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>235</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="93.75">
+      <c r="B20" s="1" t="s">
+        <v>559</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="E20" s="3">
+        <v>46043</v>
       </c>
     </row>
   </sheetData>
@@ -7911,34 +8103,41 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D01CB6-001D-4D20-8CBB-FE510A056DBA}">
-  <dimension ref="B2:C13"/>
+  <dimension ref="B1:E14"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="45.125" customWidth="1"/>
     <col min="3" max="3" width="59.5" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3">
+    <row r="1" spans="2:5">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5">
       <c r="B2" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="2:3">
+    <row r="3" spans="2:5">
       <c r="B3" s="5" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="4" spans="2:3">
+    <row r="4" spans="2:5">
       <c r="B4" s="5" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="5" spans="2:3">
+    <row r="5" spans="2:5">
       <c r="B5" s="5" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="7" spans="2:3">
+    <row r="7" spans="2:5">
       <c r="B7" s="1" t="s">
         <v>543</v>
       </c>
@@ -7946,7 +8145,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="8" spans="2:3">
+    <row r="8" spans="2:5">
       <c r="B8" t="s">
         <v>545</v>
       </c>
@@ -7954,7 +8153,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="9" spans="2:3" ht="56.25">
+    <row r="9" spans="2:5" ht="56.25">
       <c r="B9" s="1" t="s">
         <v>547</v>
       </c>
@@ -7962,7 +8161,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="37.5">
+    <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
         <v>549</v>
       </c>
@@ -7970,7 +8169,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="11" spans="2:3" ht="75">
+    <row r="11" spans="2:5" ht="75">
       <c r="B11" s="1" t="s">
         <v>551</v>
       </c>
@@ -7978,7 +8177,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="12" spans="2:3" ht="37.5">
+    <row r="12" spans="2:5" ht="37.5">
       <c r="B12" s="1" t="s">
         <v>553</v>
       </c>
@@ -7986,12 +8185,26 @@
         <v>554</v>
       </c>
     </row>
-    <row r="13" spans="2:3" ht="75">
+    <row r="13" spans="2:5" ht="75">
       <c r="B13" s="1" t="s">
         <v>555</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>556</v>
+      </c>
+      <c r="E13" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="56.25">
+      <c r="B14" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="E14" s="3">
+        <v>46043</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Update URLs in Gemini University V2 Page to include markdown formatting for better readability
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E01F30B0-272B-4A3F-B080-0AD399C13E9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424128D5-CBF3-4B2B-8F91-0BC46933C822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1173" uniqueCount="577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="576">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2154,9 +2154,6 @@
     <t xml:space="preserve">      "maxTemperature": 2</t>
   </si>
   <si>
-    <t xml:space="preserve">      "description": "Gemini 2.0 Flash",</t>
-  </si>
-  <si>
     <t xml:space="preserve">      "name": "models/gemini-2.0-flash-001",</t>
   </si>
   <si>
@@ -2784,19 +2781,7 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t xml:space="preserve">      "name": "models/gemini-2.0-flash",</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>models/gemini-2.0-flash</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">      "version": "2.0",</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash",</t>
     <phoneticPr fontId="1"/>
   </si>
   <si>
@@ -2954,6 +2939,18 @@
   </si>
   <si>
     <t>streamGenerateContent (SSE): まったく同じリクエストを受け取りますが、モデルが生成されたレスポンスのチャンクをストリーミングで返します。これにより、部分的な結果を即座に表示できるため、インタラクティブなアプリケーションにおいて優れたユーザー体験を提供します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ジェミニ2.0 フラッシュ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>You can use Gemini Code Assist in supported IDEs, such as VS Code, JetBrains IDEs, or Android Studio, for AI-powered coding assistance in many popular languages.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assistは、VS Code、JetBrains IDE、Android Studioなどの対応IDEで利用でき、多くの主要言語においてAIを活用したコーディング支援を提供します。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3356,7 +3353,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
+        <v>46044</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3539,7 +3536,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
+        <v>46044</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -3752,7 +3749,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
+        <v>46044</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3904,9 +3901,10 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F96D129-34E8-4B10-A261-7AEE00EA03AD}">
-  <dimension ref="C2:Q713"/>
+  <dimension ref="B1:Q695"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="29.375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="47.625" bestFit="1" customWidth="1"/>
@@ -3918,59 +3916,65 @@
     <col min="16" max="16" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:17">
+    <row r="1" spans="2:17">
+      <c r="B1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46044</v>
+      </c>
+    </row>
+    <row r="2" spans="2:17">
       <c r="E2" t="s">
+        <v>506</v>
+      </c>
+      <c r="F2" t="s">
+        <v>508</v>
+      </c>
+      <c r="G2" t="s">
+        <v>509</v>
+      </c>
+      <c r="H2" t="s">
+        <v>511</v>
+      </c>
+      <c r="J2" t="s">
+        <v>513</v>
+      </c>
+      <c r="K2" t="s">
+        <v>514</v>
+      </c>
+      <c r="L2" t="s">
+        <v>515</v>
+      </c>
+      <c r="M2" t="s">
+        <v>523</v>
+      </c>
+      <c r="N2" t="s">
+        <v>524</v>
+      </c>
+      <c r="O2" t="s">
+        <v>525</v>
+      </c>
+      <c r="P2" t="s">
+        <v>526</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="3" spans="2:17" ht="37.5">
+      <c r="E3" t="s">
         <v>507</v>
-      </c>
-      <c r="F2" t="s">
-        <v>509</v>
-      </c>
-      <c r="G2" t="s">
-        <v>510</v>
-      </c>
-      <c r="H2" t="s">
-        <v>512</v>
-      </c>
-      <c r="J2" t="s">
-        <v>514</v>
-      </c>
-      <c r="K2" t="s">
-        <v>515</v>
-      </c>
-      <c r="L2" t="s">
-        <v>516</v>
-      </c>
-      <c r="M2" t="s">
-        <v>524</v>
-      </c>
-      <c r="N2" t="s">
-        <v>525</v>
-      </c>
-      <c r="O2" t="s">
-        <v>526</v>
-      </c>
-      <c r="P2" t="s">
-        <v>527</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="3" spans="3:17" ht="37.5">
-      <c r="E3" t="s">
-        <v>508</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H3" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="I3" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="J3">
         <v>1024</v>
@@ -3979,24 +3983,24 @@
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="4" spans="2:17" ht="75">
+      <c r="E4" t="s">
         <v>517</v>
-      </c>
-    </row>
-    <row r="4" spans="3:17" ht="75">
-      <c r="E4" t="s">
-        <v>518</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
+        <v>518</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>519</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>520</v>
-      </c>
       <c r="I4" s="1" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="J4">
         <v>1048576</v>
@@ -4005,7 +4009,7 @@
         <v>65536</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -4023,21 +4027,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="3:17" ht="75">
+    <row r="5" spans="2:17" ht="75">
       <c r="E5" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F5">
         <v>2.5</v>
       </c>
       <c r="G5" t="s">
+        <v>529</v>
+      </c>
+      <c r="H5" t="s">
         <v>530</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>531</v>
-      </c>
-      <c r="I5" t="s">
-        <v>532</v>
       </c>
       <c r="J5">
         <v>1048576</v>
@@ -4046,7 +4050,7 @@
         <v>65536</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -4064,21 +4068,21 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:17" ht="56.25">
+    <row r="6" spans="2:17" ht="56.25">
       <c r="E6" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" t="s">
+        <v>533</v>
+      </c>
+      <c r="H6" t="s">
+        <v>533</v>
+      </c>
+      <c r="I6" t="s">
         <v>534</v>
-      </c>
-      <c r="H6" t="s">
-        <v>534</v>
-      </c>
-      <c r="I6" t="s">
-        <v>535</v>
       </c>
       <c r="J6">
         <v>1048576</v>
@@ -4087,7 +4091,7 @@
         <v>8192</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -4102,59 +4106,88 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="3:17">
+    <row r="7" spans="2:17" ht="75">
+      <c r="B7" s="3">
+        <v>46043</v>
+      </c>
       <c r="E7" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>541</v>
-      </c>
-      <c r="L7" s="1"/>
-    </row>
-    <row r="8" spans="3:17">
+        <v>537</v>
+      </c>
+      <c r="H7" t="s">
+        <v>537</v>
+      </c>
+      <c r="I7" t="s">
+        <v>573</v>
+      </c>
+      <c r="J7">
+        <v>1048576</v>
+      </c>
+      <c r="K7">
+        <v>8192</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+      <c r="N7">
+        <v>0.95</v>
+      </c>
+      <c r="O7">
+        <v>40</v>
+      </c>
+      <c r="P7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:17">
       <c r="C8" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="9" spans="3:17">
+    <row r="9" spans="2:17">
       <c r="C9" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="10" spans="3:17">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="10" spans="2:17">
       <c r="C10" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="11" spans="3:17">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17">
       <c r="C11" t="s">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="12" spans="3:17">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="12" spans="2:17">
       <c r="C12" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="13" spans="3:17">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17">
       <c r="C13" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="14" spans="3:17">
+    <row r="14" spans="2:17">
       <c r="C14" t="s">
         <v>335</v>
       </c>
     </row>
-    <row r="15" spans="3:17">
+    <row r="15" spans="2:17">
       <c r="C15" t="s">
         <v>319</v>
       </c>
     </row>
-    <row r="16" spans="3:17">
+    <row r="16" spans="2:17">
       <c r="C16" t="s">
         <v>324</v>
       </c>
@@ -4211,7 +4244,7 @@
     </row>
     <row r="27" spans="3:3">
       <c r="C27" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
     </row>
     <row r="28" spans="3:3">
@@ -4221,12 +4254,12 @@
     </row>
     <row r="29" spans="3:3">
       <c r="C29" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="30" spans="3:3">
       <c r="C30" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
     </row>
     <row r="31" spans="3:3">
@@ -4256,97 +4289,97 @@
     </row>
     <row r="36" spans="3:3">
       <c r="C36" t="s">
-        <v>326</v>
+        <v>336</v>
       </c>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="38" spans="3:3">
       <c r="C38" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="40" spans="3:3">
       <c r="C40" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="42" spans="3:3">
       <c r="C42" t="s">
-        <v>338</v>
+        <v>321</v>
       </c>
     </row>
     <row r="43" spans="3:3">
       <c r="C43" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="44" spans="3:3">
       <c r="C44" t="s">
-        <v>315</v>
+        <v>345</v>
       </c>
     </row>
     <row r="45" spans="3:3">
       <c r="C45" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
     </row>
     <row r="46" spans="3:3">
       <c r="C46" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
     </row>
     <row r="47" spans="3:3">
       <c r="C47" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
     </row>
     <row r="48" spans="3:3">
       <c r="C48" t="s">
-        <v>345</v>
+        <v>322</v>
       </c>
     </row>
     <row r="49" spans="3:3">
       <c r="C49" t="s">
-        <v>322</v>
+        <v>335</v>
       </c>
     </row>
     <row r="50" spans="3:3">
       <c r="C50" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
     </row>
     <row r="51" spans="3:3">
       <c r="C51" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="52" spans="3:3">
       <c r="C52" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="53" spans="3:3">
       <c r="C53" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="54" spans="3:3">
       <c r="C54" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
     </row>
     <row r="55" spans="3:3">
@@ -4386,7 +4419,7 @@
     </row>
     <row r="62" spans="3:3">
       <c r="C62" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="63" spans="3:3">
@@ -4396,12 +4429,12 @@
     </row>
     <row r="64" spans="3:3">
       <c r="C64" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="65" spans="3:3">
       <c r="C65" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
     </row>
     <row r="66" spans="3:3">
@@ -4476,22 +4509,22 @@
     </row>
     <row r="80" spans="3:3">
       <c r="C80" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="81" spans="3:3">
       <c r="C81" t="s">
-        <v>334</v>
+        <v>352</v>
       </c>
     </row>
     <row r="82" spans="3:3">
       <c r="C82" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="83" spans="3:3">
       <c r="C83" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="84" spans="3:3">
@@ -4566,22 +4599,22 @@
     </row>
     <row r="98" spans="3:3">
       <c r="C98" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="99" spans="3:3">
       <c r="C99" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="100" spans="3:3">
       <c r="C100" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="101" spans="3:3">
       <c r="C101" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="102" spans="3:3">
@@ -4656,22 +4689,22 @@
     </row>
     <row r="116" spans="3:3">
       <c r="C116" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="117" spans="3:3">
       <c r="C117" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
     </row>
     <row r="118" spans="3:3">
       <c r="C118" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
     </row>
     <row r="119" spans="3:3">
       <c r="C119" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
     </row>
     <row r="120" spans="3:3">
@@ -4681,7 +4714,7 @@
     </row>
     <row r="121" spans="3:3">
       <c r="C121" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
     </row>
     <row r="122" spans="3:3">
@@ -4726,62 +4759,62 @@
     </row>
     <row r="130" spans="3:3">
       <c r="C130" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="131" spans="3:3">
       <c r="C131" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
     </row>
     <row r="132" spans="3:3">
       <c r="C132" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="133" spans="3:3">
       <c r="C133" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="134" spans="3:3">
       <c r="C134" t="s">
-        <v>358</v>
+        <v>315</v>
       </c>
     </row>
     <row r="135" spans="3:3">
       <c r="C135" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
     </row>
     <row r="136" spans="3:3">
       <c r="C136" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="137" spans="3:3">
       <c r="C137" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
     </row>
     <row r="138" spans="3:3">
       <c r="C138" t="s">
-        <v>322</v>
+        <v>364</v>
       </c>
     </row>
     <row r="139" spans="3:3">
       <c r="C139" t="s">
-        <v>323</v>
+        <v>365</v>
       </c>
     </row>
     <row r="140" spans="3:3">
       <c r="C140" t="s">
-        <v>319</v>
+        <v>366</v>
       </c>
     </row>
     <row r="141" spans="3:3">
       <c r="C141" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="142" spans="3:3">
@@ -4791,232 +4824,232 @@
     </row>
     <row r="143" spans="3:3">
       <c r="C143" t="s">
-        <v>326</v>
+        <v>367</v>
       </c>
     </row>
     <row r="144" spans="3:3">
       <c r="C144" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="145" spans="3:3">
       <c r="C145" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="146" spans="3:3">
       <c r="C146" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="147" spans="3:3">
       <c r="C147" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="148" spans="3:3">
       <c r="C148" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="149" spans="3:3">
       <c r="C149" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
     </row>
     <row r="150" spans="3:3">
       <c r="C150" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
     </row>
     <row r="151" spans="3:3">
       <c r="C151" t="s">
-        <v>321</v>
+        <v>368</v>
       </c>
     </row>
     <row r="152" spans="3:3">
       <c r="C152" t="s">
-        <v>315</v>
+        <v>369</v>
       </c>
     </row>
     <row r="153" spans="3:3">
       <c r="C153" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
     </row>
     <row r="154" spans="3:3">
       <c r="C154" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
     </row>
     <row r="155" spans="3:3">
       <c r="C155" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
     </row>
     <row r="156" spans="3:3">
       <c r="C156" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="157" spans="3:3">
       <c r="C157" t="s">
-        <v>366</v>
+        <v>319</v>
       </c>
     </row>
     <row r="158" spans="3:3">
       <c r="C158" t="s">
-        <v>367</v>
+        <v>325</v>
       </c>
     </row>
     <row r="159" spans="3:3">
       <c r="C159" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="160" spans="3:3">
       <c r="C160" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="161" spans="3:3">
       <c r="C161" t="s">
-        <v>368</v>
+        <v>328</v>
       </c>
     </row>
     <row r="162" spans="3:3">
       <c r="C162" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="163" spans="3:3">
       <c r="C163" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="164" spans="3:3">
       <c r="C164" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="165" spans="3:3">
       <c r="C165" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="166" spans="3:3">
       <c r="C166" t="s">
-        <v>338</v>
+        <v>321</v>
       </c>
     </row>
     <row r="167" spans="3:3">
       <c r="C167" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="168" spans="3:3">
       <c r="C168" t="s">
-        <v>315</v>
+        <v>372</v>
       </c>
     </row>
     <row r="169" spans="3:3">
       <c r="C169" t="s">
-        <v>369</v>
+        <v>316</v>
       </c>
     </row>
     <row r="170" spans="3:3">
       <c r="C170" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="171" spans="3:3">
       <c r="C171" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="172" spans="3:3">
       <c r="C172" t="s">
-        <v>372</v>
+        <v>335</v>
       </c>
     </row>
     <row r="173" spans="3:3">
       <c r="C173" t="s">
-        <v>366</v>
+        <v>319</v>
       </c>
     </row>
     <row r="174" spans="3:3">
       <c r="C174" t="s">
-        <v>367</v>
+        <v>324</v>
       </c>
     </row>
     <row r="175" spans="3:3">
       <c r="C175" t="s">
-        <v>319</v>
+        <v>375</v>
       </c>
     </row>
     <row r="176" spans="3:3">
       <c r="C176" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="177" spans="3:3">
       <c r="C177" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="178" spans="3:3">
       <c r="C178" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="179" spans="3:3">
       <c r="C179" t="s">
-        <v>328</v>
+        <v>376</v>
       </c>
     </row>
     <row r="180" spans="3:3">
       <c r="C180" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
     </row>
     <row r="181" spans="3:3">
       <c r="C181" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="182" spans="3:3">
       <c r="C182" t="s">
-        <v>331</v>
+        <v>377</v>
       </c>
     </row>
     <row r="183" spans="3:3">
       <c r="C183" t="s">
-        <v>338</v>
+        <v>316</v>
       </c>
     </row>
     <row r="184" spans="3:3">
       <c r="C184" t="s">
-        <v>321</v>
+        <v>378</v>
       </c>
     </row>
     <row r="185" spans="3:3">
       <c r="C185" t="s">
-        <v>315</v>
+        <v>374</v>
       </c>
     </row>
     <row r="186" spans="3:3">
       <c r="C186" t="s">
-        <v>373</v>
+        <v>335</v>
       </c>
     </row>
     <row r="187" spans="3:3">
       <c r="C187" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="188" spans="3:3">
       <c r="C188" t="s">
-        <v>374</v>
+        <v>324</v>
       </c>
     </row>
     <row r="189" spans="3:3">
@@ -5026,17 +5059,17 @@
     </row>
     <row r="190" spans="3:3">
       <c r="C190" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="191" spans="3:3">
       <c r="C191" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="192" spans="3:3">
       <c r="C192" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="193" spans="3:3">
@@ -5046,47 +5079,47 @@
     </row>
     <row r="194" spans="3:3">
       <c r="C194" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="195" spans="3:3">
       <c r="C195" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="196" spans="3:3">
       <c r="C196" t="s">
-        <v>330</v>
+        <v>379</v>
       </c>
     </row>
     <row r="197" spans="3:3">
       <c r="C197" t="s">
-        <v>377</v>
+        <v>316</v>
       </c>
     </row>
     <row r="198" spans="3:3">
       <c r="C198" t="s">
-        <v>321</v>
+        <v>380</v>
       </c>
     </row>
     <row r="199" spans="3:3">
       <c r="C199" t="s">
-        <v>315</v>
+        <v>374</v>
       </c>
     </row>
     <row r="200" spans="3:3">
       <c r="C200" t="s">
-        <v>378</v>
+        <v>335</v>
       </c>
     </row>
     <row r="201" spans="3:3">
       <c r="C201" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="202" spans="3:3">
       <c r="C202" t="s">
-        <v>379</v>
+        <v>324</v>
       </c>
     </row>
     <row r="203" spans="3:3">
@@ -5096,17 +5129,17 @@
     </row>
     <row r="204" spans="3:3">
       <c r="C204" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="205" spans="3:3">
       <c r="C205" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="206" spans="3:3">
       <c r="C206" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="207" spans="3:3">
@@ -5116,47 +5149,47 @@
     </row>
     <row r="208" spans="3:3">
       <c r="C208" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="209" spans="3:3">
       <c r="C209" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="210" spans="3:3">
       <c r="C210" t="s">
-        <v>330</v>
+        <v>381</v>
       </c>
     </row>
     <row r="211" spans="3:3">
       <c r="C211" t="s">
-        <v>377</v>
+        <v>316</v>
       </c>
     </row>
     <row r="212" spans="3:3">
       <c r="C212" t="s">
-        <v>321</v>
+        <v>382</v>
       </c>
     </row>
     <row r="213" spans="3:3">
       <c r="C213" t="s">
-        <v>315</v>
+        <v>383</v>
       </c>
     </row>
     <row r="214" spans="3:3">
       <c r="C214" t="s">
-        <v>380</v>
+        <v>335</v>
       </c>
     </row>
     <row r="215" spans="3:3">
       <c r="C215" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="216" spans="3:3">
       <c r="C216" t="s">
-        <v>381</v>
+        <v>324</v>
       </c>
     </row>
     <row r="217" spans="3:3">
@@ -5166,17 +5199,17 @@
     </row>
     <row r="218" spans="3:3">
       <c r="C218" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="219" spans="3:3">
       <c r="C219" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="220" spans="3:3">
       <c r="C220" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="221" spans="3:3">
@@ -5186,67 +5219,67 @@
     </row>
     <row r="222" spans="3:3">
       <c r="C222" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="223" spans="3:3">
       <c r="C223" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="224" spans="3:3">
       <c r="C224" t="s">
-        <v>330</v>
+        <v>384</v>
       </c>
     </row>
     <row r="225" spans="3:3">
       <c r="C225" t="s">
-        <v>377</v>
+        <v>316</v>
       </c>
     </row>
     <row r="226" spans="3:3">
       <c r="C226" t="s">
-        <v>321</v>
+        <v>385</v>
       </c>
     </row>
     <row r="227" spans="3:3">
       <c r="C227" t="s">
-        <v>315</v>
+        <v>365</v>
       </c>
     </row>
     <row r="228" spans="3:3">
       <c r="C228" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
     </row>
     <row r="229" spans="3:3">
       <c r="C229" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="230" spans="3:3">
       <c r="C230" t="s">
-        <v>383</v>
+        <v>324</v>
       </c>
     </row>
     <row r="231" spans="3:3">
       <c r="C231" t="s">
-        <v>384</v>
+        <v>375</v>
       </c>
     </row>
     <row r="232" spans="3:3">
       <c r="C232" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="233" spans="3:3">
       <c r="C233" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="234" spans="3:3">
       <c r="C234" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="235" spans="3:3">
@@ -5256,67 +5289,67 @@
     </row>
     <row r="236" spans="3:3">
       <c r="C236" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="237" spans="3:3">
       <c r="C237" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="238" spans="3:3">
       <c r="C238" t="s">
-        <v>330</v>
+        <v>387</v>
       </c>
     </row>
     <row r="239" spans="3:3">
       <c r="C239" t="s">
-        <v>377</v>
+        <v>316</v>
       </c>
     </row>
     <row r="240" spans="3:3">
       <c r="C240" t="s">
-        <v>321</v>
+        <v>388</v>
       </c>
     </row>
     <row r="241" spans="3:3">
       <c r="C241" t="s">
-        <v>315</v>
+        <v>365</v>
       </c>
     </row>
     <row r="242" spans="3:3">
       <c r="C242" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="243" spans="3:3">
       <c r="C243" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="244" spans="3:3">
       <c r="C244" t="s">
-        <v>386</v>
+        <v>324</v>
       </c>
     </row>
     <row r="245" spans="3:3">
       <c r="C245" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
     </row>
     <row r="246" spans="3:3">
       <c r="C246" t="s">
-        <v>387</v>
+        <v>328</v>
       </c>
     </row>
     <row r="247" spans="3:3">
       <c r="C247" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="248" spans="3:3">
       <c r="C248" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="249" spans="3:3">
@@ -5326,437 +5359,437 @@
     </row>
     <row r="250" spans="3:3">
       <c r="C250" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="251" spans="3:3">
       <c r="C251" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="252" spans="3:3">
       <c r="C252" t="s">
-        <v>330</v>
+        <v>389</v>
       </c>
     </row>
     <row r="253" spans="3:3">
       <c r="C253" t="s">
-        <v>377</v>
+        <v>390</v>
       </c>
     </row>
     <row r="254" spans="3:3">
       <c r="C254" t="s">
-        <v>321</v>
+        <v>391</v>
       </c>
     </row>
     <row r="255" spans="3:3">
       <c r="C255" t="s">
-        <v>315</v>
+        <v>392</v>
       </c>
     </row>
     <row r="256" spans="3:3">
       <c r="C256" t="s">
-        <v>388</v>
+        <v>322</v>
       </c>
     </row>
     <row r="257" spans="3:3">
       <c r="C257" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
     </row>
     <row r="258" spans="3:3">
       <c r="C258" t="s">
-        <v>389</v>
+        <v>319</v>
       </c>
     </row>
     <row r="259" spans="3:3">
       <c r="C259" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
     </row>
     <row r="260" spans="3:3">
       <c r="C260" t="s">
-        <v>387</v>
+        <v>325</v>
       </c>
     </row>
     <row r="261" spans="3:3">
       <c r="C261" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="262" spans="3:3">
       <c r="C262" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="263" spans="3:3">
       <c r="C263" t="s">
-        <v>376</v>
+        <v>328</v>
       </c>
     </row>
     <row r="264" spans="3:3">
       <c r="C264" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="265" spans="3:3">
       <c r="C265" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="266" spans="3:3">
       <c r="C266" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="267" spans="3:3">
       <c r="C267" t="s">
-        <v>377</v>
+        <v>332</v>
       </c>
     </row>
     <row r="268" spans="3:3">
       <c r="C268" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="269" spans="3:3">
       <c r="C269" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="270" spans="3:3">
       <c r="C270" t="s">
-        <v>390</v>
+        <v>315</v>
       </c>
     </row>
     <row r="271" spans="3:3">
       <c r="C271" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="272" spans="3:3">
       <c r="C272" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="273" spans="3:3">
       <c r="C273" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="274" spans="3:3">
       <c r="C274" t="s">
-        <v>322</v>
+        <v>396</v>
       </c>
     </row>
     <row r="275" spans="3:3">
       <c r="C275" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="276" spans="3:3">
       <c r="C276" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="277" spans="3:3">
       <c r="C277" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="278" spans="3:3">
       <c r="C278" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="279" spans="3:3">
       <c r="C279" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="280" spans="3:3">
       <c r="C280" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="281" spans="3:3">
       <c r="C281" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="282" spans="3:3">
       <c r="C282" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="283" spans="3:3">
       <c r="C283" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="284" spans="3:3">
       <c r="C284" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="285" spans="3:3">
       <c r="C285" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="286" spans="3:3">
       <c r="C286" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="287" spans="3:3">
       <c r="C287" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="288" spans="3:3">
       <c r="C288" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="289" spans="3:3">
       <c r="C289" t="s">
-        <v>394</v>
+        <v>315</v>
       </c>
     </row>
     <row r="290" spans="3:3">
       <c r="C290" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="291" spans="3:3">
       <c r="C291" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="292" spans="3:3">
       <c r="C292" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="293" spans="3:3">
       <c r="C293" t="s">
-        <v>322</v>
+        <v>400</v>
       </c>
     </row>
     <row r="294" spans="3:3">
       <c r="C294" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="295" spans="3:3">
       <c r="C295" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="296" spans="3:3">
       <c r="C296" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="297" spans="3:3">
       <c r="C297" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="298" spans="3:3">
       <c r="C298" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="299" spans="3:3">
       <c r="C299" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="300" spans="3:3">
       <c r="C300" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="301" spans="3:3">
       <c r="C301" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="302" spans="3:3">
       <c r="C302" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="303" spans="3:3">
       <c r="C303" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="304" spans="3:3">
       <c r="C304" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="305" spans="3:3">
       <c r="C305" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="306" spans="3:3">
       <c r="C306" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="307" spans="3:3">
       <c r="C307" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="308" spans="3:3">
       <c r="C308" t="s">
-        <v>398</v>
+        <v>315</v>
       </c>
     </row>
     <row r="309" spans="3:3">
       <c r="C309" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="310" spans="3:3">
       <c r="C310" t="s">
-        <v>400</v>
+        <v>316</v>
       </c>
     </row>
     <row r="311" spans="3:3">
       <c r="C311" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="312" spans="3:3">
       <c r="C312" t="s">
-        <v>322</v>
+        <v>403</v>
       </c>
     </row>
     <row r="313" spans="3:3">
       <c r="C313" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="314" spans="3:3">
       <c r="C314" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="315" spans="3:3">
       <c r="C315" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="316" spans="3:3">
       <c r="C316" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="317" spans="3:3">
       <c r="C317" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="318" spans="3:3">
       <c r="C318" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="319" spans="3:3">
       <c r="C319" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="320" spans="3:3">
       <c r="C320" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="321" spans="3:3">
       <c r="C321" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="322" spans="3:3">
       <c r="C322" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="323" spans="3:3">
       <c r="C323" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="324" spans="3:3">
       <c r="C324" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="325" spans="3:3">
       <c r="C325" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="326" spans="3:3">
       <c r="C326" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="327" spans="3:3">
       <c r="C327" t="s">
-        <v>402</v>
+        <v>315</v>
       </c>
     </row>
     <row r="328" spans="3:3">
       <c r="C328" t="s">
-        <v>316</v>
+        <v>404</v>
       </c>
     </row>
     <row r="329" spans="3:3">
       <c r="C329" t="s">
-        <v>403</v>
+        <v>334</v>
       </c>
     </row>
     <row r="330" spans="3:3">
       <c r="C330" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="331" spans="3:3">
       <c r="C331" t="s">
-        <v>322</v>
+        <v>406</v>
       </c>
     </row>
     <row r="332" spans="3:3">
       <c r="C332" t="s">
-        <v>323</v>
+        <v>374</v>
       </c>
     </row>
     <row r="333" spans="3:3">
       <c r="C333" t="s">
-        <v>319</v>
+        <v>407</v>
       </c>
     </row>
     <row r="334" spans="3:3">
       <c r="C334" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="335" spans="3:3">
       <c r="C335" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="336" spans="3:3">
       <c r="C336" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="337" spans="3:3">
@@ -5786,67 +5819,67 @@
     </row>
     <row r="342" spans="3:3">
       <c r="C342" t="s">
-        <v>332</v>
+        <v>408</v>
       </c>
     </row>
     <row r="343" spans="3:3">
       <c r="C343" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="344" spans="3:3">
       <c r="C344" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="345" spans="3:3">
       <c r="C345" t="s">
-        <v>315</v>
+        <v>409</v>
       </c>
     </row>
     <row r="346" spans="3:3">
       <c r="C346" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
     </row>
     <row r="347" spans="3:3">
       <c r="C347" t="s">
-        <v>334</v>
+        <v>411</v>
       </c>
     </row>
     <row r="348" spans="3:3">
       <c r="C348" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
     </row>
     <row r="349" spans="3:3">
       <c r="C349" t="s">
-        <v>407</v>
+        <v>322</v>
       </c>
     </row>
     <row r="350" spans="3:3">
       <c r="C350" t="s">
-        <v>375</v>
+        <v>323</v>
       </c>
     </row>
     <row r="351" spans="3:3">
       <c r="C351" t="s">
-        <v>408</v>
+        <v>319</v>
       </c>
     </row>
     <row r="352" spans="3:3">
       <c r="C352" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="353" spans="3:3">
       <c r="C353" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="354" spans="3:3">
       <c r="C354" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="355" spans="3:3">
@@ -5876,352 +5909,352 @@
     </row>
     <row r="360" spans="3:3">
       <c r="C360" t="s">
-        <v>409</v>
+        <v>332</v>
       </c>
     </row>
     <row r="361" spans="3:3">
       <c r="C361" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="362" spans="3:3">
       <c r="C362" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="363" spans="3:3">
       <c r="C363" t="s">
-        <v>410</v>
+        <v>315</v>
       </c>
     </row>
     <row r="364" spans="3:3">
       <c r="C364" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
     </row>
     <row r="365" spans="3:3">
       <c r="C365" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="366" spans="3:3">
       <c r="C366" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="367" spans="3:3">
       <c r="C367" t="s">
-        <v>322</v>
+        <v>416</v>
       </c>
     </row>
     <row r="368" spans="3:3">
       <c r="C368" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="369" spans="3:3">
       <c r="C369" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="370" spans="3:3">
       <c r="C370" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="371" spans="3:3">
       <c r="C371" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="372" spans="3:3">
       <c r="C372" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="373" spans="3:3">
       <c r="C373" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="374" spans="3:3">
       <c r="C374" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="375" spans="3:3">
       <c r="C375" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="376" spans="3:3">
       <c r="C376" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="377" spans="3:3">
       <c r="C377" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="378" spans="3:3">
       <c r="C378" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="379" spans="3:3">
       <c r="C379" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="380" spans="3:3">
       <c r="C380" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="381" spans="3:3">
       <c r="C381" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="382" spans="3:3">
       <c r="C382" t="s">
-        <v>414</v>
+        <v>315</v>
       </c>
     </row>
     <row r="383" spans="3:3">
       <c r="C383" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
     </row>
     <row r="384" spans="3:3">
       <c r="C384" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="385" spans="3:3">
       <c r="C385" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="386" spans="3:3">
       <c r="C386" t="s">
-        <v>322</v>
+        <v>420</v>
       </c>
     </row>
     <row r="387" spans="3:3">
       <c r="C387" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="388" spans="3:3">
       <c r="C388" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="389" spans="3:3">
       <c r="C389" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="390" spans="3:3">
       <c r="C390" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="391" spans="3:3">
       <c r="C391" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="392" spans="3:3">
       <c r="C392" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="393" spans="3:3">
       <c r="C393" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="394" spans="3:3">
       <c r="C394" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="395" spans="3:3">
       <c r="C395" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="396" spans="3:3">
       <c r="C396" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="397" spans="3:3">
       <c r="C397" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="398" spans="3:3">
       <c r="C398" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="399" spans="3:3">
       <c r="C399" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="400" spans="3:3">
       <c r="C400" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="401" spans="3:3">
       <c r="C401" t="s">
-        <v>418</v>
+        <v>315</v>
       </c>
     </row>
     <row r="402" spans="3:3">
       <c r="C402" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="403" spans="3:3">
       <c r="C403" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="404" spans="3:3">
       <c r="C404" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="405" spans="3:3">
       <c r="C405" t="s">
-        <v>322</v>
+        <v>424</v>
       </c>
     </row>
     <row r="406" spans="3:3">
       <c r="C406" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="407" spans="3:3">
       <c r="C407" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="408" spans="3:3">
       <c r="C408" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="409" spans="3:3">
       <c r="C409" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="410" spans="3:3">
       <c r="C410" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="411" spans="3:3">
       <c r="C411" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="412" spans="3:3">
       <c r="C412" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="413" spans="3:3">
       <c r="C413" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="414" spans="3:3">
       <c r="C414" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="415" spans="3:3">
       <c r="C415" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="416" spans="3:3">
       <c r="C416" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="417" spans="3:3">
       <c r="C417" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="418" spans="3:3">
       <c r="C418" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="419" spans="3:3">
       <c r="C419" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="420" spans="3:3">
       <c r="C420" t="s">
-        <v>422</v>
+        <v>315</v>
       </c>
     </row>
     <row r="421" spans="3:3">
       <c r="C421" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="422" spans="3:3">
       <c r="C422" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="423" spans="3:3">
       <c r="C423" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="424" spans="3:3">
       <c r="C424" t="s">
-        <v>322</v>
+        <v>428</v>
       </c>
     </row>
     <row r="425" spans="3:3">
       <c r="C425" t="s">
-        <v>323</v>
+        <v>383</v>
       </c>
     </row>
     <row r="426" spans="3:3">
       <c r="C426" t="s">
-        <v>319</v>
+        <v>407</v>
       </c>
     </row>
     <row r="427" spans="3:3">
       <c r="C427" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="428" spans="3:3">
       <c r="C428" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="429" spans="3:3">
       <c r="C429" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="430" spans="3:3">
@@ -6251,7 +6284,7 @@
     </row>
     <row r="435" spans="3:3">
       <c r="C435" t="s">
-        <v>332</v>
+        <v>429</v>
       </c>
     </row>
     <row r="436" spans="3:3">
@@ -6271,32 +6304,32 @@
     </row>
     <row r="439" spans="3:3">
       <c r="C439" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
     </row>
     <row r="440" spans="3:3">
       <c r="C440" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="441" spans="3:3">
       <c r="C441" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="442" spans="3:3">
       <c r="C442" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="443" spans="3:3">
       <c r="C443" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="444" spans="3:3">
       <c r="C444" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="445" spans="3:3">
@@ -6341,7 +6374,7 @@
     </row>
     <row r="453" spans="3:3">
       <c r="C453" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="454" spans="3:3">
@@ -6366,27 +6399,27 @@
     </row>
     <row r="458" spans="3:3">
       <c r="C458" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
     </row>
     <row r="459" spans="3:3">
       <c r="C459" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
     <row r="460" spans="3:3">
       <c r="C460" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
     </row>
     <row r="461" spans="3:3">
       <c r="C461" t="s">
-        <v>384</v>
+        <v>322</v>
       </c>
     </row>
     <row r="462" spans="3:3">
       <c r="C462" t="s">
-        <v>408</v>
+        <v>323</v>
       </c>
     </row>
     <row r="463" spans="3:3">
@@ -6401,427 +6434,427 @@
     </row>
     <row r="465" spans="3:3">
       <c r="C465" t="s">
-        <v>325</v>
+        <v>375</v>
       </c>
     </row>
     <row r="466" spans="3:3">
       <c r="C466" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="467" spans="3:3">
       <c r="C467" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="468" spans="3:3">
       <c r="C468" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="469" spans="3:3">
       <c r="C469" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="470" spans="3:3">
       <c r="C470" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="471" spans="3:3">
       <c r="C471" t="s">
-        <v>430</v>
+        <v>333</v>
       </c>
     </row>
     <row r="472" spans="3:3">
       <c r="C472" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="473" spans="3:3">
       <c r="C473" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="474" spans="3:3">
       <c r="C474" t="s">
-        <v>315</v>
+        <v>435</v>
       </c>
     </row>
     <row r="475" spans="3:3">
       <c r="C475" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
     </row>
     <row r="476" spans="3:3">
       <c r="C476" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
     </row>
     <row r="477" spans="3:3">
       <c r="C477" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
     </row>
     <row r="478" spans="3:3">
       <c r="C478" t="s">
-        <v>435</v>
+        <v>383</v>
       </c>
     </row>
     <row r="479" spans="3:3">
       <c r="C479" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="480" spans="3:3">
       <c r="C480" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="481" spans="3:3">
       <c r="C481" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="482" spans="3:3">
       <c r="C482" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
     </row>
     <row r="483" spans="3:3">
       <c r="C483" t="s">
-        <v>376</v>
+        <v>328</v>
       </c>
     </row>
     <row r="484" spans="3:3">
       <c r="C484" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="485" spans="3:3">
       <c r="C485" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="486" spans="3:3">
       <c r="C486" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="487" spans="3:3">
       <c r="C487" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="488" spans="3:3">
       <c r="C488" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="489" spans="3:3">
       <c r="C489" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="490" spans="3:3">
       <c r="C490" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="491" spans="3:3">
       <c r="C491" t="s">
-        <v>315</v>
+        <v>439</v>
       </c>
     </row>
     <row r="492" spans="3:3">
       <c r="C492" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
     </row>
     <row r="493" spans="3:3">
       <c r="C493" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
     </row>
     <row r="494" spans="3:3">
       <c r="C494" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
     </row>
     <row r="495" spans="3:3">
       <c r="C495" t="s">
-        <v>439</v>
+        <v>383</v>
       </c>
     </row>
     <row r="496" spans="3:3">
       <c r="C496" t="s">
-        <v>384</v>
+        <v>323</v>
       </c>
     </row>
     <row r="497" spans="3:3">
       <c r="C497" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="498" spans="3:3">
       <c r="C498" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="499" spans="3:3">
       <c r="C499" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
     </row>
     <row r="500" spans="3:3">
       <c r="C500" t="s">
-        <v>376</v>
+        <v>328</v>
       </c>
     </row>
     <row r="501" spans="3:3">
       <c r="C501" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="502" spans="3:3">
       <c r="C502" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="503" spans="3:3">
       <c r="C503" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="504" spans="3:3">
       <c r="C504" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="505" spans="3:3">
       <c r="C505" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="506" spans="3:3">
       <c r="C506" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="507" spans="3:3">
       <c r="C507" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="508" spans="3:3">
       <c r="C508" t="s">
-        <v>315</v>
+        <v>443</v>
       </c>
     </row>
     <row r="509" spans="3:3">
       <c r="C509" t="s">
-        <v>440</v>
+        <v>316</v>
       </c>
     </row>
     <row r="510" spans="3:3">
       <c r="C510" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
     </row>
     <row r="511" spans="3:3">
       <c r="C511" t="s">
-        <v>442</v>
+        <v>317</v>
       </c>
     </row>
     <row r="512" spans="3:3">
       <c r="C512" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="513" spans="3:3">
       <c r="C513" t="s">
-        <v>384</v>
+        <v>318</v>
       </c>
     </row>
     <row r="514" spans="3:3">
       <c r="C514" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="515" spans="3:3">
       <c r="C515" t="s">
-        <v>319</v>
+        <v>446</v>
       </c>
     </row>
     <row r="516" spans="3:3">
       <c r="C516" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="517" spans="3:3">
       <c r="C517" t="s">
-        <v>376</v>
+        <v>321</v>
       </c>
     </row>
     <row r="518" spans="3:3">
       <c r="C518" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
     </row>
     <row r="519" spans="3:3">
       <c r="C519" t="s">
-        <v>329</v>
+        <v>447</v>
       </c>
     </row>
     <row r="520" spans="3:3">
       <c r="C520" t="s">
-        <v>330</v>
+        <v>448</v>
       </c>
     </row>
     <row r="521" spans="3:3">
       <c r="C521" t="s">
-        <v>331</v>
+        <v>449</v>
       </c>
     </row>
     <row r="522" spans="3:3">
       <c r="C522" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
     </row>
     <row r="523" spans="3:3">
       <c r="C523" t="s">
-        <v>333</v>
+        <v>445</v>
       </c>
     </row>
     <row r="524" spans="3:3">
       <c r="C524" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="525" spans="3:3">
       <c r="C525" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="526" spans="3:3">
       <c r="C526" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="527" spans="3:3">
       <c r="C527" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="528" spans="3:3">
       <c r="C528" t="s">
-        <v>445</v>
+        <v>321</v>
       </c>
     </row>
     <row r="529" spans="3:3">
       <c r="C529" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="530" spans="3:3">
       <c r="C530" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
     </row>
     <row r="531" spans="3:3">
       <c r="C531" t="s">
-        <v>318</v>
+        <v>451</v>
       </c>
     </row>
     <row r="532" spans="3:3">
       <c r="C532" t="s">
-        <v>319</v>
+        <v>452</v>
       </c>
     </row>
     <row r="533" spans="3:3">
       <c r="C533" t="s">
-        <v>447</v>
+        <v>317</v>
       </c>
     </row>
     <row r="534" spans="3:3">
       <c r="C534" t="s">
-        <v>320</v>
+        <v>365</v>
       </c>
     </row>
     <row r="535" spans="3:3">
       <c r="C535" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="536" spans="3:3">
       <c r="C536" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="537" spans="3:3">
       <c r="C537" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="538" spans="3:3">
       <c r="C538" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
     </row>
     <row r="539" spans="3:3">
       <c r="C539" t="s">
-        <v>450</v>
+        <v>375</v>
       </c>
     </row>
     <row r="540" spans="3:3">
       <c r="C540" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="541" spans="3:3">
       <c r="C541" t="s">
-        <v>446</v>
+        <v>321</v>
       </c>
     </row>
     <row r="542" spans="3:3">
       <c r="C542" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="543" spans="3:3">
       <c r="C543" t="s">
-        <v>319</v>
+        <v>455</v>
       </c>
     </row>
     <row r="544" spans="3:3">
       <c r="C544" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
     </row>
     <row r="545" spans="3:3">
       <c r="C545" t="s">
-        <v>320</v>
+        <v>456</v>
       </c>
     </row>
     <row r="546" spans="3:3">
       <c r="C546" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="547" spans="3:3">
       <c r="C547" t="s">
-        <v>315</v>
+        <v>365</v>
       </c>
     </row>
     <row r="548" spans="3:3">
       <c r="C548" t="s">
-        <v>451</v>
+        <v>318</v>
       </c>
     </row>
     <row r="549" spans="3:3">
       <c r="C549" t="s">
-        <v>452</v>
+        <v>319</v>
       </c>
     </row>
     <row r="550" spans="3:3">
@@ -6831,817 +6864,727 @@
     </row>
     <row r="551" spans="3:3">
       <c r="C551" t="s">
-        <v>317</v>
+        <v>454</v>
       </c>
     </row>
     <row r="552" spans="3:3">
       <c r="C552" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
     </row>
     <row r="553" spans="3:3">
       <c r="C553" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="554" spans="3:3">
       <c r="C554" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="555" spans="3:3">
       <c r="C555" t="s">
-        <v>454</v>
+        <v>315</v>
       </c>
     </row>
     <row r="556" spans="3:3">
       <c r="C556" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
     </row>
     <row r="557" spans="3:3">
       <c r="C557" t="s">
-        <v>376</v>
+        <v>316</v>
       </c>
     </row>
     <row r="558" spans="3:3">
       <c r="C558" t="s">
-        <v>320</v>
+        <v>458</v>
       </c>
     </row>
     <row r="559" spans="3:3">
       <c r="C559" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="560" spans="3:3">
       <c r="C560" t="s">
-        <v>315</v>
+        <v>445</v>
       </c>
     </row>
     <row r="561" spans="3:3">
       <c r="C561" t="s">
-        <v>456</v>
+        <v>318</v>
       </c>
     </row>
     <row r="562" spans="3:3">
       <c r="C562" t="s">
-        <v>452</v>
+        <v>319</v>
       </c>
     </row>
     <row r="563" spans="3:3">
       <c r="C563" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
     </row>
     <row r="564" spans="3:3">
       <c r="C564" t="s">
-        <v>317</v>
+        <v>454</v>
       </c>
     </row>
     <row r="565" spans="3:3">
       <c r="C565" t="s">
-        <v>366</v>
+        <v>325</v>
       </c>
     </row>
     <row r="566" spans="3:3">
       <c r="C566" t="s">
-        <v>318</v>
+        <v>459</v>
       </c>
     </row>
     <row r="567" spans="3:3">
       <c r="C567" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="568" spans="3:3">
       <c r="C568" t="s">
-        <v>454</v>
+        <v>321</v>
       </c>
     </row>
     <row r="569" spans="3:3">
       <c r="C569" t="s">
-        <v>455</v>
+        <v>315</v>
       </c>
     </row>
     <row r="570" spans="3:3">
       <c r="C570" t="s">
-        <v>376</v>
+        <v>460</v>
       </c>
     </row>
     <row r="571" spans="3:3">
       <c r="C571" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="572" spans="3:3">
       <c r="C572" t="s">
-        <v>321</v>
+        <v>461</v>
       </c>
     </row>
     <row r="573" spans="3:3">
       <c r="C573" t="s">
-        <v>315</v>
+        <v>462</v>
       </c>
     </row>
     <row r="574" spans="3:3">
       <c r="C574" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
     </row>
     <row r="575" spans="3:3">
       <c r="C575" t="s">
-        <v>316</v>
+        <v>464</v>
       </c>
     </row>
     <row r="576" spans="3:3">
       <c r="C576" t="s">
-        <v>459</v>
+        <v>319</v>
       </c>
     </row>
     <row r="577" spans="3:3">
       <c r="C577" t="s">
-        <v>317</v>
+        <v>465</v>
       </c>
     </row>
     <row r="578" spans="3:3">
       <c r="C578" t="s">
-        <v>446</v>
+        <v>328</v>
       </c>
     </row>
     <row r="579" spans="3:3">
       <c r="C579" t="s">
-        <v>318</v>
+        <v>466</v>
       </c>
     </row>
     <row r="580" spans="3:3">
       <c r="C580" t="s">
-        <v>319</v>
+        <v>467</v>
       </c>
     </row>
     <row r="581" spans="3:3">
       <c r="C581" t="s">
-        <v>454</v>
+        <v>468</v>
       </c>
     </row>
     <row r="582" spans="3:3">
       <c r="C582" t="s">
-        <v>455</v>
+        <v>321</v>
       </c>
     </row>
     <row r="583" spans="3:3">
       <c r="C583" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
     </row>
     <row r="584" spans="3:3">
       <c r="C584" t="s">
-        <v>460</v>
+        <v>469</v>
       </c>
     </row>
     <row r="585" spans="3:3">
       <c r="C585" t="s">
-        <v>320</v>
+        <v>470</v>
       </c>
     </row>
     <row r="586" spans="3:3">
       <c r="C586" t="s">
-        <v>321</v>
+        <v>471</v>
       </c>
     </row>
     <row r="587" spans="3:3">
       <c r="C587" t="s">
-        <v>315</v>
+        <v>472</v>
       </c>
     </row>
     <row r="588" spans="3:3">
       <c r="C588" t="s">
-        <v>461</v>
+        <v>473</v>
       </c>
     </row>
     <row r="589" spans="3:3">
       <c r="C589" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
     </row>
     <row r="590" spans="3:3">
       <c r="C590" t="s">
-        <v>462</v>
+        <v>319</v>
       </c>
     </row>
     <row r="591" spans="3:3">
       <c r="C591" t="s">
-        <v>463</v>
+        <v>474</v>
       </c>
     </row>
     <row r="592" spans="3:3">
       <c r="C592" t="s">
-        <v>464</v>
+        <v>320</v>
       </c>
     </row>
     <row r="593" spans="3:3">
       <c r="C593" t="s">
-        <v>465</v>
+        <v>321</v>
       </c>
     </row>
     <row r="594" spans="3:3">
       <c r="C594" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="595" spans="3:3">
       <c r="C595" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
     </row>
     <row r="596" spans="3:3">
       <c r="C596" t="s">
-        <v>328</v>
+        <v>470</v>
       </c>
     </row>
     <row r="597" spans="3:3">
       <c r="C597" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
     </row>
     <row r="598" spans="3:3">
       <c r="C598" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
     </row>
     <row r="599" spans="3:3">
       <c r="C599" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
     </row>
     <row r="600" spans="3:3">
       <c r="C600" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="601" spans="3:3">
       <c r="C601" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="602" spans="3:3">
       <c r="C602" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
     </row>
     <row r="603" spans="3:3">
       <c r="C603" t="s">
-        <v>471</v>
+        <v>320</v>
       </c>
     </row>
     <row r="604" spans="3:3">
       <c r="C604" t="s">
-        <v>472</v>
+        <v>321</v>
       </c>
     </row>
     <row r="605" spans="3:3">
       <c r="C605" t="s">
-        <v>473</v>
+        <v>315</v>
       </c>
     </row>
     <row r="606" spans="3:3">
       <c r="C606" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
     </row>
     <row r="607" spans="3:3">
       <c r="C607" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
     </row>
     <row r="608" spans="3:3">
       <c r="C608" t="s">
-        <v>319</v>
+        <v>479</v>
       </c>
     </row>
     <row r="609" spans="3:3">
       <c r="C609" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
     </row>
     <row r="610" spans="3:3">
       <c r="C610" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="611" spans="3:3">
       <c r="C611" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="612" spans="3:3">
       <c r="C612" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="613" spans="3:3">
       <c r="C613" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
     </row>
     <row r="614" spans="3:3">
       <c r="C614" t="s">
-        <v>471</v>
+        <v>320</v>
       </c>
     </row>
     <row r="615" spans="3:3">
       <c r="C615" t="s">
-        <v>477</v>
+        <v>321</v>
       </c>
     </row>
     <row r="616" spans="3:3">
       <c r="C616" t="s">
-        <v>478</v>
+        <v>315</v>
       </c>
     </row>
     <row r="617" spans="3:3">
       <c r="C617" t="s">
-        <v>474</v>
+        <v>480</v>
       </c>
     </row>
     <row r="618" spans="3:3">
       <c r="C618" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
     </row>
     <row r="619" spans="3:3">
       <c r="C619" t="s">
-        <v>319</v>
+        <v>481</v>
       </c>
     </row>
     <row r="620" spans="3:3">
       <c r="C620" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
     </row>
     <row r="621" spans="3:3">
       <c r="C621" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="622" spans="3:3">
       <c r="C622" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="623" spans="3:3">
       <c r="C623" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="624" spans="3:3">
       <c r="C624" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
     </row>
     <row r="625" spans="3:3">
       <c r="C625" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="626" spans="3:3">
       <c r="C626" t="s">
-        <v>480</v>
+        <v>321</v>
       </c>
     </row>
     <row r="627" spans="3:3">
       <c r="C627" t="s">
-        <v>473</v>
+        <v>315</v>
       </c>
     </row>
     <row r="628" spans="3:3">
       <c r="C628" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
     </row>
     <row r="629" spans="3:3">
       <c r="C629" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
     </row>
     <row r="630" spans="3:3">
       <c r="C630" t="s">
-        <v>319</v>
+        <v>483</v>
       </c>
     </row>
     <row r="631" spans="3:3">
       <c r="C631" t="s">
-        <v>475</v>
+        <v>484</v>
       </c>
     </row>
     <row r="632" spans="3:3">
       <c r="C632" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="633" spans="3:3">
       <c r="C633" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="634" spans="3:3">
       <c r="C634" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="635" spans="3:3">
       <c r="C635" t="s">
-        <v>481</v>
+        <v>474</v>
       </c>
     </row>
     <row r="636" spans="3:3">
       <c r="C636" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="637" spans="3:3">
       <c r="C637" t="s">
-        <v>482</v>
+        <v>321</v>
       </c>
     </row>
     <row r="638" spans="3:3">
       <c r="C638" t="s">
-        <v>478</v>
+        <v>315</v>
       </c>
     </row>
     <row r="639" spans="3:3">
       <c r="C639" t="s">
-        <v>474</v>
+        <v>485</v>
       </c>
     </row>
     <row r="640" spans="3:3">
       <c r="C640" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="641" spans="3:3">
       <c r="C641" t="s">
-        <v>319</v>
+        <v>486</v>
       </c>
     </row>
     <row r="642" spans="3:3">
       <c r="C642" t="s">
-        <v>475</v>
+        <v>487</v>
       </c>
     </row>
     <row r="643" spans="3:3">
       <c r="C643" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="644" spans="3:3">
       <c r="C644" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="645" spans="3:3">
       <c r="C645" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="646" spans="3:3">
       <c r="C646" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
     </row>
     <row r="647" spans="3:3">
       <c r="C647" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="648" spans="3:3">
       <c r="C648" t="s">
-        <v>484</v>
+        <v>321</v>
       </c>
     </row>
     <row r="649" spans="3:3">
       <c r="C649" t="s">
-        <v>485</v>
+        <v>315</v>
       </c>
     </row>
     <row r="650" spans="3:3">
       <c r="C650" t="s">
-        <v>474</v>
+        <v>489</v>
       </c>
     </row>
     <row r="651" spans="3:3">
       <c r="C651" t="s">
-        <v>335</v>
+        <v>426</v>
       </c>
     </row>
     <row r="652" spans="3:3">
       <c r="C652" t="s">
-        <v>319</v>
+        <v>490</v>
       </c>
     </row>
     <row r="653" spans="3:3">
       <c r="C653" t="s">
-        <v>475</v>
+        <v>491</v>
       </c>
     </row>
     <row r="654" spans="3:3">
       <c r="C654" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="655" spans="3:3">
       <c r="C655" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="656" spans="3:3">
       <c r="C656" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="657" spans="3:3">
       <c r="C657" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="658" spans="3:3">
       <c r="C658" t="s">
-        <v>334</v>
+        <v>320</v>
       </c>
     </row>
     <row r="659" spans="3:3">
       <c r="C659" t="s">
-        <v>487</v>
+        <v>321</v>
       </c>
     </row>
     <row r="660" spans="3:3">
       <c r="C660" t="s">
-        <v>488</v>
+        <v>315</v>
       </c>
     </row>
     <row r="661" spans="3:3">
       <c r="C661" t="s">
-        <v>474</v>
+        <v>492</v>
       </c>
     </row>
     <row r="662" spans="3:3">
       <c r="C662" t="s">
-        <v>335</v>
+        <v>426</v>
       </c>
     </row>
     <row r="663" spans="3:3">
       <c r="C663" t="s">
-        <v>319</v>
+        <v>493</v>
       </c>
     </row>
     <row r="664" spans="3:3">
       <c r="C664" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
     </row>
     <row r="665" spans="3:3">
       <c r="C665" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="666" spans="3:3">
       <c r="C666" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="667" spans="3:3">
       <c r="C667" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="668" spans="3:3">
       <c r="C668" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="669" spans="3:3">
       <c r="C669" t="s">
-        <v>427</v>
+        <v>320</v>
       </c>
     </row>
     <row r="670" spans="3:3">
       <c r="C670" t="s">
-        <v>491</v>
+        <v>321</v>
       </c>
     </row>
     <row r="671" spans="3:3">
       <c r="C671" t="s">
-        <v>492</v>
+        <v>315</v>
       </c>
     </row>
     <row r="672" spans="3:3">
       <c r="C672" t="s">
-        <v>474</v>
+        <v>495</v>
       </c>
     </row>
     <row r="673" spans="3:3">
       <c r="C673" t="s">
-        <v>335</v>
+        <v>496</v>
       </c>
     </row>
     <row r="674" spans="3:3">
       <c r="C674" t="s">
-        <v>319</v>
+        <v>497</v>
       </c>
     </row>
     <row r="675" spans="3:3">
       <c r="C675" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
     </row>
     <row r="676" spans="3:3">
       <c r="C676" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="677" spans="3:3">
       <c r="C677" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="678" spans="3:3">
       <c r="C678" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="679" spans="3:3">
       <c r="C679" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
     </row>
     <row r="680" spans="3:3">
       <c r="C680" t="s">
-        <v>427</v>
+        <v>320</v>
       </c>
     </row>
     <row r="681" spans="3:3">
       <c r="C681" t="s">
-        <v>494</v>
+        <v>321</v>
       </c>
     </row>
     <row r="682" spans="3:3">
       <c r="C682" t="s">
-        <v>495</v>
+        <v>315</v>
       </c>
     </row>
     <row r="683" spans="3:3">
       <c r="C683" t="s">
-        <v>474</v>
+        <v>499</v>
       </c>
     </row>
     <row r="684" spans="3:3">
       <c r="C684" t="s">
-        <v>335</v>
+        <v>496</v>
       </c>
     </row>
     <row r="685" spans="3:3">
       <c r="C685" t="s">
-        <v>319</v>
+        <v>500</v>
       </c>
     </row>
     <row r="686" spans="3:3">
       <c r="C686" t="s">
-        <v>489</v>
+        <v>501</v>
       </c>
     </row>
     <row r="687" spans="3:3">
       <c r="C687" t="s">
-        <v>320</v>
+        <v>473</v>
       </c>
     </row>
     <row r="688" spans="3:3">
       <c r="C688" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="689" spans="3:3">
       <c r="C689" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="690" spans="3:3">
       <c r="C690" t="s">
-        <v>496</v>
+        <v>488</v>
       </c>
     </row>
     <row r="691" spans="3:3">
       <c r="C691" t="s">
-        <v>497</v>
+        <v>320</v>
       </c>
     </row>
     <row r="692" spans="3:3">
       <c r="C692" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
     </row>
     <row r="693" spans="3:3">
       <c r="C693" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
     </row>
     <row r="694" spans="3:3">
       <c r="C694" t="s">
-        <v>474</v>
+        <v>504</v>
       </c>
     </row>
     <row r="695" spans="3:3">
       <c r="C695" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="696" spans="3:3">
-      <c r="C696" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="697" spans="3:3">
-      <c r="C697" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="698" spans="3:3">
-      <c r="C698" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="699" spans="3:3">
-      <c r="C699" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="700" spans="3:3">
-      <c r="C700" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="701" spans="3:3">
-      <c r="C701" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="702" spans="3:3">
-      <c r="C702" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="703" spans="3:3">
-      <c r="C703" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="704" spans="3:3">
-      <c r="C704" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="705" spans="3:3">
-      <c r="C705" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="706" spans="3:3">
-      <c r="C706" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="707" spans="3:3">
-      <c r="C707" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="708" spans="3:3">
-      <c r="C708" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="709" spans="3:3">
-      <c r="C709" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="710" spans="3:3">
-      <c r="C710" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="711" spans="3:3">
-      <c r="C711" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="712" spans="3:3">
-      <c r="C712" t="s">
         <v>505</v>
-      </c>
-    </row>
-    <row r="713" spans="3:3">
-      <c r="C713" t="s">
-        <v>506</v>
       </c>
     </row>
   </sheetData>
@@ -7663,12 +7606,12 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
+        <v>46044</v>
       </c>
     </row>
     <row r="2" spans="2:5">
       <c r="B2" s="2" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -7846,10 +7789,10 @@
     </row>
     <row r="29" spans="2:5" ht="37.5">
       <c r="B29" s="1" t="s">
-        <v>562</v>
+        <v>558</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>563</v>
+        <v>559</v>
       </c>
       <c r="E29" s="3">
         <v>46043</v>
@@ -7857,15 +7800,15 @@
     </row>
     <row r="30" spans="2:5" ht="337.5">
       <c r="B30" s="1" t="s">
-        <v>564</v>
+        <v>560</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="56.25">
       <c r="B31" s="1" t="s">
-        <v>565</v>
+        <v>561</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>566</v>
+        <v>562</v>
       </c>
       <c r="E31" s="3">
         <v>46043</v>
@@ -7873,10 +7816,10 @@
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="1" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>568</v>
+        <v>564</v>
       </c>
       <c r="E33" s="3">
         <v>46043</v>
@@ -7884,18 +7827,18 @@
     </row>
     <row r="35" spans="2:5" ht="37.5">
       <c r="B35" s="1" t="s">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>570</v>
+        <v>566</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="56.25">
       <c r="B36" s="1" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>572</v>
+        <v>568</v>
       </c>
       <c r="E36" s="3">
         <v>46043</v>
@@ -7903,10 +7846,10 @@
     </row>
     <row r="37" spans="2:5" ht="56.25">
       <c r="B37" s="1" t="s">
-        <v>573</v>
+        <v>569</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>574</v>
+        <v>570</v>
       </c>
       <c r="E37" s="3">
         <v>46043</v>
@@ -7914,10 +7857,10 @@
     </row>
     <row r="38" spans="2:5" ht="112.5">
       <c r="B38" s="1" t="s">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>576</v>
+        <v>572</v>
       </c>
       <c r="E38" s="3">
         <v>46043</v>
@@ -7938,7 +7881,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E20"/>
+  <dimension ref="B1:E25"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="73.125" customWidth="1"/>
@@ -7949,7 +7892,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
+        <v>46044</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8037,55 +7980,78 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" spans="2:5" ht="37.5">
-      <c r="B15" s="1" t="s">
+    <row r="15" spans="2:5">
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+    </row>
+    <row r="16" spans="2:5" ht="37.5">
+      <c r="B16" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C16" s="1" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="56.25">
-      <c r="B16" s="1" t="s">
+    <row r="17" spans="2:5">
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+    </row>
+    <row r="18" spans="2:5" ht="56.25">
+      <c r="B18" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>229</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5">
-      <c r="B17" s="1" t="s">
-        <v>230</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="18" spans="2:5">
-      <c r="B18" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5">
+      <c r="B20" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5">
+      <c r="B21" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C21" s="1" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="20" spans="2:5" ht="93.75">
-      <c r="B20" s="1" t="s">
-        <v>559</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="E20" s="3">
+    <row r="22" spans="2:5">
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+    </row>
+    <row r="23" spans="2:5" ht="93.75">
+      <c r="B23" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="E23" s="3">
         <v>46043</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" ht="56.25">
+      <c r="B25" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="E25" s="3">
+        <v>46044</v>
       </c>
     </row>
   </sheetData>
@@ -8114,7 +8080,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
+        <v>46044</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8134,63 +8100,63 @@
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="5" t="s">
-        <v>542</v>
+        <v>538</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" s="1" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="C7" t="s">
-        <v>544</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" t="s">
-        <v>545</v>
+        <v>541</v>
       </c>
       <c r="C8" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="56.25">
       <c r="B9" s="1" t="s">
-        <v>547</v>
+        <v>543</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>548</v>
+        <v>544</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
-        <v>549</v>
+        <v>545</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="75">
       <c r="B11" s="1" t="s">
-        <v>551</v>
+        <v>547</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="37.5">
       <c r="B12" s="1" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="75">
       <c r="B13" s="1" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>556</v>
+        <v>552</v>
       </c>
       <c r="E13" s="3">
         <v>46043</v>
@@ -8198,10 +8164,10 @@
     </row>
     <row r="14" spans="2:5" ht="56.25">
       <c r="B14" s="1" t="s">
-        <v>557</v>
+        <v>553</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="E14" s="3">
         <v>46043</v>
@@ -8887,7 +8853,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46043</v>
+        <v>46044</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
Refactor code for improved readability and consistency across multiple pages
- Updated the formatting of code blocks in `emergency_meeting_page.dart` for better readability.
- Enhanced the clarity of model filtering logic in `emergency_meeting_page.dart`.
- Improved the structure of model selection saving in `emergency_meeting_page.dart`.
- Refined the last message retrieval logic in `emergency_meeting_page.dart`.
- Standardized the formatting of strings in `gemini_university_v2_page.dart` for consistency.
- Cleaned up the mapping of supported generation methods in `morning_briefing_page.dart`.
- Enhanced the layout and readability of the AI Assistant settings display in `morning_briefing_page.dart`.
- Streamlined the task list rendering in `morning_briefing_page.dart` for better performance and clarity.
- Updated the binary file `my_web_app.xlsx` to reflect recent changes.
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424128D5-CBF3-4B2B-8F91-0BC46933C822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF847627-0433-495F-82FB-18BA80A4B175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="576">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="577">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2154,15 +2154,6 @@
     <t xml:space="preserve">      "maxTemperature": 2</t>
   </si>
   <si>
-    <t xml:space="preserve">      "name": "models/gemini-2.0-flash-001",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash 001",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "description": "Stable version of Gemini 2.0 Flash, our fast and versatile multimodal model for scaling across diverse tasks, released in January of 2025.",</t>
-  </si>
-  <si>
     <t xml:space="preserve">      "name": "models/gemini-2.0-flash-exp-image-generation",</t>
   </si>
   <si>
@@ -2951,6 +2942,22 @@
   </si>
   <si>
     <t>Gemini Code Assistは、VS Code、JetBrains IDE、Android Studioなどの対応IDEで利用でき、多くの主要言語においてAIを活用したコーディング支援を提供します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>models/gemini-2.0-flash-001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini 2.0 Flash 001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Stable version of Gemini 2.0 Flash, our fast and versatile multimodal model for scaling across diverse tasks, released in January of 2025.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>多様なタスクにスケーリング可能な高速かつ汎用性の高いマルチモーダルモデル「Gemini 2.0 Flash」の安定版が、2025年1月にリリースされました。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3901,7 +3908,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F96D129-34E8-4B10-A261-7AEE00EA03AD}">
-  <dimension ref="B1:Q695"/>
+  <dimension ref="B1:Q680"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
@@ -3924,57 +3931,57 @@
     </row>
     <row r="2" spans="2:17">
       <c r="E2" t="s">
+        <v>503</v>
+      </c>
+      <c r="F2" t="s">
+        <v>505</v>
+      </c>
+      <c r="G2" t="s">
         <v>506</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>508</v>
       </c>
-      <c r="G2" t="s">
-        <v>509</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
+        <v>510</v>
+      </c>
+      <c r="K2" t="s">
         <v>511</v>
       </c>
-      <c r="J2" t="s">
-        <v>513</v>
-      </c>
-      <c r="K2" t="s">
-        <v>514</v>
-      </c>
       <c r="L2" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="M2" t="s">
+        <v>520</v>
+      </c>
+      <c r="N2" t="s">
+        <v>521</v>
+      </c>
+      <c r="O2" t="s">
+        <v>522</v>
+      </c>
+      <c r="P2" t="s">
         <v>523</v>
       </c>
-      <c r="N2" t="s">
+      <c r="Q2" t="s">
         <v>524</v>
-      </c>
-      <c r="O2" t="s">
-        <v>525</v>
-      </c>
-      <c r="P2" t="s">
-        <v>526</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>527</v>
       </c>
     </row>
     <row r="3" spans="2:17" ht="37.5">
       <c r="E3" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="H3" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="I3" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="J3">
         <v>1024</v>
@@ -3983,24 +3990,24 @@
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" spans="2:17" ht="75">
       <c r="E4" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
+        <v>515</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>518</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>519</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>521</v>
       </c>
       <c r="J4">
         <v>1048576</v>
@@ -4009,7 +4016,7 @@
         <v>65536</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -4029,19 +4036,19 @@
     </row>
     <row r="5" spans="2:17" ht="75">
       <c r="E5" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="F5">
         <v>2.5</v>
       </c>
       <c r="G5" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="H5" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="I5" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="J5">
         <v>1048576</v>
@@ -4050,7 +4057,7 @@
         <v>65536</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -4070,19 +4077,19 @@
     </row>
     <row r="6" spans="2:17" ht="56.25">
       <c r="E6" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="H6" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="I6" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="J6">
         <v>1048576</v>
@@ -4091,7 +4098,7 @@
         <v>8192</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -4111,19 +4118,19 @@
         <v>46043</v>
       </c>
       <c r="E7" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="H7" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="I7" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="J7">
         <v>1048576</v>
@@ -4132,7 +4139,7 @@
         <v>8192</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="M7">
         <v>1</v>
@@ -4147,469 +4154,507 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:17">
-      <c r="C8" t="s">
-        <v>315</v>
+    <row r="8" spans="2:17" ht="75">
+      <c r="B8" s="3">
+        <v>46044</v>
+      </c>
+      <c r="E8" t="s">
+        <v>573</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>574</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="J8">
+        <v>1048576</v>
+      </c>
+      <c r="K8">
+        <v>8192</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+      <c r="N8">
+        <v>0.95</v>
+      </c>
+      <c r="O8">
+        <v>40</v>
+      </c>
+      <c r="P8">
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="2:17">
-      <c r="C9" t="s">
-        <v>339</v>
-      </c>
+      <c r="B9" s="3"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="L9" s="1"/>
     </row>
     <row r="10" spans="2:17">
-      <c r="C10" t="s">
-        <v>334</v>
-      </c>
+      <c r="B10" s="3"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="L10" s="1"/>
     </row>
     <row r="11" spans="2:17">
       <c r="C11" t="s">
-        <v>340</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" spans="2:17">
       <c r="C12" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="13" spans="2:17">
       <c r="C13" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
     </row>
     <row r="14" spans="2:17">
       <c r="C14" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" spans="2:17">
       <c r="C15" t="s">
-        <v>319</v>
+        <v>341</v>
       </c>
     </row>
     <row r="16" spans="2:17">
       <c r="C16" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" spans="3:3">
       <c r="C17" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="18" spans="3:3">
       <c r="C18" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="19" spans="3:3">
       <c r="C19" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="20" spans="3:3">
       <c r="C20" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="21" spans="3:3">
       <c r="C21" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="22" spans="3:3">
       <c r="C22" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="23" spans="3:3">
       <c r="C23" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
     </row>
     <row r="24" spans="3:3">
       <c r="C24" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
     </row>
     <row r="25" spans="3:3">
       <c r="C25" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
     </row>
     <row r="26" spans="3:3">
       <c r="C26" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="27" spans="3:3">
       <c r="C27" t="s">
-        <v>342</v>
+        <v>321</v>
       </c>
     </row>
     <row r="28" spans="3:3">
       <c r="C28" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="29" spans="3:3">
       <c r="C29" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="30" spans="3:3">
       <c r="C30" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
     </row>
     <row r="31" spans="3:3">
       <c r="C31" t="s">
-        <v>322</v>
+        <v>343</v>
       </c>
     </row>
     <row r="32" spans="3:3">
       <c r="C32" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
     </row>
     <row r="33" spans="3:3">
       <c r="C33" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="34" spans="3:3">
       <c r="C34" t="s">
-        <v>324</v>
+        <v>335</v>
       </c>
     </row>
     <row r="35" spans="3:3">
       <c r="C35" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="36" spans="3:3">
       <c r="C36" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
     </row>
     <row r="37" spans="3:3">
       <c r="C37" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="38" spans="3:3">
       <c r="C38" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="39" spans="3:3">
       <c r="C39" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="40" spans="3:3">
       <c r="C40" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
     </row>
     <row r="41" spans="3:3">
       <c r="C41" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="42" spans="3:3">
       <c r="C42" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="43" spans="3:3">
       <c r="C43" t="s">
-        <v>315</v>
+        <v>337</v>
       </c>
     </row>
     <row r="44" spans="3:3">
       <c r="C44" t="s">
-        <v>345</v>
+        <v>338</v>
       </c>
     </row>
     <row r="45" spans="3:3">
       <c r="C45" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
     </row>
     <row r="46" spans="3:3">
       <c r="C46" t="s">
-        <v>346</v>
+        <v>315</v>
       </c>
     </row>
     <row r="47" spans="3:3">
       <c r="C47" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="48" spans="3:3">
       <c r="C48" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
     </row>
     <row r="49" spans="3:3">
       <c r="C49" t="s">
-        <v>335</v>
+        <v>346</v>
       </c>
     </row>
     <row r="50" spans="3:3">
       <c r="C50" t="s">
-        <v>319</v>
+        <v>347</v>
       </c>
     </row>
     <row r="51" spans="3:3">
       <c r="C51" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="52" spans="3:3">
       <c r="C52" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="53" spans="3:3">
       <c r="C53" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="54" spans="3:3">
       <c r="C54" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="55" spans="3:3">
       <c r="C55" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="56" spans="3:3">
       <c r="C56" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="57" spans="3:3">
       <c r="C57" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="58" spans="3:3">
       <c r="C58" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
     </row>
     <row r="59" spans="3:3">
       <c r="C59" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="60" spans="3:3">
       <c r="C60" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="61" spans="3:3">
       <c r="C61" t="s">
-        <v>315</v>
+        <v>337</v>
       </c>
     </row>
     <row r="62" spans="3:3">
       <c r="C62" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
     </row>
     <row r="63" spans="3:3">
       <c r="C63" t="s">
-        <v>334</v>
+        <v>321</v>
       </c>
     </row>
     <row r="64" spans="3:3">
       <c r="C64" t="s">
-        <v>349</v>
+        <v>315</v>
       </c>
     </row>
     <row r="65" spans="3:3">
       <c r="C65" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="66" spans="3:3">
       <c r="C66" t="s">
-        <v>322</v>
+        <v>349</v>
       </c>
     </row>
     <row r="67" spans="3:3">
       <c r="C67" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
     </row>
     <row r="68" spans="3:3">
       <c r="C68" t="s">
-        <v>319</v>
+        <v>351</v>
       </c>
     </row>
     <row r="69" spans="3:3">
       <c r="C69" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="70" spans="3:3">
       <c r="C70" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="71" spans="3:3">
       <c r="C71" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="72" spans="3:3">
       <c r="C72" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="73" spans="3:3">
       <c r="C73" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="74" spans="3:3">
       <c r="C74" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="75" spans="3:3">
       <c r="C75" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="76" spans="3:3">
       <c r="C76" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
     </row>
     <row r="77" spans="3:3">
       <c r="C77" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="78" spans="3:3">
       <c r="C78" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="79" spans="3:3">
       <c r="C79" t="s">
-        <v>315</v>
+        <v>337</v>
       </c>
     </row>
     <row r="80" spans="3:3">
       <c r="C80" t="s">
-        <v>351</v>
+        <v>338</v>
       </c>
     </row>
     <row r="81" spans="3:3">
       <c r="C81" t="s">
-        <v>352</v>
+        <v>321</v>
       </c>
     </row>
     <row r="82" spans="3:3">
       <c r="C82" t="s">
-        <v>353</v>
+        <v>315</v>
       </c>
     </row>
     <row r="83" spans="3:3">
       <c r="C83" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="84" spans="3:3">
       <c r="C84" t="s">
-        <v>322</v>
+        <v>349</v>
       </c>
     </row>
     <row r="85" spans="3:3">
       <c r="C85" t="s">
-        <v>335</v>
+        <v>353</v>
       </c>
     </row>
     <row r="86" spans="3:3">
       <c r="C86" t="s">
-        <v>319</v>
+        <v>351</v>
       </c>
     </row>
     <row r="87" spans="3:3">
       <c r="C87" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="88" spans="3:3">
       <c r="C88" t="s">
-        <v>325</v>
+        <v>335</v>
       </c>
     </row>
     <row r="89" spans="3:3">
       <c r="C89" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="90" spans="3:3">
       <c r="C90" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="91" spans="3:3">
       <c r="C91" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="92" spans="3:3">
       <c r="C92" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="93" spans="3:3">
       <c r="C93" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="94" spans="3:3">
       <c r="C94" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
     </row>
     <row r="95" spans="3:3">
       <c r="C95" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="96" spans="3:3">
       <c r="C96" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="97" spans="3:3">
       <c r="C97" t="s">
-        <v>315</v>
+        <v>337</v>
       </c>
     </row>
     <row r="98" spans="3:3">
       <c r="C98" t="s">
-        <v>355</v>
+        <v>338</v>
       </c>
     </row>
     <row r="99" spans="3:3">
       <c r="C99" t="s">
-        <v>352</v>
+        <v>321</v>
       </c>
     </row>
     <row r="100" spans="3:3">
       <c r="C100" t="s">
-        <v>356</v>
+        <v>315</v>
       </c>
     </row>
     <row r="101" spans="3:3">
@@ -4619,287 +4664,287 @@
     </row>
     <row r="102" spans="3:3">
       <c r="C102" t="s">
-        <v>322</v>
+        <v>355</v>
       </c>
     </row>
     <row r="103" spans="3:3">
       <c r="C103" t="s">
-        <v>335</v>
+        <v>356</v>
       </c>
     </row>
     <row r="104" spans="3:3">
       <c r="C104" t="s">
-        <v>319</v>
+        <v>357</v>
       </c>
     </row>
     <row r="105" spans="3:3">
       <c r="C105" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="106" spans="3:3">
       <c r="C106" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="107" spans="3:3">
       <c r="C107" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
     </row>
     <row r="108" spans="3:3">
       <c r="C108" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="109" spans="3:3">
       <c r="C109" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="110" spans="3:3">
       <c r="C110" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="111" spans="3:3">
       <c r="C111" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="112" spans="3:3">
       <c r="C112" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
     </row>
     <row r="113" spans="3:3">
       <c r="C113" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="114" spans="3:3">
       <c r="C114" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="115" spans="3:3">
       <c r="C115" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="116" spans="3:3">
       <c r="C116" t="s">
-        <v>357</v>
+        <v>332</v>
       </c>
     </row>
     <row r="117" spans="3:3">
       <c r="C117" t="s">
-        <v>358</v>
+        <v>333</v>
       </c>
     </row>
     <row r="118" spans="3:3">
       <c r="C118" t="s">
-        <v>359</v>
+        <v>321</v>
       </c>
     </row>
     <row r="119" spans="3:3">
       <c r="C119" t="s">
-        <v>360</v>
+        <v>315</v>
       </c>
     </row>
     <row r="120" spans="3:3">
       <c r="C120" t="s">
-        <v>322</v>
+        <v>358</v>
       </c>
     </row>
     <row r="121" spans="3:3">
       <c r="C121" t="s">
-        <v>323</v>
+        <v>359</v>
       </c>
     </row>
     <row r="122" spans="3:3">
       <c r="C122" t="s">
-        <v>319</v>
+        <v>360</v>
       </c>
     </row>
     <row r="123" spans="3:3">
       <c r="C123" t="s">
-        <v>324</v>
+        <v>361</v>
       </c>
     </row>
     <row r="124" spans="3:3">
       <c r="C124" t="s">
-        <v>325</v>
+        <v>362</v>
       </c>
     </row>
     <row r="125" spans="3:3">
       <c r="C125" t="s">
-        <v>326</v>
+        <v>363</v>
       </c>
     </row>
     <row r="126" spans="3:3">
       <c r="C126" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="127" spans="3:3">
       <c r="C127" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="128" spans="3:3">
       <c r="C128" t="s">
-        <v>329</v>
+        <v>364</v>
       </c>
     </row>
     <row r="129" spans="3:3">
       <c r="C129" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="130" spans="3:3">
       <c r="C130" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="131" spans="3:3">
       <c r="C131" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="132" spans="3:3">
       <c r="C132" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="133" spans="3:3">
       <c r="C133" t="s">
-        <v>321</v>
+        <v>338</v>
       </c>
     </row>
     <row r="134" spans="3:3">
       <c r="C134" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="135" spans="3:3">
       <c r="C135" t="s">
-        <v>361</v>
+        <v>315</v>
       </c>
     </row>
     <row r="136" spans="3:3">
       <c r="C136" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="137" spans="3:3">
       <c r="C137" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="138" spans="3:3">
       <c r="C138" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="139" spans="3:3">
       <c r="C139" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="140" spans="3:3">
       <c r="C140" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
     </row>
     <row r="141" spans="3:3">
       <c r="C141" t="s">
-        <v>319</v>
+        <v>363</v>
       </c>
     </row>
     <row r="142" spans="3:3">
       <c r="C142" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="143" spans="3:3">
       <c r="C143" t="s">
-        <v>367</v>
+        <v>325</v>
       </c>
     </row>
     <row r="144" spans="3:3">
       <c r="C144" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="145" spans="3:3">
       <c r="C145" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="146" spans="3:3">
       <c r="C146" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="147" spans="3:3">
       <c r="C147" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="148" spans="3:3">
       <c r="C148" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
     </row>
     <row r="149" spans="3:3">
       <c r="C149" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="150" spans="3:3">
       <c r="C150" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
     </row>
     <row r="151" spans="3:3">
       <c r="C151" t="s">
-        <v>368</v>
+        <v>321</v>
       </c>
     </row>
     <row r="152" spans="3:3">
       <c r="C152" t="s">
-        <v>369</v>
+        <v>315</v>
       </c>
     </row>
     <row r="153" spans="3:3">
       <c r="C153" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="154" spans="3:3">
       <c r="C154" t="s">
-        <v>371</v>
+        <v>316</v>
       </c>
     </row>
     <row r="155" spans="3:3">
       <c r="C155" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
     </row>
     <row r="156" spans="3:3">
       <c r="C156" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
     </row>
     <row r="157" spans="3:3">
       <c r="C157" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
     </row>
     <row r="158" spans="3:3">
       <c r="C158" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="159" spans="3:3">
@@ -4909,7 +4954,7 @@
     </row>
     <row r="160" spans="3:3">
       <c r="C160" t="s">
-        <v>327</v>
+        <v>372</v>
       </c>
     </row>
     <row r="161" spans="3:3">
@@ -4929,172 +4974,172 @@
     </row>
     <row r="164" spans="3:3">
       <c r="C164" t="s">
-        <v>331</v>
+        <v>373</v>
       </c>
     </row>
     <row r="165" spans="3:3">
       <c r="C165" t="s">
-        <v>338</v>
+        <v>321</v>
       </c>
     </row>
     <row r="166" spans="3:3">
       <c r="C166" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="167" spans="3:3">
       <c r="C167" t="s">
-        <v>315</v>
+        <v>374</v>
       </c>
     </row>
     <row r="168" spans="3:3">
       <c r="C168" t="s">
-        <v>372</v>
+        <v>316</v>
       </c>
     </row>
     <row r="169" spans="3:3">
       <c r="C169" t="s">
-        <v>316</v>
+        <v>375</v>
       </c>
     </row>
     <row r="170" spans="3:3">
       <c r="C170" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="171" spans="3:3">
       <c r="C171" t="s">
-        <v>374</v>
+        <v>335</v>
       </c>
     </row>
     <row r="172" spans="3:3">
       <c r="C172" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
     </row>
     <row r="173" spans="3:3">
       <c r="C173" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="174" spans="3:3">
       <c r="C174" t="s">
-        <v>324</v>
+        <v>372</v>
       </c>
     </row>
     <row r="175" spans="3:3">
       <c r="C175" t="s">
-        <v>375</v>
+        <v>328</v>
       </c>
     </row>
     <row r="176" spans="3:3">
       <c r="C176" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="177" spans="3:3">
       <c r="C177" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="178" spans="3:3">
       <c r="C178" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
     </row>
     <row r="179" spans="3:3">
       <c r="C179" t="s">
-        <v>376</v>
+        <v>321</v>
       </c>
     </row>
     <row r="180" spans="3:3">
       <c r="C180" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="181" spans="3:3">
       <c r="C181" t="s">
-        <v>315</v>
+        <v>376</v>
       </c>
     </row>
     <row r="182" spans="3:3">
       <c r="C182" t="s">
-        <v>377</v>
+        <v>316</v>
       </c>
     </row>
     <row r="183" spans="3:3">
       <c r="C183" t="s">
-        <v>316</v>
+        <v>377</v>
       </c>
     </row>
     <row r="184" spans="3:3">
       <c r="C184" t="s">
-        <v>378</v>
+        <v>371</v>
       </c>
     </row>
     <row r="185" spans="3:3">
       <c r="C185" t="s">
-        <v>374</v>
+        <v>335</v>
       </c>
     </row>
     <row r="186" spans="3:3">
       <c r="C186" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
     </row>
     <row r="187" spans="3:3">
       <c r="C187" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="188" spans="3:3">
       <c r="C188" t="s">
-        <v>324</v>
+        <v>372</v>
       </c>
     </row>
     <row r="189" spans="3:3">
       <c r="C189" t="s">
-        <v>375</v>
+        <v>328</v>
       </c>
     </row>
     <row r="190" spans="3:3">
       <c r="C190" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="191" spans="3:3">
       <c r="C191" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="192" spans="3:3">
       <c r="C192" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
     </row>
     <row r="193" spans="3:3">
       <c r="C193" t="s">
-        <v>376</v>
+        <v>321</v>
       </c>
     </row>
     <row r="194" spans="3:3">
       <c r="C194" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="195" spans="3:3">
       <c r="C195" t="s">
-        <v>315</v>
+        <v>378</v>
       </c>
     </row>
     <row r="196" spans="3:3">
       <c r="C196" t="s">
-        <v>379</v>
+        <v>316</v>
       </c>
     </row>
     <row r="197" spans="3:3">
       <c r="C197" t="s">
-        <v>316</v>
+        <v>379</v>
       </c>
     </row>
     <row r="198" spans="3:3">
@@ -5104,72 +5149,72 @@
     </row>
     <row r="199" spans="3:3">
       <c r="C199" t="s">
-        <v>374</v>
+        <v>335</v>
       </c>
     </row>
     <row r="200" spans="3:3">
       <c r="C200" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
     </row>
     <row r="201" spans="3:3">
       <c r="C201" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="202" spans="3:3">
       <c r="C202" t="s">
-        <v>324</v>
+        <v>372</v>
       </c>
     </row>
     <row r="203" spans="3:3">
       <c r="C203" t="s">
-        <v>375</v>
+        <v>328</v>
       </c>
     </row>
     <row r="204" spans="3:3">
       <c r="C204" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="205" spans="3:3">
       <c r="C205" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="206" spans="3:3">
       <c r="C206" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
     </row>
     <row r="207" spans="3:3">
       <c r="C207" t="s">
-        <v>376</v>
+        <v>321</v>
       </c>
     </row>
     <row r="208" spans="3:3">
       <c r="C208" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="209" spans="3:3">
       <c r="C209" t="s">
-        <v>315</v>
+        <v>381</v>
       </c>
     </row>
     <row r="210" spans="3:3">
       <c r="C210" t="s">
-        <v>381</v>
+        <v>316</v>
       </c>
     </row>
     <row r="211" spans="3:3">
       <c r="C211" t="s">
-        <v>316</v>
+        <v>382</v>
       </c>
     </row>
     <row r="212" spans="3:3">
       <c r="C212" t="s">
-        <v>382</v>
+        <v>362</v>
       </c>
     </row>
     <row r="213" spans="3:3">
@@ -5179,122 +5224,122 @@
     </row>
     <row r="214" spans="3:3">
       <c r="C214" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
     </row>
     <row r="215" spans="3:3">
       <c r="C215" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="216" spans="3:3">
       <c r="C216" t="s">
-        <v>324</v>
+        <v>372</v>
       </c>
     </row>
     <row r="217" spans="3:3">
       <c r="C217" t="s">
-        <v>375</v>
+        <v>328</v>
       </c>
     </row>
     <row r="218" spans="3:3">
       <c r="C218" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="219" spans="3:3">
       <c r="C219" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="220" spans="3:3">
       <c r="C220" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
     </row>
     <row r="221" spans="3:3">
       <c r="C221" t="s">
-        <v>376</v>
+        <v>321</v>
       </c>
     </row>
     <row r="222" spans="3:3">
       <c r="C222" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="223" spans="3:3">
       <c r="C223" t="s">
-        <v>315</v>
+        <v>384</v>
       </c>
     </row>
     <row r="224" spans="3:3">
       <c r="C224" t="s">
-        <v>384</v>
+        <v>316</v>
       </c>
     </row>
     <row r="225" spans="3:3">
       <c r="C225" t="s">
-        <v>316</v>
+        <v>385</v>
       </c>
     </row>
     <row r="226" spans="3:3">
       <c r="C226" t="s">
-        <v>385</v>
+        <v>362</v>
       </c>
     </row>
     <row r="227" spans="3:3">
       <c r="C227" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
     </row>
     <row r="228" spans="3:3">
       <c r="C228" t="s">
-        <v>386</v>
+        <v>319</v>
       </c>
     </row>
     <row r="229" spans="3:3">
       <c r="C229" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="230" spans="3:3">
       <c r="C230" t="s">
-        <v>324</v>
+        <v>372</v>
       </c>
     </row>
     <row r="231" spans="3:3">
       <c r="C231" t="s">
-        <v>375</v>
+        <v>328</v>
       </c>
     </row>
     <row r="232" spans="3:3">
       <c r="C232" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="233" spans="3:3">
       <c r="C233" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="234" spans="3:3">
       <c r="C234" t="s">
-        <v>330</v>
+        <v>373</v>
       </c>
     </row>
     <row r="235" spans="3:3">
       <c r="C235" t="s">
-        <v>376</v>
+        <v>321</v>
       </c>
     </row>
     <row r="236" spans="3:3">
       <c r="C236" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="237" spans="3:3">
       <c r="C237" t="s">
-        <v>315</v>
+        <v>386</v>
       </c>
     </row>
     <row r="238" spans="3:3">
@@ -5304,22 +5349,22 @@
     </row>
     <row r="239" spans="3:3">
       <c r="C239" t="s">
-        <v>316</v>
+        <v>388</v>
       </c>
     </row>
     <row r="240" spans="3:3">
       <c r="C240" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="241" spans="3:3">
       <c r="C241" t="s">
-        <v>365</v>
+        <v>322</v>
       </c>
     </row>
     <row r="242" spans="3:3">
       <c r="C242" t="s">
-        <v>386</v>
+        <v>323</v>
       </c>
     </row>
     <row r="243" spans="3:3">
@@ -5334,987 +5379,987 @@
     </row>
     <row r="245" spans="3:3">
       <c r="C245" t="s">
-        <v>375</v>
+        <v>325</v>
       </c>
     </row>
     <row r="246" spans="3:3">
       <c r="C246" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="247" spans="3:3">
       <c r="C247" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
     </row>
     <row r="248" spans="3:3">
       <c r="C248" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="249" spans="3:3">
       <c r="C249" t="s">
-        <v>376</v>
+        <v>329</v>
       </c>
     </row>
     <row r="250" spans="3:3">
       <c r="C250" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="251" spans="3:3">
       <c r="C251" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="252" spans="3:3">
       <c r="C252" t="s">
-        <v>389</v>
+        <v>332</v>
       </c>
     </row>
     <row r="253" spans="3:3">
       <c r="C253" t="s">
-        <v>390</v>
+        <v>333</v>
       </c>
     </row>
     <row r="254" spans="3:3">
       <c r="C254" t="s">
-        <v>391</v>
+        <v>321</v>
       </c>
     </row>
     <row r="255" spans="3:3">
       <c r="C255" t="s">
-        <v>392</v>
+        <v>315</v>
       </c>
     </row>
     <row r="256" spans="3:3">
       <c r="C256" t="s">
-        <v>322</v>
+        <v>390</v>
       </c>
     </row>
     <row r="257" spans="3:3">
       <c r="C257" t="s">
-        <v>323</v>
+        <v>391</v>
       </c>
     </row>
     <row r="258" spans="3:3">
       <c r="C258" t="s">
-        <v>319</v>
+        <v>392</v>
       </c>
     </row>
     <row r="259" spans="3:3">
       <c r="C259" t="s">
-        <v>324</v>
+        <v>393</v>
       </c>
     </row>
     <row r="260" spans="3:3">
       <c r="C260" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="261" spans="3:3">
       <c r="C261" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="262" spans="3:3">
       <c r="C262" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="263" spans="3:3">
       <c r="C263" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="264" spans="3:3">
       <c r="C264" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="265" spans="3:3">
       <c r="C265" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="266" spans="3:3">
       <c r="C266" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="267" spans="3:3">
       <c r="C267" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="268" spans="3:3">
       <c r="C268" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="269" spans="3:3">
       <c r="C269" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="270" spans="3:3">
       <c r="C270" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="271" spans="3:3">
       <c r="C271" t="s">
-        <v>393</v>
+        <v>332</v>
       </c>
     </row>
     <row r="272" spans="3:3">
       <c r="C272" t="s">
-        <v>394</v>
+        <v>333</v>
       </c>
     </row>
     <row r="273" spans="3:3">
       <c r="C273" t="s">
-        <v>395</v>
+        <v>321</v>
       </c>
     </row>
     <row r="274" spans="3:3">
       <c r="C274" t="s">
-        <v>396</v>
+        <v>315</v>
       </c>
     </row>
     <row r="275" spans="3:3">
       <c r="C275" t="s">
-        <v>322</v>
+        <v>394</v>
       </c>
     </row>
     <row r="276" spans="3:3">
       <c r="C276" t="s">
-        <v>323</v>
+        <v>395</v>
       </c>
     </row>
     <row r="277" spans="3:3">
       <c r="C277" t="s">
-        <v>319</v>
+        <v>396</v>
       </c>
     </row>
     <row r="278" spans="3:3">
       <c r="C278" t="s">
-        <v>324</v>
+        <v>397</v>
       </c>
     </row>
     <row r="279" spans="3:3">
       <c r="C279" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="280" spans="3:3">
       <c r="C280" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="281" spans="3:3">
       <c r="C281" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="282" spans="3:3">
       <c r="C282" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="283" spans="3:3">
       <c r="C283" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="284" spans="3:3">
       <c r="C284" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="285" spans="3:3">
       <c r="C285" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="286" spans="3:3">
       <c r="C286" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="287" spans="3:3">
       <c r="C287" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="288" spans="3:3">
       <c r="C288" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="289" spans="3:3">
       <c r="C289" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="290" spans="3:3">
       <c r="C290" t="s">
-        <v>397</v>
+        <v>332</v>
       </c>
     </row>
     <row r="291" spans="3:3">
       <c r="C291" t="s">
-        <v>398</v>
+        <v>333</v>
       </c>
     </row>
     <row r="292" spans="3:3">
       <c r="C292" t="s">
-        <v>399</v>
+        <v>321</v>
       </c>
     </row>
     <row r="293" spans="3:3">
       <c r="C293" t="s">
-        <v>400</v>
+        <v>315</v>
       </c>
     </row>
     <row r="294" spans="3:3">
       <c r="C294" t="s">
-        <v>322</v>
+        <v>398</v>
       </c>
     </row>
     <row r="295" spans="3:3">
       <c r="C295" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
     </row>
     <row r="296" spans="3:3">
       <c r="C296" t="s">
-        <v>319</v>
+        <v>399</v>
       </c>
     </row>
     <row r="297" spans="3:3">
       <c r="C297" t="s">
-        <v>324</v>
+        <v>400</v>
       </c>
     </row>
     <row r="298" spans="3:3">
       <c r="C298" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="299" spans="3:3">
       <c r="C299" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="300" spans="3:3">
       <c r="C300" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="301" spans="3:3">
       <c r="C301" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="302" spans="3:3">
       <c r="C302" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="303" spans="3:3">
       <c r="C303" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="304" spans="3:3">
       <c r="C304" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="305" spans="3:3">
       <c r="C305" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="306" spans="3:3">
       <c r="C306" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="307" spans="3:3">
       <c r="C307" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="308" spans="3:3">
       <c r="C308" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="309" spans="3:3">
       <c r="C309" t="s">
-        <v>401</v>
+        <v>332</v>
       </c>
     </row>
     <row r="310" spans="3:3">
       <c r="C310" t="s">
-        <v>316</v>
+        <v>333</v>
       </c>
     </row>
     <row r="311" spans="3:3">
       <c r="C311" t="s">
-        <v>402</v>
+        <v>321</v>
       </c>
     </row>
     <row r="312" spans="3:3">
       <c r="C312" t="s">
-        <v>403</v>
+        <v>315</v>
       </c>
     </row>
     <row r="313" spans="3:3">
       <c r="C313" t="s">
-        <v>322</v>
+        <v>401</v>
       </c>
     </row>
     <row r="314" spans="3:3">
       <c r="C314" t="s">
-        <v>323</v>
+        <v>334</v>
       </c>
     </row>
     <row r="315" spans="3:3">
       <c r="C315" t="s">
-        <v>319</v>
+        <v>402</v>
       </c>
     </row>
     <row r="316" spans="3:3">
       <c r="C316" t="s">
-        <v>324</v>
+        <v>403</v>
       </c>
     </row>
     <row r="317" spans="3:3">
       <c r="C317" t="s">
-        <v>325</v>
+        <v>371</v>
       </c>
     </row>
     <row r="318" spans="3:3">
       <c r="C318" t="s">
-        <v>326</v>
+        <v>404</v>
       </c>
     </row>
     <row r="319" spans="3:3">
       <c r="C319" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="320" spans="3:3">
       <c r="C320" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="321" spans="3:3">
       <c r="C321" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="322" spans="3:3">
       <c r="C322" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="323" spans="3:3">
       <c r="C323" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="324" spans="3:3">
       <c r="C324" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="325" spans="3:3">
       <c r="C325" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="326" spans="3:3">
       <c r="C326" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="327" spans="3:3">
       <c r="C327" t="s">
-        <v>315</v>
+        <v>405</v>
       </c>
     </row>
     <row r="328" spans="3:3">
       <c r="C328" t="s">
-        <v>404</v>
+        <v>321</v>
       </c>
     </row>
     <row r="329" spans="3:3">
       <c r="C329" t="s">
-        <v>334</v>
+        <v>315</v>
       </c>
     </row>
     <row r="330" spans="3:3">
       <c r="C330" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
     </row>
     <row r="331" spans="3:3">
       <c r="C331" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
     </row>
     <row r="332" spans="3:3">
       <c r="C332" t="s">
-        <v>374</v>
+        <v>408</v>
       </c>
     </row>
     <row r="333" spans="3:3">
       <c r="C333" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
     </row>
     <row r="334" spans="3:3">
       <c r="C334" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="335" spans="3:3">
       <c r="C335" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="336" spans="3:3">
       <c r="C336" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="337" spans="3:3">
       <c r="C337" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="338" spans="3:3">
       <c r="C338" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="339" spans="3:3">
       <c r="C339" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="340" spans="3:3">
       <c r="C340" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="341" spans="3:3">
       <c r="C341" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="342" spans="3:3">
       <c r="C342" t="s">
-        <v>408</v>
+        <v>329</v>
       </c>
     </row>
     <row r="343" spans="3:3">
       <c r="C343" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="344" spans="3:3">
       <c r="C344" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="345" spans="3:3">
       <c r="C345" t="s">
-        <v>409</v>
+        <v>332</v>
       </c>
     </row>
     <row r="346" spans="3:3">
       <c r="C346" t="s">
-        <v>410</v>
+        <v>333</v>
       </c>
     </row>
     <row r="347" spans="3:3">
       <c r="C347" t="s">
-        <v>411</v>
+        <v>321</v>
       </c>
     </row>
     <row r="348" spans="3:3">
       <c r="C348" t="s">
-        <v>412</v>
+        <v>315</v>
       </c>
     </row>
     <row r="349" spans="3:3">
       <c r="C349" t="s">
-        <v>322</v>
+        <v>410</v>
       </c>
     </row>
     <row r="350" spans="3:3">
       <c r="C350" t="s">
-        <v>323</v>
+        <v>411</v>
       </c>
     </row>
     <row r="351" spans="3:3">
       <c r="C351" t="s">
-        <v>319</v>
+        <v>412</v>
       </c>
     </row>
     <row r="352" spans="3:3">
       <c r="C352" t="s">
-        <v>324</v>
+        <v>413</v>
       </c>
     </row>
     <row r="353" spans="3:3">
       <c r="C353" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="354" spans="3:3">
       <c r="C354" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="355" spans="3:3">
       <c r="C355" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="356" spans="3:3">
       <c r="C356" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="357" spans="3:3">
       <c r="C357" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="358" spans="3:3">
       <c r="C358" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="359" spans="3:3">
       <c r="C359" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="360" spans="3:3">
       <c r="C360" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="361" spans="3:3">
       <c r="C361" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="362" spans="3:3">
       <c r="C362" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="363" spans="3:3">
       <c r="C363" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="364" spans="3:3">
       <c r="C364" t="s">
-        <v>413</v>
+        <v>332</v>
       </c>
     </row>
     <row r="365" spans="3:3">
       <c r="C365" t="s">
-        <v>414</v>
+        <v>333</v>
       </c>
     </row>
     <row r="366" spans="3:3">
       <c r="C366" t="s">
-        <v>415</v>
+        <v>321</v>
       </c>
     </row>
     <row r="367" spans="3:3">
       <c r="C367" t="s">
-        <v>416</v>
+        <v>315</v>
       </c>
     </row>
     <row r="368" spans="3:3">
       <c r="C368" t="s">
-        <v>322</v>
+        <v>414</v>
       </c>
     </row>
     <row r="369" spans="3:3">
       <c r="C369" t="s">
-        <v>323</v>
+        <v>415</v>
       </c>
     </row>
     <row r="370" spans="3:3">
       <c r="C370" t="s">
-        <v>319</v>
+        <v>416</v>
       </c>
     </row>
     <row r="371" spans="3:3">
       <c r="C371" t="s">
-        <v>324</v>
+        <v>417</v>
       </c>
     </row>
     <row r="372" spans="3:3">
       <c r="C372" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="373" spans="3:3">
       <c r="C373" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="374" spans="3:3">
       <c r="C374" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="375" spans="3:3">
       <c r="C375" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="376" spans="3:3">
       <c r="C376" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="377" spans="3:3">
       <c r="C377" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="378" spans="3:3">
       <c r="C378" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="379" spans="3:3">
       <c r="C379" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="380" spans="3:3">
       <c r="C380" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="381" spans="3:3">
       <c r="C381" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="382" spans="3:3">
       <c r="C382" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="383" spans="3:3">
       <c r="C383" t="s">
-        <v>417</v>
+        <v>332</v>
       </c>
     </row>
     <row r="384" spans="3:3">
       <c r="C384" t="s">
-        <v>418</v>
+        <v>333</v>
       </c>
     </row>
     <row r="385" spans="3:3">
       <c r="C385" t="s">
-        <v>419</v>
+        <v>321</v>
       </c>
     </row>
     <row r="386" spans="3:3">
       <c r="C386" t="s">
-        <v>420</v>
+        <v>315</v>
       </c>
     </row>
     <row r="387" spans="3:3">
       <c r="C387" t="s">
-        <v>322</v>
+        <v>418</v>
       </c>
     </row>
     <row r="388" spans="3:3">
       <c r="C388" t="s">
-        <v>323</v>
+        <v>419</v>
       </c>
     </row>
     <row r="389" spans="3:3">
       <c r="C389" t="s">
-        <v>319</v>
+        <v>420</v>
       </c>
     </row>
     <row r="390" spans="3:3">
       <c r="C390" t="s">
-        <v>324</v>
+        <v>421</v>
       </c>
     </row>
     <row r="391" spans="3:3">
       <c r="C391" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="392" spans="3:3">
       <c r="C392" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="393" spans="3:3">
       <c r="C393" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="394" spans="3:3">
       <c r="C394" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="395" spans="3:3">
       <c r="C395" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="396" spans="3:3">
       <c r="C396" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="397" spans="3:3">
       <c r="C397" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="398" spans="3:3">
       <c r="C398" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
     </row>
     <row r="399" spans="3:3">
       <c r="C399" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="400" spans="3:3">
       <c r="C400" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="401" spans="3:3">
       <c r="C401" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
     </row>
     <row r="402" spans="3:3">
       <c r="C402" t="s">
-        <v>421</v>
+        <v>332</v>
       </c>
     </row>
     <row r="403" spans="3:3">
       <c r="C403" t="s">
-        <v>422</v>
+        <v>333</v>
       </c>
     </row>
     <row r="404" spans="3:3">
       <c r="C404" t="s">
-        <v>423</v>
+        <v>321</v>
       </c>
     </row>
     <row r="405" spans="3:3">
       <c r="C405" t="s">
-        <v>424</v>
+        <v>315</v>
       </c>
     </row>
     <row r="406" spans="3:3">
       <c r="C406" t="s">
-        <v>322</v>
+        <v>422</v>
       </c>
     </row>
     <row r="407" spans="3:3">
       <c r="C407" t="s">
-        <v>323</v>
+        <v>423</v>
       </c>
     </row>
     <row r="408" spans="3:3">
       <c r="C408" t="s">
-        <v>319</v>
+        <v>424</v>
       </c>
     </row>
     <row r="409" spans="3:3">
       <c r="C409" t="s">
-        <v>324</v>
+        <v>425</v>
       </c>
     </row>
     <row r="410" spans="3:3">
       <c r="C410" t="s">
-        <v>325</v>
+        <v>380</v>
       </c>
     </row>
     <row r="411" spans="3:3">
       <c r="C411" t="s">
-        <v>326</v>
+        <v>404</v>
       </c>
     </row>
     <row r="412" spans="3:3">
       <c r="C412" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="413" spans="3:3">
       <c r="C413" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="414" spans="3:3">
       <c r="C414" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="415" spans="3:3">
       <c r="C415" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="416" spans="3:3">
       <c r="C416" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="417" spans="3:3">
       <c r="C417" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="418" spans="3:3">
       <c r="C418" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="419" spans="3:3">
       <c r="C419" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="420" spans="3:3">
       <c r="C420" t="s">
-        <v>315</v>
+        <v>426</v>
       </c>
     </row>
     <row r="421" spans="3:3">
       <c r="C421" t="s">
-        <v>425</v>
+        <v>333</v>
       </c>
     </row>
     <row r="422" spans="3:3">
       <c r="C422" t="s">
-        <v>426</v>
+        <v>321</v>
       </c>
     </row>
     <row r="423" spans="3:3">
       <c r="C423" t="s">
-        <v>427</v>
+        <v>315</v>
       </c>
     </row>
     <row r="424" spans="3:3">
       <c r="C424" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="425" spans="3:3">
       <c r="C425" t="s">
-        <v>383</v>
+        <v>423</v>
       </c>
     </row>
     <row r="426" spans="3:3">
       <c r="C426" t="s">
-        <v>407</v>
+        <v>424</v>
       </c>
     </row>
     <row r="427" spans="3:3">
       <c r="C427" t="s">
-        <v>319</v>
+        <v>425</v>
       </c>
     </row>
     <row r="428" spans="3:3">
       <c r="C428" t="s">
-        <v>324</v>
+        <v>380</v>
       </c>
     </row>
     <row r="429" spans="3:3">
       <c r="C429" t="s">
-        <v>325</v>
+        <v>404</v>
       </c>
     </row>
     <row r="430" spans="3:3">
       <c r="C430" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="431" spans="3:3">
       <c r="C431" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="432" spans="3:3">
       <c r="C432" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
     </row>
     <row r="433" spans="3:3">
       <c r="C433" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="434" spans="3:3">
       <c r="C434" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
     </row>
     <row r="435" spans="3:3">
       <c r="C435" t="s">
-        <v>429</v>
+        <v>329</v>
       </c>
     </row>
     <row r="436" spans="3:3">
       <c r="C436" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="437" spans="3:3">
       <c r="C437" t="s">
-        <v>321</v>
+        <v>331</v>
       </c>
     </row>
     <row r="438" spans="3:3">
       <c r="C438" t="s">
-        <v>315</v>
+        <v>426</v>
       </c>
     </row>
     <row r="439" spans="3:3">
       <c r="C439" t="s">
-        <v>430</v>
+        <v>333</v>
       </c>
     </row>
     <row r="440" spans="3:3">
       <c r="C440" t="s">
-        <v>426</v>
+        <v>321</v>
       </c>
     </row>
     <row r="441" spans="3:3">
       <c r="C441" t="s">
-        <v>427</v>
+        <v>315</v>
       </c>
     </row>
     <row r="442" spans="3:3">
@@ -6324,502 +6369,502 @@
     </row>
     <row r="443" spans="3:3">
       <c r="C443" t="s">
-        <v>383</v>
+        <v>429</v>
       </c>
     </row>
     <row r="444" spans="3:3">
       <c r="C444" t="s">
-        <v>407</v>
+        <v>430</v>
       </c>
     </row>
     <row r="445" spans="3:3">
       <c r="C445" t="s">
-        <v>319</v>
+        <v>431</v>
       </c>
     </row>
     <row r="446" spans="3:3">
       <c r="C446" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="447" spans="3:3">
       <c r="C447" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="448" spans="3:3">
       <c r="C448" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
     </row>
     <row r="449" spans="3:3">
       <c r="C449" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="450" spans="3:3">
       <c r="C450" t="s">
-        <v>329</v>
+        <v>372</v>
       </c>
     </row>
     <row r="451" spans="3:3">
       <c r="C451" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="452" spans="3:3">
       <c r="C452" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="453" spans="3:3">
       <c r="C453" t="s">
-        <v>429</v>
+        <v>330</v>
       </c>
     </row>
     <row r="454" spans="3:3">
       <c r="C454" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="455" spans="3:3">
       <c r="C455" t="s">
-        <v>321</v>
+        <v>332</v>
       </c>
     </row>
     <row r="456" spans="3:3">
       <c r="C456" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="457" spans="3:3">
       <c r="C457" t="s">
-        <v>431</v>
+        <v>321</v>
       </c>
     </row>
     <row r="458" spans="3:3">
       <c r="C458" t="s">
-        <v>432</v>
+        <v>315</v>
       </c>
     </row>
     <row r="459" spans="3:3">
       <c r="C459" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="460" spans="3:3">
       <c r="C460" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="461" spans="3:3">
       <c r="C461" t="s">
-        <v>322</v>
+        <v>434</v>
       </c>
     </row>
     <row r="462" spans="3:3">
       <c r="C462" t="s">
-        <v>323</v>
+        <v>435</v>
       </c>
     </row>
     <row r="463" spans="3:3">
       <c r="C463" t="s">
-        <v>319</v>
+        <v>380</v>
       </c>
     </row>
     <row r="464" spans="3:3">
       <c r="C464" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="465" spans="3:3">
       <c r="C465" t="s">
-        <v>375</v>
+        <v>319</v>
       </c>
     </row>
     <row r="466" spans="3:3">
       <c r="C466" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="467" spans="3:3">
       <c r="C467" t="s">
-        <v>329</v>
+        <v>372</v>
       </c>
     </row>
     <row r="468" spans="3:3">
       <c r="C468" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="469" spans="3:3">
       <c r="C469" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="470" spans="3:3">
       <c r="C470" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="471" spans="3:3">
       <c r="C471" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="472" spans="3:3">
       <c r="C472" t="s">
-        <v>321</v>
+        <v>332</v>
       </c>
     </row>
     <row r="473" spans="3:3">
       <c r="C473" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="474" spans="3:3">
       <c r="C474" t="s">
-        <v>435</v>
+        <v>321</v>
       </c>
     </row>
     <row r="475" spans="3:3">
       <c r="C475" t="s">
-        <v>436</v>
+        <v>315</v>
       </c>
     </row>
     <row r="476" spans="3:3">
       <c r="C476" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="477" spans="3:3">
       <c r="C477" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="478" spans="3:3">
       <c r="C478" t="s">
-        <v>383</v>
+        <v>438</v>
       </c>
     </row>
     <row r="479" spans="3:3">
       <c r="C479" t="s">
-        <v>323</v>
+        <v>439</v>
       </c>
     </row>
     <row r="480" spans="3:3">
       <c r="C480" t="s">
-        <v>319</v>
+        <v>380</v>
       </c>
     </row>
     <row r="481" spans="3:3">
       <c r="C481" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="482" spans="3:3">
       <c r="C482" t="s">
-        <v>375</v>
+        <v>319</v>
       </c>
     </row>
     <row r="483" spans="3:3">
       <c r="C483" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
     </row>
     <row r="484" spans="3:3">
       <c r="C484" t="s">
-        <v>329</v>
+        <v>372</v>
       </c>
     </row>
     <row r="485" spans="3:3">
       <c r="C485" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="486" spans="3:3">
       <c r="C486" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
     </row>
     <row r="487" spans="3:3">
       <c r="C487" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="488" spans="3:3">
       <c r="C488" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="489" spans="3:3">
       <c r="C489" t="s">
-        <v>321</v>
+        <v>332</v>
       </c>
     </row>
     <row r="490" spans="3:3">
       <c r="C490" t="s">
-        <v>315</v>
+        <v>333</v>
       </c>
     </row>
     <row r="491" spans="3:3">
       <c r="C491" t="s">
-        <v>439</v>
+        <v>321</v>
       </c>
     </row>
     <row r="492" spans="3:3">
       <c r="C492" t="s">
-        <v>440</v>
+        <v>315</v>
       </c>
     </row>
     <row r="493" spans="3:3">
       <c r="C493" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="494" spans="3:3">
       <c r="C494" t="s">
-        <v>442</v>
+        <v>316</v>
       </c>
     </row>
     <row r="495" spans="3:3">
       <c r="C495" t="s">
-        <v>383</v>
+        <v>441</v>
       </c>
     </row>
     <row r="496" spans="3:3">
       <c r="C496" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
     </row>
     <row r="497" spans="3:3">
       <c r="C497" t="s">
-        <v>319</v>
+        <v>442</v>
       </c>
     </row>
     <row r="498" spans="3:3">
       <c r="C498" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="499" spans="3:3">
       <c r="C499" t="s">
-        <v>375</v>
+        <v>319</v>
       </c>
     </row>
     <row r="500" spans="3:3">
       <c r="C500" t="s">
-        <v>328</v>
+        <v>443</v>
       </c>
     </row>
     <row r="501" spans="3:3">
       <c r="C501" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
     </row>
     <row r="502" spans="3:3">
       <c r="C502" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
     </row>
     <row r="503" spans="3:3">
       <c r="C503" t="s">
-        <v>331</v>
+        <v>315</v>
       </c>
     </row>
     <row r="504" spans="3:3">
       <c r="C504" t="s">
-        <v>332</v>
+        <v>444</v>
       </c>
     </row>
     <row r="505" spans="3:3">
       <c r="C505" t="s">
-        <v>333</v>
+        <v>445</v>
       </c>
     </row>
     <row r="506" spans="3:3">
       <c r="C506" t="s">
-        <v>321</v>
+        <v>446</v>
       </c>
     </row>
     <row r="507" spans="3:3">
       <c r="C507" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="508" spans="3:3">
       <c r="C508" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="509" spans="3:3">
       <c r="C509" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="510" spans="3:3">
       <c r="C510" t="s">
-        <v>444</v>
+        <v>319</v>
       </c>
     </row>
     <row r="511" spans="3:3">
       <c r="C511" t="s">
-        <v>317</v>
+        <v>443</v>
       </c>
     </row>
     <row r="512" spans="3:3">
       <c r="C512" t="s">
-        <v>445</v>
+        <v>320</v>
       </c>
     </row>
     <row r="513" spans="3:3">
       <c r="C513" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
     </row>
     <row r="514" spans="3:3">
       <c r="C514" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="515" spans="3:3">
       <c r="C515" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
     </row>
     <row r="516" spans="3:3">
       <c r="C516" t="s">
-        <v>320</v>
+        <v>448</v>
       </c>
     </row>
     <row r="517" spans="3:3">
       <c r="C517" t="s">
-        <v>321</v>
+        <v>449</v>
       </c>
     </row>
     <row r="518" spans="3:3">
       <c r="C518" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
     </row>
     <row r="519" spans="3:3">
       <c r="C519" t="s">
-        <v>447</v>
+        <v>362</v>
       </c>
     </row>
     <row r="520" spans="3:3">
       <c r="C520" t="s">
-        <v>448</v>
+        <v>318</v>
       </c>
     </row>
     <row r="521" spans="3:3">
       <c r="C521" t="s">
-        <v>449</v>
+        <v>319</v>
       </c>
     </row>
     <row r="522" spans="3:3">
       <c r="C522" t="s">
-        <v>317</v>
+        <v>450</v>
       </c>
     </row>
     <row r="523" spans="3:3">
       <c r="C523" t="s">
-        <v>445</v>
+        <v>451</v>
       </c>
     </row>
     <row r="524" spans="3:3">
       <c r="C524" t="s">
-        <v>318</v>
+        <v>372</v>
       </c>
     </row>
     <row r="525" spans="3:3">
       <c r="C525" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="526" spans="3:3">
       <c r="C526" t="s">
-        <v>446</v>
+        <v>321</v>
       </c>
     </row>
     <row r="527" spans="3:3">
       <c r="C527" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
     </row>
     <row r="528" spans="3:3">
       <c r="C528" t="s">
-        <v>321</v>
+        <v>452</v>
       </c>
     </row>
     <row r="529" spans="3:3">
       <c r="C529" t="s">
-        <v>315</v>
+        <v>448</v>
       </c>
     </row>
     <row r="530" spans="3:3">
       <c r="C530" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
     </row>
     <row r="531" spans="3:3">
       <c r="C531" t="s">
-        <v>451</v>
+        <v>317</v>
       </c>
     </row>
     <row r="532" spans="3:3">
       <c r="C532" t="s">
-        <v>452</v>
+        <v>362</v>
       </c>
     </row>
     <row r="533" spans="3:3">
       <c r="C533" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="534" spans="3:3">
       <c r="C534" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
     </row>
     <row r="535" spans="3:3">
       <c r="C535" t="s">
-        <v>318</v>
+        <v>450</v>
       </c>
     </row>
     <row r="536" spans="3:3">
       <c r="C536" t="s">
-        <v>319</v>
+        <v>451</v>
       </c>
     </row>
     <row r="537" spans="3:3">
       <c r="C537" t="s">
-        <v>453</v>
+        <v>372</v>
       </c>
     </row>
     <row r="538" spans="3:3">
       <c r="C538" t="s">
-        <v>454</v>
+        <v>320</v>
       </c>
     </row>
     <row r="539" spans="3:3">
       <c r="C539" t="s">
-        <v>375</v>
+        <v>321</v>
       </c>
     </row>
     <row r="540" spans="3:3">
       <c r="C540" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
     </row>
     <row r="541" spans="3:3">
       <c r="C541" t="s">
-        <v>321</v>
+        <v>454</v>
       </c>
     </row>
     <row r="542" spans="3:3">
       <c r="C542" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="543" spans="3:3">
@@ -6829,762 +6874,687 @@
     </row>
     <row r="544" spans="3:3">
       <c r="C544" t="s">
-        <v>451</v>
+        <v>317</v>
       </c>
     </row>
     <row r="545" spans="3:3">
       <c r="C545" t="s">
-        <v>456</v>
+        <v>442</v>
       </c>
     </row>
     <row r="546" spans="3:3">
       <c r="C546" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="547" spans="3:3">
       <c r="C547" t="s">
-        <v>365</v>
+        <v>319</v>
       </c>
     </row>
     <row r="548" spans="3:3">
       <c r="C548" t="s">
-        <v>318</v>
+        <v>450</v>
       </c>
     </row>
     <row r="549" spans="3:3">
       <c r="C549" t="s">
-        <v>319</v>
+        <v>451</v>
       </c>
     </row>
     <row r="550" spans="3:3">
       <c r="C550" t="s">
-        <v>453</v>
+        <v>325</v>
       </c>
     </row>
     <row r="551" spans="3:3">
       <c r="C551" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="552" spans="3:3">
       <c r="C552" t="s">
-        <v>375</v>
+        <v>320</v>
       </c>
     </row>
     <row r="553" spans="3:3">
       <c r="C553" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="554" spans="3:3">
       <c r="C554" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="555" spans="3:3">
       <c r="C555" t="s">
-        <v>315</v>
+        <v>457</v>
       </c>
     </row>
     <row r="556" spans="3:3">
       <c r="C556" t="s">
-        <v>457</v>
+        <v>316</v>
       </c>
     </row>
     <row r="557" spans="3:3">
       <c r="C557" t="s">
-        <v>316</v>
+        <v>458</v>
       </c>
     </row>
     <row r="558" spans="3:3">
       <c r="C558" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="559" spans="3:3">
       <c r="C559" t="s">
-        <v>317</v>
+        <v>460</v>
       </c>
     </row>
     <row r="560" spans="3:3">
       <c r="C560" t="s">
-        <v>445</v>
+        <v>461</v>
       </c>
     </row>
     <row r="561" spans="3:3">
       <c r="C561" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
     </row>
     <row r="562" spans="3:3">
       <c r="C562" t="s">
-        <v>319</v>
+        <v>462</v>
       </c>
     </row>
     <row r="563" spans="3:3">
       <c r="C563" t="s">
-        <v>453</v>
+        <v>328</v>
       </c>
     </row>
     <row r="564" spans="3:3">
       <c r="C564" t="s">
-        <v>454</v>
+        <v>463</v>
       </c>
     </row>
     <row r="565" spans="3:3">
       <c r="C565" t="s">
-        <v>325</v>
+        <v>464</v>
       </c>
     </row>
     <row r="566" spans="3:3">
       <c r="C566" t="s">
-        <v>459</v>
+        <v>465</v>
       </c>
     </row>
     <row r="567" spans="3:3">
       <c r="C567" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="568" spans="3:3">
       <c r="C568" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="569" spans="3:3">
       <c r="C569" t="s">
-        <v>315</v>
+        <v>466</v>
       </c>
     </row>
     <row r="570" spans="3:3">
       <c r="C570" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
     </row>
     <row r="571" spans="3:3">
       <c r="C571" t="s">
-        <v>316</v>
+        <v>468</v>
       </c>
     </row>
     <row r="572" spans="3:3">
       <c r="C572" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
     </row>
     <row r="573" spans="3:3">
       <c r="C573" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
     </row>
     <row r="574" spans="3:3">
       <c r="C574" t="s">
-        <v>463</v>
+        <v>335</v>
       </c>
     </row>
     <row r="575" spans="3:3">
       <c r="C575" t="s">
-        <v>464</v>
+        <v>319</v>
       </c>
     </row>
     <row r="576" spans="3:3">
       <c r="C576" t="s">
-        <v>319</v>
+        <v>471</v>
       </c>
     </row>
     <row r="577" spans="3:3">
       <c r="C577" t="s">
-        <v>465</v>
+        <v>320</v>
       </c>
     </row>
     <row r="578" spans="3:3">
       <c r="C578" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="579" spans="3:3">
       <c r="C579" t="s">
-        <v>466</v>
+        <v>315</v>
       </c>
     </row>
     <row r="580" spans="3:3">
       <c r="C580" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
     </row>
     <row r="581" spans="3:3">
       <c r="C581" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="582" spans="3:3">
       <c r="C582" t="s">
-        <v>321</v>
+        <v>473</v>
       </c>
     </row>
     <row r="583" spans="3:3">
       <c r="C583" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="584" spans="3:3">
       <c r="C584" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="585" spans="3:3">
       <c r="C585" t="s">
-        <v>470</v>
+        <v>335</v>
       </c>
     </row>
     <row r="586" spans="3:3">
       <c r="C586" t="s">
-        <v>471</v>
+        <v>319</v>
       </c>
     </row>
     <row r="587" spans="3:3">
       <c r="C587" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="588" spans="3:3">
       <c r="C588" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="589" spans="3:3">
       <c r="C589" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="590" spans="3:3">
       <c r="C590" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="591" spans="3:3">
       <c r="C591" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
     </row>
     <row r="592" spans="3:3">
       <c r="C592" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="593" spans="3:3">
       <c r="C593" t="s">
-        <v>321</v>
+        <v>476</v>
       </c>
     </row>
     <row r="594" spans="3:3">
       <c r="C594" t="s">
-        <v>315</v>
+        <v>469</v>
       </c>
     </row>
     <row r="595" spans="3:3">
       <c r="C595" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
     </row>
     <row r="596" spans="3:3">
       <c r="C596" t="s">
-        <v>470</v>
+        <v>335</v>
       </c>
     </row>
     <row r="597" spans="3:3">
       <c r="C597" t="s">
-        <v>476</v>
+        <v>319</v>
       </c>
     </row>
     <row r="598" spans="3:3">
       <c r="C598" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
     </row>
     <row r="599" spans="3:3">
       <c r="C599" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="600" spans="3:3">
       <c r="C600" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="601" spans="3:3">
       <c r="C601" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="602" spans="3:3">
       <c r="C602" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="603" spans="3:3">
       <c r="C603" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="604" spans="3:3">
       <c r="C604" t="s">
-        <v>321</v>
+        <v>478</v>
       </c>
     </row>
     <row r="605" spans="3:3">
       <c r="C605" t="s">
-        <v>315</v>
+        <v>474</v>
       </c>
     </row>
     <row r="606" spans="3:3">
       <c r="C606" t="s">
-        <v>478</v>
+        <v>470</v>
       </c>
     </row>
     <row r="607" spans="3:3">
       <c r="C607" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
     </row>
     <row r="608" spans="3:3">
       <c r="C608" t="s">
-        <v>479</v>
+        <v>319</v>
       </c>
     </row>
     <row r="609" spans="3:3">
       <c r="C609" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="610" spans="3:3">
       <c r="C610" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="611" spans="3:3">
       <c r="C611" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="612" spans="3:3">
       <c r="C612" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="613" spans="3:3">
       <c r="C613" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
     </row>
     <row r="614" spans="3:3">
       <c r="C614" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="615" spans="3:3">
       <c r="C615" t="s">
-        <v>321</v>
+        <v>480</v>
       </c>
     </row>
     <row r="616" spans="3:3">
       <c r="C616" t="s">
-        <v>315</v>
+        <v>481</v>
       </c>
     </row>
     <row r="617" spans="3:3">
       <c r="C617" t="s">
-        <v>480</v>
+        <v>470</v>
       </c>
     </row>
     <row r="618" spans="3:3">
       <c r="C618" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
     </row>
     <row r="619" spans="3:3">
       <c r="C619" t="s">
-        <v>481</v>
+        <v>319</v>
       </c>
     </row>
     <row r="620" spans="3:3">
       <c r="C620" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
     </row>
     <row r="621" spans="3:3">
       <c r="C621" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="622" spans="3:3">
       <c r="C622" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="623" spans="3:3">
       <c r="C623" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="624" spans="3:3">
       <c r="C624" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
     </row>
     <row r="625" spans="3:3">
       <c r="C625" t="s">
-        <v>320</v>
+        <v>334</v>
       </c>
     </row>
     <row r="626" spans="3:3">
       <c r="C626" t="s">
-        <v>321</v>
+        <v>483</v>
       </c>
     </row>
     <row r="627" spans="3:3">
       <c r="C627" t="s">
-        <v>315</v>
+        <v>484</v>
       </c>
     </row>
     <row r="628" spans="3:3">
       <c r="C628" t="s">
-        <v>482</v>
+        <v>470</v>
       </c>
     </row>
     <row r="629" spans="3:3">
       <c r="C629" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
     </row>
     <row r="630" spans="3:3">
       <c r="C630" t="s">
-        <v>483</v>
+        <v>319</v>
       </c>
     </row>
     <row r="631" spans="3:3">
       <c r="C631" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="632" spans="3:3">
       <c r="C632" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="633" spans="3:3">
       <c r="C633" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="634" spans="3:3">
       <c r="C634" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="635" spans="3:3">
       <c r="C635" t="s">
-        <v>474</v>
+        <v>486</v>
       </c>
     </row>
     <row r="636" spans="3:3">
       <c r="C636" t="s">
-        <v>320</v>
+        <v>423</v>
       </c>
     </row>
     <row r="637" spans="3:3">
       <c r="C637" t="s">
-        <v>321</v>
+        <v>487</v>
       </c>
     </row>
     <row r="638" spans="3:3">
       <c r="C638" t="s">
-        <v>315</v>
+        <v>488</v>
       </c>
     </row>
     <row r="639" spans="3:3">
       <c r="C639" t="s">
-        <v>485</v>
+        <v>470</v>
       </c>
     </row>
     <row r="640" spans="3:3">
       <c r="C640" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="641" spans="3:3">
       <c r="C641" t="s">
-        <v>486</v>
+        <v>319</v>
       </c>
     </row>
     <row r="642" spans="3:3">
       <c r="C642" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="643" spans="3:3">
       <c r="C643" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="644" spans="3:3">
       <c r="C644" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="645" spans="3:3">
       <c r="C645" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="646" spans="3:3">
       <c r="C646" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
     </row>
     <row r="647" spans="3:3">
       <c r="C647" t="s">
-        <v>320</v>
+        <v>423</v>
       </c>
     </row>
     <row r="648" spans="3:3">
       <c r="C648" t="s">
-        <v>321</v>
+        <v>490</v>
       </c>
     </row>
     <row r="649" spans="3:3">
       <c r="C649" t="s">
-        <v>315</v>
+        <v>491</v>
       </c>
     </row>
     <row r="650" spans="3:3">
       <c r="C650" t="s">
-        <v>489</v>
+        <v>470</v>
       </c>
     </row>
     <row r="651" spans="3:3">
       <c r="C651" t="s">
-        <v>426</v>
+        <v>335</v>
       </c>
     </row>
     <row r="652" spans="3:3">
       <c r="C652" t="s">
-        <v>490</v>
+        <v>319</v>
       </c>
     </row>
     <row r="653" spans="3:3">
       <c r="C653" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
     </row>
     <row r="654" spans="3:3">
       <c r="C654" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="655" spans="3:3">
       <c r="C655" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="656" spans="3:3">
       <c r="C656" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="657" spans="3:3">
       <c r="C657" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
     </row>
     <row r="658" spans="3:3">
       <c r="C658" t="s">
-        <v>320</v>
+        <v>493</v>
       </c>
     </row>
     <row r="659" spans="3:3">
       <c r="C659" t="s">
-        <v>321</v>
+        <v>494</v>
       </c>
     </row>
     <row r="660" spans="3:3">
       <c r="C660" t="s">
-        <v>315</v>
+        <v>495</v>
       </c>
     </row>
     <row r="661" spans="3:3">
       <c r="C661" t="s">
-        <v>492</v>
+        <v>470</v>
       </c>
     </row>
     <row r="662" spans="3:3">
       <c r="C662" t="s">
-        <v>426</v>
+        <v>335</v>
       </c>
     </row>
     <row r="663" spans="3:3">
       <c r="C663" t="s">
-        <v>493</v>
+        <v>319</v>
       </c>
     </row>
     <row r="664" spans="3:3">
       <c r="C664" t="s">
-        <v>494</v>
+        <v>485</v>
       </c>
     </row>
     <row r="665" spans="3:3">
       <c r="C665" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="666" spans="3:3">
       <c r="C666" t="s">
-        <v>335</v>
+        <v>321</v>
       </c>
     </row>
     <row r="667" spans="3:3">
       <c r="C667" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="668" spans="3:3">
       <c r="C668" t="s">
-        <v>488</v>
+        <v>496</v>
       </c>
     </row>
     <row r="669" spans="3:3">
       <c r="C669" t="s">
-        <v>320</v>
+        <v>493</v>
       </c>
     </row>
     <row r="670" spans="3:3">
       <c r="C670" t="s">
-        <v>321</v>
+        <v>497</v>
       </c>
     </row>
     <row r="671" spans="3:3">
       <c r="C671" t="s">
-        <v>315</v>
+        <v>498</v>
       </c>
     </row>
     <row r="672" spans="3:3">
       <c r="C672" t="s">
-        <v>495</v>
+        <v>470</v>
       </c>
     </row>
     <row r="673" spans="3:3">
       <c r="C673" t="s">
-        <v>496</v>
+        <v>335</v>
       </c>
     </row>
     <row r="674" spans="3:3">
       <c r="C674" t="s">
-        <v>497</v>
+        <v>319</v>
       </c>
     </row>
     <row r="675" spans="3:3">
       <c r="C675" t="s">
-        <v>498</v>
+        <v>485</v>
       </c>
     </row>
     <row r="676" spans="3:3">
       <c r="C676" t="s">
-        <v>473</v>
+        <v>320</v>
       </c>
     </row>
     <row r="677" spans="3:3">
       <c r="C677" t="s">
-        <v>335</v>
+        <v>499</v>
       </c>
     </row>
     <row r="678" spans="3:3">
       <c r="C678" t="s">
-        <v>319</v>
+        <v>500</v>
       </c>
     </row>
     <row r="679" spans="3:3">
       <c r="C679" t="s">
-        <v>488</v>
+        <v>501</v>
       </c>
     </row>
     <row r="680" spans="3:3">
       <c r="C680" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="681" spans="3:3">
-      <c r="C681" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="682" spans="3:3">
-      <c r="C682" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="683" spans="3:3">
-      <c r="C683" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="684" spans="3:3">
-      <c r="C684" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="685" spans="3:3">
-      <c r="C685" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="686" spans="3:3">
-      <c r="C686" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="687" spans="3:3">
-      <c r="C687" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="688" spans="3:3">
-      <c r="C688" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="689" spans="3:3">
-      <c r="C689" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="690" spans="3:3">
-      <c r="C690" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="691" spans="3:3">
-      <c r="C691" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="692" spans="3:3">
-      <c r="C692" t="s">
         <v>502</v>
-      </c>
-    </row>
-    <row r="693" spans="3:3">
-      <c r="C693" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="694" spans="3:3">
-      <c r="C694" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="695" spans="3:3">
-      <c r="C695" t="s">
-        <v>505</v>
       </c>
     </row>
   </sheetData>
@@ -7611,7 +7581,7 @@
     </row>
     <row r="2" spans="2:5">
       <c r="B2" s="2" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -7789,10 +7759,10 @@
     </row>
     <row r="29" spans="2:5" ht="37.5">
       <c r="B29" s="1" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="E29" s="3">
         <v>46043</v>
@@ -7800,15 +7770,15 @@
     </row>
     <row r="30" spans="2:5" ht="337.5">
       <c r="B30" s="1" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="56.25">
       <c r="B31" s="1" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="E31" s="3">
         <v>46043</v>
@@ -7816,10 +7786,10 @@
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="1" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="E33" s="3">
         <v>46043</v>
@@ -7827,18 +7797,18 @@
     </row>
     <row r="35" spans="2:5" ht="37.5">
       <c r="B35" s="1" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="56.25">
       <c r="B36" s="1" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="E36" s="3">
         <v>46043</v>
@@ -7846,10 +7816,10 @@
     </row>
     <row r="37" spans="2:5" ht="56.25">
       <c r="B37" s="1" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="E37" s="3">
         <v>46043</v>
@@ -7857,10 +7827,10 @@
     </row>
     <row r="38" spans="2:5" ht="112.5">
       <c r="B38" s="1" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="E38" s="3">
         <v>46043</v>
@@ -8034,10 +8004,10 @@
     </row>
     <row r="23" spans="2:5" ht="93.75">
       <c r="B23" s="1" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="E23" s="3">
         <v>46043</v>
@@ -8045,10 +8015,10 @@
     </row>
     <row r="25" spans="2:5" ht="56.25">
       <c r="B25" s="1" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="E25" s="3">
         <v>46044</v>
@@ -8100,63 +8070,63 @@
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="5" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" s="1" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="C7" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C8" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="56.25">
       <c r="B9" s="1" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="75">
       <c r="B11" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="37.5">
       <c r="B12" s="1" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="75">
       <c r="B13" s="1" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="E13" s="3">
         <v>46043</v>
@@ -8164,10 +8134,10 @@
     </row>
     <row r="14" spans="2:5" ht="56.25">
       <c r="B14" s="1" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="E14" s="3">
         <v>46043</v>

</xml_diff>

<commit_message>
feat: Add EmbeddingLabPage for text embedding functionality
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF847627-0433-495F-82FB-18BA80A4B175}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8579724F-B02E-4489-9852-0796B1B4358A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -29,8 +29,8 @@
     <sheet name="Gemini API reference" sheetId="12" r:id="rId14"/>
     <sheet name="Gemini Code Assist" sheetId="15" r:id="rId15"/>
     <sheet name="Gemini Code Assist 2" sheetId="18" r:id="rId16"/>
-    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId17"/>
-    <sheet name="How to fix" sheetId="16" r:id="rId18"/>
+    <sheet name="How to fix" sheetId="16" r:id="rId17"/>
+    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="577">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="580">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2958,6 +2958,18 @@
   </si>
   <si>
     <t>多様なタスクにスケーリング可能な高速かつ汎用性の高いマルチモーダルモデル「Gemini 2.0 Flash」の安定版が、2025年1月にリリースされました。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>DETAILED_DESIGN.mdをみて、実装できていない機能があれば実装してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>They create these resolutions because everyone else does – we create a superficial meaning out of status games – but they don’t meet the requirements for true change, which goes a lot deeper than convincing yourself you’re going to be more disciplined or productive this year.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>彼らはこうした決意を立てるのは、誰もがそうするからだ——私たちは地位争いから表面的な意味を作り出す——しかしそれらは真の変化の条件を満たしていない。真の変化とは、今年こそもっと規律正しく生産的になると自分に言い聞かせるよりも、はるかに深いところにあるのだ。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3805,10 +3817,13 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="2:8">
+    <row r="6" spans="2:8" ht="37.5">
       <c r="B6">
         <f t="shared" si="0"/>
         <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>577</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -8156,6 +8171,61 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595742A4-FD4B-4501-B5BA-63CBD2F36625}">
+  <dimension ref="C2:D8"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="3" max="3" width="43.25" customWidth="1"/>
+    <col min="4" max="4" width="48.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:4">
+      <c r="C2" s="2" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4">
+      <c r="C4" t="s">
+        <v>311</v>
+      </c>
+      <c r="D4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" ht="37.5">
+      <c r="C6" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" ht="37.5">
+      <c r="C7" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" ht="112.5">
+      <c r="C8" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>579</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{2D572F08-FF13-4D66-AD9B-8810B4A82168}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
   <dimension ref="C3:E9"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
@@ -8244,53 +8314,6 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595742A4-FD4B-4501-B5BA-63CBD2F36625}">
-  <dimension ref="C2:D7"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
-  <cols>
-    <col min="3" max="3" width="35.75" customWidth="1"/>
-    <col min="4" max="4" width="48.375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="3:4">
-      <c r="C2" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="4" spans="3:4">
-      <c r="C4" t="s">
-        <v>311</v>
-      </c>
-      <c r="D4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="6" spans="3:4" ht="37.5">
-      <c r="C6" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="7" spans="3:4" ht="37.5">
-      <c r="C7" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>309</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{2D572F08-FF13-4D66-AD9B-8810B4A82168}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: Update Gemini API reference and content generation details in documentation
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8579724F-B02E-4489-9852-0796B1B4358A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781489A6-94EE-4A98-AF86-FDCE6601CFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="590">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2970,6 +2970,46 @@
   </si>
   <si>
     <t>彼らはこうした決意を立てるのは、誰もがそうするからだ——私たちは地位争いから表面的な意味を作り出す——しかしそれらは真の変化の条件を満たしていない。真の変化とは、今年こそもっと規律正しく生産的になると自分に言い聞かせるよりも、はるかに深いところにあるのだ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Request body structure</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リクエスト本文の構造</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>The request body is a JSON object that is identical for both standard and streaming modes and is built from a few core objects:</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リクエスト本体は、標準モードとストリーミングモードの両方で同一のJSONオブジェクトであり、以下のコアオブジェクトから構成されます：</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Content object: Represents a single turn in a conversation.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>コンテンツオブジェクト：会話における単一のターンを表す。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Part object: A piece of data within a Content turn (like text or an image).</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>部分オブジェクト：コンテンツターン内のデータの一部（テキストや画像など）。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>inline_data (Blob): A container for raw media bytes and their MIME type.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>inline_data (Blob): 生メディアバイトとそのMIMEタイプを格納するコンテナ。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3372,7 +3412,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3555,7 +3595,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -3768,7 +3808,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3941,7 +3981,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -7580,7 +7620,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
-  <dimension ref="B1:E38"/>
+  <dimension ref="B1:E45"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="42.5" customWidth="1"/>
@@ -7591,7 +7631,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -7849,6 +7889,52 @@
       </c>
       <c r="E38" s="3">
         <v>46043</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5">
+      <c r="B40" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" ht="56.25">
+      <c r="B42" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>583</v>
+      </c>
+      <c r="E42" s="3">
+        <v>46045</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" ht="37.5">
+      <c r="B43" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" ht="37.5">
+      <c r="B44" s="1" t="s">
+        <v>586</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" ht="37.5">
+      <c r="B45" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="E45" s="3">
+        <v>46045</v>
       </c>
     </row>
   </sheetData>
@@ -7877,7 +7963,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8065,7 +8151,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8104,7 +8190,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="56.25">
+    <row r="9" spans="2:5" ht="37.5">
       <c r="B9" s="1" t="s">
         <v>540</v>
       </c>
@@ -8172,6 +8258,9 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595742A4-FD4B-4501-B5BA-63CBD2F36625}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
   <dimension ref="C2:D8"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
@@ -8846,7 +8935,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46044</v>
+        <v>46045</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
feat: Update tasks table schema and add necessary columns for stock feature
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{781489A6-94EE-4A98-AF86-FDCE6601CFA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF83C92-38EE-4ED8-9038-D80E0D07C6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="590">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="592">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -3010,6 +3010,14 @@
   </si>
   <si>
     <t>inline_data (Blob): 生メディアバイトとそのMIMEタイプを格納するコンテナ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>You can get code completions as you write your code, generate full functions or code blocks from comments, generate unit tests, and get help with debugging, understanding, and documenting your code.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>コードを記述しながらコード補完を利用でき、コメントから完全な関数やコードブロックを生成し、ユニットテストを生成し、デバッグやコードの理解、ドキュメント作成の支援を受けられます。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -7620,6 +7628,9 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79E1C8F-6C57-4A1D-AF37-910DD10A2AE7}">
+  <sheetPr>
+    <tabColor theme="9"/>
+  </sheetPr>
   <dimension ref="B1:E45"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
@@ -7952,7 +7963,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E25"/>
+  <dimension ref="B1:E26"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="73.125" customWidth="1"/>
@@ -8123,6 +8134,17 @@
       </c>
       <c r="E25" s="3">
         <v>46044</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" ht="56.25">
+      <c r="B26" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="E26" s="3">
+        <v>46045</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: add rate limit sleep
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CF83C92-38EE-4ED8-9038-D80E0D07C6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5A4802B-EDAA-4274-8153-F1BDDE47E4B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -33,6 +33,7 @@
     <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1162" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="598">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -3018,6 +3019,51 @@
   </si>
   <si>
     <t>コードを記述しながらコード補完を利用でき、コメントから完全な関数やコードブロックを生成し、ユニットテストを生成し、デバッグやコードの理解、ドキュメント作成の支援を受けられます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>このサイトに国民民主党が衆議院選挙2026で勝利するための機能を追加してください。
+また、使用方法が分かるようにユーザーマニュアルも追加してください。AIとsupabaseを駆使する機能としてください。</t>
+    <rPh sb="45" eb="47">
+      <t>シヨウ</t>
+    </rPh>
+    <rPh sb="47" eb="49">
+      <t>ホウホウ</t>
+    </rPh>
+    <rPh sb="50" eb="51">
+      <t>ワ</t>
+    </rPh>
+    <rPh sb="66" eb="68">
+      <t>ツイカ</t>
+    </rPh>
+    <rPh sb="87" eb="89">
+      <t>クシ</t>
+    </rPh>
+    <rPh sb="91" eb="93">
+      <t>キノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>git add .
+git commit -m "fix: add rate limit sleep"
+git push</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assist provides contextualized responses to your prompts, including source citations regarding which documentation and code samples Gemini Code Assist used to generate its responses.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini Code Assistは、プロンプトに対する文脈に応じた応答を提供します。これには、応答生成に使用したドキュメントやコードサンプルに関する出典情報も含まれます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Quotas specify the amount of a countable, shared resource that you can use.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>クォータは、使用可能な共有リソースの量を指定します。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3420,7 +3466,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3603,7 +3649,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -3816,7 +3862,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3876,10 +3922,13 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:8">
+    <row r="7" spans="2:8" ht="93.75">
       <c r="B7">
         <f t="shared" si="0"/>
         <v>5</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>592</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -3989,7 +4038,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -7642,7 +7691,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -7963,7 +8012,10 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
-  <dimension ref="B1:E26"/>
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="B1:E27"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="73.125" customWidth="1"/>
@@ -7974,7 +8026,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8145,6 +8197,17 @@
       </c>
       <c r="E26" s="3">
         <v>46045</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" ht="56.25">
+      <c r="B27" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="E27" s="3">
+        <v>46050</v>
       </c>
     </row>
   </sheetData>
@@ -8162,7 +8225,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D01CB6-001D-4D20-8CBB-FE510A056DBA}">
-  <dimension ref="B1:E14"/>
+  <sheetPr>
+    <tabColor rgb="FF00B0F0"/>
+  </sheetPr>
+  <dimension ref="B1:E16"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="45.125" customWidth="1"/>
@@ -8173,106 +8239,120 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
     </row>
     <row r="2" spans="2:5">
-      <c r="B2" s="5" t="s">
-        <v>51</v>
-      </c>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" s="5" t="s">
-        <v>126</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="2:5">
       <c r="B5" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="5" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="7" spans="2:5">
-      <c r="B7" s="1" t="s">
+    <row r="8" spans="2:5">
+      <c r="B8" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="8" spans="2:5">
-      <c r="B8" t="s">
+    <row r="9" spans="2:5">
+      <c r="B9" t="s">
         <v>538</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>539</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" ht="37.5">
-      <c r="B9" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>541</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="37.5">
+      <c r="B11" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C11" s="1" t="s">
         <v>543</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="75">
-      <c r="B11" s="1" t="s">
+    <row r="12" spans="2:5" ht="75">
+      <c r="B12" s="1" t="s">
         <v>544</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="37.5">
-      <c r="B12" s="1" t="s">
+    <row r="13" spans="2:5" ht="37.5">
+      <c r="B13" s="1" t="s">
         <v>546</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C13" s="1" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="13" spans="2:5" ht="75">
-      <c r="B13" s="1" t="s">
+    <row r="14" spans="2:5" ht="75">
+      <c r="B14" s="1" t="s">
         <v>548</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C14" s="1" t="s">
         <v>549</v>
-      </c>
-      <c r="E13" s="3">
-        <v>46043</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" ht="56.25">
-      <c r="B14" s="1" t="s">
-        <v>550</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>551</v>
       </c>
       <c r="E14" s="3">
         <v>46043</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="56.25">
+      <c r="B15" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="E15" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="37.5">
+      <c r="B16" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>597</v>
+      </c>
+      <c r="E16" s="3">
+        <v>46050</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://developers.google.com/" xr:uid="{AB4DF198-4467-43BD-92E5-7F9CEA77AE2D}"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://developers.google.com/products" xr:uid="{E0788B1D-CD47-4B9D-A222-F399F4097EB5}"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{59048891-D360-4985-8E21-C2F762568942}"/>
-    <hyperlink ref="B5" r:id="rId4" display="https://developers.google.com/gemini-code-assist/resources/faqs" xr:uid="{B8E91675-F28D-4503-9C6B-4A96AC1B988B}"/>
+    <hyperlink ref="B3" r:id="rId1" display="https://developers.google.com/" xr:uid="{AB4DF198-4467-43BD-92E5-7F9CEA77AE2D}"/>
+    <hyperlink ref="B4" r:id="rId2" display="https://developers.google.com/products" xr:uid="{E0788B1D-CD47-4B9D-A222-F399F4097EB5}"/>
+    <hyperlink ref="B5" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{59048891-D360-4985-8E21-C2F762568942}"/>
+    <hyperlink ref="B6" r:id="rId4" display="https://developers.google.com/gemini-code-assist/resources/faqs" xr:uid="{B8E91675-F28D-4503-9C6B-4A96AC1B988B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8434,7 +8514,7 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="B3:D19"/>
+  <dimension ref="B3:D20"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
@@ -8456,7 +8536,7 @@
     </row>
     <row r="5" spans="2:4">
       <c r="B5">
-        <f t="shared" ref="B5:B19" si="0">B4+1</f>
+        <f t="shared" ref="B5:B20" si="0">B4+1</f>
         <v>2</v>
       </c>
       <c r="C5" t="s">
@@ -8587,6 +8667,15 @@
       </c>
       <c r="C19" s="1" t="s">
         <v>313</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" ht="56.25">
+      <c r="B20">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>593</v>
       </c>
     </row>
   </sheetData>
@@ -8957,7 +9046,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46045</v>
+        <v>46050</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
fix: correct formatting issues in ElectionStrategyPage
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED11574-E2B8-4DC9-86D3-99C0E18DD2D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{85FD3B1B-62B1-4A6F-B9EE-6AE967B33282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="9" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -3562,7 +3562,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3745,7 +3745,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -3958,7 +3958,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -4134,7 +4134,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -7737,7 +7737,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -7801,7 +7801,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="75">
+    <row r="12" spans="2:5" ht="56.25">
       <c r="B12" s="1" t="s">
         <v>64</v>
       </c>
@@ -7835,7 +7835,7 @@
       </c>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="2:5" ht="112.5">
+    <row r="19" spans="2:5" ht="93.75">
       <c r="B19" s="1" t="s">
         <v>72</v>
       </c>
@@ -7844,7 +7844,7 @@
       </c>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="2:5" ht="75">
+    <row r="20" spans="2:5" ht="56.25">
       <c r="B20" s="1" t="s">
         <v>74</v>
       </c>
@@ -7929,12 +7929,12 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="30" spans="2:5" ht="337.5">
+    <row r="30" spans="2:5" ht="318.75">
       <c r="B30" s="1" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="31" spans="2:5" ht="56.25">
+    <row r="31" spans="2:5" ht="37.5">
       <c r="B31" s="1" t="s">
         <v>553</v>
       </c>
@@ -7964,7 +7964,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="36" spans="2:5" ht="56.25">
+    <row r="36" spans="2:5" ht="37.5">
       <c r="B36" s="1" t="s">
         <v>559</v>
       </c>
@@ -7986,7 +7986,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="112.5">
+    <row r="38" spans="2:5" ht="93.75">
       <c r="B38" s="1" t="s">
         <v>563</v>
       </c>
@@ -8159,7 +8159,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8372,7 +8372,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -9187,7 +9187,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46050</v>
+        <v>46052</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
feat: Enhance AiAssistantMenu with optional SupabaseClient parameter
- Updated AiAssistantMenu to accept an optional SupabaseClient parameter for better flexibility in testing and usage.
- Modified the _handleAiAction method to utilize the provided SupabaseClient if available.
- Added comprehensive tests for AiAssistantMenu, covering various scenarios including successful function invocation and error handling.
- Removed unused AIModelService mock and related code from emergency_meeting_page_test.
- Created new mock files for AiAssistantMenu tests to facilitate isolated testing.
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{85FD3B1B-62B1-4A6F-B9EE-6AE967B33282}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F74B50-1C10-4E75-A9B7-6AF9E7D1A0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,6 @@
     <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId18"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -54,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="623">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -2152,15 +2151,6 @@
     <t xml:space="preserve">      "maxTemperature": 2</t>
   </si>
   <si>
-    <t xml:space="preserve">      "name": "models/gemini-2.0-flash-lite-001",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "displayName": "Gemini 2.0 Flash-Lite 001",</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      "description": "Stable version of Gemini 2.0 Flash-Lite",</t>
-  </si>
-  <si>
     <t xml:space="preserve">      "name": "models/gemini-2.0-flash-lite",</t>
   </si>
   <si>
@@ -3160,6 +3150,46 @@
   </si>
   <si>
     <t>高レベルでは、レスポンスボディには候補オブジェクトが含まれており、これは候補オブジェクトのリストである。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>models/gemini-2.0-flash-lite-001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini 2.0 Flash-Lite 001</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Stable version of Gemini 2.0 Flash-Lite</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Gemini 2.0 Flash-Liteの安定版</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>The Candidate object contains a Content object that has the generated response returned from the model.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Candidateオブジェクトは、モデルから返された生成済みレスポンスを含むContentオブジェクトを保持します。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Request examples</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リクエスト例</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>The following examples show how these components come together for different types of requests.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>以下の例は、これらのコンポーネントが異なる種類のリクエストに対してどのように連携するかを示しています。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3562,7 +3592,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3745,7 +3775,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -3958,7 +3988,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -4013,7 +4043,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>572</v>
+        <v>569</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -4024,7 +4054,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -4116,7 +4146,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F96D129-34E8-4B10-A261-7AEE00EA03AD}">
-  <dimension ref="B1:Q663"/>
+  <dimension ref="B1:Q645"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
@@ -4134,62 +4164,62 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="2" spans="2:17">
       <c r="E2" t="s">
+        <v>495</v>
+      </c>
+      <c r="F2" t="s">
+        <v>497</v>
+      </c>
+      <c r="G2" t="s">
         <v>498</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>500</v>
       </c>
-      <c r="G2" t="s">
-        <v>501</v>
-      </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
+        <v>502</v>
+      </c>
+      <c r="K2" t="s">
         <v>503</v>
       </c>
-      <c r="J2" t="s">
-        <v>505</v>
-      </c>
-      <c r="K2" t="s">
-        <v>506</v>
-      </c>
       <c r="L2" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="M2" t="s">
+        <v>512</v>
+      </c>
+      <c r="N2" t="s">
+        <v>513</v>
+      </c>
+      <c r="O2" t="s">
+        <v>514</v>
+      </c>
+      <c r="P2" t="s">
         <v>515</v>
       </c>
-      <c r="N2" t="s">
+      <c r="Q2" t="s">
         <v>516</v>
-      </c>
-      <c r="O2" t="s">
-        <v>517</v>
-      </c>
-      <c r="P2" t="s">
-        <v>518</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>519</v>
       </c>
     </row>
     <row r="3" spans="2:17" ht="37.5">
       <c r="E3" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="H3" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="I3" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="J3">
         <v>1024</v>
@@ -4198,24 +4228,24 @@
         <v>1</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
     </row>
     <row r="4" spans="2:17" ht="75">
       <c r="E4" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" t="s">
+        <v>507</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>510</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>511</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>513</v>
       </c>
       <c r="J4">
         <v>1048576</v>
@@ -4224,7 +4254,7 @@
         <v>65536</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="M4">
         <v>1</v>
@@ -4244,19 +4274,19 @@
     </row>
     <row r="5" spans="2:17" ht="75">
       <c r="E5" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="F5">
         <v>2.5</v>
       </c>
       <c r="G5" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H5" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="I5" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="J5">
         <v>1048576</v>
@@ -4265,7 +4295,7 @@
         <v>65536</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="M5">
         <v>1</v>
@@ -4285,19 +4315,19 @@
     </row>
     <row r="6" spans="2:17" ht="56.25">
       <c r="E6" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="H6" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="I6" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="J6">
         <v>1048576</v>
@@ -4306,7 +4336,7 @@
         <v>8192</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="M6">
         <v>1</v>
@@ -4326,19 +4356,19 @@
         <v>46043</v>
       </c>
       <c r="E7" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="H7" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="I7" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="J7">
         <v>1048576</v>
@@ -4347,7 +4377,7 @@
         <v>8192</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="M7">
         <v>1</v>
@@ -4367,19 +4397,19 @@
         <v>46044</v>
       </c>
       <c r="E8" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>569</v>
+        <v>566</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>571</v>
+        <v>568</v>
       </c>
       <c r="J8">
         <v>1048576</v>
@@ -4388,7 +4418,7 @@
         <v>8192</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="M8">
         <v>1</v>
@@ -4408,19 +4438,19 @@
         <v>46050</v>
       </c>
       <c r="E9" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="F9">
         <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="J9">
         <v>1048576</v>
@@ -4429,7 +4459,7 @@
         <v>8192</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="M9">
         <v>1</v>
@@ -4444,11 +4474,44 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:17">
+    <row r="10" spans="2:17" ht="75">
       <c r="B10" s="3"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="L10" s="1"/>
+      <c r="E10" t="s">
+        <v>613</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>614</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>615</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>616</v>
+      </c>
+      <c r="J10">
+        <v>1048576</v>
+      </c>
+      <c r="K10">
+        <v>8192</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+      <c r="N10">
+        <v>0.95</v>
+      </c>
+      <c r="O10">
+        <v>40</v>
+      </c>
+      <c r="P10">
+        <v>2</v>
+      </c>
     </row>
     <row r="11" spans="2:17">
       <c r="C11" t="s">
@@ -4552,17 +4615,17 @@
     </row>
     <row r="31" spans="3:3">
       <c r="C31" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
     </row>
     <row r="32" spans="3:3">
       <c r="C32" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="33" spans="3:3">
       <c r="C33" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="34" spans="3:3">
@@ -4637,12 +4700,12 @@
     </row>
     <row r="48" spans="3:3">
       <c r="C48" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="49" spans="3:3">
       <c r="C49" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="50" spans="3:3">
@@ -4652,7 +4715,7 @@
     </row>
     <row r="51" spans="3:3">
       <c r="C51" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="52" spans="3:3">
@@ -4727,12 +4790,12 @@
     </row>
     <row r="66" spans="3:3">
       <c r="C66" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="67" spans="3:3">
       <c r="C67" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
     </row>
     <row r="68" spans="3:3">
@@ -4742,7 +4805,7 @@
     </row>
     <row r="69" spans="3:3">
       <c r="C69" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
     </row>
     <row r="70" spans="3:3">
@@ -4752,7 +4815,7 @@
     </row>
     <row r="71" spans="3:3">
       <c r="C71" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
     </row>
     <row r="72" spans="3:3">
@@ -4797,27 +4860,27 @@
     </row>
     <row r="80" spans="3:3">
       <c r="C80" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="81" spans="3:3">
       <c r="C81" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
     </row>
     <row r="82" spans="3:3">
       <c r="C82" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="83" spans="3:3">
       <c r="C83" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="84" spans="3:3">
       <c r="C84" t="s">
-        <v>350</v>
+        <v>315</v>
       </c>
     </row>
     <row r="85" spans="3:3">
@@ -4837,22 +4900,22 @@
     </row>
     <row r="88" spans="3:3">
       <c r="C88" t="s">
-        <v>322</v>
+        <v>354</v>
       </c>
     </row>
     <row r="89" spans="3:3">
       <c r="C89" t="s">
-        <v>323</v>
+        <v>355</v>
       </c>
     </row>
     <row r="90" spans="3:3">
       <c r="C90" t="s">
-        <v>319</v>
+        <v>356</v>
       </c>
     </row>
     <row r="91" spans="3:3">
       <c r="C91" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="92" spans="3:3">
@@ -4862,642 +4925,642 @@
     </row>
     <row r="93" spans="3:3">
       <c r="C93" t="s">
-        <v>326</v>
+        <v>357</v>
       </c>
     </row>
     <row r="94" spans="3:3">
       <c r="C94" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="95" spans="3:3">
       <c r="C95" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="96" spans="3:3">
       <c r="C96" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="97" spans="3:3">
       <c r="C97" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="98" spans="3:3">
       <c r="C98" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
     </row>
     <row r="99" spans="3:3">
       <c r="C99" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
     </row>
     <row r="100" spans="3:3">
       <c r="C100" t="s">
-        <v>333</v>
+        <v>315</v>
       </c>
     </row>
     <row r="101" spans="3:3">
       <c r="C101" t="s">
-        <v>321</v>
+        <v>358</v>
       </c>
     </row>
     <row r="102" spans="3:3">
       <c r="C102" t="s">
-        <v>315</v>
+        <v>359</v>
       </c>
     </row>
     <row r="103" spans="3:3">
       <c r="C103" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
     </row>
     <row r="104" spans="3:3">
       <c r="C104" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
     </row>
     <row r="105" spans="3:3">
       <c r="C105" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="106" spans="3:3">
       <c r="C106" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="107" spans="3:3">
       <c r="C107" t="s">
-        <v>358</v>
+        <v>319</v>
       </c>
     </row>
     <row r="108" spans="3:3">
       <c r="C108" t="s">
-        <v>359</v>
+        <v>325</v>
       </c>
     </row>
     <row r="109" spans="3:3">
       <c r="C109" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="110" spans="3:3">
       <c r="C110" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="111" spans="3:3">
       <c r="C111" t="s">
-        <v>360</v>
+        <v>328</v>
       </c>
     </row>
     <row r="112" spans="3:3">
       <c r="C112" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="113" spans="3:3">
       <c r="C113" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="114" spans="3:3">
       <c r="C114" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="115" spans="3:3">
       <c r="C115" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
     </row>
     <row r="116" spans="3:3">
       <c r="C116" t="s">
-        <v>337</v>
+        <v>321</v>
       </c>
     </row>
     <row r="117" spans="3:3">
       <c r="C117" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="118" spans="3:3">
       <c r="C118" t="s">
-        <v>315</v>
+        <v>362</v>
       </c>
     </row>
     <row r="119" spans="3:3">
       <c r="C119" t="s">
-        <v>361</v>
+        <v>316</v>
       </c>
     </row>
     <row r="120" spans="3:3">
       <c r="C120" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="121" spans="3:3">
       <c r="C121" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="122" spans="3:3">
       <c r="C122" t="s">
-        <v>364</v>
+        <v>335</v>
       </c>
     </row>
     <row r="123" spans="3:3">
       <c r="C123" t="s">
-        <v>358</v>
+        <v>319</v>
       </c>
     </row>
     <row r="124" spans="3:3">
       <c r="C124" t="s">
-        <v>359</v>
+        <v>324</v>
       </c>
     </row>
     <row r="125" spans="3:3">
       <c r="C125" t="s">
-        <v>319</v>
+        <v>365</v>
       </c>
     </row>
     <row r="126" spans="3:3">
       <c r="C126" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="127" spans="3:3">
       <c r="C127" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="128" spans="3:3">
       <c r="C128" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
     </row>
     <row r="129" spans="3:3">
       <c r="C129" t="s">
-        <v>328</v>
+        <v>366</v>
       </c>
     </row>
     <row r="130" spans="3:3">
       <c r="C130" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
     </row>
     <row r="131" spans="3:3">
       <c r="C131" t="s">
-        <v>330</v>
+        <v>315</v>
       </c>
     </row>
     <row r="132" spans="3:3">
       <c r="C132" t="s">
-        <v>331</v>
+        <v>367</v>
       </c>
     </row>
     <row r="133" spans="3:3">
       <c r="C133" t="s">
-        <v>337</v>
+        <v>316</v>
       </c>
     </row>
     <row r="134" spans="3:3">
       <c r="C134" t="s">
-        <v>321</v>
+        <v>368</v>
       </c>
     </row>
     <row r="135" spans="3:3">
       <c r="C135" t="s">
-        <v>315</v>
+        <v>364</v>
       </c>
     </row>
     <row r="136" spans="3:3">
       <c r="C136" t="s">
-        <v>365</v>
+        <v>335</v>
       </c>
     </row>
     <row r="137" spans="3:3">
       <c r="C137" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="138" spans="3:3">
       <c r="C138" t="s">
-        <v>366</v>
+        <v>324</v>
       </c>
     </row>
     <row r="139" spans="3:3">
       <c r="C139" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="140" spans="3:3">
       <c r="C140" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="141" spans="3:3">
       <c r="C141" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="142" spans="3:3">
       <c r="C142" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="143" spans="3:3">
       <c r="C143" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="144" spans="3:3">
       <c r="C144" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="145" spans="3:3">
       <c r="C145" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="146" spans="3:3">
       <c r="C146" t="s">
-        <v>330</v>
+        <v>369</v>
       </c>
     </row>
     <row r="147" spans="3:3">
       <c r="C147" t="s">
-        <v>369</v>
+        <v>316</v>
       </c>
     </row>
     <row r="148" spans="3:3">
       <c r="C148" t="s">
-        <v>321</v>
+        <v>370</v>
       </c>
     </row>
     <row r="149" spans="3:3">
       <c r="C149" t="s">
-        <v>315</v>
+        <v>364</v>
       </c>
     </row>
     <row r="150" spans="3:3">
       <c r="C150" t="s">
-        <v>370</v>
+        <v>335</v>
       </c>
     </row>
     <row r="151" spans="3:3">
       <c r="C151" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="152" spans="3:3">
       <c r="C152" t="s">
-        <v>371</v>
+        <v>324</v>
       </c>
     </row>
     <row r="153" spans="3:3">
       <c r="C153" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="154" spans="3:3">
       <c r="C154" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="155" spans="3:3">
       <c r="C155" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="156" spans="3:3">
       <c r="C156" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="157" spans="3:3">
       <c r="C157" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="158" spans="3:3">
       <c r="C158" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="159" spans="3:3">
       <c r="C159" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="160" spans="3:3">
       <c r="C160" t="s">
-        <v>330</v>
+        <v>371</v>
       </c>
     </row>
     <row r="161" spans="3:3">
       <c r="C161" t="s">
-        <v>369</v>
+        <v>316</v>
       </c>
     </row>
     <row r="162" spans="3:3">
       <c r="C162" t="s">
-        <v>321</v>
+        <v>372</v>
       </c>
     </row>
     <row r="163" spans="3:3">
       <c r="C163" t="s">
-        <v>315</v>
+        <v>373</v>
       </c>
     </row>
     <row r="164" spans="3:3">
       <c r="C164" t="s">
-        <v>372</v>
+        <v>335</v>
       </c>
     </row>
     <row r="165" spans="3:3">
       <c r="C165" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="166" spans="3:3">
       <c r="C166" t="s">
-        <v>373</v>
+        <v>324</v>
       </c>
     </row>
     <row r="167" spans="3:3">
       <c r="C167" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="168" spans="3:3">
       <c r="C168" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="169" spans="3:3">
       <c r="C169" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="170" spans="3:3">
       <c r="C170" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="171" spans="3:3">
       <c r="C171" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="172" spans="3:3">
       <c r="C172" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="173" spans="3:3">
       <c r="C173" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="174" spans="3:3">
       <c r="C174" t="s">
-        <v>330</v>
+        <v>374</v>
       </c>
     </row>
     <row r="175" spans="3:3">
       <c r="C175" t="s">
-        <v>369</v>
+        <v>316</v>
       </c>
     </row>
     <row r="176" spans="3:3">
       <c r="C176" t="s">
-        <v>321</v>
+        <v>375</v>
       </c>
     </row>
     <row r="177" spans="3:3">
       <c r="C177" t="s">
-        <v>315</v>
+        <v>355</v>
       </c>
     </row>
     <row r="178" spans="3:3">
       <c r="C178" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="179" spans="3:3">
       <c r="C179" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="180" spans="3:3">
       <c r="C180" t="s">
-        <v>375</v>
+        <v>324</v>
       </c>
     </row>
     <row r="181" spans="3:3">
       <c r="C181" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
     </row>
     <row r="182" spans="3:3">
       <c r="C182" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
     </row>
     <row r="183" spans="3:3">
       <c r="C183" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="184" spans="3:3">
       <c r="C184" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="185" spans="3:3">
       <c r="C185" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="186" spans="3:3">
       <c r="C186" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="187" spans="3:3">
       <c r="C187" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="188" spans="3:3">
       <c r="C188" t="s">
-        <v>330</v>
+        <v>377</v>
       </c>
     </row>
     <row r="189" spans="3:3">
       <c r="C189" t="s">
-        <v>369</v>
+        <v>316</v>
       </c>
     </row>
     <row r="190" spans="3:3">
       <c r="C190" t="s">
-        <v>321</v>
+        <v>378</v>
       </c>
     </row>
     <row r="191" spans="3:3">
       <c r="C191" t="s">
-        <v>315</v>
+        <v>355</v>
       </c>
     </row>
     <row r="192" spans="3:3">
       <c r="C192" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="193" spans="3:3">
       <c r="C193" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="194" spans="3:3">
       <c r="C194" t="s">
-        <v>378</v>
+        <v>324</v>
       </c>
     </row>
     <row r="195" spans="3:3">
       <c r="C195" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
     </row>
     <row r="196" spans="3:3">
       <c r="C196" t="s">
-        <v>379</v>
+        <v>328</v>
       </c>
     </row>
     <row r="197" spans="3:3">
       <c r="C197" t="s">
-        <v>319</v>
+        <v>329</v>
       </c>
     </row>
     <row r="198" spans="3:3">
       <c r="C198" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
     </row>
     <row r="199" spans="3:3">
       <c r="C199" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
     </row>
     <row r="200" spans="3:3">
       <c r="C200" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
     </row>
     <row r="201" spans="3:3">
       <c r="C201" t="s">
-        <v>329</v>
+        <v>315</v>
       </c>
     </row>
     <row r="202" spans="3:3">
       <c r="C202" t="s">
-        <v>330</v>
+        <v>379</v>
       </c>
     </row>
     <row r="203" spans="3:3">
       <c r="C203" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
     </row>
     <row r="204" spans="3:3">
       <c r="C204" t="s">
-        <v>321</v>
+        <v>381</v>
       </c>
     </row>
     <row r="205" spans="3:3">
       <c r="C205" t="s">
-        <v>315</v>
+        <v>382</v>
       </c>
     </row>
     <row r="206" spans="3:3">
       <c r="C206" t="s">
-        <v>380</v>
+        <v>322</v>
       </c>
     </row>
     <row r="207" spans="3:3">
       <c r="C207" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
     </row>
     <row r="208" spans="3:3">
       <c r="C208" t="s">
-        <v>381</v>
+        <v>319</v>
       </c>
     </row>
     <row r="209" spans="3:3">
       <c r="C209" t="s">
-        <v>358</v>
+        <v>324</v>
       </c>
     </row>
     <row r="210" spans="3:3">
       <c r="C210" t="s">
-        <v>379</v>
+        <v>325</v>
       </c>
     </row>
     <row r="211" spans="3:3">
       <c r="C211" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="212" spans="3:3">
       <c r="C212" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
     </row>
     <row r="213" spans="3:3">
       <c r="C213" t="s">
-        <v>368</v>
+        <v>328</v>
       </c>
     </row>
     <row r="214" spans="3:3">
       <c r="C214" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="215" spans="3:3">
       <c r="C215" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="216" spans="3:3">
       <c r="C216" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="217" spans="3:3">
       <c r="C217" t="s">
-        <v>369</v>
+        <v>332</v>
       </c>
     </row>
     <row r="218" spans="3:3">
       <c r="C218" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="219" spans="3:3">
       <c r="C219" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="220" spans="3:3">
       <c r="C220" t="s">
-        <v>382</v>
+        <v>315</v>
       </c>
     </row>
     <row r="221" spans="3:3">
@@ -5517,82 +5580,82 @@
     </row>
     <row r="224" spans="3:3">
       <c r="C224" t="s">
-        <v>322</v>
+        <v>386</v>
       </c>
     </row>
     <row r="225" spans="3:3">
       <c r="C225" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="226" spans="3:3">
       <c r="C226" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="227" spans="3:3">
       <c r="C227" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="228" spans="3:3">
       <c r="C228" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="229" spans="3:3">
       <c r="C229" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="230" spans="3:3">
       <c r="C230" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="231" spans="3:3">
       <c r="C231" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="232" spans="3:3">
       <c r="C232" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="233" spans="3:3">
       <c r="C233" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="234" spans="3:3">
       <c r="C234" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="235" spans="3:3">
       <c r="C235" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="236" spans="3:3">
       <c r="C236" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="237" spans="3:3">
       <c r="C237" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="238" spans="3:3">
       <c r="C238" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="239" spans="3:3">
       <c r="C239" t="s">
-        <v>386</v>
+        <v>315</v>
       </c>
     </row>
     <row r="240" spans="3:3">
@@ -5612,82 +5675,82 @@
     </row>
     <row r="243" spans="3:3">
       <c r="C243" t="s">
-        <v>322</v>
+        <v>390</v>
       </c>
     </row>
     <row r="244" spans="3:3">
       <c r="C244" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="245" spans="3:3">
       <c r="C245" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="246" spans="3:3">
       <c r="C246" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="247" spans="3:3">
       <c r="C247" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="248" spans="3:3">
       <c r="C248" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="249" spans="3:3">
       <c r="C249" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="250" spans="3:3">
       <c r="C250" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="251" spans="3:3">
       <c r="C251" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="252" spans="3:3">
       <c r="C252" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="253" spans="3:3">
       <c r="C253" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="254" spans="3:3">
       <c r="C254" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="255" spans="3:3">
       <c r="C255" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="256" spans="3:3">
       <c r="C256" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="257" spans="3:3">
       <c r="C257" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="258" spans="3:3">
       <c r="C258" t="s">
-        <v>390</v>
+        <v>315</v>
       </c>
     </row>
     <row r="259" spans="3:3">
@@ -5697,137 +5760,137 @@
     </row>
     <row r="260" spans="3:3">
       <c r="C260" t="s">
-        <v>392</v>
+        <v>316</v>
       </c>
     </row>
     <row r="261" spans="3:3">
       <c r="C261" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="262" spans="3:3">
       <c r="C262" t="s">
-        <v>322</v>
+        <v>393</v>
       </c>
     </row>
     <row r="263" spans="3:3">
       <c r="C263" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="264" spans="3:3">
       <c r="C264" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="265" spans="3:3">
       <c r="C265" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="266" spans="3:3">
       <c r="C266" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="267" spans="3:3">
       <c r="C267" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="268" spans="3:3">
       <c r="C268" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="269" spans="3:3">
       <c r="C269" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="270" spans="3:3">
       <c r="C270" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="271" spans="3:3">
       <c r="C271" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="272" spans="3:3">
       <c r="C272" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="273" spans="3:3">
       <c r="C273" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="274" spans="3:3">
       <c r="C274" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="275" spans="3:3">
       <c r="C275" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="276" spans="3:3">
       <c r="C276" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="277" spans="3:3">
       <c r="C277" t="s">
-        <v>394</v>
+        <v>315</v>
       </c>
     </row>
     <row r="278" spans="3:3">
       <c r="C278" t="s">
-        <v>316</v>
+        <v>394</v>
       </c>
     </row>
     <row r="279" spans="3:3">
       <c r="C279" t="s">
-        <v>395</v>
+        <v>334</v>
       </c>
     </row>
     <row r="280" spans="3:3">
       <c r="C280" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="281" spans="3:3">
       <c r="C281" t="s">
-        <v>322</v>
+        <v>396</v>
       </c>
     </row>
     <row r="282" spans="3:3">
       <c r="C282" t="s">
-        <v>323</v>
+        <v>364</v>
       </c>
     </row>
     <row r="283" spans="3:3">
       <c r="C283" t="s">
-        <v>319</v>
+        <v>397</v>
       </c>
     </row>
     <row r="284" spans="3:3">
       <c r="C284" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="285" spans="3:3">
       <c r="C285" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="286" spans="3:3">
       <c r="C286" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="287" spans="3:3">
@@ -5857,67 +5920,67 @@
     </row>
     <row r="292" spans="3:3">
       <c r="C292" t="s">
-        <v>332</v>
+        <v>398</v>
       </c>
     </row>
     <row r="293" spans="3:3">
       <c r="C293" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="294" spans="3:3">
       <c r="C294" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="295" spans="3:3">
       <c r="C295" t="s">
-        <v>315</v>
+        <v>399</v>
       </c>
     </row>
     <row r="296" spans="3:3">
       <c r="C296" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
     </row>
     <row r="297" spans="3:3">
       <c r="C297" t="s">
-        <v>334</v>
+        <v>401</v>
       </c>
     </row>
     <row r="298" spans="3:3">
       <c r="C298" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
     </row>
     <row r="299" spans="3:3">
       <c r="C299" t="s">
-        <v>399</v>
+        <v>322</v>
       </c>
     </row>
     <row r="300" spans="3:3">
       <c r="C300" t="s">
-        <v>367</v>
+        <v>323</v>
       </c>
     </row>
     <row r="301" spans="3:3">
       <c r="C301" t="s">
-        <v>400</v>
+        <v>319</v>
       </c>
     </row>
     <row r="302" spans="3:3">
       <c r="C302" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="303" spans="3:3">
       <c r="C303" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
     </row>
     <row r="304" spans="3:3">
       <c r="C304" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="305" spans="3:3">
@@ -5947,22 +6010,22 @@
     </row>
     <row r="310" spans="3:3">
       <c r="C310" t="s">
-        <v>401</v>
+        <v>332</v>
       </c>
     </row>
     <row r="311" spans="3:3">
       <c r="C311" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="312" spans="3:3">
       <c r="C312" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="313" spans="3:3">
       <c r="C313" t="s">
-        <v>402</v>
+        <v>315</v>
       </c>
     </row>
     <row r="314" spans="3:3">
@@ -5982,177 +6045,177 @@
     </row>
     <row r="317" spans="3:3">
       <c r="C317" t="s">
-        <v>322</v>
+        <v>406</v>
       </c>
     </row>
     <row r="318" spans="3:3">
       <c r="C318" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="319" spans="3:3">
       <c r="C319" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="320" spans="3:3">
       <c r="C320" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="321" spans="3:3">
       <c r="C321" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="322" spans="3:3">
       <c r="C322" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="323" spans="3:3">
       <c r="C323" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="324" spans="3:3">
       <c r="C324" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="325" spans="3:3">
       <c r="C325" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="326" spans="3:3">
       <c r="C326" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="327" spans="3:3">
       <c r="C327" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="328" spans="3:3">
       <c r="C328" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="329" spans="3:3">
       <c r="C329" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="330" spans="3:3">
       <c r="C330" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="331" spans="3:3">
       <c r="C331" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="332" spans="3:3">
       <c r="C332" t="s">
-        <v>406</v>
+        <v>315</v>
       </c>
     </row>
     <row r="333" spans="3:3">
       <c r="C333" t="s">
-        <v>407</v>
+        <v>597</v>
       </c>
     </row>
     <row r="334" spans="3:3">
       <c r="C334" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="335" spans="3:3">
       <c r="C335" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="336" spans="3:3">
       <c r="C336" t="s">
-        <v>322</v>
+        <v>409</v>
       </c>
     </row>
     <row r="337" spans="3:3">
       <c r="C337" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="338" spans="3:3">
       <c r="C338" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="339" spans="3:3">
       <c r="C339" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="340" spans="3:3">
       <c r="C340" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="341" spans="3:3">
       <c r="C341" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="342" spans="3:3">
       <c r="C342" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="343" spans="3:3">
       <c r="C343" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="344" spans="3:3">
       <c r="C344" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="345" spans="3:3">
       <c r="C345" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="346" spans="3:3">
       <c r="C346" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="347" spans="3:3">
       <c r="C347" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="348" spans="3:3">
       <c r="C348" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="349" spans="3:3">
       <c r="C349" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="350" spans="3:3">
       <c r="C350" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="351" spans="3:3">
       <c r="C351" t="s">
-        <v>600</v>
+        <v>315</v>
       </c>
     </row>
     <row r="352" spans="3:3">
@@ -6172,82 +6235,82 @@
     </row>
     <row r="355" spans="3:3">
       <c r="C355" t="s">
-        <v>322</v>
+        <v>413</v>
       </c>
     </row>
     <row r="356" spans="3:3">
       <c r="C356" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="357" spans="3:3">
       <c r="C357" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
     </row>
     <row r="358" spans="3:3">
       <c r="C358" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="359" spans="3:3">
       <c r="C359" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="360" spans="3:3">
       <c r="C360" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="361" spans="3:3">
       <c r="C361" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="362" spans="3:3">
       <c r="C362" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="363" spans="3:3">
       <c r="C363" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="364" spans="3:3">
       <c r="C364" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="365" spans="3:3">
       <c r="C365" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="366" spans="3:3">
       <c r="C366" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="367" spans="3:3">
       <c r="C367" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="368" spans="3:3">
       <c r="C368" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
     </row>
     <row r="369" spans="3:3">
       <c r="C369" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="370" spans="3:3">
       <c r="C370" t="s">
-        <v>413</v>
+        <v>315</v>
       </c>
     </row>
     <row r="371" spans="3:3">
@@ -6267,32 +6330,32 @@
     </row>
     <row r="374" spans="3:3">
       <c r="C374" t="s">
-        <v>322</v>
+        <v>417</v>
       </c>
     </row>
     <row r="375" spans="3:3">
       <c r="C375" t="s">
-        <v>323</v>
+        <v>373</v>
       </c>
     </row>
     <row r="376" spans="3:3">
       <c r="C376" t="s">
-        <v>319</v>
+        <v>397</v>
       </c>
     </row>
     <row r="377" spans="3:3">
       <c r="C377" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
     </row>
     <row r="378" spans="3:3">
       <c r="C378" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="379" spans="3:3">
       <c r="C379" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="380" spans="3:3">
@@ -6322,7 +6385,7 @@
     </row>
     <row r="385" spans="3:3">
       <c r="C385" t="s">
-        <v>332</v>
+        <v>418</v>
       </c>
     </row>
     <row r="386" spans="3:3">
@@ -6342,32 +6405,32 @@
     </row>
     <row r="389" spans="3:3">
       <c r="C389" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="390" spans="3:3">
       <c r="C390" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
     </row>
     <row r="391" spans="3:3">
       <c r="C391" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
     </row>
     <row r="392" spans="3:3">
       <c r="C392" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="393" spans="3:3">
       <c r="C393" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="394" spans="3:3">
       <c r="C394" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="395" spans="3:3">
@@ -6412,7 +6475,7 @@
     </row>
     <row r="403" spans="3:3">
       <c r="C403" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="404" spans="3:3">
@@ -6432,32 +6495,32 @@
     </row>
     <row r="407" spans="3:3">
       <c r="C407" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
     </row>
     <row r="408" spans="3:3">
       <c r="C408" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="409" spans="3:3">
       <c r="C409" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
     </row>
     <row r="410" spans="3:3">
       <c r="C410" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="411" spans="3:3">
       <c r="C411" t="s">
-        <v>376</v>
+        <v>322</v>
       </c>
     </row>
     <row r="412" spans="3:3">
       <c r="C412" t="s">
-        <v>400</v>
+        <v>323</v>
       </c>
     </row>
     <row r="413" spans="3:3">
@@ -6472,237 +6535,237 @@
     </row>
     <row r="415" spans="3:3">
       <c r="C415" t="s">
-        <v>325</v>
+        <v>365</v>
       </c>
     </row>
     <row r="416" spans="3:3">
       <c r="C416" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="417" spans="3:3">
       <c r="C417" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="418" spans="3:3">
       <c r="C418" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="419" spans="3:3">
       <c r="C419" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="420" spans="3:3">
       <c r="C420" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="421" spans="3:3">
       <c r="C421" t="s">
-        <v>421</v>
+        <v>333</v>
       </c>
     </row>
     <row r="422" spans="3:3">
       <c r="C422" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="423" spans="3:3">
       <c r="C423" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="424" spans="3:3">
       <c r="C424" t="s">
-        <v>315</v>
+        <v>424</v>
       </c>
     </row>
     <row r="425" spans="3:3">
       <c r="C425" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="426" spans="3:3">
       <c r="C426" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
     </row>
     <row r="427" spans="3:3">
       <c r="C427" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="428" spans="3:3">
       <c r="C428" t="s">
-        <v>426</v>
+        <v>373</v>
       </c>
     </row>
     <row r="429" spans="3:3">
       <c r="C429" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="430" spans="3:3">
       <c r="C430" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="431" spans="3:3">
       <c r="C431" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="432" spans="3:3">
       <c r="C432" t="s">
-        <v>324</v>
+        <v>365</v>
       </c>
     </row>
     <row r="433" spans="3:3">
       <c r="C433" t="s">
-        <v>368</v>
+        <v>328</v>
       </c>
     </row>
     <row r="434" spans="3:3">
       <c r="C434" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="435" spans="3:3">
       <c r="C435" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="436" spans="3:3">
       <c r="C436" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="437" spans="3:3">
       <c r="C437" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="438" spans="3:3">
       <c r="C438" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="439" spans="3:3">
       <c r="C439" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="440" spans="3:3">
       <c r="C440" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="441" spans="3:3">
       <c r="C441" t="s">
-        <v>315</v>
+        <v>428</v>
       </c>
     </row>
     <row r="442" spans="3:3">
       <c r="C442" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="443" spans="3:3">
       <c r="C443" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="444" spans="3:3">
       <c r="C444" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="445" spans="3:3">
       <c r="C445" t="s">
-        <v>430</v>
+        <v>373</v>
       </c>
     </row>
     <row r="446" spans="3:3">
       <c r="C446" t="s">
-        <v>376</v>
+        <v>323</v>
       </c>
     </row>
     <row r="447" spans="3:3">
       <c r="C447" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="448" spans="3:3">
       <c r="C448" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="449" spans="3:3">
       <c r="C449" t="s">
-        <v>324</v>
+        <v>365</v>
       </c>
     </row>
     <row r="450" spans="3:3">
       <c r="C450" t="s">
-        <v>368</v>
+        <v>328</v>
       </c>
     </row>
     <row r="451" spans="3:3">
       <c r="C451" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="452" spans="3:3">
       <c r="C452" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="453" spans="3:3">
       <c r="C453" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="454" spans="3:3">
       <c r="C454" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="455" spans="3:3">
       <c r="C455" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="456" spans="3:3">
       <c r="C456" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="457" spans="3:3">
       <c r="C457" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="458" spans="3:3">
       <c r="C458" t="s">
-        <v>315</v>
+        <v>432</v>
       </c>
     </row>
     <row r="459" spans="3:3">
       <c r="C459" t="s">
-        <v>431</v>
+        <v>316</v>
       </c>
     </row>
     <row r="460" spans="3:3">
       <c r="C460" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
     </row>
     <row r="461" spans="3:3">
       <c r="C461" t="s">
-        <v>433</v>
+        <v>317</v>
       </c>
     </row>
     <row r="462" spans="3:3">
@@ -6712,67 +6775,67 @@
     </row>
     <row r="463" spans="3:3">
       <c r="C463" t="s">
-        <v>376</v>
+        <v>318</v>
       </c>
     </row>
     <row r="464" spans="3:3">
       <c r="C464" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
     </row>
     <row r="465" spans="3:3">
       <c r="C465" t="s">
-        <v>319</v>
+        <v>435</v>
       </c>
     </row>
     <row r="466" spans="3:3">
       <c r="C466" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
     </row>
     <row r="467" spans="3:3">
       <c r="C467" t="s">
-        <v>368</v>
+        <v>321</v>
       </c>
     </row>
     <row r="468" spans="3:3">
       <c r="C468" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
     </row>
     <row r="469" spans="3:3">
       <c r="C469" t="s">
-        <v>329</v>
+        <v>436</v>
       </c>
     </row>
     <row r="470" spans="3:3">
       <c r="C470" t="s">
-        <v>330</v>
+        <v>437</v>
       </c>
     </row>
     <row r="471" spans="3:3">
       <c r="C471" t="s">
-        <v>331</v>
+        <v>438</v>
       </c>
     </row>
     <row r="472" spans="3:3">
       <c r="C472" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
     </row>
     <row r="473" spans="3:3">
       <c r="C473" t="s">
-        <v>333</v>
+        <v>434</v>
       </c>
     </row>
     <row r="474" spans="3:3">
       <c r="C474" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="475" spans="3:3">
       <c r="C475" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="476" spans="3:3">
@@ -6782,147 +6845,147 @@
     </row>
     <row r="477" spans="3:3">
       <c r="C477" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="478" spans="3:3">
       <c r="C478" t="s">
-        <v>436</v>
+        <v>321</v>
       </c>
     </row>
     <row r="479" spans="3:3">
       <c r="C479" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
     </row>
     <row r="480" spans="3:3">
       <c r="C480" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="481" spans="3:3">
       <c r="C481" t="s">
-        <v>318</v>
+        <v>440</v>
       </c>
     </row>
     <row r="482" spans="3:3">
       <c r="C482" t="s">
-        <v>319</v>
+        <v>441</v>
       </c>
     </row>
     <row r="483" spans="3:3">
       <c r="C483" t="s">
-        <v>438</v>
+        <v>317</v>
       </c>
     </row>
     <row r="484" spans="3:3">
       <c r="C484" t="s">
-        <v>320</v>
+        <v>355</v>
       </c>
     </row>
     <row r="485" spans="3:3">
       <c r="C485" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="486" spans="3:3">
       <c r="C486" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="487" spans="3:3">
       <c r="C487" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
     </row>
     <row r="488" spans="3:3">
       <c r="C488" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
     </row>
     <row r="489" spans="3:3">
       <c r="C489" t="s">
-        <v>441</v>
+        <v>365</v>
       </c>
     </row>
     <row r="490" spans="3:3">
       <c r="C490" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
     </row>
     <row r="491" spans="3:3">
       <c r="C491" t="s">
-        <v>437</v>
+        <v>321</v>
       </c>
     </row>
     <row r="492" spans="3:3">
       <c r="C492" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="493" spans="3:3">
       <c r="C493" t="s">
-        <v>319</v>
+        <v>444</v>
       </c>
     </row>
     <row r="494" spans="3:3">
       <c r="C494" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="495" spans="3:3">
       <c r="C495" t="s">
-        <v>320</v>
+        <v>445</v>
       </c>
     </row>
     <row r="496" spans="3:3">
       <c r="C496" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="497" spans="3:3">
       <c r="C497" t="s">
-        <v>315</v>
+        <v>355</v>
       </c>
     </row>
     <row r="498" spans="3:3">
       <c r="C498" t="s">
-        <v>442</v>
+        <v>318</v>
       </c>
     </row>
     <row r="499" spans="3:3">
       <c r="C499" t="s">
-        <v>443</v>
+        <v>319</v>
       </c>
     </row>
     <row r="500" spans="3:3">
       <c r="C500" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
     </row>
     <row r="501" spans="3:3">
       <c r="C501" t="s">
-        <v>317</v>
+        <v>443</v>
       </c>
     </row>
     <row r="502" spans="3:3">
       <c r="C502" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
     </row>
     <row r="503" spans="3:3">
       <c r="C503" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="504" spans="3:3">
       <c r="C504" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
     </row>
     <row r="505" spans="3:3">
       <c r="C505" t="s">
-        <v>445</v>
+        <v>315</v>
       </c>
     </row>
     <row r="506" spans="3:3">
@@ -6932,317 +6995,317 @@
     </row>
     <row r="507" spans="3:3">
       <c r="C507" t="s">
-        <v>368</v>
+        <v>316</v>
       </c>
     </row>
     <row r="508" spans="3:3">
       <c r="C508" t="s">
-        <v>320</v>
+        <v>447</v>
       </c>
     </row>
     <row r="509" spans="3:3">
       <c r="C509" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
     </row>
     <row r="510" spans="3:3">
       <c r="C510" t="s">
-        <v>315</v>
+        <v>434</v>
       </c>
     </row>
     <row r="511" spans="3:3">
       <c r="C511" t="s">
-        <v>447</v>
+        <v>318</v>
       </c>
     </row>
     <row r="512" spans="3:3">
       <c r="C512" t="s">
-        <v>443</v>
+        <v>319</v>
       </c>
     </row>
     <row r="513" spans="3:3">
       <c r="C513" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
     </row>
     <row r="514" spans="3:3">
       <c r="C514" t="s">
-        <v>317</v>
+        <v>443</v>
       </c>
     </row>
     <row r="515" spans="3:3">
       <c r="C515" t="s">
-        <v>358</v>
+        <v>325</v>
       </c>
     </row>
     <row r="516" spans="3:3">
       <c r="C516" t="s">
-        <v>318</v>
+        <v>448</v>
       </c>
     </row>
     <row r="517" spans="3:3">
       <c r="C517" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
     </row>
     <row r="518" spans="3:3">
       <c r="C518" t="s">
-        <v>445</v>
+        <v>321</v>
       </c>
     </row>
     <row r="519" spans="3:3">
       <c r="C519" t="s">
-        <v>446</v>
+        <v>315</v>
       </c>
     </row>
     <row r="520" spans="3:3">
       <c r="C520" t="s">
-        <v>368</v>
+        <v>449</v>
       </c>
     </row>
     <row r="521" spans="3:3">
       <c r="C521" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
     </row>
     <row r="522" spans="3:3">
       <c r="C522" t="s">
-        <v>321</v>
+        <v>450</v>
       </c>
     </row>
     <row r="523" spans="3:3">
       <c r="C523" t="s">
-        <v>315</v>
+        <v>451</v>
       </c>
     </row>
     <row r="524" spans="3:3">
       <c r="C524" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
     </row>
     <row r="525" spans="3:3">
       <c r="C525" t="s">
-        <v>316</v>
+        <v>453</v>
       </c>
     </row>
     <row r="526" spans="3:3">
       <c r="C526" t="s">
-        <v>450</v>
+        <v>319</v>
       </c>
     </row>
     <row r="527" spans="3:3">
       <c r="C527" t="s">
-        <v>317</v>
+        <v>454</v>
       </c>
     </row>
     <row r="528" spans="3:3">
       <c r="C528" t="s">
-        <v>437</v>
+        <v>328</v>
       </c>
     </row>
     <row r="529" spans="3:3">
       <c r="C529" t="s">
-        <v>318</v>
+        <v>455</v>
       </c>
     </row>
     <row r="530" spans="3:3">
       <c r="C530" t="s">
-        <v>319</v>
+        <v>456</v>
       </c>
     </row>
     <row r="531" spans="3:3">
       <c r="C531" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
     </row>
     <row r="532" spans="3:3">
       <c r="C532" t="s">
-        <v>446</v>
+        <v>321</v>
       </c>
     </row>
     <row r="533" spans="3:3">
       <c r="C533" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
     </row>
     <row r="534" spans="3:3">
       <c r="C534" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
     </row>
     <row r="535" spans="3:3">
       <c r="C535" t="s">
-        <v>320</v>
+        <v>459</v>
       </c>
     </row>
     <row r="536" spans="3:3">
       <c r="C536" t="s">
-        <v>321</v>
+        <v>460</v>
       </c>
     </row>
     <row r="537" spans="3:3">
       <c r="C537" t="s">
-        <v>315</v>
+        <v>461</v>
       </c>
     </row>
     <row r="538" spans="3:3">
       <c r="C538" t="s">
-        <v>452</v>
+        <v>462</v>
       </c>
     </row>
     <row r="539" spans="3:3">
       <c r="C539" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
     </row>
     <row r="540" spans="3:3">
       <c r="C540" t="s">
-        <v>453</v>
+        <v>319</v>
       </c>
     </row>
     <row r="541" spans="3:3">
       <c r="C541" t="s">
-        <v>454</v>
+        <v>463</v>
       </c>
     </row>
     <row r="542" spans="3:3">
       <c r="C542" t="s">
-        <v>455</v>
+        <v>320</v>
       </c>
     </row>
     <row r="543" spans="3:3">
       <c r="C543" t="s">
-        <v>456</v>
+        <v>321</v>
       </c>
     </row>
     <row r="544" spans="3:3">
       <c r="C544" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
     </row>
     <row r="545" spans="3:3">
       <c r="C545" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
     </row>
     <row r="546" spans="3:3">
       <c r="C546" t="s">
-        <v>328</v>
+        <v>459</v>
       </c>
     </row>
     <row r="547" spans="3:3">
       <c r="C547" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
     </row>
     <row r="548" spans="3:3">
       <c r="C548" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
     </row>
     <row r="549" spans="3:3">
       <c r="C549" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
     </row>
     <row r="550" spans="3:3">
       <c r="C550" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="551" spans="3:3">
       <c r="C551" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="552" spans="3:3">
       <c r="C552" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="553" spans="3:3">
       <c r="C553" t="s">
-        <v>462</v>
+        <v>320</v>
       </c>
     </row>
     <row r="554" spans="3:3">
       <c r="C554" t="s">
-        <v>463</v>
+        <v>321</v>
       </c>
     </row>
     <row r="555" spans="3:3">
       <c r="C555" t="s">
-        <v>464</v>
+        <v>315</v>
       </c>
     </row>
     <row r="556" spans="3:3">
       <c r="C556" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="557" spans="3:3">
       <c r="C557" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
     </row>
     <row r="558" spans="3:3">
       <c r="C558" t="s">
-        <v>319</v>
+        <v>468</v>
       </c>
     </row>
     <row r="559" spans="3:3">
       <c r="C559" t="s">
-        <v>466</v>
+        <v>461</v>
       </c>
     </row>
     <row r="560" spans="3:3">
       <c r="C560" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="561" spans="3:3">
       <c r="C561" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="562" spans="3:3">
       <c r="C562" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="563" spans="3:3">
       <c r="C563" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
     </row>
     <row r="564" spans="3:3">
       <c r="C564" t="s">
-        <v>462</v>
+        <v>320</v>
       </c>
     </row>
     <row r="565" spans="3:3">
       <c r="C565" t="s">
-        <v>468</v>
+        <v>321</v>
       </c>
     </row>
     <row r="566" spans="3:3">
       <c r="C566" t="s">
-        <v>469</v>
+        <v>315</v>
       </c>
     </row>
     <row r="567" spans="3:3">
       <c r="C567" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
     </row>
     <row r="568" spans="3:3">
       <c r="C568" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
     </row>
     <row r="569" spans="3:3">
       <c r="C569" t="s">
-        <v>319</v>
+        <v>470</v>
       </c>
     </row>
     <row r="570" spans="3:3">
@@ -7252,182 +7315,182 @@
     </row>
     <row r="571" spans="3:3">
       <c r="C571" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="572" spans="3:3">
       <c r="C572" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="573" spans="3:3">
       <c r="C573" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="574" spans="3:3">
       <c r="C574" t="s">
-        <v>470</v>
+        <v>463</v>
       </c>
     </row>
     <row r="575" spans="3:3">
       <c r="C575" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="576" spans="3:3">
       <c r="C576" t="s">
-        <v>471</v>
+        <v>321</v>
       </c>
     </row>
     <row r="577" spans="3:3">
       <c r="C577" t="s">
-        <v>464</v>
+        <v>315</v>
       </c>
     </row>
     <row r="578" spans="3:3">
       <c r="C578" t="s">
-        <v>465</v>
+        <v>471</v>
       </c>
     </row>
     <row r="579" spans="3:3">
       <c r="C579" t="s">
-        <v>335</v>
+        <v>316</v>
       </c>
     </row>
     <row r="580" spans="3:3">
       <c r="C580" t="s">
-        <v>319</v>
+        <v>472</v>
       </c>
     </row>
     <row r="581" spans="3:3">
       <c r="C581" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
     </row>
     <row r="582" spans="3:3">
       <c r="C582" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="583" spans="3:3">
       <c r="C583" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="584" spans="3:3">
       <c r="C584" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="585" spans="3:3">
       <c r="C585" t="s">
-        <v>472</v>
+        <v>463</v>
       </c>
     </row>
     <row r="586" spans="3:3">
       <c r="C586" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="587" spans="3:3">
       <c r="C587" t="s">
-        <v>473</v>
+        <v>321</v>
       </c>
     </row>
     <row r="588" spans="3:3">
       <c r="C588" t="s">
-        <v>469</v>
+        <v>315</v>
       </c>
     </row>
     <row r="589" spans="3:3">
       <c r="C589" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
     </row>
     <row r="590" spans="3:3">
       <c r="C590" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="591" spans="3:3">
       <c r="C591" t="s">
-        <v>319</v>
+        <v>475</v>
       </c>
     </row>
     <row r="592" spans="3:3">
       <c r="C592" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
     </row>
     <row r="593" spans="3:3">
       <c r="C593" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="594" spans="3:3">
       <c r="C594" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="595" spans="3:3">
       <c r="C595" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="596" spans="3:3">
       <c r="C596" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="597" spans="3:3">
       <c r="C597" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="598" spans="3:3">
       <c r="C598" t="s">
-        <v>475</v>
+        <v>321</v>
       </c>
     </row>
     <row r="599" spans="3:3">
       <c r="C599" t="s">
-        <v>476</v>
+        <v>315</v>
       </c>
     </row>
     <row r="600" spans="3:3">
       <c r="C600" t="s">
-        <v>465</v>
+        <v>478</v>
       </c>
     </row>
     <row r="601" spans="3:3">
       <c r="C601" t="s">
-        <v>335</v>
+        <v>415</v>
       </c>
     </row>
     <row r="602" spans="3:3">
       <c r="C602" t="s">
-        <v>319</v>
+        <v>479</v>
       </c>
     </row>
     <row r="603" spans="3:3">
       <c r="C603" t="s">
-        <v>466</v>
+        <v>480</v>
       </c>
     </row>
     <row r="604" spans="3:3">
       <c r="C604" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="605" spans="3:3">
       <c r="C605" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="606" spans="3:3">
       <c r="C606" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="607" spans="3:3">
@@ -7437,282 +7500,192 @@
     </row>
     <row r="608" spans="3:3">
       <c r="C608" t="s">
-        <v>334</v>
+        <v>320</v>
       </c>
     </row>
     <row r="609" spans="3:3">
       <c r="C609" t="s">
-        <v>478</v>
+        <v>321</v>
       </c>
     </row>
     <row r="610" spans="3:3">
       <c r="C610" t="s">
-        <v>479</v>
+        <v>315</v>
       </c>
     </row>
     <row r="611" spans="3:3">
       <c r="C611" t="s">
-        <v>465</v>
+        <v>481</v>
       </c>
     </row>
     <row r="612" spans="3:3">
       <c r="C612" t="s">
-        <v>335</v>
+        <v>415</v>
       </c>
     </row>
     <row r="613" spans="3:3">
       <c r="C613" t="s">
-        <v>319</v>
+        <v>482</v>
       </c>
     </row>
     <row r="614" spans="3:3">
       <c r="C614" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="615" spans="3:3">
       <c r="C615" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="616" spans="3:3">
       <c r="C616" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="617" spans="3:3">
       <c r="C617" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="618" spans="3:3">
       <c r="C618" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
     </row>
     <row r="619" spans="3:3">
       <c r="C619" t="s">
-        <v>418</v>
+        <v>320</v>
       </c>
     </row>
     <row r="620" spans="3:3">
       <c r="C620" t="s">
-        <v>482</v>
+        <v>321</v>
       </c>
     </row>
     <row r="621" spans="3:3">
       <c r="C621" t="s">
-        <v>483</v>
+        <v>315</v>
       </c>
     </row>
     <row r="622" spans="3:3">
       <c r="C622" t="s">
-        <v>465</v>
+        <v>484</v>
       </c>
     </row>
     <row r="623" spans="3:3">
       <c r="C623" t="s">
-        <v>335</v>
+        <v>485</v>
       </c>
     </row>
     <row r="624" spans="3:3">
       <c r="C624" t="s">
-        <v>319</v>
+        <v>486</v>
       </c>
     </row>
     <row r="625" spans="3:3">
       <c r="C625" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
     </row>
     <row r="626" spans="3:3">
       <c r="C626" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="627" spans="3:3">
       <c r="C627" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="628" spans="3:3">
       <c r="C628" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="629" spans="3:3">
       <c r="C629" t="s">
-        <v>484</v>
+        <v>477</v>
       </c>
     </row>
     <row r="630" spans="3:3">
       <c r="C630" t="s">
-        <v>418</v>
+        <v>320</v>
       </c>
     </row>
     <row r="631" spans="3:3">
       <c r="C631" t="s">
-        <v>485</v>
+        <v>321</v>
       </c>
     </row>
     <row r="632" spans="3:3">
       <c r="C632" t="s">
-        <v>486</v>
+        <v>315</v>
       </c>
     </row>
     <row r="633" spans="3:3">
       <c r="C633" t="s">
-        <v>465</v>
+        <v>488</v>
       </c>
     </row>
     <row r="634" spans="3:3">
       <c r="C634" t="s">
-        <v>335</v>
+        <v>485</v>
       </c>
     </row>
     <row r="635" spans="3:3">
       <c r="C635" t="s">
-        <v>319</v>
+        <v>489</v>
       </c>
     </row>
     <row r="636" spans="3:3">
       <c r="C636" t="s">
-        <v>480</v>
+        <v>490</v>
       </c>
     </row>
     <row r="637" spans="3:3">
       <c r="C637" t="s">
-        <v>320</v>
+        <v>462</v>
       </c>
     </row>
     <row r="638" spans="3:3">
       <c r="C638" t="s">
-        <v>321</v>
+        <v>335</v>
       </c>
     </row>
     <row r="639" spans="3:3">
       <c r="C639" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
     </row>
     <row r="640" spans="3:3">
       <c r="C640" t="s">
-        <v>487</v>
+        <v>477</v>
       </c>
     </row>
     <row r="641" spans="3:3">
       <c r="C641" t="s">
-        <v>488</v>
+        <v>320</v>
       </c>
     </row>
     <row r="642" spans="3:3">
       <c r="C642" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="643" spans="3:3">
       <c r="C643" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="644" spans="3:3">
       <c r="C644" t="s">
-        <v>465</v>
+        <v>493</v>
       </c>
     </row>
     <row r="645" spans="3:3">
       <c r="C645" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="646" spans="3:3">
-      <c r="C646" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="647" spans="3:3">
-      <c r="C647" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="648" spans="3:3">
-      <c r="C648" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="649" spans="3:3">
-      <c r="C649" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="650" spans="3:3">
-      <c r="C650" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="651" spans="3:3">
-      <c r="C651" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="652" spans="3:3">
-      <c r="C652" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="653" spans="3:3">
-      <c r="C653" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="654" spans="3:3">
-      <c r="C654" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="655" spans="3:3">
-      <c r="C655" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="656" spans="3:3">
-      <c r="C656" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="657" spans="3:3">
-      <c r="C657" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="658" spans="3:3">
-      <c r="C658" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="659" spans="3:3">
-      <c r="C659" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="660" spans="3:3">
-      <c r="C660" t="s">
         <v>494</v>
-      </c>
-    </row>
-    <row r="661" spans="3:3">
-      <c r="C661" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="662" spans="3:3">
-      <c r="C662" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="663" spans="3:3">
-      <c r="C663" t="s">
-        <v>497</v>
       </c>
     </row>
   </sheetData>
@@ -7726,7 +7699,7 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B1:E56"/>
+  <dimension ref="B1:E61"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="51.75" customWidth="1"/>
@@ -7737,12 +7710,12 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="2" spans="2:5">
       <c r="B2" s="2" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="E2" s="3"/>
     </row>
@@ -7920,10 +7893,10 @@
     </row>
     <row r="29" spans="2:5" ht="37.5">
       <c r="B29" s="1" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="E29" s="3">
         <v>46043</v>
@@ -7931,15 +7904,15 @@
     </row>
     <row r="30" spans="2:5" ht="318.75">
       <c r="B30" s="1" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
     </row>
     <row r="31" spans="2:5" ht="37.5">
       <c r="B31" s="1" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="E31" s="3">
         <v>46043</v>
@@ -7947,10 +7920,10 @@
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="1" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="E33" s="3">
         <v>46043</v>
@@ -7958,18 +7931,18 @@
     </row>
     <row r="35" spans="2:5" ht="37.5">
       <c r="B35" s="1" t="s">
-        <v>557</v>
+        <v>554</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>558</v>
+        <v>555</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="37.5">
       <c r="B36" s="1" t="s">
-        <v>559</v>
+        <v>556</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>560</v>
+        <v>557</v>
       </c>
       <c r="E36" s="3">
         <v>46043</v>
@@ -7977,10 +7950,10 @@
     </row>
     <row r="37" spans="2:5" ht="56.25">
       <c r="B37" s="1" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="E37" s="3">
         <v>46043</v>
@@ -7988,10 +7961,10 @@
     </row>
     <row r="38" spans="2:5" ht="93.75">
       <c r="B38" s="1" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="E38" s="3">
         <v>46043</v>
@@ -7999,18 +7972,18 @@
     </row>
     <row r="40" spans="2:5">
       <c r="B40" s="1" t="s">
-        <v>575</v>
+        <v>572</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
     </row>
     <row r="42" spans="2:5" ht="56.25">
       <c r="B42" s="1" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="E42" s="3">
         <v>46045</v>
@@ -8018,26 +7991,26 @@
     </row>
     <row r="43" spans="2:5" ht="37.5">
       <c r="B43" s="1" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
     </row>
     <row r="44" spans="2:5" ht="37.5">
       <c r="B44" s="1" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
     </row>
     <row r="45" spans="2:5" ht="37.5">
       <c r="B45" s="1" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>584</v>
+        <v>581</v>
       </c>
       <c r="E45" s="3">
         <v>46045</v>
@@ -8045,10 +8018,10 @@
     </row>
     <row r="46" spans="2:5" ht="56.25">
       <c r="B46" s="1" t="s">
-        <v>593</v>
+        <v>590</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>594</v>
+        <v>591</v>
       </c>
       <c r="E46" s="3">
         <v>46050</v>
@@ -8056,10 +8029,10 @@
     </row>
     <row r="47" spans="2:5" ht="56.25">
       <c r="B47" s="1" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="E47" s="3">
         <v>46050</v>
@@ -8067,10 +8040,10 @@
     </row>
     <row r="48" spans="2:5" ht="37.5">
       <c r="B48" s="1" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="E48" s="3">
         <v>46050</v>
@@ -8078,7 +8051,7 @@
     </row>
     <row r="49" spans="2:5" ht="409.5">
       <c r="B49" s="1" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="E49" s="3">
         <v>46050</v>
@@ -8086,10 +8059,10 @@
     </row>
     <row r="51" spans="2:5">
       <c r="B51" s="1" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="E51" s="3">
         <v>46050</v>
@@ -8097,37 +8070,64 @@
     </row>
     <row r="53" spans="2:5" ht="37.5">
       <c r="B53" s="1" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="54" spans="2:5" ht="37.5">
       <c r="B54" s="1" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
     </row>
     <row r="55" spans="2:5" ht="56.25">
       <c r="B55" s="1" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="56" spans="2:5" ht="37.5">
       <c r="B56" s="1" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E56" s="3">
         <v>46050</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" ht="37.5">
+      <c r="B57" s="1" t="s">
+        <v>617</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>618</v>
+      </c>
+      <c r="E57" s="3">
+        <v>46060</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5">
+      <c r="B59" s="1" t="s">
+        <v>619</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" ht="37.5">
+      <c r="B61" s="1" t="s">
+        <v>621</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>622</v>
       </c>
     </row>
   </sheetData>
@@ -8159,7 +8159,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8301,10 +8301,10 @@
     </row>
     <row r="23" spans="2:5" ht="93.75">
       <c r="B23" s="1" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="E23" s="3">
         <v>46043</v>
@@ -8312,10 +8312,10 @@
     </row>
     <row r="25" spans="2:5" ht="56.25">
       <c r="B25" s="1" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="E25" s="3">
         <v>46044</v>
@@ -8323,10 +8323,10 @@
     </row>
     <row r="26" spans="2:5" ht="56.25">
       <c r="B26" s="1" t="s">
-        <v>585</v>
+        <v>582</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="E26" s="3">
         <v>46045</v>
@@ -8334,10 +8334,10 @@
     </row>
     <row r="27" spans="2:5" ht="56.25">
       <c r="B27" s="1" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>590</v>
+        <v>587</v>
       </c>
       <c r="E27" s="3">
         <v>46050</v>
@@ -8372,7 +8372,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8395,63 +8395,63 @@
     </row>
     <row r="6" spans="2:5">
       <c r="B6" s="5" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" s="1" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="C8" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="C9" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="37.5">
       <c r="B11" s="1" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="75">
       <c r="B12" s="1" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="13" spans="2:5" ht="37.5">
       <c r="B13" s="1" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
     </row>
     <row r="14" spans="2:5" ht="75">
       <c r="B14" s="1" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="E14" s="3">
         <v>46043</v>
@@ -8459,10 +8459,10 @@
     </row>
     <row r="15" spans="2:5" ht="56.25">
       <c r="B15" s="1" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="E15" s="3">
         <v>46043</v>
@@ -8470,10 +8470,10 @@
     </row>
     <row r="16" spans="2:5" ht="37.5">
       <c r="B16" s="1" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="E16" s="3">
         <v>46050</v>
@@ -8534,18 +8534,18 @@
     </row>
     <row r="8" spans="3:4" ht="112.5">
       <c r="C8" s="1" t="s">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="9" spans="3:4" ht="56.25">
       <c r="C9" s="1" t="s">
-        <v>595</v>
+        <v>592</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
     </row>
   </sheetData>
@@ -8816,7 +8816,7 @@
         <v>17</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
     </row>
   </sheetData>
@@ -8827,7 +8827,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB9A9986-272E-4F2B-8815-9B72212F3499}">
-  <dimension ref="B3:F7"/>
+  <dimension ref="B3:F8"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
@@ -8896,6 +8896,12 @@
       </c>
       <c r="E7" s="3">
         <v>46039</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6">
+      <c r="B8">
+        <f>B7+1</f>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -9187,7 +9193,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46052</v>
+        <v>46060</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
fix: update user count query to use 'user_profiles' table instead of 'profiles'
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F74B50-1C10-4E75-A9B7-6AF9E7D1A0DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40E05B5-05DC-4346-B465-3AEC70FB13D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="8" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1174" uniqueCount="629">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -3190,6 +3190,30 @@
   </si>
   <si>
     <t>以下の例は、これらのコンポーネントが異なる種類のリクエストに対してどのように連携するかを示しています。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Text-only prompt</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>テキストのみのプロンプト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>A simple text prompt consists of a contents array with a single Content object.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>単純なテキストプロンプトは、単一のContentオブジェクトを含むコンテンツ配列で構成されます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>That object's parts array, in turn, contains a single Part object with a text field.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>そのオブジェクトのパーツ配列は、さらに単一のPartオブジェクトを含み、そのオブジェクトにはテキストフィールドが備わっている。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -7699,7 +7723,7 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="B1:E61"/>
+  <dimension ref="B1:E66"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="51.75" customWidth="1"/>
@@ -8128,6 +8152,33 @@
       </c>
       <c r="C61" s="1" t="s">
         <v>622</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5">
+      <c r="B63" t="s">
+        <v>623</v>
+      </c>
+      <c r="C63" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" ht="37.5">
+      <c r="B65" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="E65" s="3">
+        <v>46060</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" ht="56.25">
+      <c r="B66" s="1" t="s">
+        <v>627</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>628</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add MindlessTaskPage for managing mindless tasks with date selection
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB5E2A00-3A95-43F3-A2E7-AB1D3F92A06D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D325D140-8163-4EFE-BFC6-F3770CD05214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -28,12 +28,19 @@
     <sheet name="model一覧" sheetId="17" r:id="rId13"/>
     <sheet name="Gemini API reference" sheetId="12" r:id="rId14"/>
     <sheet name="Prompt design strategies" sheetId="19" r:id="rId15"/>
-    <sheet name="Gemini Code Assist" sheetId="15" r:id="rId16"/>
-    <sheet name="Gemini Code Assist 2" sheetId="18" r:id="rId17"/>
-    <sheet name="How to fix" sheetId="16" r:id="rId18"/>
-    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId19"/>
+    <sheet name="x" sheetId="20" r:id="rId16"/>
+    <sheet name="X2" sheetId="21" r:id="rId17"/>
+    <sheet name="時記" sheetId="22" r:id="rId18"/>
+    <sheet name="Gemini Code Assist" sheetId="15" r:id="rId19"/>
+    <sheet name="Gemini Code Assist 2" sheetId="18" r:id="rId20"/>
+    <sheet name="How to fix" sheetId="16" r:id="rId21"/>
+    <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId22"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">x!$C$2:$M$117</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -54,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="801">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -3219,6 +3226,1245 @@
   </si>
   <si>
     <t>Prompt design strategies</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/i/bookmarks/1796518698825683108</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>規格外</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人生変えたきゃ、使う言葉を変えるだけ｜社員一人、億単位の営業利益を20年｜独占ニッチ市場を0から創造＆上場企業に事業売却｜とある中高一貫男子校⇨京都大学大学院中退｜新刊『すべては言葉からはじまる』 https://amzn.asia/d/aMdWcLF</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ワイの会社、社員一名なんよ。「社員何人？」と聞かれて「一人」と答えると、バカにしたような顔されることがあるけど、一人当たりの利益は億単位よ。しかも20年。さらに固定費極小、ほぼ変動費。事務所すらないからね。潰れようがない会社。大したことないけど馬鹿にされることもないと思っとるよ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>みんな、「少額浪費」の恐ろしさを分かっていない。
+毎日なんとなく買うコンビニのコーヒーや、解約し忘れのサブスク。その数千円を本や経験に置き換えるだけで、5年後の景色が激変する。
+お金がないと嘆く人に限って、財布の底に穴が空いている。豊かさの差は、能力差ではなく、規律の差。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ポスト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>少額浪費</t>
+    <rPh sb="0" eb="2">
+      <t>ショウガク</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ロウヒ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>コンビニ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>コーヒー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>解約</t>
+    <rPh sb="0" eb="2">
+      <t>カイヤク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>サブスク</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>数千円</t>
+    <rPh sb="0" eb="1">
+      <t>スウ</t>
+    </rPh>
+    <rPh sb="1" eb="3">
+      <t>センエン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>本</t>
+    <rPh sb="0" eb="1">
+      <t>ホン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>経験</t>
+    <rPh sb="0" eb="2">
+      <t>ケイケン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>5年後</t>
+    <rPh sb="1" eb="3">
+      <t>ネンゴ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>景色</t>
+    <rPh sb="0" eb="2">
+      <t>ケシキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>激変</t>
+    <rPh sb="0" eb="2">
+      <t>ゲキヘン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>お金</t>
+    <rPh sb="1" eb="2">
+      <t>カネ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>嘆く</t>
+    <rPh sb="0" eb="1">
+      <t>ナゲ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>財布</t>
+    <rPh sb="0" eb="2">
+      <t>サイフ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>底</t>
+    <rPh sb="0" eb="1">
+      <t>ソコ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>穴</t>
+    <rPh sb="0" eb="1">
+      <t>アナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>豊かさ</t>
+    <rPh sb="0" eb="1">
+      <t>ユタ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>能力</t>
+    <rPh sb="0" eb="2">
+      <t>ノウリョク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>規律</t>
+    <rPh sb="0" eb="2">
+      <t>キリツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「お金がない」と嘆く前に、財布の底に空いた穴を塞げ。毎日のコンビニ、何気ないコーヒー、使わないサブスク。その少額浪費があなたの豊かさを奪っている。数千円を浪費するな、本と経験に使え。その規律が能力に変わり、5年後の景色を激変させる。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>【貧乏マインド vs 金持ちマインド】
+× コンビニで散財する ○ 本を買って学ぶ
+× 無駄なサブスクを放置 ○ 不要な契約は即解約
+× 少額浪費で快楽を買う ○ 数千円で経験を買う
+× お金がないと嘆く ○ 財布の穴を塞ぐ
+日々の規律が能力の差を生む。 今日を変えれば、5年後に見える景色は激変する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>毎日コンビニで使う数千円と、本や経験に投じる数千円。金額は同じでも、5年後の豊かさは桁違いになる。少額浪費という財布の穴を放置して人生を嘆くな。規律を持て。その選択一つで、見える景色は激変する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/genkaidokusho/status/2022062512620114288</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>限界読書</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>X</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>読んだ人の思考を1%アップデートするアカウント｜弱者生存戦略×読書×言語化｜20歳の自分が知りたかった知恵と思考を発信｜Amazonアソシエイト参加中｜ハイライトには本紹介ポスト
+note.com/genkaidokusho/…
+Joined July 2023</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>noteでメンバーシップ「思考発酵ラボ」を運営しています。1,500名以上の方にご加入いただいています。
+「カネなし、コネなし、チカラなし」から人生を好転させるための弱者生存戦略をテーマにした200以上の記事を月額500円から読めます。ぜひご加入ください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ロールモデルとなるような人を見つけたら、その人の
+「今の行動」を真似るだけではなくて、その人が「今の状態になるまでどんな積み重ねをしてきたのか」をちゃんと聞いて、真似した方が良い。
+凄い人の「今の状態」ではなく、「そこに至る過程」にこそ、学ぶべき要素が詰まっている。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ロールモデル</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今の行動</t>
+    <rPh sb="0" eb="1">
+      <t>イマ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウドウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>真似る</t>
+    <rPh sb="0" eb="2">
+      <t>マネ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今の状態</t>
+    <rPh sb="0" eb="1">
+      <t>イマ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>ジョウタイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>積み重ね</t>
+    <rPh sb="0" eb="1">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>カサ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>真似</t>
+    <rPh sb="0" eb="2">
+      <t>マネ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>凄い人</t>
+    <rPh sb="0" eb="1">
+      <t>スゴ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ヒト</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>そこに至る過程</t>
+    <rPh sb="3" eb="4">
+      <t>イタ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>カテイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>学ぶ</t>
+    <rPh sb="0" eb="1">
+      <t>マナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>要素</t>
+    <rPh sb="0" eb="2">
+      <t>ヨウソ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>投稿</t>
+    <rPh sb="0" eb="2">
+      <t>トウコウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>インプレッション</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>このキーワードを使ってバズるポストを考えてください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>プロンプト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Folllower</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「凄い人」を見てため息をつく前に、その人がそこに至る過程を見ろ。輝かしい結果は、地味な積み重ねの氷山の一角に過ぎない。プライドを捨ててロールモデルを徹底的に真似るんだ。学ぶの語源は「真似ぶ」。思考、習慣、要素のすべてをコピーしろ。今の行動を変えない限り、今の状態は一生変わらない。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>【凡人が最短で成長する5ステップ】
+憧れのロールモデルを見つける
+その人の成功要素を分解する
+結果ではなくそこに至る過程を知る
+徹底的に真似る（TTP）
+それを毎日積み重ねる
+オリジナリティは真似の先にある。 凄い人への近道は、学ぶ（真似ぶ）こと。 今の状態を嘆く暇があるなら、今の行動を変えろ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>今の状態は、過去の自分が選んだ結果。未来を変えたいなら、今の行動を変えるしかない。凄い人も最初は凡人だった。違いはロールモデルの要素を素直に学び、狂ったように真似て、泥臭く積み重ねたかどうかだけ。憧れるな、真似るんだ。その過程だけが、あなたを本物にする。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/think_hacking/status/2021705302605787296</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>思考遊戯</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>考え方を整えるアカウント | 思考整理がテーマ | 迷い、不安、焦りが生まれる理由の分解 | 思考の変化による人生の選び方、行動の変化 | 日常と人生を題材にした思考の発信をしてます。
+note.com/think_hacking/…
+Joined March 2023</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「思考のジム」を始めました。
+仕事でも日常でも迷いが増えるのは、情報ではなく考え方の型がないからです。
+ここでは、状況整理・判断・感情の扱い方など、実務にも生きる思考の土台を毎月届けます。
+月500円で全記事読み放題。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ちゃんみなが言っていた、自由にやりたいなら先に型にはまれという話があります。
+ゴールに行くために決められた課題や、正直やりたくない作業を一度全部引き受ける。その過程を通らずに語られる自由はただの気分や憧れで終わりやすい。
+型に沿うのは個性を殺すことではありません。続けていく中で、合わない部分や無理が出てくる。その違和感こそが後から自分の色になる。
+オリジナリティは最初に出すものではなく、やるべきことをやり切ったあとに、勝手に残るものだと思います。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ちゃんみな</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自由</t>
+    <rPh sb="0" eb="2">
+      <t>ジユウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>型にはまれ</t>
+    <rPh sb="0" eb="1">
+      <t>カタ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ゴール</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>決められた課題</t>
+    <rPh sb="0" eb="1">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="5" eb="7">
+      <t>カダイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>正直</t>
+    <rPh sb="0" eb="2">
+      <t>ショウジキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>やりたくない作業</t>
+    <rPh sb="6" eb="8">
+      <t>サギョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>引き受ける</t>
+    <rPh sb="0" eb="1">
+      <t>ヒ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>過程</t>
+    <rPh sb="0" eb="2">
+      <t>カテイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>気分</t>
+    <rPh sb="0" eb="2">
+      <t>キブン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>憧れ</t>
+    <rPh sb="0" eb="1">
+      <t>アコガ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>個性</t>
+    <rPh sb="0" eb="2">
+      <t>コセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>殺す</t>
+    <rPh sb="0" eb="1">
+      <t>コロ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>続けていく</t>
+    <rPh sb="0" eb="1">
+      <t>ツヅ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>合わない部分</t>
+    <rPh sb="0" eb="1">
+      <t>ア</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ブブン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>無理</t>
+    <rPh sb="0" eb="2">
+      <t>ムリ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>違和感</t>
+    <rPh sb="0" eb="3">
+      <t>イワカン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自分の色</t>
+    <rPh sb="0" eb="2">
+      <t>ジブン</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>イロ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>オリジナリティ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>やるべきこと</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>やり切った</t>
+    <rPh sb="2" eb="3">
+      <t>キ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>勝手</t>
+    <rPh sb="0" eb="2">
+      <t>カッテ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>残る</t>
+    <rPh sb="0" eb="1">
+      <t>ノコ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「自由になりたい」と叫ぶ前に、一度黙って型にはまれ。決められた課題、やりたくない作業、全て引き受けるんだ。自分の気分なんて殺す。正直、無理だと思う瞬間もあるだろう。でも、やるべきことを徹底的にやり切った後に、どうしても合わない部分、どうしても消せずに残るもの。それこそが、誰にも真似できない自分だけの色（オリジナリティ）になる。ちゃんみなの生き様がそれを証明している。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>周りに合わせる違和感。正直、このままでいいのかという不安。でも、憧れのゴールがあるなら、その過程にある泥臭い作業も続けていくしかない。自分のエゴを殺して、型にハマってみる。それでも勝手に溢れ出てしまうもの、隠しきれずに残るもの。それが本当の個性だ。無理に探すんじゃない。やり切った先に、オリジナリティは勝手に輝く。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>オリジナリティとは、何もしない自由から生まれるんじゃない。決められた課題とやりたくない作業を完璧にこなし、自分の気分を殺してまで型にはまった結果、それでも隠しきれずに残る「違和感」のことだ。自分だけの色は、やるべきことをやり切った人間にしか見えない。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/cozeblog/status/2021736308381757789</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>こーずぶろぐ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>とにかく勉強します/新人薬剤師(27)/サウナ/読書/YouTube(7.5万)/ペンを持つことが趣味/皆様の学びをサポートしたい/ こーずぶろぐ初の著書『マジカル勉強脳』絶賛発売中http://amazon.co.jp/dp/4046068469
+ブイロガー→youtube.com/channel/UC9cn2…
+Joined April 2022</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ある日、Googleから
+「あなたは急上昇クリエイターに選ばれました」
+という一通のメールが届きました。
+正直、最初は意味が分からなくて、
+半信半疑だったけど、、
+そこから景色が変わりました。
+1週間弱で、登録者が2万人増加。
+顔出しも、声出しもなし。
+YouTube知識ゼロから始めた、
+どこにでもいる普通の大学生でも、
+急上昇クリエイターに選ばれた。
+だからこそ、この記事を書きました。
+何を考え、何を積み上げてきたのか。
+どうすれば“バズを待つ側”じゃなく、
+ “再現できる側”に回れるのか。
+全部、noteにまとめました。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 0→急上昇までの全プロセス
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 伸びた1本の裏側と、そのときの思考
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>✔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 初心者でも迷わない設計と順番
+YouTubeを本気で伸ばしたいなら、
+まずここから始めてほしい</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>⤵︎</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>勉強のスタートダッシュをうまく成功させるために、1日の始まりを私は復習から始めています。理由は以下4つです。
+①一度触れている内容なので解けやすい
+②解けた時にドーパミンが放出される
+③ドーパミンは快楽や喜びを与えてくれる
+④さらなる快楽を求めて繰り返そうとする
+復習は1番簡単に「達成感」を感じることができるのでモチベ維持に最適です。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>勉強</t>
+    <rPh sb="0" eb="2">
+      <t>ベンキョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>スタートダッシュ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>成功</t>
+    <rPh sb="0" eb="2">
+      <t>セイコウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1日の始まり</t>
+    <rPh sb="1" eb="2">
+      <t>ニチ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>ハジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>復習</t>
+    <rPh sb="0" eb="2">
+      <t>フクシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>理由</t>
+    <rPh sb="0" eb="2">
+      <t>リユウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>一度触れている内容</t>
+    <rPh sb="0" eb="2">
+      <t>イチド</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>フ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ナイヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>解けた</t>
+    <rPh sb="0" eb="1">
+      <t>ト</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ドーパミン</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>快楽</t>
+    <rPh sb="0" eb="2">
+      <t>カイラク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>喜び</t>
+    <rPh sb="0" eb="1">
+      <t>ヨロコ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>達成感</t>
+    <rPh sb="0" eb="3">
+      <t>タッセイカン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>モチベ維持</t>
+    <rPh sb="3" eb="5">
+      <t>イジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最適</t>
+    <rPh sb="0" eb="2">
+      <t>サイテキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>勉強のやる気が出ない人は、1日の始まりを間違えている。いきなり新しい問題を解くな。スタートダッシュは、必ず昨日の復習から始めろ。「一度触れている内容」だからスラスラ解けた。その瞬間の「達成感」が脳内にドーパミンをドバドバ出す。この快楽と喜びを脳に味わせるのが、最高のモチベ維持になる。朝イチは簡単な問題で脳を騙せ。これが成功への最適解だ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>【勉強で挫折する人 vs 成功する人の朝】
+× 難問から始めて絶望する ○ 復習から始めて達成感を得る
+× 無理やり机に向かう ○ 解けた！の快楽で脳を動かす
+× 気合いでモチベ維持 ○ ドーパミンを利用して自動化
+1日の始まりに「自分はできる」と脳に錯覚させろ。 一度触れている内容でスタートダッシュを決めるのが、脳科学的に最適な理由だ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1日の始まりは、昨日の復習から始めろ。なぜなら、一度触れている内容は必ず解けるからだ。その小さな成功体験が、脳に強烈な快楽（ドーパミン）を与え、勉強を「やりたくてたまらないもの」に変える。スタートダッシュで達成感を味わえ。この脳の仕組みを利用することこそが、最強のモチベ維持であり、最適な戦略だ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/yumaevo/status/2021135603333742931</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>yuma@内向哲学</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>文筆家｜早稲田大学文学部中退｜「読んだ人の思考,視点,知恵を深化する」を軸に、内向的な人に向けた人生戦略を発信しています。｜SNS,広告,文章を生業にして13年｜将棋アマ四段｜内向哲学
+@naikoutetsugaku
+｜note哲学
+@notetsugaku
+note.com/yumaevo
+Joined November 2017</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「頭の良さ」には大きく二種類あると思っています。
+ひとつは学校で測られる「頭の良さ」で、
+もうひとつは実社会で求められる「地頭の良さ」です。
+学校教育で養われる「頭の良さ」は、主に「記憶力」と「継続力」です。
+教科書に書いてあることを覚えて、テストで正確に再現する。そのために毎日コツコツと勉強を続ける。
+これができれば学校では優秀な成績を収めることができ、「頭の良い人認定」されます。
+もちろんそれはそれで大切な能力なのですが、実際のビジネスシーンなどで求められるのは、もっと別の「頭の良さ」です。
+それは言い換えれば「構造を見抜く力」だとぼくは思います。
+「構造を見抜く力」というのは、義務教育ではなかなか教われない、物事の本質を掴む力のことです。
+表面的な事象の裏側にある本質的な仕組みを理解して、
+「ああ、つまりこういうことなんだな」と悟れる力なんですよね。
+この構造把握能力は義務教育的な「マニュアル暗記力」とは異なり、
+真の意味での「地頭の良さ」のようなものだとぼくは考えています。
+構造把握能力を強化して「地頭力」を鍛えるためには、一体どうすればいいのでしょうか。
+考えていきましょう↓</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>タブーかもしれませんが、人は「同程度の頭脳レベル同士」で引き合うようになっています。
+特に夫婦関係など、深く長期的な関係だとなおさらです。
+危険なのは「片方が学び続けて日々成長してるのに、片方が現状維持(=衰退)」という場合で、長期的に見ると破綻に向かう可能性があります。
+「類は友を呼ぶ」と言いますが、それが最も顕著に現れるのは"頭脳レベル"なんです。
+人間関係を大切にしつつも、一方で、
+「孤独な時間を徹底的に確保し、頭脳を磨き、思考を深めること」は怠ってはいけないと思ってます。自戒も込めて。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>タブー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>同程度の頭脳レベル同士</t>
+    <rPh sb="0" eb="3">
+      <t>ドウテイド</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ズノウ</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ドウシ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>夫婦関係</t>
+    <rPh sb="0" eb="2">
+      <t>フウフ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンケイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>長期的な関係</t>
+    <rPh sb="0" eb="3">
+      <t>チョウキテキ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>カンケイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>危険</t>
+    <rPh sb="0" eb="2">
+      <t>キケン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>片方</t>
+    <rPh sb="0" eb="2">
+      <t>カタホウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>学び</t>
+    <rPh sb="0" eb="1">
+      <t>マナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>日々</t>
+    <rPh sb="0" eb="2">
+      <t>ヒビ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>成長</t>
+    <rPh sb="0" eb="2">
+      <t>セイチョウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>現状維持</t>
+    <rPh sb="0" eb="2">
+      <t>ゲンジョウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>イジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>衰退</t>
+    <rPh sb="0" eb="2">
+      <t>スイタイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>長期的</t>
+    <rPh sb="0" eb="3">
+      <t>チョウキテキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>破綻</t>
+    <rPh sb="0" eb="2">
+      <t>ハタン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>可能性</t>
+    <rPh sb="0" eb="3">
+      <t>カノウセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>類は友を呼ぶ</t>
+    <rPh sb="0" eb="1">
+      <t>ルイ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>トモ</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>ヨ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>顕著</t>
+    <rPh sb="0" eb="2">
+      <t>ケンチョ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>頭脳レベル</t>
+    <rPh sb="0" eb="2">
+      <t>ズノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人間関係</t>
+    <rPh sb="0" eb="2">
+      <t>ニンゲン</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>カンケイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>大切</t>
+    <rPh sb="0" eb="2">
+      <t>タイセツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>一方</t>
+    <rPh sb="0" eb="2">
+      <t>イッポウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>孤独な時間</t>
+    <rPh sb="0" eb="2">
+      <t>コドク</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>ジカン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>徹底的</t>
+    <rPh sb="0" eb="3">
+      <t>テッテイテキ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>確保</t>
+    <rPh sb="0" eb="2">
+      <t>カクホ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>頭脳</t>
+    <rPh sb="0" eb="2">
+      <t>ズノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>磨く</t>
+    <rPh sb="0" eb="1">
+      <t>ミガ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>思考</t>
+    <rPh sb="0" eb="2">
+      <t>シコウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>深める</t>
+    <rPh sb="0" eb="1">
+      <t>フカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>怠ってはいけない</t>
+    <rPh sb="0" eb="1">
+      <t>オコタ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自戒</t>
+    <rPh sb="0" eb="2">
+      <t>ジカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>あえてタブーに触れるが、夫婦関係などの長期的な関係において「同程度の頭脳レベル同士」であることは残酷なほど大切だ。片方だけが日々の学びで成長し、もう一方が現状維持を選べば、それは実質的な衰退。長期的に見れば関係の破綻は顕著になる。類は友を呼ぶは真理。孤独な時間を確保し、徹底的に思考を深めることのできる相手か。そこを妥協して急ってはいけない。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人間関係の破綻を恐れるな。日々の学びで頭脳を磨くことは、時に孤独な時間を増やす。だが、それで離れていくなら同程度の頭脳レベルではなかったというだけのこと。思考を深めることを放棄した相手との現状維持は、自分の可能性を殺すのと同じだ。徹底的に自戒し、成長を選べ。長期的に隣に残るのは、同じ速度で走れる人間だけだ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>夫婦関係の危険なサインは、喧嘩ではなく「話が通じなくなる」ことだ。片方が学び続け、もう一方が思考を止めた時、関係の破綻は静かに始まる。同程度の頭脳レベル同士でしか見えない景色がある。孤独な時間を確保してでも頭脳を磨くこと。それが長期的な関係を守る唯一の方法であり、最大の自戒だ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/hirakawa_noter/status/1992227017249722609</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ひらかわ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>有料note1記事で5年半ご飯食べています。
+Joined March 2025</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「煽って一瞬売れる」と「売れ続ける」には圧倒的な差があります。
+・1つの有料記事
+・超ニッチな分野
+・5年間販売継続
+・煽りなし
+たった1本のnoteだけでこれまで8,000万円分を手に取ってもらうために実践してきた内容をまとめてみました。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自分がこれまでnote運営してきた経験を解説したり、note運営者さんにインタビューするメンバーシップも始めてみました。
+ワンコインでいつでも入会・退会OKなので、ゆるっと覗いてみてください。
+https://note.com/hirakawa_noter/membership</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自分</t>
+    <rPh sb="0" eb="2">
+      <t>ジブン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>note</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>運営</t>
+    <rPh sb="0" eb="2">
+      <t>ウンエイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>解説</t>
+    <rPh sb="0" eb="2">
+      <t>カイセツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>note運営者</t>
+    <rPh sb="4" eb="7">
+      <t>ウンエイシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>インタビュー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>メンバーシップ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ワンコイン</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>入会</t>
+    <rPh sb="0" eb="2">
+      <t>ニュウカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>退会</t>
+    <rPh sb="0" eb="2">
+      <t>タイカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>OK</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ゆるっと</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>覗いて</t>
+    <rPh sb="0" eb="1">
+      <t>ノゾ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「noteの運営って孤独すぎる」と感じたので、自分の経験やノウハウを全部公開するメンバーシップを作りました。
+難しい解説やインタビューはありません。 あるのは、日々のリアルな運営記録と、失敗の共有だけ。
+缶コーヒー1本分（ワンコイン以下）の月額100円です。 入会も退会も自由（OK）なので、まずはゆるっと、無料部分だけでも覗いてみてください。 https://note.com/kanta0930/membership</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Webアプリ「自分株式会社」の開発日記を始めます。
+機能実装の裏側、数字の分析、デザインの迷い……。 完成品ではなく、自分が経験する「未完成の過程」をnoteで垂れ流します。
+これは僕の運営日誌であり、あなたの挑戦のヒントになるかもしれない実験記録。 月額100円で、このドキュメンタリーの証人になってくれませんか？ https://note.com/kanta0930/membership</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自分の経験をコンテンツにする実験。 note運営の裏側や開発日記を、月額100円のメンバーシップで公開し始めました。
+高尚なノウハウより、泥臭い経験談の方が役に立つと信じて。 入会も退会もOK。ゆるっとやってます。 https://note.com/kanta0930/membership</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>いいね</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>◎</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>一時間に5つ。やりたくないけどすべきことを思考停止してやる。それを記録する</t>
+    <rPh sb="0" eb="1">
+      <t>イチ</t>
+    </rPh>
+    <rPh sb="1" eb="3">
+      <t>ジカン</t>
+    </rPh>
+    <rPh sb="21" eb="23">
+      <t>シコウ</t>
+    </rPh>
+    <rPh sb="23" eb="25">
+      <t>テイシ</t>
+    </rPh>
+    <rPh sb="33" eb="35">
+      <t>キロク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>パスタを茹でる</t>
+    <rPh sb="4" eb="5">
+      <t>ユ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>お湯を沸かす</t>
+    <rPh sb="1" eb="2">
+      <t>ユ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>ワ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>日本国記</t>
+    <rPh sb="0" eb="2">
+      <t>ニホン</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>コク</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>キ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>〇</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>やるということでしかやる気はでない。とにかく思考停止して手を動かす</t>
+    <rPh sb="12" eb="13">
+      <t>キ</t>
+    </rPh>
+    <rPh sb="22" eb="24">
+      <t>シコウ</t>
+    </rPh>
+    <rPh sb="24" eb="26">
+      <t>テイシ</t>
+    </rPh>
+    <rPh sb="28" eb="29">
+      <t>テ</t>
+    </rPh>
+    <rPh sb="30" eb="31">
+      <t>ウゴ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -3268,12 +4514,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -3289,7 +4541,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -3300,6 +4552,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
@@ -3621,7 +4877,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -3804,7 +5060,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -4017,7 +5273,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -4193,7 +5449,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -7739,7 +8995,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8219,6 +9475,1827 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
+  <sheetPr filterMode="1">
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
+  <dimension ref="C2:Q117"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="67.875" customWidth="1"/>
+    <col min="6" max="6" width="59.625" customWidth="1"/>
+    <col min="7" max="7" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="54.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="48.375" customWidth="1"/>
+    <col min="11" max="11" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:17">
+      <c r="D2" t="s">
+        <v>660</v>
+      </c>
+      <c r="F2" t="s">
+        <v>635</v>
+      </c>
+      <c r="I2" t="s">
+        <v>677</v>
+      </c>
+      <c r="K2" t="s">
+        <v>674</v>
+      </c>
+      <c r="L2" t="s">
+        <v>675</v>
+      </c>
+      <c r="M2" t="s">
+        <v>678</v>
+      </c>
+      <c r="N2" t="s">
+        <v>674</v>
+      </c>
+      <c r="O2" t="s">
+        <v>675</v>
+      </c>
+      <c r="P2" t="s">
+        <v>678</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="3" spans="3:17" ht="93.75" hidden="1">
+      <c r="C3" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="D3" t="s">
+        <v>631</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="4" spans="3:17" ht="150">
+      <c r="F4" s="1" t="s">
+        <v>634</v>
+      </c>
+      <c r="G4" s="3">
+        <v>46066</v>
+      </c>
+      <c r="H4" t="s">
+        <v>636</v>
+      </c>
+      <c r="I4" t="s">
+        <v>676</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>655</v>
+      </c>
+      <c r="K4" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L4">
+        <v>31</v>
+      </c>
+      <c r="M4">
+        <v>3642</v>
+      </c>
+      <c r="N4" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O4">
+        <v>42</v>
+      </c>
+      <c r="P4">
+        <v>3639</v>
+      </c>
+      <c r="Q4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="3:17" ht="225">
+      <c r="H5" t="s">
+        <v>637</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="K5" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L5">
+        <v>19</v>
+      </c>
+      <c r="M5">
+        <v>3642</v>
+      </c>
+      <c r="N5" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O5">
+        <v>33</v>
+      </c>
+      <c r="P5">
+        <v>3639</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="3:17" ht="75">
+      <c r="H6" t="s">
+        <v>638</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="K6" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L6">
+        <v>18</v>
+      </c>
+      <c r="M6">
+        <v>3642</v>
+      </c>
+      <c r="N6" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O6">
+        <v>29</v>
+      </c>
+      <c r="P6">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="7" spans="3:17" hidden="1">
+      <c r="H7" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="8" spans="3:17" hidden="1">
+      <c r="H8" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="9" spans="3:17" hidden="1">
+      <c r="H9" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="10" spans="3:17" hidden="1">
+      <c r="H10" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="11" spans="3:17" hidden="1">
+      <c r="H11" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="12" spans="3:17" hidden="1">
+      <c r="H12" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="13" spans="3:17" hidden="1">
+      <c r="H13" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="14" spans="3:17" hidden="1">
+      <c r="H14" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="15" spans="3:17" hidden="1">
+      <c r="H15" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="16" spans="3:17" hidden="1">
+      <c r="H16" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="17" spans="3:16" hidden="1">
+      <c r="H17" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="18" spans="3:16" hidden="1">
+      <c r="H18" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="19" spans="3:16" hidden="1">
+      <c r="H19" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="20" spans="3:16" hidden="1">
+      <c r="H20" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="21" spans="3:16" hidden="1">
+      <c r="H21" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="22" spans="3:16" hidden="1">
+      <c r="H22" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="23" spans="3:16" ht="112.5" hidden="1">
+      <c r="C23" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="D23" t="s">
+        <v>659</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>661</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="24" spans="3:16" ht="131.25">
+      <c r="F24" s="1" t="s">
+        <v>663</v>
+      </c>
+      <c r="G24" s="3">
+        <v>46066</v>
+      </c>
+      <c r="H24" t="s">
+        <v>664</v>
+      </c>
+      <c r="I24" t="s">
+        <v>676</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="K24" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L24">
+        <v>26</v>
+      </c>
+      <c r="M24">
+        <v>3642</v>
+      </c>
+      <c r="N24" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O24">
+        <v>35</v>
+      </c>
+      <c r="P24">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="25" spans="3:16" ht="281.25">
+      <c r="H25" t="s">
+        <v>665</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="K25" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L25">
+        <v>24</v>
+      </c>
+      <c r="M25">
+        <v>3642</v>
+      </c>
+      <c r="N25" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O25">
+        <v>32</v>
+      </c>
+      <c r="P25">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="26" spans="3:16" ht="112.5">
+      <c r="H26" t="s">
+        <v>666</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="K26" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L26">
+        <v>28</v>
+      </c>
+      <c r="M26">
+        <v>3642</v>
+      </c>
+      <c r="N26" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O26">
+        <v>36</v>
+      </c>
+      <c r="P26">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="27" spans="3:16" hidden="1">
+      <c r="H27" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="28" spans="3:16" hidden="1">
+      <c r="H28" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="29" spans="3:16" hidden="1">
+      <c r="H29" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="30" spans="3:16" hidden="1">
+      <c r="H30" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="31" spans="3:16" hidden="1">
+      <c r="H31" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="32" spans="3:16" hidden="1">
+      <c r="H32" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="33" spans="3:16" hidden="1">
+      <c r="H33" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="34" spans="3:16" ht="112.5" hidden="1">
+      <c r="C34" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="D34" t="s">
+        <v>683</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="35" spans="3:16" ht="206.25">
+      <c r="F35" s="1" t="s">
+        <v>686</v>
+      </c>
+      <c r="G35" s="3">
+        <v>46066</v>
+      </c>
+      <c r="H35" t="s">
+        <v>687</v>
+      </c>
+      <c r="I35" t="s">
+        <v>676</v>
+      </c>
+      <c r="J35" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="K35" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L35">
+        <v>16</v>
+      </c>
+      <c r="M35">
+        <v>3642</v>
+      </c>
+      <c r="N35" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O35">
+        <v>25</v>
+      </c>
+      <c r="P35">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="36" spans="3:16" ht="131.25">
+      <c r="H36" t="s">
+        <v>688</v>
+      </c>
+      <c r="J36" s="1" t="s">
+        <v>711</v>
+      </c>
+      <c r="K36" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L36">
+        <v>28</v>
+      </c>
+      <c r="M36">
+        <v>3642</v>
+      </c>
+      <c r="N36" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O36">
+        <v>42</v>
+      </c>
+      <c r="P36">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="37" spans="3:16" ht="112.5">
+      <c r="H37" t="s">
+        <v>689</v>
+      </c>
+      <c r="J37" s="1" t="s">
+        <v>712</v>
+      </c>
+      <c r="K37" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L37">
+        <v>17</v>
+      </c>
+      <c r="M37">
+        <v>3642</v>
+      </c>
+      <c r="N37" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O37">
+        <v>27</v>
+      </c>
+      <c r="P37">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="38" spans="3:16" hidden="1">
+      <c r="H38" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="39" spans="3:16" hidden="1">
+      <c r="H39" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="40" spans="3:16" hidden="1">
+      <c r="H40" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="41" spans="3:16" hidden="1">
+      <c r="H41" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="42" spans="3:16" hidden="1">
+      <c r="H42" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="43" spans="3:16" hidden="1">
+      <c r="H43" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="44" spans="3:16" hidden="1">
+      <c r="H44" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="45" spans="3:16" hidden="1">
+      <c r="H45" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="46" spans="3:16" hidden="1">
+      <c r="H46" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="47" spans="3:16" hidden="1">
+      <c r="H47" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="48" spans="3:16" hidden="1">
+      <c r="H48" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="49" spans="3:16" hidden="1">
+      <c r="H49" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="50" spans="3:16" hidden="1">
+      <c r="H50" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="51" spans="3:16" hidden="1">
+      <c r="H51" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="52" spans="3:16" hidden="1">
+      <c r="H52" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="53" spans="3:16" hidden="1">
+      <c r="H53" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="54" spans="3:16" hidden="1">
+      <c r="H54" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="55" spans="3:16" hidden="1">
+      <c r="H55" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="56" spans="3:16" hidden="1">
+      <c r="H56" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="57" spans="3:16" hidden="1">
+      <c r="H57" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="58" spans="3:16" ht="409.5" hidden="1">
+      <c r="C58" s="2" t="s">
+        <v>713</v>
+      </c>
+      <c r="D58" t="s">
+        <v>714</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>715</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="59" spans="3:16" ht="187.5">
+      <c r="F59" s="1" t="s">
+        <v>717</v>
+      </c>
+      <c r="G59" s="3">
+        <v>46066</v>
+      </c>
+      <c r="H59" t="s">
+        <v>718</v>
+      </c>
+      <c r="I59" t="s">
+        <v>676</v>
+      </c>
+      <c r="J59" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="K59" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L59">
+        <v>13</v>
+      </c>
+      <c r="M59">
+        <v>3642</v>
+      </c>
+      <c r="N59" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O59">
+        <v>25</v>
+      </c>
+      <c r="P59">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="60" spans="3:16" ht="225">
+      <c r="H60" t="s">
+        <v>719</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>733</v>
+      </c>
+      <c r="K60" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L60">
+        <v>16</v>
+      </c>
+      <c r="M60">
+        <v>3642</v>
+      </c>
+      <c r="N60" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O60">
+        <v>27</v>
+      </c>
+      <c r="P60">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="61" spans="3:16" ht="112.5">
+      <c r="H61" t="s">
+        <v>720</v>
+      </c>
+      <c r="J61" s="1" t="s">
+        <v>734</v>
+      </c>
+      <c r="K61" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L61">
+        <v>13</v>
+      </c>
+      <c r="M61">
+        <v>3642</v>
+      </c>
+      <c r="N61" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O61">
+        <v>24</v>
+      </c>
+      <c r="P61">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="62" spans="3:16" hidden="1">
+      <c r="H62" t="s">
+        <v>721</v>
+      </c>
+      <c r="J62" s="1"/>
+    </row>
+    <row r="63" spans="3:16" hidden="1">
+      <c r="H63" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="64" spans="3:16" hidden="1">
+      <c r="H64" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="65" spans="3:16" hidden="1">
+      <c r="H65" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="66" spans="3:16" hidden="1">
+      <c r="H66" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="67" spans="3:16" hidden="1">
+      <c r="H67" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="68" spans="3:16" hidden="1">
+      <c r="H68" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="69" spans="3:16" hidden="1">
+      <c r="H69" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="70" spans="3:16" hidden="1">
+      <c r="H70" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="71" spans="3:16" hidden="1">
+      <c r="H71" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="72" spans="3:16" hidden="1">
+      <c r="H72" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="73" spans="3:16" ht="409.5" hidden="1">
+      <c r="C73" s="2" t="s">
+        <v>735</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>736</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>737</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="74" spans="3:16" ht="281.25">
+      <c r="F74" s="1" t="s">
+        <v>739</v>
+      </c>
+      <c r="G74" s="3">
+        <v>46066</v>
+      </c>
+      <c r="H74" t="s">
+        <v>740</v>
+      </c>
+      <c r="I74" t="s">
+        <v>676</v>
+      </c>
+      <c r="J74" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="K74" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L74">
+        <v>17</v>
+      </c>
+      <c r="M74">
+        <v>3642</v>
+      </c>
+      <c r="N74" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O74">
+        <v>32</v>
+      </c>
+      <c r="P74">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="75" spans="3:16" ht="131.25">
+      <c r="H75" t="s">
+        <v>741</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="K75" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L75">
+        <v>11</v>
+      </c>
+      <c r="M75">
+        <v>3642</v>
+      </c>
+      <c r="N75" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O75">
+        <v>23</v>
+      </c>
+      <c r="P75">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="76" spans="3:16" ht="112.5">
+      <c r="H76" t="s">
+        <v>742</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="K76" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L76">
+        <v>15</v>
+      </c>
+      <c r="M76">
+        <v>3642</v>
+      </c>
+      <c r="N76" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O76">
+        <v>29</v>
+      </c>
+      <c r="P76">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="77" spans="3:16" hidden="1">
+      <c r="H77" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="78" spans="3:16" hidden="1">
+      <c r="H78" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="79" spans="3:16" hidden="1">
+      <c r="H79" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="80" spans="3:16" hidden="1">
+      <c r="H80" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="81" spans="8:8" hidden="1">
+      <c r="H81" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="82" spans="8:8" hidden="1">
+      <c r="H82" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="83" spans="8:8" hidden="1">
+      <c r="H83" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="84" spans="8:8" hidden="1">
+      <c r="H84" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="85" spans="8:8" hidden="1">
+      <c r="H85" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="86" spans="8:8" hidden="1">
+      <c r="H86" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="87" spans="8:8" hidden="1">
+      <c r="H87" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="88" spans="8:8" hidden="1">
+      <c r="H88" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="89" spans="8:8" hidden="1">
+      <c r="H89" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="90" spans="8:8" hidden="1">
+      <c r="H90" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="91" spans="8:8" hidden="1">
+      <c r="H91" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="92" spans="8:8" hidden="1">
+      <c r="H92" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="93" spans="8:8" hidden="1">
+      <c r="H93" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="94" spans="8:8" hidden="1">
+      <c r="H94" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="95" spans="8:8" hidden="1">
+      <c r="H95" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="96" spans="8:8" hidden="1">
+      <c r="H96" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="97" spans="3:16" hidden="1">
+      <c r="H97" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="98" spans="3:16" hidden="1">
+      <c r="H98" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="99" spans="3:16" hidden="1">
+      <c r="H99" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="100" spans="3:16" hidden="1">
+      <c r="H100" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="101" spans="3:16" hidden="1">
+      <c r="H101" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="102" spans="3:16" hidden="1">
+      <c r="H102" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="103" spans="3:16" ht="168.75" hidden="1">
+      <c r="C103" s="2" t="s">
+        <v>772</v>
+      </c>
+      <c r="D103" t="s">
+        <v>773</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>774</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="104" spans="3:16" ht="206.25">
+      <c r="F104" s="1" t="s">
+        <v>776</v>
+      </c>
+      <c r="G104" s="3">
+        <v>46066</v>
+      </c>
+      <c r="H104" t="s">
+        <v>777</v>
+      </c>
+      <c r="I104" t="s">
+        <v>676</v>
+      </c>
+      <c r="J104" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="K104" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L104">
+        <v>3</v>
+      </c>
+      <c r="M104">
+        <v>3642</v>
+      </c>
+      <c r="N104" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O104">
+        <v>23</v>
+      </c>
+      <c r="P104">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="105" spans="3:16" ht="187.5">
+      <c r="H105" t="s">
+        <v>778</v>
+      </c>
+      <c r="J105" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="K105" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L105">
+        <v>3</v>
+      </c>
+      <c r="M105">
+        <v>3642</v>
+      </c>
+      <c r="N105" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O105">
+        <v>33</v>
+      </c>
+      <c r="P105">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="106" spans="3:16" ht="131.25">
+      <c r="H106" t="s">
+        <v>779</v>
+      </c>
+      <c r="J106" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="K106" s="3">
+        <v>46066</v>
+      </c>
+      <c r="L106">
+        <v>3</v>
+      </c>
+      <c r="M106">
+        <v>3642</v>
+      </c>
+      <c r="N106" s="3">
+        <v>46067</v>
+      </c>
+      <c r="O106">
+        <v>20</v>
+      </c>
+      <c r="P106">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="107" spans="3:16" hidden="1">
+      <c r="H107" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="108" spans="3:16" hidden="1">
+      <c r="H108" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="109" spans="3:16" hidden="1">
+      <c r="H109" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="110" spans="3:16" hidden="1">
+      <c r="H110" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="111" spans="3:16" hidden="1">
+      <c r="H111" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="112" spans="3:16" hidden="1">
+      <c r="H112" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="113" spans="8:8" hidden="1">
+      <c r="H113" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="114" spans="8:8" hidden="1">
+      <c r="H114" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="115" spans="8:8" hidden="1">
+      <c r="H115" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="116" spans="8:8" hidden="1">
+      <c r="H116" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="117" spans="8:8" hidden="1">
+      <c r="H117" t="s">
+        <v>789</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="C2:M117" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
+    <filterColumn colId="8">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{C897C6D6-16A8-4618-9776-831A651C49AE}"/>
+    <hyperlink ref="C23" r:id="rId2" xr:uid="{BE504C4C-F69D-4324-A180-161A02DAC9DC}"/>
+    <hyperlink ref="C34" r:id="rId3" xr:uid="{BD19965A-B265-4188-8708-2E5B80BD19AB}"/>
+    <hyperlink ref="C58" r:id="rId4" xr:uid="{25990352-46B9-4C85-982A-98F73BBB9104}"/>
+    <hyperlink ref="C73" r:id="rId5" xr:uid="{AE1289EC-5E13-44B2-914C-DD143CE7FDD9}"/>
+    <hyperlink ref="D73" r:id="rId6" xr:uid="{0D4EEA7C-455E-45DF-A93D-F93B0AFD534B}"/>
+    <hyperlink ref="C103" r:id="rId7" xr:uid="{9EA14625-33D5-4EF7-8F21-0B01E5AFD468}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970790C5-0376-420E-A317-55DF989D7F43}">
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr defaultColWidth="73.25" defaultRowHeight="18.75"/>
+  <cols>
+    <col min="1" max="1" width="77.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="B1" t="s">
+        <v>674</v>
+      </c>
+      <c r="C1" t="s">
+        <v>675</v>
+      </c>
+      <c r="D1" t="s">
+        <v>678</v>
+      </c>
+      <c r="E1" t="s">
+        <v>674</v>
+      </c>
+      <c r="F1" t="s">
+        <v>675</v>
+      </c>
+      <c r="G1" t="s">
+        <v>678</v>
+      </c>
+      <c r="H1" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="93.75">
+      <c r="A2" s="1" t="s">
+        <v>792</v>
+      </c>
+      <c r="B2" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>3642</v>
+      </c>
+      <c r="E2" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F2">
+        <v>20</v>
+      </c>
+      <c r="G2">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="75">
+      <c r="A3" s="1" t="s">
+        <v>770</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C3">
+        <v>11</v>
+      </c>
+      <c r="D3">
+        <v>3642</v>
+      </c>
+      <c r="E3" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F3">
+        <v>23</v>
+      </c>
+      <c r="G3">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="168.75">
+      <c r="A4" s="1" t="s">
+        <v>790</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>3642</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F4">
+        <v>23</v>
+      </c>
+      <c r="G4">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="75">
+      <c r="A5" s="1" t="s">
+        <v>734</v>
+      </c>
+      <c r="B5" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C5">
+        <v>13</v>
+      </c>
+      <c r="D5">
+        <v>3642</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F5">
+        <v>24</v>
+      </c>
+      <c r="G5">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="93.75">
+      <c r="A6" s="1" t="s">
+        <v>710</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <v>3642</v>
+      </c>
+      <c r="E6" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F6">
+        <v>25</v>
+      </c>
+      <c r="G6">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="93.75">
+      <c r="A7" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C7">
+        <v>13</v>
+      </c>
+      <c r="D7">
+        <v>3642</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F7">
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="75">
+      <c r="A8" s="1" t="s">
+        <v>712</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C8">
+        <v>17</v>
+      </c>
+      <c r="D8">
+        <v>3642</v>
+      </c>
+      <c r="E8" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F8">
+        <v>27</v>
+      </c>
+      <c r="G8">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="187.5">
+      <c r="A9" s="1" t="s">
+        <v>733</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C9">
+        <v>16</v>
+      </c>
+      <c r="D9">
+        <v>3642</v>
+      </c>
+      <c r="E9" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F9">
+        <v>27</v>
+      </c>
+      <c r="G9">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="56.25">
+      <c r="A10" s="1" t="s">
+        <v>657</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C10">
+        <v>18</v>
+      </c>
+      <c r="D10">
+        <v>3642</v>
+      </c>
+      <c r="E10" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F10">
+        <v>29</v>
+      </c>
+      <c r="G10">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="75">
+      <c r="A11" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C11">
+        <v>15</v>
+      </c>
+      <c r="D11">
+        <v>3642</v>
+      </c>
+      <c r="E11" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F11">
+        <v>29</v>
+      </c>
+      <c r="G11">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="262.5">
+      <c r="A12" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C12">
+        <v>24</v>
+      </c>
+      <c r="D12">
+        <v>3642</v>
+      </c>
+      <c r="E12" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F12">
+        <v>32</v>
+      </c>
+      <c r="G12">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="93.75">
+      <c r="A13" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="B13" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C13">
+        <v>17</v>
+      </c>
+      <c r="D13">
+        <v>3642</v>
+      </c>
+      <c r="E13" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F13">
+        <v>32</v>
+      </c>
+      <c r="G13">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="206.25">
+      <c r="A14" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B14" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C14">
+        <v>19</v>
+      </c>
+      <c r="D14">
+        <v>3642</v>
+      </c>
+      <c r="E14" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F14">
+        <v>33</v>
+      </c>
+      <c r="G14">
+        <v>3639</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="150">
+      <c r="A15" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="B15" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C15">
+        <v>3</v>
+      </c>
+      <c r="D15">
+        <v>3642</v>
+      </c>
+      <c r="E15" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F15">
+        <v>33</v>
+      </c>
+      <c r="G15">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="75">
+      <c r="A16" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="B16" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C16">
+        <v>26</v>
+      </c>
+      <c r="D16">
+        <v>3642</v>
+      </c>
+      <c r="E16" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F16">
+        <v>35</v>
+      </c>
+      <c r="G16">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="75">
+      <c r="A17" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="B17" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C17">
+        <v>28</v>
+      </c>
+      <c r="D17">
+        <v>3642</v>
+      </c>
+      <c r="E17" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F17">
+        <v>36</v>
+      </c>
+      <c r="G17">
+        <v>3639</v>
+      </c>
+      <c r="I17" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="56.25">
+      <c r="A18" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="B18" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C18">
+        <v>31</v>
+      </c>
+      <c r="D18">
+        <v>3642</v>
+      </c>
+      <c r="E18" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F18">
+        <v>42</v>
+      </c>
+      <c r="G18">
+        <v>3639</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="75">
+      <c r="A19" s="6" t="s">
+        <v>711</v>
+      </c>
+      <c r="B19" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C19">
+        <v>28</v>
+      </c>
+      <c r="D19">
+        <v>3642</v>
+      </c>
+      <c r="E19" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F19">
+        <v>42</v>
+      </c>
+      <c r="G19">
+        <v>3639</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H19">
+    <sortCondition ref="F2:F19"/>
+  </sortState>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CEE3D6-6F68-4B25-8FF2-FA5306076EAF}">
+  <dimension ref="B2:I34"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9">
+      <c r="C2" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="3" spans="2:9">
+      <c r="C3" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9">
+      <c r="B5" s="3"/>
+      <c r="D5" s="3">
+        <v>46067</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46068</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3">
+        <v>46069</v>
+      </c>
+      <c r="H5" s="3">
+        <v>46070</v>
+      </c>
+      <c r="I5" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9">
+      <c r="C6" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9">
+      <c r="C7" s="7">
+        <v>4.1666666666666664E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9">
+      <c r="C8" s="7">
+        <v>8.3333333333333301E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9">
+      <c r="C9" s="7">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9">
+      <c r="C10" s="7">
+        <v>0.16666666666666699</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9">
+      <c r="C11" s="7">
+        <v>0.20833333333333301</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9">
+      <c r="C12" s="7">
+        <v>0.25</v>
+      </c>
+      <c r="E12" t="s">
+        <v>797</v>
+      </c>
+      <c r="F12" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9">
+      <c r="C13" s="7"/>
+      <c r="E13" t="s">
+        <v>796</v>
+      </c>
+      <c r="F13" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9">
+      <c r="C14" s="7"/>
+      <c r="E14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9">
+      <c r="C15" s="7"/>
+      <c r="E15" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9">
+      <c r="C16" s="7"/>
+      <c r="E16" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" s="7">
+        <v>0.29166666666666702</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3">
+      <c r="C18" s="7">
+        <v>0.33333333333333298</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3">
+      <c r="C19" s="7">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3">
+      <c r="C20" s="7">
+        <v>0.41666666666666702</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3">
+      <c r="C21" s="7">
+        <v>0.45833333333333298</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3">
+      <c r="C22" s="7">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3">
+      <c r="C23" s="7">
+        <v>0.54166666666666696</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3">
+      <c r="C24" s="7">
+        <v>0.58333333333333304</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3">
+      <c r="C25" s="7">
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="26" spans="3:3">
+      <c r="C26" s="7">
+        <v>0.66666666666666696</v>
+      </c>
+    </row>
+    <row r="27" spans="3:3">
+      <c r="C27" s="7">
+        <v>0.70833333333333304</v>
+      </c>
+    </row>
+    <row r="28" spans="3:3">
+      <c r="C28" s="7">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="29" spans="3:3">
+      <c r="C29" s="7">
+        <v>0.79166666666666696</v>
+      </c>
+    </row>
+    <row r="30" spans="3:3">
+      <c r="C30" s="7">
+        <v>0.83333333333333304</v>
+      </c>
+    </row>
+    <row r="31" spans="3:3">
+      <c r="C31" s="7">
+        <v>0.875</v>
+      </c>
+    </row>
+    <row r="32" spans="3:3">
+      <c r="C32" s="7">
+        <v>0.91666666666666696</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3">
+      <c r="C33" s="7">
+        <v>0.95833333333333304</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3">
+      <c r="C34" s="7"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2804FBA8-A624-4312-90D5-A46193547956}">
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
@@ -8234,7 +11311,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -8427,300 +11504,6 @@
     <hyperlink ref="B6" r:id="rId4" display="https://developers.google.com/gemini-code-assist/docs/overview" xr:uid="{D4606693-ABC6-4C4C-8030-AFF9956F016B}"/>
     <hyperlink ref="B2" r:id="rId5" xr:uid="{F2F2C855-BA2E-4DBF-BDB7-B571F8EBFB8B}"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D01CB6-001D-4D20-8CBB-FE510A056DBA}">
-  <sheetPr>
-    <tabColor rgb="FF00B0F0"/>
-  </sheetPr>
-  <dimension ref="B1:E16"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
-  <cols>
-    <col min="2" max="2" width="45.125" customWidth="1"/>
-    <col min="3" max="3" width="59.5" customWidth="1"/>
-    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="2:5">
-      <c r="E1" s="3">
-        <f ca="1">TODAY()</f>
-        <v>46064</v>
-      </c>
-    </row>
-    <row r="2" spans="2:5">
-      <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="2:5">
-      <c r="B3" s="5" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5">
-      <c r="B4" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5">
-      <c r="B5" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5">
-      <c r="B6" s="5" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5">
-      <c r="B8" s="1" t="s">
-        <v>528</v>
-      </c>
-      <c r="C8" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5">
-      <c r="B9" t="s">
-        <v>530</v>
-      </c>
-      <c r="C9" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" ht="37.5">
-      <c r="B10" s="1" t="s">
-        <v>532</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="11" spans="2:5" ht="37.5">
-      <c r="B11" s="1" t="s">
-        <v>534</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>535</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" ht="75">
-      <c r="B12" s="1" t="s">
-        <v>536</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>537</v>
-      </c>
-    </row>
-    <row r="13" spans="2:5" ht="37.5">
-      <c r="B13" s="1" t="s">
-        <v>538</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="14" spans="2:5" ht="75">
-      <c r="B14" s="1" t="s">
-        <v>540</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>541</v>
-      </c>
-      <c r="E14" s="3">
-        <v>46043</v>
-      </c>
-    </row>
-    <row r="15" spans="2:5" ht="56.25">
-      <c r="B15" s="1" t="s">
-        <v>542</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>543</v>
-      </c>
-      <c r="E15" s="3">
-        <v>46043</v>
-      </c>
-    </row>
-    <row r="16" spans="2:5" ht="37.5">
-      <c r="B16" s="1" t="s">
-        <v>588</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>589</v>
-      </c>
-      <c r="E16" s="3">
-        <v>46050</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" display="https://developers.google.com/" xr:uid="{AB4DF198-4467-43BD-92E5-7F9CEA77AE2D}"/>
-    <hyperlink ref="B4" r:id="rId2" display="https://developers.google.com/products" xr:uid="{E0788B1D-CD47-4B9D-A222-F399F4097EB5}"/>
-    <hyperlink ref="B5" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{59048891-D360-4985-8E21-C2F762568942}"/>
-    <hyperlink ref="B6" r:id="rId4" display="https://developers.google.com/gemini-code-assist/resources/faqs" xr:uid="{B8E91675-F28D-4503-9C6B-4A96AC1B988B}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595742A4-FD4B-4501-B5BA-63CBD2F36625}">
-  <sheetPr>
-    <tabColor rgb="FFFF0000"/>
-  </sheetPr>
-  <dimension ref="C2:D9"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
-  <cols>
-    <col min="3" max="3" width="43.25" customWidth="1"/>
-    <col min="4" max="4" width="48.375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="3:4">
-      <c r="C2" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="4" spans="3:4">
-      <c r="C4" t="s">
-        <v>311</v>
-      </c>
-      <c r="D4" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="6" spans="3:4" ht="37.5">
-      <c r="C6" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="7" spans="3:4" ht="37.5">
-      <c r="C7" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="8" spans="3:4" ht="112.5">
-      <c r="C8" s="1" t="s">
-        <v>570</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="9" spans="3:4" ht="56.25">
-      <c r="C9" s="1" t="s">
-        <v>592</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>593</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{2D572F08-FF13-4D66-AD9B-8810B4A82168}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
-  <dimension ref="C3:E9"/>
-  <sheetFormatPr defaultRowHeight="18.75"/>
-  <cols>
-    <col min="3" max="3" width="31.625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="94" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="3:5" ht="206.25">
-      <c r="C3" t="s">
-        <v>91</v>
-      </c>
-      <c r="D3" t="s">
-        <v>92</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="4" spans="3:5" ht="150">
-      <c r="C4" t="s">
-        <v>94</v>
-      </c>
-      <c r="D4" t="s">
-        <v>96</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="3:5" ht="300">
-      <c r="C5" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="3:5" ht="409.5">
-      <c r="C6" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" t="s">
-        <v>113</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="7" spans="3:5" ht="409.5">
-      <c r="C7" t="s">
-        <v>115</v>
-      </c>
-      <c r="D7" t="s">
-        <v>116</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="3:5" ht="262.5">
-      <c r="C8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="9" spans="3:5" ht="131.25">
-      <c r="C9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -8892,6 +11675,300 @@
       </c>
       <c r="C20" s="1" t="s">
         <v>585</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D01CB6-001D-4D20-8CBB-FE510A056DBA}">
+  <sheetPr>
+    <tabColor rgb="FF00B0F0"/>
+  </sheetPr>
+  <dimension ref="B1:E16"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="2" max="2" width="45.125" customWidth="1"/>
+    <col min="3" max="3" width="59.5" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:5">
+      <c r="E1" s="3">
+        <f ca="1">TODAY()</f>
+        <v>46068</v>
+      </c>
+    </row>
+    <row r="2" spans="2:5">
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="2:5">
+      <c r="B3" s="5" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="5" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="C8" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" t="s">
+        <v>530</v>
+      </c>
+      <c r="C9" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="37.5">
+      <c r="B10" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="37.5">
+      <c r="B11" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="75">
+      <c r="B12" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5" ht="37.5">
+      <c r="B13" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5" ht="75">
+      <c r="B14" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="E14" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5" ht="56.25">
+      <c r="B15" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="E15" s="3">
+        <v>46043</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" ht="37.5">
+      <c r="B16" s="1" t="s">
+        <v>588</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>589</v>
+      </c>
+      <c r="E16" s="3">
+        <v>46050</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" display="https://developers.google.com/" xr:uid="{AB4DF198-4467-43BD-92E5-7F9CEA77AE2D}"/>
+    <hyperlink ref="B4" r:id="rId2" display="https://developers.google.com/products" xr:uid="{E0788B1D-CD47-4B9D-A222-F399F4097EB5}"/>
+    <hyperlink ref="B5" r:id="rId3" display="https://developers.google.com/gemini-code-assist" xr:uid="{59048891-D360-4985-8E21-C2F762568942}"/>
+    <hyperlink ref="B6" r:id="rId4" display="https://developers.google.com/gemini-code-assist/resources/faqs" xr:uid="{B8E91675-F28D-4503-9C6B-4A96AC1B988B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595742A4-FD4B-4501-B5BA-63CBD2F36625}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="C2:D9"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="3" max="3" width="43.25" customWidth="1"/>
+    <col min="4" max="4" width="48.375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:4">
+      <c r="C2" s="2" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="4" spans="3:4">
+      <c r="C4" t="s">
+        <v>311</v>
+      </c>
+      <c r="D4" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" ht="37.5">
+      <c r="C6" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" ht="37.5">
+      <c r="C7" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" ht="112.5">
+      <c r="C8" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" ht="56.25">
+      <c r="C9" s="1" t="s">
+        <v>592</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>593</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{2D572F08-FF13-4D66-AD9B-8810B4A82168}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
+  <dimension ref="C3:E9"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
+  <cols>
+    <col min="3" max="3" width="31.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="94" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:5" ht="206.25">
+      <c r="C3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="3:5" ht="150">
+      <c r="C4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="3:5" ht="300">
+      <c r="C5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="3:5" ht="409.5">
+      <c r="C6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="7" spans="3:5" ht="409.5">
+      <c r="C7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="3:5" ht="262.5">
+      <c r="C8" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="9" spans="3:5" ht="131.25">
+      <c r="C9" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -9268,7 +12345,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46064</v>
+        <v>46068</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
feat: integrate Supabase for asset management and update KPI summary with total assets
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D325D140-8163-4EFE-BFC6-F3770CD05214}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C48EE9B-EB5A-4AF6-89F9-52AA45091B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="17" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="801">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1455" uniqueCount="868">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -4465,6 +4465,531 @@
     <rPh sb="30" eb="31">
       <t>ウゴ</t>
     </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/genmai_tokyo/status/2021783281461866788</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>玄米</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">会社売却2回・事業売却1回。30代。AI×プロダクトの設計・実装、ヘルスケア、IPまわり。個人でハンズオン投資。拠点は日本と東南アジア。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>🗼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Joined December 2025</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>玄米の自己紹介｜2回のExitと売却前提の事業づくり</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>【本を読む技術】
+海外でバズってる記事。読書が苦手な方はこれマスト。
+脳が情報収集に最適化されすぎてて、「本を読んだのに、何も身についていない気がする」という体感ある人多いと思う。
+ニュースをAIに要約させ、わかった気になる。情報を知れても理解には至らない。はい図星。
+誰もがアクセスできる「情報」に価値はなく、そこから自分だけの「理解」を抽出できるかどうか。本を読む技術をマスターしよう。
+要約
+1. 「情報」vs「理解」
+単なる情報収集を超え、著者の思考の骨格を見抜き、自分の言葉で批判的に再構築できる状態（= 理解）を目指すべき。
+2. 戦略的な「点検読書」
+1ページ目から読み始めるのは非効率。目次から、本全体の構造を把握する予習が大事。
+3. アイデアを戦わせる「シントピカル読書」
+一冊に心酔するのではなく、同じテーマの複数冊を読み比べる。著者同士を脳内で対話させ、矛盾や共通点から自分なりの答えを導き出す。これこそが理解を生み出すプロセス。
+4. 社会的な帰結
+複雑な社会は、判断力を失い、感情的な操作に屈しやすくなる。読書術を磨くことは、個人の知性を高めるだけでなく、判断力を守ることと同義である。
+詳しい方法は全文翻訳がおすすめ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>読む</t>
+    <rPh sb="0" eb="1">
+      <t>ヨ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>技術</t>
+    <rPh sb="0" eb="2">
+      <t>ギジュツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>海外</t>
+    <rPh sb="0" eb="2">
+      <t>カイガイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>バズっている記事</t>
+    <rPh sb="6" eb="8">
+      <t>キジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>読書</t>
+    <rPh sb="0" eb="2">
+      <t>ドクショ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>苦手</t>
+    <rPh sb="0" eb="2">
+      <t>ニガテ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>マスト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>脳</t>
+    <rPh sb="0" eb="1">
+      <t>ノウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>情報収集</t>
+    <rPh sb="0" eb="2">
+      <t>ジョウホウ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>シュウシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最適化</t>
+    <rPh sb="0" eb="3">
+      <t>サイテキカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>本を読んだ</t>
+    <rPh sb="0" eb="1">
+      <t>ホン</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ヨ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>何も身についていない</t>
+    <rPh sb="0" eb="1">
+      <t>ナニ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ミ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ニュース</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>AI</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>わかった気</t>
+    <rPh sb="4" eb="5">
+      <t>キ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>情報</t>
+    <rPh sb="0" eb="2">
+      <t>ジョウホウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>理解</t>
+    <rPh sb="0" eb="2">
+      <t>リカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>図星</t>
+    <rPh sb="0" eb="2">
+      <t>ズボシ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>誰もがアクセスできる</t>
+    <rPh sb="0" eb="1">
+      <t>ダレ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>価値</t>
+    <rPh sb="0" eb="2">
+      <t>カチ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>抽出</t>
+    <rPh sb="0" eb="2">
+      <t>チュウシュツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>本を読む技術</t>
+    <rPh sb="0" eb="1">
+      <t>ホン</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ヨ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ギジュツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>マスター</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「情報」vs「理解」</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>著者の思考の骨格</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>批判的</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>再構築</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>戦略的な「点検読書」</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1ページ目</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>非効率</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>目次</t>
+    <rPh sb="0" eb="2">
+      <t>モクジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>本全体の構造</t>
+    <rPh sb="0" eb="1">
+      <t>ホン</t>
+    </rPh>
+    <rPh sb="1" eb="3">
+      <t>ゼンタイ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>コウゾウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>把握</t>
+    <rPh sb="0" eb="2">
+      <t>ハアク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>予習</t>
+    <rPh sb="0" eb="2">
+      <t>ヨシュウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>大事</t>
+    <rPh sb="0" eb="2">
+      <t>ダイジ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>アイデア</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>シントピカル読書</t>
+    <rPh sb="6" eb="8">
+      <t>ドクショ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1冊</t>
+    <rPh sb="1" eb="2">
+      <t>サツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>心酔</t>
+    <rPh sb="0" eb="2">
+      <t>シンスイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>同じテーマ</t>
+    <rPh sb="0" eb="1">
+      <t>オナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>複数冊</t>
+    <rPh sb="0" eb="2">
+      <t>フクスウ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>サツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>著者</t>
+    <rPh sb="0" eb="2">
+      <t>チョシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>脳内</t>
+    <rPh sb="0" eb="2">
+      <t>ノウナイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>対話</t>
+    <rPh sb="0" eb="2">
+      <t>タイワ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>矛盾</t>
+    <rPh sb="0" eb="2">
+      <t>ムジュン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>共通点</t>
+    <rPh sb="0" eb="3">
+      <t>キョウツウテン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>自分なり</t>
+    <rPh sb="0" eb="2">
+      <t>ジブン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>答え</t>
+    <rPh sb="0" eb="1">
+      <t>コタ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>導き出す</t>
+    <rPh sb="0" eb="1">
+      <t>ミチビ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ダ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>プロセス</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>社会的な帰結</t>
+    <rPh sb="0" eb="3">
+      <t>シャカイテキ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>キケツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>複雑な社会</t>
+    <rPh sb="0" eb="2">
+      <t>フクザツ</t>
+    </rPh>
+    <rPh sb="3" eb="5">
+      <t>シャカイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>判断力</t>
+    <rPh sb="0" eb="2">
+      <t>ハンダン</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>リョク</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>感情的な操作</t>
+    <rPh sb="0" eb="3">
+      <t>カンジョウテキ</t>
+    </rPh>
+    <rPh sb="4" eb="6">
+      <t>ソウサ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>読書術</t>
+    <rPh sb="0" eb="2">
+      <t>ドクショ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>ジュツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>知性</t>
+    <rPh sb="0" eb="2">
+      <t>チセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>判断力を守る</t>
+    <rPh sb="0" eb="3">
+      <t>ハンダンリョク</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>マモ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>同義</t>
+    <rPh sb="0" eb="2">
+      <t>ドウギ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>このキーワードを使ってバズるポストを考えてください。Xでバズる方法としては以下を参考にしてください。
+目に入った人がどうしても一言コメントしたくなるような文章にしてください。コメント、リポスト、引用リポストおよび、ポスト滞在時間がインプレッションを増やすために必要です。</t>
+    <rPh sb="31" eb="33">
+      <t>ホウホウ</t>
+    </rPh>
+    <rPh sb="37" eb="39">
+      <t>イカ</t>
+    </rPh>
+    <rPh sb="40" eb="42">
+      <t>サンコウ</t>
+    </rPh>
+    <rPh sb="52" eb="53">
+      <t>メ</t>
+    </rPh>
+    <rPh sb="54" eb="55">
+      <t>ハイ</t>
+    </rPh>
+    <rPh sb="57" eb="58">
+      <t>ヒト</t>
+    </rPh>
+    <rPh sb="64" eb="66">
+      <t>ヒトコト</t>
+    </rPh>
+    <rPh sb="78" eb="80">
+      <t>ブンショウ</t>
+    </rPh>
+    <rPh sb="98" eb="100">
+      <t>インヨウ</t>
+    </rPh>
+    <rPh sb="111" eb="113">
+      <t>タイザイ</t>
+    </rPh>
+    <rPh sb="113" eb="115">
+      <t>ジカン</t>
+    </rPh>
+    <rPh sb="125" eb="126">
+      <t>フ</t>
+    </rPh>
+    <rPh sb="131" eb="133">
+      <t>ヒツヨウ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>あえて言いますが、AIの要約を読んで「わかった気」になるのは、知的な自殺行為に等しい。 情報は誰でもアクセスできる時代。そこにあるのは単なる「データ」であって「理解」じゃない。 非効率に見える1ページ目からの通読、著者との脳内対話、そこから生まれる矛盾への違和感。このプロセスを飛ばして得た答えに、何の価値がある？ 判断力を守るために、あえて苦手な本を読め。「情報」を喰うな、「知性」を磨け。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>本を1冊読んで信じ込むのは危険だ。 本当に知性を磨きたいなら、同じテーマの本を複数冊読み、脳内で著者同士を戦わせろ（シントピカル読書）。 A氏の主張とB氏の主張、その矛盾と共通点を見つけ、自分なりの答えを導き出す。 AIが抽出した「正解っぽいもの」を受け入れるな。情報を再構築し、自分の脳で批判的に検証する。それが、この複雑な社会で騙されないための唯一の技術だ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「情報」と「理解」は同義じゃない。 スマホでニュースを見るのは「情報収集」。 苦手な本と格闘し、著者の思考の骨格を自分なりに再構築するのが「読書」。 AIに要約させて効率化したつもりになるな。手間と時間をかけたプロセスの中にしか、本物の判断力は宿らない。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -9476,10 +10001,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="C2:Q117"/>
+  <dimension ref="C2:Q178"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
@@ -9529,7 +10054,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="3" spans="3:17" ht="93.75" hidden="1">
+    <row r="3" spans="3:17" ht="93.75">
       <c r="C3" s="2" t="s">
         <v>630</v>
       </c>
@@ -9636,87 +10161,87 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="7" spans="3:17" hidden="1">
+    <row r="7" spans="3:17">
       <c r="H7" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="8" spans="3:17" hidden="1">
+    <row r="8" spans="3:17">
       <c r="H8" t="s">
         <v>640</v>
       </c>
     </row>
-    <row r="9" spans="3:17" hidden="1">
+    <row r="9" spans="3:17">
       <c r="H9" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="10" spans="3:17" hidden="1">
+    <row r="10" spans="3:17">
       <c r="H10" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="11" spans="3:17" hidden="1">
+    <row r="11" spans="3:17">
       <c r="H11" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="12" spans="3:17" hidden="1">
+    <row r="12" spans="3:17">
       <c r="H12" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="13" spans="3:17" hidden="1">
+    <row r="13" spans="3:17">
       <c r="H13" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="14" spans="3:17" hidden="1">
+    <row r="14" spans="3:17">
       <c r="H14" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="15" spans="3:17" hidden="1">
+    <row r="15" spans="3:17">
       <c r="H15" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="16" spans="3:17" hidden="1">
+    <row r="16" spans="3:17">
       <c r="H16" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="17" spans="3:16" hidden="1">
+    <row r="17" spans="3:16">
       <c r="H17" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="18" spans="3:16" hidden="1">
+    <row r="18" spans="3:16">
       <c r="H18" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="19" spans="3:16" hidden="1">
+    <row r="19" spans="3:16">
       <c r="H19" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="20" spans="3:16" hidden="1">
+    <row r="20" spans="3:16">
       <c r="H20" t="s">
         <v>652</v>
       </c>
     </row>
-    <row r="21" spans="3:16" hidden="1">
+    <row r="21" spans="3:16">
       <c r="H21" t="s">
         <v>653</v>
       </c>
     </row>
-    <row r="22" spans="3:16" hidden="1">
+    <row r="22" spans="3:16">
       <c r="H22" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="23" spans="3:16" ht="112.5" hidden="1">
+    <row r="23" spans="3:16" ht="112.5">
       <c r="C23" s="2" t="s">
         <v>658</v>
       </c>
@@ -9817,42 +10342,42 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="27" spans="3:16" hidden="1">
+    <row r="27" spans="3:16">
       <c r="H27" t="s">
         <v>667</v>
       </c>
     </row>
-    <row r="28" spans="3:16" hidden="1">
+    <row r="28" spans="3:16">
       <c r="H28" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="29" spans="3:16" hidden="1">
+    <row r="29" spans="3:16">
       <c r="H29" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="30" spans="3:16" hidden="1">
+    <row r="30" spans="3:16">
       <c r="H30" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="31" spans="3:16" hidden="1">
+    <row r="31" spans="3:16">
       <c r="H31" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="32" spans="3:16" hidden="1">
+    <row r="32" spans="3:16">
       <c r="H32" t="s">
         <v>672</v>
       </c>
     </row>
-    <row r="33" spans="3:16" hidden="1">
+    <row r="33" spans="3:16">
       <c r="H33" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="34" spans="3:16" ht="112.5" hidden="1">
+    <row r="34" spans="3:16" ht="112.5">
       <c r="C34" s="2" t="s">
         <v>682</v>
       </c>
@@ -9953,107 +10478,107 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="38" spans="3:16" hidden="1">
+    <row r="38" spans="3:16">
       <c r="H38" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="39" spans="3:16" hidden="1">
+    <row r="39" spans="3:16">
       <c r="H39" t="s">
         <v>691</v>
       </c>
     </row>
-    <row r="40" spans="3:16" hidden="1">
+    <row r="40" spans="3:16">
       <c r="H40" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="41" spans="3:16" hidden="1">
+    <row r="41" spans="3:16">
       <c r="H41" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="42" spans="3:16" hidden="1">
+    <row r="42" spans="3:16">
       <c r="H42" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="43" spans="3:16" hidden="1">
+    <row r="43" spans="3:16">
       <c r="H43" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="44" spans="3:16" hidden="1">
+    <row r="44" spans="3:16">
       <c r="H44" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="45" spans="3:16" hidden="1">
+    <row r="45" spans="3:16">
       <c r="H45" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="46" spans="3:16" hidden="1">
+    <row r="46" spans="3:16">
       <c r="H46" t="s">
         <v>698</v>
       </c>
     </row>
-    <row r="47" spans="3:16" hidden="1">
+    <row r="47" spans="3:16">
       <c r="H47" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="48" spans="3:16" hidden="1">
+    <row r="48" spans="3:16">
       <c r="H48" t="s">
         <v>700</v>
       </c>
     </row>
-    <row r="49" spans="3:16" hidden="1">
+    <row r="49" spans="3:16">
       <c r="H49" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="50" spans="3:16" hidden="1">
+    <row r="50" spans="3:16">
       <c r="H50" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="51" spans="3:16" hidden="1">
+    <row r="51" spans="3:16">
       <c r="H51" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="52" spans="3:16" hidden="1">
+    <row r="52" spans="3:16">
       <c r="H52" t="s">
         <v>704</v>
       </c>
     </row>
-    <row r="53" spans="3:16" hidden="1">
+    <row r="53" spans="3:16">
       <c r="H53" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="54" spans="3:16" hidden="1">
+    <row r="54" spans="3:16">
       <c r="H54" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="55" spans="3:16" hidden="1">
+    <row r="55" spans="3:16">
       <c r="H55" t="s">
         <v>707</v>
       </c>
     </row>
-    <row r="56" spans="3:16" hidden="1">
+    <row r="56" spans="3:16">
       <c r="H56" t="s">
         <v>708</v>
       </c>
     </row>
-    <row r="57" spans="3:16" hidden="1">
+    <row r="57" spans="3:16">
       <c r="H57" t="s">
         <v>709</v>
       </c>
     </row>
-    <row r="58" spans="3:16" ht="409.5" hidden="1">
+    <row r="58" spans="3:16" ht="409.5">
       <c r="C58" s="2" t="s">
         <v>713</v>
       </c>
@@ -10154,63 +10679,63 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="62" spans="3:16" hidden="1">
+    <row r="62" spans="3:16">
       <c r="H62" t="s">
         <v>721</v>
       </c>
       <c r="J62" s="1"/>
     </row>
-    <row r="63" spans="3:16" hidden="1">
+    <row r="63" spans="3:16">
       <c r="H63" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="64" spans="3:16" hidden="1">
+    <row r="64" spans="3:16">
       <c r="H64" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="65" spans="3:16" hidden="1">
+    <row r="65" spans="3:16">
       <c r="H65" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="66" spans="3:16" hidden="1">
+    <row r="66" spans="3:16">
       <c r="H66" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="67" spans="3:16" hidden="1">
+    <row r="67" spans="3:16">
       <c r="H67" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="68" spans="3:16" hidden="1">
+    <row r="68" spans="3:16">
       <c r="H68" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="69" spans="3:16" hidden="1">
+    <row r="69" spans="3:16">
       <c r="H69" t="s">
         <v>728</v>
       </c>
     </row>
-    <row r="70" spans="3:16" hidden="1">
+    <row r="70" spans="3:16">
       <c r="H70" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="71" spans="3:16" hidden="1">
+    <row r="71" spans="3:16">
       <c r="H71" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="72" spans="3:16" hidden="1">
+    <row r="72" spans="3:16">
       <c r="H72" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="73" spans="3:16" ht="409.5" hidden="1">
+    <row r="73" spans="3:16" ht="409.5">
       <c r="C73" s="2" t="s">
         <v>735</v>
       </c>
@@ -10311,137 +10836,137 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="77" spans="3:16" hidden="1">
+    <row r="77" spans="3:16">
       <c r="H77" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="78" spans="3:16" hidden="1">
+    <row r="78" spans="3:16">
       <c r="H78" t="s">
         <v>744</v>
       </c>
     </row>
-    <row r="79" spans="3:16" hidden="1">
+    <row r="79" spans="3:16">
       <c r="H79" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="80" spans="3:16" hidden="1">
+    <row r="80" spans="3:16">
       <c r="H80" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="81" spans="8:8" hidden="1">
+    <row r="81" spans="8:8">
       <c r="H81" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="82" spans="8:8" hidden="1">
+    <row r="82" spans="8:8">
       <c r="H82" t="s">
         <v>748</v>
       </c>
     </row>
-    <row r="83" spans="8:8" hidden="1">
+    <row r="83" spans="8:8">
       <c r="H83" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="84" spans="8:8" hidden="1">
+    <row r="84" spans="8:8">
       <c r="H84" t="s">
         <v>750</v>
       </c>
     </row>
-    <row r="85" spans="8:8" hidden="1">
+    <row r="85" spans="8:8">
       <c r="H85" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="86" spans="8:8" hidden="1">
+    <row r="86" spans="8:8">
       <c r="H86" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="87" spans="8:8" hidden="1">
+    <row r="87" spans="8:8">
       <c r="H87" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="88" spans="8:8" hidden="1">
+    <row r="88" spans="8:8">
       <c r="H88" t="s">
         <v>754</v>
       </c>
     </row>
-    <row r="89" spans="8:8" hidden="1">
+    <row r="89" spans="8:8">
       <c r="H89" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="90" spans="8:8" hidden="1">
+    <row r="90" spans="8:8">
       <c r="H90" t="s">
         <v>756</v>
       </c>
     </row>
-    <row r="91" spans="8:8" hidden="1">
+    <row r="91" spans="8:8">
       <c r="H91" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="92" spans="8:8" hidden="1">
+    <row r="92" spans="8:8">
       <c r="H92" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="93" spans="8:8" hidden="1">
+    <row r="93" spans="8:8">
       <c r="H93" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="94" spans="8:8" hidden="1">
+    <row r="94" spans="8:8">
       <c r="H94" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="95" spans="8:8" hidden="1">
+    <row r="95" spans="8:8">
       <c r="H95" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="96" spans="8:8" hidden="1">
+    <row r="96" spans="8:8">
       <c r="H96" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="97" spans="3:16" hidden="1">
+    <row r="97" spans="3:16">
       <c r="H97" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="98" spans="3:16" hidden="1">
+    <row r="98" spans="3:16">
       <c r="H98" t="s">
         <v>764</v>
       </c>
     </row>
-    <row r="99" spans="3:16" hidden="1">
+    <row r="99" spans="3:16">
       <c r="H99" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="100" spans="3:16" hidden="1">
+    <row r="100" spans="3:16">
       <c r="H100" t="s">
         <v>766</v>
       </c>
     </row>
-    <row r="101" spans="3:16" hidden="1">
+    <row r="101" spans="3:16">
       <c r="H101" t="s">
         <v>767</v>
       </c>
     </row>
-    <row r="102" spans="3:16" hidden="1">
+    <row r="102" spans="3:16">
       <c r="H102" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="103" spans="3:16" ht="168.75" hidden="1">
+    <row r="103" spans="3:16" ht="168.75">
       <c r="C103" s="2" t="s">
         <v>772</v>
       </c>
@@ -10542,69 +11067,422 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="107" spans="3:16" hidden="1">
+    <row r="107" spans="3:16">
       <c r="H107" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="108" spans="3:16" hidden="1">
+    <row r="108" spans="3:16">
       <c r="H108" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="109" spans="3:16" hidden="1">
+    <row r="109" spans="3:16">
       <c r="H109" t="s">
         <v>781</v>
       </c>
     </row>
-    <row r="110" spans="3:16" hidden="1">
+    <row r="110" spans="3:16">
       <c r="H110" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="111" spans="3:16" hidden="1">
+    <row r="111" spans="3:16">
       <c r="H111" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="112" spans="3:16" hidden="1">
+    <row r="112" spans="3:16">
       <c r="H112" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="113" spans="8:8" hidden="1">
+    <row r="113" spans="3:13">
       <c r="H113" t="s">
         <v>785</v>
       </c>
     </row>
-    <row r="114" spans="8:8" hidden="1">
+    <row r="114" spans="3:13">
       <c r="H114" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="115" spans="8:8" hidden="1">
+    <row r="115" spans="3:13">
       <c r="H115" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="116" spans="8:8" hidden="1">
+    <row r="116" spans="3:13">
       <c r="H116" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="117" spans="8:8" hidden="1">
+    <row r="117" spans="3:13">
       <c r="H117" t="s">
         <v>789</v>
       </c>
     </row>
+    <row r="118" spans="3:13" ht="75">
+      <c r="C118" s="2" t="s">
+        <v>801</v>
+      </c>
+      <c r="D118" t="s">
+        <v>802</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>803</v>
+      </c>
+      <c r="F118" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="119" spans="3:13" ht="409.5">
+      <c r="F119" s="1" t="s">
+        <v>805</v>
+      </c>
+      <c r="G119" s="3">
+        <v>46068</v>
+      </c>
+      <c r="H119" t="s">
+        <v>642</v>
+      </c>
+      <c r="I119" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="J119" s="1" t="s">
+        <v>865</v>
+      </c>
+      <c r="K119" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L119">
+        <v>2</v>
+      </c>
+      <c r="M119">
+        <v>3640</v>
+      </c>
+    </row>
+    <row r="120" spans="3:13" ht="150">
+      <c r="H120" t="s">
+        <v>806</v>
+      </c>
+      <c r="J120" s="1" t="s">
+        <v>866</v>
+      </c>
+      <c r="K120" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L120">
+        <v>3</v>
+      </c>
+      <c r="M120">
+        <v>3640</v>
+      </c>
+    </row>
+    <row r="121" spans="3:13" ht="93.75">
+      <c r="H121" t="s">
+        <v>807</v>
+      </c>
+      <c r="J121" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="K121" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L121">
+        <v>7</v>
+      </c>
+      <c r="M121">
+        <v>3640</v>
+      </c>
+    </row>
+    <row r="122" spans="3:13">
+      <c r="H122" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="123" spans="3:13">
+      <c r="H123" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="124" spans="3:13">
+      <c r="H124" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="125" spans="3:13">
+      <c r="H125" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="126" spans="3:13">
+      <c r="H126" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="127" spans="3:13">
+      <c r="H127" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="128" spans="3:13">
+      <c r="H128" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="129" spans="8:8">
+      <c r="H129" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="130" spans="8:8">
+      <c r="H130" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="131" spans="8:8">
+      <c r="H131" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="132" spans="8:8">
+      <c r="H132" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="133" spans="8:8">
+      <c r="H133" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="134" spans="8:8">
+      <c r="H134" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="135" spans="8:8">
+      <c r="H135" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="136" spans="8:8">
+      <c r="H136" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="137" spans="8:8">
+      <c r="H137" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="138" spans="8:8">
+      <c r="H138" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="139" spans="8:8">
+      <c r="H139" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="140" spans="8:8">
+      <c r="H140" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="141" spans="8:8">
+      <c r="H141" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="142" spans="8:8">
+      <c r="H142" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="143" spans="8:8">
+      <c r="H143" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="144" spans="8:8">
+      <c r="H144" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="145" spans="8:8">
+      <c r="H145" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="146" spans="8:8">
+      <c r="H146" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="147" spans="8:8">
+      <c r="H147" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="148" spans="8:8">
+      <c r="H148" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="149" spans="8:8">
+      <c r="H149" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="150" spans="8:8">
+      <c r="H150" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="151" spans="8:8">
+      <c r="H151" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="152" spans="8:8">
+      <c r="H152" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="153" spans="8:8">
+      <c r="H153" t="s">
+        <v>838</v>
+      </c>
+    </row>
+    <row r="154" spans="8:8">
+      <c r="H154" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="155" spans="8:8">
+      <c r="H155" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="156" spans="8:8">
+      <c r="H156" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="157" spans="8:8">
+      <c r="H157" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="158" spans="8:8">
+      <c r="H158" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="159" spans="8:8">
+      <c r="H159" t="s">
+        <v>844</v>
+      </c>
+    </row>
+    <row r="160" spans="8:8">
+      <c r="H160" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="161" spans="8:8">
+      <c r="H161" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="162" spans="8:8">
+      <c r="H162" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="163" spans="8:8">
+      <c r="H163" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="164" spans="8:8">
+      <c r="H164" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="165" spans="8:8">
+      <c r="H165" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="166" spans="8:8">
+      <c r="H166" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="167" spans="8:8">
+      <c r="H167" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="168" spans="8:8">
+      <c r="H168" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="169" spans="8:8">
+      <c r="H169" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="170" spans="8:8">
+      <c r="H170" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="171" spans="8:8">
+      <c r="H171" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="172" spans="8:8">
+      <c r="H172" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="173" spans="8:8">
+      <c r="H173" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="174" spans="8:8">
+      <c r="H174" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="175" spans="8:8">
+      <c r="H175" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="176" spans="8:8">
+      <c r="H176" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="177" spans="8:8">
+      <c r="H177" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="178" spans="8:8">
+      <c r="H178" t="s">
+        <v>863</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="C2:M117" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
-    <filterColumn colId="8">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="C2:M117" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}"/>
   <phoneticPr fontId="1"/>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" xr:uid="{C897C6D6-16A8-4618-9776-831A651C49AE}"/>
@@ -10614,6 +11492,7 @@
     <hyperlink ref="C73" r:id="rId5" xr:uid="{AE1289EC-5E13-44B2-914C-DD143CE7FDD9}"/>
     <hyperlink ref="D73" r:id="rId6" xr:uid="{0D4EEA7C-455E-45DF-A93D-F93B0AFD534B}"/>
     <hyperlink ref="C103" r:id="rId7" xr:uid="{9EA14625-33D5-4EF7-8F21-0B01E5AFD468}"/>
+    <hyperlink ref="C118" r:id="rId8" xr:uid="{CF96628D-0F57-4F99-94C8-6E77305F553D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11081,6 +11960,9 @@
       </c>
       <c r="G19">
         <v>3639</v>
+      </c>
+      <c r="I19" t="s">
+        <v>794</v>
       </c>
     </row>
   </sheetData>
@@ -11193,6 +12075,9 @@
       <c r="C15" s="7"/>
       <c r="E15" t="s">
         <v>45</v>
+      </c>
+      <c r="F15" t="s">
+        <v>799</v>
       </c>
     </row>
     <row r="16" spans="2:9">

</xml_diff>

<commit_message>
feat: add chart display mode toggle and legend for asset management
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C48EE9B-EB5A-4AF6-89F9-52AA45091B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0214F12-5E2C-48D5-8977-84E1157DC91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1455" uniqueCount="868">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="895">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -4990,6 +4990,178 @@
   </si>
   <si>
     <t>「情報」と「理解」は同義じゃない。 スマホでニュースを見るのは「情報収集」。 苦手な本と格闘し、著者の思考の骨格を自分なりに再構築するのが「読書」。 AIに要約させて効率化したつもりになるな。手間と時間をかけたプロセスの中にしか、本物の判断力は宿らない。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/naikoutetsugaku/status/2022868444484636714</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>内向哲学</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>中の人
+@yumaevo
+｜「読んだ人の思考,視点,知恵を深化する」を軸に、内向的な人に向けた人生戦略を発信しています。
+note.com/yumaevo
+Joined October 2025</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>地頭の良さとは「構造を見抜く力」だとぼくは思います。
+構造を見抜く力というのは、義務教育ではなかなか教われない「物事の本質を掴む力」であり、頭いい人に共通する力でもあります。
+構造把握能力を強化するためには、一体どうすればいいのでしょうか。
+解説しました↓</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>頭がいい人とは「孤独でいられる人」のこと</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>XにArticleを投稿したいです。下記を参考にバズるArticleの文面を考えてください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/kanta13jp1/status/2022918189710217415</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/kanta13jp1/status/2022919786657681574</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/kanta13jp1/status/2022920488784400571</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/jungo_FanMarke/status/2022885834572337545</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>じゅんご</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>賢い生き方が学べる｜副業、ビジネス、独立の考え方が学べる｜人間関係が上手くいくコツ｜フォローすると人生にやる気が出る｜メンタルマネジメント｜経営歴25年｜全て経験談と本音｜ 著書『60%の力でうまいこと結果を出す思考100』をKADOKAWAより出版
+Entrepreneur↓著書「60%の力でうまいこと結果を出す思考100」amazon.co.jp/dp/4046056002?…Born March 23
+Joined June 2018
+1,623 Following
+140.3K Followers</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>起業して25年。1000人以上の、起業家や経営車と、話して感じる共通点は○○○です。これがある人は、どんな業種でも結果を出す。その考え方とは…今夜2/15の21時から90分間。zoomセミナー『稼ぐマインドの作り方』を開催します。参加費は1000円です。アーカイブのみの購入も1000円で可能です。参加希望の方はDM下さい。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>覚えておいて。人間関係で気をつけたいことは、「相手に尽くし過ぎないこと」です。最初は感謝されても、やってくれることに慣れてくると、雑に扱われるので要注意。人という生き物は、最初は感謝していても、慣れてきて当たり前になると、やってくれないとイライラしたりする。人間関係を良好にしたいなら、都合の良い人認定だけは、されてはいけない。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>気をつけたいこと</t>
+    <rPh sb="0" eb="1">
+      <t>キ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>相手に尽くし過ぎないこと</t>
+    <rPh sb="0" eb="2">
+      <t>アイテ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>ツ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>ス</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最初</t>
+    <rPh sb="0" eb="2">
+      <t>サイショ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>感謝</t>
+    <rPh sb="0" eb="2">
+      <t>カンシャ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>慣れてくる</t>
+    <rPh sb="0" eb="1">
+      <t>ナ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>雑に扱われる</t>
+    <rPh sb="0" eb="1">
+      <t>ザツ</t>
+    </rPh>
+    <rPh sb="2" eb="3">
+      <t>アツカ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>要注意</t>
+    <rPh sb="0" eb="3">
+      <t>ヨウチュウイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人という生き物</t>
+    <rPh sb="0" eb="1">
+      <t>ヒト</t>
+    </rPh>
+    <rPh sb="4" eb="5">
+      <t>イ</t>
+    </rPh>
+    <rPh sb="6" eb="7">
+      <t>モノ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>イライラ</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>都合の良い人認定</t>
+    <rPh sb="0" eb="2">
+      <t>ツゴウ</t>
+    </rPh>
+    <rPh sb="3" eb="4">
+      <t>ヨ</t>
+    </rPh>
+    <rPh sb="5" eb="6">
+      <t>ヒト</t>
+    </rPh>
+    <rPh sb="6" eb="8">
+      <t>ニンテイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人間関係で一番気をつけたいこと。 最初は「ありがとう」と感謝されていたのに、尽くし過ぎると相手はそれが「日常」になり、次第に「慣れて」くる。 そして最終的には、やらないと「なんでやってくれないの？」とイライラされ、雑に扱われるようになる。
+これが「都合の良い人認定」されるまでの黄金ルート。 人という生き物は、与えられすぎると感謝を忘れるバグがある。 最初から100点で飛ばすな。60点でいろ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>「相手に尽くし過ぎないこと」。 これは冷たさではなく、自衛のための必須スキルです。
+悲しいけど、人という生き物は「無償の愛」を注ぎ続けると、それを「安売り」だと勘違いして雑に扱ってくる生き物です。 最初は感謝されても、慣れてくればただの「便利な人」。 尽くせば愛されるなんて幻想です。 自分の価値を守るために、あえて「やらない」という選択肢を持ってください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>人間関係の教訓。 「最初」に頑張りすぎると、後で絶対に自分が苦しくなる。 相手はあなたの優しさに「慣れ」、感謝は消え、要求だけがエスカレートする。 そして気づけば「都合の良い人」に認定完了。 イライラしたくないなら、適度な距離感と「断る勇気」を最初から見せておくこと。 自分を安売りしない人が、結局一番大切にされる。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -10004,7 +10176,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="C2:Q178"/>
+  <dimension ref="C2:Q194"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
@@ -10014,7 +10186,7 @@
     <col min="7" max="7" width="10.25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="54.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="48.375" customWidth="1"/>
+    <col min="10" max="10" width="52.5" customWidth="1"/>
     <col min="11" max="11" width="10.25" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="17.125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="10.25" bestFit="1" customWidth="1"/>
@@ -11156,7 +11328,7 @@
         <v>46068</v>
       </c>
       <c r="L119">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="M119">
         <v>3640</v>
@@ -11173,7 +11345,7 @@
         <v>46068</v>
       </c>
       <c r="L120">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="M120">
         <v>3640</v>
@@ -11190,7 +11362,7 @@
         <v>46068</v>
       </c>
       <c r="L121">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="M121">
         <v>3640</v>
@@ -11471,14 +11643,190 @@
         <v>861</v>
       </c>
     </row>
-    <row r="177" spans="8:8">
+    <row r="177" spans="3:13">
       <c r="H177" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="178" spans="8:8">
+    <row r="178" spans="3:13">
       <c r="H178" t="s">
         <v>863</v>
+      </c>
+    </row>
+    <row r="179" spans="3:13" ht="168.75">
+      <c r="C179" s="2" t="s">
+        <v>868</v>
+      </c>
+      <c r="D179" t="s">
+        <v>869</v>
+      </c>
+      <c r="E179" s="1" t="s">
+        <v>870</v>
+      </c>
+      <c r="F179" s="1" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="180" spans="3:13" ht="37.5">
+      <c r="F180" t="s">
+        <v>872</v>
+      </c>
+      <c r="G180" s="3">
+        <v>46068</v>
+      </c>
+      <c r="I180" s="1" t="s">
+        <v>873</v>
+      </c>
+      <c r="J180" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="K180" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L180">
+        <v>6</v>
+      </c>
+      <c r="M180">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="181" spans="3:13">
+      <c r="J181" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="K181" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L181">
+        <v>8</v>
+      </c>
+      <c r="M181">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="182" spans="3:13">
+      <c r="J182" s="2" t="s">
+        <v>876</v>
+      </c>
+      <c r="K182" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L182">
+        <v>5</v>
+      </c>
+      <c r="M182">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="183" spans="3:13" ht="168.75">
+      <c r="C183" s="2" t="s">
+        <v>877</v>
+      </c>
+      <c r="D183" t="s">
+        <v>878</v>
+      </c>
+      <c r="E183" s="1" t="s">
+        <v>879</v>
+      </c>
+      <c r="F183" s="1" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="184" spans="3:13" ht="168.75">
+      <c r="F184" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="H184" t="s">
+        <v>757</v>
+      </c>
+      <c r="I184" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="J184" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="K184" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L184">
+        <v>8</v>
+      </c>
+      <c r="M184">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="185" spans="3:13" ht="168.75">
+      <c r="H185" t="s">
+        <v>882</v>
+      </c>
+      <c r="J185" s="1" t="s">
+        <v>893</v>
+      </c>
+      <c r="K185" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L185">
+        <v>3</v>
+      </c>
+      <c r="M185">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="186" spans="3:13" ht="112.5">
+      <c r="H186" t="s">
+        <v>883</v>
+      </c>
+      <c r="J186" s="1" t="s">
+        <v>894</v>
+      </c>
+      <c r="K186" s="3">
+        <v>46068</v>
+      </c>
+      <c r="L186">
+        <v>1</v>
+      </c>
+      <c r="M186">
+        <v>3639</v>
+      </c>
+    </row>
+    <row r="187" spans="3:13">
+      <c r="H187" t="s">
+        <v>884</v>
+      </c>
+    </row>
+    <row r="188" spans="3:13">
+      <c r="H188" t="s">
+        <v>885</v>
+      </c>
+    </row>
+    <row r="189" spans="3:13">
+      <c r="H189" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="190" spans="3:13">
+      <c r="H190" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="191" spans="3:13">
+      <c r="H191" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="192" spans="3:13">
+      <c r="H192" t="s">
+        <v>889</v>
+      </c>
+    </row>
+    <row r="193" spans="8:8">
+      <c r="H193" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="194" spans="8:8">
+      <c r="H194" t="s">
+        <v>891</v>
       </c>
     </row>
   </sheetData>
@@ -11493,6 +11841,11 @@
     <hyperlink ref="D73" r:id="rId6" xr:uid="{0D4EEA7C-455E-45DF-A93D-F93B0AFD534B}"/>
     <hyperlink ref="C103" r:id="rId7" xr:uid="{9EA14625-33D5-4EF7-8F21-0B01E5AFD468}"/>
     <hyperlink ref="C118" r:id="rId8" xr:uid="{CF96628D-0F57-4F99-94C8-6E77305F553D}"/>
+    <hyperlink ref="C179" r:id="rId9" xr:uid="{49A61CBE-F584-431C-8996-0777D9F3031C}"/>
+    <hyperlink ref="J180" r:id="rId10" xr:uid="{C5CC7172-5FB3-4105-966C-94AD7C8F1806}"/>
+    <hyperlink ref="J181" r:id="rId11" xr:uid="{74EB677D-91E5-4907-B4F5-3ACA421B4E80}"/>
+    <hyperlink ref="J182" r:id="rId12" xr:uid="{EA7E52DD-41C5-45C2-9A18-446254898E6D}"/>
+    <hyperlink ref="C183" r:id="rId13" xr:uid="{08131E02-FD4B-431B-973E-3929F7D77638}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: implement wealth struggle tracking and UI enhancements for asset management
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0214F12-5E2C-48D5-8977-84E1157DC91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D9BB346-4738-4A92-9208-5C3E0CACFC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId22"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">x!$C$2:$M$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">x!$C$2:$M$207</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1484" uniqueCount="895">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1563" uniqueCount="958">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -5164,6 +5164,379 @@
     <t>人間関係の教訓。 「最初」に頑張りすぎると、後で絶対に自分が苦しくなる。 相手はあなたの優しさに「慣れ」、感謝は消え、要求だけがエスカレートする。 そして気づけば「都合の良い人」に認定完了。 イライラしたくないなら、適度な距離感と「断る勇気」を最初から見せておくこと。 自分を安売りしない人が、結局一番大切にされる。</t>
     <phoneticPr fontId="1"/>
   </si>
+  <si>
+    <t>https://x.com/yuruazabu/status/2022919233131450549</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ゆる麻布｜3万部突破</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t>すぐに動ける人になる｜起業家思考が学べる｜仕事のモチベが上がる｜半年で6万フォロワー｜起業、経営、投資、会社売却、経営者の恋愛｜全て本音、忖度無し｜起業家｜1ヶ月で3万部突破｜PHP研究所「こうやって、すぐに動ける人になる。」https://amzn.asia/d/5mpOrRf
+ゆる麻布の詳細はこちら</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>👉</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>yuruazabu.com
+Joined July 2023</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最高の本ができた。1年間の時間をかけて大切に育て上げてきた、初めての本が完成した。Xで発信していたことを、もっと深く、もっと広く多くの人に届けたい。みんながもっと動き出して、もっと日本を盛り上げていきたい。そんな想いの詰まった、これから頑張りたい全ての人に贈る、ワイの最高傑作です。
+まずは今まで、みんなXを見てくれてありがとう。半年で6万人以上の方からフォローしていただき、たくさんの方に応援していただけたことを、心から感謝しとる。これからもよろしくな。
+今までXで発信してきたことを、もっと深く、もっと実践的に、たくさんの人にお伝えできればいいなと思って、魂を込めて本気で本を書くことにした。
+昔の変わりたくても行動できなかった自分を思い出しながら、どんなことを書いたらみんなの役に立つのか、人生がより良くなるのか、そして楽しくなるのか。
+そんなことばかりを考えて、執筆を始めて、そして想いを詰め込みまくって、何度も書いたり消したりを繰り返してたら、気づいたら1年が経っていた。
+あと1ヶ月ちょっとで2025年も終わり。この本を読めば、2026年までに絶対変わる。そして、2026年はめっちゃ楽しくて、めっちゃ有意義な1年になることをワイが保証する。
+学生さん、新卒や第二新卒の方、若手の方、これから頑張りたい方、経営者の方など、何かを変えたい全ての方にとって、必ず気づきやヒントがある本に仕上がった。
+本当にめっちゃいい内容になったと心から思ってるから、この本を絶対にベストセラーにしたいと思っとる。
+これから、この本を少しでも多くの人に届けるために、色々な活動をしていこうと思っているけど、まずは最初の1冊をぜひ手に取って欲しい。
+そして、出版にあたり、大切な友人から嬉しい推薦をいただいたので、紹介させて欲しい。
+「先延ばし民への最終警告。この本で動けなかったら、マジで人生詰みです。」
+高野秀敏さん 
+@keyplayers
+ （キープレイヤーズ代表、『ベンチャーの作法』著者）
+「やる気不要、「仕組み」で動ける体質に変える革新的な本。」
+三宅裕之さん 
+@hiroyuki_miyake
+ （教育実業家、『奇跡が起きる 毎朝１分日記』著者）
+「どんな悩みもスッキリ解決！“納得して生きる力”が身につく本です。　」
+森川亮さん 
+@moriakit
+ （元LINE代表、『シンプルに考える』著者）
+今日からAmazonで予約開始だから、ぜひみんな予約してな。そして届いたら、ぜひ感想を教えてな。
+Amazon限定の特典として、この本を書くに至った裏話の音声特典をつけとるで。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>これな。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デジタル全盛</t>
+    <rPh sb="4" eb="6">
+      <t>ゼンセイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>時代</t>
+    <rPh sb="0" eb="2">
+      <t>ジダイ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>手紙</t>
+    <rPh sb="0" eb="2">
+      <t>テガミ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>書け</t>
+    <rPh sb="0" eb="1">
+      <t>カ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>侍ジャパン</t>
+    <rPh sb="0" eb="1">
+      <t>サムライ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>選手</t>
+    <rPh sb="0" eb="2">
+      <t>センシュ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>私</t>
+    <rPh sb="0" eb="1">
+      <t>ワタシ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>思い</t>
+    <rPh sb="0" eb="1">
+      <t>オモ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>毛筆</t>
+    <rPh sb="0" eb="2">
+      <t>モウヒツ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>英語</t>
+    <rPh sb="0" eb="2">
+      <t>エイゴ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>訳文</t>
+    <rPh sb="0" eb="2">
+      <t>ヤクブン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>できることはすべてやる</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デジタル全盛の時代に、あえて「手紙」を書け。 侍ジャパンの選手を口説く時、私はパソコンを開かなかった。 毛筆で、英語の訳文を添えて、ただひたすらに思いを綴った。 効率？そんなものはない。 でも、相手の心を動かすのはいつだって、泥臭い「手間」と「熱量」だけだ。 「できることはすべてやる」とは、そういうことだ。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>最後に手書きの手紙を書いたのはいつですか？ メールやLINEで済ませるのが当たり前の今だからこそ、直筆の「重み」が相手に刺さる。 侍ジャパンの選手へのオファーも、私は毛筆の手紙に英語の訳文を添えて送った。 デジタルで何でもできる時代に、あえてアナログを選ぶ。 その「非効率」こそが、相手への最大の敬意になると思いませんか？</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>デジタル全盛だからこそ、最強の武器は「手紙」だ。 侍ジャパンへのオファーも、毛筆で、英語訳を添えて。 「できることはすべてやる」 その覚悟は、画面越しの文字じゃ伝わらない。 思いを伝えたいなら、書け。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>リポスト</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/ysk_motoyama/status/2023181173418262611</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>もとやま</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <r>
+      <t>1人社長兼会社員の「自由気ままな働き方」を発信｜著書『投資としての読書』『仕事ができる人のキリの悪い時間の使い方』｜生成AIとかコンテンツマーケとかDXが得意｜株式会社Shikumu代表｜グロービス講師｜元PwCコンサルタント｜Globis MBA←慶應商｜福岡住み｜お問い合わせはDMまで
+View more
+自由気ままな働き方note「シゴデキ部屋」はこちら</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="2"/>
+      </rPr>
+      <t>👇</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>note.com/yusuke_motoyam…
+Joined January 2019</t>
+    </r>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>マネジメント本20冊読んで初管理職に挑んだ結果、どうなったのか、約3万字の学びを全部noteに綴ってみました。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>解説『科学的根拠に基づく最高の勉強法』を試してみたら効果抜群すぎた</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/kanta13jp1/status/2023258195121365261</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/RayDalio/status/2022788750388998543</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Ray Dalio</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Official account of Ray Dalio, founder of Bridgewater Associates, author of #1 New York Times bestseller 'Principles,' professional mistake maker
+View more
+wmi.edu.sg/dmp-online/?ut…
+Joined August 2009</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>レイ・ダリオ公式アカウント
+ブリッジウォーター・アソシエイツ創業者
+『プリンシプルズ』ニューヨーク・タイムズベストセラー第1位著者
+プロの失敗製造者
+もっと見る
+wmi.edu.sg/dmp-online/?ut…
+2009年8月参加</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>It’s Official: The World Order Has Broken Down</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>At the Munich Security Conference, the post-1945 world order was pronounced dead by most leaders and the picture behind it was laid out in the Security Report 2026, entitled “Under Destruction,” which you can read here if you're interested.  More specifically, German Chancellor Friedrich Merz said, “The world order as it has stood for decades no longer exists,” and that we are in a period “great power politics.”   He made clear that freedom “is no longer a given” in this new era. French President Emmanuel Macron echoed Merz’s assessment and said that Europe’s old security structures tied to the previous world order don't exist and that Europe must prepare for war. U.S. Secretary of State Marco Rubio said that we are in a “new geopolitics era” because the “old world” is gone.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ミュンヘン安全保障会議では、1945 年以降の世界秩序は終焉を迎えたとほとんどの指導者が宣言し、その背景については「破壊下」と題された 2026 年の安全保障報告書にまとめられています。ご興味があれば、こちらでご覧いただけます。具体的には、ドイツのフリードリッヒ・メルツ首相は、「何十年も続いてきた世界秩序はもはや存在せず、我々は『大国の政治』の時代に突入している」と述べています。  彼は、この新しい時代では自由は「もはや当然のものではない」ことを明らかにしました。フランスのエマニュエル・マクロン大統領は、メルツ氏の評価に賛同し、これまでの世界秩序に結びついたヨーロッパの古い安全保障構造はもはや存在せず、ヨーロッパは戦争に備える必要があると述べました。米国のマルコ・ルビオ国務長官は、「旧世界」は終わったため、私たちは「新しい地政学の時代」にあると述べています。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>公式発表：世界秩序は崩壊した</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>In my parlance, we are in the Stage 6 part of the Big Cycle in which there is great disorder arising from being in a period in which there are no rules, might is right, and there is a clash of great powers. How Stage 6 works is explained in detail in Chapter 6, “The Big Cycle of External Order and Disorder,” in my book Principles for Dealing with the Changing World Order. While I previously shared a lengthy set of excerpts from Chapter 5 ("The Big Cycle of Internal Order and Disorder"), so you could see how what is going on with the United States tracks the classic cycle explained in that chapter, I am including all of Chapter 6 here for your review.  Given the now nearly universal agreement that the post-1945 world order has broken down and that we are entering a new world order, I think it would be worth your time to read.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>私の用語では、我々はビッグサイクルの第6段階にあり、そこではルールが存在せず、力こそが正義であり、大国間の衝突が起こる時期であることから、大きな混乱が生じている。第6段階の仕組みについては、私の著書『変化する世界秩序に対処するための原則』の第6章「外部秩序と無秩序のビッグサイクル」で詳細に説明している。以前、第5章「内部秩序と無秩序のビッグサイクル」から長文の抜粋を共有し、米国で起きていることが同章で説明される古典的サイクルに沿っていることを示しましたが、今回は第6章全文を掲載します。 1945年以降の世界秩序が崩壊し、新たな世界秩序へ移行しつつあるという認識がほぼ普遍化した今、本書を読む価値は十分にあると考えます。</t>
+  </si>
+  <si>
+    <t>Chapter 6: The Big Cycle of External Order and Disorder
+Relationships between people and the orders that govern them work in basically the same ways, whether they are internal or external, and they blend together. In fact, it wasn’t long ago that there were no distinctions between internal and external orders because there were no clearly defined and mutually recognized boundaries between countries. For that reason, the six-stage cycle of going between order and disorder that I described in the last chapter about what happens within countries works the same way between countries, with one big exception: international relations are driven much more by raw power dynamics. That is because all governance systems require effective and agreed-upon 1) laws and law-making abilities, 2) law enforcement capabilities (e.g., police), 3) ways of adjudicating (e.g., judges), and 4) clear and specified consequences that both suit crimes and are enforced (e.g., fines and incarcerations), and those things either don’t exist or are not as effective in guiding relations between countries as they are in guiding relations within them.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>第6章：外部秩序と無秩序の大きな循環
+人間とそれを支配する秩序との関係は、内部であれ外部であれ基本的に同じ仕組みで機能し、それらは混ざり合う。実際、国家間の境界が明確に定義され相互に認識されていなかったため、内部秩序と外部秩序の区別が存在しなかったのは、それほど昔のことではない。そのため、前章で国内における秩序と無秩序の循環として説明した六段階のサイクルは、国家間においても同様に機能する。ただし、一つの大きな例外がある：国際関係は、より直接的な力関係によって駆動される傾向が強い。これは、あらゆる統治システムが以下の要素を必要とするためである：1) 効果的で合意された法律と立法能力、2) 法執行能力（例：警察）、 3) 裁定方法（例：裁判官）、4) 犯罪に適合し執行される明確かつ規定された結果（例：罰金や投獄）を必要とするが、これらの要素は国家間の関係を導く上で、国家内の関係を導く場合ほど存在しないか、あるいは効果的ではない。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>While attempts have been made to make the external order more rule-abiding (e.g., via the League of Nations and the United Nations), by and large they have failed because these organizations have not had more wealth and power than the most powerful countries. When individual countries have more power than the collectives of countries, the more powerful individual countries rule. For example, if the US, China, or other countries have more power than the United Nations, then the US, China, or other countries will determine how things go rather than the United Nations. That is because power prevails, and wealth and power among equals is rarely given up without a fight.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>国際秩序をより規範遵守的なものとする試み（国際連盟や国際連合など）がなされてきたが、概して失敗に終わっている。これらの組織は、最も強力な国々よりも富と権力を有していなかったためである。個々の国が国家集団よりも強い力を持つ場合、より強力な個々の国が支配する。例えば、米国や中国、その他の国々が国連よりも大きな力を持つ場合、事態の行方は国連ではなく米国や中国、その他の国々によって決定される。なぜなら力は常に優先され、対等な立場にある者同士の富と権力は、争いなくして放棄されることは稀だからである。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>When powerful countries have disputes, they don’t get their lawyers to plead their cases to judges. Instead, they threaten each other and either reach agreements or fight. The international order follows the law of the jungle much more than it follows international law.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>強国同士が争いを起こす時、弁護士を立てて裁判官に訴えを請うことはない。代わりに互いに威嚇し合い、合意に達するか、あるいは戦う。国際秩序は国際法よりも、むしろ弱肉強食の法則に従っている。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>There are five major kinds of fights between countries: trade/economic wars, technology wars, capital wars, geopolitical wars, and military wars. Let’s begin by briefly defining them.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>国家間の主要な争いは五つに分類される：貿易・経済戦争、技術戦争、資本戦争、地政学的戦争、そして軍事戦争である。まずこれらを簡潔に定義することから始めよう。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1. Trade/economic wars: Conflicts over tariffs, import/export restrictions, and other ways of damaging a rival economically
+2. Technology wars: Conflicts over which technologies are shared and which are held as protected aspects of national security
+3. Geopolitical wars: Conflicts over territory and alliances that are resolved through negotiations and explicit or implicit commitments, not fighting
+4. Capital wars: Conflicts imposed through financial tools such as sanctions (e.g., cutting off money and credit by punishing institutions and governments that offer it) and limiting foreign access to capital markets
+5. Military wars: Conflicts that involve actual shooting and the deployment of military forces</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1. 貿易・経済戦争：関税、輸出入制限、その他経済的手段による相手国への損害を与える紛争
+2. 技術戦争：どの技術を共有し、どの技術を国家安全保障上の保護対象とするかに関する紛争
+3. 地政学的戦争：領土や同盟をめぐる紛争で、戦闘ではなく交渉や明示的・暗黙の約束によって解決されるもの
+4. 資本戦争：制裁（例：資金・信用を提供する機関や政府を罰することで遮断する）や外国資本市場へのアクセス制限といった金融手段による対立
+5. 軍事戦争：実際の戦闘や軍事力の展開を伴う対立</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Most fights between nations fall under one or more of those categories (cyber warfare, for example, has a role in all of them). They are over wealth and power and the ideologies pertaining to them.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>国家間の紛争の大半は、これらのカテゴリーの一つまたは複数に該当する（例えばサイバー戦争は全てに関与している）。その争いは富と権力、そしてそれらに関連するイデオロギーを巡るものである。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>While most of these types of wars don’t involve shooting and killing, they all are power struggles. In most cases, the first four kinds of war will evolve over time as intense competitions between rival nations until a military war begins. These struggles and wars, whether or not they involve shooting and killing, are exertions of power of one side over the other. They can be all-out or contained, depending on how important the issue is and what the relative powers of the opponents are. But once a military war begins, all four of the other dimensions will be weaponized to the greatest extent possible.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>こうした戦争の大半は銃撃や殺戮を伴わないものの、いずれも権力闘争である。多くの場合、最初の四種類の戦争は、軍事戦争が始まるまで、対立する国家間の激しい競争として時間をかけて発展する。こうした闘争や戦争は、銃撃や殺戮を伴うか否かにかかわらず、一方の側が他方に対して権力を行使する行為である。その重要度や対立する双方の相対的な力関係に応じて、全面的なものにも限定的なものにもなり得る。しかし軍事戦争が始まると、他の四つの次元は可能な限り最大限に武器化される。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>As discussed in the last several chapters, all of the factors that drive internal and external cycles tend to improve and worsen together. When things get bad, there are more things to argue over, which leads to greater inclinations to fight. That’s human nature, and it is why we have the Big Cycle, which oscillates between good times and bad ones.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>過去数章で論じた通り、内部サイクルと外部サイクルを駆動する要因はすべて、共に改善と悪化を繰り返す傾向にある。状況が悪化すれば、争点が増え、対立する傾向が強まる。これは人間の本性であり、好況と不況の間で揺れ動くビッグサイクルが存在する理由である。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>All-out wars typically occur when existential issues (ones that are so essential to the country’s existence that people are willing to fight and die for them) are at stake and they cannot be resolved by peaceful means. The wars that result from them make it clear which side gets its way and has supremacy in subsequent matters. That clarity over who sets the rules then becomes the basis of a new international order.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>全面戦争は通常、国家の存亡に関わる問題（国民が戦って死ぬ覚悟で守るほど重要な問題）が懸かり、平和的手段では解決できない場合に発生する。その結果生じる戦争は、どちらの側が自らの主張を通し、その後の事柄において優位性を得るかを明らかにする。誰がルールを決めるかという明確さが、新たな国際秩序の基盤となるのである。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>The following chart shows the cycles of internal and external peace and conflict in Europe going back to 1500 as reflected in the deaths they caused. As you can see, there were three big cycles of rising and declining conflict, averaging about 150 years each. Though big civil and external wars last only a short time, they are typically the culmination of the longstanding conflicts that led up to them.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>以下の図表は、1500年まで遡るヨーロッパにおける内戦と対外戦争の平和と紛争の周期を、それらが引き起こした死者数に基づいて示したものである。ご覧の通り、紛争の増減を示す3つの大きな周期が存在し、それぞれ平均約150年続いている。大規模な内戦や対外戦争は短期間で終わるものの、それらは通常、それ以前に長期間にわたって蓄積された紛争の頂点として発生するものである。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>While World Wars I and II were separately driven by the classic cycle, they were also interrelated.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>第一次世界大戦と第二次世界大戦はそれぞれ古典的サイクルによって駆動されたが、相互に関連し合っていた。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>As you can see, each cycle consisted of a relatively long period of peace and prosperity (e.g., the Renaissance, the Enlightenment, and the Industrial Revolution) that sowed the seeds for terrible and violent external wars (e.g., the Thirty Years’ War, the Napoleonic Wars, and the two World Wars). Both the upswings (the periods of peace and prosperity) and the downswings (the periods of depression and war) affected the whole world. Not all countries prosper when the leading powers do because countries gain at the expense of others. For example, the decline of China from around 1840 to 1949, known as the “Century of Humiliation,” came about because the Western powers and Japan exploited China.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ご覧の通り、各サイクルは比較的長い平和と繁栄の時代（例：ルネサンス、啓蒙時代、産業革命）で構成され、それが恐ろしい暴力的な対外戦争（例：三十年戦争、ナポレオン戦争、二度の世界大戦）の種を蒔いた。上昇局面（平和と繁栄の時代）も下降局面（不況と戦争の時代）も、世界全体に影響を及ぼしました。主要国が繁栄しても、すべての国が繁栄するわけではありません。なぜなら、ある国が利益を得ることは、他の国が犠牲になることを意味するからです。例えば、1840年頃から1949年にかけての中国の衰退期は「屈辱の世紀」と呼ばれ、これは欧米諸国と日本による中国搾取の結果でした。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>As you read on, keep in mind that * the two things about war that one can be most confident in are 1) that it won’t go as planned and 2) that it will be far worse than imagined. It is for those reasons that so many of the principles that follow are about ways to avoid shooting wars. Still, whether they are fought for good reasons or bad, shooting wars happen. To be clear, while I believe most are tragic and fought for nonsensical reasons, some are worth fighting because the consequences of not fighting them (e.g., the loss of freedom) would be intolerable.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>読み進めるにあたり、次の二点を心に留めておいてほしい。戦争に関して最も確信を持って言えることは、1）計画通りには進まないこと、2）想像をはるかに超える惨事になることだ。だからこそ、以下に述べる原則の多くは武力衝突を回避する方法に焦点を当てている。とはいえ、正当な理由によるものであれ不当な理由によるものであれ、武力衝突は発生する。明確にしておくと、私はその大半が悲劇的で無意味な理由で戦われていると考えるが、戦わなければ生じる結果（例えば自由の喪失）が耐え難いものとなるため、戦う価値のある戦争も存在する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
 </sst>
 </file>
 
@@ -5211,18 +5584,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -5238,7 +5605,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -5248,9 +5615,6 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -5574,7 +5938,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -5757,7 +6121,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -5970,7 +6334,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -6146,7 +6510,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -9692,7 +10056,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -10176,11 +10540,11 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="C2:Q194"/>
+  <dimension ref="C2:Q225"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="67.875" customWidth="1"/>
     <col min="6" max="6" width="59.625" customWidth="1"/>
     <col min="7" max="7" width="10.25" bestFit="1" customWidth="1"/>
@@ -11790,8 +12154,17 @@
       </c>
     </row>
     <row r="187" spans="3:13">
+      <c r="C187" s="2"/>
+      <c r="E187" s="1"/>
+      <c r="F187" s="1"/>
       <c r="H187" t="s">
         <v>884</v>
+      </c>
+      <c r="J187" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="K187" s="3">
+        <v>46069</v>
       </c>
     </row>
     <row r="188" spans="3:13">
@@ -11819,18 +12192,308 @@
         <v>889</v>
       </c>
     </row>
-    <row r="193" spans="8:8">
+    <row r="193" spans="3:13">
       <c r="H193" t="s">
         <v>890</v>
       </c>
     </row>
-    <row r="194" spans="8:8">
+    <row r="194" spans="3:13">
       <c r="H194" t="s">
         <v>891</v>
       </c>
     </row>
+    <row r="195" spans="3:13" ht="409.5">
+      <c r="C195" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="D195" t="s">
+        <v>896</v>
+      </c>
+      <c r="E195" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="F195" s="1" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="196" spans="3:13" ht="112.5">
+      <c r="F196" t="s">
+        <v>899</v>
+      </c>
+      <c r="G196" s="3">
+        <v>46069</v>
+      </c>
+      <c r="H196" t="s">
+        <v>900</v>
+      </c>
+      <c r="I196" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="J196" s="1" t="s">
+        <v>912</v>
+      </c>
+      <c r="K196" s="3">
+        <v>46069</v>
+      </c>
+      <c r="L196">
+        <v>17</v>
+      </c>
+      <c r="M196">
+        <v>3642</v>
+      </c>
+    </row>
+    <row r="197" spans="3:13" ht="112.5">
+      <c r="H197" t="s">
+        <v>901</v>
+      </c>
+      <c r="J197" s="1" t="s">
+        <v>913</v>
+      </c>
+      <c r="K197" s="3">
+        <v>46069</v>
+      </c>
+      <c r="L197">
+        <v>21</v>
+      </c>
+      <c r="M197">
+        <v>3642</v>
+      </c>
+    </row>
+    <row r="198" spans="3:13" ht="75">
+      <c r="H198" t="s">
+        <v>902</v>
+      </c>
+      <c r="J198" s="1" t="s">
+        <v>914</v>
+      </c>
+      <c r="K198" s="3">
+        <v>46069</v>
+      </c>
+      <c r="L198">
+        <v>23</v>
+      </c>
+      <c r="M198">
+        <v>3642</v>
+      </c>
+    </row>
+    <row r="199" spans="3:13">
+      <c r="H199" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="200" spans="3:13">
+      <c r="H200" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="201" spans="3:13">
+      <c r="H201" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="202" spans="3:13">
+      <c r="H202" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="203" spans="3:13">
+      <c r="H203" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="204" spans="3:13">
+      <c r="H204" t="s">
+        <v>908</v>
+      </c>
+    </row>
+    <row r="205" spans="3:13">
+      <c r="H205" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="206" spans="3:13">
+      <c r="H206" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="207" spans="3:13">
+      <c r="H207" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="208" spans="3:13" ht="150">
+      <c r="C208" s="2" t="s">
+        <v>916</v>
+      </c>
+      <c r="D208" t="s">
+        <v>917</v>
+      </c>
+      <c r="E208" s="1" t="s">
+        <v>918</v>
+      </c>
+      <c r="F208" s="1" t="s">
+        <v>919</v>
+      </c>
+      <c r="G208" s="3">
+        <v>46069</v>
+      </c>
+    </row>
+    <row r="209" spans="3:10" ht="37.5">
+      <c r="F209" s="1" t="s">
+        <v>920</v>
+      </c>
+      <c r="G209" s="3">
+        <v>46069</v>
+      </c>
+      <c r="I209" s="1" t="s">
+        <v>873</v>
+      </c>
+      <c r="J209" s="2" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="210" spans="3:10" ht="93.75">
+      <c r="C210" s="2" t="s">
+        <v>922</v>
+      </c>
+      <c r="D210" t="s">
+        <v>923</v>
+      </c>
+      <c r="E210" s="1" t="s">
+        <v>924</v>
+      </c>
+      <c r="F210" t="s">
+        <v>926</v>
+      </c>
+      <c r="I210" t="s">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="211" spans="3:10" ht="262.5">
+      <c r="E211" s="1" t="s">
+        <v>925</v>
+      </c>
+      <c r="F211" s="1" t="s">
+        <v>927</v>
+      </c>
+      <c r="I211" s="1" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="212" spans="3:10" ht="243.75">
+      <c r="F212" s="1" t="s">
+        <v>930</v>
+      </c>
+      <c r="I212" s="1" t="s">
+        <v>931</v>
+      </c>
+    </row>
+    <row r="213" spans="3:10" ht="337.5">
+      <c r="F213" s="1" t="s">
+        <v>932</v>
+      </c>
+      <c r="I213" s="1" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="214" spans="3:10" ht="206.25">
+      <c r="F214" s="1" t="s">
+        <v>934</v>
+      </c>
+      <c r="I214" s="1" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="215" spans="3:10" ht="75">
+      <c r="F215" s="1" t="s">
+        <v>936</v>
+      </c>
+      <c r="I215" s="1" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="216" spans="3:10" ht="56.25">
+      <c r="F216" s="1" t="s">
+        <v>938</v>
+      </c>
+      <c r="I216" s="1" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="217" spans="3:10" ht="243.75">
+      <c r="F217" s="1" t="s">
+        <v>940</v>
+      </c>
+      <c r="I217" s="1" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="218" spans="3:10" ht="75">
+      <c r="F218" s="1" t="s">
+        <v>942</v>
+      </c>
+      <c r="I218" s="1" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="219" spans="3:10" ht="168.75">
+      <c r="F219" s="1" t="s">
+        <v>944</v>
+      </c>
+      <c r="I219" s="1" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="220" spans="3:10" ht="112.5">
+      <c r="F220" s="1" t="s">
+        <v>946</v>
+      </c>
+      <c r="I220" s="1" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="221" spans="3:10" ht="131.25">
+      <c r="F221" s="1" t="s">
+        <v>948</v>
+      </c>
+      <c r="I221" s="1" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="222" spans="3:10" ht="131.25">
+      <c r="F222" s="1" t="s">
+        <v>950</v>
+      </c>
+      <c r="I222" s="1" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="223" spans="3:10" ht="37.5">
+      <c r="F223" s="1" t="s">
+        <v>952</v>
+      </c>
+      <c r="I223" s="1" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="224" spans="3:10" ht="206.25">
+      <c r="F224" s="1" t="s">
+        <v>954</v>
+      </c>
+      <c r="I224" s="1" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="225" spans="6:9" ht="168.75">
+      <c r="F225" s="1" t="s">
+        <v>956</v>
+      </c>
+      <c r="I225" s="1" t="s">
+        <v>957</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="C2:M117" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}"/>
+  <autoFilter ref="C2:M207" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}"/>
   <phoneticPr fontId="1"/>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" xr:uid="{C897C6D6-16A8-4618-9776-831A651C49AE}"/>
@@ -11846,6 +12509,10 @@
     <hyperlink ref="J181" r:id="rId11" xr:uid="{74EB677D-91E5-4907-B4F5-3ACA421B4E80}"/>
     <hyperlink ref="J182" r:id="rId12" xr:uid="{EA7E52DD-41C5-45C2-9A18-446254898E6D}"/>
     <hyperlink ref="C183" r:id="rId13" xr:uid="{08131E02-FD4B-431B-973E-3929F7D77638}"/>
+    <hyperlink ref="C195" r:id="rId14" xr:uid="{39E432C6-4E9C-4343-9815-52F316B64658}"/>
+    <hyperlink ref="C208" r:id="rId15" xr:uid="{3BB45995-7DA2-4F11-900F-84AFACB633B1}"/>
+    <hyperlink ref="J209" r:id="rId16" xr:uid="{9220184A-77DE-47EA-97A3-9205D7952A4A}"/>
+    <hyperlink ref="C210" r:id="rId17" xr:uid="{90934316-82E9-4DC7-B9EE-F6BEE341122B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11853,7 +12520,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970790C5-0376-420E-A317-55DF989D7F43}">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr defaultColWidth="73.25" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="77.5" bestFit="1" customWidth="1"/>
@@ -11864,9 +12531,10 @@
     <col min="6" max="6" width="17.125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="B1" t="s">
         <v>674</v>
       </c>
@@ -11888,200 +12556,227 @@
       <c r="H1" t="s">
         <v>793</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="93.75">
-      <c r="A2" s="1" t="s">
-        <v>792</v>
+      <c r="I1" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="2" t="s">
+        <v>876</v>
       </c>
       <c r="B2" s="3">
-        <v>46066</v>
+        <v>46068</v>
       </c>
       <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="D2">
+        <v>3639</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>3643</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="112.5">
+      <c r="A3" s="1" t="s">
+        <v>893</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C3">
         <v>3</v>
       </c>
-      <c r="D2">
-        <v>3642</v>
-      </c>
-      <c r="E2" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F2">
+      <c r="D3">
+        <v>3639</v>
+      </c>
+      <c r="F3">
+        <v>13</v>
+      </c>
+      <c r="G3">
+        <v>3643</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="75">
+      <c r="A4" s="1" t="s">
+        <v>894</v>
+      </c>
+      <c r="B4" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>3639</v>
+      </c>
+      <c r="F4">
+        <v>13</v>
+      </c>
+      <c r="G4">
+        <v>3643</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="93.75">
+      <c r="A5" s="1" t="s">
+        <v>866</v>
+      </c>
+      <c r="B5" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C5">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>3640</v>
+      </c>
+      <c r="F5">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <v>3643</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="2" t="s">
+        <v>874</v>
+      </c>
+      <c r="B6" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C6">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>3639</v>
+      </c>
+      <c r="F6">
+        <v>14</v>
+      </c>
+      <c r="G6">
+        <v>3643</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
+        <v>875</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C7">
+        <v>8</v>
+      </c>
+      <c r="D7">
+        <v>3639</v>
+      </c>
+      <c r="F7">
+        <v>14</v>
+      </c>
+      <c r="G7">
+        <v>3643</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="93.75">
+      <c r="A8" s="1" t="s">
+        <v>865</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C8">
+        <v>13</v>
+      </c>
+      <c r="D8">
+        <v>3640</v>
+      </c>
+      <c r="F8">
+        <v>18</v>
+      </c>
+      <c r="G8">
+        <v>3643</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="75">
+      <c r="A9" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C9">
+        <v>13</v>
+      </c>
+      <c r="D9">
+        <v>3640</v>
+      </c>
+      <c r="F9">
         <v>20</v>
       </c>
-      <c r="G2">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="75">
-      <c r="A3" s="1" t="s">
-        <v>770</v>
-      </c>
-      <c r="B3" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C3">
-        <v>11</v>
-      </c>
-      <c r="D3">
-        <v>3642</v>
-      </c>
-      <c r="E3" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F3">
-        <v>23</v>
-      </c>
-      <c r="G3">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="168.75">
-      <c r="A4" s="1" t="s">
+      <c r="G9">
+        <v>3643</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="168.75">
+      <c r="A10" s="1" t="s">
         <v>790</v>
-      </c>
-      <c r="B4" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C4">
-        <v>3</v>
-      </c>
-      <c r="D4">
-        <v>3642</v>
-      </c>
-      <c r="E4" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F4">
-        <v>23</v>
-      </c>
-      <c r="G4">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="75">
-      <c r="A5" s="1" t="s">
-        <v>734</v>
-      </c>
-      <c r="B5" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C5">
-        <v>13</v>
-      </c>
-      <c r="D5">
-        <v>3642</v>
-      </c>
-      <c r="E5" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F5">
-        <v>24</v>
-      </c>
-      <c r="G5">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="93.75">
-      <c r="A6" s="1" t="s">
-        <v>710</v>
-      </c>
-      <c r="B6" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>3642</v>
-      </c>
-      <c r="E6" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F6">
-        <v>25</v>
-      </c>
-      <c r="G6">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="93.75">
-      <c r="A7" s="1" t="s">
-        <v>732</v>
-      </c>
-      <c r="B7" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C7">
-        <v>13</v>
-      </c>
-      <c r="D7">
-        <v>3642</v>
-      </c>
-      <c r="E7" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F7">
-        <v>25</v>
-      </c>
-      <c r="G7">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="75">
-      <c r="A8" s="1" t="s">
-        <v>712</v>
-      </c>
-      <c r="B8" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C8">
-        <v>17</v>
-      </c>
-      <c r="D8">
-        <v>3642</v>
-      </c>
-      <c r="E8" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F8">
-        <v>27</v>
-      </c>
-      <c r="G8">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="187.5">
-      <c r="A9" s="1" t="s">
-        <v>733</v>
-      </c>
-      <c r="B9" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C9">
-        <v>16</v>
-      </c>
-      <c r="D9">
-        <v>3642</v>
-      </c>
-      <c r="E9" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F9">
-        <v>27</v>
-      </c>
-      <c r="G9">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="56.25">
-      <c r="A10" s="1" t="s">
-        <v>657</v>
       </c>
       <c r="B10" s="3">
         <v>46066</v>
       </c>
       <c r="C10">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="D10">
         <v>3642</v>
@@ -12090,21 +12785,27 @@
         <v>46067</v>
       </c>
       <c r="F10">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G10">
         <v>3639</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" ht="75">
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="93.75">
       <c r="A11" s="1" t="s">
-        <v>771</v>
+        <v>732</v>
       </c>
       <c r="B11" s="3">
         <v>46066</v>
       </c>
       <c r="C11">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D11">
         <v>3642</v>
@@ -12113,21 +12814,27 @@
         <v>46067</v>
       </c>
       <c r="F11">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G11">
         <v>3639</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="262.5">
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="75">
       <c r="A12" s="1" t="s">
-        <v>680</v>
+        <v>734</v>
       </c>
       <c r="B12" s="3">
         <v>46066</v>
       </c>
       <c r="C12">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D12">
         <v>3642</v>
@@ -12136,21 +12843,27 @@
         <v>46067</v>
       </c>
       <c r="F12">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G12">
         <v>3639</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" ht="93.75">
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="75">
       <c r="A13" s="1" t="s">
-        <v>769</v>
+        <v>770</v>
       </c>
       <c r="B13" s="3">
         <v>46066</v>
       </c>
       <c r="C13">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="D13">
         <v>3642</v>
@@ -12159,21 +12872,27 @@
         <v>46067</v>
       </c>
       <c r="F13">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G13">
         <v>3639</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" ht="206.25">
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="93.75">
       <c r="A14" s="1" t="s">
-        <v>656</v>
+        <v>792</v>
       </c>
       <c r="B14" s="3">
         <v>46066</v>
       </c>
       <c r="C14">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="D14">
         <v>3642</v>
@@ -12182,7 +12901,7 @@
         <v>46067</v>
       </c>
       <c r="F14">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G14">
         <v>3639</v>
@@ -12190,16 +12909,19 @@
       <c r="H14">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" ht="150">
+      <c r="I14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="93.75">
       <c r="A15" s="1" t="s">
-        <v>791</v>
+        <v>710</v>
       </c>
       <c r="B15" s="3">
         <v>46066</v>
       </c>
       <c r="C15">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="D15">
         <v>3642</v>
@@ -12208,44 +12930,53 @@
         <v>46067</v>
       </c>
       <c r="F15">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="G15">
         <v>3639</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="75">
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="75">
       <c r="A16" s="1" t="s">
-        <v>679</v>
+        <v>912</v>
       </c>
       <c r="B16" s="3">
-        <v>46066</v>
+        <v>46069</v>
       </c>
       <c r="C16">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="D16">
         <v>3642</v>
       </c>
-      <c r="E16" s="3">
-        <v>46067</v>
-      </c>
       <c r="F16">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G16">
-        <v>3639</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="75">
-      <c r="A17" s="6" t="s">
-        <v>681</v>
+        <v>3643</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="75">
+      <c r="A17" s="1" t="s">
+        <v>712</v>
       </c>
       <c r="B17" s="3">
         <v>46066</v>
       </c>
       <c r="C17">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D17">
         <v>3642</v>
@@ -12254,24 +12985,27 @@
         <v>46067</v>
       </c>
       <c r="F17">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G17">
         <v>3639</v>
       </c>
-      <c r="I17" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="56.25">
-      <c r="A18" s="6" t="s">
-        <v>655</v>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="187.5">
+      <c r="A18" s="1" t="s">
+        <v>733</v>
       </c>
       <c r="B18" s="3">
         <v>46066</v>
       </c>
       <c r="C18">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="D18">
         <v>3642</v>
@@ -12280,7 +13014,7 @@
         <v>46067</v>
       </c>
       <c r="F18">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G18">
         <v>3639</v>
@@ -12288,19 +13022,19 @@
       <c r="H18">
         <v>1</v>
       </c>
-      <c r="I18" t="s">
-        <v>794</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="75">
-      <c r="A19" s="6" t="s">
-        <v>711</v>
+      <c r="I18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="56.25">
+      <c r="A19" s="1" t="s">
+        <v>657</v>
       </c>
       <c r="B19" s="3">
         <v>46066</v>
       </c>
       <c r="C19">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="D19">
         <v>3642</v>
@@ -12309,20 +13043,384 @@
         <v>46067</v>
       </c>
       <c r="F19">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="G19">
         <v>3639</v>
       </c>
-      <c r="I19" t="s">
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="56.25">
+      <c r="A20" s="1" t="s">
+        <v>914</v>
+      </c>
+      <c r="B20" s="3">
+        <v>46069</v>
+      </c>
+      <c r="C20">
+        <v>23</v>
+      </c>
+      <c r="D20">
+        <v>3642</v>
+      </c>
+      <c r="F20">
+        <v>32</v>
+      </c>
+      <c r="G20">
+        <v>3643</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="75">
+      <c r="A21" s="1" t="s">
+        <v>913</v>
+      </c>
+      <c r="B21" s="3">
+        <v>46069</v>
+      </c>
+      <c r="C21">
+        <v>21</v>
+      </c>
+      <c r="D21">
+        <v>3642</v>
+      </c>
+      <c r="F21">
+        <v>33</v>
+      </c>
+      <c r="G21">
+        <v>3643</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="75">
+      <c r="A22" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="B22" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C22">
+        <v>15</v>
+      </c>
+      <c r="D22">
+        <v>3642</v>
+      </c>
+      <c r="E22" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F22">
+        <v>34</v>
+      </c>
+      <c r="G22">
+        <v>3639</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="93.75">
+      <c r="A23" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C23">
+        <v>17</v>
+      </c>
+      <c r="D23">
+        <v>3642</v>
+      </c>
+      <c r="E23" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F23">
+        <v>35</v>
+      </c>
+      <c r="G23">
+        <v>3639</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="206.25">
+      <c r="A24" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B24" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C24">
+        <v>19</v>
+      </c>
+      <c r="D24">
+        <v>3642</v>
+      </c>
+      <c r="E24" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F24">
+        <v>37</v>
+      </c>
+      <c r="G24">
+        <v>3639</v>
+      </c>
+      <c r="H24">
+        <v>2</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="262.5">
+      <c r="A25" s="1" t="s">
+        <v>680</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C25">
+        <v>24</v>
+      </c>
+      <c r="D25">
+        <v>3642</v>
+      </c>
+      <c r="E25" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F25">
+        <v>37</v>
+      </c>
+      <c r="G25">
+        <v>3639</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
+      <c r="I25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="150">
+      <c r="A26" s="1" t="s">
+        <v>791</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C26">
+        <v>3</v>
+      </c>
+      <c r="D26">
+        <v>3642</v>
+      </c>
+      <c r="E26" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F26">
+        <v>37</v>
+      </c>
+      <c r="G26">
+        <v>3639</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="75">
+      <c r="A27" s="1" t="s">
+        <v>679</v>
+      </c>
+      <c r="B27" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C27">
+        <v>26</v>
+      </c>
+      <c r="D27">
+        <v>3642</v>
+      </c>
+      <c r="E27" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F27">
+        <v>38</v>
+      </c>
+      <c r="G27">
+        <v>3639</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="112.5">
+      <c r="A28" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="B28" s="3">
+        <v>46068</v>
+      </c>
+      <c r="C28">
+        <v>8</v>
+      </c>
+      <c r="D28">
+        <v>3639</v>
+      </c>
+      <c r="F28">
+        <v>39</v>
+      </c>
+      <c r="G28">
+        <v>3643</v>
+      </c>
+      <c r="H28">
+        <v>2</v>
+      </c>
+      <c r="I28">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="75">
+      <c r="A29" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="B29" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C29">
+        <v>28</v>
+      </c>
+      <c r="D29">
+        <v>3642</v>
+      </c>
+      <c r="E29" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F29">
+        <v>68</v>
+      </c>
+      <c r="G29">
+        <v>3639</v>
+      </c>
+      <c r="H29">
+        <v>3</v>
+      </c>
+      <c r="I29">
+        <v>2</v>
+      </c>
+      <c r="J29" t="s">
         <v>794</v>
       </c>
     </row>
+    <row r="30" spans="1:10" ht="75">
+      <c r="A30" s="1" t="s">
+        <v>711</v>
+      </c>
+      <c r="B30" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C30">
+        <v>28</v>
+      </c>
+      <c r="D30">
+        <v>3642</v>
+      </c>
+      <c r="E30" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F30">
+        <v>71</v>
+      </c>
+      <c r="G30">
+        <v>3639</v>
+      </c>
+      <c r="H30">
+        <v>3</v>
+      </c>
+      <c r="I30">
+        <v>2</v>
+      </c>
+      <c r="J30" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="56.25">
+      <c r="A31" s="1" t="s">
+        <v>655</v>
+      </c>
+      <c r="B31" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C31">
+        <v>31</v>
+      </c>
+      <c r="D31">
+        <v>3642</v>
+      </c>
+      <c r="E31" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F31">
+        <v>95</v>
+      </c>
+      <c r="G31">
+        <v>3639</v>
+      </c>
+      <c r="H31">
+        <v>3</v>
+      </c>
+      <c r="I31">
+        <v>2</v>
+      </c>
+      <c r="J31" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="B32" s="3">
+        <v>46069</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H19">
-    <sortCondition ref="F2:F19"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I32">
+    <sortCondition ref="F2:F32"/>
   </sortState>
   <phoneticPr fontId="1"/>
+  <hyperlinks>
+    <hyperlink ref="A6" r:id="rId1" xr:uid="{652F4804-A291-4908-8DB0-F790956B309E}"/>
+    <hyperlink ref="A7" r:id="rId2" xr:uid="{11FEC87D-3AF9-45D5-A4CE-AC44976C500C}"/>
+    <hyperlink ref="A2" r:id="rId3" xr:uid="{331C7376-F1B6-4EE5-8CFD-0EE5CD109EC0}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -12369,37 +13467,37 @@
       </c>
     </row>
     <row r="6" spans="2:9">
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="2:9">
-      <c r="C7" s="7">
+      <c r="C7" s="6">
         <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="8" spans="2:9">
-      <c r="C8" s="7">
+      <c r="C8" s="6">
         <v>8.3333333333333301E-2</v>
       </c>
     </row>
     <row r="9" spans="2:9">
-      <c r="C9" s="7">
+      <c r="C9" s="6">
         <v>0.125</v>
       </c>
     </row>
     <row r="10" spans="2:9">
-      <c r="C10" s="7">
+      <c r="C10" s="6">
         <v>0.16666666666666699</v>
       </c>
     </row>
     <row r="11" spans="2:9">
-      <c r="C11" s="7">
+      <c r="C11" s="6">
         <v>0.20833333333333301</v>
       </c>
     </row>
     <row r="12" spans="2:9">
-      <c r="C12" s="7">
+      <c r="C12" s="6">
         <v>0.25</v>
       </c>
       <c r="E12" t="s">
@@ -12410,7 +13508,7 @@
       </c>
     </row>
     <row r="13" spans="2:9">
-      <c r="C13" s="7"/>
+      <c r="C13" s="6"/>
       <c r="E13" t="s">
         <v>796</v>
       </c>
@@ -12419,13 +13517,13 @@
       </c>
     </row>
     <row r="14" spans="2:9">
-      <c r="C14" s="7"/>
+      <c r="C14" s="6"/>
       <c r="E14" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="15" spans="2:9">
-      <c r="C15" s="7"/>
+      <c r="C15" s="6"/>
       <c r="E15" t="s">
         <v>45</v>
       </c>
@@ -12434,98 +13532,98 @@
       </c>
     </row>
     <row r="16" spans="2:9">
-      <c r="C16" s="7"/>
+      <c r="C16" s="6"/>
       <c r="E16" t="s">
         <v>798</v>
       </c>
     </row>
     <row r="17" spans="3:3">
-      <c r="C17" s="7">
+      <c r="C17" s="6">
         <v>0.29166666666666702</v>
       </c>
     </row>
     <row r="18" spans="3:3">
-      <c r="C18" s="7">
+      <c r="C18" s="6">
         <v>0.33333333333333298</v>
       </c>
     </row>
     <row r="19" spans="3:3">
-      <c r="C19" s="7">
+      <c r="C19" s="6">
         <v>0.375</v>
       </c>
     </row>
     <row r="20" spans="3:3">
-      <c r="C20" s="7">
+      <c r="C20" s="6">
         <v>0.41666666666666702</v>
       </c>
     </row>
     <row r="21" spans="3:3">
-      <c r="C21" s="7">
+      <c r="C21" s="6">
         <v>0.45833333333333298</v>
       </c>
     </row>
     <row r="22" spans="3:3">
-      <c r="C22" s="7">
+      <c r="C22" s="6">
         <v>0.5</v>
       </c>
     </row>
     <row r="23" spans="3:3">
-      <c r="C23" s="7">
+      <c r="C23" s="6">
         <v>0.54166666666666696</v>
       </c>
     </row>
     <row r="24" spans="3:3">
-      <c r="C24" s="7">
+      <c r="C24" s="6">
         <v>0.58333333333333304</v>
       </c>
     </row>
     <row r="25" spans="3:3">
-      <c r="C25" s="7">
+      <c r="C25" s="6">
         <v>0.625</v>
       </c>
     </row>
     <row r="26" spans="3:3">
-      <c r="C26" s="7">
+      <c r="C26" s="6">
         <v>0.66666666666666696</v>
       </c>
     </row>
     <row r="27" spans="3:3">
-      <c r="C27" s="7">
+      <c r="C27" s="6">
         <v>0.70833333333333304</v>
       </c>
     </row>
     <row r="28" spans="3:3">
-      <c r="C28" s="7">
+      <c r="C28" s="6">
         <v>0.75</v>
       </c>
     </row>
     <row r="29" spans="3:3">
-      <c r="C29" s="7">
+      <c r="C29" s="6">
         <v>0.79166666666666696</v>
       </c>
     </row>
     <row r="30" spans="3:3">
-      <c r="C30" s="7">
+      <c r="C30" s="6">
         <v>0.83333333333333304</v>
       </c>
     </row>
     <row r="31" spans="3:3">
-      <c r="C31" s="7">
+      <c r="C31" s="6">
         <v>0.875</v>
       </c>
     </row>
     <row r="32" spans="3:3">
-      <c r="C32" s="7">
+      <c r="C32" s="6">
         <v>0.91666666666666696</v>
       </c>
     </row>
     <row r="33" spans="3:3">
-      <c r="C33" s="7">
+      <c r="C33" s="6">
         <v>0.95833333333333304</v>
       </c>
     </row>
     <row r="34" spans="3:3">
-      <c r="C34" s="7"/>
+      <c r="C34" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -12549,7 +13647,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -12937,7 +14035,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -13583,7 +14681,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46068</v>
+        <v>46070</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
feat: update asset management UI to include investment tracking and enhance struggle logic
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D9BB346-4738-4A92-9208-5C3E0CACFC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1515EEE6-F32C-4D4A-BB1F-E98BAB8385FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
     <sheet name="1日で人生を立て直す方法" sheetId="14" r:id="rId22"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">x!$C$2:$M$207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">x!$C$2:$M$231</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1563" uniqueCount="958">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="969">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -5421,9 +5421,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>私の用語では、我々はビッグサイクルの第6段階にあり、そこではルールが存在せず、力こそが正義であり、大国間の衝突が起こる時期であることから、大きな混乱が生じている。第6段階の仕組みについては、私の著書『変化する世界秩序に対処するための原則』の第6章「外部秩序と無秩序のビッグサイクル」で詳細に説明している。以前、第5章「内部秩序と無秩序のビッグサイクル」から長文の抜粋を共有し、米国で起きていることが同章で説明される古典的サイクルに沿っていることを示しましたが、今回は第6章全文を掲載します。 1945年以降の世界秩序が崩壊し、新たな世界秩序へ移行しつつあるという認識がほぼ普遍化した今、本書を読む価値は十分にあると考えます。</t>
-  </si>
-  <si>
     <t>Chapter 6: The Big Cycle of External Order and Disorder
 Relationships between people and the orders that govern them work in basically the same ways, whether they are internal or external, and they blend together. In fact, it wasn’t long ago that there were no distinctions between internal and external orders because there were no clearly defined and mutually recognized boundaries between countries. For that reason, the six-stage cycle of going between order and disorder that I described in the last chapter about what happens within countries works the same way between countries, with one big exception: international relations are driven much more by raw power dynamics. That is because all governance systems require effective and agreed-upon 1) laws and law-making abilities, 2) law enforcement capabilities (e.g., police), 3) ways of adjudicating (e.g., judges), and 4) clear and specified consequences that both suit crimes and are enforced (e.g., fines and incarcerations), and those things either don’t exist or are not as effective in guiding relations between countries as they are in guiding relations within them.</t>
     <phoneticPr fontId="1"/>
@@ -5535,6 +5532,63 @@
   </si>
   <si>
     <t>読み進めるにあたり、次の二点を心に留めておいてほしい。戦争に関して最も確信を持って言えることは、1）計画通りには進まないこと、2）想像をはるかに超える惨事になることだ。だからこそ、以下に述べる原則の多くは武力衝突を回避する方法に焦点を当てている。とはいえ、正当な理由によるものであれ不当な理由によるものであれ、武力衝突は発生する。明確にしておくと、私はその大半が悲劇的で無意味な理由で戦われていると考えるが、戦わなければ生じる結果（例えば自由の喪失）が耐え難いものとなるため、戦う価値のある戦争も存在する。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>THE TIMELESS AND UNIVERSAL FORCES THAT PRODUCE CHANGES TO THE EXTERNAL ORDER</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>外部の秩序に変化をもたらす、時代を超え普遍的な力</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>私の用語では、我々はビッグサイクルの第6段階にあり、そこではルールが存在せず、力こそが正義であり、大国間の衝突が起こる時期であることから、大きな混乱が生じている。第6段階の仕組みについては、私の著書『変化する世界秩序に対処するための原則』の第6章「外部秩序と無秩序のビッグサイクル」で詳細に説明している。以前、第5章「内部秩序と無秩序のビッグサイクル」から長文の抜粋を共有し、米国で起きていることが同章で説明される古典的サイクルに沿っていることを示しましたが、今回は第6章全文を掲載します。 1945年以降の世界秩序が崩壊し、新たな世界秩序へ移行しつつあるという認識がほぼ普遍化した今、本書を読む価値は十分にあると考えます。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/gokko_ceo/status/2014587657779872073</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>田中 聡 ♧ GOKKO_CEO</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>(株) GOKKO 代表取締役｜-日常で忘れがちな小さな愛- 『ごっこ倶楽部』 
+@gokko5club
+ | ~あなたのスキマに、感動を。~ 『POPCORN』 
+@popcorndrama505
+ 縦型ショートドラマ、エンタメ、スタートアップ、組織論、ときどき犬
+View more
+Entrepreneur知恵の差は“小” なり,行動の差は “大”なり　応募は→gokkoclub.jp/recruit/
+Joined October 2019</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>バズってるだけで意味ある？？
+自分達へのアンチテーゼ。
+GOKKOがやるからこその本当の価値ある作品。ぜひ、来てください！</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">前提が壊れた時代に、舞台役者の価値が上がる理由 </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t xml:space="preserve">IP事業を本気でやろうとしている人だけ読んでほしい。 </t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/kanta13jp1/status/2023828035288637730</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/kanta13jp1/status/2023829338475634704</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>https://x.com/kanta13jp1/status/2023829776843370629</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -5938,7 +5992,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -6121,7 +6175,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -6334,7 +6388,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -6510,7 +6564,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -10056,7 +10110,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -10537,10 +10591,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="C2:Q225"/>
+  <dimension ref="C2:Q231"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
@@ -10568,6 +10622,9 @@
       <c r="I2" t="s">
         <v>677</v>
       </c>
+      <c r="J2" t="s">
+        <v>635</v>
+      </c>
       <c r="K2" t="s">
         <v>674</v>
       </c>
@@ -10590,7 +10647,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="3" spans="3:17" ht="93.75">
+    <row r="3" spans="3:17" ht="93.75" hidden="1">
       <c r="C3" s="2" t="s">
         <v>630</v>
       </c>
@@ -10697,87 +10754,87 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="7" spans="3:17">
+    <row r="7" spans="3:17" hidden="1">
       <c r="H7" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="8" spans="3:17">
+    <row r="8" spans="3:17" hidden="1">
       <c r="H8" t="s">
         <v>640</v>
       </c>
     </row>
-    <row r="9" spans="3:17">
+    <row r="9" spans="3:17" hidden="1">
       <c r="H9" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="10" spans="3:17">
+    <row r="10" spans="3:17" hidden="1">
       <c r="H10" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="11" spans="3:17">
+    <row r="11" spans="3:17" hidden="1">
       <c r="H11" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="12" spans="3:17">
+    <row r="12" spans="3:17" hidden="1">
       <c r="H12" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="13" spans="3:17">
+    <row r="13" spans="3:17" hidden="1">
       <c r="H13" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="14" spans="3:17">
+    <row r="14" spans="3:17" hidden="1">
       <c r="H14" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="15" spans="3:17">
+    <row r="15" spans="3:17" hidden="1">
       <c r="H15" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="16" spans="3:17">
+    <row r="16" spans="3:17" hidden="1">
       <c r="H16" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="17" spans="3:16">
+    <row r="17" spans="3:16" hidden="1">
       <c r="H17" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="18" spans="3:16">
+    <row r="18" spans="3:16" hidden="1">
       <c r="H18" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="19" spans="3:16">
+    <row r="19" spans="3:16" hidden="1">
       <c r="H19" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="20" spans="3:16">
+    <row r="20" spans="3:16" hidden="1">
       <c r="H20" t="s">
         <v>652</v>
       </c>
     </row>
-    <row r="21" spans="3:16">
+    <row r="21" spans="3:16" hidden="1">
       <c r="H21" t="s">
         <v>653</v>
       </c>
     </row>
-    <row r="22" spans="3:16">
+    <row r="22" spans="3:16" hidden="1">
       <c r="H22" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="23" spans="3:16" ht="112.5">
+    <row r="23" spans="3:16" ht="112.5" hidden="1">
       <c r="C23" s="2" t="s">
         <v>658</v>
       </c>
@@ -10878,42 +10935,42 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="27" spans="3:16">
+    <row r="27" spans="3:16" hidden="1">
       <c r="H27" t="s">
         <v>667</v>
       </c>
     </row>
-    <row r="28" spans="3:16">
+    <row r="28" spans="3:16" hidden="1">
       <c r="H28" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="29" spans="3:16">
+    <row r="29" spans="3:16" hidden="1">
       <c r="H29" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="30" spans="3:16">
+    <row r="30" spans="3:16" hidden="1">
       <c r="H30" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="31" spans="3:16">
+    <row r="31" spans="3:16" hidden="1">
       <c r="H31" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="32" spans="3:16">
+    <row r="32" spans="3:16" hidden="1">
       <c r="H32" t="s">
         <v>672</v>
       </c>
     </row>
-    <row r="33" spans="3:16">
+    <row r="33" spans="3:16" hidden="1">
       <c r="H33" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="34" spans="3:16" ht="112.5">
+    <row r="34" spans="3:16" ht="112.5" hidden="1">
       <c r="C34" s="2" t="s">
         <v>682</v>
       </c>
@@ -11014,107 +11071,107 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="38" spans="3:16">
+    <row r="38" spans="3:16" hidden="1">
       <c r="H38" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="39" spans="3:16">
+    <row r="39" spans="3:16" hidden="1">
       <c r="H39" t="s">
         <v>691</v>
       </c>
     </row>
-    <row r="40" spans="3:16">
+    <row r="40" spans="3:16" hidden="1">
       <c r="H40" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="41" spans="3:16">
+    <row r="41" spans="3:16" hidden="1">
       <c r="H41" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="42" spans="3:16">
+    <row r="42" spans="3:16" hidden="1">
       <c r="H42" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="43" spans="3:16">
+    <row r="43" spans="3:16" hidden="1">
       <c r="H43" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="44" spans="3:16">
+    <row r="44" spans="3:16" hidden="1">
       <c r="H44" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="45" spans="3:16">
+    <row r="45" spans="3:16" hidden="1">
       <c r="H45" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="46" spans="3:16">
+    <row r="46" spans="3:16" hidden="1">
       <c r="H46" t="s">
         <v>698</v>
       </c>
     </row>
-    <row r="47" spans="3:16">
+    <row r="47" spans="3:16" hidden="1">
       <c r="H47" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="48" spans="3:16">
+    <row r="48" spans="3:16" hidden="1">
       <c r="H48" t="s">
         <v>700</v>
       </c>
     </row>
-    <row r="49" spans="3:16">
+    <row r="49" spans="3:16" hidden="1">
       <c r="H49" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="50" spans="3:16">
+    <row r="50" spans="3:16" hidden="1">
       <c r="H50" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="51" spans="3:16">
+    <row r="51" spans="3:16" hidden="1">
       <c r="H51" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="52" spans="3:16">
+    <row r="52" spans="3:16" hidden="1">
       <c r="H52" t="s">
         <v>704</v>
       </c>
     </row>
-    <row r="53" spans="3:16">
+    <row r="53" spans="3:16" hidden="1">
       <c r="H53" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="54" spans="3:16">
+    <row r="54" spans="3:16" hidden="1">
       <c r="H54" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="55" spans="3:16">
+    <row r="55" spans="3:16" hidden="1">
       <c r="H55" t="s">
         <v>707</v>
       </c>
     </row>
-    <row r="56" spans="3:16">
+    <row r="56" spans="3:16" hidden="1">
       <c r="H56" t="s">
         <v>708</v>
       </c>
     </row>
-    <row r="57" spans="3:16">
+    <row r="57" spans="3:16" hidden="1">
       <c r="H57" t="s">
         <v>709</v>
       </c>
     </row>
-    <row r="58" spans="3:16" ht="409.5">
+    <row r="58" spans="3:16" ht="409.5" hidden="1">
       <c r="C58" s="2" t="s">
         <v>713</v>
       </c>
@@ -11215,63 +11272,63 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="62" spans="3:16">
+    <row r="62" spans="3:16" hidden="1">
       <c r="H62" t="s">
         <v>721</v>
       </c>
       <c r="J62" s="1"/>
     </row>
-    <row r="63" spans="3:16">
+    <row r="63" spans="3:16" hidden="1">
       <c r="H63" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="64" spans="3:16">
+    <row r="64" spans="3:16" hidden="1">
       <c r="H64" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="65" spans="3:16">
+    <row r="65" spans="3:16" hidden="1">
       <c r="H65" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="66" spans="3:16">
+    <row r="66" spans="3:16" hidden="1">
       <c r="H66" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="67" spans="3:16">
+    <row r="67" spans="3:16" hidden="1">
       <c r="H67" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="68" spans="3:16">
+    <row r="68" spans="3:16" hidden="1">
       <c r="H68" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="69" spans="3:16">
+    <row r="69" spans="3:16" hidden="1">
       <c r="H69" t="s">
         <v>728</v>
       </c>
     </row>
-    <row r="70" spans="3:16">
+    <row r="70" spans="3:16" hidden="1">
       <c r="H70" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="71" spans="3:16">
+    <row r="71" spans="3:16" hidden="1">
       <c r="H71" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="72" spans="3:16">
+    <row r="72" spans="3:16" hidden="1">
       <c r="H72" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="73" spans="3:16" ht="409.5">
+    <row r="73" spans="3:16" ht="409.5" hidden="1">
       <c r="C73" s="2" t="s">
         <v>735</v>
       </c>
@@ -11372,137 +11429,137 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="77" spans="3:16">
+    <row r="77" spans="3:16" hidden="1">
       <c r="H77" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="78" spans="3:16">
+    <row r="78" spans="3:16" hidden="1">
       <c r="H78" t="s">
         <v>744</v>
       </c>
     </row>
-    <row r="79" spans="3:16">
+    <row r="79" spans="3:16" hidden="1">
       <c r="H79" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="80" spans="3:16">
+    <row r="80" spans="3:16" hidden="1">
       <c r="H80" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="81" spans="8:8">
+    <row r="81" spans="8:8" hidden="1">
       <c r="H81" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="82" spans="8:8">
+    <row r="82" spans="8:8" hidden="1">
       <c r="H82" t="s">
         <v>748</v>
       </c>
     </row>
-    <row r="83" spans="8:8">
+    <row r="83" spans="8:8" hidden="1">
       <c r="H83" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="84" spans="8:8">
+    <row r="84" spans="8:8" hidden="1">
       <c r="H84" t="s">
         <v>750</v>
       </c>
     </row>
-    <row r="85" spans="8:8">
+    <row r="85" spans="8:8" hidden="1">
       <c r="H85" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="86" spans="8:8">
+    <row r="86" spans="8:8" hidden="1">
       <c r="H86" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="87" spans="8:8">
+    <row r="87" spans="8:8" hidden="1">
       <c r="H87" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="88" spans="8:8">
+    <row r="88" spans="8:8" hidden="1">
       <c r="H88" t="s">
         <v>754</v>
       </c>
     </row>
-    <row r="89" spans="8:8">
+    <row r="89" spans="8:8" hidden="1">
       <c r="H89" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="90" spans="8:8">
+    <row r="90" spans="8:8" hidden="1">
       <c r="H90" t="s">
         <v>756</v>
       </c>
     </row>
-    <row r="91" spans="8:8">
+    <row r="91" spans="8:8" hidden="1">
       <c r="H91" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="92" spans="8:8">
+    <row r="92" spans="8:8" hidden="1">
       <c r="H92" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="93" spans="8:8">
+    <row r="93" spans="8:8" hidden="1">
       <c r="H93" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="94" spans="8:8">
+    <row r="94" spans="8:8" hidden="1">
       <c r="H94" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="95" spans="8:8">
+    <row r="95" spans="8:8" hidden="1">
       <c r="H95" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="96" spans="8:8">
+    <row r="96" spans="8:8" hidden="1">
       <c r="H96" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="97" spans="3:16">
+    <row r="97" spans="3:16" hidden="1">
       <c r="H97" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="98" spans="3:16">
+    <row r="98" spans="3:16" hidden="1">
       <c r="H98" t="s">
         <v>764</v>
       </c>
     </row>
-    <row r="99" spans="3:16">
+    <row r="99" spans="3:16" hidden="1">
       <c r="H99" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="100" spans="3:16">
+    <row r="100" spans="3:16" hidden="1">
       <c r="H100" t="s">
         <v>766</v>
       </c>
     </row>
-    <row r="101" spans="3:16">
+    <row r="101" spans="3:16" hidden="1">
       <c r="H101" t="s">
         <v>767</v>
       </c>
     </row>
-    <row r="102" spans="3:16">
+    <row r="102" spans="3:16" hidden="1">
       <c r="H102" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="103" spans="3:16" ht="168.75">
+    <row r="103" spans="3:16" ht="168.75" hidden="1">
       <c r="C103" s="2" t="s">
         <v>772</v>
       </c>
@@ -11603,62 +11660,62 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="107" spans="3:16">
+    <row r="107" spans="3:16" hidden="1">
       <c r="H107" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="108" spans="3:16">
+    <row r="108" spans="3:16" hidden="1">
       <c r="H108" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="109" spans="3:16">
+    <row r="109" spans="3:16" hidden="1">
       <c r="H109" t="s">
         <v>781</v>
       </c>
     </row>
-    <row r="110" spans="3:16">
+    <row r="110" spans="3:16" hidden="1">
       <c r="H110" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="111" spans="3:16">
+    <row r="111" spans="3:16" hidden="1">
       <c r="H111" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="112" spans="3:16">
+    <row r="112" spans="3:16" hidden="1">
       <c r="H112" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="113" spans="3:13">
+    <row r="113" spans="3:13" hidden="1">
       <c r="H113" t="s">
         <v>785</v>
       </c>
     </row>
-    <row r="114" spans="3:13">
+    <row r="114" spans="3:13" hidden="1">
       <c r="H114" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="115" spans="3:13">
+    <row r="115" spans="3:13" hidden="1">
       <c r="H115" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="116" spans="3:13">
+    <row r="116" spans="3:13" hidden="1">
       <c r="H116" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="117" spans="3:13">
+    <row r="117" spans="3:13" hidden="1">
       <c r="H117" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="118" spans="3:13" ht="75">
+    <row r="118" spans="3:13" ht="75" hidden="1">
       <c r="C118" s="2" t="s">
         <v>801</v>
       </c>
@@ -11732,292 +11789,292 @@
         <v>3640</v>
       </c>
     </row>
-    <row r="122" spans="3:13">
+    <row r="122" spans="3:13" hidden="1">
       <c r="H122" t="s">
         <v>808</v>
       </c>
     </row>
-    <row r="123" spans="3:13">
+    <row r="123" spans="3:13" hidden="1">
       <c r="H123" t="s">
         <v>809</v>
       </c>
     </row>
-    <row r="124" spans="3:13">
+    <row r="124" spans="3:13" hidden="1">
       <c r="H124" t="s">
         <v>810</v>
       </c>
     </row>
-    <row r="125" spans="3:13">
+    <row r="125" spans="3:13" hidden="1">
       <c r="H125" t="s">
         <v>811</v>
       </c>
     </row>
-    <row r="126" spans="3:13">
+    <row r="126" spans="3:13" hidden="1">
       <c r="H126" t="s">
         <v>812</v>
       </c>
     </row>
-    <row r="127" spans="3:13">
+    <row r="127" spans="3:13" hidden="1">
       <c r="H127" t="s">
         <v>813</v>
       </c>
     </row>
-    <row r="128" spans="3:13">
+    <row r="128" spans="3:13" hidden="1">
       <c r="H128" t="s">
         <v>814</v>
       </c>
     </row>
-    <row r="129" spans="8:8">
+    <row r="129" spans="8:8" hidden="1">
       <c r="H129" t="s">
         <v>815</v>
       </c>
     </row>
-    <row r="130" spans="8:8">
+    <row r="130" spans="8:8" hidden="1">
       <c r="H130" t="s">
         <v>816</v>
       </c>
     </row>
-    <row r="131" spans="8:8">
+    <row r="131" spans="8:8" hidden="1">
       <c r="H131" t="s">
         <v>817</v>
       </c>
     </row>
-    <row r="132" spans="8:8">
+    <row r="132" spans="8:8" hidden="1">
       <c r="H132" t="s">
         <v>818</v>
       </c>
     </row>
-    <row r="133" spans="8:8">
+    <row r="133" spans="8:8" hidden="1">
       <c r="H133" t="s">
         <v>819</v>
       </c>
     </row>
-    <row r="134" spans="8:8">
+    <row r="134" spans="8:8" hidden="1">
       <c r="H134" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="135" spans="8:8">
+    <row r="135" spans="8:8" hidden="1">
       <c r="H135" t="s">
         <v>820</v>
       </c>
     </row>
-    <row r="136" spans="8:8">
+    <row r="136" spans="8:8" hidden="1">
       <c r="H136" t="s">
         <v>821</v>
       </c>
     </row>
-    <row r="137" spans="8:8">
+    <row r="137" spans="8:8" hidden="1">
       <c r="H137" t="s">
         <v>822</v>
       </c>
     </row>
-    <row r="138" spans="8:8">
+    <row r="138" spans="8:8" hidden="1">
       <c r="H138" t="s">
         <v>823</v>
       </c>
     </row>
-    <row r="139" spans="8:8">
+    <row r="139" spans="8:8" hidden="1">
       <c r="H139" t="s">
         <v>824</v>
       </c>
     </row>
-    <row r="140" spans="8:8">
+    <row r="140" spans="8:8" hidden="1">
       <c r="H140" t="s">
         <v>825</v>
       </c>
     </row>
-    <row r="141" spans="8:8">
+    <row r="141" spans="8:8" hidden="1">
       <c r="H141" t="s">
         <v>826</v>
       </c>
     </row>
-    <row r="142" spans="8:8">
+    <row r="142" spans="8:8" hidden="1">
       <c r="H142" t="s">
         <v>827</v>
       </c>
     </row>
-    <row r="143" spans="8:8">
+    <row r="143" spans="8:8" hidden="1">
       <c r="H143" t="s">
         <v>828</v>
       </c>
     </row>
-    <row r="144" spans="8:8">
+    <row r="144" spans="8:8" hidden="1">
       <c r="H144" t="s">
         <v>829</v>
       </c>
     </row>
-    <row r="145" spans="8:8">
+    <row r="145" spans="8:8" hidden="1">
       <c r="H145" t="s">
         <v>830</v>
       </c>
     </row>
-    <row r="146" spans="8:8">
+    <row r="146" spans="8:8" hidden="1">
       <c r="H146" t="s">
         <v>831</v>
       </c>
     </row>
-    <row r="147" spans="8:8">
+    <row r="147" spans="8:8" hidden="1">
       <c r="H147" t="s">
         <v>832</v>
       </c>
     </row>
-    <row r="148" spans="8:8">
+    <row r="148" spans="8:8" hidden="1">
       <c r="H148" t="s">
         <v>833</v>
       </c>
     </row>
-    <row r="149" spans="8:8">
+    <row r="149" spans="8:8" hidden="1">
       <c r="H149" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="150" spans="8:8">
+    <row r="150" spans="8:8" hidden="1">
       <c r="H150" t="s">
         <v>835</v>
       </c>
     </row>
-    <row r="151" spans="8:8">
+    <row r="151" spans="8:8" hidden="1">
       <c r="H151" t="s">
         <v>836</v>
       </c>
     </row>
-    <row r="152" spans="8:8">
+    <row r="152" spans="8:8" hidden="1">
       <c r="H152" t="s">
         <v>837</v>
       </c>
     </row>
-    <row r="153" spans="8:8">
+    <row r="153" spans="8:8" hidden="1">
       <c r="H153" t="s">
         <v>838</v>
       </c>
     </row>
-    <row r="154" spans="8:8">
+    <row r="154" spans="8:8" hidden="1">
       <c r="H154" t="s">
         <v>839</v>
       </c>
     </row>
-    <row r="155" spans="8:8">
+    <row r="155" spans="8:8" hidden="1">
       <c r="H155" t="s">
         <v>840</v>
       </c>
     </row>
-    <row r="156" spans="8:8">
+    <row r="156" spans="8:8" hidden="1">
       <c r="H156" t="s">
         <v>841</v>
       </c>
     </row>
-    <row r="157" spans="8:8">
+    <row r="157" spans="8:8" hidden="1">
       <c r="H157" t="s">
         <v>842</v>
       </c>
     </row>
-    <row r="158" spans="8:8">
+    <row r="158" spans="8:8" hidden="1">
       <c r="H158" t="s">
         <v>843</v>
       </c>
     </row>
-    <row r="159" spans="8:8">
+    <row r="159" spans="8:8" hidden="1">
       <c r="H159" t="s">
         <v>844</v>
       </c>
     </row>
-    <row r="160" spans="8:8">
+    <row r="160" spans="8:8" hidden="1">
       <c r="H160" t="s">
         <v>845</v>
       </c>
     </row>
-    <row r="161" spans="8:8">
+    <row r="161" spans="8:8" hidden="1">
       <c r="H161" t="s">
         <v>846</v>
       </c>
     </row>
-    <row r="162" spans="8:8">
+    <row r="162" spans="8:8" hidden="1">
       <c r="H162" t="s">
         <v>847</v>
       </c>
     </row>
-    <row r="163" spans="8:8">
+    <row r="163" spans="8:8" hidden="1">
       <c r="H163" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="164" spans="8:8">
+    <row r="164" spans="8:8" hidden="1">
       <c r="H164" t="s">
         <v>849</v>
       </c>
     </row>
-    <row r="165" spans="8:8">
+    <row r="165" spans="8:8" hidden="1">
       <c r="H165" t="s">
         <v>850</v>
       </c>
     </row>
-    <row r="166" spans="8:8">
+    <row r="166" spans="8:8" hidden="1">
       <c r="H166" t="s">
         <v>851</v>
       </c>
     </row>
-    <row r="167" spans="8:8">
+    <row r="167" spans="8:8" hidden="1">
       <c r="H167" t="s">
         <v>852</v>
       </c>
     </row>
-    <row r="168" spans="8:8">
+    <row r="168" spans="8:8" hidden="1">
       <c r="H168" t="s">
         <v>853</v>
       </c>
     </row>
-    <row r="169" spans="8:8">
+    <row r="169" spans="8:8" hidden="1">
       <c r="H169" t="s">
         <v>854</v>
       </c>
     </row>
-    <row r="170" spans="8:8">
+    <row r="170" spans="8:8" hidden="1">
       <c r="H170" t="s">
         <v>855</v>
       </c>
     </row>
-    <row r="171" spans="8:8">
+    <row r="171" spans="8:8" hidden="1">
       <c r="H171" t="s">
         <v>856</v>
       </c>
     </row>
-    <row r="172" spans="8:8">
+    <row r="172" spans="8:8" hidden="1">
       <c r="H172" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="173" spans="8:8">
+    <row r="173" spans="8:8" hidden="1">
       <c r="H173" t="s">
         <v>858</v>
       </c>
     </row>
-    <row r="174" spans="8:8">
+    <row r="174" spans="8:8" hidden="1">
       <c r="H174" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="175" spans="8:8">
+    <row r="175" spans="8:8" hidden="1">
       <c r="H175" t="s">
         <v>860</v>
       </c>
     </row>
-    <row r="176" spans="8:8">
+    <row r="176" spans="8:8" hidden="1">
       <c r="H176" t="s">
         <v>861</v>
       </c>
     </row>
-    <row r="177" spans="3:13">
+    <row r="177" spans="3:13" hidden="1">
       <c r="H177" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="178" spans="3:13">
+    <row r="178" spans="3:13" hidden="1">
       <c r="H178" t="s">
         <v>863</v>
       </c>
     </row>
-    <row r="179" spans="3:13" ht="168.75">
+    <row r="179" spans="3:13" ht="168.75" hidden="1">
       <c r="C179" s="2" t="s">
         <v>868</v>
       </c>
@@ -12082,7 +12139,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="183" spans="3:13" ht="168.75">
+    <row r="183" spans="3:13" ht="168.75" hidden="1">
       <c r="C183" s="2" t="s">
         <v>877</v>
       </c>
@@ -12167,42 +12224,42 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="188" spans="3:13">
+    <row r="188" spans="3:13" hidden="1">
       <c r="H188" t="s">
         <v>885</v>
       </c>
     </row>
-    <row r="189" spans="3:13">
+    <row r="189" spans="3:13" hidden="1">
       <c r="H189" t="s">
         <v>886</v>
       </c>
     </row>
-    <row r="190" spans="3:13">
+    <row r="190" spans="3:13" hidden="1">
       <c r="H190" t="s">
         <v>887</v>
       </c>
     </row>
-    <row r="191" spans="3:13">
+    <row r="191" spans="3:13" hidden="1">
       <c r="H191" t="s">
         <v>888</v>
       </c>
     </row>
-    <row r="192" spans="3:13">
+    <row r="192" spans="3:13" hidden="1">
       <c r="H192" t="s">
         <v>889</v>
       </c>
     </row>
-    <row r="193" spans="3:13">
+    <row r="193" spans="3:13" hidden="1">
       <c r="H193" t="s">
         <v>890</v>
       </c>
     </row>
-    <row r="194" spans="3:13">
+    <row r="194" spans="3:13" hidden="1">
       <c r="H194" t="s">
         <v>891</v>
       </c>
     </row>
-    <row r="195" spans="3:13" ht="409.5">
+    <row r="195" spans="3:13" ht="409.5" hidden="1">
       <c r="C195" s="2" t="s">
         <v>895</v>
       </c>
@@ -12276,52 +12333,52 @@
         <v>3642</v>
       </c>
     </row>
-    <row r="199" spans="3:13">
+    <row r="199" spans="3:13" hidden="1">
       <c r="H199" t="s">
         <v>903</v>
       </c>
     </row>
-    <row r="200" spans="3:13">
+    <row r="200" spans="3:13" hidden="1">
       <c r="H200" t="s">
         <v>904</v>
       </c>
     </row>
-    <row r="201" spans="3:13">
+    <row r="201" spans="3:13" hidden="1">
       <c r="H201" t="s">
         <v>905</v>
       </c>
     </row>
-    <row r="202" spans="3:13">
+    <row r="202" spans="3:13" hidden="1">
       <c r="H202" t="s">
         <v>906</v>
       </c>
     </row>
-    <row r="203" spans="3:13">
+    <row r="203" spans="3:13" hidden="1">
       <c r="H203" t="s">
         <v>907</v>
       </c>
     </row>
-    <row r="204" spans="3:13">
+    <row r="204" spans="3:13" hidden="1">
       <c r="H204" t="s">
         <v>908</v>
       </c>
     </row>
-    <row r="205" spans="3:13">
+    <row r="205" spans="3:13" hidden="1">
       <c r="H205" t="s">
         <v>909</v>
       </c>
     </row>
-    <row r="206" spans="3:13">
+    <row r="206" spans="3:13" hidden="1">
       <c r="H206" t="s">
         <v>910</v>
       </c>
     </row>
-    <row r="207" spans="3:13">
+    <row r="207" spans="3:13" hidden="1">
       <c r="H207" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="208" spans="3:13" ht="150">
+    <row r="208" spans="3:13" ht="150" hidden="1">
       <c r="C208" s="2" t="s">
         <v>916</v>
       </c>
@@ -12338,7 +12395,7 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="209" spans="3:10" ht="37.5">
+    <row r="209" spans="3:11" ht="37.5">
       <c r="F209" s="1" t="s">
         <v>920</v>
       </c>
@@ -12351,149 +12408,285 @@
       <c r="J209" s="2" t="s">
         <v>921</v>
       </c>
-    </row>
-    <row r="210" spans="3:10" ht="93.75">
+      <c r="K209" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="210" spans="3:11" ht="168.75" hidden="1">
       <c r="C210" s="2" t="s">
+        <v>960</v>
+      </c>
+      <c r="D210" t="s">
+        <v>961</v>
+      </c>
+      <c r="E210" s="1" t="s">
+        <v>962</v>
+      </c>
+      <c r="F210" s="1" t="s">
+        <v>963</v>
+      </c>
+      <c r="G210" s="3"/>
+      <c r="I210" s="1"/>
+      <c r="J210" s="2"/>
+    </row>
+    <row r="211" spans="3:11" hidden="1">
+      <c r="C211" s="2"/>
+      <c r="E211" s="1"/>
+      <c r="F211" s="1" t="s">
+        <v>964</v>
+      </c>
+      <c r="G211" s="3">
+        <v>46071</v>
+      </c>
+      <c r="I211" s="1"/>
+      <c r="J211" s="2"/>
+    </row>
+    <row r="212" spans="3:11" ht="37.5">
+      <c r="C212" s="2"/>
+      <c r="E212" s="1"/>
+      <c r="F212" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="G212" s="3">
+        <v>46071</v>
+      </c>
+      <c r="I212" s="1" t="s">
+        <v>873</v>
+      </c>
+      <c r="J212" s="2" t="s">
+        <v>966</v>
+      </c>
+      <c r="K212" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="213" spans="3:11">
+      <c r="C213" s="2"/>
+      <c r="E213" s="1"/>
+      <c r="F213" s="1"/>
+      <c r="G213" s="3"/>
+      <c r="I213" s="1"/>
+      <c r="J213" s="2" t="s">
+        <v>967</v>
+      </c>
+      <c r="K213" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="214" spans="3:11">
+      <c r="C214" s="2"/>
+      <c r="E214" s="1"/>
+      <c r="F214" s="1"/>
+      <c r="G214" s="3"/>
+      <c r="I214" s="1"/>
+      <c r="J214" s="2" t="s">
+        <v>968</v>
+      </c>
+      <c r="K214" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="215" spans="3:11" ht="93.75" hidden="1">
+      <c r="C215" s="2" t="s">
         <v>922</v>
       </c>
-      <c r="D210" t="s">
+      <c r="D215" t="s">
         <v>923</v>
       </c>
-      <c r="E210" s="1" t="s">
+      <c r="E215" s="1" t="s">
         <v>924</v>
       </c>
-      <c r="F210" t="s">
+      <c r="F215" t="s">
         <v>926</v>
       </c>
-      <c r="I210" t="s">
+      <c r="I215" t="s">
         <v>929</v>
       </c>
     </row>
-    <row r="211" spans="3:10" ht="262.5">
-      <c r="E211" s="1" t="s">
+    <row r="216" spans="3:11" ht="262.5" hidden="1">
+      <c r="E216" s="1" t="s">
         <v>925</v>
       </c>
-      <c r="F211" s="1" t="s">
+      <c r="F216" s="1" t="s">
         <v>927</v>
       </c>
-      <c r="I211" s="1" t="s">
+      <c r="I216" s="1" t="s">
         <v>928</v>
       </c>
-    </row>
-    <row r="212" spans="3:10" ht="243.75">
-      <c r="F212" s="1" t="s">
+      <c r="J216" s="1" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="217" spans="3:11" ht="243.75" hidden="1">
+      <c r="F217" s="1" t="s">
         <v>930</v>
       </c>
-      <c r="I212" s="1" t="s">
+      <c r="I217" s="1" t="s">
+        <v>959</v>
+      </c>
+      <c r="J217" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="218" spans="3:11" ht="337.5" hidden="1">
+      <c r="F218" s="1" t="s">
         <v>931</v>
       </c>
-    </row>
-    <row r="213" spans="3:10" ht="337.5">
-      <c r="F213" s="1" t="s">
+      <c r="I218" s="1" t="s">
         <v>932</v>
       </c>
-      <c r="I213" s="1" t="s">
+      <c r="J218" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="219" spans="3:11" ht="206.25" hidden="1">
+      <c r="F219" s="1" t="s">
         <v>933</v>
       </c>
-    </row>
-    <row r="214" spans="3:10" ht="206.25">
-      <c r="F214" s="1" t="s">
+      <c r="I219" s="1" t="s">
         <v>934</v>
       </c>
-      <c r="I214" s="1" t="s">
+      <c r="J219" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="220" spans="3:11" ht="75" hidden="1">
+      <c r="F220" s="1" t="s">
         <v>935</v>
       </c>
-    </row>
-    <row r="215" spans="3:10" ht="75">
-      <c r="F215" s="1" t="s">
+      <c r="I220" s="1" t="s">
         <v>936</v>
       </c>
-      <c r="I215" s="1" t="s">
+      <c r="J220" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="221" spans="3:11" ht="56.25" hidden="1">
+      <c r="F221" s="1" t="s">
         <v>937</v>
       </c>
-    </row>
-    <row r="216" spans="3:10" ht="56.25">
-      <c r="F216" s="1" t="s">
+      <c r="I221" s="1" t="s">
         <v>938</v>
       </c>
-      <c r="I216" s="1" t="s">
+      <c r="J221" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="222" spans="3:11" ht="243.75" hidden="1">
+      <c r="F222" s="1" t="s">
         <v>939</v>
       </c>
-    </row>
-    <row r="217" spans="3:10" ht="243.75">
-      <c r="F217" s="1" t="s">
+      <c r="I222" s="1" t="s">
         <v>940</v>
       </c>
-      <c r="I217" s="1" t="s">
+      <c r="J222" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="223" spans="3:11" ht="75" hidden="1">
+      <c r="F223" s="1" t="s">
         <v>941</v>
       </c>
-    </row>
-    <row r="218" spans="3:10" ht="75">
-      <c r="F218" s="1" t="s">
+      <c r="I223" s="1" t="s">
         <v>942</v>
       </c>
-      <c r="I218" s="1" t="s">
+      <c r="J223" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="224" spans="3:11" ht="168.75" hidden="1">
+      <c r="F224" s="1" t="s">
         <v>943</v>
       </c>
-    </row>
-    <row r="219" spans="3:10" ht="168.75">
-      <c r="F219" s="1" t="s">
+      <c r="I224" s="1" t="s">
         <v>944</v>
       </c>
-      <c r="I219" s="1" t="s">
+      <c r="J224" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="225" spans="6:10" ht="112.5" hidden="1">
+      <c r="F225" s="1" t="s">
         <v>945</v>
       </c>
-    </row>
-    <row r="220" spans="3:10" ht="112.5">
-      <c r="F220" s="1" t="s">
+      <c r="I225" s="1" t="s">
         <v>946</v>
       </c>
-      <c r="I220" s="1" t="s">
+      <c r="J225" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="226" spans="6:10" ht="131.25" hidden="1">
+      <c r="F226" s="1" t="s">
         <v>947</v>
       </c>
-    </row>
-    <row r="221" spans="3:10" ht="131.25">
-      <c r="F221" s="1" t="s">
+      <c r="I226" s="1" t="s">
         <v>948</v>
       </c>
-      <c r="I221" s="1" t="s">
+      <c r="J226" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="227" spans="6:10" ht="131.25" hidden="1">
+      <c r="F227" s="1" t="s">
         <v>949</v>
       </c>
-    </row>
-    <row r="222" spans="3:10" ht="131.25">
-      <c r="F222" s="1" t="s">
+      <c r="I227" s="1" t="s">
         <v>950</v>
       </c>
-      <c r="I222" s="1" t="s">
+      <c r="J227" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="228" spans="6:10" ht="37.5" hidden="1">
+      <c r="F228" s="1" t="s">
         <v>951</v>
       </c>
-    </row>
-    <row r="223" spans="3:10" ht="37.5">
-      <c r="F223" s="1" t="s">
+      <c r="I228" s="1" t="s">
         <v>952</v>
       </c>
-      <c r="I223" s="1" t="s">
+      <c r="J228" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="229" spans="6:10" ht="206.25" hidden="1">
+      <c r="F229" s="1" t="s">
         <v>953</v>
       </c>
-    </row>
-    <row r="224" spans="3:10" ht="206.25">
-      <c r="F224" s="1" t="s">
+      <c r="I229" s="1" t="s">
         <v>954</v>
       </c>
-      <c r="I224" s="1" t="s">
+      <c r="J229" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="230" spans="6:10" ht="168.75" hidden="1">
+      <c r="F230" s="1" t="s">
         <v>955</v>
       </c>
-    </row>
-    <row r="225" spans="6:9" ht="168.75">
-      <c r="F225" s="1" t="s">
+      <c r="I230" s="1" t="s">
         <v>956</v>
       </c>
-      <c r="I225" s="1" t="s">
+      <c r="J230" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="231" spans="6:10" ht="37.5" hidden="1">
+      <c r="F231" s="1" t="s">
         <v>957</v>
       </c>
+      <c r="I231" s="1" t="s">
+        <v>958</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="C2:M207" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}"/>
+  <autoFilter ref="C2:M231" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
+    <filterColumn colId="8">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="1"/>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" xr:uid="{C897C6D6-16A8-4618-9776-831A651C49AE}"/>
@@ -12512,7 +12705,11 @@
     <hyperlink ref="C195" r:id="rId14" xr:uid="{39E432C6-4E9C-4343-9815-52F316B64658}"/>
     <hyperlink ref="C208" r:id="rId15" xr:uid="{3BB45995-7DA2-4F11-900F-84AFACB633B1}"/>
     <hyperlink ref="J209" r:id="rId16" xr:uid="{9220184A-77DE-47EA-97A3-9205D7952A4A}"/>
-    <hyperlink ref="C210" r:id="rId17" xr:uid="{90934316-82E9-4DC7-B9EE-F6BEE341122B}"/>
+    <hyperlink ref="C215" r:id="rId17" xr:uid="{90934316-82E9-4DC7-B9EE-F6BEE341122B}"/>
+    <hyperlink ref="C210" r:id="rId18" xr:uid="{5BDF6C17-4D24-458A-9CF3-B882D353E8DA}"/>
+    <hyperlink ref="J212" r:id="rId19" xr:uid="{71F52FA6-1FAB-4126-B29F-1E7E41C83F60}"/>
+    <hyperlink ref="J213" r:id="rId20" xr:uid="{C2906471-C6FC-4CA7-A604-3B66D9D2AFFA}"/>
+    <hyperlink ref="J214" r:id="rId21" xr:uid="{E558B1F8-18E8-46BA-834A-9F0F97BEF2FC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12520,7 +12717,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970790C5-0376-420E-A317-55DF989D7F43}">
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultColWidth="73.25" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="77.5" bestFit="1" customWidth="1"/>
@@ -12534,7 +12731,10 @@
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>635</v>
+      </c>
       <c r="B1" t="s">
         <v>674</v>
       </c>
@@ -12560,50 +12760,59 @@
         <v>915</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
-      <c r="A2" s="2" t="s">
-        <v>876</v>
+    <row r="2" spans="1:10" ht="56.25">
+      <c r="A2" s="1" t="s">
+        <v>655</v>
       </c>
       <c r="B2" s="3">
-        <v>46068</v>
+        <v>46066</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D2">
+        <v>3642</v>
+      </c>
+      <c r="E2" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F2">
+        <v>136</v>
+      </c>
+      <c r="G2">
+        <v>3649</v>
+      </c>
+      <c r="H2">
+        <v>2</v>
+      </c>
+      <c r="I2">
+        <v>3</v>
+      </c>
+      <c r="J2" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="206.25">
+      <c r="A3" s="1" t="s">
+        <v>656</v>
+      </c>
+      <c r="B3" s="3">
+        <v>46066</v>
+      </c>
+      <c r="C3">
+        <v>19</v>
+      </c>
+      <c r="D3">
+        <v>3642</v>
+      </c>
+      <c r="E3" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F3">
+        <v>33</v>
+      </c>
+      <c r="G3">
         <v>3639</v>
-      </c>
-      <c r="F2">
-        <v>10</v>
-      </c>
-      <c r="G2">
-        <v>3643</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" ht="112.5">
-      <c r="A3" s="1" t="s">
-        <v>893</v>
-      </c>
-      <c r="B3" s="3">
-        <v>46068</v>
-      </c>
-      <c r="C3">
-        <v>3</v>
-      </c>
-      <c r="D3">
-        <v>3639</v>
-      </c>
-      <c r="F3">
-        <v>13</v>
-      </c>
-      <c r="G3">
-        <v>3643</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -12612,171 +12821,171 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="75">
+    <row r="4" spans="1:10" ht="56.25">
       <c r="A4" s="1" t="s">
-        <v>894</v>
+        <v>657</v>
       </c>
       <c r="B4" s="3">
-        <v>46068</v>
+        <v>46066</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D4">
+        <v>3642</v>
+      </c>
+      <c r="E4" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F4">
+        <v>29</v>
+      </c>
+      <c r="G4">
         <v>3639</v>
-      </c>
-      <c r="F4">
-        <v>13</v>
-      </c>
-      <c r="G4">
-        <v>3643</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
       </c>
       <c r="I4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="93.75">
+    <row r="5" spans="1:10" ht="75">
       <c r="A5" s="1" t="s">
-        <v>866</v>
+        <v>679</v>
       </c>
       <c r="B5" s="3">
-        <v>46068</v>
+        <v>46066</v>
       </c>
       <c r="C5">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="D5">
-        <v>3640</v>
+        <v>3642</v>
+      </c>
+      <c r="E5" s="3">
+        <v>46067</v>
       </c>
       <c r="F5">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="G5">
-        <v>3643</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
+        <v>3639</v>
       </c>
       <c r="I5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="2" t="s">
-        <v>874</v>
+    <row r="6" spans="1:10" ht="262.5">
+      <c r="A6" s="1" t="s">
+        <v>680</v>
       </c>
       <c r="B6" s="3">
-        <v>46068</v>
+        <v>46066</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D6">
+        <v>3642</v>
+      </c>
+      <c r="E6" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F6">
+        <v>32</v>
+      </c>
+      <c r="G6">
         <v>3639</v>
-      </c>
-      <c r="F6">
-        <v>14</v>
-      </c>
-      <c r="G6">
-        <v>3643</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
       </c>
       <c r="I6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="2" t="s">
-        <v>875</v>
+    <row r="7" spans="1:10" ht="75">
+      <c r="A7" s="1" t="s">
+        <v>681</v>
       </c>
       <c r="B7" s="3">
-        <v>46068</v>
+        <v>46066</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D7">
+        <v>3642</v>
+      </c>
+      <c r="E7" s="3">
+        <v>46067</v>
+      </c>
+      <c r="F7">
+        <v>36</v>
+      </c>
+      <c r="G7">
         <v>3639</v>
-      </c>
-      <c r="F7">
-        <v>14</v>
-      </c>
-      <c r="G7">
-        <v>3643</v>
-      </c>
-      <c r="H7">
-        <v>1</v>
       </c>
       <c r="I7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="93.75">
+    <row r="8" spans="1:10" ht="93.75">
       <c r="A8" s="1" t="s">
-        <v>865</v>
+        <v>710</v>
       </c>
       <c r="B8" s="3">
-        <v>46068</v>
+        <v>46066</v>
       </c>
       <c r="C8">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D8">
-        <v>3640</v>
+        <v>3642</v>
+      </c>
+      <c r="E8" s="3">
+        <v>46067</v>
       </c>
       <c r="F8">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G8">
-        <v>3643</v>
-      </c>
-      <c r="H8">
-        <v>1</v>
+        <v>3639</v>
       </c>
       <c r="I8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="75">
+    <row r="9" spans="1:10" ht="75">
       <c r="A9" s="1" t="s">
-        <v>867</v>
+        <v>711</v>
       </c>
       <c r="B9" s="3">
-        <v>46068</v>
+        <v>46066</v>
       </c>
       <c r="C9">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D9">
-        <v>3640</v>
+        <v>3642</v>
+      </c>
+      <c r="E9" s="3">
+        <v>46067</v>
       </c>
       <c r="F9">
-        <v>20</v>
+        <v>42</v>
       </c>
       <c r="G9">
-        <v>3643</v>
-      </c>
-      <c r="H9">
-        <v>1</v>
+        <v>3639</v>
       </c>
       <c r="I9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="168.75">
+    <row r="10" spans="1:10" ht="75">
       <c r="A10" s="1" t="s">
-        <v>790</v>
+        <v>712</v>
       </c>
       <c r="B10" s="3">
         <v>46066</v>
       </c>
       <c r="C10">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D10">
         <v>3642</v>
@@ -12785,19 +12994,16 @@
         <v>46067</v>
       </c>
       <c r="F10">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G10">
         <v>3639</v>
       </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
       <c r="I10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="93.75">
+    <row r="11" spans="1:10" ht="93.75">
       <c r="A11" s="1" t="s">
         <v>732</v>
       </c>
@@ -12814,27 +13020,24 @@
         <v>46067</v>
       </c>
       <c r="F11">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G11">
         <v>3639</v>
       </c>
-      <c r="H11">
-        <v>1</v>
-      </c>
       <c r="I11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="75">
+    <row r="12" spans="1:10" ht="187.5">
       <c r="A12" s="1" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="B12" s="3">
         <v>46066</v>
       </c>
       <c r="C12">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D12">
         <v>3642</v>
@@ -12848,22 +13051,19 @@
       <c r="G12">
         <v>3639</v>
       </c>
-      <c r="H12">
-        <v>1</v>
-      </c>
       <c r="I12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="75">
+    <row r="13" spans="1:10" ht="75">
       <c r="A13" s="1" t="s">
-        <v>770</v>
+        <v>734</v>
       </c>
       <c r="B13" s="3">
         <v>46066</v>
       </c>
       <c r="C13">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D13">
         <v>3642</v>
@@ -12872,27 +13072,24 @@
         <v>46067</v>
       </c>
       <c r="F13">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="G13">
         <v>3639</v>
       </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
       <c r="I13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="93.75">
+    <row r="14" spans="1:10" ht="93.75">
       <c r="A14" s="1" t="s">
-        <v>792</v>
+        <v>769</v>
       </c>
       <c r="B14" s="3">
         <v>46066</v>
       </c>
       <c r="C14">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="D14">
         <v>3642</v>
@@ -12901,27 +13098,24 @@
         <v>46067</v>
       </c>
       <c r="F14">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G14">
         <v>3639</v>
       </c>
-      <c r="H14">
-        <v>1</v>
-      </c>
       <c r="I14">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="93.75">
+    <row r="15" spans="1:10" ht="75">
       <c r="A15" s="1" t="s">
-        <v>710</v>
+        <v>770</v>
       </c>
       <c r="B15" s="3">
         <v>46066</v>
       </c>
       <c r="C15">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D15">
         <v>3642</v>
@@ -12930,53 +13124,50 @@
         <v>46067</v>
       </c>
       <c r="F15">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G15">
         <v>3639</v>
       </c>
-      <c r="H15">
-        <v>1</v>
-      </c>
       <c r="I15">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="75">
+    <row r="16" spans="1:10" ht="75">
       <c r="A16" s="1" t="s">
-        <v>912</v>
+        <v>771</v>
       </c>
       <c r="B16" s="3">
-        <v>46069</v>
+        <v>46066</v>
       </c>
       <c r="C16">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D16">
         <v>3642</v>
       </c>
+      <c r="E16" s="3">
+        <v>46067</v>
+      </c>
       <c r="F16">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G16">
-        <v>3643</v>
-      </c>
-      <c r="H16">
-        <v>1</v>
+        <v>3639</v>
       </c>
       <c r="I16">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="75">
+    <row r="17" spans="1:10" ht="168.75">
       <c r="A17" s="1" t="s">
-        <v>712</v>
+        <v>790</v>
       </c>
       <c r="B17" s="3">
         <v>46066</v>
       </c>
       <c r="C17">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="D17">
         <v>3642</v>
@@ -12985,27 +13176,24 @@
         <v>46067</v>
       </c>
       <c r="F17">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="G17">
         <v>3639</v>
       </c>
-      <c r="H17">
-        <v>1</v>
-      </c>
       <c r="I17">
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="187.5">
+    <row r="18" spans="1:10" ht="150">
       <c r="A18" s="1" t="s">
-        <v>733</v>
+        <v>791</v>
       </c>
       <c r="B18" s="3">
         <v>46066</v>
       </c>
       <c r="C18">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="D18">
         <v>3642</v>
@@ -13014,27 +13202,24 @@
         <v>46067</v>
       </c>
       <c r="F18">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G18">
         <v>3639</v>
       </c>
-      <c r="H18">
-        <v>1</v>
-      </c>
       <c r="I18">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="56.25">
+    <row r="19" spans="1:10" ht="93.75">
       <c r="A19" s="1" t="s">
-        <v>657</v>
+        <v>792</v>
       </c>
       <c r="B19" s="3">
         <v>46066</v>
       </c>
       <c r="C19">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="D19">
         <v>3642</v>
@@ -13043,65 +13228,44 @@
         <v>46067</v>
       </c>
       <c r="F19">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G19">
         <v>3639</v>
       </c>
-      <c r="H19">
-        <v>1</v>
-      </c>
       <c r="I19">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="56.25">
+    <row r="20" spans="1:10" ht="93.75">
       <c r="A20" s="1" t="s">
-        <v>914</v>
+        <v>865</v>
       </c>
       <c r="B20" s="3">
-        <v>46069</v>
+        <v>46068</v>
       </c>
       <c r="C20">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="D20">
-        <v>3642</v>
-      </c>
-      <c r="F20">
-        <v>32</v>
-      </c>
-      <c r="G20">
-        <v>3643</v>
-      </c>
-      <c r="H20">
-        <v>1</v>
+        <v>3640</v>
       </c>
       <c r="I20">
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="75">
+    <row r="21" spans="1:10" ht="93.75">
       <c r="A21" s="1" t="s">
-        <v>913</v>
+        <v>866</v>
       </c>
       <c r="B21" s="3">
-        <v>46069</v>
+        <v>46068</v>
       </c>
       <c r="C21">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D21">
-        <v>3642</v>
-      </c>
-      <c r="F21">
-        <v>33</v>
-      </c>
-      <c r="G21">
-        <v>3643</v>
-      </c>
-      <c r="H21">
-        <v>1</v>
+        <v>3640</v>
       </c>
       <c r="I21">
         <v>1</v>
@@ -13109,228 +13273,129 @@
     </row>
     <row r="22" spans="1:10" ht="75">
       <c r="A22" s="1" t="s">
-        <v>771</v>
+        <v>867</v>
       </c>
       <c r="B22" s="3">
-        <v>46066</v>
+        <v>46068</v>
       </c>
       <c r="C22">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D22">
-        <v>3642</v>
-      </c>
-      <c r="E22" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F22">
-        <v>34</v>
-      </c>
-      <c r="G22">
-        <v>3639</v>
-      </c>
-      <c r="H22">
-        <v>1</v>
+        <v>3640</v>
       </c>
       <c r="I22">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="93.75">
-      <c r="A23" s="1" t="s">
-        <v>769</v>
+    <row r="23" spans="1:10">
+      <c r="A23" s="2" t="s">
+        <v>874</v>
       </c>
       <c r="B23" s="3">
-        <v>46066</v>
+        <v>46068</v>
       </c>
       <c r="C23">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="D23">
-        <v>3642</v>
-      </c>
-      <c r="E23" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F23">
-        <v>35</v>
-      </c>
-      <c r="G23">
         <v>3639</v>
-      </c>
-      <c r="H23">
-        <v>1</v>
       </c>
       <c r="I23">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="206.25">
-      <c r="A24" s="1" t="s">
-        <v>656</v>
+    <row r="24" spans="1:10">
+      <c r="A24" s="2" t="s">
+        <v>875</v>
       </c>
       <c r="B24" s="3">
-        <v>46066</v>
+        <v>46068</v>
       </c>
       <c r="C24">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="D24">
-        <v>3642</v>
-      </c>
-      <c r="E24" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F24">
-        <v>37</v>
-      </c>
-      <c r="G24">
         <v>3639</v>
-      </c>
-      <c r="H24">
-        <v>2</v>
       </c>
       <c r="I24">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="262.5">
-      <c r="A25" s="1" t="s">
-        <v>680</v>
+    <row r="25" spans="1:10">
+      <c r="A25" s="2" t="s">
+        <v>876</v>
       </c>
       <c r="B25" s="3">
-        <v>46066</v>
+        <v>46068</v>
       </c>
       <c r="C25">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="D25">
-        <v>3642</v>
-      </c>
-      <c r="E25" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F25">
-        <v>37</v>
-      </c>
-      <c r="G25">
         <v>3639</v>
-      </c>
-      <c r="H25">
-        <v>1</v>
       </c>
       <c r="I25">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="150">
+    <row r="26" spans="1:10" ht="112.5">
       <c r="A26" s="1" t="s">
-        <v>791</v>
+        <v>892</v>
       </c>
       <c r="B26" s="3">
-        <v>46066</v>
+        <v>46068</v>
       </c>
       <c r="C26">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D26">
-        <v>3642</v>
-      </c>
-      <c r="E26" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F26">
-        <v>37</v>
-      </c>
-      <c r="G26">
         <v>3639</v>
-      </c>
-      <c r="H26">
-        <v>1</v>
       </c>
       <c r="I26">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="75">
+    <row r="27" spans="1:10" ht="112.5">
       <c r="A27" s="1" t="s">
-        <v>679</v>
+        <v>893</v>
       </c>
       <c r="B27" s="3">
-        <v>46066</v>
+        <v>46068</v>
       </c>
       <c r="C27">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="D27">
-        <v>3642</v>
-      </c>
-      <c r="E27" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F27">
-        <v>38</v>
-      </c>
-      <c r="G27">
         <v>3639</v>
-      </c>
-      <c r="H27">
-        <v>1</v>
       </c>
       <c r="I27">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="112.5">
+    <row r="28" spans="1:10" ht="75">
       <c r="A28" s="1" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="B28" s="3">
         <v>46068</v>
       </c>
       <c r="C28">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D28">
         <v>3639</v>
       </c>
-      <c r="F28">
-        <v>39</v>
-      </c>
-      <c r="G28">
-        <v>3643</v>
-      </c>
-      <c r="H28">
-        <v>2</v>
-      </c>
       <c r="I28">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="75">
+    <row r="29" spans="1:10">
       <c r="A29" s="1" t="s">
-        <v>681</v>
+        <v>899</v>
       </c>
       <c r="B29" s="3">
-        <v>46066</v>
-      </c>
-      <c r="C29">
-        <v>28</v>
-      </c>
-      <c r="D29">
-        <v>3642</v>
-      </c>
-      <c r="E29" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F29">
-        <v>68</v>
-      </c>
-      <c r="G29">
-        <v>3639</v>
-      </c>
-      <c r="H29">
-        <v>3</v>
+        <v>46069</v>
       </c>
       <c r="I29">
         <v>2</v>
@@ -13341,29 +13406,17 @@
     </row>
     <row r="30" spans="1:10" ht="75">
       <c r="A30" s="1" t="s">
-        <v>711</v>
+        <v>912</v>
       </c>
       <c r="B30" s="3">
-        <v>46066</v>
+        <v>46069</v>
       </c>
       <c r="C30">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="D30">
         <v>3642</v>
       </c>
-      <c r="E30" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F30">
-        <v>71</v>
-      </c>
-      <c r="G30">
-        <v>3639</v>
-      </c>
-      <c r="H30">
-        <v>3</v>
-      </c>
       <c r="I30">
         <v>2</v>
       </c>
@@ -13371,31 +13424,19 @@
         <v>794</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="56.25">
+    <row r="31" spans="1:10" ht="75">
       <c r="A31" s="1" t="s">
-        <v>655</v>
+        <v>913</v>
       </c>
       <c r="B31" s="3">
-        <v>46066</v>
+        <v>46069</v>
       </c>
       <c r="C31">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D31">
         <v>3642</v>
       </c>
-      <c r="E31" s="3">
-        <v>46067</v>
-      </c>
-      <c r="F31">
-        <v>95</v>
-      </c>
-      <c r="G31">
-        <v>3639</v>
-      </c>
-      <c r="H31">
-        <v>3</v>
-      </c>
       <c r="I31">
         <v>2</v>
       </c>
@@ -13403,12 +13444,50 @@
         <v>794</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" ht="56.25">
       <c r="A32" s="1" t="s">
-        <v>899</v>
+        <v>914</v>
       </c>
       <c r="B32" s="3">
         <v>46069</v>
+      </c>
+      <c r="C32">
+        <v>23</v>
+      </c>
+      <c r="D32">
+        <v>3642</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" s="2" t="s">
+        <v>921</v>
+      </c>
+      <c r="B33" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="2" t="s">
+        <v>966</v>
+      </c>
+      <c r="B34" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="2" t="s">
+        <v>967</v>
+      </c>
+      <c r="B35" s="3">
+        <v>46071</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="2" t="s">
+        <v>968</v>
+      </c>
+      <c r="B36" s="3">
+        <v>46071</v>
       </c>
     </row>
   </sheetData>
@@ -13417,9 +13496,13 @@
   </sortState>
   <phoneticPr fontId="1"/>
   <hyperlinks>
-    <hyperlink ref="A6" r:id="rId1" xr:uid="{652F4804-A291-4908-8DB0-F790956B309E}"/>
-    <hyperlink ref="A7" r:id="rId2" xr:uid="{11FEC87D-3AF9-45D5-A4CE-AC44976C500C}"/>
-    <hyperlink ref="A2" r:id="rId3" xr:uid="{331C7376-F1B6-4EE5-8CFD-0EE5CD109EC0}"/>
+    <hyperlink ref="A23" r:id="rId1" xr:uid="{37DE3294-D0FE-4C41-82C6-A053F898D96C}"/>
+    <hyperlink ref="A24" r:id="rId2" xr:uid="{C26843F4-B085-48AF-BF5E-2915CC32483A}"/>
+    <hyperlink ref="A25" r:id="rId3" xr:uid="{B43E9FB8-107C-4957-A1BD-53FF80634BBE}"/>
+    <hyperlink ref="A33" r:id="rId4" xr:uid="{CA997FE4-29B4-4561-A04B-87B2E7741A2E}"/>
+    <hyperlink ref="A34" r:id="rId5" xr:uid="{ED174808-7EA1-49A1-9686-D90A0BEABA41}"/>
+    <hyperlink ref="A35" r:id="rId6" xr:uid="{5ACD6FF0-625D-4EAB-91E4-7FF3DB672BC0}"/>
+    <hyperlink ref="A36" r:id="rId7" xr:uid="{3522D58F-6205-4458-8474-88FD15B79747}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13647,7 +13730,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -14035,7 +14118,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -14681,7 +14764,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46071</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
feat: enhance asset management UI with gradualism mission tracking and struggle logic improvements
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1515EEE6-F32C-4D4A-BB1F-E98BAB8385FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D878C62A-47BD-44D4-9B7C-7A60ABCE7BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="16" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="969">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1629" uniqueCount="971">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -5589,6 +5589,14 @@
   </si>
   <si>
     <t>https://x.com/kanta13jp1/status/2023829776843370629</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>As I explained in Chapter 2, after self-interest and self-survival, the quest for wealth and power is what most motivates individuals, families, companies, states, and countries. Because wealth equals power in terms of the ability to build military strength, control trade, and influence other nations,  domestic and military strength go hand in hand. It takes money to buy guns (military power) and it takes money to buy butter (domestic social spending needs). When a country fails to provide adequate amounts of either, it becomes vulnerable to domestic and foreign opposition. From my study of Chinese dynasties and European empires, I’ve learned that  the financial strength to outspend one’s rivals is one of the most important strengths a country can have. That is how the United States beat the Soviet Union in the Cold War. Spend enough money in the right ways, and you don’t have to have a shooting war. Long-term success depends on sustaining both the “guns” and the “butter” without producing the excesses that lead to their declines. In other words, a country must be strong enough financially to give its people both a good living standard and protection from outside enemies. The really successful countries have been able to do that for 200 to 300 years. None has been able to do it forever.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>第2章で説明したように、自己利益と自己保存に次いで、富と権力の追求こそが個人、家族、企業、国家、そして国々を最も強く駆り立てる動機である。なぜなら富は軍事力の構築、貿易の支配、他国への影響力という点で権力に等しく、国内の力と軍事力は表裏一体だからだ。銃（軍事力）を買うにも金が必要であり、バター（国内の社会支出需要）を買うにも金が必要だ。いずれかの供給が十分でないと、国家は国内外の反対勢力に脆弱となる。中国の王朝やヨーロッパ帝国を研究する中で、私は「ライバルよりも多く支出できる財政力」が国家が持つべき最重要の強みの一つであることを学んだ。これが冷戦においてアメリカがソ連に勝利した理由である。適切な方法で十分な資金を投入すれば、武力衝突を避けられるのだ。長期的な成功は、「銃」と「バター」の両方を、衰退を招く過剰を生み出さずに持続させることに依存する。つまり、国家は国民に良好な生活水準と外敵からの保護の両方を提供できるだけの財政的強さを備えていなければならない。真に成功した国々は200年から300年にわたりこれを達成してきた。永遠にこれを成し遂げた国は存在しない。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -5992,7 +6000,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -6175,7 +6183,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -6388,7 +6396,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -6564,7 +6572,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -10110,7 +10118,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -10591,10 +10599,10 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="C2:Q231"/>
+  <dimension ref="C2:Q232"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
@@ -10647,7 +10655,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="3" spans="3:17" ht="93.75" hidden="1">
+    <row r="3" spans="3:17" ht="93.75">
       <c r="C3" s="2" t="s">
         <v>630</v>
       </c>
@@ -10754,87 +10762,87 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="7" spans="3:17" hidden="1">
+    <row r="7" spans="3:17">
       <c r="H7" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="8" spans="3:17" hidden="1">
+    <row r="8" spans="3:17">
       <c r="H8" t="s">
         <v>640</v>
       </c>
     </row>
-    <row r="9" spans="3:17" hidden="1">
+    <row r="9" spans="3:17">
       <c r="H9" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="10" spans="3:17" hidden="1">
+    <row r="10" spans="3:17">
       <c r="H10" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="11" spans="3:17" hidden="1">
+    <row r="11" spans="3:17">
       <c r="H11" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="12" spans="3:17" hidden="1">
+    <row r="12" spans="3:17">
       <c r="H12" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="13" spans="3:17" hidden="1">
+    <row r="13" spans="3:17">
       <c r="H13" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="14" spans="3:17" hidden="1">
+    <row r="14" spans="3:17">
       <c r="H14" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="15" spans="3:17" hidden="1">
+    <row r="15" spans="3:17">
       <c r="H15" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="16" spans="3:17" hidden="1">
+    <row r="16" spans="3:17">
       <c r="H16" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="17" spans="3:16" hidden="1">
+    <row r="17" spans="3:16">
       <c r="H17" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="18" spans="3:16" hidden="1">
+    <row r="18" spans="3:16">
       <c r="H18" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="19" spans="3:16" hidden="1">
+    <row r="19" spans="3:16">
       <c r="H19" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="20" spans="3:16" hidden="1">
+    <row r="20" spans="3:16">
       <c r="H20" t="s">
         <v>652</v>
       </c>
     </row>
-    <row r="21" spans="3:16" hidden="1">
+    <row r="21" spans="3:16">
       <c r="H21" t="s">
         <v>653</v>
       </c>
     </row>
-    <row r="22" spans="3:16" hidden="1">
+    <row r="22" spans="3:16">
       <c r="H22" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="23" spans="3:16" ht="112.5" hidden="1">
+    <row r="23" spans="3:16" ht="112.5">
       <c r="C23" s="2" t="s">
         <v>658</v>
       </c>
@@ -10935,42 +10943,42 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="27" spans="3:16" hidden="1">
+    <row r="27" spans="3:16">
       <c r="H27" t="s">
         <v>667</v>
       </c>
     </row>
-    <row r="28" spans="3:16" hidden="1">
+    <row r="28" spans="3:16">
       <c r="H28" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="29" spans="3:16" hidden="1">
+    <row r="29" spans="3:16">
       <c r="H29" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="30" spans="3:16" hidden="1">
+    <row r="30" spans="3:16">
       <c r="H30" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="31" spans="3:16" hidden="1">
+    <row r="31" spans="3:16">
       <c r="H31" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="32" spans="3:16" hidden="1">
+    <row r="32" spans="3:16">
       <c r="H32" t="s">
         <v>672</v>
       </c>
     </row>
-    <row r="33" spans="3:16" hidden="1">
+    <row r="33" spans="3:16">
       <c r="H33" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="34" spans="3:16" ht="112.5" hidden="1">
+    <row r="34" spans="3:16" ht="112.5">
       <c r="C34" s="2" t="s">
         <v>682</v>
       </c>
@@ -11071,107 +11079,107 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="38" spans="3:16" hidden="1">
+    <row r="38" spans="3:16">
       <c r="H38" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="39" spans="3:16" hidden="1">
+    <row r="39" spans="3:16">
       <c r="H39" t="s">
         <v>691</v>
       </c>
     </row>
-    <row r="40" spans="3:16" hidden="1">
+    <row r="40" spans="3:16">
       <c r="H40" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="41" spans="3:16" hidden="1">
+    <row r="41" spans="3:16">
       <c r="H41" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="42" spans="3:16" hidden="1">
+    <row r="42" spans="3:16">
       <c r="H42" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="43" spans="3:16" hidden="1">
+    <row r="43" spans="3:16">
       <c r="H43" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="44" spans="3:16" hidden="1">
+    <row r="44" spans="3:16">
       <c r="H44" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="45" spans="3:16" hidden="1">
+    <row r="45" spans="3:16">
       <c r="H45" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="46" spans="3:16" hidden="1">
+    <row r="46" spans="3:16">
       <c r="H46" t="s">
         <v>698</v>
       </c>
     </row>
-    <row r="47" spans="3:16" hidden="1">
+    <row r="47" spans="3:16">
       <c r="H47" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="48" spans="3:16" hidden="1">
+    <row r="48" spans="3:16">
       <c r="H48" t="s">
         <v>700</v>
       </c>
     </row>
-    <row r="49" spans="3:16" hidden="1">
+    <row r="49" spans="3:16">
       <c r="H49" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="50" spans="3:16" hidden="1">
+    <row r="50" spans="3:16">
       <c r="H50" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="51" spans="3:16" hidden="1">
+    <row r="51" spans="3:16">
       <c r="H51" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="52" spans="3:16" hidden="1">
+    <row r="52" spans="3:16">
       <c r="H52" t="s">
         <v>704</v>
       </c>
     </row>
-    <row r="53" spans="3:16" hidden="1">
+    <row r="53" spans="3:16">
       <c r="H53" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="54" spans="3:16" hidden="1">
+    <row r="54" spans="3:16">
       <c r="H54" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="55" spans="3:16" hidden="1">
+    <row r="55" spans="3:16">
       <c r="H55" t="s">
         <v>707</v>
       </c>
     </row>
-    <row r="56" spans="3:16" hidden="1">
+    <row r="56" spans="3:16">
       <c r="H56" t="s">
         <v>708</v>
       </c>
     </row>
-    <row r="57" spans="3:16" hidden="1">
+    <row r="57" spans="3:16">
       <c r="H57" t="s">
         <v>709</v>
       </c>
     </row>
-    <row r="58" spans="3:16" ht="409.5" hidden="1">
+    <row r="58" spans="3:16" ht="409.5">
       <c r="C58" s="2" t="s">
         <v>713</v>
       </c>
@@ -11272,63 +11280,63 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="62" spans="3:16" hidden="1">
+    <row r="62" spans="3:16">
       <c r="H62" t="s">
         <v>721</v>
       </c>
       <c r="J62" s="1"/>
     </row>
-    <row r="63" spans="3:16" hidden="1">
+    <row r="63" spans="3:16">
       <c r="H63" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="64" spans="3:16" hidden="1">
+    <row r="64" spans="3:16">
       <c r="H64" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="65" spans="3:16" hidden="1">
+    <row r="65" spans="3:16">
       <c r="H65" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="66" spans="3:16" hidden="1">
+    <row r="66" spans="3:16">
       <c r="H66" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="67" spans="3:16" hidden="1">
+    <row r="67" spans="3:16">
       <c r="H67" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="68" spans="3:16" hidden="1">
+    <row r="68" spans="3:16">
       <c r="H68" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="69" spans="3:16" hidden="1">
+    <row r="69" spans="3:16">
       <c r="H69" t="s">
         <v>728</v>
       </c>
     </row>
-    <row r="70" spans="3:16" hidden="1">
+    <row r="70" spans="3:16">
       <c r="H70" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="71" spans="3:16" hidden="1">
+    <row r="71" spans="3:16">
       <c r="H71" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="72" spans="3:16" hidden="1">
+    <row r="72" spans="3:16">
       <c r="H72" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="73" spans="3:16" ht="409.5" hidden="1">
+    <row r="73" spans="3:16" ht="409.5">
       <c r="C73" s="2" t="s">
         <v>735</v>
       </c>
@@ -11429,137 +11437,137 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="77" spans="3:16" hidden="1">
+    <row r="77" spans="3:16">
       <c r="H77" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="78" spans="3:16" hidden="1">
+    <row r="78" spans="3:16">
       <c r="H78" t="s">
         <v>744</v>
       </c>
     </row>
-    <row r="79" spans="3:16" hidden="1">
+    <row r="79" spans="3:16">
       <c r="H79" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="80" spans="3:16" hidden="1">
+    <row r="80" spans="3:16">
       <c r="H80" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="81" spans="8:8" hidden="1">
+    <row r="81" spans="8:8">
       <c r="H81" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="82" spans="8:8" hidden="1">
+    <row r="82" spans="8:8">
       <c r="H82" t="s">
         <v>748</v>
       </c>
     </row>
-    <row r="83" spans="8:8" hidden="1">
+    <row r="83" spans="8:8">
       <c r="H83" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="84" spans="8:8" hidden="1">
+    <row r="84" spans="8:8">
       <c r="H84" t="s">
         <v>750</v>
       </c>
     </row>
-    <row r="85" spans="8:8" hidden="1">
+    <row r="85" spans="8:8">
       <c r="H85" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="86" spans="8:8" hidden="1">
+    <row r="86" spans="8:8">
       <c r="H86" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="87" spans="8:8" hidden="1">
+    <row r="87" spans="8:8">
       <c r="H87" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="88" spans="8:8" hidden="1">
+    <row r="88" spans="8:8">
       <c r="H88" t="s">
         <v>754</v>
       </c>
     </row>
-    <row r="89" spans="8:8" hidden="1">
+    <row r="89" spans="8:8">
       <c r="H89" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="90" spans="8:8" hidden="1">
+    <row r="90" spans="8:8">
       <c r="H90" t="s">
         <v>756</v>
       </c>
     </row>
-    <row r="91" spans="8:8" hidden="1">
+    <row r="91" spans="8:8">
       <c r="H91" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="92" spans="8:8" hidden="1">
+    <row r="92" spans="8:8">
       <c r="H92" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="93" spans="8:8" hidden="1">
+    <row r="93" spans="8:8">
       <c r="H93" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="94" spans="8:8" hidden="1">
+    <row r="94" spans="8:8">
       <c r="H94" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="95" spans="8:8" hidden="1">
+    <row r="95" spans="8:8">
       <c r="H95" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="96" spans="8:8" hidden="1">
+    <row r="96" spans="8:8">
       <c r="H96" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="97" spans="3:16" hidden="1">
+    <row r="97" spans="3:16">
       <c r="H97" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="98" spans="3:16" hidden="1">
+    <row r="98" spans="3:16">
       <c r="H98" t="s">
         <v>764</v>
       </c>
     </row>
-    <row r="99" spans="3:16" hidden="1">
+    <row r="99" spans="3:16">
       <c r="H99" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="100" spans="3:16" hidden="1">
+    <row r="100" spans="3:16">
       <c r="H100" t="s">
         <v>766</v>
       </c>
     </row>
-    <row r="101" spans="3:16" hidden="1">
+    <row r="101" spans="3:16">
       <c r="H101" t="s">
         <v>767</v>
       </c>
     </row>
-    <row r="102" spans="3:16" hidden="1">
+    <row r="102" spans="3:16">
       <c r="H102" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="103" spans="3:16" ht="168.75" hidden="1">
+    <row r="103" spans="3:16" ht="168.75">
       <c r="C103" s="2" t="s">
         <v>772</v>
       </c>
@@ -11660,62 +11668,62 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="107" spans="3:16" hidden="1">
+    <row r="107" spans="3:16">
       <c r="H107" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="108" spans="3:16" hidden="1">
+    <row r="108" spans="3:16">
       <c r="H108" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="109" spans="3:16" hidden="1">
+    <row r="109" spans="3:16">
       <c r="H109" t="s">
         <v>781</v>
       </c>
     </row>
-    <row r="110" spans="3:16" hidden="1">
+    <row r="110" spans="3:16">
       <c r="H110" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="111" spans="3:16" hidden="1">
+    <row r="111" spans="3:16">
       <c r="H111" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="112" spans="3:16" hidden="1">
+    <row r="112" spans="3:16">
       <c r="H112" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="113" spans="3:13" hidden="1">
+    <row r="113" spans="3:13">
       <c r="H113" t="s">
         <v>785</v>
       </c>
     </row>
-    <row r="114" spans="3:13" hidden="1">
+    <row r="114" spans="3:13">
       <c r="H114" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="115" spans="3:13" hidden="1">
+    <row r="115" spans="3:13">
       <c r="H115" t="s">
         <v>787</v>
       </c>
     </row>
-    <row r="116" spans="3:13" hidden="1">
+    <row r="116" spans="3:13">
       <c r="H116" t="s">
         <v>788</v>
       </c>
     </row>
-    <row r="117" spans="3:13" hidden="1">
+    <row r="117" spans="3:13">
       <c r="H117" t="s">
         <v>789</v>
       </c>
     </row>
-    <row r="118" spans="3:13" ht="75" hidden="1">
+    <row r="118" spans="3:13" ht="75">
       <c r="C118" s="2" t="s">
         <v>801</v>
       </c>
@@ -11789,292 +11797,292 @@
         <v>3640</v>
       </c>
     </row>
-    <row r="122" spans="3:13" hidden="1">
+    <row r="122" spans="3:13">
       <c r="H122" t="s">
         <v>808</v>
       </c>
     </row>
-    <row r="123" spans="3:13" hidden="1">
+    <row r="123" spans="3:13">
       <c r="H123" t="s">
         <v>809</v>
       </c>
     </row>
-    <row r="124" spans="3:13" hidden="1">
+    <row r="124" spans="3:13">
       <c r="H124" t="s">
         <v>810</v>
       </c>
     </row>
-    <row r="125" spans="3:13" hidden="1">
+    <row r="125" spans="3:13">
       <c r="H125" t="s">
         <v>811</v>
       </c>
     </row>
-    <row r="126" spans="3:13" hidden="1">
+    <row r="126" spans="3:13">
       <c r="H126" t="s">
         <v>812</v>
       </c>
     </row>
-    <row r="127" spans="3:13" hidden="1">
+    <row r="127" spans="3:13">
       <c r="H127" t="s">
         <v>813</v>
       </c>
     </row>
-    <row r="128" spans="3:13" hidden="1">
+    <row r="128" spans="3:13">
       <c r="H128" t="s">
         <v>814</v>
       </c>
     </row>
-    <row r="129" spans="8:8" hidden="1">
+    <row r="129" spans="8:8">
       <c r="H129" t="s">
         <v>815</v>
       </c>
     </row>
-    <row r="130" spans="8:8" hidden="1">
+    <row r="130" spans="8:8">
       <c r="H130" t="s">
         <v>816</v>
       </c>
     </row>
-    <row r="131" spans="8:8" hidden="1">
+    <row r="131" spans="8:8">
       <c r="H131" t="s">
         <v>817</v>
       </c>
     </row>
-    <row r="132" spans="8:8" hidden="1">
+    <row r="132" spans="8:8">
       <c r="H132" t="s">
         <v>818</v>
       </c>
     </row>
-    <row r="133" spans="8:8" hidden="1">
+    <row r="133" spans="8:8">
       <c r="H133" t="s">
         <v>819</v>
       </c>
     </row>
-    <row r="134" spans="8:8" hidden="1">
+    <row r="134" spans="8:8">
       <c r="H134" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="135" spans="8:8" hidden="1">
+    <row r="135" spans="8:8">
       <c r="H135" t="s">
         <v>820</v>
       </c>
     </row>
-    <row r="136" spans="8:8" hidden="1">
+    <row r="136" spans="8:8">
       <c r="H136" t="s">
         <v>821</v>
       </c>
     </row>
-    <row r="137" spans="8:8" hidden="1">
+    <row r="137" spans="8:8">
       <c r="H137" t="s">
         <v>822</v>
       </c>
     </row>
-    <row r="138" spans="8:8" hidden="1">
+    <row r="138" spans="8:8">
       <c r="H138" t="s">
         <v>823</v>
       </c>
     </row>
-    <row r="139" spans="8:8" hidden="1">
+    <row r="139" spans="8:8">
       <c r="H139" t="s">
         <v>824</v>
       </c>
     </row>
-    <row r="140" spans="8:8" hidden="1">
+    <row r="140" spans="8:8">
       <c r="H140" t="s">
         <v>825</v>
       </c>
     </row>
-    <row r="141" spans="8:8" hidden="1">
+    <row r="141" spans="8:8">
       <c r="H141" t="s">
         <v>826</v>
       </c>
     </row>
-    <row r="142" spans="8:8" hidden="1">
+    <row r="142" spans="8:8">
       <c r="H142" t="s">
         <v>827</v>
       </c>
     </row>
-    <row r="143" spans="8:8" hidden="1">
+    <row r="143" spans="8:8">
       <c r="H143" t="s">
         <v>828</v>
       </c>
     </row>
-    <row r="144" spans="8:8" hidden="1">
+    <row r="144" spans="8:8">
       <c r="H144" t="s">
         <v>829</v>
       </c>
     </row>
-    <row r="145" spans="8:8" hidden="1">
+    <row r="145" spans="8:8">
       <c r="H145" t="s">
         <v>830</v>
       </c>
     </row>
-    <row r="146" spans="8:8" hidden="1">
+    <row r="146" spans="8:8">
       <c r="H146" t="s">
         <v>831</v>
       </c>
     </row>
-    <row r="147" spans="8:8" hidden="1">
+    <row r="147" spans="8:8">
       <c r="H147" t="s">
         <v>832</v>
       </c>
     </row>
-    <row r="148" spans="8:8" hidden="1">
+    <row r="148" spans="8:8">
       <c r="H148" t="s">
         <v>833</v>
       </c>
     </row>
-    <row r="149" spans="8:8" hidden="1">
+    <row r="149" spans="8:8">
       <c r="H149" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="150" spans="8:8" hidden="1">
+    <row r="150" spans="8:8">
       <c r="H150" t="s">
         <v>835</v>
       </c>
     </row>
-    <row r="151" spans="8:8" hidden="1">
+    <row r="151" spans="8:8">
       <c r="H151" t="s">
         <v>836</v>
       </c>
     </row>
-    <row r="152" spans="8:8" hidden="1">
+    <row r="152" spans="8:8">
       <c r="H152" t="s">
         <v>837</v>
       </c>
     </row>
-    <row r="153" spans="8:8" hidden="1">
+    <row r="153" spans="8:8">
       <c r="H153" t="s">
         <v>838</v>
       </c>
     </row>
-    <row r="154" spans="8:8" hidden="1">
+    <row r="154" spans="8:8">
       <c r="H154" t="s">
         <v>839</v>
       </c>
     </row>
-    <row r="155" spans="8:8" hidden="1">
+    <row r="155" spans="8:8">
       <c r="H155" t="s">
         <v>840</v>
       </c>
     </row>
-    <row r="156" spans="8:8" hidden="1">
+    <row r="156" spans="8:8">
       <c r="H156" t="s">
         <v>841</v>
       </c>
     </row>
-    <row r="157" spans="8:8" hidden="1">
+    <row r="157" spans="8:8">
       <c r="H157" t="s">
         <v>842</v>
       </c>
     </row>
-    <row r="158" spans="8:8" hidden="1">
+    <row r="158" spans="8:8">
       <c r="H158" t="s">
         <v>843</v>
       </c>
     </row>
-    <row r="159" spans="8:8" hidden="1">
+    <row r="159" spans="8:8">
       <c r="H159" t="s">
         <v>844</v>
       </c>
     </row>
-    <row r="160" spans="8:8" hidden="1">
+    <row r="160" spans="8:8">
       <c r="H160" t="s">
         <v>845</v>
       </c>
     </row>
-    <row r="161" spans="8:8" hidden="1">
+    <row r="161" spans="8:8">
       <c r="H161" t="s">
         <v>846</v>
       </c>
     </row>
-    <row r="162" spans="8:8" hidden="1">
+    <row r="162" spans="8:8">
       <c r="H162" t="s">
         <v>847</v>
       </c>
     </row>
-    <row r="163" spans="8:8" hidden="1">
+    <row r="163" spans="8:8">
       <c r="H163" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="164" spans="8:8" hidden="1">
+    <row r="164" spans="8:8">
       <c r="H164" t="s">
         <v>849</v>
       </c>
     </row>
-    <row r="165" spans="8:8" hidden="1">
+    <row r="165" spans="8:8">
       <c r="H165" t="s">
         <v>850</v>
       </c>
     </row>
-    <row r="166" spans="8:8" hidden="1">
+    <row r="166" spans="8:8">
       <c r="H166" t="s">
         <v>851</v>
       </c>
     </row>
-    <row r="167" spans="8:8" hidden="1">
+    <row r="167" spans="8:8">
       <c r="H167" t="s">
         <v>852</v>
       </c>
     </row>
-    <row r="168" spans="8:8" hidden="1">
+    <row r="168" spans="8:8">
       <c r="H168" t="s">
         <v>853</v>
       </c>
     </row>
-    <row r="169" spans="8:8" hidden="1">
+    <row r="169" spans="8:8">
       <c r="H169" t="s">
         <v>854</v>
       </c>
     </row>
-    <row r="170" spans="8:8" hidden="1">
+    <row r="170" spans="8:8">
       <c r="H170" t="s">
         <v>855</v>
       </c>
     </row>
-    <row r="171" spans="8:8" hidden="1">
+    <row r="171" spans="8:8">
       <c r="H171" t="s">
         <v>856</v>
       </c>
     </row>
-    <row r="172" spans="8:8" hidden="1">
+    <row r="172" spans="8:8">
       <c r="H172" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="173" spans="8:8" hidden="1">
+    <row r="173" spans="8:8">
       <c r="H173" t="s">
         <v>858</v>
       </c>
     </row>
-    <row r="174" spans="8:8" hidden="1">
+    <row r="174" spans="8:8">
       <c r="H174" t="s">
         <v>859</v>
       </c>
     </row>
-    <row r="175" spans="8:8" hidden="1">
+    <row r="175" spans="8:8">
       <c r="H175" t="s">
         <v>860</v>
       </c>
     </row>
-    <row r="176" spans="8:8" hidden="1">
+    <row r="176" spans="8:8">
       <c r="H176" t="s">
         <v>861</v>
       </c>
     </row>
-    <row r="177" spans="3:13" hidden="1">
+    <row r="177" spans="3:13">
       <c r="H177" t="s">
         <v>862</v>
       </c>
     </row>
-    <row r="178" spans="3:13" hidden="1">
+    <row r="178" spans="3:13">
       <c r="H178" t="s">
         <v>863</v>
       </c>
     </row>
-    <row r="179" spans="3:13" ht="168.75" hidden="1">
+    <row r="179" spans="3:13" ht="168.75">
       <c r="C179" s="2" t="s">
         <v>868</v>
       </c>
@@ -12139,7 +12147,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="183" spans="3:13" ht="168.75" hidden="1">
+    <row r="183" spans="3:13" ht="168.75">
       <c r="C183" s="2" t="s">
         <v>877</v>
       </c>
@@ -12224,42 +12232,42 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="188" spans="3:13" hidden="1">
+    <row r="188" spans="3:13">
       <c r="H188" t="s">
         <v>885</v>
       </c>
     </row>
-    <row r="189" spans="3:13" hidden="1">
+    <row r="189" spans="3:13">
       <c r="H189" t="s">
         <v>886</v>
       </c>
     </row>
-    <row r="190" spans="3:13" hidden="1">
+    <row r="190" spans="3:13">
       <c r="H190" t="s">
         <v>887</v>
       </c>
     </row>
-    <row r="191" spans="3:13" hidden="1">
+    <row r="191" spans="3:13">
       <c r="H191" t="s">
         <v>888</v>
       </c>
     </row>
-    <row r="192" spans="3:13" hidden="1">
+    <row r="192" spans="3:13">
       <c r="H192" t="s">
         <v>889</v>
       </c>
     </row>
-    <row r="193" spans="3:13" hidden="1">
+    <row r="193" spans="3:13">
       <c r="H193" t="s">
         <v>890</v>
       </c>
     </row>
-    <row r="194" spans="3:13" hidden="1">
+    <row r="194" spans="3:13">
       <c r="H194" t="s">
         <v>891</v>
       </c>
     </row>
-    <row r="195" spans="3:13" ht="409.5" hidden="1">
+    <row r="195" spans="3:13" ht="409.5">
       <c r="C195" s="2" t="s">
         <v>895</v>
       </c>
@@ -12333,52 +12341,52 @@
         <v>3642</v>
       </c>
     </row>
-    <row r="199" spans="3:13" hidden="1">
+    <row r="199" spans="3:13">
       <c r="H199" t="s">
         <v>903</v>
       </c>
     </row>
-    <row r="200" spans="3:13" hidden="1">
+    <row r="200" spans="3:13">
       <c r="H200" t="s">
         <v>904</v>
       </c>
     </row>
-    <row r="201" spans="3:13" hidden="1">
+    <row r="201" spans="3:13">
       <c r="H201" t="s">
         <v>905</v>
       </c>
     </row>
-    <row r="202" spans="3:13" hidden="1">
+    <row r="202" spans="3:13">
       <c r="H202" t="s">
         <v>906</v>
       </c>
     </row>
-    <row r="203" spans="3:13" hidden="1">
+    <row r="203" spans="3:13">
       <c r="H203" t="s">
         <v>907</v>
       </c>
     </row>
-    <row r="204" spans="3:13" hidden="1">
+    <row r="204" spans="3:13">
       <c r="H204" t="s">
         <v>908</v>
       </c>
     </row>
-    <row r="205" spans="3:13" hidden="1">
+    <row r="205" spans="3:13">
       <c r="H205" t="s">
         <v>909</v>
       </c>
     </row>
-    <row r="206" spans="3:13" hidden="1">
+    <row r="206" spans="3:13">
       <c r="H206" t="s">
         <v>910</v>
       </c>
     </row>
-    <row r="207" spans="3:13" hidden="1">
+    <row r="207" spans="3:13">
       <c r="H207" t="s">
         <v>911</v>
       </c>
     </row>
-    <row r="208" spans="3:13" ht="150" hidden="1">
+    <row r="208" spans="3:13" ht="150">
       <c r="C208" s="2" t="s">
         <v>916</v>
       </c>
@@ -12412,7 +12420,7 @@
         <v>46071</v>
       </c>
     </row>
-    <row r="210" spans="3:11" ht="168.75" hidden="1">
+    <row r="210" spans="3:11" ht="168.75">
       <c r="C210" s="2" t="s">
         <v>960</v>
       </c>
@@ -12429,7 +12437,7 @@
       <c r="I210" s="1"/>
       <c r="J210" s="2"/>
     </row>
-    <row r="211" spans="3:11" hidden="1">
+    <row r="211" spans="3:11">
       <c r="C211" s="2"/>
       <c r="E211" s="1"/>
       <c r="F211" s="1" t="s">
@@ -12486,7 +12494,7 @@
         <v>46071</v>
       </c>
     </row>
-    <row r="215" spans="3:11" ht="93.75" hidden="1">
+    <row r="215" spans="3:11" ht="93.75">
       <c r="C215" s="2" t="s">
         <v>922</v>
       </c>
@@ -12503,7 +12511,7 @@
         <v>929</v>
       </c>
     </row>
-    <row r="216" spans="3:11" ht="262.5" hidden="1">
+    <row r="216" spans="3:11" ht="262.5">
       <c r="E216" s="1" t="s">
         <v>925</v>
       </c>
@@ -12517,7 +12525,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="217" spans="3:11" ht="243.75" hidden="1">
+    <row r="217" spans="3:11" ht="243.75">
       <c r="F217" s="1" t="s">
         <v>930</v>
       </c>
@@ -12528,7 +12536,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="218" spans="3:11" ht="337.5" hidden="1">
+    <row r="218" spans="3:11" ht="337.5">
       <c r="F218" s="1" t="s">
         <v>931</v>
       </c>
@@ -12539,7 +12547,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="219" spans="3:11" ht="206.25" hidden="1">
+    <row r="219" spans="3:11" ht="206.25">
       <c r="F219" s="1" t="s">
         <v>933</v>
       </c>
@@ -12550,7 +12558,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="220" spans="3:11" ht="75" hidden="1">
+    <row r="220" spans="3:11" ht="75">
       <c r="F220" s="1" t="s">
         <v>935</v>
       </c>
@@ -12561,7 +12569,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="221" spans="3:11" ht="56.25" hidden="1">
+    <row r="221" spans="3:11" ht="56.25">
       <c r="F221" s="1" t="s">
         <v>937</v>
       </c>
@@ -12572,7 +12580,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="222" spans="3:11" ht="243.75" hidden="1">
+    <row r="222" spans="3:11" ht="243.75">
       <c r="F222" s="1" t="s">
         <v>939</v>
       </c>
@@ -12583,7 +12591,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="223" spans="3:11" ht="75" hidden="1">
+    <row r="223" spans="3:11" ht="75">
       <c r="F223" s="1" t="s">
         <v>941</v>
       </c>
@@ -12594,7 +12602,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="224" spans="3:11" ht="168.75" hidden="1">
+    <row r="224" spans="3:11" ht="168.75">
       <c r="F224" s="1" t="s">
         <v>943</v>
       </c>
@@ -12605,7 +12613,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="225" spans="6:10" ht="112.5" hidden="1">
+    <row r="225" spans="6:10" ht="112.5">
       <c r="F225" s="1" t="s">
         <v>945</v>
       </c>
@@ -12616,7 +12624,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="226" spans="6:10" ht="131.25" hidden="1">
+    <row r="226" spans="6:10" ht="131.25">
       <c r="F226" s="1" t="s">
         <v>947</v>
       </c>
@@ -12627,7 +12635,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="227" spans="6:10" ht="131.25" hidden="1">
+    <row r="227" spans="6:10" ht="131.25">
       <c r="F227" s="1" t="s">
         <v>949</v>
       </c>
@@ -12638,7 +12646,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="228" spans="6:10" ht="37.5" hidden="1">
+    <row r="228" spans="6:10" ht="37.5">
       <c r="F228" s="1" t="s">
         <v>951</v>
       </c>
@@ -12649,7 +12657,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="229" spans="6:10" ht="206.25" hidden="1">
+    <row r="229" spans="6:10" ht="206.25">
       <c r="F229" s="1" t="s">
         <v>953</v>
       </c>
@@ -12660,7 +12668,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="230" spans="6:10" ht="168.75" hidden="1">
+    <row r="230" spans="6:10" ht="168.75">
       <c r="F230" s="1" t="s">
         <v>955</v>
       </c>
@@ -12671,7 +12679,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="231" spans="6:10" ht="37.5" hidden="1">
+    <row r="231" spans="6:10" ht="37.5">
       <c r="F231" s="1" t="s">
         <v>957</v>
       </c>
@@ -12679,14 +12687,16 @@
         <v>958</v>
       </c>
     </row>
+    <row r="232" spans="6:10" ht="375">
+      <c r="F232" s="1" t="s">
+        <v>969</v>
+      </c>
+      <c r="I232" s="1" t="s">
+        <v>970</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="C2:M231" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}">
-    <filterColumn colId="8">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="C2:M231" xr:uid="{69928822-4B0A-479C-837F-2ECBAF654BC2}"/>
   <phoneticPr fontId="1"/>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" xr:uid="{C897C6D6-16A8-4618-9776-831A651C49AE}"/>
@@ -12727,8 +12737,8 @@
     <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17.125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.25" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -12754,10 +12764,10 @@
         <v>678</v>
       </c>
       <c r="H1" t="s">
+        <v>915</v>
+      </c>
+      <c r="I1" t="s">
         <v>793</v>
-      </c>
-      <c r="I1" t="s">
-        <v>915</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="56.25">
@@ -12809,16 +12819,19 @@
         <v>46067</v>
       </c>
       <c r="F3">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="G3">
-        <v>3639</v>
+        <v>3649</v>
       </c>
       <c r="H3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I3">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J3" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="56.25">
@@ -12838,13 +12851,19 @@
         <v>46067</v>
       </c>
       <c r="F4">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="G4">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
       </c>
       <c r="I4">
         <v>1</v>
+      </c>
+      <c r="J4" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="75">
@@ -12864,13 +12883,19 @@
         <v>46067</v>
       </c>
       <c r="F5">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="G5">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
       </c>
       <c r="I5">
         <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="262.5">
@@ -12890,13 +12915,19 @@
         <v>46067</v>
       </c>
       <c r="F6">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="G6">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
       </c>
       <c r="I6">
         <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="75">
@@ -12919,10 +12950,16 @@
         <v>36</v>
       </c>
       <c r="G7">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="J7" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="93.75">
@@ -12942,13 +12979,19 @@
         <v>46067</v>
       </c>
       <c r="F8">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G8">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J8" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="75">
@@ -12968,13 +13011,19 @@
         <v>46067</v>
       </c>
       <c r="F9">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="G9">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H9">
+        <v>2</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="J9" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="75">
@@ -12994,13 +13043,19 @@
         <v>46067</v>
       </c>
       <c r="F10">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="G10">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
       </c>
       <c r="I10">
         <v>1</v>
+      </c>
+      <c r="J10" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="93.75">
@@ -13020,13 +13075,19 @@
         <v>46067</v>
       </c>
       <c r="F11">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="G11">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
       </c>
       <c r="I11">
         <v>1</v>
+      </c>
+      <c r="J11" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="187.5">
@@ -13046,13 +13107,19 @@
         <v>46067</v>
       </c>
       <c r="F12">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="G12">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
       </c>
       <c r="I12">
         <v>1</v>
+      </c>
+      <c r="J12" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="75">
@@ -13072,13 +13139,19 @@
         <v>46067</v>
       </c>
       <c r="F13">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="G13">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
       </c>
       <c r="I13">
         <v>1</v>
+      </c>
+      <c r="J13" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="93.75">
@@ -13098,13 +13171,19 @@
         <v>46067</v>
       </c>
       <c r="F14">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="G14">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
       </c>
       <c r="I14">
         <v>1</v>
+      </c>
+      <c r="J14" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="75">
@@ -13124,13 +13203,19 @@
         <v>46067</v>
       </c>
       <c r="F15">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="G15">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
       </c>
       <c r="I15">
         <v>1</v>
+      </c>
+      <c r="J15" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="75">
@@ -13150,13 +13235,19 @@
         <v>46067</v>
       </c>
       <c r="F16">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G16">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
       </c>
       <c r="I16">
         <v>1</v>
+      </c>
+      <c r="J16" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="168.75">
@@ -13176,13 +13267,19 @@
         <v>46067</v>
       </c>
       <c r="F17">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="G17">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
       </c>
       <c r="I17">
         <v>1</v>
+      </c>
+      <c r="J17" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="150">
@@ -13202,13 +13299,19 @@
         <v>46067</v>
       </c>
       <c r="F18">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="G18">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
       </c>
       <c r="I18">
         <v>1</v>
+      </c>
+      <c r="J18" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="93.75">
@@ -13228,13 +13331,19 @@
         <v>46067</v>
       </c>
       <c r="F19">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G19">
-        <v>3639</v>
+        <v>3649</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
       </c>
       <c r="I19">
         <v>1</v>
+      </c>
+      <c r="J19" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="93.75">
@@ -13250,8 +13359,23 @@
       <c r="D20">
         <v>3640</v>
       </c>
+      <c r="E20" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F20">
+        <v>32</v>
+      </c>
+      <c r="G20">
+        <v>3649</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
       <c r="I20">
         <v>1</v>
+      </c>
+      <c r="J20" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="93.75">
@@ -13267,8 +13391,23 @@
       <c r="D21">
         <v>3640</v>
       </c>
+      <c r="E21" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F21">
+        <v>25</v>
+      </c>
+      <c r="G21">
+        <v>3649</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
       <c r="I21">
         <v>1</v>
+      </c>
+      <c r="J21" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="75">
@@ -13284,8 +13423,23 @@
       <c r="D22">
         <v>3640</v>
       </c>
+      <c r="E22" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F22">
+        <v>35</v>
+      </c>
+      <c r="G22">
+        <v>3649</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
       <c r="I22">
         <v>1</v>
+      </c>
+      <c r="J22" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -13301,8 +13455,23 @@
       <c r="D23">
         <v>3639</v>
       </c>
+      <c r="E23" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F23">
+        <v>27</v>
+      </c>
+      <c r="G23">
+        <v>3649</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
       <c r="I23">
         <v>1</v>
+      </c>
+      <c r="J23" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="24" spans="1:10">
@@ -13318,8 +13487,23 @@
       <c r="D24">
         <v>3639</v>
       </c>
+      <c r="E24" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F24">
+        <v>24</v>
+      </c>
+      <c r="G24">
+        <v>3649</v>
+      </c>
+      <c r="H24">
+        <v>1</v>
+      </c>
       <c r="I24">
         <v>1</v>
+      </c>
+      <c r="J24" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="25" spans="1:10">
@@ -13335,8 +13519,23 @@
       <c r="D25">
         <v>3639</v>
       </c>
+      <c r="E25" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F25">
+        <v>23</v>
+      </c>
+      <c r="G25">
+        <v>3649</v>
+      </c>
+      <c r="H25">
+        <v>1</v>
+      </c>
       <c r="I25">
         <v>1</v>
+      </c>
+      <c r="J25" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="112.5">
@@ -13352,8 +13551,23 @@
       <c r="D26">
         <v>3639</v>
       </c>
+      <c r="E26" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F26">
+        <v>51</v>
+      </c>
+      <c r="G26">
+        <v>3649</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
       <c r="I26">
         <v>1</v>
+      </c>
+      <c r="J26" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="112.5">
@@ -13369,8 +13583,23 @@
       <c r="D27">
         <v>3639</v>
       </c>
+      <c r="E27" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F27">
+        <v>23</v>
+      </c>
+      <c r="G27">
+        <v>3649</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
       <c r="I27">
         <v>1</v>
+      </c>
+      <c r="J27" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="75">
@@ -13386,8 +13615,23 @@
       <c r="D28">
         <v>3639</v>
       </c>
+      <c r="E28" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F28">
+        <v>27</v>
+      </c>
+      <c r="G28">
+        <v>3649</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
       <c r="I28">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="J28" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="29" spans="1:10">
@@ -13397,11 +13641,8 @@
       <c r="B29" s="3">
         <v>46069</v>
       </c>
-      <c r="I29">
+      <c r="H29">
         <v>2</v>
-      </c>
-      <c r="J29" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="75">
@@ -13417,8 +13658,20 @@
       <c r="D30">
         <v>3642</v>
       </c>
+      <c r="E30" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F30">
+        <v>35</v>
+      </c>
+      <c r="G30">
+        <v>3649</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
       <c r="I30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" t="s">
         <v>794</v>
@@ -13437,8 +13690,20 @@
       <c r="D31">
         <v>3642</v>
       </c>
+      <c r="E31" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F31">
+        <v>51</v>
+      </c>
+      <c r="G31">
+        <v>3649</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
       <c r="I31">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J31" t="s">
         <v>794</v>
@@ -13457,37 +13722,127 @@
       <c r="D32">
         <v>3642</v>
       </c>
-    </row>
-    <row r="33" spans="1:2">
+      <c r="E32" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F32">
+        <v>50</v>
+      </c>
+      <c r="G32">
+        <v>3649</v>
+      </c>
+      <c r="H32">
+        <v>1</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
+      </c>
+      <c r="J32" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10">
       <c r="A33" s="2" t="s">
         <v>921</v>
       </c>
       <c r="B33" s="3">
         <v>46071</v>
       </c>
-    </row>
-    <row r="34" spans="1:2">
+      <c r="E33" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F33">
+        <v>14</v>
+      </c>
+      <c r="G33">
+        <v>3649</v>
+      </c>
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33">
+        <v>1</v>
+      </c>
+      <c r="J33" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10">
       <c r="A34" s="2" t="s">
         <v>966</v>
       </c>
       <c r="B34" s="3">
         <v>46071</v>
       </c>
-    </row>
-    <row r="35" spans="1:2">
+      <c r="E34" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F34">
+        <v>5</v>
+      </c>
+      <c r="G34">
+        <v>3649</v>
+      </c>
+      <c r="H34">
+        <v>1</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10">
       <c r="A35" s="2" t="s">
         <v>967</v>
       </c>
       <c r="B35" s="3">
         <v>46071</v>
       </c>
-    </row>
-    <row r="36" spans="1:2">
+      <c r="E35" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F35">
+        <v>6</v>
+      </c>
+      <c r="G35">
+        <v>3649</v>
+      </c>
+      <c r="H35">
+        <v>1</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10">
       <c r="A36" s="2" t="s">
         <v>968</v>
       </c>
       <c r="B36" s="3">
         <v>46071</v>
+      </c>
+      <c r="E36" s="3">
+        <v>46071</v>
+      </c>
+      <c r="F36">
+        <v>3</v>
+      </c>
+      <c r="G36">
+        <v>3649</v>
+      </c>
+      <c r="H36">
+        <v>1</v>
+      </c>
+      <c r="I36">
+        <v>1</v>
+      </c>
+      <c r="J36" t="s">
+        <v>794</v>
       </c>
     </row>
   </sheetData>
@@ -13730,7 +14085,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -14118,7 +14473,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -14764,7 +15119,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46071</v>
+        <v>46072</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
中 CHRO の主要導線 People Help が Coming soon の死に導線でした。実運用で詰まるので、chro_office_page.dart:102 から新設の people_help_page.dart:8 へ接続し、notes / onboarding memo / rewards / stats の即時導線に置き換えました。
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5F273B-7127-409E-8D8C-01FA9146A173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9055A55F-239E-49E7-89BE-FD974CD6A682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="23" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1730" uniqueCount="1067">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1732" uniqueCount="1069">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -6499,6 +6499,14 @@
   </si>
   <si>
     <t>プロジェクト全体をレビューして改善してください。</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>Skilled collaborations to produce win-win relationships that both increase and divide up wealth and power well are much more rewarding and much less painful than wars that lead to one side subjugating the other. Seeing things through your adversary’s eyes and clearly identifying and communicating your red lines to them (i.e., what cannot be compromised) are the keys to doing this well. * Winning means getting the things that are most important without losing the things that are most important, so wars that cost much more in lives and money than they provide in benefits are stupid. But “stupid” wars still happen all the time for reasons that I will explain.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>熟練した協力関係によって、富と権力を増大させつつ適切に分配するウィンウィンの関係を築くことは、一方の側が他方を征服する戦争よりもはるかに有益で、はるかに苦痛が少ない。敵対者の視点で物事を捉え、自らのレッドライン（つまり妥協できない点）を明確に認識し、それを相手に伝えることが、これを成功させる鍵である。* 勝利とは、最も重要なものを失うことなく獲得することである。ゆえに、もたらす利益よりもはるかに多くの命と資金を犠牲にする戦争は愚かである。しかし「愚かな」戦争は、これから説明する理由により、今なお頻繁に発生している。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6928,7 +6936,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -7111,7 +7119,7 @@
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -7324,7 +7332,7 @@
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -7500,7 +7508,7 @@
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -11046,7 +11054,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -11541,7 +11549,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -11765,7 +11773,7 @@
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -12236,7 +12244,7 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="C2:Q267"/>
+  <dimension ref="C2:Q268"/>
   <sheetFormatPr defaultRowHeight="18"/>
   <cols>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
@@ -14877,6 +14885,14 @@
       </c>
       <c r="I267" s="1" t="s">
         <v>1050</v>
+      </c>
+    </row>
+    <row r="268" spans="6:10" ht="180">
+      <c r="F268" s="1" t="s">
+        <v>1067</v>
+      </c>
+      <c r="I268" s="1" t="s">
+        <v>1068</v>
       </c>
     </row>
   </sheetData>
@@ -16742,7 +16758,7 @@
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46087</v>
+        <v>46093</v>
       </c>
       <c r="G1">
         <v>107</v>

</xml_diff>

<commit_message>
embedding_lab_page.dart を embedding-gecko-001:embedText から gemini-embedding-001:embedContent ベースへ移行しました。
</commit_message>
<xml_diff>
--- a/my_web_app.xlsx
+++ b/my_web_app.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kanta\GitHub\my_web_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AA18259-F803-410C-915D-574688DE2997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB9C8FF-A92D-4CC3-BECD-4CA804C999F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" firstSheet="10" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="15" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="目次" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1728" uniqueCount="1072">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1730" uniqueCount="1074">
   <si>
     <t>linterエラーを0にする</t>
     <phoneticPr fontId="1"/>
@@ -6522,6 +6522,14 @@
   </si>
   <si>
     <t>Gemini 2.0 Flash-Lite</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>I’ve quit 10x more goals than I’ve achieved.</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>達成した目標の10倍もの目標を、途中で諦めてきた。</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -6912,9 +6920,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="C3:C4"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:3">
@@ -6940,18 +6948,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32515FA5-1C1F-4EBA-80C2-D5F40752231E}">
   <dimension ref="B1:H19"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.59765625" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -7123,18 +7131,18 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A27E184-E904-4778-A996-9404F32C3EC7}">
   <dimension ref="B1:I19"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="6" max="7" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9">
       <c r="F1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="2" spans="2:9">
@@ -7151,7 +7159,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="90">
+    <row r="3" spans="2:9" ht="93.75">
       <c r="B3">
         <v>1</v>
       </c>
@@ -7188,7 +7196,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="2:9" ht="90">
+    <row r="6" spans="2:9" ht="93.75">
       <c r="B6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -7206,7 +7214,7 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="7" spans="2:9" ht="36">
+    <row r="7" spans="2:9" ht="37.5">
       <c r="B7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -7224,7 +7232,7 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="8" spans="2:9" ht="72">
+    <row r="8" spans="2:9" ht="75">
       <c r="B8">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -7248,7 +7256,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="10" spans="2:9" ht="36">
+    <row r="10" spans="2:9" ht="37.5">
       <c r="B10">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -7259,7 +7267,7 @@
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
     </row>
-    <row r="11" spans="2:9" ht="36">
+    <row r="11" spans="2:9" ht="37.5">
       <c r="B11">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -7277,7 +7285,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="13" spans="2:9" ht="36">
+    <row r="13" spans="2:9" ht="37.5">
       <c r="B13">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -7336,18 +7344,18 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{475FE61E-6EC0-4C61-9FD0-98172694F2E5}">
   <dimension ref="B1:H19"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.59765625" customWidth="1"/>
-    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.625" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="2" spans="2:8">
@@ -7374,7 +7382,7 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="2:8" ht="36">
+    <row r="4" spans="2:8" ht="37.5">
       <c r="B4">
         <f t="shared" ref="B4:B19" si="0">B3+1</f>
         <v>2</v>
@@ -7385,7 +7393,7 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
     </row>
-    <row r="5" spans="2:8" ht="36">
+    <row r="5" spans="2:8" ht="37.5">
       <c r="B5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -7396,7 +7404,7 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
     </row>
-    <row r="6" spans="2:8" ht="36">
+    <row r="6" spans="2:8" ht="37.5">
       <c r="B6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -7407,7 +7415,7 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
     </row>
-    <row r="7" spans="2:8" ht="90">
+    <row r="7" spans="2:8" ht="93.75">
       <c r="B7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -7506,24 +7514,24 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F96D129-34E8-4B10-A261-7AEE00EA03AD}">
   <dimension ref="B1:Q629"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="46.09765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="48.19921875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="47.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="47.69921875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="46.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.25" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="47.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="47.75" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.25" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.09765625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.09765625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="16.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:17">
       <c r="B1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="2" spans="2:17">
@@ -7564,7 +7572,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="3" spans="2:17" ht="36">
+    <row r="3" spans="2:17" ht="37.5">
       <c r="E3" t="s">
         <v>493</v>
       </c>
@@ -7590,7 +7598,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="4" spans="2:17" ht="72">
+    <row r="4" spans="2:17" ht="75">
       <c r="E4" t="s">
         <v>503</v>
       </c>
@@ -7631,7 +7639,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:17" ht="72">
+    <row r="5" spans="2:17" ht="75">
       <c r="E5" t="s">
         <v>514</v>
       </c>
@@ -7672,7 +7680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:17" ht="54">
+    <row r="6" spans="2:17" ht="56.25">
       <c r="E6" t="s">
         <v>518</v>
       </c>
@@ -7710,7 +7718,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:17" ht="72">
+    <row r="7" spans="2:17" ht="75">
       <c r="B7" s="3">
         <v>46043</v>
       </c>
@@ -7751,7 +7759,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:17" ht="72">
+    <row r="8" spans="2:17" ht="75">
       <c r="B8" s="3">
         <v>46044</v>
       </c>
@@ -7792,7 +7800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:17" ht="54">
+    <row r="9" spans="2:17" ht="56.25">
       <c r="B9" s="3">
         <v>46050</v>
       </c>
@@ -7833,7 +7841,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:17" ht="72">
+    <row r="10" spans="2:17" ht="75">
       <c r="B10" s="3">
         <v>46096</v>
       </c>
@@ -7874,7 +7882,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="2:17" ht="72">
+    <row r="11" spans="2:17" ht="75">
       <c r="B11" s="3">
         <v>46096</v>
       </c>
@@ -11017,17 +11025,17 @@
     <tabColor theme="9"/>
   </sheetPr>
   <dimension ref="B1:E66"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="51.69921875" customWidth="1"/>
-    <col min="3" max="3" width="51.19921875" customWidth="1"/>
-    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.75" customWidth="1"/>
+    <col min="3" max="3" width="51.25" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -11067,7 +11075,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="54">
+    <row r="9" spans="2:5" ht="56.25">
       <c r="B9" s="1" t="s">
         <v>58</v>
       </c>
@@ -11075,7 +11083,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="36">
+    <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
         <v>60</v>
       </c>
@@ -11083,7 +11091,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="36">
+    <row r="11" spans="2:5" ht="37.5">
       <c r="B11" s="1" t="s">
         <v>62</v>
       </c>
@@ -11091,7 +11099,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="54">
+    <row r="12" spans="2:5" ht="56.25">
       <c r="B12" s="1" t="s">
         <v>64</v>
       </c>
@@ -11108,7 +11116,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="36">
+    <row r="16" spans="2:5" ht="37.5">
       <c r="B16" s="1" t="s">
         <v>68</v>
       </c>
@@ -11116,7 +11124,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="72">
+    <row r="18" spans="2:5" ht="93.75">
       <c r="B18" s="1" t="s">
         <v>70</v>
       </c>
@@ -11125,7 +11133,7 @@
       </c>
       <c r="E18" s="3"/>
     </row>
-    <row r="19" spans="2:5" ht="90">
+    <row r="19" spans="2:5" ht="93.75">
       <c r="B19" s="1" t="s">
         <v>72</v>
       </c>
@@ -11134,7 +11142,7 @@
       </c>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="2:5" ht="54">
+    <row r="20" spans="2:5" ht="56.25">
       <c r="B20" s="1" t="s">
         <v>74</v>
       </c>
@@ -11145,7 +11153,7 @@
         <v>46037</v>
       </c>
     </row>
-    <row r="21" spans="2:5" ht="54">
+    <row r="21" spans="2:5" ht="56.25">
       <c r="B21" s="1" t="s">
         <v>81</v>
       </c>
@@ -11156,7 +11164,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="22" spans="2:5" ht="36">
+    <row r="22" spans="2:5" ht="56.25">
       <c r="B22" s="1" t="s">
         <v>89</v>
       </c>
@@ -11167,7 +11175,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="23" spans="2:5" ht="72">
+    <row r="23" spans="2:5" ht="93.75">
       <c r="B23" s="1" t="s">
         <v>124</v>
       </c>
@@ -11178,7 +11186,7 @@
         <v>46038</v>
       </c>
     </row>
-    <row r="24" spans="2:5" ht="54">
+    <row r="24" spans="2:5" ht="56.25">
       <c r="B24" s="1" t="s">
         <v>291</v>
       </c>
@@ -11197,7 +11205,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="28" spans="2:5" ht="54">
+    <row r="28" spans="2:5" ht="56.25">
       <c r="B28" s="1" t="s">
         <v>294</v>
       </c>
@@ -11208,7 +11216,7 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="29" spans="2:5" ht="36">
+    <row r="29" spans="2:5" ht="37.5">
       <c r="B29" s="1" t="s">
         <v>544</v>
       </c>
@@ -11219,12 +11227,12 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="30" spans="2:5" ht="306">
+    <row r="30" spans="2:5" ht="318.75">
       <c r="B30" s="1" t="s">
         <v>546</v>
       </c>
     </row>
-    <row r="31" spans="2:5" ht="36">
+    <row r="31" spans="2:5" ht="37.5">
       <c r="B31" s="1" t="s">
         <v>547</v>
       </c>
@@ -11246,7 +11254,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="35" spans="2:5" ht="36">
+    <row r="35" spans="2:5" ht="37.5">
       <c r="B35" s="1" t="s">
         <v>551</v>
       </c>
@@ -11254,7 +11262,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="36" spans="2:5" ht="36">
+    <row r="36" spans="2:5" ht="37.5">
       <c r="B36" s="1" t="s">
         <v>553</v>
       </c>
@@ -11265,7 +11273,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="37" spans="2:5" ht="54">
+    <row r="37" spans="2:5" ht="56.25">
       <c r="B37" s="1" t="s">
         <v>555</v>
       </c>
@@ -11276,7 +11284,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="38" spans="2:5" ht="90">
+    <row r="38" spans="2:5" ht="93.75">
       <c r="B38" s="1" t="s">
         <v>557</v>
       </c>
@@ -11295,7 +11303,7 @@
         <v>570</v>
       </c>
     </row>
-    <row r="42" spans="2:5" ht="54">
+    <row r="42" spans="2:5" ht="56.25">
       <c r="B42" s="1" t="s">
         <v>571</v>
       </c>
@@ -11306,7 +11314,7 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="43" spans="2:5">
+    <row r="43" spans="2:5" ht="37.5">
       <c r="B43" s="1" t="s">
         <v>573</v>
       </c>
@@ -11314,7 +11322,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="44" spans="2:5" ht="36">
+    <row r="44" spans="2:5" ht="37.5">
       <c r="B44" s="1" t="s">
         <v>575</v>
       </c>
@@ -11322,7 +11330,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="45" spans="2:5" ht="36">
+    <row r="45" spans="2:5" ht="37.5">
       <c r="B45" s="1" t="s">
         <v>577</v>
       </c>
@@ -11333,7 +11341,7 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="46" spans="2:5" ht="54">
+    <row r="46" spans="2:5" ht="56.25">
       <c r="B46" s="1" t="s">
         <v>587</v>
       </c>
@@ -11344,7 +11352,7 @@
         <v>46050</v>
       </c>
     </row>
-    <row r="47" spans="2:5" ht="54">
+    <row r="47" spans="2:5" ht="56.25">
       <c r="B47" s="1" t="s">
         <v>595</v>
       </c>
@@ -11355,7 +11363,7 @@
         <v>46050</v>
       </c>
     </row>
-    <row r="48" spans="2:5" ht="36">
+    <row r="48" spans="2:5" ht="37.5">
       <c r="B48" s="1" t="s">
         <v>597</v>
       </c>
@@ -11366,7 +11374,7 @@
         <v>46050</v>
       </c>
     </row>
-    <row r="49" spans="2:5" ht="396">
+    <row r="49" spans="2:5" ht="409.5">
       <c r="B49" s="1" t="s">
         <v>599</v>
       </c>
@@ -11385,7 +11393,7 @@
         <v>46050</v>
       </c>
     </row>
-    <row r="53" spans="2:5" ht="36">
+    <row r="53" spans="2:5" ht="37.5">
       <c r="B53" s="1" t="s">
         <v>602</v>
       </c>
@@ -11393,7 +11401,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="54" spans="2:5" ht="36">
+    <row r="54" spans="2:5" ht="37.5">
       <c r="B54" s="1" t="s">
         <v>604</v>
       </c>
@@ -11401,7 +11409,7 @@
         <v>605</v>
       </c>
     </row>
-    <row r="55" spans="2:5" ht="54">
+    <row r="55" spans="2:5" ht="56.25">
       <c r="B55" s="1" t="s">
         <v>606</v>
       </c>
@@ -11409,7 +11417,7 @@
         <v>607</v>
       </c>
     </row>
-    <row r="56" spans="2:5" ht="36">
+    <row r="56" spans="2:5" ht="37.5">
       <c r="B56" s="1" t="s">
         <v>608</v>
       </c>
@@ -11420,7 +11428,7 @@
         <v>46050</v>
       </c>
     </row>
-    <row r="57" spans="2:5" ht="36">
+    <row r="57" spans="2:5" ht="37.5">
       <c r="B57" s="1" t="s">
         <v>614</v>
       </c>
@@ -11439,7 +11447,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="61" spans="2:5" ht="36">
+    <row r="61" spans="2:5" ht="37.5">
       <c r="B61" s="1" t="s">
         <v>618</v>
       </c>
@@ -11455,7 +11463,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="65" spans="2:5" ht="36">
+    <row r="65" spans="2:5" ht="37.5">
       <c r="B65" s="1" t="s">
         <v>622</v>
       </c>
@@ -11466,7 +11474,7 @@
         <v>46060</v>
       </c>
     </row>
-    <row r="66" spans="2:5" ht="54">
+    <row r="66" spans="2:5" ht="56.25">
       <c r="B66" s="1" t="s">
         <v>624</v>
       </c>
@@ -11490,9 +11498,9 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF8ED9BD-4903-45DB-A379-2F8E5B42F77F}">
   <dimension ref="C3"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="81.69921875" customWidth="1"/>
+    <col min="3" max="3" width="81.75" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:3">
@@ -11512,17 +11520,17 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="B1:E28"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="73.09765625" customWidth="1"/>
+    <col min="2" max="2" width="73.125" customWidth="1"/>
     <col min="3" max="3" width="72.5" customWidth="1"/>
-    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -11562,7 +11570,7 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="9" spans="2:5" ht="36">
+    <row r="9" spans="2:5" ht="37.5">
       <c r="B9" s="1" t="s">
         <v>132</v>
       </c>
@@ -11570,7 +11578,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="36">
+    <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
         <v>134</v>
       </c>
@@ -11578,7 +11586,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="36">
+    <row r="11" spans="2:5" ht="37.5">
       <c r="B11" s="1" t="s">
         <v>136</v>
       </c>
@@ -11586,7 +11594,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="36">
+    <row r="12" spans="2:5" ht="37.5">
       <c r="B12" s="1" t="s">
         <v>138</v>
       </c>
@@ -11594,7 +11602,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="13" spans="2:5" ht="36">
+    <row r="13" spans="2:5" ht="37.5">
       <c r="B13" s="1" t="s">
         <v>140</v>
       </c>
@@ -11602,7 +11610,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="36">
+    <row r="14" spans="2:5" ht="37.5">
       <c r="B14" s="1" t="s">
         <v>142</v>
       </c>
@@ -11614,7 +11622,7 @@
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
     </row>
-    <row r="16" spans="2:5" ht="36">
+    <row r="16" spans="2:5" ht="37.5">
       <c r="B16" s="1" t="s">
         <v>226</v>
       </c>
@@ -11626,7 +11634,7 @@
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
     </row>
-    <row r="18" spans="2:5" ht="54">
+    <row r="18" spans="2:5" ht="56.25">
       <c r="B18" s="1" t="s">
         <v>228</v>
       </c>
@@ -11662,7 +11670,7 @@
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
     </row>
-    <row r="23" spans="2:5" ht="90">
+    <row r="23" spans="2:5" ht="93.75">
       <c r="B23" s="1" t="s">
         <v>541</v>
       </c>
@@ -11673,7 +11681,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="25" spans="2:5" ht="36">
+    <row r="25" spans="2:5" ht="56.25">
       <c r="B25" s="1" t="s">
         <v>560</v>
       </c>
@@ -11684,7 +11692,7 @@
         <v>46044</v>
       </c>
     </row>
-    <row r="26" spans="2:5" ht="54">
+    <row r="26" spans="2:5" ht="56.25">
       <c r="B26" s="1" t="s">
         <v>579</v>
       </c>
@@ -11695,7 +11703,7 @@
         <v>46045</v>
       </c>
     </row>
-    <row r="27" spans="2:5" ht="54">
+    <row r="27" spans="2:5" ht="56.25">
       <c r="B27" s="1" t="s">
         <v>583</v>
       </c>
@@ -11706,7 +11714,7 @@
         <v>46050</v>
       </c>
     </row>
-    <row r="28" spans="2:5" ht="72">
+    <row r="28" spans="2:5" ht="75">
       <c r="B28" s="1" t="s">
         <v>1054</v>
       </c>
@@ -11736,17 +11744,17 @@
     <tabColor rgb="FF00B0F0"/>
   </sheetPr>
   <dimension ref="B1:E16"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="45.09765625" customWidth="1"/>
+    <col min="2" max="2" width="45.125" customWidth="1"/>
     <col min="3" max="3" width="59.5" customWidth="1"/>
-    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:5">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
     </row>
     <row r="2" spans="2:5">
@@ -11788,7 +11796,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="36">
+    <row r="10" spans="2:5" ht="37.5">
       <c r="B10" s="1" t="s">
         <v>529</v>
       </c>
@@ -11796,7 +11804,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="36">
+    <row r="11" spans="2:5" ht="37.5">
       <c r="B11" s="1" t="s">
         <v>531</v>
       </c>
@@ -11804,7 +11812,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="72">
+    <row r="12" spans="2:5" ht="75">
       <c r="B12" s="1" t="s">
         <v>533</v>
       </c>
@@ -11812,7 +11820,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="13" spans="2:5" ht="36">
+    <row r="13" spans="2:5" ht="37.5">
       <c r="B13" s="1" t="s">
         <v>535</v>
       </c>
@@ -11820,7 +11828,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="72">
+    <row r="14" spans="2:5" ht="75">
       <c r="B14" s="1" t="s">
         <v>537</v>
       </c>
@@ -11831,7 +11839,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="15" spans="2:5" ht="54">
+    <row r="15" spans="2:5" ht="56.25">
       <c r="B15" s="1" t="s">
         <v>539</v>
       </c>
@@ -11842,7 +11850,7 @@
         <v>46043</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="36">
+    <row r="16" spans="2:5" ht="37.5">
       <c r="B16" s="1" t="s">
         <v>585</v>
       </c>
@@ -11871,7 +11879,7 @@
     <tabColor theme="5"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <sheetData/>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11883,11 +11891,11 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="C2:D9"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <dimension ref="C2:D10"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="43.19921875" customWidth="1"/>
-    <col min="4" max="4" width="48.3984375" customWidth="1"/>
+    <col min="3" max="3" width="43.25" customWidth="1"/>
+    <col min="4" max="4" width="48.375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:4">
@@ -11903,7 +11911,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="6" spans="3:4" ht="36">
+    <row r="6" spans="3:4" ht="37.5">
       <c r="C6" s="1" t="s">
         <v>306</v>
       </c>
@@ -11911,7 +11919,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="7" spans="3:4" ht="36">
+    <row r="7" spans="3:4" ht="37.5">
       <c r="C7" s="1" t="s">
         <v>308</v>
       </c>
@@ -11919,7 +11927,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="8" spans="3:4" ht="108">
+    <row r="8" spans="3:4" ht="112.5">
       <c r="C8" s="1" t="s">
         <v>567</v>
       </c>
@@ -11927,12 +11935,20 @@
         <v>568</v>
       </c>
     </row>
-    <row r="9" spans="3:4" ht="36">
+    <row r="9" spans="3:4" ht="56.25">
       <c r="C9" s="1" t="s">
         <v>589</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>590</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4">
+      <c r="C10" s="1" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>1073</v>
       </c>
     </row>
   </sheetData>
@@ -11950,7 +11966,7 @@
     <tabColor rgb="FFC00000"/>
   </sheetPr>
   <dimension ref="B3:D20"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="60" bestFit="1" customWidth="1"/>
@@ -11996,7 +12012,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="72">
+    <row r="8" spans="2:4" ht="75">
       <c r="B8">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -12014,7 +12030,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="198">
+    <row r="10" spans="2:4" ht="206.25">
       <c r="B10">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -12023,7 +12039,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="36">
+    <row r="11" spans="2:4" ht="37.5">
       <c r="B11">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -12104,7 +12120,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="20" spans="2:3" ht="54">
+    <row r="20" spans="2:3" ht="56.25">
       <c r="B20">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -12122,14 +12138,14 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C540C251-7928-4CED-B9EB-2D2B5444C0F0}">
   <dimension ref="C3:E9"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="31.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="46.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="46.625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="94" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:5" ht="198">
+    <row r="3" spans="3:5" ht="206.25">
       <c r="C3" t="s">
         <v>91</v>
       </c>
@@ -12140,7 +12156,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="4" spans="3:5" ht="144">
+    <row r="4" spans="3:5" ht="150">
       <c r="C4" t="s">
         <v>94</v>
       </c>
@@ -12151,7 +12167,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="5" spans="3:5" ht="288">
+    <row r="5" spans="3:5" ht="300">
       <c r="C5" s="1" t="s">
         <v>97</v>
       </c>
@@ -12162,7 +12178,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="3:5" ht="409.6">
+    <row r="6" spans="3:5" ht="409.5">
       <c r="C6" t="s">
         <v>112</v>
       </c>
@@ -12173,7 +12189,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="7" spans="3:5" ht="409.6">
+    <row r="7" spans="3:5" ht="409.5">
       <c r="C7" t="s">
         <v>115</v>
       </c>
@@ -12184,7 +12200,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="8" spans="3:5" ht="252">
+    <row r="8" spans="3:5" ht="262.5">
       <c r="C8" t="s">
         <v>118</v>
       </c>
@@ -12195,7 +12211,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" spans="3:5" ht="126">
+    <row r="9" spans="3:5" ht="131.25">
       <c r="C9" t="s">
         <v>121</v>
       </c>
@@ -12218,21 +12234,21 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="C2:Q270"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="3" max="3" width="58" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.09765625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="67.8984375" customWidth="1"/>
-    <col min="6" max="6" width="59.59765625" customWidth="1"/>
-    <col min="7" max="7" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="67.875" customWidth="1"/>
+    <col min="6" max="6" width="59.625" customWidth="1"/>
+    <col min="7" max="7" width="10.25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="54.5" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="52.5" customWidth="1"/>
-    <col min="11" max="11" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.09765625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="17.09765625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="7.09765625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:17">
@@ -12270,7 +12286,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="3" spans="3:17" ht="90">
+    <row r="3" spans="3:17" ht="93.75">
       <c r="C3" s="2" t="s">
         <v>627</v>
       </c>
@@ -12284,7 +12300,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="4" spans="3:17" ht="126">
+    <row r="4" spans="3:17" ht="150">
       <c r="F4" s="1" t="s">
         <v>631</v>
       </c>
@@ -12322,7 +12338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="3:17" ht="216">
+    <row r="5" spans="3:17" ht="225">
       <c r="H5" t="s">
         <v>634</v>
       </c>
@@ -12351,7 +12367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="3:17" ht="72">
+    <row r="6" spans="3:17" ht="75">
       <c r="H6" t="s">
         <v>635</v>
       </c>
@@ -12457,7 +12473,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="23" spans="3:16" ht="108">
+    <row r="23" spans="3:16" ht="112.5">
       <c r="C23" s="2" t="s">
         <v>655</v>
       </c>
@@ -12471,7 +12487,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="24" spans="3:16" ht="126">
+    <row r="24" spans="3:16" ht="131.25">
       <c r="F24" s="1" t="s">
         <v>660</v>
       </c>
@@ -12506,7 +12522,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="25" spans="3:16" ht="270">
+    <row r="25" spans="3:16" ht="281.25">
       <c r="H25" t="s">
         <v>662</v>
       </c>
@@ -12532,7 +12548,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="26" spans="3:16" ht="90">
+    <row r="26" spans="3:16" ht="93.75">
       <c r="H26" t="s">
         <v>663</v>
       </c>
@@ -12593,7 +12609,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="34" spans="3:16" ht="108">
+    <row r="34" spans="3:16" ht="112.5">
       <c r="C34" s="2" t="s">
         <v>679</v>
       </c>
@@ -12607,7 +12623,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="35" spans="3:16" ht="180">
+    <row r="35" spans="3:16" ht="206.25">
       <c r="F35" s="1" t="s">
         <v>683</v>
       </c>
@@ -12642,7 +12658,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="36" spans="3:16" ht="108">
+    <row r="36" spans="3:16" ht="112.5">
       <c r="H36" t="s">
         <v>685</v>
       </c>
@@ -12668,7 +12684,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="37" spans="3:16" ht="90">
+    <row r="37" spans="3:16" ht="93.75">
       <c r="H37" t="s">
         <v>686</v>
       </c>
@@ -12794,7 +12810,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="58" spans="3:16" ht="409.6">
+    <row r="58" spans="3:16" ht="409.5">
       <c r="C58" s="2" t="s">
         <v>710</v>
       </c>
@@ -12808,7 +12824,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="59" spans="3:16" ht="180">
+    <row r="59" spans="3:16" ht="187.5">
       <c r="F59" s="1" t="s">
         <v>714</v>
       </c>
@@ -12843,7 +12859,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="60" spans="3:16" ht="198">
+    <row r="60" spans="3:16" ht="206.25">
       <c r="H60" t="s">
         <v>716</v>
       </c>
@@ -12869,7 +12885,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="61" spans="3:16" ht="108">
+    <row r="61" spans="3:16" ht="112.5">
       <c r="H61" t="s">
         <v>717</v>
       </c>
@@ -12951,7 +12967,7 @@
         <v>728</v>
       </c>
     </row>
-    <row r="73" spans="3:16" ht="409.6">
+    <row r="73" spans="3:16" ht="409.5">
       <c r="C73" s="2" t="s">
         <v>732</v>
       </c>
@@ -12965,7 +12981,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="74" spans="3:16" ht="252">
+    <row r="74" spans="3:16" ht="281.25">
       <c r="F74" s="1" t="s">
         <v>736</v>
       </c>
@@ -13000,7 +13016,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="75" spans="3:16" ht="108">
+    <row r="75" spans="3:16" ht="112.5">
       <c r="H75" t="s">
         <v>738</v>
       </c>
@@ -13026,7 +13042,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="76" spans="3:16" ht="90">
+    <row r="76" spans="3:16" ht="112.5">
       <c r="H76" t="s">
         <v>739</v>
       </c>
@@ -13182,7 +13198,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="103" spans="3:16" ht="162">
+    <row r="103" spans="3:16" ht="168.75">
       <c r="C103" s="2" t="s">
         <v>769</v>
       </c>
@@ -13196,7 +13212,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="104" spans="3:16" ht="180">
+    <row r="104" spans="3:16" ht="187.5">
       <c r="F104" s="1" t="s">
         <v>773</v>
       </c>
@@ -13231,7 +13247,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="105" spans="3:16" ht="180">
+    <row r="105" spans="3:16" ht="187.5">
       <c r="H105" t="s">
         <v>775</v>
       </c>
@@ -13257,7 +13273,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="106" spans="3:16" ht="108">
+    <row r="106" spans="3:16" ht="112.5">
       <c r="H106" t="s">
         <v>776</v>
       </c>
@@ -13338,7 +13354,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="118" spans="3:13" ht="72">
+    <row r="118" spans="3:13" ht="75">
       <c r="C118" s="2" t="s">
         <v>798</v>
       </c>
@@ -13352,7 +13368,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="119" spans="3:13" ht="409.6">
+    <row r="119" spans="3:13" ht="409.5">
       <c r="F119" s="1" t="s">
         <v>802</v>
       </c>
@@ -13378,7 +13394,7 @@
         <v>3640</v>
       </c>
     </row>
-    <row r="120" spans="3:13" ht="126">
+    <row r="120" spans="3:13" ht="131.25">
       <c r="H120" t="s">
         <v>803</v>
       </c>
@@ -13395,7 +13411,7 @@
         <v>3640</v>
       </c>
     </row>
-    <row r="121" spans="3:13" ht="90">
+    <row r="121" spans="3:13" ht="93.75">
       <c r="H121" t="s">
         <v>804</v>
       </c>
@@ -13697,7 +13713,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="179" spans="3:13" ht="144">
+    <row r="179" spans="3:13" ht="168.75">
       <c r="C179" s="2" t="s">
         <v>865</v>
       </c>
@@ -13711,7 +13727,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="180" spans="3:13" ht="36">
+    <row r="180" spans="3:13" ht="37.5">
       <c r="F180" t="s">
         <v>869</v>
       </c>
@@ -13762,7 +13778,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="183" spans="3:13" ht="162">
+    <row r="183" spans="3:13" ht="168.75">
       <c r="C183" s="2" t="s">
         <v>874</v>
       </c>
@@ -13776,7 +13792,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="184" spans="3:13" ht="162">
+    <row r="184" spans="3:13" ht="168.75">
       <c r="F184" s="1" t="s">
         <v>878</v>
       </c>
@@ -13799,7 +13815,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="185" spans="3:13" ht="144">
+    <row r="185" spans="3:13" ht="168.75">
       <c r="H185" t="s">
         <v>879</v>
       </c>
@@ -13816,7 +13832,7 @@
         <v>3639</v>
       </c>
     </row>
-    <row r="186" spans="3:13" ht="108">
+    <row r="186" spans="3:13" ht="112.5">
       <c r="H186" t="s">
         <v>880</v>
       </c>
@@ -13882,7 +13898,7 @@
         <v>888</v>
       </c>
     </row>
-    <row r="195" spans="3:13" ht="409.6">
+    <row r="195" spans="3:13" ht="409.5">
       <c r="C195" s="2" t="s">
         <v>892</v>
       </c>
@@ -13896,7 +13912,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="196" spans="3:13" ht="108">
+    <row r="196" spans="3:13" ht="112.5">
       <c r="F196" t="s">
         <v>896</v>
       </c>
@@ -13922,7 +13938,7 @@
         <v>3642</v>
       </c>
     </row>
-    <row r="197" spans="3:13" ht="108">
+    <row r="197" spans="3:13" ht="112.5">
       <c r="H197" t="s">
         <v>898</v>
       </c>
@@ -13939,7 +13955,7 @@
         <v>3642</v>
       </c>
     </row>
-    <row r="198" spans="3:13" ht="72">
+    <row r="198" spans="3:13" ht="75">
       <c r="H198" t="s">
         <v>899</v>
       </c>
@@ -14001,7 +14017,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="208" spans="3:13" ht="144">
+    <row r="208" spans="3:13" ht="150">
       <c r="C208" s="2" t="s">
         <v>913</v>
       </c>
@@ -14018,7 +14034,7 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="209" spans="3:11" ht="36">
+    <row r="209" spans="3:11" ht="37.5">
       <c r="F209" s="1" t="s">
         <v>917</v>
       </c>
@@ -14035,7 +14051,7 @@
         <v>46071</v>
       </c>
     </row>
-    <row r="210" spans="3:11" ht="162">
+    <row r="210" spans="3:11" ht="168.75">
       <c r="C210" s="2" t="s">
         <v>957</v>
       </c>
@@ -14064,7 +14080,7 @@
       <c r="I211" s="1"/>
       <c r="J211" s="2"/>
     </row>
-    <row r="212" spans="3:11" ht="36">
+    <row r="212" spans="3:11" ht="37.5">
       <c r="C212" s="2"/>
       <c r="E212" s="1"/>
       <c r="F212" s="1" t="s">
@@ -14109,7 +14125,7 @@
         <v>46071</v>
       </c>
     </row>
-    <row r="215" spans="3:11" ht="126">
+    <row r="215" spans="3:11" ht="131.25">
       <c r="C215" s="2" t="s">
         <v>970</v>
       </c>
@@ -14129,7 +14145,7 @@
       <c r="J215" s="2"/>
       <c r="K215" s="3"/>
     </row>
-    <row r="216" spans="3:11" ht="180">
+    <row r="216" spans="3:11" ht="187.5">
       <c r="C216" s="2"/>
       <c r="E216" s="1"/>
       <c r="F216" s="1" t="s">
@@ -14142,7 +14158,7 @@
       <c r="J216" s="2"/>
       <c r="K216" s="3"/>
     </row>
-    <row r="217" spans="3:11" ht="108">
+    <row r="217" spans="3:11" ht="112.5">
       <c r="C217" s="2" t="s">
         <v>995</v>
       </c>
@@ -14162,7 +14178,7 @@
       <c r="J217" s="2"/>
       <c r="K217" s="3"/>
     </row>
-    <row r="218" spans="3:11" ht="72">
+    <row r="218" spans="3:11" ht="75">
       <c r="C218" s="2"/>
       <c r="E218" s="1"/>
       <c r="F218" s="1" t="s">
@@ -14175,7 +14191,7 @@
       <c r="J218" s="2"/>
       <c r="K218" s="3"/>
     </row>
-    <row r="219" spans="3:11" ht="126">
+    <row r="219" spans="3:11" ht="131.25">
       <c r="C219" s="2" t="s">
         <v>1000</v>
       </c>
@@ -14208,7 +14224,7 @@
       <c r="J220" s="2"/>
       <c r="K220" s="3"/>
     </row>
-    <row r="221" spans="3:11" ht="144">
+    <row r="221" spans="3:11" ht="150">
       <c r="C221" s="2" t="s">
         <v>1004</v>
       </c>
@@ -14228,7 +14244,7 @@
       <c r="J221" s="2"/>
       <c r="K221" s="3"/>
     </row>
-    <row r="222" spans="3:11" ht="36">
+    <row r="222" spans="3:11" ht="37.5">
       <c r="C222" s="2"/>
       <c r="E222" s="1"/>
       <c r="F222" s="1" t="s">
@@ -14241,7 +14257,7 @@
       <c r="J222" s="2"/>
       <c r="K222" s="3"/>
     </row>
-    <row r="223" spans="3:11" ht="409.6">
+    <row r="223" spans="3:11" ht="409.5">
       <c r="C223" s="2" t="s">
         <v>975</v>
       </c>
@@ -14261,7 +14277,7 @@
       <c r="J223" s="2"/>
       <c r="K223" s="3"/>
     </row>
-    <row r="224" spans="3:11" ht="90">
+    <row r="224" spans="3:11" ht="93.75">
       <c r="C224" s="2"/>
       <c r="E224" s="1"/>
       <c r="F224" s="1" t="s">
@@ -14274,7 +14290,7 @@
       <c r="J224" s="2"/>
       <c r="K224" s="3"/>
     </row>
-    <row r="225" spans="3:11" ht="108">
+    <row r="225" spans="3:11" ht="131.25">
       <c r="C225" s="2" t="s">
         <v>1010</v>
       </c>
@@ -14307,7 +14323,7 @@
       <c r="J226" s="2"/>
       <c r="K226" s="3"/>
     </row>
-    <row r="227" spans="3:11" ht="306">
+    <row r="227" spans="3:11" ht="318.75">
       <c r="C227" s="2" t="s">
         <v>980</v>
       </c>
@@ -14340,7 +14356,7 @@
       <c r="J228" s="2"/>
       <c r="K228" s="3"/>
     </row>
-    <row r="229" spans="3:11" ht="180">
+    <row r="229" spans="3:11" ht="187.5">
       <c r="C229" s="2" t="s">
         <v>1015</v>
       </c>
@@ -14373,7 +14389,7 @@
       <c r="J230" s="2"/>
       <c r="K230" s="3"/>
     </row>
-    <row r="231" spans="3:11" ht="162">
+    <row r="231" spans="3:11" ht="168.75">
       <c r="C231" s="2" t="s">
         <v>985</v>
       </c>
@@ -14393,7 +14409,7 @@
       <c r="J231" s="2"/>
       <c r="K231" s="3"/>
     </row>
-    <row r="232" spans="3:11" ht="180">
+    <row r="232" spans="3:11" ht="187.5">
       <c r="C232" s="2"/>
       <c r="E232" s="1"/>
       <c r="F232" s="1" t="s">
@@ -14406,7 +14422,7 @@
       <c r="J232" s="2"/>
       <c r="K232" s="3"/>
     </row>
-    <row r="233" spans="3:11" ht="144">
+    <row r="233" spans="3:11" ht="150">
       <c r="C233" s="2" t="s">
         <v>990</v>
       </c>
@@ -14426,7 +14442,7 @@
       <c r="J233" s="2"/>
       <c r="K233" s="3"/>
     </row>
-    <row r="234" spans="3:11" ht="36">
+    <row r="234" spans="3:11" ht="37.5">
       <c r="C234" s="2"/>
       <c r="E234" s="1"/>
       <c r="F234" s="1" t="s">
@@ -14441,7 +14457,7 @@
       <c r="J234" s="2"/>
       <c r="K234" s="3"/>
     </row>
-    <row r="235" spans="3:11" ht="54">
+    <row r="235" spans="3:11" ht="75">
       <c r="C235" s="2"/>
       <c r="E235" s="1"/>
       <c r="F235" s="1" t="s">
@@ -14452,7 +14468,7 @@
       <c r="J235" s="2"/>
       <c r="K235" s="3"/>
     </row>
-    <row r="236" spans="3:11" ht="162">
+    <row r="236" spans="3:11" ht="187.5">
       <c r="C236" s="2" t="s">
         <v>1021</v>
       </c>
@@ -14485,7 +14501,7 @@
       </c>
       <c r="K237" s="3"/>
     </row>
-    <row r="238" spans="3:11" ht="76.2">
+    <row r="238" spans="3:11" ht="78.75">
       <c r="C238" s="2" t="s">
         <v>1031</v>
       </c>
@@ -14516,7 +14532,7 @@
       </c>
       <c r="K239" s="3"/>
     </row>
-    <row r="240" spans="3:11" ht="162">
+    <row r="240" spans="3:11" ht="168.75">
       <c r="C240" s="2" t="s">
         <v>1036</v>
       </c>
@@ -14536,7 +14552,7 @@
       <c r="J240" s="2"/>
       <c r="K240" s="3"/>
     </row>
-    <row r="241" spans="3:11" ht="162">
+    <row r="241" spans="3:11" ht="168.75">
       <c r="C241" s="2"/>
       <c r="E241" s="8"/>
       <c r="F241" s="1" t="s">
@@ -14547,7 +14563,7 @@
       <c r="J241" s="2"/>
       <c r="K241" s="3"/>
     </row>
-    <row r="242" spans="3:11" ht="144">
+    <row r="242" spans="3:11" ht="150">
       <c r="C242" s="2" t="s">
         <v>1041</v>
       </c>
@@ -14567,7 +14583,7 @@
       <c r="J242" s="2"/>
       <c r="K242" s="3"/>
     </row>
-    <row r="243" spans="3:11" ht="144">
+    <row r="243" spans="3:11" ht="150">
       <c r="C243" s="2"/>
       <c r="E243" s="8"/>
       <c r="F243" s="1" t="s">
@@ -14580,7 +14596,7 @@
       <c r="J243" s="2"/>
       <c r="K243" s="3"/>
     </row>
-    <row r="244" spans="3:11" ht="112.2">
+    <row r="244" spans="3:11" ht="116.25">
       <c r="C244" s="2" t="s">
         <v>1048</v>
       </c>
@@ -14609,7 +14625,7 @@
       <c r="J245" s="2"/>
       <c r="K245" s="3"/>
     </row>
-    <row r="246" spans="3:11" ht="54">
+    <row r="246" spans="3:11" ht="56.25">
       <c r="C246" s="2"/>
       <c r="E246" s="8"/>
       <c r="F246" s="1" t="s">
@@ -14623,7 +14639,7 @@
       <c r="J246" s="2"/>
       <c r="K246" s="3"/>
     </row>
-    <row r="247" spans="3:11" ht="90">
+    <row r="247" spans="3:11" ht="93.75">
       <c r="C247" s="2" t="s">
         <v>919</v>
       </c>
@@ -14640,7 +14656,7 @@
         <v>926</v>
       </c>
     </row>
-    <row r="248" spans="3:11" ht="234">
+    <row r="248" spans="3:11" ht="262.5">
       <c r="E248" s="1" t="s">
         <v>922</v>
       </c>
@@ -14657,7 +14673,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="249" spans="3:11" ht="234">
+    <row r="249" spans="3:11" ht="243.75">
       <c r="F249" s="1" t="s">
         <v>927</v>
       </c>
@@ -14668,7 +14684,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="250" spans="3:11" ht="306">
+    <row r="250" spans="3:11" ht="337.5">
       <c r="F250" s="1" t="s">
         <v>928</v>
       </c>
@@ -14679,7 +14695,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="251" spans="3:11" ht="180">
+    <row r="251" spans="3:11" ht="206.25">
       <c r="F251" s="1" t="s">
         <v>930</v>
       </c>
@@ -14690,7 +14706,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="252" spans="3:11" ht="72">
+    <row r="252" spans="3:11" ht="75">
       <c r="F252" s="1" t="s">
         <v>932</v>
       </c>
@@ -14701,7 +14717,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="253" spans="3:11" ht="54">
+    <row r="253" spans="3:11" ht="56.25">
       <c r="F253" s="1" t="s">
         <v>934</v>
       </c>
@@ -14712,7 +14728,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="254" spans="3:11" ht="234">
+    <row r="254" spans="3:11" ht="243.75">
       <c r="F254" s="1" t="s">
         <v>936</v>
       </c>
@@ -14723,7 +14739,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="255" spans="3:11" ht="72">
+    <row r="255" spans="3:11" ht="75">
       <c r="F255" s="1" t="s">
         <v>938</v>
       </c>
@@ -14734,7 +14750,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="256" spans="3:11" ht="162">
+    <row r="256" spans="3:11" ht="168.75">
       <c r="F256" s="1" t="s">
         <v>940</v>
       </c>
@@ -14745,7 +14761,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="257" spans="6:10" ht="90">
+    <row r="257" spans="6:10" ht="112.5">
       <c r="F257" s="1" t="s">
         <v>942</v>
       </c>
@@ -14756,7 +14772,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="258" spans="6:10" ht="108">
+    <row r="258" spans="6:10" ht="131.25">
       <c r="F258" s="1" t="s">
         <v>944</v>
       </c>
@@ -14767,7 +14783,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="259" spans="6:10" ht="126">
+    <row r="259" spans="6:10" ht="131.25">
       <c r="F259" s="1" t="s">
         <v>946</v>
       </c>
@@ -14778,7 +14794,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="260" spans="6:10" ht="36">
+    <row r="260" spans="6:10" ht="37.5">
       <c r="F260" s="1" t="s">
         <v>948</v>
       </c>
@@ -14789,7 +14805,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="261" spans="6:10" ht="198">
+    <row r="261" spans="6:10" ht="206.25">
       <c r="F261" s="1" t="s">
         <v>950</v>
       </c>
@@ -14800,7 +14816,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="262" spans="6:10" ht="162">
+    <row r="262" spans="6:10" ht="168.75">
       <c r="F262" s="1" t="s">
         <v>952</v>
       </c>
@@ -14811,7 +14827,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="263" spans="6:10" ht="36">
+    <row r="263" spans="6:10" ht="37.5">
       <c r="F263" s="1" t="s">
         <v>954</v>
       </c>
@@ -14822,7 +14838,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="264" spans="6:10" ht="342">
+    <row r="264" spans="6:10" ht="375">
       <c r="F264" s="1" t="s">
         <v>966</v>
       </c>
@@ -14833,7 +14849,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="265" spans="6:10" ht="108">
+    <row r="265" spans="6:10" ht="131.25">
       <c r="F265" s="1" t="s">
         <v>968</v>
       </c>
@@ -14844,7 +14860,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="266" spans="6:10" ht="144">
+    <row r="266" spans="6:10" ht="150">
       <c r="F266" s="1" t="s">
         <v>1028</v>
       </c>
@@ -14855,7 +14871,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="267" spans="6:10" ht="144">
+    <row r="267" spans="6:10" ht="150">
       <c r="F267" s="1" t="s">
         <v>1046</v>
       </c>
@@ -14866,7 +14882,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="268" spans="6:10" ht="180">
+    <row r="268" spans="6:10" ht="187.5">
       <c r="F268" s="1" t="s">
         <v>1064</v>
       </c>
@@ -14877,7 +14893,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="269" spans="6:10" ht="180">
+    <row r="269" spans="6:10" ht="187.5">
       <c r="F269" s="1" t="s">
         <v>1066</v>
       </c>
@@ -14888,7 +14904,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="270" spans="6:10" ht="126">
+    <row r="270" spans="6:10" ht="131.25">
       <c r="F270" s="1" t="s">
         <v>1068</v>
       </c>
@@ -14950,17 +14966,17 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{970790C5-0376-420E-A317-55DF989D7F43}">
   <dimension ref="A1:J36"/>
-  <sheetFormatPr defaultColWidth="73.19921875" defaultRowHeight="18"/>
+  <sheetFormatPr defaultColWidth="73.25" defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="77.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.09765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.19921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.09765625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.09765625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -14992,7 +15008,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="54">
+    <row r="2" spans="1:10" ht="56.25">
       <c r="A2" s="1" t="s">
         <v>652</v>
       </c>
@@ -15024,7 +15040,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="198">
+    <row r="3" spans="1:10" ht="206.25">
       <c r="A3" s="1" t="s">
         <v>653</v>
       </c>
@@ -15056,7 +15072,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="54">
+    <row r="4" spans="1:10" ht="56.25">
       <c r="A4" s="1" t="s">
         <v>654</v>
       </c>
@@ -15088,7 +15104,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="72">
+    <row r="5" spans="1:10" ht="75">
       <c r="A5" s="1" t="s">
         <v>676</v>
       </c>
@@ -15120,7 +15136,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="252">
+    <row r="6" spans="1:10" ht="262.5">
       <c r="A6" s="1" t="s">
         <v>677</v>
       </c>
@@ -15152,7 +15168,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="72">
+    <row r="7" spans="1:10" ht="75">
       <c r="A7" s="1" t="s">
         <v>678</v>
       </c>
@@ -15184,7 +15200,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="90">
+    <row r="8" spans="1:10" ht="93.75">
       <c r="A8" s="1" t="s">
         <v>707</v>
       </c>
@@ -15216,7 +15232,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="72">
+    <row r="9" spans="1:10" ht="75">
       <c r="A9" s="1" t="s">
         <v>708</v>
       </c>
@@ -15248,7 +15264,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="54">
+    <row r="10" spans="1:10" ht="75">
       <c r="A10" s="1" t="s">
         <v>709</v>
       </c>
@@ -15280,7 +15296,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="90">
+    <row r="11" spans="1:10" ht="93.75">
       <c r="A11" s="1" t="s">
         <v>729</v>
       </c>
@@ -15312,7 +15328,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="180">
+    <row r="12" spans="1:10" ht="187.5">
       <c r="A12" s="1" t="s">
         <v>730</v>
       </c>
@@ -15344,7 +15360,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="72">
+    <row r="13" spans="1:10" ht="75">
       <c r="A13" s="1" t="s">
         <v>731</v>
       </c>
@@ -15376,7 +15392,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="90">
+    <row r="14" spans="1:10" ht="93.75">
       <c r="A14" s="1" t="s">
         <v>766</v>
       </c>
@@ -15408,7 +15424,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="72">
+    <row r="15" spans="1:10" ht="75">
       <c r="A15" s="1" t="s">
         <v>767</v>
       </c>
@@ -15440,7 +15456,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="72">
+    <row r="16" spans="1:10" ht="75">
       <c r="A16" s="1" t="s">
         <v>768</v>
       </c>
@@ -15472,7 +15488,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="162">
+    <row r="17" spans="1:10" ht="168.75">
       <c r="A17" s="1" t="s">
         <v>787</v>
       </c>
@@ -15504,7 +15520,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="144">
+    <row r="18" spans="1:10" ht="150">
       <c r="A18" s="1" t="s">
         <v>788</v>
       </c>
@@ -15536,7 +15552,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="90">
+    <row r="19" spans="1:10" ht="93.75">
       <c r="A19" s="1" t="s">
         <v>789</v>
       </c>
@@ -15568,7 +15584,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="90">
+    <row r="20" spans="1:10" ht="93.75">
       <c r="A20" s="1" t="s">
         <v>862</v>
       </c>
@@ -15600,7 +15616,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="90">
+    <row r="21" spans="1:10" ht="93.75">
       <c r="A21" s="1" t="s">
         <v>863</v>
       </c>
@@ -15632,7 +15648,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="54">
+    <row r="22" spans="1:10" ht="75">
       <c r="A22" s="1" t="s">
         <v>864</v>
       </c>
@@ -15760,7 +15776,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="108">
+    <row r="26" spans="1:10" ht="112.5">
       <c r="A26" s="1" t="s">
         <v>889</v>
       </c>
@@ -15792,7 +15808,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="108">
+    <row r="27" spans="1:10" ht="112.5">
       <c r="A27" s="1" t="s">
         <v>890</v>
       </c>
@@ -15824,7 +15840,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="72">
+    <row r="28" spans="1:10" ht="75">
       <c r="A28" s="1" t="s">
         <v>891</v>
       </c>
@@ -15867,7 +15883,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="72">
+    <row r="30" spans="1:10" ht="75">
       <c r="A30" s="1" t="s">
         <v>909</v>
       </c>
@@ -15899,7 +15915,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="72">
+    <row r="31" spans="1:10" ht="75">
       <c r="A31" s="1" t="s">
         <v>910</v>
       </c>
@@ -15931,7 +15947,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="54">
+    <row r="32" spans="1:10" ht="56.25">
       <c r="A32" s="1" t="s">
         <v>911</v>
       </c>
@@ -16088,13 +16104,13 @@
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CEE3D6-6F68-4B25-8FF2-FA5306076EAF}">
   <dimension ref="B2:I34"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.09765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.3984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="9" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9">
@@ -16294,13 +16310,13 @@
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56AA8B76-448C-412D-8BE5-3DD6B31F5B46}">
   <dimension ref="C3:E10"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="39.8984375" customWidth="1"/>
-    <col min="4" max="4" width="9.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="39.875" customWidth="1"/>
+    <col min="4" max="4" width="9.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:5" ht="54">
+    <row r="3" spans="3:5" ht="56.25">
       <c r="C3" s="1" t="s">
         <v>1060</v>
       </c>
@@ -16311,7 +16327,7 @@
         <v>0.86041666666666672</v>
       </c>
     </row>
-    <row r="4" spans="3:5" ht="72">
+    <row r="4" spans="3:5" ht="75">
       <c r="C4" s="1" t="s">
         <v>1056</v>
       </c>
@@ -16322,7 +16338,7 @@
         <v>0.86041666666666672</v>
       </c>
     </row>
-    <row r="5" spans="3:5" ht="54">
+    <row r="5" spans="3:5" ht="75">
       <c r="C5" s="1" t="s">
         <v>1057</v>
       </c>
@@ -16333,7 +16349,7 @@
         <v>0.86111111111111116</v>
       </c>
     </row>
-    <row r="6" spans="3:5" ht="162">
+    <row r="6" spans="3:5" ht="187.5">
       <c r="C6" s="1" t="s">
         <v>1058</v>
       </c>
@@ -16344,7 +16360,7 @@
         <v>0.89513888888888893</v>
       </c>
     </row>
-    <row r="7" spans="3:5" ht="90">
+    <row r="7" spans="3:5" ht="112.5">
       <c r="C7" s="1" t="s">
         <v>1059</v>
       </c>
@@ -16355,7 +16371,7 @@
         <v>0.91319444444444442</v>
       </c>
     </row>
-    <row r="8" spans="3:5" ht="54">
+    <row r="8" spans="3:5" ht="56.25">
       <c r="C8" s="1" t="s">
         <v>1061</v>
       </c>
@@ -16366,7 +16382,7 @@
         <v>0.69722222222222219</v>
       </c>
     </row>
-    <row r="9" spans="3:5" ht="36">
+    <row r="9" spans="3:5" ht="37.5">
       <c r="C9" s="1" t="s">
         <v>1062</v>
       </c>
@@ -16377,7 +16393,7 @@
         <v>0.69722222222222219</v>
       </c>
     </row>
-    <row r="10" spans="3:5" ht="36">
+    <row r="10" spans="3:5" ht="37.5">
       <c r="C10" s="1" t="s">
         <v>1063</v>
       </c>
@@ -16397,13 +16413,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB9A9986-272E-4F2B-8815-9B72212F3499}">
   <dimension ref="B3:F8"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.3984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:6">
@@ -16488,10 +16504,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBEF53A6-A89B-421F-A561-8936407ADCF5}">
   <dimension ref="C2:E11"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="3" max="3" width="157.59765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="157.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="3:5">
@@ -16574,12 +16590,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62C7C188-6DA4-4CDE-8831-D70FA561BA5F}">
   <dimension ref="B3:H12"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.8984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -16746,23 +16762,23 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{831F138C-7B13-4940-8512-4B95D1A24D44}">
   <dimension ref="B1:L8"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.09765625" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10.19921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.25" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="78" customWidth="1"/>
     <col min="9" max="9" width="117.5" customWidth="1"/>
     <col min="10" max="10" width="101.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="196.59765625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="80.19921875" customWidth="1"/>
+    <col min="11" max="11" width="196.625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="80.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:12">
       <c r="E1" s="3">
         <f ca="1">TODAY()</f>
-        <v>46096</v>
+        <v>46098</v>
       </c>
       <c r="G1">
         <v>107</v>
@@ -16794,7 +16810,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="3" spans="2:12" ht="144">
+    <row r="3" spans="2:12" ht="150">
       <c r="B3">
         <v>1</v>
       </c>
@@ -16826,7 +16842,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="4" spans="2:12" ht="234">
+    <row r="4" spans="2:12" ht="243.75">
       <c r="B4">
         <f>B3+1</f>
         <v>2</v>
@@ -16859,7 +16875,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="2:12" ht="72">
+    <row r="5" spans="2:12" ht="75">
       <c r="B5">
         <f>B4+1</f>
         <v>3</v>
@@ -16892,7 +16908,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="6" spans="2:12" ht="234">
+    <row r="6" spans="2:12" ht="243.75">
       <c r="B6">
         <f>B5+1</f>
         <v>4</v>
@@ -16958,30 +16974,30 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A08533-9740-4130-8AB5-7E4127B4922F}">
   <dimension ref="B2:X13"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
-    <col min="2" max="2" width="3.69921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.09765625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.69921875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.19921875" customWidth="1"/>
-    <col min="6" max="6" width="54.8984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.8984375" customWidth="1"/>
-    <col min="8" max="8" width="22.59765625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.59765625" customWidth="1"/>
-    <col min="10" max="10" width="35.69921875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.09765625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.8984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="41.69921875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="32.59765625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.75" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="34.25" customWidth="1"/>
+    <col min="6" max="6" width="54.875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.875" customWidth="1"/>
+    <col min="8" max="8" width="22.625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.625" customWidth="1"/>
+    <col min="10" max="10" width="35.75" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="41.75" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="32.625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="75.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="65.69921875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="65.69921875" customWidth="1"/>
-    <col min="19" max="19" width="50.09765625" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="50.09765625" customWidth="1"/>
-    <col min="22" max="22" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="65.75" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="65.75" customWidth="1"/>
+    <col min="19" max="19" width="50.125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="50.125" customWidth="1"/>
+    <col min="22" max="22" width="10.25" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="47" customWidth="1"/>
-    <col min="24" max="24" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:24">
@@ -17049,7 +17065,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:24" ht="198">
+    <row r="3" spans="2:24" ht="225">
       <c r="B3">
         <v>1</v>
       </c>
@@ -17118,7 +17134,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="4" spans="2:24" ht="360">
+    <row r="4" spans="2:24" ht="375">
       <c r="B4">
         <f t="shared" ref="B4:B13" si="0">B3+1</f>
         <v>2</v>
@@ -17186,7 +17202,7 @@
         <v>46036</v>
       </c>
     </row>
-    <row r="5" spans="2:24" ht="198">
+    <row r="5" spans="2:24" ht="206.25">
       <c r="B5">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -17248,7 +17264,7 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="6" spans="2:24" ht="324">
+    <row r="6" spans="2:24" ht="337.5">
       <c r="B6">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -17310,7 +17326,7 @@
         <v>46039</v>
       </c>
     </row>
-    <row r="7" spans="2:24" ht="162">
+    <row r="7" spans="2:24" ht="187.5">
       <c r="B7">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -17349,7 +17365,7 @@
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
     </row>
-    <row r="9" spans="2:24" ht="144">
+    <row r="9" spans="2:24" ht="150">
       <c r="B9">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -17377,7 +17393,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="10" spans="2:24" ht="162">
+    <row r="10" spans="2:24" ht="168.75">
       <c r="B10">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -17405,7 +17421,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="11" spans="2:24" ht="126">
+    <row r="11" spans="2:24" ht="131.25">
       <c r="B11">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -17432,7 +17448,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="12" spans="2:24" ht="126">
+    <row r="12" spans="2:24" ht="131.25">
       <c r="B12">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -17460,7 +17476,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="13" spans="2:24" ht="126">
+    <row r="13" spans="2:24" ht="131.25">
       <c r="B13">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -17497,11 +17513,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCCFC25C-982C-4873-AE2A-E40A864E9987}">
   <dimension ref="B3:D3"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="2.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4">
@@ -17524,13 +17540,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EE8B69-0038-4D7F-ACFE-E2E709E6B1D2}">
   <dimension ref="B2:I26"/>
-  <sheetFormatPr defaultRowHeight="18"/>
+  <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="2" max="2" width="3.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="29.59765625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.09765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="10.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="29.625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="10.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:9">

</xml_diff>